<commit_message>
Actualizacion pedidos al 23/09/2026 con fichero Pedidos 24.09 comerciales
</commit_message>
<xml_diff>
--- a/Seguimiento_Presupuesto_Sep_2026.xlsx
+++ b/Seguimiento_Presupuesto_Sep_2026.xlsx
@@ -905,7 +905,7 @@
     <row r="3" ht="20" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Comparativa Budget Septiembre (Unidades) vs Pedidos Reales a Fecha 22/09/2026 | Generado: 23/09/2026 12:32</t>
+          <t>Comparativa Budget Septiembre (Unidades) vs Pedidos Reales a Fecha 23/09/2026 | Generado: 24/09/2026 07:12</t>
         </is>
       </c>
     </row>
@@ -943,31 +943,31 @@
     <row r="6" ht="28" customHeight="1">
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>172,503 u</t>
+          <t>181,966 u</t>
         </is>
       </c>
       <c r="C6" s="4" t="n"/>
       <c r="D6" s="8" t="inlineStr">
         <is>
-          <t>170,801 u</t>
+          <t>173,601 u</t>
         </is>
       </c>
       <c r="E6" s="4" t="n"/>
       <c r="F6" s="9" t="inlineStr">
         <is>
-          <t>99.0%</t>
+          <t>95.4%</t>
         </is>
       </c>
       <c r="G6" s="4" t="n"/>
       <c r="H6" s="10" t="inlineStr">
         <is>
-          <t>34,884 u</t>
+          <t>39,570 u</t>
         </is>
       </c>
       <c r="I6" s="4" t="n"/>
       <c r="J6" s="7" t="inlineStr">
         <is>
-          <t>90,844 u</t>
+          <t>93,644 u</t>
         </is>
       </c>
     </row>
@@ -1035,7 +1035,7 @@
         <v>10</v>
       </c>
       <c r="D10" s="15" t="n">
-        <v>2199.351043172263</v>
+        <v>2320</v>
       </c>
       <c r="E10" s="15" t="n">
         <v>10110</v>
@@ -1069,16 +1069,16 @@
         <v>5</v>
       </c>
       <c r="D11" s="19" t="n">
-        <v>35864.58994193666</v>
+        <v>37832</v>
       </c>
       <c r="E11" s="19" t="n">
-        <v>51772</v>
+        <v>52772</v>
       </c>
       <c r="F11" s="19" t="n">
         <v>2556</v>
       </c>
       <c r="G11" s="19" t="n">
-        <v>49216</v>
+        <v>50216</v>
       </c>
       <c r="H11" s="19">
         <f>MAX(0, D11-E11)</f>
@@ -1103,7 +1103,7 @@
         <v>3</v>
       </c>
       <c r="D12" s="15" t="n">
-        <v>20774.3873965849</v>
+        <v>21914</v>
       </c>
       <c r="E12" s="15" t="n">
         <v>12806</v>
@@ -1137,7 +1137,7 @@
         <v>8</v>
       </c>
       <c r="D13" s="19" t="n">
-        <v>16210.73398200246</v>
+        <v>17100</v>
       </c>
       <c r="E13" s="19" t="n">
         <v>25575</v>
@@ -1171,7 +1171,7 @@
         <v>1</v>
       </c>
       <c r="D14" s="15" t="n">
-        <v>37407.92765671444</v>
+        <v>39460</v>
       </c>
       <c r="E14" s="15" t="n">
         <v>32828</v>
@@ -1205,16 +1205,16 @@
         <v>3</v>
       </c>
       <c r="D15" s="19" t="n">
-        <v>16438.25305543407</v>
+        <v>17340</v>
       </c>
       <c r="E15" s="19" t="n">
-        <v>5860</v>
+        <v>7660</v>
       </c>
       <c r="F15" s="19" t="n">
         <v>5860</v>
       </c>
       <c r="G15" s="19" t="n">
-        <v>0</v>
+        <v>1800</v>
       </c>
       <c r="H15" s="19">
         <f>MAX(0, D15-E15)</f>
@@ -1239,7 +1239,7 @@
         <v>3</v>
       </c>
       <c r="D16" s="15" t="n">
-        <v>43607.8224077259</v>
+        <v>46000</v>
       </c>
       <c r="E16" s="15" t="n">
         <v>31850</v>
@@ -1330,17 +1330,17 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="2" ht="36" customHeight="1">
@@ -1353,7 +1353,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 22/09/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 23/09/2026</t>
         </is>
       </c>
     </row>
@@ -1392,7 +1392,7 @@
     <row r="6" ht="25" customHeight="1">
       <c r="B6" s="25" t="inlineStr">
         <is>
-          <t>2,199 u</t>
+          <t>2,320 u</t>
         </is>
       </c>
       <c r="C6" s="4" t="n"/>
@@ -1404,7 +1404,7 @@
       <c r="E6" s="4" t="n"/>
       <c r="F6" s="26" t="inlineStr">
         <is>
-          <t>459.7%</t>
+          <t>435.8%</t>
         </is>
       </c>
       <c r="G6" s="4" t="n"/>
@@ -1466,12 +1466,12 @@
       </c>
       <c r="I9" s="12" t="inlineStr">
         <is>
-          <t>Falta Conseguir (u)</t>
+          <t>Falta (u)</t>
         </is>
       </c>
       <c r="J9" s="12" t="inlineStr">
         <is>
-          <t>Desviación (u)</t>
+          <t>Desv. (u)</t>
         </is>
       </c>
       <c r="K9" s="12" t="inlineStr">
@@ -1502,7 +1502,7 @@
         </is>
       </c>
       <c r="E10" s="15" t="n">
-        <v>910.0762937264537</v>
+        <v>960</v>
       </c>
       <c r="F10" s="15" t="n">
         <v>1280</v>
@@ -1548,7 +1548,7 @@
         </is>
       </c>
       <c r="E11" s="19" t="n">
-        <v>910.0762937264537</v>
+        <v>960</v>
       </c>
       <c r="F11" s="19" t="n">
         <v>1920</v>
@@ -1732,7 +1732,7 @@
         </is>
       </c>
       <c r="E15" s="19" t="n">
-        <v>379.1984557193557</v>
+        <v>400</v>
       </c>
       <c r="F15" s="19" t="n">
         <v>320</v>
@@ -2663,17 +2663,17 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="2" ht="36" customHeight="1">
@@ -2686,7 +2686,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 22/09/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 23/09/2026</t>
         </is>
       </c>
     </row>
@@ -2725,19 +2725,19 @@
     <row r="6" ht="25" customHeight="1">
       <c r="B6" s="25" t="inlineStr">
         <is>
-          <t>35,865 u</t>
+          <t>37,832 u</t>
         </is>
       </c>
       <c r="C6" s="4" t="n"/>
       <c r="D6" s="26" t="inlineStr">
         <is>
-          <t>51,772 u</t>
+          <t>52,772 u</t>
         </is>
       </c>
       <c r="E6" s="4" t="n"/>
       <c r="F6" s="26" t="inlineStr">
         <is>
-          <t>144.4%</t>
+          <t>139.5%</t>
         </is>
       </c>
       <c r="G6" s="4" t="n"/>
@@ -2749,7 +2749,7 @@
       <c r="I6" s="4" t="n"/>
       <c r="J6" s="25" t="inlineStr">
         <is>
-          <t>49,216 u</t>
+          <t>50,216 u</t>
         </is>
       </c>
       <c r="K6" s="4" t="n"/>
@@ -2799,12 +2799,12 @@
       </c>
       <c r="I9" s="12" t="inlineStr">
         <is>
-          <t>Falta Conseguir (u)</t>
+          <t>Falta (u)</t>
         </is>
       </c>
       <c r="J9" s="12" t="inlineStr">
         <is>
-          <t>Desviación (u)</t>
+          <t>Desv. (u)</t>
         </is>
       </c>
       <c r="K9" s="12" t="inlineStr">
@@ -2835,7 +2835,7 @@
         </is>
       </c>
       <c r="E10" s="15" t="n">
-        <v>663.5972975088725</v>
+        <v>700</v>
       </c>
       <c r="F10" s="15" t="n">
         <v>0</v>
@@ -2881,7 +2881,7 @@
         </is>
       </c>
       <c r="E11" s="19" t="n">
-        <v>1895.992278596779</v>
+        <v>2000</v>
       </c>
       <c r="F11" s="19" t="n">
         <v>0</v>
@@ -2927,7 +2927,7 @@
         </is>
       </c>
       <c r="E12" s="15" t="n">
-        <v>284.3988417895168</v>
+        <v>300</v>
       </c>
       <c r="F12" s="15" t="n">
         <v>0</v>
@@ -3019,7 +3019,7 @@
         </is>
       </c>
       <c r="E14" s="15" t="n">
-        <v>2085.591506456457</v>
+        <v>2200</v>
       </c>
       <c r="F14" s="15" t="n">
         <v>1100</v>
@@ -3065,7 +3065,7 @@
         </is>
       </c>
       <c r="E15" s="19" t="n">
-        <v>1820.152587452907</v>
+        <v>1920</v>
       </c>
       <c r="F15" s="19" t="n">
         <v>640</v>
@@ -3111,16 +3111,16 @@
         </is>
       </c>
       <c r="E16" s="15" t="n">
-        <v>4739.980696491946</v>
+        <v>5000</v>
       </c>
       <c r="F16" s="15" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="G16" s="15" t="n">
         <v>0</v>
       </c>
       <c r="H16" s="15" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="I16" s="15">
         <f>MAX(0, E16-F16)</f>
@@ -3134,9 +3134,9 @@
         <f>IF(E16&gt;0, F16/E16, IF(F16&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L16" s="36" t="inlineStr">
-        <is>
-          <t>Sin Pedido</t>
+      <c r="L16" s="37" t="inlineStr">
+        <is>
+          <t>Rezagado</t>
         </is>
       </c>
     </row>
@@ -3157,7 +3157,7 @@
         </is>
       </c>
       <c r="E17" s="19" t="n">
-        <v>473.9980696491947</v>
+        <v>500</v>
       </c>
       <c r="F17" s="19" t="n">
         <v>0</v>
@@ -3203,7 +3203,7 @@
         </is>
       </c>
       <c r="E18" s="15" t="n">
-        <v>1042.795753228228</v>
+        <v>1100</v>
       </c>
       <c r="F18" s="15" t="n">
         <v>0</v>
@@ -3249,7 +3249,7 @@
         </is>
       </c>
       <c r="E19" s="19" t="n">
-        <v>189.5992278596779</v>
+        <v>200</v>
       </c>
       <c r="F19" s="19" t="n">
         <v>0</v>
@@ -3295,7 +3295,7 @@
         </is>
       </c>
       <c r="E20" s="15" t="n">
-        <v>284.3988417895168</v>
+        <v>300</v>
       </c>
       <c r="F20" s="15" t="n">
         <v>0</v>
@@ -3341,7 +3341,7 @@
         </is>
       </c>
       <c r="E21" s="19" t="n">
-        <v>94.79961392983893</v>
+        <v>100</v>
       </c>
       <c r="F21" s="19" t="n">
         <v>0</v>
@@ -3387,7 +3387,7 @@
         </is>
       </c>
       <c r="E22" s="15" t="n">
-        <v>284.3988417895168</v>
+        <v>300</v>
       </c>
       <c r="F22" s="15" t="n">
         <v>0</v>
@@ -3433,7 +3433,7 @@
         </is>
       </c>
       <c r="E23" s="19" t="n">
-        <v>189.5992278596779</v>
+        <v>200</v>
       </c>
       <c r="F23" s="19" t="n">
         <v>0</v>
@@ -3479,7 +3479,7 @@
         </is>
       </c>
       <c r="E24" s="15" t="n">
-        <v>189.5992278596779</v>
+        <v>200</v>
       </c>
       <c r="F24" s="15" t="n">
         <v>0</v>
@@ -3525,7 +3525,7 @@
         </is>
       </c>
       <c r="E25" s="19" t="n">
-        <v>18959.92278596778</v>
+        <v>20000</v>
       </c>
       <c r="F25" s="19" t="n">
         <v>21000</v>
@@ -3801,7 +3801,7 @@
         </is>
       </c>
       <c r="E31" s="19" t="n">
-        <v>606.7175291509692</v>
+        <v>640</v>
       </c>
       <c r="F31" s="19" t="n">
         <v>0</v>
@@ -3847,7 +3847,7 @@
         </is>
       </c>
       <c r="E32" s="15" t="n">
-        <v>56.87976835790336</v>
+        <v>60</v>
       </c>
       <c r="F32" s="15" t="n">
         <v>0</v>
@@ -4399,7 +4399,7 @@
         </is>
       </c>
       <c r="E44" s="15" t="n">
-        <v>189.5992278596779</v>
+        <v>200</v>
       </c>
       <c r="F44" s="15" t="n">
         <v>0</v>
@@ -4491,7 +4491,7 @@
         </is>
       </c>
       <c r="E46" s="15" t="n">
-        <v>94.79961392983893</v>
+        <v>100</v>
       </c>
       <c r="F46" s="15" t="n">
         <v>120</v>
@@ -4537,7 +4537,7 @@
         </is>
       </c>
       <c r="E47" s="19" t="n">
-        <v>11.37595367158067</v>
+        <v>12</v>
       </c>
       <c r="F47" s="19" t="n">
         <v>12</v>
@@ -4583,7 +4583,7 @@
         </is>
       </c>
       <c r="E48" s="15" t="n">
-        <v>284.3988417895168</v>
+        <v>300</v>
       </c>
       <c r="F48" s="15" t="n">
         <v>0</v>
@@ -4721,7 +4721,7 @@
         </is>
       </c>
       <c r="E51" s="19" t="n">
-        <v>284.3988417895168</v>
+        <v>300</v>
       </c>
       <c r="F51" s="19" t="n">
         <v>160</v>
@@ -4767,7 +4767,7 @@
         </is>
       </c>
       <c r="E52" s="15" t="n">
-        <v>94.79961392983893</v>
+        <v>100</v>
       </c>
       <c r="F52" s="15" t="n">
         <v>120</v>
@@ -4859,7 +4859,7 @@
         </is>
       </c>
       <c r="E54" s="15" t="n">
-        <v>1042.795753228228</v>
+        <v>1100</v>
       </c>
       <c r="F54" s="15" t="n">
         <v>0</v>
@@ -4896,7 +4896,7 @@
       </c>
       <c r="C55" s="34" t="inlineStr">
         <is>
-          <t>233 líneas</t>
+          <t>234 líneas</t>
         </is>
       </c>
       <c r="D55" s="35" t="inlineStr"/>
@@ -4962,17 +4962,17 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="2" ht="36" customHeight="1">
@@ -4985,7 +4985,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 22/09/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 23/09/2026</t>
         </is>
       </c>
     </row>
@@ -5024,7 +5024,7 @@
     <row r="6" ht="25" customHeight="1">
       <c r="B6" s="25" t="inlineStr">
         <is>
-          <t>20,774 u</t>
+          <t>21,914 u</t>
         </is>
       </c>
       <c r="C6" s="4" t="n"/>
@@ -5036,13 +5036,13 @@
       <c r="E6" s="4" t="n"/>
       <c r="F6" s="38" t="inlineStr">
         <is>
-          <t>61.6%</t>
+          <t>58.4%</t>
         </is>
       </c>
       <c r="G6" s="4" t="n"/>
       <c r="H6" s="38" t="inlineStr">
         <is>
-          <t>7,968 u</t>
+          <t>9,108 u</t>
         </is>
       </c>
       <c r="I6" s="4" t="n"/>
@@ -5098,12 +5098,12 @@
       </c>
       <c r="I9" s="12" t="inlineStr">
         <is>
-          <t>Falta Conseguir (u)</t>
+          <t>Falta (u)</t>
         </is>
       </c>
       <c r="J9" s="12" t="inlineStr">
         <is>
-          <t>Desviación (u)</t>
+          <t>Desv. (u)</t>
         </is>
       </c>
       <c r="K9" s="12" t="inlineStr">
@@ -5134,7 +5134,7 @@
         </is>
       </c>
       <c r="E10" s="15" t="n">
-        <v>189.5992278596779</v>
+        <v>200</v>
       </c>
       <c r="F10" s="15" t="n">
         <v>0</v>
@@ -5226,7 +5226,7 @@
         </is>
       </c>
       <c r="E12" s="15" t="n">
-        <v>1820.152587452907</v>
+        <v>1920</v>
       </c>
       <c r="F12" s="15" t="n">
         <v>0</v>
@@ -5272,7 +5272,7 @@
         </is>
       </c>
       <c r="E13" s="19" t="n">
-        <v>284.3988417895168</v>
+        <v>300</v>
       </c>
       <c r="F13" s="19" t="n">
         <v>0</v>
@@ -5318,7 +5318,7 @@
         </is>
       </c>
       <c r="E14" s="15" t="n">
-        <v>910.0762937264537</v>
+        <v>960</v>
       </c>
       <c r="F14" s="15" t="n">
         <v>640</v>
@@ -5364,7 +5364,7 @@
         </is>
       </c>
       <c r="E15" s="19" t="n">
-        <v>606.7175291509692</v>
+        <v>640</v>
       </c>
       <c r="F15" s="19" t="n">
         <v>0</v>
@@ -5410,7 +5410,7 @@
         </is>
       </c>
       <c r="E16" s="15" t="n">
-        <v>56.87976835790336</v>
+        <v>60</v>
       </c>
       <c r="F16" s="15" t="n">
         <v>0</v>
@@ -5456,7 +5456,7 @@
         </is>
       </c>
       <c r="E17" s="19" t="n">
-        <v>284.3988417895168</v>
+        <v>300</v>
       </c>
       <c r="F17" s="19" t="n">
         <v>0</v>
@@ -5502,7 +5502,7 @@
         </is>
       </c>
       <c r="E18" s="15" t="n">
-        <v>45.50381468632268</v>
+        <v>48</v>
       </c>
       <c r="F18" s="15" t="n">
         <v>36</v>
@@ -5548,7 +5548,7 @@
         </is>
       </c>
       <c r="E19" s="19" t="n">
-        <v>379.1984557193557</v>
+        <v>400</v>
       </c>
       <c r="F19" s="19" t="n">
         <v>700</v>
@@ -5594,7 +5594,7 @@
         </is>
       </c>
       <c r="E20" s="15" t="n">
-        <v>758.3969114387114</v>
+        <v>800</v>
       </c>
       <c r="F20" s="15" t="n">
         <v>100</v>
@@ -5640,7 +5640,7 @@
         </is>
       </c>
       <c r="E21" s="19" t="n">
-        <v>1213.435058301938</v>
+        <v>1280</v>
       </c>
       <c r="F21" s="19" t="n">
         <v>640</v>
@@ -5686,7 +5686,7 @@
         </is>
       </c>
       <c r="E22" s="15" t="n">
-        <v>94.79961392983893</v>
+        <v>100</v>
       </c>
       <c r="F22" s="15" t="n">
         <v>0</v>
@@ -5732,7 +5732,7 @@
         </is>
       </c>
       <c r="E23" s="19" t="n">
-        <v>3033.587645754846</v>
+        <v>3200</v>
       </c>
       <c r="F23" s="19" t="n">
         <v>0</v>
@@ -5778,7 +5778,7 @@
         </is>
       </c>
       <c r="E24" s="15" t="n">
-        <v>606.7175291509692</v>
+        <v>640</v>
       </c>
       <c r="F24" s="15" t="n">
         <v>0</v>
@@ -5824,7 +5824,7 @@
         </is>
       </c>
       <c r="E25" s="19" t="n">
-        <v>94.79961392983893</v>
+        <v>100</v>
       </c>
       <c r="F25" s="19" t="n">
         <v>100</v>
@@ -5870,7 +5870,7 @@
         </is>
       </c>
       <c r="E26" s="15" t="n">
-        <v>3033.587645754846</v>
+        <v>3200</v>
       </c>
       <c r="F26" s="15" t="n">
         <v>0</v>
@@ -5916,7 +5916,7 @@
         </is>
       </c>
       <c r="E27" s="19" t="n">
-        <v>379.1984557193557</v>
+        <v>400</v>
       </c>
       <c r="F27" s="19" t="n">
         <v>0</v>
@@ -5962,7 +5962,7 @@
         </is>
       </c>
       <c r="E28" s="15" t="n">
-        <v>1137.595367158067</v>
+        <v>1200</v>
       </c>
       <c r="F28" s="15" t="n">
         <v>0</v>
@@ -6008,7 +6008,7 @@
         </is>
       </c>
       <c r="E29" s="19" t="n">
-        <v>189.5992278596779</v>
+        <v>200</v>
       </c>
       <c r="F29" s="19" t="n">
         <v>0</v>
@@ -6054,7 +6054,7 @@
         </is>
       </c>
       <c r="E30" s="15" t="n">
-        <v>284.3988417895168</v>
+        <v>300</v>
       </c>
       <c r="F30" s="15" t="n">
         <v>0</v>
@@ -6100,7 +6100,7 @@
         </is>
       </c>
       <c r="E31" s="19" t="n">
-        <v>606.7175291509692</v>
+        <v>640</v>
       </c>
       <c r="F31" s="19" t="n">
         <v>0</v>
@@ -6146,7 +6146,7 @@
         </is>
       </c>
       <c r="E32" s="15" t="n">
-        <v>1213.435058301938</v>
+        <v>1280</v>
       </c>
       <c r="F32" s="15" t="n">
         <v>0</v>
@@ -6192,7 +6192,7 @@
         </is>
       </c>
       <c r="E33" s="19" t="n">
-        <v>94.79961392983893</v>
+        <v>100</v>
       </c>
       <c r="F33" s="19" t="n">
         <v>0</v>
@@ -6238,7 +6238,7 @@
         </is>
       </c>
       <c r="E34" s="15" t="n">
-        <v>1175.515212730003</v>
+        <v>1240</v>
       </c>
       <c r="F34" s="15" t="n">
         <v>0</v>
@@ -6330,7 +6330,7 @@
         </is>
       </c>
       <c r="E36" s="15" t="n">
-        <v>47.39980696491946</v>
+        <v>50</v>
       </c>
       <c r="F36" s="15" t="n">
         <v>50</v>
@@ -6376,7 +6376,7 @@
         </is>
       </c>
       <c r="E37" s="19" t="n">
-        <v>189.5992278596779</v>
+        <v>200</v>
       </c>
       <c r="F37" s="19" t="n">
         <v>200</v>
@@ -6422,7 +6422,7 @@
         </is>
       </c>
       <c r="E38" s="15" t="n">
-        <v>606.7175291509692</v>
+        <v>640</v>
       </c>
       <c r="F38" s="15" t="n">
         <v>640</v>
@@ -6468,7 +6468,7 @@
         </is>
       </c>
       <c r="E39" s="19" t="n">
-        <v>75.83969114387115</v>
+        <v>80</v>
       </c>
       <c r="F39" s="19" t="n">
         <v>80</v>
@@ -6514,7 +6514,7 @@
         </is>
       </c>
       <c r="E40" s="15" t="n">
-        <v>568.7976835790336</v>
+        <v>600</v>
       </c>
       <c r="F40" s="15" t="n">
         <v>600</v>
@@ -6560,7 +6560,7 @@
         </is>
       </c>
       <c r="E41" s="19" t="n">
-        <v>34.12786101474202</v>
+        <v>36</v>
       </c>
       <c r="F41" s="19" t="n">
         <v>0</v>
@@ -6606,7 +6606,7 @@
         </is>
       </c>
       <c r="E42" s="15" t="n">
-        <v>758.3969114387114</v>
+        <v>800</v>
       </c>
       <c r="F42" s="15" t="n">
         <v>800</v>
@@ -6755,17 +6755,17 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="2" ht="36" customHeight="1">
@@ -6778,7 +6778,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 22/09/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 23/09/2026</t>
         </is>
       </c>
     </row>
@@ -6817,7 +6817,7 @@
     <row r="6" ht="25" customHeight="1">
       <c r="B6" s="25" t="inlineStr">
         <is>
-          <t>16,211 u</t>
+          <t>17,100 u</t>
         </is>
       </c>
       <c r="C6" s="4" t="n"/>
@@ -6829,7 +6829,7 @@
       <c r="E6" s="4" t="n"/>
       <c r="F6" s="26" t="inlineStr">
         <is>
-          <t>157.8%</t>
+          <t>149.6%</t>
         </is>
       </c>
       <c r="G6" s="4" t="n"/>
@@ -6891,12 +6891,12 @@
       </c>
       <c r="I9" s="12" t="inlineStr">
         <is>
-          <t>Falta Conseguir (u)</t>
+          <t>Falta (u)</t>
         </is>
       </c>
       <c r="J9" s="12" t="inlineStr">
         <is>
-          <t>Desviación (u)</t>
+          <t>Desv. (u)</t>
         </is>
       </c>
       <c r="K9" s="12" t="inlineStr">
@@ -6927,7 +6927,7 @@
         </is>
       </c>
       <c r="E10" s="15" t="n">
-        <v>1516.793822877423</v>
+        <v>1600</v>
       </c>
       <c r="F10" s="15" t="n">
         <v>1600</v>
@@ -7019,7 +7019,7 @@
         </is>
       </c>
       <c r="E12" s="15" t="n">
-        <v>1042.795753228228</v>
+        <v>1100</v>
       </c>
       <c r="F12" s="15" t="n">
         <v>1100</v>
@@ -7479,7 +7479,7 @@
         </is>
       </c>
       <c r="E22" s="15" t="n">
-        <v>6256.77451936937</v>
+        <v>6600</v>
       </c>
       <c r="F22" s="15" t="n">
         <v>4400</v>
@@ -7663,7 +7663,7 @@
         </is>
       </c>
       <c r="E26" s="15" t="n">
-        <v>189.5992278596779</v>
+        <v>200</v>
       </c>
       <c r="F26" s="15" t="n">
         <v>200</v>
@@ -7709,7 +7709,7 @@
         </is>
       </c>
       <c r="E27" s="19" t="n">
-        <v>606.7175291509692</v>
+        <v>640</v>
       </c>
       <c r="F27" s="19" t="n">
         <v>640</v>
@@ -8261,7 +8261,7 @@
         </is>
       </c>
       <c r="E39" s="19" t="n">
-        <v>4171.183012912913</v>
+        <v>4400</v>
       </c>
       <c r="F39" s="19" t="n">
         <v>4400</v>
@@ -8307,7 +8307,7 @@
         </is>
       </c>
       <c r="E40" s="15" t="n">
-        <v>2426.870116603877</v>
+        <v>2560</v>
       </c>
       <c r="F40" s="15" t="n">
         <v>1280</v>
@@ -8452,21 +8452,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:L20"/>
+  <dimension ref="B2:L16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="2" ht="36" customHeight="1">
@@ -8479,7 +8479,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 22/09/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 23/09/2026</t>
         </is>
       </c>
     </row>
@@ -8518,7 +8518,7 @@
     <row r="6" ht="25" customHeight="1">
       <c r="B6" s="25" t="inlineStr">
         <is>
-          <t>37,408 u</t>
+          <t>39,460 u</t>
         </is>
       </c>
       <c r="C6" s="4" t="n"/>
@@ -8530,13 +8530,13 @@
       <c r="E6" s="4" t="n"/>
       <c r="F6" s="38" t="inlineStr">
         <is>
-          <t>87.8%</t>
+          <t>83.2%</t>
         </is>
       </c>
       <c r="G6" s="4" t="n"/>
       <c r="H6" s="38" t="inlineStr">
         <is>
-          <t>4,580 u</t>
+          <t>6,632 u</t>
         </is>
       </c>
       <c r="I6" s="4" t="n"/>
@@ -8592,12 +8592,12 @@
       </c>
       <c r="I9" s="12" t="inlineStr">
         <is>
-          <t>Falta Conseguir (u)</t>
+          <t>Falta (u)</t>
         </is>
       </c>
       <c r="J9" s="12" t="inlineStr">
         <is>
-          <t>Desviación (u)</t>
+          <t>Desv. (u)</t>
         </is>
       </c>
       <c r="K9" s="12" t="inlineStr">
@@ -8614,7 +8614,7 @@
     <row r="10">
       <c r="B10" s="28" t="inlineStr">
         <is>
-          <t>DOGA TARIM TIC.SAN.VE TUR. LTD. STI</t>
+          <t>ÇITAR ÇIÇEK TARIM TIC. LTD. STI</t>
         </is>
       </c>
       <c r="C10" s="29" t="inlineStr">
@@ -8628,16 +8628,16 @@
         </is>
       </c>
       <c r="E10" s="15" t="n">
-        <v>5213.978766141141</v>
+        <v>5500</v>
       </c>
       <c r="F10" s="15" t="n">
-        <v>0</v>
+        <v>3300</v>
       </c>
       <c r="G10" s="15" t="n">
         <v>0</v>
       </c>
       <c r="H10" s="15" t="n">
-        <v>0</v>
+        <v>3300</v>
       </c>
       <c r="I10" s="15">
         <f>MAX(0, E10-F10)</f>
@@ -8651,16 +8651,16 @@
         <f>IF(E10&gt;0, F10/E10, IF(F10&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L10" s="36" t="inlineStr">
-        <is>
-          <t>Sin Pedido</t>
+      <c r="L10" s="33" t="inlineStr">
+        <is>
+          <t>En Curso</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="B11" s="31" t="inlineStr">
         <is>
-          <t>DOGA TARIM TIC.SAN.VE TUR. LTD. STI</t>
+          <t>ÇITAR ÇIÇEK TARIM TIC. LTD. STI</t>
         </is>
       </c>
       <c r="C11" s="32" t="inlineStr">
@@ -8674,16 +8674,16 @@
         </is>
       </c>
       <c r="E11" s="19" t="n">
-        <v>9479.961392983892</v>
+        <v>10000</v>
       </c>
       <c r="F11" s="19" t="n">
-        <v>0</v>
+        <v>10060</v>
       </c>
       <c r="G11" s="19" t="n">
         <v>0</v>
       </c>
       <c r="H11" s="19" t="n">
-        <v>0</v>
+        <v>10060</v>
       </c>
       <c r="I11" s="19">
         <f>MAX(0, E11-F11)</f>
@@ -8697,16 +8697,16 @@
         <f>IF(E11&gt;0, F11/E11, IF(F11&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L11" s="36" t="inlineStr">
-        <is>
-          <t>Sin Pedido</t>
+      <c r="L11" s="30" t="inlineStr">
+        <is>
+          <t>Superado</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="B12" s="28" t="inlineStr">
         <is>
-          <t>DOGA TARIM TIC.SAN.VE TUR. LTD. STI</t>
+          <t>ÇITAR ÇIÇEK TARIM TIC. LTD. STI</t>
         </is>
       </c>
       <c r="C12" s="29" t="inlineStr">
@@ -8720,16 +8720,16 @@
         </is>
       </c>
       <c r="E12" s="15" t="n">
-        <v>9479.961392983892</v>
+        <v>10000</v>
       </c>
       <c r="F12" s="15" t="n">
-        <v>0</v>
+        <v>11000</v>
       </c>
       <c r="G12" s="15" t="n">
         <v>0</v>
       </c>
       <c r="H12" s="15" t="n">
-        <v>0</v>
+        <v>11000</v>
       </c>
       <c r="I12" s="15">
         <f>MAX(0, E12-F12)</f>
@@ -8743,16 +8743,16 @@
         <f>IF(E12&gt;0, F12/E12, IF(F12&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L12" s="36" t="inlineStr">
-        <is>
-          <t>Sin Pedido</t>
+      <c r="L12" s="30" t="inlineStr">
+        <is>
+          <t>Superado</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="B13" s="31" t="inlineStr">
         <is>
-          <t>DOGA TARIM TIC.SAN.VE TUR. LTD. STI</t>
+          <t>ÇITAR ÇIÇEK TARIM TIC. LTD. STI</t>
         </is>
       </c>
       <c r="C13" s="32" t="inlineStr">
@@ -8766,16 +8766,16 @@
         </is>
       </c>
       <c r="E13" s="19" t="n">
-        <v>1895.992278596779</v>
+        <v>2000</v>
       </c>
       <c r="F13" s="19" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="G13" s="19" t="n">
         <v>0</v>
       </c>
       <c r="H13" s="19" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="I13" s="19">
         <f>MAX(0, E13-F13)</f>
@@ -8789,9 +8789,9 @@
         <f>IF(E13&gt;0, F13/E13, IF(F13&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L13" s="36" t="inlineStr">
-        <is>
-          <t>Sin Pedido</t>
+      <c r="L13" s="33" t="inlineStr">
+        <is>
+          <t>En Curso</t>
         </is>
       </c>
     </row>
@@ -8803,25 +8803,25 @@
       </c>
       <c r="C14" s="29" t="inlineStr">
         <is>
-          <t>AN0005</t>
+          <t>FTK0005</t>
         </is>
       </c>
       <c r="D14" s="28" t="inlineStr">
         <is>
-          <t>ALCAPLANT NEW</t>
+          <t>FITOKONTROL CA FLOW, 5 KG</t>
         </is>
       </c>
       <c r="E14" s="15" t="n">
-        <v>0</v>
+        <v>10000</v>
       </c>
       <c r="F14" s="15" t="n">
-        <v>3300</v>
+        <v>5500</v>
       </c>
       <c r="G14" s="15" t="n">
         <v>0</v>
       </c>
       <c r="H14" s="15" t="n">
-        <v>3300</v>
+        <v>5500</v>
       </c>
       <c r="I14" s="15">
         <f>MAX(0, E14-F14)</f>
@@ -8835,9 +8835,9 @@
         <f>IF(E14&gt;0, F14/E14, IF(F14&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L14" s="30" t="inlineStr">
-        <is>
-          <t>Extra Budget</t>
+      <c r="L14" s="33" t="inlineStr">
+        <is>
+          <t>En Curso</t>
         </is>
       </c>
     </row>
@@ -8849,25 +8849,25 @@
       </c>
       <c r="C15" s="32" t="inlineStr">
         <is>
-          <t>BIO0020</t>
+          <t>RUN0001</t>
         </is>
       </c>
       <c r="D15" s="31" t="inlineStr">
         <is>
-          <t>BIORAD-20, 20 L</t>
+          <t>RUN STRESS, 1 L</t>
         </is>
       </c>
       <c r="E15" s="19" t="n">
-        <v>0</v>
+        <v>1960</v>
       </c>
       <c r="F15" s="19" t="n">
-        <v>10060</v>
+        <v>1968</v>
       </c>
       <c r="G15" s="19" t="n">
         <v>0</v>
       </c>
       <c r="H15" s="19" t="n">
-        <v>10060</v>
+        <v>1968</v>
       </c>
       <c r="I15" s="19">
         <f>MAX(0, E15-F15)</f>
@@ -8883,236 +8883,52 @@
       </c>
       <c r="L15" s="30" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="B16" s="28" t="inlineStr">
-        <is>
-          <t>ÇITAR ÇIÇEK TARIM TIC. LTD. STI</t>
-        </is>
-      </c>
-      <c r="C16" s="29" t="inlineStr">
-        <is>
-          <t>BIO1000</t>
-        </is>
-      </c>
-      <c r="D16" s="28" t="inlineStr">
-        <is>
-          <t>BIORAD-20, 1000 L</t>
-        </is>
-      </c>
-      <c r="E16" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="F16" s="15" t="n">
-        <v>11000</v>
-      </c>
-      <c r="G16" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H16" s="15" t="n">
-        <v>11000</v>
-      </c>
-      <c r="I16" s="15">
-        <f>MAX(0, E16-F16)</f>
-        <v/>
-      </c>
-      <c r="J16" s="15">
-        <f>F16-E16</f>
-        <v/>
-      </c>
-      <c r="K16" s="16">
-        <f>IF(E16&gt;0, F16/E16, IF(F16&gt;0, 1, 0))</f>
-        <v/>
-      </c>
-      <c r="L16" s="30" t="inlineStr">
-        <is>
-          <t>Extra Budget</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="B17" s="31" t="inlineStr">
-        <is>
-          <t>ÇITAR ÇIÇEK TARIM TIC. LTD. STI</t>
-        </is>
-      </c>
-      <c r="C17" s="32" t="inlineStr">
-        <is>
-          <t>C-CU1000</t>
-        </is>
-      </c>
-      <c r="D17" s="31" t="inlineStr">
-        <is>
-          <t>CODICOBRE, 1000 L</t>
-        </is>
-      </c>
-      <c r="E17" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="F17" s="19" t="n">
-        <v>1000</v>
-      </c>
-      <c r="G17" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="H17" s="19" t="n">
-        <v>1000</v>
-      </c>
-      <c r="I17" s="19">
-        <f>MAX(0, E17-F17)</f>
-        <v/>
-      </c>
-      <c r="J17" s="19">
-        <f>F17-E17</f>
-        <v/>
-      </c>
-      <c r="K17" s="20">
-        <f>IF(E17&gt;0, F17/E17, IF(F17&gt;0, 1, 0))</f>
-        <v/>
-      </c>
-      <c r="L17" s="30" t="inlineStr">
-        <is>
-          <t>Extra Budget</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="B18" s="28" t="inlineStr">
-        <is>
-          <t>ÇITAR ÇIÇEK TARIM TIC. LTD. STI</t>
-        </is>
-      </c>
-      <c r="C18" s="29" t="inlineStr">
-        <is>
-          <t>FTK0005</t>
-        </is>
-      </c>
-      <c r="D18" s="28" t="inlineStr">
-        <is>
-          <t>FITOKONTROL CA FLOW, 5 KG</t>
-        </is>
-      </c>
-      <c r="E18" s="15" t="n">
-        <v>9479.961392983892</v>
-      </c>
-      <c r="F18" s="15" t="n">
-        <v>5500</v>
-      </c>
-      <c r="G18" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H18" s="15" t="n">
-        <v>5500</v>
-      </c>
-      <c r="I18" s="15">
-        <f>MAX(0, E18-F18)</f>
-        <v/>
-      </c>
-      <c r="J18" s="15">
-        <f>F18-E18</f>
-        <v/>
-      </c>
-      <c r="K18" s="16">
-        <f>IF(E18&gt;0, F18/E18, IF(F18&gt;0, 1, 0))</f>
-        <v/>
-      </c>
-      <c r="L18" s="33" t="inlineStr">
-        <is>
-          <t>En Curso</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="B19" s="31" t="inlineStr">
-        <is>
-          <t>ÇITAR ÇIÇEK TARIM TIC. LTD. STI</t>
-        </is>
-      </c>
-      <c r="C19" s="32" t="inlineStr">
-        <is>
-          <t>RUN0001</t>
-        </is>
-      </c>
-      <c r="D19" s="31" t="inlineStr">
-        <is>
-          <t>RUN STRESS, 1 L</t>
-        </is>
-      </c>
-      <c r="E19" s="19" t="n">
-        <v>1858.072433024843</v>
-      </c>
-      <c r="F19" s="19" t="n">
-        <v>1968</v>
-      </c>
-      <c r="G19" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="H19" s="19" t="n">
-        <v>1968</v>
-      </c>
-      <c r="I19" s="19">
-        <f>MAX(0, E19-F19)</f>
-        <v/>
-      </c>
-      <c r="J19" s="19">
-        <f>F19-E19</f>
-        <v/>
-      </c>
-      <c r="K19" s="20">
-        <f>IF(E19&gt;0, F19/E19, IF(F19&gt;0, 1, 0))</f>
-        <v/>
-      </c>
-      <c r="L19" s="30" t="inlineStr">
-        <is>
           <t>Superado</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="24" customHeight="1">
-      <c r="B20" s="21" t="inlineStr">
+    <row r="16" ht="24" customHeight="1">
+      <c r="B16" s="21" t="inlineStr">
         <is>
           <t>TOTAL MEHMET</t>
         </is>
       </c>
-      <c r="C20" s="34" t="inlineStr">
-        <is>
-          <t>65 líneas</t>
-        </is>
-      </c>
-      <c r="D20" s="35" t="inlineStr"/>
-      <c r="E20" s="23">
-        <f>SUM(E10:E19)</f>
-        <v/>
-      </c>
-      <c r="F20" s="23">
-        <f>SUM(F10:F19)</f>
-        <v/>
-      </c>
-      <c r="G20" s="23">
-        <f>SUM(G10:G19)</f>
-        <v/>
-      </c>
-      <c r="H20" s="23">
-        <f>SUM(H10:H19)</f>
-        <v/>
-      </c>
-      <c r="I20" s="23">
-        <f>SUM(I10:I19)</f>
-        <v/>
-      </c>
-      <c r="J20" s="23">
-        <f>SUM(J10:J19)</f>
-        <v/>
-      </c>
-      <c r="K20" s="24">
-        <f>IF(E20&gt;0, F20/E20, 0)</f>
-        <v/>
-      </c>
-      <c r="L20" s="22">
-        <f>IF(K20&gt;=1, "SUPERADO", "EN CURSO")</f>
+      <c r="C16" s="34" t="inlineStr">
+        <is>
+          <t>61 líneas</t>
+        </is>
+      </c>
+      <c r="D16" s="35" t="inlineStr"/>
+      <c r="E16" s="23">
+        <f>SUM(E10:E15)</f>
+        <v/>
+      </c>
+      <c r="F16" s="23">
+        <f>SUM(F10:F15)</f>
+        <v/>
+      </c>
+      <c r="G16" s="23">
+        <f>SUM(G10:G15)</f>
+        <v/>
+      </c>
+      <c r="H16" s="23">
+        <f>SUM(H10:H15)</f>
+        <v/>
+      </c>
+      <c r="I16" s="23">
+        <f>SUM(I10:I15)</f>
+        <v/>
+      </c>
+      <c r="J16" s="23">
+        <f>SUM(J10:J15)</f>
+        <v/>
+      </c>
+      <c r="K16" s="24">
+        <f>IF(E16&gt;0, F16/E16, 0)</f>
+        <v/>
+      </c>
+      <c r="L16" s="22">
+        <f>IF(K16&gt;=1, "SUPERADO", "EN CURSO")</f>
         <v/>
       </c>
     </row>
@@ -9141,21 +8957,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:L26"/>
+  <dimension ref="B2:L29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="2" ht="36" customHeight="1">
@@ -9168,7 +8984,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 22/09/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 23/09/2026</t>
         </is>
       </c>
     </row>
@@ -9207,31 +9023,31 @@
     <row r="6" ht="25" customHeight="1">
       <c r="B6" s="25" t="inlineStr">
         <is>
-          <t>16,438 u</t>
+          <t>17,340 u</t>
         </is>
       </c>
       <c r="C6" s="4" t="n"/>
       <c r="D6" s="25" t="inlineStr">
         <is>
-          <t>5,860 u</t>
+          <t>7,660 u</t>
         </is>
       </c>
       <c r="E6" s="4" t="n"/>
       <c r="F6" s="38" t="inlineStr">
         <is>
-          <t>35.6%</t>
+          <t>44.2%</t>
         </is>
       </c>
       <c r="G6" s="4" t="n"/>
       <c r="H6" s="38" t="inlineStr">
         <is>
-          <t>10,578 u</t>
+          <t>9,680 u</t>
         </is>
       </c>
       <c r="I6" s="4" t="n"/>
       <c r="J6" s="25" t="inlineStr">
         <is>
-          <t>0 u</t>
+          <t>1,800 u</t>
         </is>
       </c>
       <c r="K6" s="4" t="n"/>
@@ -9281,12 +9097,12 @@
       </c>
       <c r="I9" s="12" t="inlineStr">
         <is>
-          <t>Falta Conseguir (u)</t>
+          <t>Falta (u)</t>
         </is>
       </c>
       <c r="J9" s="12" t="inlineStr">
         <is>
-          <t>Desviación (u)</t>
+          <t>Desv. (u)</t>
         </is>
       </c>
       <c r="K9" s="12" t="inlineStr">
@@ -9317,7 +9133,7 @@
         </is>
       </c>
       <c r="E10" s="15" t="n">
-        <v>606.7175291509692</v>
+        <v>640</v>
       </c>
       <c r="F10" s="15" t="n">
         <v>0</v>
@@ -9363,7 +9179,7 @@
         </is>
       </c>
       <c r="E11" s="19" t="n">
-        <v>284.3988417895168</v>
+        <v>300</v>
       </c>
       <c r="F11" s="19" t="n">
         <v>0</v>
@@ -9409,7 +9225,7 @@
         </is>
       </c>
       <c r="E12" s="15" t="n">
-        <v>1213.435058301938</v>
+        <v>1280</v>
       </c>
       <c r="F12" s="15" t="n">
         <v>0</v>
@@ -9455,7 +9271,7 @@
         </is>
       </c>
       <c r="E13" s="19" t="n">
-        <v>1213.435058301938</v>
+        <v>1280</v>
       </c>
       <c r="F13" s="19" t="n">
         <v>0</v>
@@ -9501,7 +9317,7 @@
         </is>
       </c>
       <c r="E14" s="15" t="n">
-        <v>2426.870116603877</v>
+        <v>2560</v>
       </c>
       <c r="F14" s="15" t="n">
         <v>1920</v>
@@ -9547,7 +9363,7 @@
         </is>
       </c>
       <c r="E15" s="19" t="n">
-        <v>379.1984557193557</v>
+        <v>400</v>
       </c>
       <c r="F15" s="19" t="n">
         <v>0</v>
@@ -9593,7 +9409,7 @@
         </is>
       </c>
       <c r="E16" s="15" t="n">
-        <v>1895.992278596779</v>
+        <v>2000</v>
       </c>
       <c r="F16" s="15" t="n">
         <v>0</v>
@@ -9639,7 +9455,7 @@
         </is>
       </c>
       <c r="E17" s="19" t="n">
-        <v>2085.591506456457</v>
+        <v>2200</v>
       </c>
       <c r="F17" s="19" t="n">
         <v>2200</v>
@@ -9722,25 +9538,25 @@
       </c>
       <c r="C19" s="32" t="inlineStr">
         <is>
-          <t>S0020</t>
+          <t>N0200</t>
         </is>
       </c>
       <c r="D19" s="31" t="inlineStr">
         <is>
-          <t>SAL-WAX STAR, 20 L</t>
+          <t>NUTRICALE, 200 L</t>
         </is>
       </c>
       <c r="E19" s="19" t="n">
-        <v>606.7175291509692</v>
+        <v>0</v>
       </c>
       <c r="F19" s="19" t="n">
-        <v>640</v>
+        <v>200</v>
       </c>
       <c r="G19" s="19" t="n">
-        <v>640</v>
+        <v>0</v>
       </c>
       <c r="H19" s="19" t="n">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="I19" s="19">
         <f>MAX(0, E19-F19)</f>
@@ -9756,7 +9572,7 @@
       </c>
       <c r="L19" s="30" t="inlineStr">
         <is>
-          <t>Superado</t>
+          <t>Extra Budget</t>
         </is>
       </c>
     </row>
@@ -9768,25 +9584,25 @@
       </c>
       <c r="C20" s="29" t="inlineStr">
         <is>
-          <t>S0200</t>
+          <t>PT0200</t>
         </is>
       </c>
       <c r="D20" s="28" t="inlineStr">
         <is>
-          <t>SAL-WAX STAR, 200 L</t>
+          <t>AGROPOTASION, 200 L</t>
         </is>
       </c>
       <c r="E20" s="15" t="n">
-        <v>379.1984557193557</v>
+        <v>0</v>
       </c>
       <c r="F20" s="15" t="n">
-        <v>0</v>
+        <v>600</v>
       </c>
       <c r="G20" s="15" t="n">
         <v>0</v>
       </c>
       <c r="H20" s="15" t="n">
-        <v>0</v>
+        <v>600</v>
       </c>
       <c r="I20" s="15">
         <f>MAX(0, E20-F20)</f>
@@ -9800,9 +9616,9 @@
         <f>IF(E20&gt;0, F20/E20, IF(F20&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L20" s="36" t="inlineStr">
-        <is>
-          <t>Sin Pedido</t>
+      <c r="L20" s="30" t="inlineStr">
+        <is>
+          <t>Extra Budget</t>
         </is>
       </c>
     </row>
@@ -9814,25 +9630,25 @@
       </c>
       <c r="C21" s="32" t="inlineStr">
         <is>
-          <t>S1000</t>
+          <t>PT1000</t>
         </is>
       </c>
       <c r="D21" s="31" t="inlineStr">
         <is>
-          <t>SAL-WAX STAR, 1000 L</t>
+          <t>AGROPOTASION, 1000 L</t>
         </is>
       </c>
       <c r="E21" s="19" t="n">
-        <v>4739.980696491946</v>
+        <v>0</v>
       </c>
       <c r="F21" s="19" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="G21" s="19" t="n">
         <v>0</v>
       </c>
       <c r="H21" s="19" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="I21" s="19">
         <f>MAX(0, E21-F21)</f>
@@ -9846,9 +9662,9 @@
         <f>IF(E21&gt;0, F21/E21, IF(F21&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L21" s="36" t="inlineStr">
-        <is>
-          <t>Sin Pedido</t>
+      <c r="L21" s="30" t="inlineStr">
+        <is>
+          <t>Extra Budget</t>
         </is>
       </c>
     </row>
@@ -9860,22 +9676,22 @@
       </c>
       <c r="C22" s="29" t="inlineStr">
         <is>
-          <t>SPCE2B0020</t>
+          <t>S0020</t>
         </is>
       </c>
       <c r="D22" s="28" t="inlineStr">
         <is>
-          <t>SPRINTENE CON BORO, 20 L</t>
+          <t>SAL-WAX STAR, 20 L</t>
         </is>
       </c>
       <c r="E22" s="15" t="n">
-        <v>606.7175291509692</v>
+        <v>640</v>
       </c>
       <c r="F22" s="15" t="n">
-        <v>0</v>
+        <v>640</v>
       </c>
       <c r="G22" s="15" t="n">
-        <v>0</v>
+        <v>640</v>
       </c>
       <c r="H22" s="15" t="n">
         <v>0</v>
@@ -9892,9 +9708,9 @@
         <f>IF(E22&gt;0, F22/E22, IF(F22&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L22" s="36" t="inlineStr">
-        <is>
-          <t>Sin Pedido</t>
+      <c r="L22" s="30" t="inlineStr">
+        <is>
+          <t>Superado</t>
         </is>
       </c>
     </row>
@@ -9906,22 +9722,22 @@
       </c>
       <c r="C23" s="32" t="inlineStr">
         <is>
-          <t>SS0020</t>
+          <t>S0200</t>
         </is>
       </c>
       <c r="D23" s="31" t="inlineStr">
         <is>
-          <t>SAL-WAX-Ca sólido, 20 KG</t>
+          <t>SAL-WAX STAR, 200 L</t>
         </is>
       </c>
       <c r="E23" s="19" t="n">
-        <v>0</v>
+        <v>400</v>
       </c>
       <c r="F23" s="19" t="n">
-        <v>400</v>
+        <v>0</v>
       </c>
       <c r="G23" s="19" t="n">
-        <v>400</v>
+        <v>0</v>
       </c>
       <c r="H23" s="19" t="n">
         <v>0</v>
@@ -9938,36 +9754,36 @@
         <f>IF(E23&gt;0, F23/E23, IF(F23&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L23" s="30" t="inlineStr">
-        <is>
-          <t>Extra Budget</t>
+      <c r="L23" s="36" t="inlineStr">
+        <is>
+          <t>Sin Pedido</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="B24" s="28" t="inlineStr">
         <is>
-          <t>FITOMURCIA S.L.</t>
+          <t>COMERCIAL TÉCNICA FITOCARTHAGO, S.L.</t>
         </is>
       </c>
       <c r="C24" s="29" t="inlineStr">
         <is>
-          <t>SPCE2B0020</t>
+          <t>S1000</t>
         </is>
       </c>
       <c r="D24" s="28" t="inlineStr">
         <is>
-          <t>SPRINTENE CON BORO, 20 L</t>
+          <t>SAL-WAX STAR, 1000 L</t>
         </is>
       </c>
       <c r="E24" s="15" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="F24" s="15" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="G24" s="15" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="H24" s="15" t="n">
         <v>0</v>
@@ -9984,36 +9800,36 @@
         <f>IF(E24&gt;0, F24/E24, IF(F24&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L24" s="30" t="inlineStr">
-        <is>
-          <t>Extra Budget</t>
+      <c r="L24" s="36" t="inlineStr">
+        <is>
+          <t>Sin Pedido</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="B25" s="31" t="inlineStr">
         <is>
-          <t>FITOMURCIA S.L.</t>
+          <t>COMERCIAL TÉCNICA FITOCARTHAGO, S.L.</t>
         </is>
       </c>
       <c r="C25" s="32" t="inlineStr">
         <is>
-          <t>SS0005</t>
+          <t>SPCE2B0020</t>
         </is>
       </c>
       <c r="D25" s="31" t="inlineStr">
         <is>
-          <t>SAL-WAX-Ca sólido, 5 KG</t>
+          <t>SPRINTENE CON BORO, 20 L</t>
         </is>
       </c>
       <c r="E25" s="19" t="n">
-        <v>0</v>
+        <v>640</v>
       </c>
       <c r="F25" s="19" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="G25" s="19" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="H25" s="19" t="n">
         <v>0</v>
@@ -10030,54 +9846,192 @@
         <f>IF(E25&gt;0, F25/E25, IF(F25&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L25" s="30" t="inlineStr">
+      <c r="L25" s="36" t="inlineStr">
+        <is>
+          <t>Sin Pedido</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="28" t="inlineStr">
+        <is>
+          <t>COMERCIAL TÉCNICA FITOCARTHAGO, S.L.</t>
+        </is>
+      </c>
+      <c r="C26" s="29" t="inlineStr">
+        <is>
+          <t>SS0020</t>
+        </is>
+      </c>
+      <c r="D26" s="28" t="inlineStr">
+        <is>
+          <t>SAL-WAX-Ca sólido, 20 KG</t>
+        </is>
+      </c>
+      <c r="E26" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" s="15" t="n">
+        <v>400</v>
+      </c>
+      <c r="G26" s="15" t="n">
+        <v>400</v>
+      </c>
+      <c r="H26" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I26" s="15">
+        <f>MAX(0, E26-F26)</f>
+        <v/>
+      </c>
+      <c r="J26" s="15">
+        <f>F26-E26</f>
+        <v/>
+      </c>
+      <c r="K26" s="16">
+        <f>IF(E26&gt;0, F26/E26, IF(F26&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L26" s="30" t="inlineStr">
         <is>
           <t>Extra Budget</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="24" customHeight="1">
-      <c r="B26" s="21" t="inlineStr">
+    <row r="27">
+      <c r="B27" s="31" t="inlineStr">
+        <is>
+          <t>FITOMURCIA S.L.</t>
+        </is>
+      </c>
+      <c r="C27" s="32" t="inlineStr">
+        <is>
+          <t>SPCE2B0020</t>
+        </is>
+      </c>
+      <c r="D27" s="31" t="inlineStr">
+        <is>
+          <t>SPRINTENE CON BORO, 20 L</t>
+        </is>
+      </c>
+      <c r="E27" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" s="19" t="n">
+        <v>200</v>
+      </c>
+      <c r="G27" s="19" t="n">
+        <v>200</v>
+      </c>
+      <c r="H27" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I27" s="19">
+        <f>MAX(0, E27-F27)</f>
+        <v/>
+      </c>
+      <c r="J27" s="19">
+        <f>F27-E27</f>
+        <v/>
+      </c>
+      <c r="K27" s="20">
+        <f>IF(E27&gt;0, F27/E27, IF(F27&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L27" s="30" t="inlineStr">
+        <is>
+          <t>Extra Budget</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="28" t="inlineStr">
+        <is>
+          <t>FITOMURCIA S.L.</t>
+        </is>
+      </c>
+      <c r="C28" s="29" t="inlineStr">
+        <is>
+          <t>SS0005</t>
+        </is>
+      </c>
+      <c r="D28" s="28" t="inlineStr">
+        <is>
+          <t>SAL-WAX-Ca sólido, 5 KG</t>
+        </is>
+      </c>
+      <c r="E28" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" s="15" t="n">
+        <v>300</v>
+      </c>
+      <c r="G28" s="15" t="n">
+        <v>300</v>
+      </c>
+      <c r="H28" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I28" s="15">
+        <f>MAX(0, E28-F28)</f>
+        <v/>
+      </c>
+      <c r="J28" s="15">
+        <f>F28-E28</f>
+        <v/>
+      </c>
+      <c r="K28" s="16">
+        <f>IF(E28&gt;0, F28/E28, IF(F28&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L28" s="30" t="inlineStr">
+        <is>
+          <t>Extra Budget</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="24" customHeight="1">
+      <c r="B29" s="21" t="inlineStr">
         <is>
           <t>TOTAL PEDRO</t>
         </is>
       </c>
-      <c r="C26" s="34" t="inlineStr">
-        <is>
-          <t>103 líneas</t>
-        </is>
-      </c>
-      <c r="D26" s="35" t="inlineStr"/>
-      <c r="E26" s="23">
-        <f>SUM(E10:E25)</f>
-        <v/>
-      </c>
-      <c r="F26" s="23">
-        <f>SUM(F10:F25)</f>
-        <v/>
-      </c>
-      <c r="G26" s="23">
-        <f>SUM(G10:G25)</f>
-        <v/>
-      </c>
-      <c r="H26" s="23">
-        <f>SUM(H10:H25)</f>
-        <v/>
-      </c>
-      <c r="I26" s="23">
-        <f>SUM(I10:I25)</f>
-        <v/>
-      </c>
-      <c r="J26" s="23">
-        <f>SUM(J10:J25)</f>
-        <v/>
-      </c>
-      <c r="K26" s="24">
-        <f>IF(E26&gt;0, F26/E26, 0)</f>
-        <v/>
-      </c>
-      <c r="L26" s="22">
-        <f>IF(K26&gt;=1, "SUPERADO", "EN CURSO")</f>
+      <c r="C29" s="34" t="inlineStr">
+        <is>
+          <t>105 líneas</t>
+        </is>
+      </c>
+      <c r="D29" s="35" t="inlineStr"/>
+      <c r="E29" s="23">
+        <f>SUM(E10:E28)</f>
+        <v/>
+      </c>
+      <c r="F29" s="23">
+        <f>SUM(F10:F28)</f>
+        <v/>
+      </c>
+      <c r="G29" s="23">
+        <f>SUM(G10:G28)</f>
+        <v/>
+      </c>
+      <c r="H29" s="23">
+        <f>SUM(H10:H28)</f>
+        <v/>
+      </c>
+      <c r="I29" s="23">
+        <f>SUM(I10:I28)</f>
+        <v/>
+      </c>
+      <c r="J29" s="23">
+        <f>SUM(J10:J28)</f>
+        <v/>
+      </c>
+      <c r="K29" s="24">
+        <f>IF(E29&gt;0, F29/E29, 0)</f>
+        <v/>
+      </c>
+      <c r="L29" s="22">
+        <f>IF(K29&gt;=1, "SUPERADO", "EN CURSO")</f>
         <v/>
       </c>
     </row>
@@ -10110,17 +10064,17 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="2" ht="36" customHeight="1">
@@ -10133,7 +10087,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 22/09/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 23/09/2026</t>
         </is>
       </c>
     </row>
@@ -10172,7 +10126,7 @@
     <row r="6" ht="25" customHeight="1">
       <c r="B6" s="25" t="inlineStr">
         <is>
-          <t>43,608 u</t>
+          <t>46,000 u</t>
         </is>
       </c>
       <c r="C6" s="4" t="n"/>
@@ -10184,13 +10138,13 @@
       <c r="E6" s="4" t="n"/>
       <c r="F6" s="38" t="inlineStr">
         <is>
-          <t>73.0%</t>
+          <t>69.2%</t>
         </is>
       </c>
       <c r="G6" s="4" t="n"/>
       <c r="H6" s="38" t="inlineStr">
         <is>
-          <t>11,758 u</t>
+          <t>14,150 u</t>
         </is>
       </c>
       <c r="I6" s="4" t="n"/>
@@ -10246,12 +10200,12 @@
       </c>
       <c r="I9" s="12" t="inlineStr">
         <is>
-          <t>Falta Conseguir (u)</t>
+          <t>Falta (u)</t>
         </is>
       </c>
       <c r="J9" s="12" t="inlineStr">
         <is>
-          <t>Desviación (u)</t>
+          <t>Desv. (u)</t>
         </is>
       </c>
       <c r="K9" s="12" t="inlineStr">
@@ -10420,7 +10374,7 @@
         </is>
       </c>
       <c r="E13" s="19" t="n">
-        <v>1895.992278596779</v>
+        <v>2000</v>
       </c>
       <c r="F13" s="19" t="n">
         <v>0</v>
@@ -10926,7 +10880,7 @@
         </is>
       </c>
       <c r="E24" s="15" t="n">
-        <v>41711.83012912912</v>
+        <v>44000</v>
       </c>
       <c r="F24" s="15" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Fix carga dashboard web y sincronizar fecha corte 28/09/2026
</commit_message>
<xml_diff>
--- a/Seguimiento_Presupuesto_Sep_2026.xlsx
+++ b/Seguimiento_Presupuesto_Sep_2026.xlsx
@@ -437,7 +437,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Budget Septiembre vs Pedidos Reales por Comercial (Unidades)</a:t>
+              <a:t>Estimación Septiembre vs Pedidos Reales por Comercial (Unidades)</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -902,14 +902,14 @@
     <row r="3" ht="20" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Comparativa Budget Septiembre (Unidades) vs Pedidos Reales a Fecha 25/09/2026 | Generado: 25/09/2026 07:40</t>
+          <t>Comparativa Estimación Septiembre (Unidades) vs Pedidos Reales a Fecha 28/09/2026 | Generado: 29/09/2026 07:26</t>
         </is>
       </c>
     </row>
     <row r="5" ht="18" customHeight="1">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>BUDGET SEP (UDS)</t>
+          <t>ESTIMACIÓN SEP (UDS)</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
@@ -946,13 +946,13 @@
       <c r="C6" s="4" t="n"/>
       <c r="D6" s="8" t="inlineStr">
         <is>
-          <t>186,385 u</t>
+          <t>203,399 u</t>
         </is>
       </c>
       <c r="E6" s="4" t="n"/>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>102.4%</t>
+          <t>111.8%</t>
         </is>
       </c>
       <c r="G6" s="4" t="n"/>
@@ -964,7 +964,7 @@
       <c r="I6" s="4" t="n"/>
       <c r="J6" s="7" t="inlineStr">
         <is>
-          <t>103,628 u</t>
+          <t>104,818 u</t>
         </is>
       </c>
     </row>
@@ -988,7 +988,7 @@
       </c>
       <c r="D9" s="11" t="inlineStr">
         <is>
-          <t>Budget Sep (u)</t>
+          <t>Estimación Sep (u)</t>
         </is>
       </c>
       <c r="E9" s="11" t="inlineStr">
@@ -1035,10 +1035,10 @@
         <v>2320</v>
       </c>
       <c r="E10" s="14" t="n">
-        <v>10110</v>
+        <v>11410</v>
       </c>
       <c r="F10" s="14" t="n">
-        <v>10110</v>
+        <v>11410</v>
       </c>
       <c r="G10" s="14" t="n">
         <v>0</v>
@@ -1063,19 +1063,19 @@
         </is>
       </c>
       <c r="C11" s="17" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D11" s="18" t="n">
         <v>37832</v>
       </c>
       <c r="E11" s="18" t="n">
-        <v>52772</v>
+        <v>55612</v>
       </c>
       <c r="F11" s="18" t="n">
-        <v>3556</v>
+        <v>5296</v>
       </c>
       <c r="G11" s="18" t="n">
-        <v>49216</v>
+        <v>50316</v>
       </c>
       <c r="H11" s="18">
         <f>MAX(0, D11-E11)</f>
@@ -1140,10 +1140,10 @@
         <v>38359</v>
       </c>
       <c r="F13" s="18" t="n">
-        <v>25575</v>
+        <v>38359</v>
       </c>
       <c r="G13" s="18" t="n">
-        <v>12784</v>
+        <v>0</v>
       </c>
       <c r="H13" s="18">
         <f>MAX(0, D13-E13)</f>
@@ -1323,7 +1323,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:L34"/>
+  <dimension ref="B2:L36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1350,14 +1350,14 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 25/09/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 28/09/2026</t>
         </is>
       </c>
     </row>
     <row r="5" ht="16" customHeight="1">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>BUDGET SEP (U)</t>
+          <t>ESTIMACIÓN SEP (U)</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
@@ -1395,13 +1395,13 @@
       <c r="C6" s="4" t="n"/>
       <c r="D6" s="25" t="inlineStr">
         <is>
-          <t>10,110 u</t>
+          <t>11,410 u</t>
         </is>
       </c>
       <c r="E6" s="4" t="n"/>
       <c r="F6" s="25" t="inlineStr">
         <is>
-          <t>435.8%</t>
+          <t>491.8%</t>
         </is>
       </c>
       <c r="G6" s="4" t="n"/>
@@ -1443,7 +1443,7 @@
       </c>
       <c r="E9" s="11" t="inlineStr">
         <is>
-          <t>Budget Sep (u)</t>
+          <t>Estimación Sep (u)</t>
         </is>
       </c>
       <c r="F9" s="11" t="inlineStr">
@@ -1594,10 +1594,10 @@
         <v>0</v>
       </c>
       <c r="F12" s="14" t="n">
-        <v>300</v>
+        <v>500</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>300</v>
+        <v>500</v>
       </c>
       <c r="H12" s="14" t="n">
         <v>0</v>
@@ -1616,7 +1616,7 @@
       </c>
       <c r="L12" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -1662,24 +1662,24 @@
       </c>
       <c r="L13" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="B14" s="27" t="inlineStr">
         <is>
-          <t>AGROVEYCA,S.L</t>
+          <t>AGROTÉCNICA DEL NORTE, S.L</t>
         </is>
       </c>
       <c r="C14" s="28" t="inlineStr">
         <is>
-          <t>A-50(2)0005</t>
+          <t>PT0005</t>
         </is>
       </c>
       <c r="D14" s="27" t="inlineStr">
         <is>
-          <t>CODIORGAN-A50, 5 KG</t>
+          <t>AGROPOTASION, 5 L</t>
         </is>
       </c>
       <c r="E14" s="14" t="n">
@@ -1708,7 +1708,7 @@
       </c>
       <c r="L14" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -1720,22 +1720,22 @@
       </c>
       <c r="C15" s="31" t="inlineStr">
         <is>
-          <t>BIO0020</t>
+          <t>A-50(2)0005</t>
         </is>
       </c>
       <c r="D15" s="30" t="inlineStr">
         <is>
-          <t>BIORAD-20, 20 L</t>
+          <t>CODIORGAN-A50, 5 KG</t>
         </is>
       </c>
       <c r="E15" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="18" t="n">
         <v>400</v>
       </c>
-      <c r="F15" s="18" t="n">
-        <v>320</v>
-      </c>
       <c r="G15" s="18" t="n">
-        <v>320</v>
+        <v>400</v>
       </c>
       <c r="H15" s="18" t="n">
         <v>0</v>
@@ -1752,36 +1752,36 @@
         <f>IF(E15&gt;0, F15/E15, IF(F15&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L15" s="32" t="inlineStr">
-        <is>
-          <t>En Curso</t>
+      <c r="L15" s="29" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="27" t="inlineStr">
         <is>
-          <t>ASOC. HORTICULTORES DE VILLA DEL PRADO</t>
+          <t>AGROVEYCA,S.L</t>
         </is>
       </c>
       <c r="C16" s="28" t="inlineStr">
         <is>
-          <t>A-50(2)0005</t>
+          <t>BIO0020</t>
         </is>
       </c>
       <c r="D16" s="27" t="inlineStr">
         <is>
-          <t>CODIORGAN A-50, 5 KG</t>
+          <t>BIORAD-20, 20 L</t>
         </is>
       </c>
       <c r="E16" s="14" t="n">
-        <v>0</v>
+        <v>400</v>
       </c>
       <c r="F16" s="14" t="n">
-        <v>50</v>
+        <v>320</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>50</v>
+        <v>320</v>
       </c>
       <c r="H16" s="14" t="n">
         <v>0</v>
@@ -1798,9 +1798,9 @@
         <f>IF(E16&gt;0, F16/E16, IF(F16&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L16" s="29" t="inlineStr">
-        <is>
-          <t>Extra Budget</t>
+      <c r="L16" s="32" t="inlineStr">
+        <is>
+          <t>En Curso</t>
         </is>
       </c>
     </row>
@@ -1812,22 +1812,22 @@
       </c>
       <c r="C17" s="31" t="inlineStr">
         <is>
-          <t>AVAN0005</t>
+          <t>A-50(2)0005</t>
         </is>
       </c>
       <c r="D17" s="30" t="inlineStr">
         <is>
-          <t>FLORAMEC AVANCE, 5 L</t>
+          <t>CODIORGAN A-50, 5 KG</t>
         </is>
       </c>
       <c r="E17" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F17" s="18" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="G17" s="18" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="H17" s="18" t="n">
         <v>0</v>
@@ -1846,7 +1846,7 @@
       </c>
       <c r="L17" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -1858,22 +1858,22 @@
       </c>
       <c r="C18" s="28" t="inlineStr">
         <is>
-          <t>C-CU0005</t>
+          <t>AVAN0005</t>
         </is>
       </c>
       <c r="D18" s="27" t="inlineStr">
         <is>
-          <t>CODICOBRE, 5 L</t>
+          <t>FLORAMEC AVANCE, 5 L</t>
         </is>
       </c>
       <c r="E18" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F18" s="14" t="n">
-        <v>20</v>
+        <v>100</v>
       </c>
       <c r="G18" s="14" t="n">
-        <v>20</v>
+        <v>100</v>
       </c>
       <c r="H18" s="14" t="n">
         <v>0</v>
@@ -1892,7 +1892,7 @@
       </c>
       <c r="L18" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -1904,22 +1904,22 @@
       </c>
       <c r="C19" s="31" t="inlineStr">
         <is>
-          <t>S0020</t>
+          <t>C-CU0005</t>
         </is>
       </c>
       <c r="D19" s="30" t="inlineStr">
         <is>
-          <t>SALWAX STAR, 20 L</t>
+          <t>CODICOBRE, 5 L</t>
         </is>
       </c>
       <c r="E19" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F19" s="18" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="G19" s="18" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="H19" s="18" t="n">
         <v>0</v>
@@ -1938,34 +1938,34 @@
       </c>
       <c r="L19" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="B20" s="27" t="inlineStr">
         <is>
-          <t>BARDENAS COMERCIAL, S.L.</t>
+          <t>ASOC. HORTICULTORES DE VILLA DEL PRADO</t>
         </is>
       </c>
       <c r="C20" s="28" t="inlineStr">
         <is>
-          <t>AGRMG0005</t>
+          <t>S0020</t>
         </is>
       </c>
       <c r="D20" s="27" t="inlineStr">
         <is>
-          <t>AGROXIGREEN-MG, 5 L</t>
+          <t>SALWAX STAR, 20 L</t>
         </is>
       </c>
       <c r="E20" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F20" s="14" t="n">
-        <v>300</v>
+        <v>40</v>
       </c>
       <c r="G20" s="14" t="n">
-        <v>300</v>
+        <v>40</v>
       </c>
       <c r="H20" s="14" t="n">
         <v>0</v>
@@ -1984,7 +1984,7 @@
       </c>
       <c r="L20" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -1996,12 +1996,12 @@
       </c>
       <c r="C21" s="31" t="inlineStr">
         <is>
-          <t>PT0005</t>
+          <t>AGRMG0005</t>
         </is>
       </c>
       <c r="D21" s="30" t="inlineStr">
         <is>
-          <t>AGROPOTASION, 5 L</t>
+          <t>AGROXIGREEN-MG, 5 L</t>
         </is>
       </c>
       <c r="E21" s="18" t="n">
@@ -2030,34 +2030,34 @@
       </c>
       <c r="L21" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="B22" s="27" t="inlineStr">
         <is>
-          <t>COMERCIAL NORTE AGROCAMPO, S.L.</t>
+          <t>BARDENAS COMERCIAL, S.L.</t>
         </is>
       </c>
       <c r="C22" s="28" t="inlineStr">
         <is>
-          <t>A-50(2)0020</t>
+          <t>PT0005</t>
         </is>
       </c>
       <c r="D22" s="27" t="inlineStr">
         <is>
-          <t>CODIORGAN-A50, 20 KG</t>
+          <t>AGROPOTASION, 5 L</t>
         </is>
       </c>
       <c r="E22" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F22" s="14" t="n">
-        <v>40</v>
+        <v>300</v>
       </c>
       <c r="G22" s="14" t="n">
-        <v>40</v>
+        <v>300</v>
       </c>
       <c r="H22" s="14" t="n">
         <v>0</v>
@@ -2076,7 +2076,7 @@
       </c>
       <c r="L22" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -2088,22 +2088,22 @@
       </c>
       <c r="C23" s="31" t="inlineStr">
         <is>
-          <t>AN0005</t>
+          <t>A-50(2)0020</t>
         </is>
       </c>
       <c r="D23" s="30" t="inlineStr">
         <is>
-          <t>ALCAPLANT NEW, 5 KG</t>
+          <t>CODIORGAN-A50, 20 KG</t>
         </is>
       </c>
       <c r="E23" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F23" s="18" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="G23" s="18" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="H23" s="18" t="n">
         <v>0</v>
@@ -2122,7 +2122,7 @@
       </c>
       <c r="L23" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -2134,22 +2134,22 @@
       </c>
       <c r="C24" s="28" t="inlineStr">
         <is>
-          <t>BR-590005</t>
+          <t>AN0005</t>
         </is>
       </c>
       <c r="D24" s="27" t="inlineStr">
         <is>
-          <t>BR-59, 5 KG</t>
+          <t>ALCAPLANT NEW, 5 KG</t>
         </is>
       </c>
       <c r="E24" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F24" s="14" t="n">
-        <v>60</v>
+        <v>20</v>
       </c>
       <c r="G24" s="14" t="n">
-        <v>60</v>
+        <v>20</v>
       </c>
       <c r="H24" s="14" t="n">
         <v>0</v>
@@ -2168,7 +2168,7 @@
       </c>
       <c r="L24" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -2180,22 +2180,22 @@
       </c>
       <c r="C25" s="31" t="inlineStr">
         <is>
-          <t>BROTA0020</t>
+          <t>BR-590005</t>
         </is>
       </c>
       <c r="D25" s="30" t="inlineStr">
         <is>
-          <t>BROTAMEC, 20 L</t>
+          <t>BR-59, 5 KG</t>
         </is>
       </c>
       <c r="E25" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F25" s="18" t="n">
-        <v>20</v>
+        <v>60</v>
       </c>
       <c r="G25" s="18" t="n">
-        <v>20</v>
+        <v>60</v>
       </c>
       <c r="H25" s="18" t="n">
         <v>0</v>
@@ -2214,7 +2214,7 @@
       </c>
       <c r="L25" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -2226,12 +2226,12 @@
       </c>
       <c r="C26" s="28" t="inlineStr">
         <is>
-          <t>C-CU0005</t>
+          <t>BROTA0020</t>
         </is>
       </c>
       <c r="D26" s="27" t="inlineStr">
         <is>
-          <t>CODICOBRE, 5 L</t>
+          <t>BROTAMEC, 20 L</t>
         </is>
       </c>
       <c r="E26" s="14" t="n">
@@ -2260,7 +2260,7 @@
       </c>
       <c r="L26" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -2272,12 +2272,12 @@
       </c>
       <c r="C27" s="31" t="inlineStr">
         <is>
-          <t>PT0020</t>
+          <t>C-CU0005</t>
         </is>
       </c>
       <c r="D27" s="30" t="inlineStr">
         <is>
-          <t>AGROPOTASION, 20 L</t>
+          <t>CODICOBRE, 5 L</t>
         </is>
       </c>
       <c r="E27" s="18" t="n">
@@ -2306,7 +2306,7 @@
       </c>
       <c r="L27" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -2318,22 +2318,22 @@
       </c>
       <c r="C28" s="28" t="inlineStr">
         <is>
-          <t>S0020</t>
+          <t>PT0020</t>
         </is>
       </c>
       <c r="D28" s="27" t="inlineStr">
         <is>
-          <t>SALWAX STAR, 20 L</t>
+          <t>AGROPOTASION, 20 L</t>
         </is>
       </c>
       <c r="E28" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F28" s="14" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="G28" s="14" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="H28" s="14" t="n">
         <v>0</v>
@@ -2352,34 +2352,34 @@
       </c>
       <c r="L28" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="B29" s="30" t="inlineStr">
         <is>
-          <t>MAJ AGROQUIMICOS S.L.</t>
+          <t>COMERCIAL NORTE AGROCAMPO, S.L.</t>
         </is>
       </c>
       <c r="C29" s="31" t="inlineStr">
         <is>
-          <t>CPLUS0005</t>
+          <t>S0020</t>
         </is>
       </c>
       <c r="D29" s="30" t="inlineStr">
         <is>
-          <t>CALCIPLUS, 5 L</t>
+          <t>SALWAX STAR, 20 L</t>
         </is>
       </c>
       <c r="E29" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F29" s="18" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="G29" s="18" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="H29" s="18" t="n">
         <v>0</v>
@@ -2398,34 +2398,34 @@
       </c>
       <c r="L29" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="B30" s="27" t="inlineStr">
         <is>
-          <t>SAFIAGRO, S.A.</t>
+          <t>MAJ AGROQUIMICOS S.L.</t>
         </is>
       </c>
       <c r="C30" s="28" t="inlineStr">
         <is>
-          <t>AGXK0020</t>
+          <t>CPLUS0005</t>
         </is>
       </c>
       <c r="D30" s="27" t="inlineStr">
         <is>
-          <t>AGROXILATO-K, 20 L</t>
+          <t>CALCIPLUS, 5 L</t>
         </is>
       </c>
       <c r="E30" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F30" s="14" t="n">
-        <v>640</v>
+        <v>20</v>
       </c>
       <c r="G30" s="14" t="n">
-        <v>640</v>
+        <v>20</v>
       </c>
       <c r="H30" s="14" t="n">
         <v>0</v>
@@ -2444,34 +2444,34 @@
       </c>
       <c r="L30" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="B31" s="30" t="inlineStr">
         <is>
-          <t>T.J AGRICULTURA S.L.</t>
+          <t>MAJ AGROQUIMICOS S.L.</t>
         </is>
       </c>
       <c r="C31" s="31" t="inlineStr">
         <is>
-          <t>AN0020</t>
+          <t>FTK0005</t>
         </is>
       </c>
       <c r="D31" s="30" t="inlineStr">
         <is>
-          <t>ALCAPLANT NEW, 20 KG</t>
+          <t>FITOKONTROL CA FLOW, 5 KG</t>
         </is>
       </c>
       <c r="E31" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F31" s="18" t="n">
-        <v>600</v>
+        <v>40</v>
       </c>
       <c r="G31" s="18" t="n">
-        <v>600</v>
+        <v>40</v>
       </c>
       <c r="H31" s="18" t="n">
         <v>0</v>
@@ -2490,34 +2490,34 @@
       </c>
       <c r="L31" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="B32" s="27" t="inlineStr">
         <is>
-          <t>T.J AGRICULTURA S.L.</t>
+          <t>SAFIAGRO, S.A.</t>
         </is>
       </c>
       <c r="C32" s="28" t="inlineStr">
         <is>
-          <t>SS0020</t>
+          <t>AGXK0020</t>
         </is>
       </c>
       <c r="D32" s="27" t="inlineStr">
         <is>
-          <t>SALWAX-CA, 20 KG</t>
+          <t>AGROXILATO-K, 20 L</t>
         </is>
       </c>
       <c r="E32" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F32" s="14" t="n">
-        <v>500</v>
+        <v>640</v>
       </c>
       <c r="G32" s="14" t="n">
-        <v>500</v>
+        <v>640</v>
       </c>
       <c r="H32" s="14" t="n">
         <v>0</v>
@@ -2536,34 +2536,34 @@
       </c>
       <c r="L32" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="B33" s="30" t="inlineStr">
         <is>
-          <t>VILLALTA SATIVUM, S.L.</t>
+          <t>T.J AGRICULTURA S.L.</t>
         </is>
       </c>
       <c r="C33" s="31" t="inlineStr">
         <is>
-          <t>WHITE0020</t>
+          <t>AN0020</t>
         </is>
       </c>
       <c r="D33" s="30" t="inlineStr">
         <is>
-          <t>AGROWHITE, 20 KG</t>
+          <t>ALCAPLANT NEW, 20 KG</t>
         </is>
       </c>
       <c r="E33" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F33" s="18" t="n">
-        <v>2800</v>
+        <v>600</v>
       </c>
       <c r="G33" s="18" t="n">
-        <v>2800</v>
+        <v>600</v>
       </c>
       <c r="H33" s="18" t="n">
         <v>0</v>
@@ -2582,52 +2582,144 @@
       </c>
       <c r="L33" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="24" customHeight="1">
-      <c r="B34" s="20" t="inlineStr">
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="27" t="inlineStr">
+        <is>
+          <t>T.J AGRICULTURA S.L.</t>
+        </is>
+      </c>
+      <c r="C34" s="28" t="inlineStr">
+        <is>
+          <t>SS0020</t>
+        </is>
+      </c>
+      <c r="D34" s="27" t="inlineStr">
+        <is>
+          <t>SALWAX-CA, 20 KG</t>
+        </is>
+      </c>
+      <c r="E34" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" s="14" t="n">
+        <v>500</v>
+      </c>
+      <c r="G34" s="14" t="n">
+        <v>500</v>
+      </c>
+      <c r="H34" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I34" s="14">
+        <f>MAX(0, E34-F34)</f>
+        <v/>
+      </c>
+      <c r="J34" s="14">
+        <f>F34-E34</f>
+        <v/>
+      </c>
+      <c r="K34" s="15">
+        <f>IF(E34&gt;0, F34/E34, IF(F34&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L34" s="29" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="30" t="inlineStr">
+        <is>
+          <t>VILLALTA SATIVUM, S.L.</t>
+        </is>
+      </c>
+      <c r="C35" s="31" t="inlineStr">
+        <is>
+          <t>WHITE0020</t>
+        </is>
+      </c>
+      <c r="D35" s="30" t="inlineStr">
+        <is>
+          <t>AGROWHITE, 20 KG</t>
+        </is>
+      </c>
+      <c r="E35" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F35" s="18" t="n">
+        <v>3460</v>
+      </c>
+      <c r="G35" s="18" t="n">
+        <v>3460</v>
+      </c>
+      <c r="H35" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="I35" s="18">
+        <f>MAX(0, E35-F35)</f>
+        <v/>
+      </c>
+      <c r="J35" s="18">
+        <f>F35-E35</f>
+        <v/>
+      </c>
+      <c r="K35" s="19">
+        <f>IF(E35&gt;0, F35/E35, IF(F35&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L35" s="29" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="24" customHeight="1">
+      <c r="B36" s="20" t="inlineStr">
         <is>
           <t>TOTAL ALFONSO</t>
         </is>
       </c>
-      <c r="C34" s="33" t="inlineStr">
-        <is>
-          <t>279 líneas</t>
-        </is>
-      </c>
-      <c r="D34" s="34" t="inlineStr"/>
-      <c r="E34" s="22">
-        <f>SUM(E10:E33)</f>
-        <v/>
-      </c>
-      <c r="F34" s="22">
-        <f>SUM(F10:F33)</f>
-        <v/>
-      </c>
-      <c r="G34" s="22">
-        <f>SUM(G10:G33)</f>
-        <v/>
-      </c>
-      <c r="H34" s="22">
-        <f>SUM(H10:H33)</f>
-        <v/>
-      </c>
-      <c r="I34" s="22">
-        <f>SUM(I10:I33)</f>
-        <v/>
-      </c>
-      <c r="J34" s="22">
-        <f>SUM(J10:J33)</f>
-        <v/>
-      </c>
-      <c r="K34" s="23">
-        <f>IF(E34&gt;0, F34/E34, 0)</f>
-        <v/>
-      </c>
-      <c r="L34" s="21">
-        <f>IF(K34&gt;=1, "SUPERADO", "EN CURSO")</f>
+      <c r="C36" s="33" t="inlineStr">
+        <is>
+          <t>280 líneas</t>
+        </is>
+      </c>
+      <c r="D36" s="34" t="inlineStr"/>
+      <c r="E36" s="22">
+        <f>SUM(E10:E35)</f>
+        <v/>
+      </c>
+      <c r="F36" s="22">
+        <f>SUM(F10:F35)</f>
+        <v/>
+      </c>
+      <c r="G36" s="22">
+        <f>SUM(G10:G35)</f>
+        <v/>
+      </c>
+      <c r="H36" s="22">
+        <f>SUM(H10:H35)</f>
+        <v/>
+      </c>
+      <c r="I36" s="22">
+        <f>SUM(I10:I35)</f>
+        <v/>
+      </c>
+      <c r="J36" s="22">
+        <f>SUM(J10:J35)</f>
+        <v/>
+      </c>
+      <c r="K36" s="23">
+        <f>IF(E36&gt;0, F36/E36, 0)</f>
+        <v/>
+      </c>
+      <c r="L36" s="21">
+        <f>IF(K36&gt;=1, "SUPERADO", "EN CURSO")</f>
         <v/>
       </c>
     </row>
@@ -2656,7 +2748,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:L55"/>
+  <dimension ref="B2:L56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -2683,14 +2775,14 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 25/09/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 28/09/2026</t>
         </is>
       </c>
     </row>
     <row r="5" ht="16" customHeight="1">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>BUDGET SEP (U)</t>
+          <t>ESTIMACIÓN SEP (U)</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
@@ -2728,13 +2820,13 @@
       <c r="C6" s="4" t="n"/>
       <c r="D6" s="25" t="inlineStr">
         <is>
-          <t>52,772 u</t>
+          <t>55,612 u</t>
         </is>
       </c>
       <c r="E6" s="4" t="n"/>
       <c r="F6" s="25" t="inlineStr">
         <is>
-          <t>139.5%</t>
+          <t>147.0%</t>
         </is>
       </c>
       <c r="G6" s="4" t="n"/>
@@ -2746,7 +2838,7 @@
       <c r="I6" s="4" t="n"/>
       <c r="J6" s="24" t="inlineStr">
         <is>
-          <t>49,216 u</t>
+          <t>50,316 u</t>
         </is>
       </c>
       <c r="K6" s="4" t="n"/>
@@ -2776,7 +2868,7 @@
       </c>
       <c r="E9" s="11" t="inlineStr">
         <is>
-          <t>Budget Sep (u)</t>
+          <t>Estimación Sep (u)</t>
         </is>
       </c>
       <c r="F9" s="11" t="inlineStr">
@@ -2995,7 +3087,7 @@
       </c>
       <c r="L13" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -3065,10 +3157,10 @@
         <v>1920</v>
       </c>
       <c r="F15" s="18" t="n">
-        <v>640</v>
+        <v>1280</v>
       </c>
       <c r="G15" s="18" t="n">
-        <v>640</v>
+        <v>1280</v>
       </c>
       <c r="H15" s="18" t="n">
         <v>0</v>
@@ -3085,9 +3177,9 @@
         <f>IF(E15&gt;0, F15/E15, IF(F15&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L15" s="36" t="inlineStr">
-        <is>
-          <t>Rezagado</t>
+      <c r="L15" s="32" t="inlineStr">
+        <is>
+          <t>En Curso</t>
         </is>
       </c>
     </row>
@@ -3593,7 +3685,7 @@
       </c>
       <c r="L26" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -3639,7 +3731,7 @@
       </c>
       <c r="L27" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -3685,7 +3777,7 @@
       </c>
       <c r="L28" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -3731,7 +3823,7 @@
       </c>
       <c r="L29" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -3777,37 +3869,37 @@
       </c>
       <c r="L30" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="B31" s="30" t="inlineStr">
         <is>
-          <t>INIESTA DEL PINO DISTRIBUCIONES S.L.U</t>
+          <t>EL PINAR BERRIES, S.L.</t>
         </is>
       </c>
       <c r="C31" s="31" t="inlineStr">
         <is>
-          <t>AGXK0020</t>
+          <t>AN0005</t>
         </is>
       </c>
       <c r="D31" s="30" t="inlineStr">
         <is>
-          <t>AGROXILATO-K, 20 L</t>
+          <t>ALCAPLANT NEW, 5 KG</t>
         </is>
       </c>
       <c r="E31" s="18" t="n">
-        <v>640</v>
+        <v>0</v>
       </c>
       <c r="F31" s="18" t="n">
-        <v>0</v>
+        <v>1100</v>
       </c>
       <c r="G31" s="18" t="n">
         <v>0</v>
       </c>
       <c r="H31" s="18" t="n">
-        <v>0</v>
+        <v>1100</v>
       </c>
       <c r="I31" s="18">
         <f>MAX(0, E31-F31)</f>
@@ -3821,9 +3913,9 @@
         <f>IF(E31&gt;0, F31/E31, IF(F31&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L31" s="35" t="inlineStr">
-        <is>
-          <t>Sin Pedido</t>
+      <c r="L31" s="29" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -3835,16 +3927,16 @@
       </c>
       <c r="C32" s="28" t="inlineStr">
         <is>
-          <t>TRI0005</t>
+          <t>AGXK0020</t>
         </is>
       </c>
       <c r="D32" s="27" t="inlineStr">
         <is>
-          <t>TRIFENO-94, 5L</t>
+          <t>AGROXILATO-K, 20 L</t>
         </is>
       </c>
       <c r="E32" s="14" t="n">
-        <v>60</v>
+        <v>640</v>
       </c>
       <c r="F32" s="14" t="n">
         <v>0</v>
@@ -3876,30 +3968,30 @@
     <row r="33">
       <c r="B33" s="30" t="inlineStr">
         <is>
-          <t>SC MARCOSER S.R.L.</t>
+          <t>INIESTA DEL PINO DISTRIBUCIONES S.L.U</t>
         </is>
       </c>
       <c r="C33" s="31" t="inlineStr">
         <is>
-          <t>A-500001</t>
+          <t>TRI0005</t>
         </is>
       </c>
       <c r="D33" s="30" t="inlineStr">
         <is>
-          <t>CODIORGAN  A-50</t>
+          <t>TRIFENO-94, 5L</t>
         </is>
       </c>
       <c r="E33" s="18" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="F33" s="18" t="n">
-        <v>1056</v>
+        <v>0</v>
       </c>
       <c r="G33" s="18" t="n">
         <v>0</v>
       </c>
       <c r="H33" s="18" t="n">
-        <v>1056</v>
+        <v>0</v>
       </c>
       <c r="I33" s="18">
         <f>MAX(0, E33-F33)</f>
@@ -3913,9 +4005,9 @@
         <f>IF(E33&gt;0, F33/E33, IF(F33&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L33" s="29" t="inlineStr">
-        <is>
-          <t>Extra Budget</t>
+      <c r="L33" s="35" t="inlineStr">
+        <is>
+          <t>Sin Pedido</t>
         </is>
       </c>
     </row>
@@ -3927,25 +4019,25 @@
       </c>
       <c r="C34" s="28" t="inlineStr">
         <is>
-          <t>AGMG0001</t>
+          <t>A-500001</t>
         </is>
       </c>
       <c r="D34" s="27" t="inlineStr">
         <is>
-          <t>AGROXILATO Mg</t>
+          <t>CODIORGAN  A-50</t>
         </is>
       </c>
       <c r="E34" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F34" s="14" t="n">
-        <v>528</v>
+        <v>1056</v>
       </c>
       <c r="G34" s="14" t="n">
         <v>0</v>
       </c>
       <c r="H34" s="14" t="n">
-        <v>528</v>
+        <v>1056</v>
       </c>
       <c r="I34" s="14">
         <f>MAX(0, E34-F34)</f>
@@ -3961,7 +4053,7 @@
       </c>
       <c r="L34" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -3973,25 +4065,25 @@
       </c>
       <c r="C35" s="31" t="inlineStr">
         <is>
-          <t>AGXKAEP0001</t>
+          <t>AGMG0001</t>
         </is>
       </c>
       <c r="D35" s="30" t="inlineStr">
         <is>
-          <t>BIOCULTURE POTASIO PLUS, 1 L</t>
+          <t>AGROXILATO Mg</t>
         </is>
       </c>
       <c r="E35" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F35" s="18" t="n">
-        <v>396</v>
+        <v>528</v>
       </c>
       <c r="G35" s="18" t="n">
         <v>0</v>
       </c>
       <c r="H35" s="18" t="n">
-        <v>396</v>
+        <v>528</v>
       </c>
       <c r="I35" s="18">
         <f>MAX(0, E35-F35)</f>
@@ -4007,7 +4099,7 @@
       </c>
       <c r="L35" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -4019,25 +4111,25 @@
       </c>
       <c r="C36" s="28" t="inlineStr">
         <is>
-          <t>BIO0001</t>
+          <t>AGXKAEP0001</t>
         </is>
       </c>
       <c r="D36" s="27" t="inlineStr">
         <is>
-          <t>BIORAD-20</t>
+          <t>BIOCULTURE POTASIO PLUS, 1 L</t>
         </is>
       </c>
       <c r="E36" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F36" s="14" t="n">
-        <v>792</v>
+        <v>396</v>
       </c>
       <c r="G36" s="14" t="n">
         <v>0</v>
       </c>
       <c r="H36" s="14" t="n">
-        <v>792</v>
+        <v>396</v>
       </c>
       <c r="I36" s="14">
         <f>MAX(0, E36-F36)</f>
@@ -4053,7 +4145,7 @@
       </c>
       <c r="L36" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -4065,7 +4157,7 @@
       </c>
       <c r="C37" s="31" t="inlineStr">
         <is>
-          <t>BIO0005</t>
+          <t>BIO0001</t>
         </is>
       </c>
       <c r="D37" s="30" t="inlineStr">
@@ -4077,13 +4169,13 @@
         <v>0</v>
       </c>
       <c r="F37" s="18" t="n">
-        <v>600</v>
+        <v>792</v>
       </c>
       <c r="G37" s="18" t="n">
         <v>0</v>
       </c>
       <c r="H37" s="18" t="n">
-        <v>600</v>
+        <v>792</v>
       </c>
       <c r="I37" s="18">
         <f>MAX(0, E37-F37)</f>
@@ -4099,7 +4191,7 @@
       </c>
       <c r="L37" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -4111,7 +4203,7 @@
       </c>
       <c r="C38" s="28" t="inlineStr">
         <is>
-          <t>BIO0020</t>
+          <t>BIO0005</t>
         </is>
       </c>
       <c r="D38" s="27" t="inlineStr">
@@ -4123,13 +4215,13 @@
         <v>0</v>
       </c>
       <c r="F38" s="14" t="n">
-        <v>640</v>
+        <v>600</v>
       </c>
       <c r="G38" s="14" t="n">
         <v>0</v>
       </c>
       <c r="H38" s="14" t="n">
-        <v>640</v>
+        <v>600</v>
       </c>
       <c r="I38" s="14">
         <f>MAX(0, E38-F38)</f>
@@ -4145,7 +4237,7 @@
       </c>
       <c r="L38" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -4157,25 +4249,25 @@
       </c>
       <c r="C39" s="31" t="inlineStr">
         <is>
-          <t>C-L0001</t>
+          <t>BIO0020</t>
         </is>
       </c>
       <c r="D39" s="30" t="inlineStr">
         <is>
-          <t>CODIBOR-L</t>
+          <t>BIORAD-20</t>
         </is>
       </c>
       <c r="E39" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F39" s="18" t="n">
-        <v>792</v>
+        <v>640</v>
       </c>
       <c r="G39" s="18" t="n">
         <v>0</v>
       </c>
       <c r="H39" s="18" t="n">
-        <v>792</v>
+        <v>640</v>
       </c>
       <c r="I39" s="18">
         <f>MAX(0, E39-F39)</f>
@@ -4191,7 +4283,7 @@
       </c>
       <c r="L39" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -4203,25 +4295,25 @@
       </c>
       <c r="C40" s="28" t="inlineStr">
         <is>
-          <t>P-5X0020RU</t>
+          <t>C-L0001</t>
         </is>
       </c>
       <c r="D40" s="27" t="inlineStr">
         <is>
-          <t>P.M.S. 5x, 20 L</t>
+          <t>CODIBOR-L</t>
         </is>
       </c>
       <c r="E40" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F40" s="14" t="n">
-        <v>640</v>
+        <v>792</v>
       </c>
       <c r="G40" s="14" t="n">
         <v>0</v>
       </c>
       <c r="H40" s="14" t="n">
-        <v>640</v>
+        <v>792</v>
       </c>
       <c r="I40" s="14">
         <f>MAX(0, E40-F40)</f>
@@ -4237,7 +4329,7 @@
       </c>
       <c r="L40" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -4249,25 +4341,25 @@
       </c>
       <c r="C41" s="31" t="inlineStr">
         <is>
-          <t>SPCE0001</t>
+          <t>P-5X0020RU</t>
         </is>
       </c>
       <c r="D41" s="30" t="inlineStr">
         <is>
-          <t>SPRINTENE</t>
+          <t>P.M.S. 5x, 20 L</t>
         </is>
       </c>
       <c r="E41" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F41" s="18" t="n">
-        <v>792</v>
+        <v>640</v>
       </c>
       <c r="G41" s="18" t="n">
         <v>0</v>
       </c>
       <c r="H41" s="18" t="n">
-        <v>792</v>
+        <v>640</v>
       </c>
       <c r="I41" s="18">
         <f>MAX(0, E41-F41)</f>
@@ -4283,7 +4375,7 @@
       </c>
       <c r="L41" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -4295,7 +4387,7 @@
       </c>
       <c r="C42" s="28" t="inlineStr">
         <is>
-          <t>SPCE0020</t>
+          <t>SPCE0001</t>
         </is>
       </c>
       <c r="D42" s="27" t="inlineStr">
@@ -4307,13 +4399,13 @@
         <v>0</v>
       </c>
       <c r="F42" s="14" t="n">
-        <v>640</v>
+        <v>792</v>
       </c>
       <c r="G42" s="14" t="n">
         <v>0</v>
       </c>
       <c r="H42" s="14" t="n">
-        <v>640</v>
+        <v>792</v>
       </c>
       <c r="I42" s="14">
         <f>MAX(0, E42-F42)</f>
@@ -4329,7 +4421,7 @@
       </c>
       <c r="L42" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -4341,25 +4433,25 @@
       </c>
       <c r="C43" s="31" t="inlineStr">
         <is>
-          <t>SS0001</t>
+          <t>SPCE0020</t>
         </is>
       </c>
       <c r="D43" s="30" t="inlineStr">
         <is>
-          <t>SAL-WAX Ca</t>
+          <t>SPRINTENE</t>
         </is>
       </c>
       <c r="E43" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F43" s="18" t="n">
-        <v>1056</v>
+        <v>640</v>
       </c>
       <c r="G43" s="18" t="n">
         <v>0</v>
       </c>
       <c r="H43" s="18" t="n">
-        <v>1056</v>
+        <v>640</v>
       </c>
       <c r="I43" s="18">
         <f>MAX(0, E43-F43)</f>
@@ -4375,37 +4467,37 @@
       </c>
       <c r="L43" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="B44" s="27" t="inlineStr">
         <is>
-          <t>SERVIAGRI´ 97, S.L.</t>
+          <t>SC MARCOSER S.R.L.</t>
         </is>
       </c>
       <c r="C44" s="28" t="inlineStr">
         <is>
-          <t>AGXK0005</t>
+          <t>SS0001</t>
         </is>
       </c>
       <c r="D44" s="27" t="inlineStr">
         <is>
-          <t>AGROXILATO-K, 5 L</t>
+          <t>SAL-WAX Ca</t>
         </is>
       </c>
       <c r="E44" s="14" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="F44" s="14" t="n">
-        <v>0</v>
+        <v>1056</v>
       </c>
       <c r="G44" s="14" t="n">
         <v>0</v>
       </c>
       <c r="H44" s="14" t="n">
-        <v>0</v>
+        <v>1056</v>
       </c>
       <c r="I44" s="14">
         <f>MAX(0, E44-F44)</f>
@@ -4419,9 +4511,9 @@
         <f>IF(E44&gt;0, F44/E44, IF(F44&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L44" s="35" t="inlineStr">
-        <is>
-          <t>Sin Pedido</t>
+      <c r="L44" s="29" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -4433,22 +4525,22 @@
       </c>
       <c r="C45" s="31" t="inlineStr">
         <is>
-          <t>AGXK0020</t>
+          <t>AGXK0005</t>
         </is>
       </c>
       <c r="D45" s="30" t="inlineStr">
         <is>
-          <t>AGROXILATO-K, 20 L</t>
+          <t>AGROXILATO-K, 5 L</t>
         </is>
       </c>
       <c r="E45" s="18" t="n">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="F45" s="18" t="n">
-        <v>120</v>
+        <v>0</v>
       </c>
       <c r="G45" s="18" t="n">
-        <v>120</v>
+        <v>0</v>
       </c>
       <c r="H45" s="18" t="n">
         <v>0</v>
@@ -4465,9 +4557,9 @@
         <f>IF(E45&gt;0, F45/E45, IF(F45&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L45" s="29" t="inlineStr">
-        <is>
-          <t>Extra Budget</t>
+      <c r="L45" s="35" t="inlineStr">
+        <is>
+          <t>Sin Pedido</t>
         </is>
       </c>
     </row>
@@ -4479,16 +4571,16 @@
       </c>
       <c r="C46" s="28" t="inlineStr">
         <is>
-          <t>AVAN0005</t>
+          <t>AGXK0020</t>
         </is>
       </c>
       <c r="D46" s="27" t="inlineStr">
         <is>
-          <t>FLORAMEC AVANCE, 5 L</t>
+          <t>AGROXILATO-K, 20 L</t>
         </is>
       </c>
       <c r="E46" s="14" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="F46" s="14" t="n">
         <v>120</v>
@@ -4513,7 +4605,7 @@
       </c>
       <c r="L46" s="29" t="inlineStr">
         <is>
-          <t>Superado</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -4525,22 +4617,22 @@
       </c>
       <c r="C47" s="31" t="inlineStr">
         <is>
-          <t>B0001</t>
+          <t>AVAN0005</t>
         </is>
       </c>
       <c r="D47" s="30" t="inlineStr">
         <is>
-          <t>BOROCAL,1 L</t>
+          <t>FLORAMEC AVANCE, 5 L</t>
         </is>
       </c>
       <c r="E47" s="18" t="n">
-        <v>12</v>
+        <v>100</v>
       </c>
       <c r="F47" s="18" t="n">
-        <v>12</v>
+        <v>120</v>
       </c>
       <c r="G47" s="18" t="n">
-        <v>12</v>
+        <v>120</v>
       </c>
       <c r="H47" s="18" t="n">
         <v>0</v>
@@ -4571,22 +4663,22 @@
       </c>
       <c r="C48" s="28" t="inlineStr">
         <is>
-          <t>BIO0005</t>
+          <t>B0001</t>
         </is>
       </c>
       <c r="D48" s="27" t="inlineStr">
         <is>
-          <t>BIORAD-20, 5L</t>
+          <t>BOROCAL,1 L</t>
         </is>
       </c>
       <c r="E48" s="14" t="n">
-        <v>300</v>
+        <v>12</v>
       </c>
       <c r="F48" s="14" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="G48" s="14" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="H48" s="14" t="n">
         <v>0</v>
@@ -4603,9 +4695,9 @@
         <f>IF(E48&gt;0, F48/E48, IF(F48&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L48" s="35" t="inlineStr">
-        <is>
-          <t>Sin Pedido</t>
+      <c r="L48" s="29" t="inlineStr">
+        <is>
+          <t>Superado</t>
         </is>
       </c>
     </row>
@@ -4617,22 +4709,22 @@
       </c>
       <c r="C49" s="31" t="inlineStr">
         <is>
-          <t>BROTA0001</t>
+          <t>BIO0005</t>
         </is>
       </c>
       <c r="D49" s="30" t="inlineStr">
         <is>
-          <t>BROTAMEC, 1 L</t>
+          <t>BIORAD-20, 5L</t>
         </is>
       </c>
       <c r="E49" s="18" t="n">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="F49" s="18" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="G49" s="18" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="H49" s="18" t="n">
         <v>0</v>
@@ -4649,9 +4741,9 @@
         <f>IF(E49&gt;0, F49/E49, IF(F49&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L49" s="29" t="inlineStr">
-        <is>
-          <t>Extra Budget</t>
+      <c r="L49" s="35" t="inlineStr">
+        <is>
+          <t>Sin Pedido</t>
         </is>
       </c>
     </row>
@@ -4663,22 +4755,22 @@
       </c>
       <c r="C50" s="28" t="inlineStr">
         <is>
-          <t>BROTA0005</t>
+          <t>BROTA0001</t>
         </is>
       </c>
       <c r="D50" s="27" t="inlineStr">
         <is>
-          <t>BROTAMEC, 5 L</t>
+          <t>BROTAMEC, 1 L</t>
         </is>
       </c>
       <c r="E50" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F50" s="14" t="n">
-        <v>100</v>
+        <v>24</v>
       </c>
       <c r="G50" s="14" t="n">
-        <v>100</v>
+        <v>24</v>
       </c>
       <c r="H50" s="14" t="n">
         <v>0</v>
@@ -4697,7 +4789,7 @@
       </c>
       <c r="L50" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -4709,22 +4801,22 @@
       </c>
       <c r="C51" s="31" t="inlineStr">
         <is>
-          <t>FTK0005</t>
+          <t>BROTA0005</t>
         </is>
       </c>
       <c r="D51" s="30" t="inlineStr">
         <is>
-          <t>FITOKONTROL CA FLOW, 5 KG</t>
+          <t>BROTAMEC, 5 L</t>
         </is>
       </c>
       <c r="E51" s="18" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="F51" s="18" t="n">
-        <v>160</v>
+        <v>100</v>
       </c>
       <c r="G51" s="18" t="n">
-        <v>160</v>
+        <v>100</v>
       </c>
       <c r="H51" s="18" t="n">
         <v>0</v>
@@ -4741,9 +4833,9 @@
         <f>IF(E51&gt;0, F51/E51, IF(F51&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L51" s="32" t="inlineStr">
-        <is>
-          <t>En Curso</t>
+      <c r="L51" s="29" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -4755,22 +4847,22 @@
       </c>
       <c r="C52" s="28" t="inlineStr">
         <is>
-          <t>JF0005</t>
+          <t>FTK0005</t>
         </is>
       </c>
       <c r="D52" s="27" t="inlineStr">
         <is>
-          <t>CODIGIN-FOS, 5 L</t>
+          <t>FITOKONTROL CA FLOW, 5 KG</t>
         </is>
       </c>
       <c r="E52" s="14" t="n">
-        <v>100</v>
+        <v>300</v>
       </c>
       <c r="F52" s="14" t="n">
-        <v>120</v>
+        <v>160</v>
       </c>
       <c r="G52" s="14" t="n">
-        <v>120</v>
+        <v>160</v>
       </c>
       <c r="H52" s="14" t="n">
         <v>0</v>
@@ -4787,9 +4879,9 @@
         <f>IF(E52&gt;0, F52/E52, IF(F52&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L52" s="29" t="inlineStr">
-        <is>
-          <t>Superado</t>
+      <c r="L52" s="32" t="inlineStr">
+        <is>
+          <t>En Curso</t>
         </is>
       </c>
     </row>
@@ -4801,22 +4893,22 @@
       </c>
       <c r="C53" s="31" t="inlineStr">
         <is>
-          <t>SSAE0005</t>
+          <t>JF0005</t>
         </is>
       </c>
       <c r="D53" s="30" t="inlineStr">
         <is>
-          <t>MAGNIFIC-VIETS-AE, 5 KG</t>
+          <t>CODIGIN-FOS, 5 L</t>
         </is>
       </c>
       <c r="E53" s="18" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="F53" s="18" t="n">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="G53" s="18" t="n">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="H53" s="18" t="n">
         <v>0</v>
@@ -4835,34 +4927,34 @@
       </c>
       <c r="L53" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Superado</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="B54" s="27" t="inlineStr">
         <is>
-          <t>TRATAMIENTOS AGRICOLAS BRENES, S.L.</t>
+          <t>SERVIAGRI´ 97, S.L.</t>
         </is>
       </c>
       <c r="C54" s="28" t="inlineStr">
         <is>
-          <t>WHITE0020</t>
+          <t>SSAE0005</t>
         </is>
       </c>
       <c r="D54" s="27" t="inlineStr">
         <is>
-          <t>AGROWHITE, 20 KG</t>
+          <t>MAGNIFIC-VIETS-AE, 5 KG</t>
         </is>
       </c>
       <c r="E54" s="14" t="n">
-        <v>1100</v>
+        <v>0</v>
       </c>
       <c r="F54" s="14" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="G54" s="14" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="H54" s="14" t="n">
         <v>0</v>
@@ -4879,54 +4971,100 @@
         <f>IF(E54&gt;0, F54/E54, IF(F54&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L54" s="35" t="inlineStr">
-        <is>
-          <t>Sin Pedido</t>
-        </is>
-      </c>
-    </row>
-    <row r="55" ht="24" customHeight="1">
-      <c r="B55" s="20" t="inlineStr">
+      <c r="L54" s="29" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="B55" s="30" t="inlineStr">
+        <is>
+          <t>TRATAMIENTOS AGRICOLAS BRENES, S.L.</t>
+        </is>
+      </c>
+      <c r="C55" s="31" t="inlineStr">
+        <is>
+          <t>WHITE0020</t>
+        </is>
+      </c>
+      <c r="D55" s="30" t="inlineStr">
+        <is>
+          <t>AGROWHITE, 20 KG</t>
+        </is>
+      </c>
+      <c r="E55" s="18" t="n">
+        <v>1100</v>
+      </c>
+      <c r="F55" s="18" t="n">
+        <v>1100</v>
+      </c>
+      <c r="G55" s="18" t="n">
+        <v>1100</v>
+      </c>
+      <c r="H55" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="I55" s="18">
+        <f>MAX(0, E55-F55)</f>
+        <v/>
+      </c>
+      <c r="J55" s="18">
+        <f>F55-E55</f>
+        <v/>
+      </c>
+      <c r="K55" s="19">
+        <f>IF(E55&gt;0, F55/E55, IF(F55&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L55" s="29" t="inlineStr">
+        <is>
+          <t>Superado</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="24" customHeight="1">
+      <c r="B56" s="20" t="inlineStr">
         <is>
           <t>TOTAL GARCÍA</t>
         </is>
       </c>
-      <c r="C55" s="33" t="inlineStr">
-        <is>
-          <t>234 líneas</t>
-        </is>
-      </c>
-      <c r="D55" s="34" t="inlineStr"/>
-      <c r="E55" s="22">
-        <f>SUM(E10:E54)</f>
-        <v/>
-      </c>
-      <c r="F55" s="22">
-        <f>SUM(F10:F54)</f>
-        <v/>
-      </c>
-      <c r="G55" s="22">
-        <f>SUM(G10:G54)</f>
-        <v/>
-      </c>
-      <c r="H55" s="22">
-        <f>SUM(H10:H54)</f>
-        <v/>
-      </c>
-      <c r="I55" s="22">
-        <f>SUM(I10:I54)</f>
-        <v/>
-      </c>
-      <c r="J55" s="22">
-        <f>SUM(J10:J54)</f>
-        <v/>
-      </c>
-      <c r="K55" s="23">
-        <f>IF(E55&gt;0, F55/E55, 0)</f>
-        <v/>
-      </c>
-      <c r="L55" s="21">
-        <f>IF(K55&gt;=1, "SUPERADO", "EN CURSO")</f>
+      <c r="C56" s="33" t="inlineStr">
+        <is>
+          <t>235 líneas</t>
+        </is>
+      </c>
+      <c r="D56" s="34" t="inlineStr"/>
+      <c r="E56" s="22">
+        <f>SUM(E10:E55)</f>
+        <v/>
+      </c>
+      <c r="F56" s="22">
+        <f>SUM(F10:F55)</f>
+        <v/>
+      </c>
+      <c r="G56" s="22">
+        <f>SUM(G10:G55)</f>
+        <v/>
+      </c>
+      <c r="H56" s="22">
+        <f>SUM(H10:H55)</f>
+        <v/>
+      </c>
+      <c r="I56" s="22">
+        <f>SUM(I10:I55)</f>
+        <v/>
+      </c>
+      <c r="J56" s="22">
+        <f>SUM(J10:J55)</f>
+        <v/>
+      </c>
+      <c r="K56" s="23">
+        <f>IF(E56&gt;0, F56/E56, 0)</f>
+        <v/>
+      </c>
+      <c r="L56" s="21">
+        <f>IF(K56&gt;=1, "SUPERADO", "EN CURSO")</f>
         <v/>
       </c>
     </row>
@@ -4982,14 +5120,14 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 25/09/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 28/09/2026</t>
         </is>
       </c>
     </row>
     <row r="5" ht="16" customHeight="1">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>BUDGET SEP (U)</t>
+          <t>ESTIMACIÓN SEP (U)</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
@@ -5075,7 +5213,7 @@
       </c>
       <c r="E9" s="11" t="inlineStr">
         <is>
-          <t>Budget Sep (u)</t>
+          <t>Estimación Sep (u)</t>
         </is>
       </c>
       <c r="F9" s="11" t="inlineStr">
@@ -5202,7 +5340,7 @@
       </c>
       <c r="L11" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -6306,7 +6444,7 @@
       </c>
       <c r="L35" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -6674,7 +6812,7 @@
       </c>
       <c r="L43" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -6775,14 +6913,14 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 25/09/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 28/09/2026</t>
         </is>
       </c>
     </row>
     <row r="5" ht="16" customHeight="1">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>BUDGET SEP (U)</t>
+          <t>ESTIMACIÓN SEP (U)</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
@@ -6838,7 +6976,7 @@
       <c r="I6" s="4" t="n"/>
       <c r="J6" s="24" t="inlineStr">
         <is>
-          <t>12,784 u</t>
+          <t>0 u</t>
         </is>
       </c>
       <c r="K6" s="4" t="n"/>
@@ -6868,7 +7006,7 @@
       </c>
       <c r="E9" s="11" t="inlineStr">
         <is>
-          <t>Budget Sep (u)</t>
+          <t>Estimación Sep (u)</t>
         </is>
       </c>
       <c r="F9" s="11" t="inlineStr">
@@ -6995,7 +7133,7 @@
       </c>
       <c r="L11" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -7087,7 +7225,7 @@
       </c>
       <c r="L13" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -7133,7 +7271,7 @@
       </c>
       <c r="L14" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -7179,7 +7317,7 @@
       </c>
       <c r="L15" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -7225,7 +7363,7 @@
       </c>
       <c r="L16" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -7271,7 +7409,7 @@
       </c>
       <c r="L17" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -7317,7 +7455,7 @@
       </c>
       <c r="L18" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -7363,7 +7501,7 @@
       </c>
       <c r="L19" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -7409,7 +7547,7 @@
       </c>
       <c r="L20" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -7455,7 +7593,7 @@
       </c>
       <c r="L21" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -7547,7 +7685,7 @@
       </c>
       <c r="L23" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -7593,7 +7731,7 @@
       </c>
       <c r="L24" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -7639,7 +7777,7 @@
       </c>
       <c r="L25" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -7777,7 +7915,7 @@
       </c>
       <c r="L28" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -7823,7 +7961,7 @@
       </c>
       <c r="L29" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -7869,7 +8007,7 @@
       </c>
       <c r="L30" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -7915,7 +8053,7 @@
       </c>
       <c r="L31" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -7961,7 +8099,7 @@
       </c>
       <c r="L32" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -8007,7 +8145,7 @@
       </c>
       <c r="L33" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -8053,7 +8191,7 @@
       </c>
       <c r="L34" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -8099,7 +8237,7 @@
       </c>
       <c r="L35" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -8145,7 +8283,7 @@
       </c>
       <c r="L36" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -8191,7 +8329,7 @@
       </c>
       <c r="L37" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -8218,10 +8356,10 @@
         <v>1600</v>
       </c>
       <c r="G38" s="14" t="n">
-        <v>0</v>
+        <v>1600</v>
       </c>
       <c r="H38" s="14" t="n">
-        <v>1600</v>
+        <v>0</v>
       </c>
       <c r="I38" s="14">
         <f>MAX(0, E38-F38)</f>
@@ -8237,7 +8375,7 @@
       </c>
       <c r="L38" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -8264,10 +8402,10 @@
         <v>10000</v>
       </c>
       <c r="G39" s="18" t="n">
-        <v>2000</v>
+        <v>10000</v>
       </c>
       <c r="H39" s="18" t="n">
-        <v>8000</v>
+        <v>0</v>
       </c>
       <c r="I39" s="18">
         <f>MAX(0, E39-F39)</f>
@@ -8283,7 +8421,7 @@
       </c>
       <c r="L39" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -8310,10 +8448,10 @@
         <v>24</v>
       </c>
       <c r="G40" s="14" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="H40" s="14" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="I40" s="14">
         <f>MAX(0, E40-F40)</f>
@@ -8329,7 +8467,7 @@
       </c>
       <c r="L40" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -8356,10 +8494,10 @@
         <v>1280</v>
       </c>
       <c r="G41" s="18" t="n">
-        <v>0</v>
+        <v>1280</v>
       </c>
       <c r="H41" s="18" t="n">
-        <v>1280</v>
+        <v>0</v>
       </c>
       <c r="I41" s="18">
         <f>MAX(0, E41-F41)</f>
@@ -8375,7 +8513,7 @@
       </c>
       <c r="L41" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -8402,10 +8540,10 @@
         <v>400</v>
       </c>
       <c r="G42" s="14" t="n">
-        <v>0</v>
+        <v>400</v>
       </c>
       <c r="H42" s="14" t="n">
-        <v>400</v>
+        <v>0</v>
       </c>
       <c r="I42" s="14">
         <f>MAX(0, E42-F42)</f>
@@ -8421,7 +8559,7 @@
       </c>
       <c r="L42" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -8448,10 +8586,10 @@
         <v>640</v>
       </c>
       <c r="G43" s="18" t="n">
-        <v>0</v>
+        <v>640</v>
       </c>
       <c r="H43" s="18" t="n">
-        <v>640</v>
+        <v>0</v>
       </c>
       <c r="I43" s="18">
         <f>MAX(0, E43-F43)</f>
@@ -8467,7 +8605,7 @@
       </c>
       <c r="L43" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -8494,10 +8632,10 @@
         <v>800</v>
       </c>
       <c r="G44" s="14" t="n">
-        <v>0</v>
+        <v>800</v>
       </c>
       <c r="H44" s="14" t="n">
-        <v>800</v>
+        <v>0</v>
       </c>
       <c r="I44" s="14">
         <f>MAX(0, E44-F44)</f>
@@ -8513,7 +8651,7 @@
       </c>
       <c r="L44" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -8540,10 +8678,10 @@
         <v>40</v>
       </c>
       <c r="G45" s="18" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="H45" s="18" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="I45" s="18">
         <f>MAX(0, E45-F45)</f>
@@ -8559,7 +8697,7 @@
       </c>
       <c r="L45" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -8697,7 +8835,7 @@
       </c>
       <c r="L48" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -8798,14 +8936,14 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 25/09/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 28/09/2026</t>
         </is>
       </c>
     </row>
     <row r="5" ht="16" customHeight="1">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>BUDGET SEP (U)</t>
+          <t>ESTIMACIÓN SEP (U)</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
@@ -8891,7 +9029,7 @@
       </c>
       <c r="E9" s="11" t="inlineStr">
         <is>
-          <t>Budget Sep (u)</t>
+          <t>Estimación Sep (u)</t>
         </is>
       </c>
       <c r="F9" s="11" t="inlineStr">
@@ -9303,14 +9441,14 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 25/09/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 28/09/2026</t>
         </is>
       </c>
     </row>
     <row r="5" ht="16" customHeight="1">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>BUDGET SEP (U)</t>
+          <t>ESTIMACIÓN SEP (U)</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
@@ -9396,7 +9534,7 @@
       </c>
       <c r="E9" s="11" t="inlineStr">
         <is>
-          <t>Budget Sep (u)</t>
+          <t>Estimación Sep (u)</t>
         </is>
       </c>
       <c r="F9" s="11" t="inlineStr">
@@ -9845,7 +9983,7 @@
       </c>
       <c r="L18" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -9891,7 +10029,7 @@
       </c>
       <c r="L19" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -9937,7 +10075,7 @@
       </c>
       <c r="L20" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -9983,7 +10121,7 @@
       </c>
       <c r="L21" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -10213,7 +10351,7 @@
       </c>
       <c r="L26" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -10259,7 +10397,7 @@
       </c>
       <c r="L27" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -10305,7 +10443,7 @@
       </c>
       <c r="L28" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -10406,14 +10544,14 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 25/09/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 28/09/2026</t>
         </is>
       </c>
     </row>
     <row r="5" ht="16" customHeight="1">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>BUDGET SEP (U)</t>
+          <t>ESTIMACIÓN SEP (U)</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
@@ -10499,7 +10637,7 @@
       </c>
       <c r="E9" s="11" t="inlineStr">
         <is>
-          <t>Budget Sep (u)</t>
+          <t>Estimación Sep (u)</t>
         </is>
       </c>
       <c r="F9" s="11" t="inlineStr">
@@ -10580,7 +10718,7 @@
       </c>
       <c r="L10" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -10626,7 +10764,7 @@
       </c>
       <c r="L11" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -10672,7 +10810,7 @@
       </c>
       <c r="L12" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -10764,7 +10902,7 @@
       </c>
       <c r="L14" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -10810,7 +10948,7 @@
       </c>
       <c r="L15" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -10856,7 +10994,7 @@
       </c>
       <c r="L16" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -10902,7 +11040,7 @@
       </c>
       <c r="L17" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -10948,7 +11086,7 @@
       </c>
       <c r="L18" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -10994,7 +11132,7 @@
       </c>
       <c r="L19" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -11040,7 +11178,7 @@
       </c>
       <c r="L20" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -11086,7 +11224,7 @@
       </c>
       <c r="L21" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -11132,7 +11270,7 @@
       </c>
       <c r="L22" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -11178,7 +11316,7 @@
       </c>
       <c r="L23" s="29" t="inlineStr">
         <is>
-          <t>Extra Budget</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizar pedidos a 29/09/2026 y sincronizar dashboard y Excel
</commit_message>
<xml_diff>
--- a/Seguimiento_Presupuesto_Sep_2026.xlsx
+++ b/Seguimiento_Presupuesto_Sep_2026.xlsx
@@ -902,7 +902,7 @@
     <row r="3" ht="20" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Comparativa Estimación Septiembre (Unidades) vs Pedidos Reales a Fecha 28/09/2026 | Generado: 29/09/2026 07:26</t>
+          <t>Comparativa Estimación Septiembre (Unidades) vs Pedidos Reales a Fecha 29/09/2026 | Generado: 29/09/2026 07:41</t>
         </is>
       </c>
     </row>
@@ -946,25 +946,25 @@
       <c r="C6" s="4" t="n"/>
       <c r="D6" s="8" t="inlineStr">
         <is>
-          <t>203,399 u</t>
+          <t>206,419 u</t>
         </is>
       </c>
       <c r="E6" s="4" t="n"/>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>111.8%</t>
+          <t>113.4%</t>
         </is>
       </c>
       <c r="G6" s="4" t="n"/>
       <c r="H6" s="9" t="inlineStr">
         <is>
-          <t>39,570 u</t>
+          <t>24,576 u</t>
         </is>
       </c>
       <c r="I6" s="4" t="n"/>
       <c r="J6" s="7" t="inlineStr">
         <is>
-          <t>104,818 u</t>
+          <t>104,718 u</t>
         </is>
       </c>
     </row>
@@ -1029,16 +1029,16 @@
         </is>
       </c>
       <c r="C10" s="13" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D10" s="14" t="n">
         <v>2320</v>
       </c>
       <c r="E10" s="14" t="n">
-        <v>11410</v>
+        <v>11710</v>
       </c>
       <c r="F10" s="14" t="n">
-        <v>11410</v>
+        <v>11710</v>
       </c>
       <c r="G10" s="14" t="n">
         <v>0</v>
@@ -1063,16 +1063,16 @@
         </is>
       </c>
       <c r="C11" s="17" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D11" s="18" t="n">
         <v>37832</v>
       </c>
       <c r="E11" s="18" t="n">
-        <v>55612</v>
+        <v>56212</v>
       </c>
       <c r="F11" s="18" t="n">
-        <v>5296</v>
+        <v>5896</v>
       </c>
       <c r="G11" s="18" t="n">
         <v>50316</v>
@@ -1103,10 +1103,10 @@
         <v>21914</v>
       </c>
       <c r="E12" s="14" t="n">
-        <v>12806</v>
+        <v>14826</v>
       </c>
       <c r="F12" s="14" t="n">
-        <v>12806</v>
+        <v>14826</v>
       </c>
       <c r="G12" s="14" t="n">
         <v>0</v>
@@ -1171,13 +1171,13 @@
         <v>39460</v>
       </c>
       <c r="E14" s="14" t="n">
-        <v>32828</v>
+        <v>32728</v>
       </c>
       <c r="F14" s="14" t="n">
         <v>0</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>32828</v>
+        <v>32728</v>
       </c>
       <c r="H14" s="14">
         <f>MAX(0, D14-E14)</f>
@@ -1205,10 +1205,10 @@
         <v>17340</v>
       </c>
       <c r="E15" s="18" t="n">
-        <v>7660</v>
+        <v>7860</v>
       </c>
       <c r="F15" s="18" t="n">
-        <v>7660</v>
+        <v>7860</v>
       </c>
       <c r="G15" s="18" t="n">
         <v>0</v>
@@ -1233,19 +1233,19 @@
         </is>
       </c>
       <c r="C16" s="13" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D16" s="14" t="n">
         <v>46000</v>
       </c>
       <c r="E16" s="14" t="n">
-        <v>31850</v>
+        <v>44724</v>
       </c>
       <c r="F16" s="14" t="n">
         <v>23050</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>8800</v>
+        <v>21674</v>
       </c>
       <c r="H16" s="14">
         <f>MAX(0, D16-E16)</f>
@@ -1323,7 +1323,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:L36"/>
+  <dimension ref="B2:L38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1350,7 +1350,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 28/09/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 29/09/2026</t>
         </is>
       </c>
     </row>
@@ -1395,13 +1395,13 @@
       <c r="C6" s="4" t="n"/>
       <c r="D6" s="25" t="inlineStr">
         <is>
-          <t>11,410 u</t>
+          <t>11,710 u</t>
         </is>
       </c>
       <c r="E6" s="4" t="n"/>
       <c r="F6" s="25" t="inlineStr">
         <is>
-          <t>491.8%</t>
+          <t>504.7%</t>
         </is>
       </c>
       <c r="G6" s="4" t="n"/>
@@ -1577,27 +1577,27 @@
     <row r="12">
       <c r="B12" s="27" t="inlineStr">
         <is>
-          <t>AGROTÉCNICA DEL NORTE, S.L</t>
+          <t>AGRICOLA DEL JUCAR DE CUENCA, S.L.</t>
         </is>
       </c>
       <c r="C12" s="28" t="inlineStr">
         <is>
-          <t>A-50(2)0005</t>
+          <t>C-CU0020</t>
         </is>
       </c>
       <c r="D12" s="27" t="inlineStr">
         <is>
-          <t>CODIORGAN-A50, 5 KG</t>
+          <t>CODICOBRE, 20 L</t>
         </is>
       </c>
       <c r="E12" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F12" s="14" t="n">
-        <v>500</v>
+        <v>100</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>500</v>
+        <v>100</v>
       </c>
       <c r="H12" s="14" t="n">
         <v>0</v>
@@ -1623,27 +1623,27 @@
     <row r="13">
       <c r="B13" s="30" t="inlineStr">
         <is>
-          <t>AGROTÉCNICA DEL NORTE, S.L</t>
+          <t>AGRICOLA DEL JUCAR DE CUENCA, S.L.</t>
         </is>
       </c>
       <c r="C13" s="31" t="inlineStr">
         <is>
-          <t>AGRMG0005</t>
+          <t>C-L0020</t>
         </is>
       </c>
       <c r="D13" s="30" t="inlineStr">
         <is>
-          <t>AGROXIGREEN-MG, 5 L</t>
+          <t>CODIBOR-L, 20 L</t>
         </is>
       </c>
       <c r="E13" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F13" s="18" t="n">
-        <v>300</v>
+        <v>200</v>
       </c>
       <c r="G13" s="18" t="n">
-        <v>300</v>
+        <v>200</v>
       </c>
       <c r="H13" s="18" t="n">
         <v>0</v>
@@ -1674,22 +1674,22 @@
       </c>
       <c r="C14" s="28" t="inlineStr">
         <is>
-          <t>PT0005</t>
+          <t>A-50(2)0005</t>
         </is>
       </c>
       <c r="D14" s="27" t="inlineStr">
         <is>
-          <t>AGROPOTASION, 5 L</t>
+          <t>CODIORGAN-A50, 5 KG</t>
         </is>
       </c>
       <c r="E14" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F14" s="14" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="H14" s="14" t="n">
         <v>0</v>
@@ -1715,27 +1715,27 @@
     <row r="15">
       <c r="B15" s="30" t="inlineStr">
         <is>
-          <t>AGROVEYCA,S.L</t>
+          <t>AGROTÉCNICA DEL NORTE, S.L</t>
         </is>
       </c>
       <c r="C15" s="31" t="inlineStr">
         <is>
-          <t>A-50(2)0005</t>
+          <t>AGRMG0005</t>
         </is>
       </c>
       <c r="D15" s="30" t="inlineStr">
         <is>
-          <t>CODIORGAN-A50, 5 KG</t>
+          <t>AGROXIGREEN-MG, 5 L</t>
         </is>
       </c>
       <c r="E15" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F15" s="18" t="n">
-        <v>400</v>
+        <v>300</v>
       </c>
       <c r="G15" s="18" t="n">
-        <v>400</v>
+        <v>300</v>
       </c>
       <c r="H15" s="18" t="n">
         <v>0</v>
@@ -1761,27 +1761,27 @@
     <row r="16">
       <c r="B16" s="27" t="inlineStr">
         <is>
-          <t>AGROVEYCA,S.L</t>
+          <t>AGROTÉCNICA DEL NORTE, S.L</t>
         </is>
       </c>
       <c r="C16" s="28" t="inlineStr">
         <is>
-          <t>BIO0020</t>
+          <t>PT0005</t>
         </is>
       </c>
       <c r="D16" s="27" t="inlineStr">
         <is>
-          <t>BIORAD-20, 20 L</t>
+          <t>AGROPOTASION, 5 L</t>
         </is>
       </c>
       <c r="E16" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="14" t="n">
         <v>400</v>
       </c>
-      <c r="F16" s="14" t="n">
-        <v>320</v>
-      </c>
       <c r="G16" s="14" t="n">
-        <v>320</v>
+        <v>400</v>
       </c>
       <c r="H16" s="14" t="n">
         <v>0</v>
@@ -1798,16 +1798,16 @@
         <f>IF(E16&gt;0, F16/E16, IF(F16&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L16" s="32" t="inlineStr">
-        <is>
-          <t>En Curso</t>
+      <c r="L16" s="29" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="30" t="inlineStr">
         <is>
-          <t>ASOC. HORTICULTORES DE VILLA DEL PRADO</t>
+          <t>AGROVEYCA,S.L</t>
         </is>
       </c>
       <c r="C17" s="31" t="inlineStr">
@@ -1817,17 +1817,17 @@
       </c>
       <c r="D17" s="30" t="inlineStr">
         <is>
-          <t>CODIORGAN A-50, 5 KG</t>
+          <t>CODIORGAN-A50, 5 KG</t>
         </is>
       </c>
       <c r="E17" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F17" s="18" t="n">
-        <v>50</v>
+        <v>400</v>
       </c>
       <c r="G17" s="18" t="n">
-        <v>50</v>
+        <v>400</v>
       </c>
       <c r="H17" s="18" t="n">
         <v>0</v>
@@ -1853,27 +1853,27 @@
     <row r="18">
       <c r="B18" s="27" t="inlineStr">
         <is>
-          <t>ASOC. HORTICULTORES DE VILLA DEL PRADO</t>
+          <t>AGROVEYCA,S.L</t>
         </is>
       </c>
       <c r="C18" s="28" t="inlineStr">
         <is>
-          <t>AVAN0005</t>
+          <t>BIO0020</t>
         </is>
       </c>
       <c r="D18" s="27" t="inlineStr">
         <is>
-          <t>FLORAMEC AVANCE, 5 L</t>
+          <t>BIORAD-20, 20 L</t>
         </is>
       </c>
       <c r="E18" s="14" t="n">
-        <v>0</v>
+        <v>400</v>
       </c>
       <c r="F18" s="14" t="n">
-        <v>100</v>
+        <v>320</v>
       </c>
       <c r="G18" s="14" t="n">
-        <v>100</v>
+        <v>320</v>
       </c>
       <c r="H18" s="14" t="n">
         <v>0</v>
@@ -1890,9 +1890,9 @@
         <f>IF(E18&gt;0, F18/E18, IF(F18&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L18" s="29" t="inlineStr">
-        <is>
-          <t>Extra Estimación</t>
+      <c r="L18" s="32" t="inlineStr">
+        <is>
+          <t>En Curso</t>
         </is>
       </c>
     </row>
@@ -1904,22 +1904,22 @@
       </c>
       <c r="C19" s="31" t="inlineStr">
         <is>
-          <t>C-CU0005</t>
+          <t>A-50(2)0005</t>
         </is>
       </c>
       <c r="D19" s="30" t="inlineStr">
         <is>
-          <t>CODICOBRE, 5 L</t>
+          <t>CODIORGAN A-50, 5 KG</t>
         </is>
       </c>
       <c r="E19" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F19" s="18" t="n">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="G19" s="18" t="n">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="H19" s="18" t="n">
         <v>0</v>
@@ -1950,22 +1950,22 @@
       </c>
       <c r="C20" s="28" t="inlineStr">
         <is>
-          <t>S0020</t>
+          <t>AVAN0005</t>
         </is>
       </c>
       <c r="D20" s="27" t="inlineStr">
         <is>
-          <t>SALWAX STAR, 20 L</t>
+          <t>FLORAMEC AVANCE, 5 L</t>
         </is>
       </c>
       <c r="E20" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F20" s="14" t="n">
-        <v>40</v>
+        <v>100</v>
       </c>
       <c r="G20" s="14" t="n">
-        <v>40</v>
+        <v>100</v>
       </c>
       <c r="H20" s="14" t="n">
         <v>0</v>
@@ -1991,27 +1991,27 @@
     <row r="21">
       <c r="B21" s="30" t="inlineStr">
         <is>
-          <t>BARDENAS COMERCIAL, S.L.</t>
+          <t>ASOC. HORTICULTORES DE VILLA DEL PRADO</t>
         </is>
       </c>
       <c r="C21" s="31" t="inlineStr">
         <is>
-          <t>AGRMG0005</t>
+          <t>C-CU0005</t>
         </is>
       </c>
       <c r="D21" s="30" t="inlineStr">
         <is>
-          <t>AGROXIGREEN-MG, 5 L</t>
+          <t>CODICOBRE, 5 L</t>
         </is>
       </c>
       <c r="E21" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F21" s="18" t="n">
-        <v>300</v>
+        <v>20</v>
       </c>
       <c r="G21" s="18" t="n">
-        <v>300</v>
+        <v>20</v>
       </c>
       <c r="H21" s="18" t="n">
         <v>0</v>
@@ -2037,27 +2037,27 @@
     <row r="22">
       <c r="B22" s="27" t="inlineStr">
         <is>
-          <t>BARDENAS COMERCIAL, S.L.</t>
+          <t>ASOC. HORTICULTORES DE VILLA DEL PRADO</t>
         </is>
       </c>
       <c r="C22" s="28" t="inlineStr">
         <is>
-          <t>PT0005</t>
+          <t>S0020</t>
         </is>
       </c>
       <c r="D22" s="27" t="inlineStr">
         <is>
-          <t>AGROPOTASION, 5 L</t>
+          <t>SALWAX STAR, 20 L</t>
         </is>
       </c>
       <c r="E22" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F22" s="14" t="n">
-        <v>300</v>
+        <v>40</v>
       </c>
       <c r="G22" s="14" t="n">
-        <v>300</v>
+        <v>40</v>
       </c>
       <c r="H22" s="14" t="n">
         <v>0</v>
@@ -2083,27 +2083,27 @@
     <row r="23">
       <c r="B23" s="30" t="inlineStr">
         <is>
-          <t>COMERCIAL NORTE AGROCAMPO, S.L.</t>
+          <t>BARDENAS COMERCIAL, S.L.</t>
         </is>
       </c>
       <c r="C23" s="31" t="inlineStr">
         <is>
-          <t>A-50(2)0020</t>
+          <t>AGRMG0005</t>
         </is>
       </c>
       <c r="D23" s="30" t="inlineStr">
         <is>
-          <t>CODIORGAN-A50, 20 KG</t>
+          <t>AGROXIGREEN-MG, 5 L</t>
         </is>
       </c>
       <c r="E23" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F23" s="18" t="n">
-        <v>40</v>
+        <v>300</v>
       </c>
       <c r="G23" s="18" t="n">
-        <v>40</v>
+        <v>300</v>
       </c>
       <c r="H23" s="18" t="n">
         <v>0</v>
@@ -2129,27 +2129,27 @@
     <row r="24">
       <c r="B24" s="27" t="inlineStr">
         <is>
-          <t>COMERCIAL NORTE AGROCAMPO, S.L.</t>
+          <t>BARDENAS COMERCIAL, S.L.</t>
         </is>
       </c>
       <c r="C24" s="28" t="inlineStr">
         <is>
-          <t>AN0005</t>
+          <t>PT0005</t>
         </is>
       </c>
       <c r="D24" s="27" t="inlineStr">
         <is>
-          <t>ALCAPLANT NEW, 5 KG</t>
+          <t>AGROPOTASION, 5 L</t>
         </is>
       </c>
       <c r="E24" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F24" s="14" t="n">
-        <v>20</v>
+        <v>300</v>
       </c>
       <c r="G24" s="14" t="n">
-        <v>20</v>
+        <v>300</v>
       </c>
       <c r="H24" s="14" t="n">
         <v>0</v>
@@ -2180,22 +2180,22 @@
       </c>
       <c r="C25" s="31" t="inlineStr">
         <is>
-          <t>BR-590005</t>
+          <t>A-50(2)0020</t>
         </is>
       </c>
       <c r="D25" s="30" t="inlineStr">
         <is>
-          <t>BR-59, 5 KG</t>
+          <t>CODIORGAN-A50, 20 KG</t>
         </is>
       </c>
       <c r="E25" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F25" s="18" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="G25" s="18" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="H25" s="18" t="n">
         <v>0</v>
@@ -2226,12 +2226,12 @@
       </c>
       <c r="C26" s="28" t="inlineStr">
         <is>
-          <t>BROTA0020</t>
+          <t>AN0005</t>
         </is>
       </c>
       <c r="D26" s="27" t="inlineStr">
         <is>
-          <t>BROTAMEC, 20 L</t>
+          <t>ALCAPLANT NEW, 5 KG</t>
         </is>
       </c>
       <c r="E26" s="14" t="n">
@@ -2272,22 +2272,22 @@
       </c>
       <c r="C27" s="31" t="inlineStr">
         <is>
-          <t>C-CU0005</t>
+          <t>BR-590005</t>
         </is>
       </c>
       <c r="D27" s="30" t="inlineStr">
         <is>
-          <t>CODICOBRE, 5 L</t>
+          <t>BR-59, 5 KG</t>
         </is>
       </c>
       <c r="E27" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F27" s="18" t="n">
-        <v>20</v>
+        <v>60</v>
       </c>
       <c r="G27" s="18" t="n">
-        <v>20</v>
+        <v>60</v>
       </c>
       <c r="H27" s="18" t="n">
         <v>0</v>
@@ -2318,12 +2318,12 @@
       </c>
       <c r="C28" s="28" t="inlineStr">
         <is>
-          <t>PT0020</t>
+          <t>BROTA0020</t>
         </is>
       </c>
       <c r="D28" s="27" t="inlineStr">
         <is>
-          <t>AGROPOTASION, 20 L</t>
+          <t>BROTAMEC, 20 L</t>
         </is>
       </c>
       <c r="E28" s="14" t="n">
@@ -2364,22 +2364,22 @@
       </c>
       <c r="C29" s="31" t="inlineStr">
         <is>
-          <t>S0020</t>
+          <t>C-CU0005</t>
         </is>
       </c>
       <c r="D29" s="30" t="inlineStr">
         <is>
-          <t>SALWAX STAR, 20 L</t>
+          <t>CODICOBRE, 5 L</t>
         </is>
       </c>
       <c r="E29" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F29" s="18" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="G29" s="18" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="H29" s="18" t="n">
         <v>0</v>
@@ -2405,17 +2405,17 @@
     <row r="30">
       <c r="B30" s="27" t="inlineStr">
         <is>
-          <t>MAJ AGROQUIMICOS S.L.</t>
+          <t>COMERCIAL NORTE AGROCAMPO, S.L.</t>
         </is>
       </c>
       <c r="C30" s="28" t="inlineStr">
         <is>
-          <t>CPLUS0005</t>
+          <t>PT0020</t>
         </is>
       </c>
       <c r="D30" s="27" t="inlineStr">
         <is>
-          <t>CALCIPLUS, 5 L</t>
+          <t>AGROPOTASION, 20 L</t>
         </is>
       </c>
       <c r="E30" s="14" t="n">
@@ -2451,17 +2451,17 @@
     <row r="31">
       <c r="B31" s="30" t="inlineStr">
         <is>
-          <t>MAJ AGROQUIMICOS S.L.</t>
+          <t>COMERCIAL NORTE AGROCAMPO, S.L.</t>
         </is>
       </c>
       <c r="C31" s="31" t="inlineStr">
         <is>
-          <t>FTK0005</t>
+          <t>S0020</t>
         </is>
       </c>
       <c r="D31" s="30" t="inlineStr">
         <is>
-          <t>FITOKONTROL CA FLOW, 5 KG</t>
+          <t>SALWAX STAR, 20 L</t>
         </is>
       </c>
       <c r="E31" s="18" t="n">
@@ -2497,27 +2497,27 @@
     <row r="32">
       <c r="B32" s="27" t="inlineStr">
         <is>
-          <t>SAFIAGRO, S.A.</t>
+          <t>MAJ AGROQUIMICOS S.L.</t>
         </is>
       </c>
       <c r="C32" s="28" t="inlineStr">
         <is>
-          <t>AGXK0020</t>
+          <t>CPLUS0005</t>
         </is>
       </c>
       <c r="D32" s="27" t="inlineStr">
         <is>
-          <t>AGROXILATO-K, 20 L</t>
+          <t>CALCIPLUS, 5 L</t>
         </is>
       </c>
       <c r="E32" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F32" s="14" t="n">
-        <v>640</v>
+        <v>20</v>
       </c>
       <c r="G32" s="14" t="n">
-        <v>640</v>
+        <v>20</v>
       </c>
       <c r="H32" s="14" t="n">
         <v>0</v>
@@ -2543,27 +2543,27 @@
     <row r="33">
       <c r="B33" s="30" t="inlineStr">
         <is>
-          <t>T.J AGRICULTURA S.L.</t>
+          <t>MAJ AGROQUIMICOS S.L.</t>
         </is>
       </c>
       <c r="C33" s="31" t="inlineStr">
         <is>
-          <t>AN0020</t>
+          <t>FTK0005</t>
         </is>
       </c>
       <c r="D33" s="30" t="inlineStr">
         <is>
-          <t>ALCAPLANT NEW, 20 KG</t>
+          <t>FITOKONTROL CA FLOW, 5 KG</t>
         </is>
       </c>
       <c r="E33" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F33" s="18" t="n">
-        <v>600</v>
+        <v>40</v>
       </c>
       <c r="G33" s="18" t="n">
-        <v>600</v>
+        <v>40</v>
       </c>
       <c r="H33" s="18" t="n">
         <v>0</v>
@@ -2589,27 +2589,27 @@
     <row r="34">
       <c r="B34" s="27" t="inlineStr">
         <is>
-          <t>T.J AGRICULTURA S.L.</t>
+          <t>SAFIAGRO, S.A.</t>
         </is>
       </c>
       <c r="C34" s="28" t="inlineStr">
         <is>
-          <t>SS0020</t>
+          <t>AGXK0020</t>
         </is>
       </c>
       <c r="D34" s="27" t="inlineStr">
         <is>
-          <t>SALWAX-CA, 20 KG</t>
+          <t>AGROXILATO-K, 20 L</t>
         </is>
       </c>
       <c r="E34" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F34" s="14" t="n">
-        <v>500</v>
+        <v>640</v>
       </c>
       <c r="G34" s="14" t="n">
-        <v>500</v>
+        <v>640</v>
       </c>
       <c r="H34" s="14" t="n">
         <v>0</v>
@@ -2635,27 +2635,27 @@
     <row r="35">
       <c r="B35" s="30" t="inlineStr">
         <is>
-          <t>VILLALTA SATIVUM, S.L.</t>
+          <t>T.J AGRICULTURA S.L.</t>
         </is>
       </c>
       <c r="C35" s="31" t="inlineStr">
         <is>
-          <t>WHITE0020</t>
+          <t>AN0020</t>
         </is>
       </c>
       <c r="D35" s="30" t="inlineStr">
         <is>
-          <t>AGROWHITE, 20 KG</t>
+          <t>ALCAPLANT NEW, 20 KG</t>
         </is>
       </c>
       <c r="E35" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F35" s="18" t="n">
-        <v>3460</v>
+        <v>600</v>
       </c>
       <c r="G35" s="18" t="n">
-        <v>3460</v>
+        <v>600</v>
       </c>
       <c r="H35" s="18" t="n">
         <v>0</v>
@@ -2678,48 +2678,140 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="24" customHeight="1">
-      <c r="B36" s="20" t="inlineStr">
+    <row r="36">
+      <c r="B36" s="27" t="inlineStr">
+        <is>
+          <t>T.J AGRICULTURA S.L.</t>
+        </is>
+      </c>
+      <c r="C36" s="28" t="inlineStr">
+        <is>
+          <t>SS0020</t>
+        </is>
+      </c>
+      <c r="D36" s="27" t="inlineStr">
+        <is>
+          <t>SALWAX-CA, 20 KG</t>
+        </is>
+      </c>
+      <c r="E36" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F36" s="14" t="n">
+        <v>500</v>
+      </c>
+      <c r="G36" s="14" t="n">
+        <v>500</v>
+      </c>
+      <c r="H36" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I36" s="14">
+        <f>MAX(0, E36-F36)</f>
+        <v/>
+      </c>
+      <c r="J36" s="14">
+        <f>F36-E36</f>
+        <v/>
+      </c>
+      <c r="K36" s="15">
+        <f>IF(E36&gt;0, F36/E36, IF(F36&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L36" s="29" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" s="30" t="inlineStr">
+        <is>
+          <t>VILLALTA SATIVUM, S.L.</t>
+        </is>
+      </c>
+      <c r="C37" s="31" t="inlineStr">
+        <is>
+          <t>WHITE0020</t>
+        </is>
+      </c>
+      <c r="D37" s="30" t="inlineStr">
+        <is>
+          <t>AGROWHITE, 20 KG</t>
+        </is>
+      </c>
+      <c r="E37" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F37" s="18" t="n">
+        <v>3460</v>
+      </c>
+      <c r="G37" s="18" t="n">
+        <v>3460</v>
+      </c>
+      <c r="H37" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="I37" s="18">
+        <f>MAX(0, E37-F37)</f>
+        <v/>
+      </c>
+      <c r="J37" s="18">
+        <f>F37-E37</f>
+        <v/>
+      </c>
+      <c r="K37" s="19">
+        <f>IF(E37&gt;0, F37/E37, IF(F37&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L37" s="29" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="24" customHeight="1">
+      <c r="B38" s="20" t="inlineStr">
         <is>
           <t>TOTAL ALFONSO</t>
         </is>
       </c>
-      <c r="C36" s="33" t="inlineStr">
+      <c r="C38" s="33" t="inlineStr">
         <is>
           <t>280 líneas</t>
         </is>
       </c>
-      <c r="D36" s="34" t="inlineStr"/>
-      <c r="E36" s="22">
-        <f>SUM(E10:E35)</f>
-        <v/>
-      </c>
-      <c r="F36" s="22">
-        <f>SUM(F10:F35)</f>
-        <v/>
-      </c>
-      <c r="G36" s="22">
-        <f>SUM(G10:G35)</f>
-        <v/>
-      </c>
-      <c r="H36" s="22">
-        <f>SUM(H10:H35)</f>
-        <v/>
-      </c>
-      <c r="I36" s="22">
-        <f>SUM(I10:I35)</f>
-        <v/>
-      </c>
-      <c r="J36" s="22">
-        <f>SUM(J10:J35)</f>
-        <v/>
-      </c>
-      <c r="K36" s="23">
-        <f>IF(E36&gt;0, F36/E36, 0)</f>
-        <v/>
-      </c>
-      <c r="L36" s="21">
-        <f>IF(K36&gt;=1, "SUPERADO", "EN CURSO")</f>
+      <c r="D38" s="34" t="inlineStr"/>
+      <c r="E38" s="22">
+        <f>SUM(E10:E37)</f>
+        <v/>
+      </c>
+      <c r="F38" s="22">
+        <f>SUM(F10:F37)</f>
+        <v/>
+      </c>
+      <c r="G38" s="22">
+        <f>SUM(G10:G37)</f>
+        <v/>
+      </c>
+      <c r="H38" s="22">
+        <f>SUM(H10:H37)</f>
+        <v/>
+      </c>
+      <c r="I38" s="22">
+        <f>SUM(I10:I37)</f>
+        <v/>
+      </c>
+      <c r="J38" s="22">
+        <f>SUM(J10:J37)</f>
+        <v/>
+      </c>
+      <c r="K38" s="23">
+        <f>IF(E38&gt;0, F38/E38, 0)</f>
+        <v/>
+      </c>
+      <c r="L38" s="21">
+        <f>IF(K38&gt;=1, "SUPERADO", "EN CURSO")</f>
         <v/>
       </c>
     </row>
@@ -2775,7 +2867,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 28/09/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 29/09/2026</t>
         </is>
       </c>
     </row>
@@ -2820,13 +2912,13 @@
       <c r="C6" s="4" t="n"/>
       <c r="D6" s="25" t="inlineStr">
         <is>
-          <t>55,612 u</t>
+          <t>56,212 u</t>
         </is>
       </c>
       <c r="E6" s="4" t="n"/>
       <c r="F6" s="25" t="inlineStr">
         <is>
-          <t>147.0%</t>
+          <t>148.6%</t>
         </is>
       </c>
       <c r="G6" s="4" t="n"/>
@@ -3433,10 +3525,10 @@
         <v>100</v>
       </c>
       <c r="F21" s="18" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="G21" s="18" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="H21" s="18" t="n">
         <v>0</v>
@@ -3453,9 +3545,9 @@
         <f>IF(E21&gt;0, F21/E21, IF(F21&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L21" s="35" t="inlineStr">
-        <is>
-          <t>Sin Pedido</t>
+      <c r="L21" s="29" t="inlineStr">
+        <is>
+          <t>Superado</t>
         </is>
       </c>
     </row>
@@ -3479,10 +3571,10 @@
         <v>300</v>
       </c>
       <c r="F22" s="14" t="n">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="G22" s="14" t="n">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="H22" s="14" t="n">
         <v>0</v>
@@ -3499,9 +3591,9 @@
         <f>IF(E22&gt;0, F22/E22, IF(F22&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L22" s="35" t="inlineStr">
-        <is>
-          <t>Sin Pedido</t>
+      <c r="L22" s="29" t="inlineStr">
+        <is>
+          <t>Superado</t>
         </is>
       </c>
     </row>
@@ -3525,10 +3617,10 @@
         <v>200</v>
       </c>
       <c r="F23" s="18" t="n">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="G23" s="18" t="n">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="H23" s="18" t="n">
         <v>0</v>
@@ -3545,9 +3637,9 @@
         <f>IF(E23&gt;0, F23/E23, IF(F23&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L23" s="35" t="inlineStr">
-        <is>
-          <t>Sin Pedido</t>
+      <c r="L23" s="29" t="inlineStr">
+        <is>
+          <t>Superado</t>
         </is>
       </c>
     </row>
@@ -5093,7 +5185,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:L44"/>
+  <dimension ref="B2:L45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -5120,7 +5212,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 28/09/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 29/09/2026</t>
         </is>
       </c>
     </row>
@@ -5165,19 +5257,19 @@
       <c r="C6" s="4" t="n"/>
       <c r="D6" s="24" t="inlineStr">
         <is>
-          <t>12,806 u</t>
+          <t>14,826 u</t>
         </is>
       </c>
       <c r="E6" s="4" t="n"/>
       <c r="F6" s="37" t="inlineStr">
         <is>
-          <t>58.4%</t>
+          <t>67.7%</t>
         </is>
       </c>
       <c r="G6" s="4" t="n"/>
       <c r="H6" s="37" t="inlineStr">
         <is>
-          <t>9,108 u</t>
+          <t>7,088 u</t>
         </is>
       </c>
       <c r="I6" s="4" t="n"/>
@@ -5272,10 +5364,10 @@
         <v>200</v>
       </c>
       <c r="F10" s="14" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="H10" s="14" t="n">
         <v>0</v>
@@ -5292,9 +5384,9 @@
         <f>IF(E10&gt;0, F10/E10, IF(F10&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L10" s="35" t="inlineStr">
-        <is>
-          <t>Sin Pedido</t>
+      <c r="L10" s="32" t="inlineStr">
+        <is>
+          <t>En Curso</t>
         </is>
       </c>
     </row>
@@ -5364,10 +5456,10 @@
         <v>1920</v>
       </c>
       <c r="F12" s="14" t="n">
-        <v>0</v>
+        <v>640</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>0</v>
+        <v>640</v>
       </c>
       <c r="H12" s="14" t="n">
         <v>0</v>
@@ -5384,9 +5476,9 @@
         <f>IF(E12&gt;0, F12/E12, IF(F12&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L12" s="35" t="inlineStr">
-        <is>
-          <t>Sin Pedido</t>
+      <c r="L12" s="36" t="inlineStr">
+        <is>
+          <t>Rezagado</t>
         </is>
       </c>
     </row>
@@ -5870,10 +5962,10 @@
         <v>3200</v>
       </c>
       <c r="F23" s="18" t="n">
-        <v>0</v>
+        <v>640</v>
       </c>
       <c r="G23" s="18" t="n">
-        <v>0</v>
+        <v>640</v>
       </c>
       <c r="H23" s="18" t="n">
         <v>0</v>
@@ -5890,9 +5982,9 @@
         <f>IF(E23&gt;0, F23/E23, IF(F23&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L23" s="35" t="inlineStr">
-        <is>
-          <t>Sin Pedido</t>
+      <c r="L23" s="36" t="inlineStr">
+        <is>
+          <t>Rezagado</t>
         </is>
       </c>
     </row>
@@ -6778,22 +6870,22 @@
       </c>
       <c r="C43" s="31" t="inlineStr">
         <is>
-          <t>AVAN0020</t>
+          <t>AGXK0020</t>
         </is>
       </c>
       <c r="D43" s="30" t="inlineStr">
         <is>
-          <t>FLORAMEC AVANCE, 20 L</t>
+          <t>AGROXILATO-K, 20 L</t>
         </is>
       </c>
       <c r="E43" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F43" s="18" t="n">
-        <v>200</v>
+        <v>640</v>
       </c>
       <c r="G43" s="18" t="n">
-        <v>200</v>
+        <v>640</v>
       </c>
       <c r="H43" s="18" t="n">
         <v>0</v>
@@ -6816,48 +6908,94 @@
         </is>
       </c>
     </row>
-    <row r="44" ht="24" customHeight="1">
-      <c r="B44" s="20" t="inlineStr">
+    <row r="44">
+      <c r="B44" s="27" t="inlineStr">
+        <is>
+          <t>SUCA, S.C.A.</t>
+        </is>
+      </c>
+      <c r="C44" s="28" t="inlineStr">
+        <is>
+          <t>AVAN0020</t>
+        </is>
+      </c>
+      <c r="D44" s="27" t="inlineStr">
+        <is>
+          <t>FLORAMEC AVANCE, 20 L</t>
+        </is>
+      </c>
+      <c r="E44" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F44" s="14" t="n">
+        <v>200</v>
+      </c>
+      <c r="G44" s="14" t="n">
+        <v>200</v>
+      </c>
+      <c r="H44" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I44" s="14">
+        <f>MAX(0, E44-F44)</f>
+        <v/>
+      </c>
+      <c r="J44" s="14">
+        <f>F44-E44</f>
+        <v/>
+      </c>
+      <c r="K44" s="15">
+        <f>IF(E44&gt;0, F44/E44, IF(F44&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L44" s="29" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="24" customHeight="1">
+      <c r="B45" s="20" t="inlineStr">
         <is>
           <t>TOTAL IRENE</t>
         </is>
       </c>
-      <c r="C44" s="33" t="inlineStr">
+      <c r="C45" s="33" t="inlineStr">
         <is>
           <t>89 líneas</t>
         </is>
       </c>
-      <c r="D44" s="34" t="inlineStr"/>
-      <c r="E44" s="22">
-        <f>SUM(E10:E43)</f>
-        <v/>
-      </c>
-      <c r="F44" s="22">
-        <f>SUM(F10:F43)</f>
-        <v/>
-      </c>
-      <c r="G44" s="22">
-        <f>SUM(G10:G43)</f>
-        <v/>
-      </c>
-      <c r="H44" s="22">
-        <f>SUM(H10:H43)</f>
-        <v/>
-      </c>
-      <c r="I44" s="22">
-        <f>SUM(I10:I43)</f>
-        <v/>
-      </c>
-      <c r="J44" s="22">
-        <f>SUM(J10:J43)</f>
-        <v/>
-      </c>
-      <c r="K44" s="23">
-        <f>IF(E44&gt;0, F44/E44, 0)</f>
-        <v/>
-      </c>
-      <c r="L44" s="21">
-        <f>IF(K44&gt;=1, "SUPERADO", "EN CURSO")</f>
+      <c r="D45" s="34" t="inlineStr"/>
+      <c r="E45" s="22">
+        <f>SUM(E10:E44)</f>
+        <v/>
+      </c>
+      <c r="F45" s="22">
+        <f>SUM(F10:F44)</f>
+        <v/>
+      </c>
+      <c r="G45" s="22">
+        <f>SUM(G10:G44)</f>
+        <v/>
+      </c>
+      <c r="H45" s="22">
+        <f>SUM(H10:H44)</f>
+        <v/>
+      </c>
+      <c r="I45" s="22">
+        <f>SUM(I10:I44)</f>
+        <v/>
+      </c>
+      <c r="J45" s="22">
+        <f>SUM(J10:J44)</f>
+        <v/>
+      </c>
+      <c r="K45" s="23">
+        <f>IF(E45&gt;0, F45/E45, 0)</f>
+        <v/>
+      </c>
+      <c r="L45" s="21">
+        <f>IF(K45&gt;=1, "SUPERADO", "EN CURSO")</f>
         <v/>
       </c>
     </row>
@@ -6913,7 +7051,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 28/09/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 29/09/2026</t>
         </is>
       </c>
     </row>
@@ -8909,7 +9047,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:L16"/>
+  <dimension ref="B2:L17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -8936,7 +9074,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 28/09/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 29/09/2026</t>
         </is>
       </c>
     </row>
@@ -8981,25 +9119,25 @@
       <c r="C6" s="4" t="n"/>
       <c r="D6" s="24" t="inlineStr">
         <is>
-          <t>32,828 u</t>
+          <t>32,728 u</t>
         </is>
       </c>
       <c r="E6" s="4" t="n"/>
       <c r="F6" s="37" t="inlineStr">
         <is>
-          <t>83.2%</t>
+          <t>82.9%</t>
         </is>
       </c>
       <c r="G6" s="4" t="n"/>
       <c r="H6" s="37" t="inlineStr">
         <is>
-          <t>6,632 u</t>
+          <t>6,732 u</t>
         </is>
       </c>
       <c r="I6" s="4" t="n"/>
       <c r="J6" s="24" t="inlineStr">
         <is>
-          <t>32,828 u</t>
+          <t>32,728 u</t>
         </is>
       </c>
       <c r="K6" s="4" t="n"/>
@@ -9088,13 +9226,13 @@
         <v>5500</v>
       </c>
       <c r="F10" s="14" t="n">
-        <v>3300</v>
+        <v>2200</v>
       </c>
       <c r="G10" s="14" t="n">
         <v>0</v>
       </c>
       <c r="H10" s="14" t="n">
-        <v>3300</v>
+        <v>2200</v>
       </c>
       <c r="I10" s="14">
         <f>MAX(0, E10-F10)</f>
@@ -9108,9 +9246,9 @@
         <f>IF(E10&gt;0, F10/E10, IF(F10&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L10" s="32" t="inlineStr">
-        <is>
-          <t>En Curso</t>
+      <c r="L10" s="36" t="inlineStr">
+        <is>
+          <t>Rezagado</t>
         </is>
       </c>
     </row>
@@ -9306,25 +9444,25 @@
       </c>
       <c r="C15" s="31" t="inlineStr">
         <is>
-          <t>RUN0001</t>
+          <t>FU1000</t>
         </is>
       </c>
       <c r="D15" s="30" t="inlineStr">
         <is>
-          <t>RUN STRESS, 1 L</t>
+          <t>FULVIGIN, 1000 L</t>
         </is>
       </c>
       <c r="E15" s="18" t="n">
-        <v>1960</v>
+        <v>0</v>
       </c>
       <c r="F15" s="18" t="n">
-        <v>1968</v>
+        <v>1000</v>
       </c>
       <c r="G15" s="18" t="n">
         <v>0</v>
       </c>
       <c r="H15" s="18" t="n">
-        <v>1968</v>
+        <v>1000</v>
       </c>
       <c r="I15" s="18">
         <f>MAX(0, E15-F15)</f>
@@ -9340,52 +9478,98 @@
       </c>
       <c r="L15" s="29" t="inlineStr">
         <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="27" t="inlineStr">
+        <is>
+          <t>ÇITAR ÇIÇEK TARIM TIC. LTD. STI</t>
+        </is>
+      </c>
+      <c r="C16" s="28" t="inlineStr">
+        <is>
+          <t>RUN0001</t>
+        </is>
+      </c>
+      <c r="D16" s="27" t="inlineStr">
+        <is>
+          <t>RUN STRESS, 1 L</t>
+        </is>
+      </c>
+      <c r="E16" s="14" t="n">
+        <v>1960</v>
+      </c>
+      <c r="F16" s="14" t="n">
+        <v>1968</v>
+      </c>
+      <c r="G16" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="14" t="n">
+        <v>1968</v>
+      </c>
+      <c r="I16" s="14">
+        <f>MAX(0, E16-F16)</f>
+        <v/>
+      </c>
+      <c r="J16" s="14">
+        <f>F16-E16</f>
+        <v/>
+      </c>
+      <c r="K16" s="15">
+        <f>IF(E16&gt;0, F16/E16, IF(F16&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L16" s="29" t="inlineStr">
+        <is>
           <t>Superado</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="24" customHeight="1">
-      <c r="B16" s="20" t="inlineStr">
+    <row r="17" ht="24" customHeight="1">
+      <c r="B17" s="20" t="inlineStr">
         <is>
           <t>TOTAL MEHMET</t>
         </is>
       </c>
-      <c r="C16" s="33" t="inlineStr">
+      <c r="C17" s="33" t="inlineStr">
         <is>
           <t>61 líneas</t>
         </is>
       </c>
-      <c r="D16" s="34" t="inlineStr"/>
-      <c r="E16" s="22">
-        <f>SUM(E10:E15)</f>
-        <v/>
-      </c>
-      <c r="F16" s="22">
-        <f>SUM(F10:F15)</f>
-        <v/>
-      </c>
-      <c r="G16" s="22">
-        <f>SUM(G10:G15)</f>
-        <v/>
-      </c>
-      <c r="H16" s="22">
-        <f>SUM(H10:H15)</f>
-        <v/>
-      </c>
-      <c r="I16" s="22">
-        <f>SUM(I10:I15)</f>
-        <v/>
-      </c>
-      <c r="J16" s="22">
-        <f>SUM(J10:J15)</f>
-        <v/>
-      </c>
-      <c r="K16" s="23">
-        <f>IF(E16&gt;0, F16/E16, 0)</f>
-        <v/>
-      </c>
-      <c r="L16" s="21">
-        <f>IF(K16&gt;=1, "SUPERADO", "EN CURSO")</f>
+      <c r="D17" s="34" t="inlineStr"/>
+      <c r="E17" s="22">
+        <f>SUM(E10:E16)</f>
+        <v/>
+      </c>
+      <c r="F17" s="22">
+        <f>SUM(F10:F16)</f>
+        <v/>
+      </c>
+      <c r="G17" s="22">
+        <f>SUM(G10:G16)</f>
+        <v/>
+      </c>
+      <c r="H17" s="22">
+        <f>SUM(H10:H16)</f>
+        <v/>
+      </c>
+      <c r="I17" s="22">
+        <f>SUM(I10:I16)</f>
+        <v/>
+      </c>
+      <c r="J17" s="22">
+        <f>SUM(J10:J16)</f>
+        <v/>
+      </c>
+      <c r="K17" s="23">
+        <f>IF(E17&gt;0, F17/E17, 0)</f>
+        <v/>
+      </c>
+      <c r="L17" s="21">
+        <f>IF(K17&gt;=1, "SUPERADO", "EN CURSO")</f>
         <v/>
       </c>
     </row>
@@ -9414,7 +9598,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:L29"/>
+  <dimension ref="B2:L30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -9441,7 +9625,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 28/09/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 29/09/2026</t>
         </is>
       </c>
     </row>
@@ -9486,19 +9670,19 @@
       <c r="C6" s="4" t="n"/>
       <c r="D6" s="24" t="inlineStr">
         <is>
-          <t>7,660 u</t>
+          <t>7,860 u</t>
         </is>
       </c>
       <c r="E6" s="4" t="n"/>
       <c r="F6" s="37" t="inlineStr">
         <is>
-          <t>44.2%</t>
+          <t>45.3%</t>
         </is>
       </c>
       <c r="G6" s="4" t="n"/>
       <c r="H6" s="37" t="inlineStr">
         <is>
-          <t>9,680 u</t>
+          <t>9,480 u</t>
         </is>
       </c>
       <c r="I6" s="4" t="n"/>
@@ -10363,12 +10547,12 @@
       </c>
       <c r="C27" s="31" t="inlineStr">
         <is>
-          <t>SPCE2B0020</t>
+          <t>AGZNP0005</t>
         </is>
       </c>
       <c r="D27" s="30" t="inlineStr">
         <is>
-          <t>SPRINTENE CON BORO, 20 L</t>
+          <t>AGROXILATO-ZN PLUS, 5 KG</t>
         </is>
       </c>
       <c r="E27" s="18" t="n">
@@ -10409,22 +10593,22 @@
       </c>
       <c r="C28" s="28" t="inlineStr">
         <is>
-          <t>SS0005</t>
+          <t>SPCE2B0020</t>
         </is>
       </c>
       <c r="D28" s="27" t="inlineStr">
         <is>
-          <t>SAL-WAX-Ca sólido, 5 KG</t>
+          <t>SPRINTENE CON BORO, 20 L</t>
         </is>
       </c>
       <c r="E28" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F28" s="14" t="n">
-        <v>300</v>
+        <v>200</v>
       </c>
       <c r="G28" s="14" t="n">
-        <v>300</v>
+        <v>200</v>
       </c>
       <c r="H28" s="14" t="n">
         <v>0</v>
@@ -10447,48 +10631,94 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="24" customHeight="1">
-      <c r="B29" s="20" t="inlineStr">
+    <row r="29">
+      <c r="B29" s="30" t="inlineStr">
+        <is>
+          <t>FITOMURCIA S.L.</t>
+        </is>
+      </c>
+      <c r="C29" s="31" t="inlineStr">
+        <is>
+          <t>SS0005</t>
+        </is>
+      </c>
+      <c r="D29" s="30" t="inlineStr">
+        <is>
+          <t>SAL-WAX-Ca sólido, 5 KG</t>
+        </is>
+      </c>
+      <c r="E29" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F29" s="18" t="n">
+        <v>300</v>
+      </c>
+      <c r="G29" s="18" t="n">
+        <v>300</v>
+      </c>
+      <c r="H29" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="I29" s="18">
+        <f>MAX(0, E29-F29)</f>
+        <v/>
+      </c>
+      <c r="J29" s="18">
+        <f>F29-E29</f>
+        <v/>
+      </c>
+      <c r="K29" s="19">
+        <f>IF(E29&gt;0, F29/E29, IF(F29&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L29" s="29" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="24" customHeight="1">
+      <c r="B30" s="20" t="inlineStr">
         <is>
           <t>TOTAL PEDRO</t>
         </is>
       </c>
-      <c r="C29" s="33" t="inlineStr">
-        <is>
-          <t>105 líneas</t>
-        </is>
-      </c>
-      <c r="D29" s="34" t="inlineStr"/>
-      <c r="E29" s="22">
-        <f>SUM(E10:E28)</f>
-        <v/>
-      </c>
-      <c r="F29" s="22">
-        <f>SUM(F10:F28)</f>
-        <v/>
-      </c>
-      <c r="G29" s="22">
-        <f>SUM(G10:G28)</f>
-        <v/>
-      </c>
-      <c r="H29" s="22">
-        <f>SUM(H10:H28)</f>
-        <v/>
-      </c>
-      <c r="I29" s="22">
-        <f>SUM(I10:I28)</f>
-        <v/>
-      </c>
-      <c r="J29" s="22">
-        <f>SUM(J10:J28)</f>
-        <v/>
-      </c>
-      <c r="K29" s="23">
-        <f>IF(E29&gt;0, F29/E29, 0)</f>
-        <v/>
-      </c>
-      <c r="L29" s="21">
-        <f>IF(K29&gt;=1, "SUPERADO", "EN CURSO")</f>
+      <c r="C30" s="33" t="inlineStr">
+        <is>
+          <t>106 líneas</t>
+        </is>
+      </c>
+      <c r="D30" s="34" t="inlineStr"/>
+      <c r="E30" s="22">
+        <f>SUM(E10:E29)</f>
+        <v/>
+      </c>
+      <c r="F30" s="22">
+        <f>SUM(F10:F29)</f>
+        <v/>
+      </c>
+      <c r="G30" s="22">
+        <f>SUM(G10:G29)</f>
+        <v/>
+      </c>
+      <c r="H30" s="22">
+        <f>SUM(H10:H29)</f>
+        <v/>
+      </c>
+      <c r="I30" s="22">
+        <f>SUM(I10:I29)</f>
+        <v/>
+      </c>
+      <c r="J30" s="22">
+        <f>SUM(J10:J29)</f>
+        <v/>
+      </c>
+      <c r="K30" s="23">
+        <f>IF(E30&gt;0, F30/E30, 0)</f>
+        <v/>
+      </c>
+      <c r="L30" s="21">
+        <f>IF(K30&gt;=1, "SUPERADO", "EN CURSO")</f>
         <v/>
       </c>
     </row>
@@ -10517,7 +10747,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:L25"/>
+  <dimension ref="B2:L36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -10544,7 +10774,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 28/09/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 29/09/2026</t>
         </is>
       </c>
     </row>
@@ -10589,25 +10819,25 @@
       <c r="C6" s="4" t="n"/>
       <c r="D6" s="24" t="inlineStr">
         <is>
-          <t>31,850 u</t>
+          <t>44,724 u</t>
         </is>
       </c>
       <c r="E6" s="4" t="n"/>
       <c r="F6" s="37" t="inlineStr">
         <is>
-          <t>69.2%</t>
+          <t>97.2%</t>
         </is>
       </c>
       <c r="G6" s="4" t="n"/>
       <c r="H6" s="37" t="inlineStr">
         <is>
-          <t>14,150 u</t>
+          <t>1,276 u</t>
         </is>
       </c>
       <c r="I6" s="4" t="n"/>
       <c r="J6" s="24" t="inlineStr">
         <is>
-          <t>8,800 u</t>
+          <t>21,674 u</t>
         </is>
       </c>
       <c r="K6" s="4" t="n"/>
@@ -11366,48 +11596,554 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="24" customHeight="1">
-      <c r="B25" s="20" t="inlineStr">
+    <row r="25">
+      <c r="B25" s="30" t="inlineStr">
+        <is>
+          <t>TÉCNICAS AGRÍCOLAS, S.A.</t>
+        </is>
+      </c>
+      <c r="C25" s="31" t="inlineStr">
+        <is>
+          <t>A-500001</t>
+        </is>
+      </c>
+      <c r="D25" s="30" t="inlineStr">
+        <is>
+          <t>CODIORGAN-A50, 1 KG</t>
+        </is>
+      </c>
+      <c r="E25" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" s="18" t="n">
+        <v>368</v>
+      </c>
+      <c r="G25" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" s="18" t="n">
+        <v>368</v>
+      </c>
+      <c r="I25" s="18">
+        <f>MAX(0, E25-F25)</f>
+        <v/>
+      </c>
+      <c r="J25" s="18">
+        <f>F25-E25</f>
+        <v/>
+      </c>
+      <c r="K25" s="19">
+        <f>IF(E25&gt;0, F25/E25, IF(F25&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L25" s="29" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="27" t="inlineStr">
+        <is>
+          <t>TÉCNICAS AGRÍCOLAS, S.A.</t>
+        </is>
+      </c>
+      <c r="C26" s="28" t="inlineStr">
+        <is>
+          <t>AGXCR0001</t>
+        </is>
+      </c>
+      <c r="D26" s="27" t="inlineStr">
+        <is>
+          <t>AGROXILATO-K, 1 L</t>
+        </is>
+      </c>
+      <c r="E26" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" s="14" t="n">
+        <v>540</v>
+      </c>
+      <c r="G26" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" s="14" t="n">
+        <v>540</v>
+      </c>
+      <c r="I26" s="14">
+        <f>MAX(0, E26-F26)</f>
+        <v/>
+      </c>
+      <c r="J26" s="14">
+        <f>F26-E26</f>
+        <v/>
+      </c>
+      <c r="K26" s="15">
+        <f>IF(E26&gt;0, F26/E26, IF(F26&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L26" s="29" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="30" t="inlineStr">
+        <is>
+          <t>TÉCNICAS AGRÍCOLAS, S.A.</t>
+        </is>
+      </c>
+      <c r="C27" s="31" t="inlineStr">
+        <is>
+          <t>AGXCR0005</t>
+        </is>
+      </c>
+      <c r="D27" s="30" t="inlineStr">
+        <is>
+          <t>AGROXILATO-K, 5 L</t>
+        </is>
+      </c>
+      <c r="E27" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" s="18" t="n">
+        <v>300</v>
+      </c>
+      <c r="G27" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H27" s="18" t="n">
+        <v>300</v>
+      </c>
+      <c r="I27" s="18">
+        <f>MAX(0, E27-F27)</f>
+        <v/>
+      </c>
+      <c r="J27" s="18">
+        <f>F27-E27</f>
+        <v/>
+      </c>
+      <c r="K27" s="19">
+        <f>IF(E27&gt;0, F27/E27, IF(F27&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L27" s="29" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="27" t="inlineStr">
+        <is>
+          <t>TÉCNICAS AGRÍCOLAS, S.A.</t>
+        </is>
+      </c>
+      <c r="C28" s="28" t="inlineStr">
+        <is>
+          <t>AN0005</t>
+        </is>
+      </c>
+      <c r="D28" s="27" t="inlineStr">
+        <is>
+          <t>ALCAPLANT, 5 KG</t>
+        </is>
+      </c>
+      <c r="E28" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" s="14" t="n">
+        <v>7920</v>
+      </c>
+      <c r="G28" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H28" s="14" t="n">
+        <v>7920</v>
+      </c>
+      <c r="I28" s="14">
+        <f>MAX(0, E28-F28)</f>
+        <v/>
+      </c>
+      <c r="J28" s="14">
+        <f>F28-E28</f>
+        <v/>
+      </c>
+      <c r="K28" s="15">
+        <f>IF(E28&gt;0, F28/E28, IF(F28&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L28" s="29" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="30" t="inlineStr">
+        <is>
+          <t>TÉCNICAS AGRÍCOLAS, S.A.</t>
+        </is>
+      </c>
+      <c r="C29" s="31" t="inlineStr">
+        <is>
+          <t>B0001</t>
+        </is>
+      </c>
+      <c r="D29" s="30" t="inlineStr">
+        <is>
+          <t>FORTALEZA,1 L</t>
+        </is>
+      </c>
+      <c r="E29" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F29" s="18" t="n">
+        <v>540</v>
+      </c>
+      <c r="G29" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H29" s="18" t="n">
+        <v>540</v>
+      </c>
+      <c r="I29" s="18">
+        <f>MAX(0, E29-F29)</f>
+        <v/>
+      </c>
+      <c r="J29" s="18">
+        <f>F29-E29</f>
+        <v/>
+      </c>
+      <c r="K29" s="19">
+        <f>IF(E29&gt;0, F29/E29, IF(F29&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L29" s="29" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="27" t="inlineStr">
+        <is>
+          <t>TÉCNICAS AGRÍCOLAS, S.A.</t>
+        </is>
+      </c>
+      <c r="C30" s="28" t="inlineStr">
+        <is>
+          <t>C-CU0001</t>
+        </is>
+      </c>
+      <c r="D30" s="27" t="inlineStr">
+        <is>
+          <t>CODICOBRE, 1 L</t>
+        </is>
+      </c>
+      <c r="E30" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" s="14" t="n">
+        <v>840</v>
+      </c>
+      <c r="G30" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H30" s="14" t="n">
+        <v>840</v>
+      </c>
+      <c r="I30" s="14">
+        <f>MAX(0, E30-F30)</f>
+        <v/>
+      </c>
+      <c r="J30" s="14">
+        <f>F30-E30</f>
+        <v/>
+      </c>
+      <c r="K30" s="15">
+        <f>IF(E30&gt;0, F30/E30, IF(F30&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L30" s="29" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="30" t="inlineStr">
+        <is>
+          <t>TÉCNICAS AGRÍCOLAS, S.A.</t>
+        </is>
+      </c>
+      <c r="C31" s="31" t="inlineStr">
+        <is>
+          <t>C-CU0005</t>
+        </is>
+      </c>
+      <c r="D31" s="30" t="inlineStr">
+        <is>
+          <t>CODICOBRE, 5 L</t>
+        </is>
+      </c>
+      <c r="E31" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" s="18" t="n">
+        <v>600</v>
+      </c>
+      <c r="G31" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H31" s="18" t="n">
+        <v>600</v>
+      </c>
+      <c r="I31" s="18">
+        <f>MAX(0, E31-F31)</f>
+        <v/>
+      </c>
+      <c r="J31" s="18">
+        <f>F31-E31</f>
+        <v/>
+      </c>
+      <c r="K31" s="19">
+        <f>IF(E31&gt;0, F31/E31, IF(F31&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L31" s="29" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="27" t="inlineStr">
+        <is>
+          <t>TÉCNICAS AGRÍCOLAS, S.A.</t>
+        </is>
+      </c>
+      <c r="C32" s="28" t="inlineStr">
+        <is>
+          <t>SERVFLETE</t>
+        </is>
+      </c>
+      <c r="D32" s="27" t="inlineStr">
+        <is>
+          <t>FREIGHT</t>
+        </is>
+      </c>
+      <c r="E32" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F32" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="G32" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H32" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="I32" s="14">
+        <f>MAX(0, E32-F32)</f>
+        <v/>
+      </c>
+      <c r="J32" s="14">
+        <f>F32-E32</f>
+        <v/>
+      </c>
+      <c r="K32" s="15">
+        <f>IF(E32&gt;0, F32/E32, IF(F32&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L32" s="29" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="30" t="inlineStr">
+        <is>
+          <t>TÉCNICAS AGRÍCOLAS, S.A.</t>
+        </is>
+      </c>
+      <c r="C33" s="31" t="inlineStr">
+        <is>
+          <t>SERVSEGURO</t>
+        </is>
+      </c>
+      <c r="D33" s="30" t="inlineStr">
+        <is>
+          <t>INSURANCE</t>
+        </is>
+      </c>
+      <c r="E33" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F33" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="G33" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H33" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="I33" s="18">
+        <f>MAX(0, E33-F33)</f>
+        <v/>
+      </c>
+      <c r="J33" s="18">
+        <f>F33-E33</f>
+        <v/>
+      </c>
+      <c r="K33" s="19">
+        <f>IF(E33&gt;0, F33/E33, IF(F33&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L33" s="29" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="27" t="inlineStr">
+        <is>
+          <t>TÉCNICAS AGRÍCOLAS, S.A.</t>
+        </is>
+      </c>
+      <c r="C34" s="28" t="inlineStr">
+        <is>
+          <t>SPCE0001</t>
+        </is>
+      </c>
+      <c r="D34" s="27" t="inlineStr">
+        <is>
+          <t>SPRINTENE ABONO CE, 1 L</t>
+        </is>
+      </c>
+      <c r="E34" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" s="14" t="n">
+        <v>180</v>
+      </c>
+      <c r="G34" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H34" s="14" t="n">
+        <v>180</v>
+      </c>
+      <c r="I34" s="14">
+        <f>MAX(0, E34-F34)</f>
+        <v/>
+      </c>
+      <c r="J34" s="14">
+        <f>F34-E34</f>
+        <v/>
+      </c>
+      <c r="K34" s="15">
+        <f>IF(E34&gt;0, F34/E34, IF(F34&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L34" s="29" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="30" t="inlineStr">
+        <is>
+          <t>TÉCNICAS AGRÍCOLAS, S.A.</t>
+        </is>
+      </c>
+      <c r="C35" s="31" t="inlineStr">
+        <is>
+          <t>SS0001</t>
+        </is>
+      </c>
+      <c r="D35" s="30" t="inlineStr">
+        <is>
+          <t>SAL WAX MAX, 1 KG</t>
+        </is>
+      </c>
+      <c r="E35" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F35" s="18" t="n">
+        <v>1584</v>
+      </c>
+      <c r="G35" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H35" s="18" t="n">
+        <v>1584</v>
+      </c>
+      <c r="I35" s="18">
+        <f>MAX(0, E35-F35)</f>
+        <v/>
+      </c>
+      <c r="J35" s="18">
+        <f>F35-E35</f>
+        <v/>
+      </c>
+      <c r="K35" s="19">
+        <f>IF(E35&gt;0, F35/E35, IF(F35&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L35" s="29" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="24" customHeight="1">
+      <c r="B36" s="20" t="inlineStr">
         <is>
           <t>TOTAL RICARDO</t>
         </is>
       </c>
-      <c r="C25" s="33" t="inlineStr">
-        <is>
-          <t>125 líneas</t>
-        </is>
-      </c>
-      <c r="D25" s="34" t="inlineStr"/>
-      <c r="E25" s="22">
-        <f>SUM(E10:E24)</f>
-        <v/>
-      </c>
-      <c r="F25" s="22">
-        <f>SUM(F10:F24)</f>
-        <v/>
-      </c>
-      <c r="G25" s="22">
-        <f>SUM(G10:G24)</f>
-        <v/>
-      </c>
-      <c r="H25" s="22">
-        <f>SUM(H10:H24)</f>
-        <v/>
-      </c>
-      <c r="I25" s="22">
-        <f>SUM(I10:I24)</f>
-        <v/>
-      </c>
-      <c r="J25" s="22">
-        <f>SUM(J10:J24)</f>
-        <v/>
-      </c>
-      <c r="K25" s="23">
-        <f>IF(E25&gt;0, F25/E25, 0)</f>
-        <v/>
-      </c>
-      <c r="L25" s="21">
-        <f>IF(K25&gt;=1, "SUPERADO", "EN CURSO")</f>
+      <c r="C36" s="33" t="inlineStr">
+        <is>
+          <t>136 líneas</t>
+        </is>
+      </c>
+      <c r="D36" s="34" t="inlineStr"/>
+      <c r="E36" s="22">
+        <f>SUM(E10:E35)</f>
+        <v/>
+      </c>
+      <c r="F36" s="22">
+        <f>SUM(F10:F35)</f>
+        <v/>
+      </c>
+      <c r="G36" s="22">
+        <f>SUM(G10:G35)</f>
+        <v/>
+      </c>
+      <c r="H36" s="22">
+        <f>SUM(H10:H35)</f>
+        <v/>
+      </c>
+      <c r="I36" s="22">
+        <f>SUM(I10:I35)</f>
+        <v/>
+      </c>
+      <c r="J36" s="22">
+        <f>SUM(J10:J35)</f>
+        <v/>
+      </c>
+      <c r="K36" s="23">
+        <f>IF(E36&gt;0, F36/E36, 0)</f>
+        <v/>
+      </c>
+      <c r="L36" s="21">
+        <f>IF(K36&gt;=1, "SUPERADO", "EN CURSO")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizar pedidos a 30/09/2026 y sincronizar dashboard web y Excel
</commit_message>
<xml_diff>
--- a/Seguimiento_Presupuesto_Sep_2026.xlsx
+++ b/Seguimiento_Presupuesto_Sep_2026.xlsx
@@ -902,7 +902,7 @@
     <row r="3" ht="20" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Comparativa Estimación Septiembre (Unidades) vs Pedidos Reales a Fecha 29/09/2026 | Generado: 29/09/2026 07:41</t>
+          <t>Comparativa Estimación Septiembre (Unidades) vs Pedidos Reales a Fecha 30/09/2026 | Generado: 30/09/2026 07:33</t>
         </is>
       </c>
     </row>
@@ -946,25 +946,25 @@
       <c r="C6" s="4" t="n"/>
       <c r="D6" s="8" t="inlineStr">
         <is>
-          <t>206,419 u</t>
+          <t>233,625 u</t>
         </is>
       </c>
       <c r="E6" s="4" t="n"/>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>113.4%</t>
+          <t>128.4%</t>
         </is>
       </c>
       <c r="G6" s="4" t="n"/>
       <c r="H6" s="9" t="inlineStr">
         <is>
-          <t>24,576 u</t>
+          <t>15,512 u</t>
         </is>
       </c>
       <c r="I6" s="4" t="n"/>
       <c r="J6" s="7" t="inlineStr">
         <is>
-          <t>104,718 u</t>
+          <t>130,660 u</t>
         </is>
       </c>
     </row>
@@ -1029,16 +1029,16 @@
         </is>
       </c>
       <c r="C10" s="13" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D10" s="14" t="n">
         <v>2320</v>
       </c>
       <c r="E10" s="14" t="n">
-        <v>11710</v>
+        <v>11874</v>
       </c>
       <c r="F10" s="14" t="n">
-        <v>11710</v>
+        <v>11874</v>
       </c>
       <c r="G10" s="14" t="n">
         <v>0</v>
@@ -1072,10 +1072,10 @@
         <v>56212</v>
       </c>
       <c r="F11" s="18" t="n">
-        <v>5896</v>
+        <v>6996</v>
       </c>
       <c r="G11" s="18" t="n">
-        <v>50316</v>
+        <v>49216</v>
       </c>
       <c r="H11" s="18">
         <f>MAX(0, D11-E11)</f>
@@ -1103,13 +1103,13 @@
         <v>21914</v>
       </c>
       <c r="E12" s="14" t="n">
-        <v>14826</v>
+        <v>23674</v>
       </c>
       <c r="F12" s="14" t="n">
         <v>14826</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>0</v>
+        <v>8848</v>
       </c>
       <c r="H12" s="14">
         <f>MAX(0, D12-E12)</f>
@@ -1137,13 +1137,13 @@
         <v>17100</v>
       </c>
       <c r="E13" s="18" t="n">
-        <v>38359</v>
+        <v>45669</v>
       </c>
       <c r="F13" s="18" t="n">
         <v>38359</v>
       </c>
       <c r="G13" s="18" t="n">
-        <v>0</v>
+        <v>7310</v>
       </c>
       <c r="H13" s="18">
         <f>MAX(0, D13-E13)</f>
@@ -1205,13 +1205,13 @@
         <v>17340</v>
       </c>
       <c r="E15" s="18" t="n">
-        <v>7860</v>
+        <v>8560</v>
       </c>
       <c r="F15" s="18" t="n">
         <v>7860</v>
       </c>
       <c r="G15" s="18" t="n">
-        <v>0</v>
+        <v>700</v>
       </c>
       <c r="H15" s="18">
         <f>MAX(0, D15-E15)</f>
@@ -1233,19 +1233,19 @@
         </is>
       </c>
       <c r="C16" s="13" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D16" s="14" t="n">
         <v>46000</v>
       </c>
       <c r="E16" s="14" t="n">
-        <v>44724</v>
+        <v>54908</v>
       </c>
       <c r="F16" s="14" t="n">
         <v>23050</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>21674</v>
+        <v>31858</v>
       </c>
       <c r="H16" s="14">
         <f>MAX(0, D16-E16)</f>
@@ -1323,7 +1323,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:L38"/>
+  <dimension ref="B2:L41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1350,7 +1350,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 29/09/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 30/09/2026</t>
         </is>
       </c>
     </row>
@@ -1395,13 +1395,13 @@
       <c r="C6" s="4" t="n"/>
       <c r="D6" s="25" t="inlineStr">
         <is>
-          <t>11,710 u</t>
+          <t>11,874 u</t>
         </is>
       </c>
       <c r="E6" s="4" t="n"/>
       <c r="F6" s="25" t="inlineStr">
         <is>
-          <t>504.7%</t>
+          <t>511.8%</t>
         </is>
       </c>
       <c r="G6" s="4" t="n"/>
@@ -2589,27 +2589,27 @@
     <row r="34">
       <c r="B34" s="27" t="inlineStr">
         <is>
-          <t>SAFIAGRO, S.A.</t>
+          <t>MUNDOHUERTO-CARMEN SOLAZ BLANCO</t>
         </is>
       </c>
       <c r="C34" s="28" t="inlineStr">
         <is>
-          <t>AGXK0020</t>
+          <t>PT0001</t>
         </is>
       </c>
       <c r="D34" s="27" t="inlineStr">
         <is>
-          <t>AGROXILATO-K, 20 L</t>
+          <t>AGROPOTASION, 1 L</t>
         </is>
       </c>
       <c r="E34" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F34" s="14" t="n">
-        <v>640</v>
+        <v>24</v>
       </c>
       <c r="G34" s="14" t="n">
-        <v>640</v>
+        <v>24</v>
       </c>
       <c r="H34" s="14" t="n">
         <v>0</v>
@@ -2635,27 +2635,27 @@
     <row r="35">
       <c r="B35" s="30" t="inlineStr">
         <is>
-          <t>T.J AGRICULTURA S.L.</t>
+          <t>MUNDOHUERTO-CARMEN SOLAZ BLANCO</t>
         </is>
       </c>
       <c r="C35" s="31" t="inlineStr">
         <is>
-          <t>AN0020</t>
+          <t>PT0005</t>
         </is>
       </c>
       <c r="D35" s="30" t="inlineStr">
         <is>
-          <t>ALCAPLANT NEW, 20 KG</t>
+          <t>AGROPOTASION, 5 L</t>
         </is>
       </c>
       <c r="E35" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F35" s="18" t="n">
-        <v>600</v>
+        <v>80</v>
       </c>
       <c r="G35" s="18" t="n">
-        <v>600</v>
+        <v>80</v>
       </c>
       <c r="H35" s="18" t="n">
         <v>0</v>
@@ -2681,27 +2681,27 @@
     <row r="36">
       <c r="B36" s="27" t="inlineStr">
         <is>
-          <t>T.J AGRICULTURA S.L.</t>
+          <t>MUNDOHUERTO-CARMEN SOLAZ BLANCO</t>
         </is>
       </c>
       <c r="C36" s="28" t="inlineStr">
         <is>
-          <t>SS0020</t>
+          <t>PT0020</t>
         </is>
       </c>
       <c r="D36" s="27" t="inlineStr">
         <is>
-          <t>SALWAX-CA, 20 KG</t>
+          <t>AGROPOTASION, 20 L</t>
         </is>
       </c>
       <c r="E36" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F36" s="14" t="n">
-        <v>500</v>
+        <v>60</v>
       </c>
       <c r="G36" s="14" t="n">
-        <v>500</v>
+        <v>60</v>
       </c>
       <c r="H36" s="14" t="n">
         <v>0</v>
@@ -2727,27 +2727,27 @@
     <row r="37">
       <c r="B37" s="30" t="inlineStr">
         <is>
-          <t>VILLALTA SATIVUM, S.L.</t>
+          <t>SAFIAGRO, S.A.</t>
         </is>
       </c>
       <c r="C37" s="31" t="inlineStr">
         <is>
-          <t>WHITE0020</t>
+          <t>AGXK0020</t>
         </is>
       </c>
       <c r="D37" s="30" t="inlineStr">
         <is>
-          <t>AGROWHITE, 20 KG</t>
+          <t>AGROXILATO-K, 20 L</t>
         </is>
       </c>
       <c r="E37" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F37" s="18" t="n">
-        <v>3460</v>
+        <v>640</v>
       </c>
       <c r="G37" s="18" t="n">
-        <v>3460</v>
+        <v>640</v>
       </c>
       <c r="H37" s="18" t="n">
         <v>0</v>
@@ -2770,48 +2770,186 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="24" customHeight="1">
-      <c r="B38" s="20" t="inlineStr">
+    <row r="38">
+      <c r="B38" s="27" t="inlineStr">
+        <is>
+          <t>T.J AGRICULTURA S.L.</t>
+        </is>
+      </c>
+      <c r="C38" s="28" t="inlineStr">
+        <is>
+          <t>AN0020</t>
+        </is>
+      </c>
+      <c r="D38" s="27" t="inlineStr">
+        <is>
+          <t>ALCAPLANT NEW, 20 KG</t>
+        </is>
+      </c>
+      <c r="E38" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F38" s="14" t="n">
+        <v>600</v>
+      </c>
+      <c r="G38" s="14" t="n">
+        <v>600</v>
+      </c>
+      <c r="H38" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I38" s="14">
+        <f>MAX(0, E38-F38)</f>
+        <v/>
+      </c>
+      <c r="J38" s="14">
+        <f>F38-E38</f>
+        <v/>
+      </c>
+      <c r="K38" s="15">
+        <f>IF(E38&gt;0, F38/E38, IF(F38&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L38" s="29" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" s="30" t="inlineStr">
+        <is>
+          <t>T.J AGRICULTURA S.L.</t>
+        </is>
+      </c>
+      <c r="C39" s="31" t="inlineStr">
+        <is>
+          <t>SS0020</t>
+        </is>
+      </c>
+      <c r="D39" s="30" t="inlineStr">
+        <is>
+          <t>SALWAX-CA, 20 KG</t>
+        </is>
+      </c>
+      <c r="E39" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F39" s="18" t="n">
+        <v>500</v>
+      </c>
+      <c r="G39" s="18" t="n">
+        <v>500</v>
+      </c>
+      <c r="H39" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="I39" s="18">
+        <f>MAX(0, E39-F39)</f>
+        <v/>
+      </c>
+      <c r="J39" s="18">
+        <f>F39-E39</f>
+        <v/>
+      </c>
+      <c r="K39" s="19">
+        <f>IF(E39&gt;0, F39/E39, IF(F39&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L39" s="29" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" s="27" t="inlineStr">
+        <is>
+          <t>VILLALTA SATIVUM, S.L.</t>
+        </is>
+      </c>
+      <c r="C40" s="28" t="inlineStr">
+        <is>
+          <t>WHITE0020</t>
+        </is>
+      </c>
+      <c r="D40" s="27" t="inlineStr">
+        <is>
+          <t>AGROWHITE, 20 KG</t>
+        </is>
+      </c>
+      <c r="E40" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F40" s="14" t="n">
+        <v>3460</v>
+      </c>
+      <c r="G40" s="14" t="n">
+        <v>3460</v>
+      </c>
+      <c r="H40" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I40" s="14">
+        <f>MAX(0, E40-F40)</f>
+        <v/>
+      </c>
+      <c r="J40" s="14">
+        <f>F40-E40</f>
+        <v/>
+      </c>
+      <c r="K40" s="15">
+        <f>IF(E40&gt;0, F40/E40, IF(F40&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L40" s="29" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="24" customHeight="1">
+      <c r="B41" s="20" t="inlineStr">
         <is>
           <t>TOTAL ALFONSO</t>
         </is>
       </c>
-      <c r="C38" s="33" t="inlineStr">
-        <is>
-          <t>280 líneas</t>
-        </is>
-      </c>
-      <c r="D38" s="34" t="inlineStr"/>
-      <c r="E38" s="22">
-        <f>SUM(E10:E37)</f>
-        <v/>
-      </c>
-      <c r="F38" s="22">
-        <f>SUM(F10:F37)</f>
-        <v/>
-      </c>
-      <c r="G38" s="22">
-        <f>SUM(G10:G37)</f>
-        <v/>
-      </c>
-      <c r="H38" s="22">
-        <f>SUM(H10:H37)</f>
-        <v/>
-      </c>
-      <c r="I38" s="22">
-        <f>SUM(I10:I37)</f>
-        <v/>
-      </c>
-      <c r="J38" s="22">
-        <f>SUM(J10:J37)</f>
-        <v/>
-      </c>
-      <c r="K38" s="23">
-        <f>IF(E38&gt;0, F38/E38, 0)</f>
-        <v/>
-      </c>
-      <c r="L38" s="21">
-        <f>IF(K38&gt;=1, "SUPERADO", "EN CURSO")</f>
+      <c r="C41" s="33" t="inlineStr">
+        <is>
+          <t>282 líneas</t>
+        </is>
+      </c>
+      <c r="D41" s="34" t="inlineStr"/>
+      <c r="E41" s="22">
+        <f>SUM(E10:E40)</f>
+        <v/>
+      </c>
+      <c r="F41" s="22">
+        <f>SUM(F10:F40)</f>
+        <v/>
+      </c>
+      <c r="G41" s="22">
+        <f>SUM(G10:G40)</f>
+        <v/>
+      </c>
+      <c r="H41" s="22">
+        <f>SUM(H10:H40)</f>
+        <v/>
+      </c>
+      <c r="I41" s="22">
+        <f>SUM(I10:I40)</f>
+        <v/>
+      </c>
+      <c r="J41" s="22">
+        <f>SUM(J10:J40)</f>
+        <v/>
+      </c>
+      <c r="K41" s="23">
+        <f>IF(E41&gt;0, F41/E41, 0)</f>
+        <v/>
+      </c>
+      <c r="L41" s="21">
+        <f>IF(K41&gt;=1, "SUPERADO", "EN CURSO")</f>
         <v/>
       </c>
     </row>
@@ -2867,7 +3005,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 29/09/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 30/09/2026</t>
         </is>
       </c>
     </row>
@@ -2930,7 +3068,7 @@
       <c r="I6" s="4" t="n"/>
       <c r="J6" s="24" t="inlineStr">
         <is>
-          <t>50,316 u</t>
+          <t>49,216 u</t>
         </is>
       </c>
       <c r="K6" s="4" t="n"/>
@@ -3988,10 +4126,10 @@
         <v>1100</v>
       </c>
       <c r="G31" s="18" t="n">
-        <v>0</v>
+        <v>1100</v>
       </c>
       <c r="H31" s="18" t="n">
-        <v>1100</v>
+        <v>0</v>
       </c>
       <c r="I31" s="18">
         <f>MAX(0, E31-F31)</f>
@@ -5185,7 +5323,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:L45"/>
+  <dimension ref="B2:L46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -5212,7 +5350,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 29/09/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 30/09/2026</t>
         </is>
       </c>
     </row>
@@ -5223,19 +5361,19 @@
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D5" s="5" t="inlineStr">
         <is>
           <t>PEDIDOS REALES (U)</t>
         </is>
       </c>
       <c r="E5" s="4" t="n"/>
-      <c r="F5" s="6" t="inlineStr">
+      <c r="F5" s="5" t="inlineStr">
         <is>
           <t>% CONSECUCIÓN</t>
         </is>
       </c>
       <c r="G5" s="4" t="n"/>
-      <c r="H5" s="6" t="inlineStr">
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>FALTA CONSEGUIR (GAP)</t>
         </is>
@@ -5255,27 +5393,27 @@
         </is>
       </c>
       <c r="C6" s="4" t="n"/>
-      <c r="D6" s="24" t="inlineStr">
-        <is>
-          <t>14,826 u</t>
+      <c r="D6" s="25" t="inlineStr">
+        <is>
+          <t>23,674 u</t>
         </is>
       </c>
       <c r="E6" s="4" t="n"/>
-      <c r="F6" s="37" t="inlineStr">
-        <is>
-          <t>67.7%</t>
+      <c r="F6" s="25" t="inlineStr">
+        <is>
+          <t>108.0%</t>
         </is>
       </c>
       <c r="G6" s="4" t="n"/>
-      <c r="H6" s="37" t="inlineStr">
-        <is>
-          <t>7,088 u</t>
+      <c r="H6" s="25" t="inlineStr">
+        <is>
+          <t>0 u</t>
         </is>
       </c>
       <c r="I6" s="4" t="n"/>
       <c r="J6" s="24" t="inlineStr">
         <is>
-          <t>0 u</t>
+          <t>8,848 u</t>
         </is>
       </c>
       <c r="K6" s="4" t="n"/>
@@ -5548,13 +5686,13 @@
         <v>960</v>
       </c>
       <c r="F14" s="14" t="n">
-        <v>640</v>
+        <v>2560</v>
       </c>
       <c r="G14" s="14" t="n">
         <v>640</v>
       </c>
       <c r="H14" s="14" t="n">
-        <v>0</v>
+        <v>1920</v>
       </c>
       <c r="I14" s="14">
         <f>MAX(0, E14-F14)</f>
@@ -5568,9 +5706,9 @@
         <f>IF(E14&gt;0, F14/E14, IF(F14&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L14" s="32" t="inlineStr">
-        <is>
-          <t>En Curso</t>
+      <c r="L14" s="29" t="inlineStr">
+        <is>
+          <t>Superado</t>
         </is>
       </c>
     </row>
@@ -5594,13 +5732,13 @@
         <v>640</v>
       </c>
       <c r="F15" s="18" t="n">
-        <v>0</v>
+        <v>640</v>
       </c>
       <c r="G15" s="18" t="n">
         <v>0</v>
       </c>
       <c r="H15" s="18" t="n">
-        <v>0</v>
+        <v>640</v>
       </c>
       <c r="I15" s="18">
         <f>MAX(0, E15-F15)</f>
@@ -5614,9 +5752,9 @@
         <f>IF(E15&gt;0, F15/E15, IF(F15&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L15" s="35" t="inlineStr">
-        <is>
-          <t>Sin Pedido</t>
+      <c r="L15" s="29" t="inlineStr">
+        <is>
+          <t>Superado</t>
         </is>
       </c>
     </row>
@@ -5778,13 +5916,13 @@
         <v>400</v>
       </c>
       <c r="F19" s="18" t="n">
-        <v>700</v>
+        <v>1300</v>
       </c>
       <c r="G19" s="18" t="n">
         <v>700</v>
       </c>
       <c r="H19" s="18" t="n">
-        <v>0</v>
+        <v>600</v>
       </c>
       <c r="I19" s="18">
         <f>MAX(0, E19-F19)</f>
@@ -5824,13 +5962,13 @@
         <v>800</v>
       </c>
       <c r="F20" s="14" t="n">
-        <v>100</v>
+        <v>1600</v>
       </c>
       <c r="G20" s="14" t="n">
         <v>100</v>
       </c>
       <c r="H20" s="14" t="n">
-        <v>0</v>
+        <v>1500</v>
       </c>
       <c r="I20" s="14">
         <f>MAX(0, E20-F20)</f>
@@ -5844,9 +5982,9 @@
         <f>IF(E20&gt;0, F20/E20, IF(F20&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L20" s="36" t="inlineStr">
-        <is>
-          <t>Rezagado</t>
+      <c r="L20" s="29" t="inlineStr">
+        <is>
+          <t>Superado</t>
         </is>
       </c>
     </row>
@@ -5870,13 +6008,13 @@
         <v>1280</v>
       </c>
       <c r="F21" s="18" t="n">
-        <v>640</v>
+        <v>4480</v>
       </c>
       <c r="G21" s="18" t="n">
         <v>640</v>
       </c>
       <c r="H21" s="18" t="n">
-        <v>0</v>
+        <v>3840</v>
       </c>
       <c r="I21" s="18">
         <f>MAX(0, E21-F21)</f>
@@ -5890,9 +6028,9 @@
         <f>IF(E21&gt;0, F21/E21, IF(F21&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L21" s="32" t="inlineStr">
-        <is>
-          <t>En Curso</t>
+      <c r="L21" s="29" t="inlineStr">
+        <is>
+          <t>Superado</t>
         </is>
       </c>
     </row>
@@ -5904,25 +6042,25 @@
       </c>
       <c r="C22" s="28" t="inlineStr">
         <is>
-          <t>PHD0005</t>
+          <t>PHD0001</t>
         </is>
       </c>
       <c r="D22" s="27" t="inlineStr">
         <is>
-          <t>PH-DOWNER, 5 L</t>
+          <t>PH-DOWNER, 1 L</t>
         </is>
       </c>
       <c r="E22" s="14" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="F22" s="14" t="n">
-        <v>0</v>
+        <v>48</v>
       </c>
       <c r="G22" s="14" t="n">
         <v>0</v>
       </c>
       <c r="H22" s="14" t="n">
-        <v>0</v>
+        <v>48</v>
       </c>
       <c r="I22" s="14">
         <f>MAX(0, E22-F22)</f>
@@ -5936,9 +6074,9 @@
         <f>IF(E22&gt;0, F22/E22, IF(F22&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L22" s="35" t="inlineStr">
-        <is>
-          <t>Sin Pedido</t>
+      <c r="L22" s="29" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -5950,25 +6088,25 @@
       </c>
       <c r="C23" s="31" t="inlineStr">
         <is>
-          <t>PIV0020</t>
+          <t>PHD0005</t>
         </is>
       </c>
       <c r="D23" s="30" t="inlineStr">
         <is>
-          <t>PGR IV, 20 L</t>
+          <t>PH-DOWNER, 5 L</t>
         </is>
       </c>
       <c r="E23" s="18" t="n">
-        <v>3200</v>
+        <v>100</v>
       </c>
       <c r="F23" s="18" t="n">
-        <v>640</v>
+        <v>300</v>
       </c>
       <c r="G23" s="18" t="n">
-        <v>640</v>
+        <v>0</v>
       </c>
       <c r="H23" s="18" t="n">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="I23" s="18">
         <f>MAX(0, E23-F23)</f>
@@ -5982,9 +6120,9 @@
         <f>IF(E23&gt;0, F23/E23, IF(F23&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L23" s="36" t="inlineStr">
-        <is>
-          <t>Rezagado</t>
+      <c r="L23" s="29" t="inlineStr">
+        <is>
+          <t>Superado</t>
         </is>
       </c>
     </row>
@@ -5996,22 +6134,22 @@
       </c>
       <c r="C24" s="28" t="inlineStr">
         <is>
-          <t>S0020</t>
+          <t>PIV0020</t>
         </is>
       </c>
       <c r="D24" s="27" t="inlineStr">
         <is>
-          <t>SAL-WAX STAR, 20 L</t>
+          <t>PGR IV, 20 L</t>
         </is>
       </c>
       <c r="E24" s="14" t="n">
+        <v>3200</v>
+      </c>
+      <c r="F24" s="14" t="n">
         <v>640</v>
       </c>
-      <c r="F24" s="14" t="n">
-        <v>0</v>
-      </c>
       <c r="G24" s="14" t="n">
-        <v>0</v>
+        <v>640</v>
       </c>
       <c r="H24" s="14" t="n">
         <v>0</v>
@@ -6028,9 +6166,9 @@
         <f>IF(E24&gt;0, F24/E24, IF(F24&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L24" s="35" t="inlineStr">
-        <is>
-          <t>Sin Pedido</t>
+      <c r="L24" s="36" t="inlineStr">
+        <is>
+          <t>Rezagado</t>
         </is>
       </c>
     </row>
@@ -6042,22 +6180,22 @@
       </c>
       <c r="C25" s="31" t="inlineStr">
         <is>
-          <t>TRI0005</t>
+          <t>S0020</t>
         </is>
       </c>
       <c r="D25" s="30" t="inlineStr">
         <is>
-          <t>TRIFENO-94, 5L</t>
+          <t>SAL-WAX STAR, 20 L</t>
         </is>
       </c>
       <c r="E25" s="18" t="n">
-        <v>100</v>
+        <v>640</v>
       </c>
       <c r="F25" s="18" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G25" s="18" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="H25" s="18" t="n">
         <v>0</v>
@@ -6074,36 +6212,36 @@
         <f>IF(E25&gt;0, F25/E25, IF(F25&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L25" s="29" t="inlineStr">
-        <is>
-          <t>Superado</t>
+      <c r="L25" s="35" t="inlineStr">
+        <is>
+          <t>Sin Pedido</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="B26" s="27" t="inlineStr">
         <is>
-          <t>COOP.AGRIC. SAN ISIDRO S.C.A.</t>
+          <t>CAMPOEJIDO S.C.A.</t>
         </is>
       </c>
       <c r="C26" s="28" t="inlineStr">
         <is>
-          <t>AGXK0020</t>
+          <t>TRI0005</t>
         </is>
       </c>
       <c r="D26" s="27" t="inlineStr">
         <is>
-          <t>AGROXILATO-K, 20 L</t>
+          <t>TRIFENO-94, 5L</t>
         </is>
       </c>
       <c r="E26" s="14" t="n">
-        <v>3200</v>
+        <v>100</v>
       </c>
       <c r="F26" s="14" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="G26" s="14" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="H26" s="14" t="n">
         <v>0</v>
@@ -6120,9 +6258,9 @@
         <f>IF(E26&gt;0, F26/E26, IF(F26&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L26" s="35" t="inlineStr">
-        <is>
-          <t>Sin Pedido</t>
+      <c r="L26" s="29" t="inlineStr">
+        <is>
+          <t>Superado</t>
         </is>
       </c>
     </row>
@@ -6134,16 +6272,16 @@
       </c>
       <c r="C27" s="31" t="inlineStr">
         <is>
-          <t>AGXK0200</t>
+          <t>AGXK0020</t>
         </is>
       </c>
       <c r="D27" s="30" t="inlineStr">
         <is>
-          <t>AGROXILATO-K, 200 L</t>
+          <t>AGROXILATO-K, 20 L</t>
         </is>
       </c>
       <c r="E27" s="18" t="n">
-        <v>400</v>
+        <v>3200</v>
       </c>
       <c r="F27" s="18" t="n">
         <v>0</v>
@@ -6180,16 +6318,16 @@
       </c>
       <c r="C28" s="28" t="inlineStr">
         <is>
-          <t>AVAN0005</t>
+          <t>AGXK0200</t>
         </is>
       </c>
       <c r="D28" s="27" t="inlineStr">
         <is>
-          <t>FLORAMEC AVANCE, 5 L</t>
+          <t>AGROXILATO-K, 200 L</t>
         </is>
       </c>
       <c r="E28" s="14" t="n">
-        <v>1200</v>
+        <v>400</v>
       </c>
       <c r="F28" s="14" t="n">
         <v>0</v>
@@ -6226,16 +6364,16 @@
       </c>
       <c r="C29" s="31" t="inlineStr">
         <is>
-          <t>C-L0005</t>
+          <t>AVAN0005</t>
         </is>
       </c>
       <c r="D29" s="30" t="inlineStr">
         <is>
-          <t>CODIBOR-L, 5 L</t>
+          <t>FLORAMEC AVANCE, 5 L</t>
         </is>
       </c>
       <c r="E29" s="18" t="n">
-        <v>200</v>
+        <v>1200</v>
       </c>
       <c r="F29" s="18" t="n">
         <v>0</v>
@@ -6272,16 +6410,16 @@
       </c>
       <c r="C30" s="28" t="inlineStr">
         <is>
-          <t>C-MB0005</t>
+          <t>C-L0005</t>
         </is>
       </c>
       <c r="D30" s="27" t="inlineStr">
         <is>
-          <t>CODIFOL-MB, 5 L</t>
+          <t>CODIBOR-L, 5 L</t>
         </is>
       </c>
       <c r="E30" s="14" t="n">
-        <v>300</v>
+        <v>200</v>
       </c>
       <c r="F30" s="14" t="n">
         <v>0</v>
@@ -6318,16 +6456,16 @@
       </c>
       <c r="C31" s="31" t="inlineStr">
         <is>
-          <t>CPLUS0020</t>
+          <t>C-MB0005</t>
         </is>
       </c>
       <c r="D31" s="30" t="inlineStr">
         <is>
-          <t>CALCIPLUS, 20 L</t>
+          <t>CODIFOL-MB, 5 L</t>
         </is>
       </c>
       <c r="E31" s="18" t="n">
-        <v>640</v>
+        <v>300</v>
       </c>
       <c r="F31" s="18" t="n">
         <v>0</v>
@@ -6364,16 +6502,16 @@
       </c>
       <c r="C32" s="28" t="inlineStr">
         <is>
-          <t>PIV0020</t>
+          <t>CPLUS0020</t>
         </is>
       </c>
       <c r="D32" s="27" t="inlineStr">
         <is>
-          <t>PGR IV, 20 L</t>
+          <t>CALCIPLUS, 20 L</t>
         </is>
       </c>
       <c r="E32" s="14" t="n">
-        <v>1280</v>
+        <v>640</v>
       </c>
       <c r="F32" s="14" t="n">
         <v>0</v>
@@ -6405,21 +6543,21 @@
     <row r="33">
       <c r="B33" s="30" t="inlineStr">
         <is>
-          <t>GUIVARTO AGRICOLA, S.L.</t>
+          <t>COOP.AGRIC. SAN ISIDRO S.C.A.</t>
         </is>
       </c>
       <c r="C33" s="31" t="inlineStr">
         <is>
-          <t>A-50(2)0005</t>
+          <t>PIV0020</t>
         </is>
       </c>
       <c r="D33" s="30" t="inlineStr">
         <is>
-          <t>CODIORGAN A-50, 5 KG</t>
+          <t>PGR IV, 20 L</t>
         </is>
       </c>
       <c r="E33" s="18" t="n">
-        <v>100</v>
+        <v>1280</v>
       </c>
       <c r="F33" s="18" t="n">
         <v>0</v>
@@ -6456,16 +6594,16 @@
       </c>
       <c r="C34" s="28" t="inlineStr">
         <is>
-          <t>AGXK0020</t>
+          <t>A-50(2)0005</t>
         </is>
       </c>
       <c r="D34" s="27" t="inlineStr">
         <is>
-          <t>AGROXILATO-K, 20 L</t>
+          <t>CODIORGAN A-50, 5 KG</t>
         </is>
       </c>
       <c r="E34" s="14" t="n">
-        <v>1240</v>
+        <v>100</v>
       </c>
       <c r="F34" s="14" t="n">
         <v>0</v>
@@ -6502,22 +6640,22 @@
       </c>
       <c r="C35" s="31" t="inlineStr">
         <is>
-          <t>AGXK1000</t>
+          <t>AGXK0020</t>
         </is>
       </c>
       <c r="D35" s="30" t="inlineStr">
         <is>
-          <t>AGROXILATO-K, 1000 L</t>
+          <t>AGROXILATO-K, 20 L</t>
         </is>
       </c>
       <c r="E35" s="18" t="n">
-        <v>0</v>
+        <v>1240</v>
       </c>
       <c r="F35" s="18" t="n">
-        <v>8000</v>
+        <v>0</v>
       </c>
       <c r="G35" s="18" t="n">
-        <v>8000</v>
+        <v>0</v>
       </c>
       <c r="H35" s="18" t="n">
         <v>0</v>
@@ -6534,9 +6672,9 @@
         <f>IF(E35&gt;0, F35/E35, IF(F35&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L35" s="29" t="inlineStr">
-        <is>
-          <t>Extra Estimación</t>
+      <c r="L35" s="35" t="inlineStr">
+        <is>
+          <t>Sin Pedido</t>
         </is>
       </c>
     </row>
@@ -6548,22 +6686,22 @@
       </c>
       <c r="C36" s="28" t="inlineStr">
         <is>
-          <t>AGZNP0005</t>
+          <t>AGXK1000</t>
         </is>
       </c>
       <c r="D36" s="27" t="inlineStr">
         <is>
-          <t>AGROXILATO-ZN PLUS, 5 KG</t>
+          <t>AGROXILATO-K, 1000 L</t>
         </is>
       </c>
       <c r="E36" s="14" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="F36" s="14" t="n">
-        <v>50</v>
+        <v>8000</v>
       </c>
       <c r="G36" s="14" t="n">
-        <v>50</v>
+        <v>8000</v>
       </c>
       <c r="H36" s="14" t="n">
         <v>0</v>
@@ -6582,7 +6720,7 @@
       </c>
       <c r="L36" s="29" t="inlineStr">
         <is>
-          <t>Superado</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -6594,22 +6732,22 @@
       </c>
       <c r="C37" s="31" t="inlineStr">
         <is>
-          <t>AQUOM0005</t>
+          <t>AGZNP0005</t>
         </is>
       </c>
       <c r="D37" s="30" t="inlineStr">
         <is>
-          <t>AQUOM, 5 L</t>
+          <t>AGROXILATO-ZN PLUS, 5 KG</t>
         </is>
       </c>
       <c r="E37" s="18" t="n">
-        <v>200</v>
+        <v>50</v>
       </c>
       <c r="F37" s="18" t="n">
-        <v>200</v>
+        <v>50</v>
       </c>
       <c r="G37" s="18" t="n">
-        <v>200</v>
+        <v>50</v>
       </c>
       <c r="H37" s="18" t="n">
         <v>0</v>
@@ -6640,22 +6778,22 @@
       </c>
       <c r="C38" s="28" t="inlineStr">
         <is>
-          <t>AVAN0020</t>
+          <t>AQUOM0005</t>
         </is>
       </c>
       <c r="D38" s="27" t="inlineStr">
         <is>
-          <t>FLORAMEC AVANCE, 20 L</t>
+          <t>AQUOM, 5 L</t>
         </is>
       </c>
       <c r="E38" s="14" t="n">
-        <v>640</v>
+        <v>200</v>
       </c>
       <c r="F38" s="14" t="n">
-        <v>640</v>
+        <v>200</v>
       </c>
       <c r="G38" s="14" t="n">
-        <v>640</v>
+        <v>200</v>
       </c>
       <c r="H38" s="14" t="n">
         <v>0</v>
@@ -6686,22 +6824,22 @@
       </c>
       <c r="C39" s="31" t="inlineStr">
         <is>
-          <t>BEY0020</t>
+          <t>AVAN0020</t>
         </is>
       </c>
       <c r="D39" s="30" t="inlineStr">
         <is>
-          <t>FLORAMEC PLUS 20 L</t>
+          <t>FLORAMEC AVANCE, 20 L</t>
         </is>
       </c>
       <c r="E39" s="18" t="n">
-        <v>80</v>
+        <v>640</v>
       </c>
       <c r="F39" s="18" t="n">
-        <v>80</v>
+        <v>640</v>
       </c>
       <c r="G39" s="18" t="n">
-        <v>80</v>
+        <v>640</v>
       </c>
       <c r="H39" s="18" t="n">
         <v>0</v>
@@ -6732,22 +6870,22 @@
       </c>
       <c r="C40" s="28" t="inlineStr">
         <is>
-          <t>BROTA0005</t>
+          <t>BEY0020</t>
         </is>
       </c>
       <c r="D40" s="27" t="inlineStr">
         <is>
-          <t>BROTAMEC, 5 L</t>
+          <t>FLORAMEC PLUS 20 L</t>
         </is>
       </c>
       <c r="E40" s="14" t="n">
-        <v>600</v>
+        <v>80</v>
       </c>
       <c r="F40" s="14" t="n">
-        <v>600</v>
+        <v>80</v>
       </c>
       <c r="G40" s="14" t="n">
-        <v>600</v>
+        <v>80</v>
       </c>
       <c r="H40" s="14" t="n">
         <v>0</v>
@@ -6778,22 +6916,22 @@
       </c>
       <c r="C41" s="31" t="inlineStr">
         <is>
-          <t>C-M-P0001</t>
+          <t>BROTA0005</t>
         </is>
       </c>
       <c r="D41" s="30" t="inlineStr">
         <is>
-          <t>CODIFOL Mo-PLUS, 1 L</t>
+          <t>BROTAMEC, 5 L</t>
         </is>
       </c>
       <c r="E41" s="18" t="n">
-        <v>36</v>
+        <v>600</v>
       </c>
       <c r="F41" s="18" t="n">
-        <v>0</v>
+        <v>600</v>
       </c>
       <c r="G41" s="18" t="n">
-        <v>0</v>
+        <v>600</v>
       </c>
       <c r="H41" s="18" t="n">
         <v>0</v>
@@ -6810,9 +6948,9 @@
         <f>IF(E41&gt;0, F41/E41, IF(F41&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L41" s="35" t="inlineStr">
-        <is>
-          <t>Sin Pedido</t>
+      <c r="L41" s="29" t="inlineStr">
+        <is>
+          <t>Superado</t>
         </is>
       </c>
     </row>
@@ -6824,22 +6962,22 @@
       </c>
       <c r="C42" s="28" t="inlineStr">
         <is>
-          <t>FTK0005</t>
+          <t>C-M-P0001</t>
         </is>
       </c>
       <c r="D42" s="27" t="inlineStr">
         <is>
-          <t>FITOKONTROL CA FLOW, 5 KG</t>
+          <t>CODIFOL Mo-PLUS, 1 L</t>
         </is>
       </c>
       <c r="E42" s="14" t="n">
-        <v>800</v>
+        <v>36</v>
       </c>
       <c r="F42" s="14" t="n">
-        <v>800</v>
+        <v>0</v>
       </c>
       <c r="G42" s="14" t="n">
-        <v>800</v>
+        <v>0</v>
       </c>
       <c r="H42" s="14" t="n">
         <v>0</v>
@@ -6856,36 +6994,36 @@
         <f>IF(E42&gt;0, F42/E42, IF(F42&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L42" s="29" t="inlineStr">
-        <is>
-          <t>Superado</t>
+      <c r="L42" s="35" t="inlineStr">
+        <is>
+          <t>Sin Pedido</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="B43" s="30" t="inlineStr">
         <is>
-          <t>SUCA, S.C.A.</t>
+          <t>GUIVARTO AGRICOLA, S.L.</t>
         </is>
       </c>
       <c r="C43" s="31" t="inlineStr">
         <is>
-          <t>AGXK0020</t>
+          <t>FTK0005</t>
         </is>
       </c>
       <c r="D43" s="30" t="inlineStr">
         <is>
-          <t>AGROXILATO-K, 20 L</t>
+          <t>FITOKONTROL CA FLOW, 5 KG</t>
         </is>
       </c>
       <c r="E43" s="18" t="n">
-        <v>0</v>
+        <v>800</v>
       </c>
       <c r="F43" s="18" t="n">
-        <v>640</v>
+        <v>800</v>
       </c>
       <c r="G43" s="18" t="n">
-        <v>640</v>
+        <v>800</v>
       </c>
       <c r="H43" s="18" t="n">
         <v>0</v>
@@ -6904,7 +7042,7 @@
       </c>
       <c r="L43" s="29" t="inlineStr">
         <is>
-          <t>Extra Estimación</t>
+          <t>Superado</t>
         </is>
       </c>
     </row>
@@ -6916,22 +7054,22 @@
       </c>
       <c r="C44" s="28" t="inlineStr">
         <is>
-          <t>AVAN0020</t>
+          <t>AGXK0020</t>
         </is>
       </c>
       <c r="D44" s="27" t="inlineStr">
         <is>
-          <t>FLORAMEC AVANCE, 20 L</t>
+          <t>AGROXILATO-K, 20 L</t>
         </is>
       </c>
       <c r="E44" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F44" s="14" t="n">
-        <v>200</v>
+        <v>640</v>
       </c>
       <c r="G44" s="14" t="n">
-        <v>200</v>
+        <v>640</v>
       </c>
       <c r="H44" s="14" t="n">
         <v>0</v>
@@ -6954,48 +7092,94 @@
         </is>
       </c>
     </row>
-    <row r="45" ht="24" customHeight="1">
-      <c r="B45" s="20" t="inlineStr">
+    <row r="45">
+      <c r="B45" s="30" t="inlineStr">
+        <is>
+          <t>SUCA, S.C.A.</t>
+        </is>
+      </c>
+      <c r="C45" s="31" t="inlineStr">
+        <is>
+          <t>AVAN0020</t>
+        </is>
+      </c>
+      <c r="D45" s="30" t="inlineStr">
+        <is>
+          <t>FLORAMEC AVANCE, 20 L</t>
+        </is>
+      </c>
+      <c r="E45" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F45" s="18" t="n">
+        <v>200</v>
+      </c>
+      <c r="G45" s="18" t="n">
+        <v>200</v>
+      </c>
+      <c r="H45" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="I45" s="18">
+        <f>MAX(0, E45-F45)</f>
+        <v/>
+      </c>
+      <c r="J45" s="18">
+        <f>F45-E45</f>
+        <v/>
+      </c>
+      <c r="K45" s="19">
+        <f>IF(E45&gt;0, F45/E45, IF(F45&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L45" s="29" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="24" customHeight="1">
+      <c r="B46" s="20" t="inlineStr">
         <is>
           <t>TOTAL IRENE</t>
         </is>
       </c>
-      <c r="C45" s="33" t="inlineStr">
+      <c r="C46" s="33" t="inlineStr">
         <is>
           <t>89 líneas</t>
         </is>
       </c>
-      <c r="D45" s="34" t="inlineStr"/>
-      <c r="E45" s="22">
-        <f>SUM(E10:E44)</f>
-        <v/>
-      </c>
-      <c r="F45" s="22">
-        <f>SUM(F10:F44)</f>
-        <v/>
-      </c>
-      <c r="G45" s="22">
-        <f>SUM(G10:G44)</f>
-        <v/>
-      </c>
-      <c r="H45" s="22">
-        <f>SUM(H10:H44)</f>
-        <v/>
-      </c>
-      <c r="I45" s="22">
-        <f>SUM(I10:I44)</f>
-        <v/>
-      </c>
-      <c r="J45" s="22">
-        <f>SUM(J10:J44)</f>
-        <v/>
-      </c>
-      <c r="K45" s="23">
-        <f>IF(E45&gt;0, F45/E45, 0)</f>
-        <v/>
-      </c>
-      <c r="L45" s="21">
-        <f>IF(K45&gt;=1, "SUPERADO", "EN CURSO")</f>
+      <c r="D46" s="34" t="inlineStr"/>
+      <c r="E46" s="22">
+        <f>SUM(E10:E45)</f>
+        <v/>
+      </c>
+      <c r="F46" s="22">
+        <f>SUM(F10:F45)</f>
+        <v/>
+      </c>
+      <c r="G46" s="22">
+        <f>SUM(G10:G45)</f>
+        <v/>
+      </c>
+      <c r="H46" s="22">
+        <f>SUM(H10:H45)</f>
+        <v/>
+      </c>
+      <c r="I46" s="22">
+        <f>SUM(I10:I45)</f>
+        <v/>
+      </c>
+      <c r="J46" s="22">
+        <f>SUM(J10:J45)</f>
+        <v/>
+      </c>
+      <c r="K46" s="23">
+        <f>IF(E46&gt;0, F46/E46, 0)</f>
+        <v/>
+      </c>
+      <c r="L46" s="21">
+        <f>IF(K46&gt;=1, "SUPERADO", "EN CURSO")</f>
         <v/>
       </c>
     </row>
@@ -7024,7 +7208,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:L49"/>
+  <dimension ref="B2:L54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -7051,7 +7235,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 29/09/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 30/09/2026</t>
         </is>
       </c>
     </row>
@@ -7096,13 +7280,13 @@
       <c r="C6" s="4" t="n"/>
       <c r="D6" s="25" t="inlineStr">
         <is>
-          <t>38,359 u</t>
+          <t>45,669 u</t>
         </is>
       </c>
       <c r="E6" s="4" t="n"/>
       <c r="F6" s="25" t="inlineStr">
         <is>
-          <t>224.3%</t>
+          <t>267.1%</t>
         </is>
       </c>
       <c r="G6" s="4" t="n"/>
@@ -7114,7 +7298,7 @@
       <c r="I6" s="4" t="n"/>
       <c r="J6" s="24" t="inlineStr">
         <is>
-          <t>0 u</t>
+          <t>7,310 u</t>
         </is>
       </c>
       <c r="K6" s="4" t="n"/>
@@ -7203,13 +7387,13 @@
         <v>1600</v>
       </c>
       <c r="F10" s="14" t="n">
-        <v>1600</v>
+        <v>3200</v>
       </c>
       <c r="G10" s="14" t="n">
         <v>1600</v>
       </c>
       <c r="H10" s="14" t="n">
-        <v>0</v>
+        <v>1600</v>
       </c>
       <c r="I10" s="14">
         <f>MAX(0, E10-F10)</f>
@@ -7605,25 +7789,25 @@
       </c>
       <c r="C19" s="31" t="inlineStr">
         <is>
-          <t>PHD0005</t>
+          <t>JF0020</t>
         </is>
       </c>
       <c r="D19" s="30" t="inlineStr">
         <is>
-          <t>PH-DOWNER, 5 L</t>
+          <t>DRAGO-FOS, 20 L</t>
         </is>
       </c>
       <c r="E19" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F19" s="18" t="n">
-        <v>40</v>
+        <v>1280</v>
       </c>
       <c r="G19" s="18" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="H19" s="18" t="n">
-        <v>0</v>
+        <v>1280</v>
       </c>
       <c r="I19" s="18">
         <f>MAX(0, E19-F19)</f>
@@ -7646,27 +7830,27 @@
     <row r="20">
       <c r="B20" s="27" t="inlineStr">
         <is>
-          <t>ALMENDRALIA IBÉRICA, S.L.U.</t>
+          <t>AGROQUIMICAS DRAGO S.L.</t>
         </is>
       </c>
       <c r="C20" s="28" t="inlineStr">
         <is>
-          <t>AN0020</t>
+          <t>PHD0005</t>
         </is>
       </c>
       <c r="D20" s="27" t="inlineStr">
         <is>
-          <t>ALCAPLANT NEW, 20 KG</t>
+          <t>PH-DOWNER, 5 L</t>
         </is>
       </c>
       <c r="E20" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F20" s="14" t="n">
-        <v>1100</v>
+        <v>40</v>
       </c>
       <c r="G20" s="14" t="n">
-        <v>1100</v>
+        <v>40</v>
       </c>
       <c r="H20" s="14" t="n">
         <v>0</v>
@@ -7692,30 +7876,30 @@
     <row r="21">
       <c r="B21" s="30" t="inlineStr">
         <is>
-          <t>CABRERA MORALES FRANCISCO</t>
+          <t>AGROQUIMICAS DRAGO S.L.</t>
         </is>
       </c>
       <c r="C21" s="31" t="inlineStr">
         <is>
-          <t>A-50(2)0005</t>
+          <t>S0020</t>
         </is>
       </c>
       <c r="D21" s="30" t="inlineStr">
         <is>
-          <t>CODIORGAN A-50, 5 KG</t>
+          <t>SAL-WAX STAR, 20 L</t>
         </is>
       </c>
       <c r="E21" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F21" s="18" t="n">
-        <v>375</v>
+        <v>1280</v>
       </c>
       <c r="G21" s="18" t="n">
-        <v>375</v>
+        <v>0</v>
       </c>
       <c r="H21" s="18" t="n">
-        <v>0</v>
+        <v>1280</v>
       </c>
       <c r="I21" s="18">
         <f>MAX(0, E21-F21)</f>
@@ -7738,27 +7922,27 @@
     <row r="22">
       <c r="B22" s="27" t="inlineStr">
         <is>
-          <t>CABRERA MORALES FRANCISCO</t>
+          <t>ALMENDRALIA IBÉRICA, S.L.U.</t>
         </is>
       </c>
       <c r="C22" s="28" t="inlineStr">
         <is>
-          <t>ANAE0005</t>
+          <t>AN0020</t>
         </is>
       </c>
       <c r="D22" s="27" t="inlineStr">
         <is>
-          <t>ALCAPLANT NEW AE, 5 KG</t>
+          <t>ALCAPLANT NEW, 20 KG</t>
         </is>
       </c>
       <c r="E22" s="14" t="n">
-        <v>6600</v>
+        <v>0</v>
       </c>
       <c r="F22" s="14" t="n">
-        <v>4400</v>
+        <v>1100</v>
       </c>
       <c r="G22" s="14" t="n">
-        <v>4400</v>
+        <v>1100</v>
       </c>
       <c r="H22" s="14" t="n">
         <v>0</v>
@@ -7775,9 +7959,9 @@
         <f>IF(E22&gt;0, F22/E22, IF(F22&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L22" s="32" t="inlineStr">
-        <is>
-          <t>En Curso</t>
+      <c r="L22" s="29" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -7789,25 +7973,25 @@
       </c>
       <c r="C23" s="31" t="inlineStr">
         <is>
-          <t>BIO0005</t>
+          <t>A-50(2)0005</t>
         </is>
       </c>
       <c r="D23" s="30" t="inlineStr">
         <is>
-          <t>BIORAD-20, 5L</t>
+          <t>CODIORGAN A-50, 5 KG</t>
         </is>
       </c>
       <c r="E23" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F23" s="18" t="n">
-        <v>600</v>
+        <v>625</v>
       </c>
       <c r="G23" s="18" t="n">
-        <v>600</v>
+        <v>375</v>
       </c>
       <c r="H23" s="18" t="n">
-        <v>0</v>
+        <v>250</v>
       </c>
       <c r="I23" s="18">
         <f>MAX(0, E23-F23)</f>
@@ -7835,25 +8019,25 @@
       </c>
       <c r="C24" s="28" t="inlineStr">
         <is>
-          <t>BIO0020</t>
+          <t>A-50(2)0020</t>
         </is>
       </c>
       <c r="D24" s="27" t="inlineStr">
         <is>
-          <t>BIORAD-20, 20 L</t>
+          <t>CODIORGAN A-50, 20 KG</t>
         </is>
       </c>
       <c r="E24" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F24" s="14" t="n">
-        <v>1280</v>
+        <v>100</v>
       </c>
       <c r="G24" s="14" t="n">
-        <v>1280</v>
+        <v>0</v>
       </c>
       <c r="H24" s="14" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="I24" s="14">
         <f>MAX(0, E24-F24)</f>
@@ -7881,25 +8065,25 @@
       </c>
       <c r="C25" s="31" t="inlineStr">
         <is>
-          <t>C-L0005</t>
+          <t>ANAE0005</t>
         </is>
       </c>
       <c r="D25" s="30" t="inlineStr">
         <is>
-          <t>CODIBOR-L, 5 L</t>
+          <t>ALCAPLANT NEW AE, 5 KG</t>
         </is>
       </c>
       <c r="E25" s="18" t="n">
-        <v>0</v>
+        <v>6600</v>
       </c>
       <c r="F25" s="18" t="n">
-        <v>200</v>
+        <v>6600</v>
       </c>
       <c r="G25" s="18" t="n">
-        <v>200</v>
+        <v>4400</v>
       </c>
       <c r="H25" s="18" t="n">
-        <v>0</v>
+        <v>2200</v>
       </c>
       <c r="I25" s="18">
         <f>MAX(0, E25-F25)</f>
@@ -7915,34 +8099,34 @@
       </c>
       <c r="L25" s="29" t="inlineStr">
         <is>
-          <t>Extra Estimación</t>
+          <t>Superado</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="B26" s="27" t="inlineStr">
         <is>
-          <t>CODIMED EXPORT, S.L.</t>
+          <t>CABRERA MORALES FRANCISCO</t>
         </is>
       </c>
       <c r="C26" s="28" t="inlineStr">
         <is>
-          <t>C-L0005</t>
+          <t>BIO0005</t>
         </is>
       </c>
       <c r="D26" s="27" t="inlineStr">
         <is>
-          <t>CODIBOR-L, 5 L</t>
+          <t>BIORAD-20, 5L</t>
         </is>
       </c>
       <c r="E26" s="14" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="F26" s="14" t="n">
-        <v>200</v>
+        <v>600</v>
       </c>
       <c r="G26" s="14" t="n">
-        <v>200</v>
+        <v>600</v>
       </c>
       <c r="H26" s="14" t="n">
         <v>0</v>
@@ -7961,34 +8145,34 @@
       </c>
       <c r="L26" s="29" t="inlineStr">
         <is>
-          <t>Superado</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="B27" s="30" t="inlineStr">
         <is>
-          <t>CODIMED EXPORT, S.L.</t>
+          <t>CABRERA MORALES FRANCISCO</t>
         </is>
       </c>
       <c r="C27" s="31" t="inlineStr">
         <is>
-          <t>C-L0020</t>
+          <t>BIO0020</t>
         </is>
       </c>
       <c r="D27" s="30" t="inlineStr">
         <is>
-          <t>CODIBOR-L, 20 L</t>
+          <t>BIORAD-20, 20 L</t>
         </is>
       </c>
       <c r="E27" s="18" t="n">
-        <v>640</v>
+        <v>0</v>
       </c>
       <c r="F27" s="18" t="n">
-        <v>640</v>
+        <v>1280</v>
       </c>
       <c r="G27" s="18" t="n">
-        <v>640</v>
+        <v>1280</v>
       </c>
       <c r="H27" s="18" t="n">
         <v>0</v>
@@ -8007,37 +8191,37 @@
       </c>
       <c r="L27" s="29" t="inlineStr">
         <is>
-          <t>Superado</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="B28" s="27" t="inlineStr">
         <is>
-          <t>CODIMED EXPORT, S.L.</t>
+          <t>CABRERA MORALES FRANCISCO</t>
         </is>
       </c>
       <c r="C28" s="28" t="inlineStr">
         <is>
-          <t>PT0005</t>
+          <t>C-L0005</t>
         </is>
       </c>
       <c r="D28" s="27" t="inlineStr">
         <is>
-          <t>AGROPOTASION, 5 L</t>
+          <t>CODIBOR-L, 5 L</t>
         </is>
       </c>
       <c r="E28" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F28" s="14" t="n">
-        <v>100</v>
+        <v>400</v>
       </c>
       <c r="G28" s="14" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="H28" s="14" t="n">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="I28" s="14">
         <f>MAX(0, E28-F28)</f>
@@ -8060,17 +8244,17 @@
     <row r="29">
       <c r="B29" s="30" t="inlineStr">
         <is>
-          <t>CODIMED EXPORT, S.L.</t>
+          <t>CABRERA MORALES FRANCISCO</t>
         </is>
       </c>
       <c r="C29" s="31" t="inlineStr">
         <is>
-          <t>PT0020</t>
+          <t>PIV0005</t>
         </is>
       </c>
       <c r="D29" s="30" t="inlineStr">
         <is>
-          <t>AGROPOTASION, 20 L</t>
+          <t>PGR IV, 5 L</t>
         </is>
       </c>
       <c r="E29" s="18" t="n">
@@ -8080,10 +8264,10 @@
         <v>200</v>
       </c>
       <c r="G29" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H29" s="18" t="n">
         <v>200</v>
-      </c>
-      <c r="H29" s="18" t="n">
-        <v>0</v>
       </c>
       <c r="I29" s="18">
         <f>MAX(0, E29-F29)</f>
@@ -8106,30 +8290,30 @@
     <row r="30">
       <c r="B30" s="27" t="inlineStr">
         <is>
-          <t>CODIMED EXPORT, S.L.</t>
+          <t>CABRERA MORALES FRANCISCO</t>
         </is>
       </c>
       <c r="C30" s="28" t="inlineStr">
         <is>
-          <t>SPCE2B0020</t>
+          <t>PIV0020</t>
         </is>
       </c>
       <c r="D30" s="27" t="inlineStr">
         <is>
-          <t>SPRINTENE CON BORO, 20 L</t>
+          <t>PGR IV, 20 L</t>
         </is>
       </c>
       <c r="E30" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F30" s="14" t="n">
-        <v>320</v>
+        <v>200</v>
       </c>
       <c r="G30" s="14" t="n">
-        <v>320</v>
+        <v>0</v>
       </c>
       <c r="H30" s="14" t="n">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="I30" s="14">
         <f>MAX(0, E30-F30)</f>
@@ -8152,27 +8336,27 @@
     <row r="31">
       <c r="B31" s="30" t="inlineStr">
         <is>
-          <t>FINCA DOÑA ANA C.B.</t>
+          <t>CODIMED EXPORT, S.L.</t>
         </is>
       </c>
       <c r="C31" s="31" t="inlineStr">
         <is>
-          <t>A-50(2)0020</t>
+          <t>C-L0005</t>
         </is>
       </c>
       <c r="D31" s="30" t="inlineStr">
         <is>
-          <t>CODIORGAN-A50, 20 KG</t>
+          <t>CODIBOR-L, 5 L</t>
         </is>
       </c>
       <c r="E31" s="18" t="n">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="F31" s="18" t="n">
-        <v>120</v>
+        <v>200</v>
       </c>
       <c r="G31" s="18" t="n">
-        <v>120</v>
+        <v>200</v>
       </c>
       <c r="H31" s="18" t="n">
         <v>0</v>
@@ -8191,34 +8375,34 @@
       </c>
       <c r="L31" s="29" t="inlineStr">
         <is>
-          <t>Extra Estimación</t>
+          <t>Superado</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="B32" s="27" t="inlineStr">
         <is>
-          <t>FINCA DOÑA ANA C.B.</t>
+          <t>CODIMED EXPORT, S.L.</t>
         </is>
       </c>
       <c r="C32" s="28" t="inlineStr">
         <is>
-          <t>C-CU1000</t>
+          <t>C-L0020</t>
         </is>
       </c>
       <c r="D32" s="27" t="inlineStr">
         <is>
-          <t>CODICOBRE, 1000 L</t>
+          <t>CODIBOR-L, 20 L</t>
         </is>
       </c>
       <c r="E32" s="14" t="n">
-        <v>0</v>
+        <v>640</v>
       </c>
       <c r="F32" s="14" t="n">
-        <v>1000</v>
+        <v>640</v>
       </c>
       <c r="G32" s="14" t="n">
-        <v>1000</v>
+        <v>640</v>
       </c>
       <c r="H32" s="14" t="n">
         <v>0</v>
@@ -8237,24 +8421,24 @@
       </c>
       <c r="L32" s="29" t="inlineStr">
         <is>
-          <t>Extra Estimación</t>
+          <t>Superado</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="B33" s="30" t="inlineStr">
         <is>
-          <t>FITOSANITARIOS CARCAIXENT, S.L.</t>
+          <t>CODIMED EXPORT, S.L.</t>
         </is>
       </c>
       <c r="C33" s="31" t="inlineStr">
         <is>
-          <t>C-CU0005</t>
+          <t>PT0005</t>
         </is>
       </c>
       <c r="D33" s="30" t="inlineStr">
         <is>
-          <t>CODICOBRE, 5 L</t>
+          <t>AGROPOTASION, 5 L</t>
         </is>
       </c>
       <c r="E33" s="18" t="n">
@@ -8290,17 +8474,17 @@
     <row r="34">
       <c r="B34" s="27" t="inlineStr">
         <is>
-          <t>FITOSANITARIOS CARCAIXENT, S.L.</t>
+          <t>CODIMED EXPORT, S.L.</t>
         </is>
       </c>
       <c r="C34" s="28" t="inlineStr">
         <is>
-          <t>G30020</t>
+          <t>PT0020</t>
         </is>
       </c>
       <c r="D34" s="27" t="inlineStr">
         <is>
-          <t>GREEN-UP, 20 L</t>
+          <t>AGROPOTASION, 20 L</t>
         </is>
       </c>
       <c r="E34" s="14" t="n">
@@ -8336,27 +8520,27 @@
     <row r="35">
       <c r="B35" s="30" t="inlineStr">
         <is>
-          <t>FITOSANITARIOS CARCAIXENT, S.L.</t>
+          <t>CODIMED EXPORT, S.L.</t>
         </is>
       </c>
       <c r="C35" s="31" t="inlineStr">
         <is>
-          <t>HST0020</t>
+          <t>SPCE2B0020</t>
         </is>
       </c>
       <c r="D35" s="30" t="inlineStr">
         <is>
-          <t>HIDROSTRESS-40, 20 L</t>
+          <t>SPRINTENE CON BORO, 20 L</t>
         </is>
       </c>
       <c r="E35" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F35" s="18" t="n">
-        <v>100</v>
+        <v>320</v>
       </c>
       <c r="G35" s="18" t="n">
-        <v>100</v>
+        <v>320</v>
       </c>
       <c r="H35" s="18" t="n">
         <v>0</v>
@@ -8382,27 +8566,27 @@
     <row r="36">
       <c r="B36" s="27" t="inlineStr">
         <is>
-          <t>FITOSANITARIOS CARCAIXENT, S.L.</t>
+          <t>FINCA DOÑA ANA C.B.</t>
         </is>
       </c>
       <c r="C36" s="28" t="inlineStr">
         <is>
-          <t>PT0005</t>
+          <t>A-50(2)0020</t>
         </is>
       </c>
       <c r="D36" s="27" t="inlineStr">
         <is>
-          <t>AGROPOTASION, 5 L</t>
+          <t>CODIORGAN-A50, 20 KG</t>
         </is>
       </c>
       <c r="E36" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F36" s="14" t="n">
-        <v>600</v>
+        <v>120</v>
       </c>
       <c r="G36" s="14" t="n">
-        <v>600</v>
+        <v>120</v>
       </c>
       <c r="H36" s="14" t="n">
         <v>0</v>
@@ -8428,27 +8612,27 @@
     <row r="37">
       <c r="B37" s="30" t="inlineStr">
         <is>
-          <t>FITOSANITARIOS CARCAIXENT, S.L.</t>
+          <t>FINCA DOÑA ANA C.B.</t>
         </is>
       </c>
       <c r="C37" s="31" t="inlineStr">
         <is>
-          <t>PT0020</t>
+          <t>C-CU1000</t>
         </is>
       </c>
       <c r="D37" s="30" t="inlineStr">
         <is>
-          <t>AGROPOTASION, 20 L</t>
+          <t>CODICOBRE, 1000 L</t>
         </is>
       </c>
       <c r="E37" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F37" s="18" t="n">
-        <v>1920</v>
+        <v>1000</v>
       </c>
       <c r="G37" s="18" t="n">
-        <v>1920</v>
+        <v>1000</v>
       </c>
       <c r="H37" s="18" t="n">
         <v>0</v>
@@ -8474,27 +8658,27 @@
     <row r="38">
       <c r="B38" s="27" t="inlineStr">
         <is>
-          <t>FITOSANITARIOS DRAGO S.L.U</t>
+          <t>FITOSANITARIOS CARCAIXENT, S.L.</t>
         </is>
       </c>
       <c r="C38" s="28" t="inlineStr">
         <is>
-          <t>AGXK0200</t>
+          <t>C-CU0005</t>
         </is>
       </c>
       <c r="D38" s="27" t="inlineStr">
         <is>
-          <t>AGROXILATO-K, 200 L</t>
+          <t>CODICOBRE, 5 L</t>
         </is>
       </c>
       <c r="E38" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F38" s="14" t="n">
-        <v>1600</v>
+        <v>100</v>
       </c>
       <c r="G38" s="14" t="n">
-        <v>1600</v>
+        <v>100</v>
       </c>
       <c r="H38" s="14" t="n">
         <v>0</v>
@@ -8520,27 +8704,27 @@
     <row r="39">
       <c r="B39" s="30" t="inlineStr">
         <is>
-          <t>FITOSANITARIOS DRAGO S.L.U</t>
+          <t>FITOSANITARIOS CARCAIXENT, S.L.</t>
         </is>
       </c>
       <c r="C39" s="31" t="inlineStr">
         <is>
-          <t>AGXK1000</t>
+          <t>G30020</t>
         </is>
       </c>
       <c r="D39" s="30" t="inlineStr">
         <is>
-          <t>AGROXILATO-K, 1000 L</t>
+          <t>GREEN-UP, 20 L</t>
         </is>
       </c>
       <c r="E39" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F39" s="18" t="n">
-        <v>10000</v>
+        <v>200</v>
       </c>
       <c r="G39" s="18" t="n">
-        <v>10000</v>
+        <v>200</v>
       </c>
       <c r="H39" s="18" t="n">
         <v>0</v>
@@ -8566,27 +8750,27 @@
     <row r="40">
       <c r="B40" s="27" t="inlineStr">
         <is>
-          <t>FITOSANITARIOS DRAGO S.L.U</t>
+          <t>FITOSANITARIOS CARCAIXENT, S.L.</t>
         </is>
       </c>
       <c r="C40" s="28" t="inlineStr">
         <is>
-          <t>C-CU0001</t>
+          <t>HST0020</t>
         </is>
       </c>
       <c r="D40" s="27" t="inlineStr">
         <is>
-          <t>CODICOBRE, 1 L</t>
+          <t>HIDROSTRESS-40, 20 L</t>
         </is>
       </c>
       <c r="E40" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F40" s="14" t="n">
-        <v>24</v>
+        <v>100</v>
       </c>
       <c r="G40" s="14" t="n">
-        <v>24</v>
+        <v>100</v>
       </c>
       <c r="H40" s="14" t="n">
         <v>0</v>
@@ -8612,27 +8796,27 @@
     <row r="41">
       <c r="B41" s="30" t="inlineStr">
         <is>
-          <t>FITOSANITARIOS DRAGO S.L.U</t>
+          <t>FITOSANITARIOS CARCAIXENT, S.L.</t>
         </is>
       </c>
       <c r="C41" s="31" t="inlineStr">
         <is>
-          <t>JF0020</t>
+          <t>PT0005</t>
         </is>
       </c>
       <c r="D41" s="30" t="inlineStr">
         <is>
-          <t>DRAGO-FOS, 20 L</t>
+          <t>AGROPOTASION, 5 L</t>
         </is>
       </c>
       <c r="E41" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F41" s="18" t="n">
-        <v>1280</v>
+        <v>600</v>
       </c>
       <c r="G41" s="18" t="n">
-        <v>1280</v>
+        <v>600</v>
       </c>
       <c r="H41" s="18" t="n">
         <v>0</v>
@@ -8658,27 +8842,27 @@
     <row r="42">
       <c r="B42" s="27" t="inlineStr">
         <is>
-          <t>FITOSANITARIOS DRAGO S.L.U</t>
+          <t>FITOSANITARIOS CARCAIXENT, S.L.</t>
         </is>
       </c>
       <c r="C42" s="28" t="inlineStr">
         <is>
-          <t>PHD0005</t>
+          <t>PT0020</t>
         </is>
       </c>
       <c r="D42" s="27" t="inlineStr">
         <is>
-          <t xml:space="preserve">PH-DOWNER, 5 L   </t>
+          <t>AGROPOTASION, 20 L</t>
         </is>
       </c>
       <c r="E42" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F42" s="14" t="n">
-        <v>400</v>
+        <v>1920</v>
       </c>
       <c r="G42" s="14" t="n">
-        <v>400</v>
+        <v>1920</v>
       </c>
       <c r="H42" s="14" t="n">
         <v>0</v>
@@ -8709,22 +8893,22 @@
       </c>
       <c r="C43" s="31" t="inlineStr">
         <is>
-          <t>PHD0020</t>
+          <t>AGXK0200</t>
         </is>
       </c>
       <c r="D43" s="30" t="inlineStr">
         <is>
-          <t>PH-DOWNER, 20 L</t>
+          <t>AGROXILATO-K, 200 L</t>
         </is>
       </c>
       <c r="E43" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F43" s="18" t="n">
-        <v>640</v>
+        <v>1600</v>
       </c>
       <c r="G43" s="18" t="n">
-        <v>640</v>
+        <v>1600</v>
       </c>
       <c r="H43" s="18" t="n">
         <v>0</v>
@@ -8755,22 +8939,22 @@
       </c>
       <c r="C44" s="28" t="inlineStr">
         <is>
-          <t>S0200</t>
+          <t>AGXK1000</t>
         </is>
       </c>
       <c r="D44" s="27" t="inlineStr">
         <is>
-          <t>SAL-WAX STAR, 200 L</t>
+          <t>AGROXILATO-K, 1000 L</t>
         </is>
       </c>
       <c r="E44" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F44" s="14" t="n">
-        <v>800</v>
+        <v>10000</v>
       </c>
       <c r="G44" s="14" t="n">
-        <v>800</v>
+        <v>10000</v>
       </c>
       <c r="H44" s="14" t="n">
         <v>0</v>
@@ -8801,22 +8985,22 @@
       </c>
       <c r="C45" s="31" t="inlineStr">
         <is>
-          <t>SS0020</t>
+          <t>C-CU0001</t>
         </is>
       </c>
       <c r="D45" s="30" t="inlineStr">
         <is>
-          <t>SALWAX-CA, 20 KG</t>
+          <t>CODICOBRE, 1 L</t>
         </is>
       </c>
       <c r="E45" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F45" s="18" t="n">
-        <v>40</v>
+        <v>24</v>
       </c>
       <c r="G45" s="18" t="n">
-        <v>40</v>
+        <v>24</v>
       </c>
       <c r="H45" s="18" t="n">
         <v>0</v>
@@ -8842,27 +9026,27 @@
     <row r="46">
       <c r="B46" s="27" t="inlineStr">
         <is>
-          <t>FITOXENT S.C.L.V.</t>
+          <t>FITOSANITARIOS DRAGO S.L.U</t>
         </is>
       </c>
       <c r="C46" s="28" t="inlineStr">
         <is>
-          <t>FTK0005</t>
+          <t>JF0020</t>
         </is>
       </c>
       <c r="D46" s="27" t="inlineStr">
         <is>
-          <t>FITOKONTROL CA FLOW, 5 KG</t>
+          <t>DRAGO-FOS, 20 L</t>
         </is>
       </c>
       <c r="E46" s="14" t="n">
-        <v>4400</v>
+        <v>0</v>
       </c>
       <c r="F46" s="14" t="n">
-        <v>4400</v>
+        <v>1280</v>
       </c>
       <c r="G46" s="14" t="n">
-        <v>4400</v>
+        <v>1280</v>
       </c>
       <c r="H46" s="14" t="n">
         <v>0</v>
@@ -8881,34 +9065,34 @@
       </c>
       <c r="L46" s="29" t="inlineStr">
         <is>
-          <t>Superado</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="B47" s="30" t="inlineStr">
         <is>
-          <t>FITOXENT S.C.L.V.</t>
+          <t>FITOSANITARIOS DRAGO S.L.U</t>
         </is>
       </c>
       <c r="C47" s="31" t="inlineStr">
         <is>
-          <t>PT0020</t>
+          <t>PHD0005</t>
         </is>
       </c>
       <c r="D47" s="30" t="inlineStr">
         <is>
-          <t>AGROPOTASION, 20 L</t>
+          <t xml:space="preserve">PH-DOWNER, 5 L   </t>
         </is>
       </c>
       <c r="E47" s="18" t="n">
-        <v>2560</v>
+        <v>0</v>
       </c>
       <c r="F47" s="18" t="n">
-        <v>1280</v>
+        <v>400</v>
       </c>
       <c r="G47" s="18" t="n">
-        <v>1280</v>
+        <v>400</v>
       </c>
       <c r="H47" s="18" t="n">
         <v>0</v>
@@ -8925,36 +9109,36 @@
         <f>IF(E47&gt;0, F47/E47, IF(F47&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L47" s="32" t="inlineStr">
-        <is>
-          <t>En Curso</t>
+      <c r="L47" s="29" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="B48" s="27" t="inlineStr">
         <is>
-          <t>FITOXENT S.C.L.V.</t>
+          <t>FITOSANITARIOS DRAGO S.L.U</t>
         </is>
       </c>
       <c r="C48" s="28" t="inlineStr">
         <is>
-          <t>S0020</t>
+          <t>PHD0020</t>
         </is>
       </c>
       <c r="D48" s="27" t="inlineStr">
         <is>
-          <t>SALWAX STAR, 20 L</t>
+          <t>PH-DOWNER, 20 L</t>
         </is>
       </c>
       <c r="E48" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F48" s="14" t="n">
-        <v>200</v>
+        <v>640</v>
       </c>
       <c r="G48" s="14" t="n">
-        <v>200</v>
+        <v>640</v>
       </c>
       <c r="H48" s="14" t="n">
         <v>0</v>
@@ -8977,48 +9161,278 @@
         </is>
       </c>
     </row>
-    <row r="49" ht="24" customHeight="1">
-      <c r="B49" s="20" t="inlineStr">
+    <row r="49">
+      <c r="B49" s="30" t="inlineStr">
+        <is>
+          <t>FITOSANITARIOS DRAGO S.L.U</t>
+        </is>
+      </c>
+      <c r="C49" s="31" t="inlineStr">
+        <is>
+          <t>S0200</t>
+        </is>
+      </c>
+      <c r="D49" s="30" t="inlineStr">
+        <is>
+          <t>SAL-WAX STAR, 200 L</t>
+        </is>
+      </c>
+      <c r="E49" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F49" s="18" t="n">
+        <v>800</v>
+      </c>
+      <c r="G49" s="18" t="n">
+        <v>800</v>
+      </c>
+      <c r="H49" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="I49" s="18">
+        <f>MAX(0, E49-F49)</f>
+        <v/>
+      </c>
+      <c r="J49" s="18">
+        <f>F49-E49</f>
+        <v/>
+      </c>
+      <c r="K49" s="19">
+        <f>IF(E49&gt;0, F49/E49, IF(F49&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L49" s="29" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="B50" s="27" t="inlineStr">
+        <is>
+          <t>FITOSANITARIOS DRAGO S.L.U</t>
+        </is>
+      </c>
+      <c r="C50" s="28" t="inlineStr">
+        <is>
+          <t>SS0020</t>
+        </is>
+      </c>
+      <c r="D50" s="27" t="inlineStr">
+        <is>
+          <t>SALWAX-CA, 20 KG</t>
+        </is>
+      </c>
+      <c r="E50" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F50" s="14" t="n">
+        <v>40</v>
+      </c>
+      <c r="G50" s="14" t="n">
+        <v>40</v>
+      </c>
+      <c r="H50" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I50" s="14">
+        <f>MAX(0, E50-F50)</f>
+        <v/>
+      </c>
+      <c r="J50" s="14">
+        <f>F50-E50</f>
+        <v/>
+      </c>
+      <c r="K50" s="15">
+        <f>IF(E50&gt;0, F50/E50, IF(F50&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L50" s="29" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="B51" s="30" t="inlineStr">
+        <is>
+          <t>FITOXENT S.C.L.V.</t>
+        </is>
+      </c>
+      <c r="C51" s="31" t="inlineStr">
+        <is>
+          <t>FTK0005</t>
+        </is>
+      </c>
+      <c r="D51" s="30" t="inlineStr">
+        <is>
+          <t>FITOKONTROL CA FLOW, 5 KG</t>
+        </is>
+      </c>
+      <c r="E51" s="18" t="n">
+        <v>4400</v>
+      </c>
+      <c r="F51" s="18" t="n">
+        <v>4400</v>
+      </c>
+      <c r="G51" s="18" t="n">
+        <v>4400</v>
+      </c>
+      <c r="H51" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="I51" s="18">
+        <f>MAX(0, E51-F51)</f>
+        <v/>
+      </c>
+      <c r="J51" s="18">
+        <f>F51-E51</f>
+        <v/>
+      </c>
+      <c r="K51" s="19">
+        <f>IF(E51&gt;0, F51/E51, IF(F51&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L51" s="29" t="inlineStr">
+        <is>
+          <t>Superado</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="B52" s="27" t="inlineStr">
+        <is>
+          <t>FITOXENT S.C.L.V.</t>
+        </is>
+      </c>
+      <c r="C52" s="28" t="inlineStr">
+        <is>
+          <t>PT0020</t>
+        </is>
+      </c>
+      <c r="D52" s="27" t="inlineStr">
+        <is>
+          <t>AGROPOTASION, 20 L</t>
+        </is>
+      </c>
+      <c r="E52" s="14" t="n">
+        <v>2560</v>
+      </c>
+      <c r="F52" s="14" t="n">
+        <v>1280</v>
+      </c>
+      <c r="G52" s="14" t="n">
+        <v>1280</v>
+      </c>
+      <c r="H52" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I52" s="14">
+        <f>MAX(0, E52-F52)</f>
+        <v/>
+      </c>
+      <c r="J52" s="14">
+        <f>F52-E52</f>
+        <v/>
+      </c>
+      <c r="K52" s="15">
+        <f>IF(E52&gt;0, F52/E52, IF(F52&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L52" s="32" t="inlineStr">
+        <is>
+          <t>En Curso</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="B53" s="30" t="inlineStr">
+        <is>
+          <t>FITOXENT S.C.L.V.</t>
+        </is>
+      </c>
+      <c r="C53" s="31" t="inlineStr">
+        <is>
+          <t>S0020</t>
+        </is>
+      </c>
+      <c r="D53" s="30" t="inlineStr">
+        <is>
+          <t>SALWAX STAR, 20 L</t>
+        </is>
+      </c>
+      <c r="E53" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F53" s="18" t="n">
+        <v>200</v>
+      </c>
+      <c r="G53" s="18" t="n">
+        <v>200</v>
+      </c>
+      <c r="H53" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="I53" s="18">
+        <f>MAX(0, E53-F53)</f>
+        <v/>
+      </c>
+      <c r="J53" s="18">
+        <f>F53-E53</f>
+        <v/>
+      </c>
+      <c r="K53" s="19">
+        <f>IF(E53&gt;0, F53/E53, IF(F53&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L53" s="29" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="24" customHeight="1">
+      <c r="B54" s="20" t="inlineStr">
         <is>
           <t>TOTAL JAVIER</t>
         </is>
       </c>
-      <c r="C49" s="33" t="inlineStr">
-        <is>
-          <t>184 líneas</t>
-        </is>
-      </c>
-      <c r="D49" s="34" t="inlineStr"/>
-      <c r="E49" s="22">
-        <f>SUM(E10:E48)</f>
-        <v/>
-      </c>
-      <c r="F49" s="22">
-        <f>SUM(F10:F48)</f>
-        <v/>
-      </c>
-      <c r="G49" s="22">
-        <f>SUM(G10:G48)</f>
-        <v/>
-      </c>
-      <c r="H49" s="22">
-        <f>SUM(H10:H48)</f>
-        <v/>
-      </c>
-      <c r="I49" s="22">
-        <f>SUM(I10:I48)</f>
-        <v/>
-      </c>
-      <c r="J49" s="22">
-        <f>SUM(J10:J48)</f>
-        <v/>
-      </c>
-      <c r="K49" s="23">
-        <f>IF(E49&gt;0, F49/E49, 0)</f>
-        <v/>
-      </c>
-      <c r="L49" s="21">
-        <f>IF(K49&gt;=1, "SUPERADO", "EN CURSO")</f>
+      <c r="C54" s="33" t="inlineStr">
+        <is>
+          <t>186 líneas</t>
+        </is>
+      </c>
+      <c r="D54" s="34" t="inlineStr"/>
+      <c r="E54" s="22">
+        <f>SUM(E10:E53)</f>
+        <v/>
+      </c>
+      <c r="F54" s="22">
+        <f>SUM(F10:F53)</f>
+        <v/>
+      </c>
+      <c r="G54" s="22">
+        <f>SUM(G10:G53)</f>
+        <v/>
+      </c>
+      <c r="H54" s="22">
+        <f>SUM(H10:H53)</f>
+        <v/>
+      </c>
+      <c r="I54" s="22">
+        <f>SUM(I10:I53)</f>
+        <v/>
+      </c>
+      <c r="J54" s="22">
+        <f>SUM(J10:J53)</f>
+        <v/>
+      </c>
+      <c r="K54" s="23">
+        <f>IF(E54&gt;0, F54/E54, 0)</f>
+        <v/>
+      </c>
+      <c r="L54" s="21">
+        <f>IF(K54&gt;=1, "SUPERADO", "EN CURSO")</f>
         <v/>
       </c>
     </row>
@@ -9074,7 +9488,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 29/09/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 30/09/2026</t>
         </is>
       </c>
     </row>
@@ -9598,7 +10012,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:L30"/>
+  <dimension ref="B2:L33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -9625,7 +10039,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 29/09/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 30/09/2026</t>
         </is>
       </c>
     </row>
@@ -9670,25 +10084,25 @@
       <c r="C6" s="4" t="n"/>
       <c r="D6" s="24" t="inlineStr">
         <is>
-          <t>7,860 u</t>
+          <t>8,560 u</t>
         </is>
       </c>
       <c r="E6" s="4" t="n"/>
       <c r="F6" s="37" t="inlineStr">
         <is>
-          <t>45.3%</t>
+          <t>49.4%</t>
         </is>
       </c>
       <c r="G6" s="4" t="n"/>
       <c r="H6" s="37" t="inlineStr">
         <is>
-          <t>9,480 u</t>
+          <t>8,780 u</t>
         </is>
       </c>
       <c r="I6" s="4" t="n"/>
       <c r="J6" s="24" t="inlineStr">
         <is>
-          <t>0 u</t>
+          <t>700 u</t>
         </is>
       </c>
       <c r="K6" s="4" t="n"/>
@@ -10593,25 +11007,25 @@
       </c>
       <c r="C28" s="28" t="inlineStr">
         <is>
-          <t>SPCE2B0020</t>
+          <t>C-L0020</t>
         </is>
       </c>
       <c r="D28" s="27" t="inlineStr">
         <is>
-          <t>SPRINTENE CON BORO, 20 L</t>
+          <t>CODIBOR-L, 20 L</t>
         </is>
       </c>
       <c r="E28" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F28" s="14" t="n">
-        <v>200</v>
+        <v>320</v>
       </c>
       <c r="G28" s="14" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="H28" s="14" t="n">
-        <v>0</v>
+        <v>320</v>
       </c>
       <c r="I28" s="14">
         <f>MAX(0, E28-F28)</f>
@@ -10639,25 +11053,25 @@
       </c>
       <c r="C29" s="31" t="inlineStr">
         <is>
-          <t>SS0005</t>
+          <t>C-MB0005</t>
         </is>
       </c>
       <c r="D29" s="30" t="inlineStr">
         <is>
-          <t>SAL-WAX-Ca sólido, 5 KG</t>
+          <t>CODIFOL-MB, 5 L</t>
         </is>
       </c>
       <c r="E29" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F29" s="18" t="n">
-        <v>300</v>
+        <v>60</v>
       </c>
       <c r="G29" s="18" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="H29" s="18" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="I29" s="18">
         <f>MAX(0, E29-F29)</f>
@@ -10677,48 +11091,186 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="24" customHeight="1">
-      <c r="B30" s="20" t="inlineStr">
+    <row r="30">
+      <c r="B30" s="27" t="inlineStr">
+        <is>
+          <t>FITOMURCIA S.L.</t>
+        </is>
+      </c>
+      <c r="C30" s="28" t="inlineStr">
+        <is>
+          <t>C-MB0020</t>
+        </is>
+      </c>
+      <c r="D30" s="27" t="inlineStr">
+        <is>
+          <t>CODIFOL-MB, 20 L</t>
+        </is>
+      </c>
+      <c r="E30" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" s="14" t="n">
+        <v>320</v>
+      </c>
+      <c r="G30" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H30" s="14" t="n">
+        <v>320</v>
+      </c>
+      <c r="I30" s="14">
+        <f>MAX(0, E30-F30)</f>
+        <v/>
+      </c>
+      <c r="J30" s="14">
+        <f>F30-E30</f>
+        <v/>
+      </c>
+      <c r="K30" s="15">
+        <f>IF(E30&gt;0, F30/E30, IF(F30&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L30" s="29" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="30" t="inlineStr">
+        <is>
+          <t>FITOMURCIA S.L.</t>
+        </is>
+      </c>
+      <c r="C31" s="31" t="inlineStr">
+        <is>
+          <t>SPCE2B0020</t>
+        </is>
+      </c>
+      <c r="D31" s="30" t="inlineStr">
+        <is>
+          <t>SPRINTENE CON BORO, 20 L</t>
+        </is>
+      </c>
+      <c r="E31" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" s="18" t="n">
+        <v>200</v>
+      </c>
+      <c r="G31" s="18" t="n">
+        <v>200</v>
+      </c>
+      <c r="H31" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="I31" s="18">
+        <f>MAX(0, E31-F31)</f>
+        <v/>
+      </c>
+      <c r="J31" s="18">
+        <f>F31-E31</f>
+        <v/>
+      </c>
+      <c r="K31" s="19">
+        <f>IF(E31&gt;0, F31/E31, IF(F31&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L31" s="29" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="27" t="inlineStr">
+        <is>
+          <t>FITOMURCIA S.L.</t>
+        </is>
+      </c>
+      <c r="C32" s="28" t="inlineStr">
+        <is>
+          <t>SS0005</t>
+        </is>
+      </c>
+      <c r="D32" s="27" t="inlineStr">
+        <is>
+          <t>SAL-WAX-Ca sólido, 5 KG</t>
+        </is>
+      </c>
+      <c r="E32" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F32" s="14" t="n">
+        <v>300</v>
+      </c>
+      <c r="G32" s="14" t="n">
+        <v>300</v>
+      </c>
+      <c r="H32" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I32" s="14">
+        <f>MAX(0, E32-F32)</f>
+        <v/>
+      </c>
+      <c r="J32" s="14">
+        <f>F32-E32</f>
+        <v/>
+      </c>
+      <c r="K32" s="15">
+        <f>IF(E32&gt;0, F32/E32, IF(F32&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L32" s="29" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="24" customHeight="1">
+      <c r="B33" s="20" t="inlineStr">
         <is>
           <t>TOTAL PEDRO</t>
         </is>
       </c>
-      <c r="C30" s="33" t="inlineStr">
+      <c r="C33" s="33" t="inlineStr">
         <is>
           <t>106 líneas</t>
         </is>
       </c>
-      <c r="D30" s="34" t="inlineStr"/>
-      <c r="E30" s="22">
-        <f>SUM(E10:E29)</f>
-        <v/>
-      </c>
-      <c r="F30" s="22">
-        <f>SUM(F10:F29)</f>
-        <v/>
-      </c>
-      <c r="G30" s="22">
-        <f>SUM(G10:G29)</f>
-        <v/>
-      </c>
-      <c r="H30" s="22">
-        <f>SUM(H10:H29)</f>
-        <v/>
-      </c>
-      <c r="I30" s="22">
-        <f>SUM(I10:I29)</f>
-        <v/>
-      </c>
-      <c r="J30" s="22">
-        <f>SUM(J10:J29)</f>
-        <v/>
-      </c>
-      <c r="K30" s="23">
-        <f>IF(E30&gt;0, F30/E30, 0)</f>
-        <v/>
-      </c>
-      <c r="L30" s="21">
-        <f>IF(K30&gt;=1, "SUPERADO", "EN CURSO")</f>
+      <c r="D33" s="34" t="inlineStr"/>
+      <c r="E33" s="22">
+        <f>SUM(E10:E32)</f>
+        <v/>
+      </c>
+      <c r="F33" s="22">
+        <f>SUM(F10:F32)</f>
+        <v/>
+      </c>
+      <c r="G33" s="22">
+        <f>SUM(G10:G32)</f>
+        <v/>
+      </c>
+      <c r="H33" s="22">
+        <f>SUM(H10:H32)</f>
+        <v/>
+      </c>
+      <c r="I33" s="22">
+        <f>SUM(I10:I32)</f>
+        <v/>
+      </c>
+      <c r="J33" s="22">
+        <f>SUM(J10:J32)</f>
+        <v/>
+      </c>
+      <c r="K33" s="23">
+        <f>IF(E33&gt;0, F33/E33, 0)</f>
+        <v/>
+      </c>
+      <c r="L33" s="21">
+        <f>IF(K33&gt;=1, "SUPERADO", "EN CURSO")</f>
         <v/>
       </c>
     </row>
@@ -10747,7 +11299,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:L36"/>
+  <dimension ref="B2:L44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -10774,7 +11326,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 29/09/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 30/09/2026</t>
         </is>
       </c>
     </row>
@@ -10785,19 +11337,19 @@
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D5" s="5" t="inlineStr">
         <is>
           <t>PEDIDOS REALES (U)</t>
         </is>
       </c>
       <c r="E5" s="4" t="n"/>
-      <c r="F5" s="6" t="inlineStr">
+      <c r="F5" s="5" t="inlineStr">
         <is>
           <t>% CONSECUCIÓN</t>
         </is>
       </c>
       <c r="G5" s="4" t="n"/>
-      <c r="H5" s="6" t="inlineStr">
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>FALTA CONSEGUIR (GAP)</t>
         </is>
@@ -10817,27 +11369,27 @@
         </is>
       </c>
       <c r="C6" s="4" t="n"/>
-      <c r="D6" s="24" t="inlineStr">
-        <is>
-          <t>44,724 u</t>
+      <c r="D6" s="25" t="inlineStr">
+        <is>
+          <t>54,908 u</t>
         </is>
       </c>
       <c r="E6" s="4" t="n"/>
-      <c r="F6" s="37" t="inlineStr">
-        <is>
-          <t>97.2%</t>
+      <c r="F6" s="25" t="inlineStr">
+        <is>
+          <t>119.4%</t>
         </is>
       </c>
       <c r="G6" s="4" t="n"/>
-      <c r="H6" s="37" t="inlineStr">
-        <is>
-          <t>1,276 u</t>
+      <c r="H6" s="25" t="inlineStr">
+        <is>
+          <t>0 u</t>
         </is>
       </c>
       <c r="I6" s="4" t="n"/>
       <c r="J6" s="24" t="inlineStr">
         <is>
-          <t>21,674 u</t>
+          <t>31,858 u</t>
         </is>
       </c>
       <c r="K6" s="4" t="n"/>
@@ -10955,30 +11507,30 @@
     <row r="11">
       <c r="B11" s="30" t="inlineStr">
         <is>
-          <t>ECUAQUIMICA</t>
+          <t>CAMPO ABIERTO, S.A.S.</t>
         </is>
       </c>
       <c r="C11" s="31" t="inlineStr">
         <is>
-          <t>AN0005</t>
+          <t>AGXCR0001</t>
         </is>
       </c>
       <c r="D11" s="30" t="inlineStr">
         <is>
-          <t>ALCAPLANT NEW</t>
+          <t>AGROXILATO-K</t>
         </is>
       </c>
       <c r="E11" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F11" s="18" t="n">
-        <v>2200</v>
+        <v>840</v>
       </c>
       <c r="G11" s="18" t="n">
         <v>0</v>
       </c>
       <c r="H11" s="18" t="n">
-        <v>2200</v>
+        <v>840</v>
       </c>
       <c r="I11" s="18">
         <f>MAX(0, E11-F11)</f>
@@ -11001,30 +11553,30 @@
     <row r="12">
       <c r="B12" s="27" t="inlineStr">
         <is>
-          <t>ECUAQUIMICA</t>
+          <t>CAMPO ABIERTO, S.A.S.</t>
         </is>
       </c>
       <c r="C12" s="28" t="inlineStr">
         <is>
-          <t>AN0020</t>
+          <t>AGXCR0020</t>
         </is>
       </c>
       <c r="D12" s="27" t="inlineStr">
         <is>
-          <t>ALCAPLANT NEW</t>
+          <t>AGROXILATO-K</t>
         </is>
       </c>
       <c r="E12" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F12" s="14" t="n">
-        <v>6600</v>
+        <v>2000</v>
       </c>
       <c r="G12" s="14" t="n">
         <v>0</v>
       </c>
       <c r="H12" s="14" t="n">
-        <v>6600</v>
+        <v>2000</v>
       </c>
       <c r="I12" s="14">
         <f>MAX(0, E12-F12)</f>
@@ -11047,30 +11599,30 @@
     <row r="13">
       <c r="B13" s="30" t="inlineStr">
         <is>
-          <t>EUROFERTIL, S.A.</t>
+          <t>CAMPO ABIERTO, S.A.S.</t>
         </is>
       </c>
       <c r="C13" s="31" t="inlineStr">
         <is>
-          <t>F-A1000</t>
+          <t>AN0020</t>
         </is>
       </c>
       <c r="D13" s="30" t="inlineStr">
         <is>
-          <t>FITOLIN AGRO</t>
+          <t>ALCAPLANT NEW</t>
         </is>
       </c>
       <c r="E13" s="18" t="n">
-        <v>2000</v>
+        <v>0</v>
       </c>
       <c r="F13" s="18" t="n">
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="G13" s="18" t="n">
         <v>0</v>
       </c>
       <c r="H13" s="18" t="n">
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="I13" s="18">
         <f>MAX(0, E13-F13)</f>
@@ -11084,39 +11636,39 @@
         <f>IF(E13&gt;0, F13/E13, IF(F13&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L13" s="35" t="inlineStr">
-        <is>
-          <t>Sin Pedido</t>
+      <c r="L13" s="29" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="B14" s="27" t="inlineStr">
         <is>
-          <t xml:space="preserve">EUROFERTIL, S.A.    </t>
+          <t>CAMPO ABIERTO, S.A.S.</t>
         </is>
       </c>
       <c r="C14" s="28" t="inlineStr">
         <is>
-          <t>AGXCR1000</t>
+          <t>G30001</t>
         </is>
       </c>
       <c r="D14" s="27" t="inlineStr">
         <is>
-          <t>AGROXILATO-K, 1000 L</t>
+          <t>GREEN-UP, 1 L</t>
         </is>
       </c>
       <c r="E14" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F14" s="14" t="n">
-        <v>3000</v>
+        <v>240</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="H14" s="14" t="n">
-        <v>0</v>
+        <v>240</v>
       </c>
       <c r="I14" s="14">
         <f>MAX(0, E14-F14)</f>
@@ -11139,30 +11691,30 @@
     <row r="15">
       <c r="B15" s="30" t="inlineStr">
         <is>
-          <t xml:space="preserve">EUROFERTIL, S.A.    </t>
+          <t>CAMPO ABIERTO, S.A.S.</t>
         </is>
       </c>
       <c r="C15" s="31" t="inlineStr">
         <is>
-          <t>AN0005</t>
+          <t>SSEG0001</t>
         </is>
       </c>
       <c r="D15" s="30" t="inlineStr">
         <is>
-          <t>ALCAPLANT, 5 KG</t>
+          <t>SALWAX CALCIO</t>
         </is>
       </c>
       <c r="E15" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F15" s="18" t="n">
-        <v>3300</v>
+        <v>324</v>
       </c>
       <c r="G15" s="18" t="n">
-        <v>3300</v>
+        <v>0</v>
       </c>
       <c r="H15" s="18" t="n">
-        <v>0</v>
+        <v>324</v>
       </c>
       <c r="I15" s="18">
         <f>MAX(0, E15-F15)</f>
@@ -11185,30 +11737,30 @@
     <row r="16">
       <c r="B16" s="27" t="inlineStr">
         <is>
-          <t xml:space="preserve">EUROFERTIL, S.A.    </t>
+          <t>CAMPO ABIERTO, S.A.S.</t>
         </is>
       </c>
       <c r="C16" s="28" t="inlineStr">
         <is>
-          <t>AN0020</t>
+          <t>SSEG0005</t>
         </is>
       </c>
       <c r="D16" s="27" t="inlineStr">
         <is>
-          <t>ALCAPLANT, 20 KG</t>
+          <t>SALWAX CALCIO EGIPTO, 5 KG</t>
         </is>
       </c>
       <c r="E16" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F16" s="14" t="n">
-        <v>4400</v>
+        <v>480</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>4400</v>
+        <v>0</v>
       </c>
       <c r="H16" s="14" t="n">
-        <v>0</v>
+        <v>480</v>
       </c>
       <c r="I16" s="14">
         <f>MAX(0, E16-F16)</f>
@@ -11231,30 +11783,30 @@
     <row r="17">
       <c r="B17" s="30" t="inlineStr">
         <is>
-          <t xml:space="preserve">EUROFERTIL, S.A.    </t>
+          <t>CAMPO ABIERTO, S.A.S.</t>
         </is>
       </c>
       <c r="C17" s="31" t="inlineStr">
         <is>
-          <t>B1000</t>
+          <t>SSEG0020</t>
         </is>
       </c>
       <c r="D17" s="30" t="inlineStr">
         <is>
-          <t>FORTALEZA, 1000 L</t>
+          <t>SALWAX CALCIO EGIPTO, 20 KG</t>
         </is>
       </c>
       <c r="E17" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F17" s="18" t="n">
-        <v>2000</v>
+        <v>1200</v>
       </c>
       <c r="G17" s="18" t="n">
-        <v>2000</v>
+        <v>0</v>
       </c>
       <c r="H17" s="18" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="I17" s="18">
         <f>MAX(0, E17-F17)</f>
@@ -11277,30 +11829,30 @@
     <row r="18">
       <c r="B18" s="27" t="inlineStr">
         <is>
-          <t xml:space="preserve">EUROFERTIL, S.A.    </t>
+          <t>ECUAQUIMICA</t>
         </is>
       </c>
       <c r="C18" s="28" t="inlineStr">
         <is>
-          <t>C-CU1000</t>
+          <t>AN0005</t>
         </is>
       </c>
       <c r="D18" s="27" t="inlineStr">
         <is>
-          <t>CODICOBRE, 1000 L</t>
+          <t>ALCAPLANT NEW</t>
         </is>
       </c>
       <c r="E18" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F18" s="14" t="n">
-        <v>1000</v>
+        <v>2200</v>
       </c>
       <c r="G18" s="14" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="H18" s="14" t="n">
-        <v>0</v>
+        <v>2200</v>
       </c>
       <c r="I18" s="14">
         <f>MAX(0, E18-F18)</f>
@@ -11323,30 +11875,30 @@
     <row r="19">
       <c r="B19" s="30" t="inlineStr">
         <is>
-          <t xml:space="preserve">EUROFERTIL, S.A.    </t>
+          <t>ECUAQUIMICA</t>
         </is>
       </c>
       <c r="C19" s="31" t="inlineStr">
         <is>
-          <t>CODIR1000</t>
+          <t>AN0020</t>
         </is>
       </c>
       <c r="D19" s="30" t="inlineStr">
         <is>
-          <t>CODIRESIST, 1000 L</t>
+          <t>ALCAPLANT NEW</t>
         </is>
       </c>
       <c r="E19" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F19" s="18" t="n">
-        <v>1000</v>
+        <v>6600</v>
       </c>
       <c r="G19" s="18" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="H19" s="18" t="n">
-        <v>0</v>
+        <v>6600</v>
       </c>
       <c r="I19" s="18">
         <f>MAX(0, E19-F19)</f>
@@ -11369,27 +11921,27 @@
     <row r="20">
       <c r="B20" s="27" t="inlineStr">
         <is>
-          <t xml:space="preserve">EUROFERTIL, S.A.    </t>
+          <t>EUROFERTIL, S.A.</t>
         </is>
       </c>
       <c r="C20" s="28" t="inlineStr">
         <is>
-          <t>DECA0005</t>
+          <t>F-A1000</t>
         </is>
       </c>
       <c r="D20" s="27" t="inlineStr">
         <is>
-          <t>DEFENS-CA-AE, 5 KG</t>
+          <t>FITOLIN AGRO</t>
         </is>
       </c>
       <c r="E20" s="14" t="n">
-        <v>0</v>
+        <v>2000</v>
       </c>
       <c r="F20" s="14" t="n">
-        <v>750</v>
+        <v>0</v>
       </c>
       <c r="G20" s="14" t="n">
-        <v>750</v>
+        <v>0</v>
       </c>
       <c r="H20" s="14" t="n">
         <v>0</v>
@@ -11406,9 +11958,9 @@
         <f>IF(E20&gt;0, F20/E20, IF(F20&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L20" s="29" t="inlineStr">
-        <is>
-          <t>Extra Estimación</t>
+      <c r="L20" s="35" t="inlineStr">
+        <is>
+          <t>Sin Pedido</t>
         </is>
       </c>
     </row>
@@ -11420,22 +11972,22 @@
       </c>
       <c r="C21" s="31" t="inlineStr">
         <is>
-          <t>F-A1000</t>
+          <t>AGXCR1000</t>
         </is>
       </c>
       <c r="D21" s="30" t="inlineStr">
         <is>
-          <t xml:space="preserve">FITOLIN AGRO, 1000 L </t>
+          <t>AGROXILATO-K, 1000 L</t>
         </is>
       </c>
       <c r="E21" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F21" s="18" t="n">
-        <v>1000</v>
+        <v>3000</v>
       </c>
       <c r="G21" s="18" t="n">
-        <v>1000</v>
+        <v>3000</v>
       </c>
       <c r="H21" s="18" t="n">
         <v>0</v>
@@ -11466,22 +12018,22 @@
       </c>
       <c r="C22" s="28" t="inlineStr">
         <is>
-          <t>NB1000</t>
+          <t>AN0005</t>
         </is>
       </c>
       <c r="D22" s="27" t="inlineStr">
         <is>
-          <t>NITROBALANCE, 1000 L</t>
+          <t>ALCAPLANT, 5 KG</t>
         </is>
       </c>
       <c r="E22" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F22" s="14" t="n">
-        <v>2000</v>
+        <v>3300</v>
       </c>
       <c r="G22" s="14" t="n">
-        <v>2000</v>
+        <v>3300</v>
       </c>
       <c r="H22" s="14" t="n">
         <v>0</v>
@@ -11512,22 +12064,22 @@
       </c>
       <c r="C23" s="31" t="inlineStr">
         <is>
-          <t>SS0020</t>
+          <t>AN0020</t>
         </is>
       </c>
       <c r="D23" s="30" t="inlineStr">
         <is>
-          <t>SAL WAX MAX, 20 KG</t>
+          <t>ALCAPLANT, 20 KG</t>
         </is>
       </c>
       <c r="E23" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F23" s="18" t="n">
-        <v>1600</v>
+        <v>4400</v>
       </c>
       <c r="G23" s="18" t="n">
-        <v>1600</v>
+        <v>4400</v>
       </c>
       <c r="H23" s="18" t="n">
         <v>0</v>
@@ -11553,27 +12105,27 @@
     <row r="24">
       <c r="B24" s="27" t="inlineStr">
         <is>
-          <t>LEKKERBIO B.V.</t>
+          <t xml:space="preserve">EUROFERTIL, S.A.    </t>
         </is>
       </c>
       <c r="C24" s="28" t="inlineStr">
         <is>
-          <t>AO0020</t>
+          <t>B1000</t>
         </is>
       </c>
       <c r="D24" s="27" t="inlineStr">
         <is>
-          <t>ALCAPLANT NEW</t>
+          <t>FORTALEZA, 1000 L</t>
         </is>
       </c>
       <c r="E24" s="14" t="n">
-        <v>44000</v>
+        <v>0</v>
       </c>
       <c r="F24" s="14" t="n">
-        <v>0</v>
+        <v>2000</v>
       </c>
       <c r="G24" s="14" t="n">
-        <v>0</v>
+        <v>2000</v>
       </c>
       <c r="H24" s="14" t="n">
         <v>0</v>
@@ -11590,39 +12142,39 @@
         <f>IF(E24&gt;0, F24/E24, IF(F24&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L24" s="35" t="inlineStr">
-        <is>
-          <t>Sin Pedido</t>
+      <c r="L24" s="29" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="B25" s="30" t="inlineStr">
         <is>
-          <t>TÉCNICAS AGRÍCOLAS, S.A.</t>
+          <t xml:space="preserve">EUROFERTIL, S.A.    </t>
         </is>
       </c>
       <c r="C25" s="31" t="inlineStr">
         <is>
-          <t>A-500001</t>
+          <t>C-CU1000</t>
         </is>
       </c>
       <c r="D25" s="30" t="inlineStr">
         <is>
-          <t>CODIORGAN-A50, 1 KG</t>
+          <t>CODICOBRE, 1000 L</t>
         </is>
       </c>
       <c r="E25" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F25" s="18" t="n">
-        <v>368</v>
+        <v>1000</v>
       </c>
       <c r="G25" s="18" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="H25" s="18" t="n">
-        <v>368</v>
+        <v>0</v>
       </c>
       <c r="I25" s="18">
         <f>MAX(0, E25-F25)</f>
@@ -11645,30 +12197,30 @@
     <row r="26">
       <c r="B26" s="27" t="inlineStr">
         <is>
-          <t>TÉCNICAS AGRÍCOLAS, S.A.</t>
+          <t xml:space="preserve">EUROFERTIL, S.A.    </t>
         </is>
       </c>
       <c r="C26" s="28" t="inlineStr">
         <is>
-          <t>AGXCR0001</t>
+          <t>CODIR1000</t>
         </is>
       </c>
       <c r="D26" s="27" t="inlineStr">
         <is>
-          <t>AGROXILATO-K, 1 L</t>
+          <t>CODIRESIST, 1000 L</t>
         </is>
       </c>
       <c r="E26" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F26" s="14" t="n">
-        <v>540</v>
+        <v>1000</v>
       </c>
       <c r="G26" s="14" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="H26" s="14" t="n">
-        <v>540</v>
+        <v>0</v>
       </c>
       <c r="I26" s="14">
         <f>MAX(0, E26-F26)</f>
@@ -11691,30 +12243,30 @@
     <row r="27">
       <c r="B27" s="30" t="inlineStr">
         <is>
-          <t>TÉCNICAS AGRÍCOLAS, S.A.</t>
+          <t xml:space="preserve">EUROFERTIL, S.A.    </t>
         </is>
       </c>
       <c r="C27" s="31" t="inlineStr">
         <is>
-          <t>AGXCR0005</t>
+          <t>DECA0005</t>
         </is>
       </c>
       <c r="D27" s="30" t="inlineStr">
         <is>
-          <t>AGROXILATO-K, 5 L</t>
+          <t>DEFENS-CA-AE, 5 KG</t>
         </is>
       </c>
       <c r="E27" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F27" s="18" t="n">
-        <v>300</v>
+        <v>750</v>
       </c>
       <c r="G27" s="18" t="n">
-        <v>0</v>
+        <v>750</v>
       </c>
       <c r="H27" s="18" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="I27" s="18">
         <f>MAX(0, E27-F27)</f>
@@ -11737,30 +12289,30 @@
     <row r="28">
       <c r="B28" s="27" t="inlineStr">
         <is>
-          <t>TÉCNICAS AGRÍCOLAS, S.A.</t>
+          <t xml:space="preserve">EUROFERTIL, S.A.    </t>
         </is>
       </c>
       <c r="C28" s="28" t="inlineStr">
         <is>
-          <t>AN0005</t>
+          <t>F-A1000</t>
         </is>
       </c>
       <c r="D28" s="27" t="inlineStr">
         <is>
-          <t>ALCAPLANT, 5 KG</t>
+          <t xml:space="preserve">FITOLIN AGRO, 1000 L </t>
         </is>
       </c>
       <c r="E28" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F28" s="14" t="n">
-        <v>7920</v>
+        <v>1000</v>
       </c>
       <c r="G28" s="14" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="H28" s="14" t="n">
-        <v>7920</v>
+        <v>0</v>
       </c>
       <c r="I28" s="14">
         <f>MAX(0, E28-F28)</f>
@@ -11783,30 +12335,30 @@
     <row r="29">
       <c r="B29" s="30" t="inlineStr">
         <is>
-          <t>TÉCNICAS AGRÍCOLAS, S.A.</t>
+          <t xml:space="preserve">EUROFERTIL, S.A.    </t>
         </is>
       </c>
       <c r="C29" s="31" t="inlineStr">
         <is>
-          <t>B0001</t>
+          <t>NB1000</t>
         </is>
       </c>
       <c r="D29" s="30" t="inlineStr">
         <is>
-          <t>FORTALEZA,1 L</t>
+          <t>NITROBALANCE, 1000 L</t>
         </is>
       </c>
       <c r="E29" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F29" s="18" t="n">
-        <v>540</v>
+        <v>2000</v>
       </c>
       <c r="G29" s="18" t="n">
-        <v>0</v>
+        <v>2000</v>
       </c>
       <c r="H29" s="18" t="n">
-        <v>540</v>
+        <v>0</v>
       </c>
       <c r="I29" s="18">
         <f>MAX(0, E29-F29)</f>
@@ -11829,30 +12381,30 @@
     <row r="30">
       <c r="B30" s="27" t="inlineStr">
         <is>
-          <t>TÉCNICAS AGRÍCOLAS, S.A.</t>
+          <t xml:space="preserve">EUROFERTIL, S.A.    </t>
         </is>
       </c>
       <c r="C30" s="28" t="inlineStr">
         <is>
-          <t>C-CU0001</t>
+          <t>SS0020</t>
         </is>
       </c>
       <c r="D30" s="27" t="inlineStr">
         <is>
-          <t>CODICOBRE, 1 L</t>
+          <t>SAL WAX MAX, 20 KG</t>
         </is>
       </c>
       <c r="E30" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F30" s="14" t="n">
-        <v>840</v>
+        <v>1600</v>
       </c>
       <c r="G30" s="14" t="n">
-        <v>0</v>
+        <v>1600</v>
       </c>
       <c r="H30" s="14" t="n">
-        <v>840</v>
+        <v>0</v>
       </c>
       <c r="I30" s="14">
         <f>MAX(0, E30-F30)</f>
@@ -11875,30 +12427,30 @@
     <row r="31">
       <c r="B31" s="30" t="inlineStr">
         <is>
-          <t>TÉCNICAS AGRÍCOLAS, S.A.</t>
+          <t>HORTIFRUT - PERU, S.A.C.</t>
         </is>
       </c>
       <c r="C31" s="31" t="inlineStr">
         <is>
-          <t>C-CU0005</t>
+          <t>AN0020</t>
         </is>
       </c>
       <c r="D31" s="30" t="inlineStr">
         <is>
-          <t>CODICOBRE, 5 L</t>
+          <t>ALCAPLANT NEW, 20 KG</t>
         </is>
       </c>
       <c r="E31" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F31" s="18" t="n">
-        <v>600</v>
+        <v>1100</v>
       </c>
       <c r="G31" s="18" t="n">
         <v>0</v>
       </c>
       <c r="H31" s="18" t="n">
-        <v>600</v>
+        <v>1100</v>
       </c>
       <c r="I31" s="18">
         <f>MAX(0, E31-F31)</f>
@@ -11921,30 +12473,30 @@
     <row r="32">
       <c r="B32" s="27" t="inlineStr">
         <is>
-          <t>TÉCNICAS AGRÍCOLAS, S.A.</t>
+          <t>LEKKERBIO B.V.</t>
         </is>
       </c>
       <c r="C32" s="28" t="inlineStr">
         <is>
-          <t>SERVFLETE</t>
+          <t>AO0020</t>
         </is>
       </c>
       <c r="D32" s="27" t="inlineStr">
         <is>
-          <t>FREIGHT</t>
+          <t>ALCAPLANT NEW</t>
         </is>
       </c>
       <c r="E32" s="14" t="n">
-        <v>0</v>
+        <v>44000</v>
       </c>
       <c r="F32" s="14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G32" s="14" t="n">
         <v>0</v>
       </c>
       <c r="H32" s="14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I32" s="14">
         <f>MAX(0, E32-F32)</f>
@@ -11958,39 +12510,39 @@
         <f>IF(E32&gt;0, F32/E32, IF(F32&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L32" s="29" t="inlineStr">
-        <is>
-          <t>Extra Estimación</t>
+      <c r="L32" s="35" t="inlineStr">
+        <is>
+          <t>Sin Pedido</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="B33" s="30" t="inlineStr">
         <is>
-          <t>TÉCNICAS AGRÍCOLAS, S.A.</t>
+          <t xml:space="preserve">SERVICIOS AGROPECUARIOS EL LLANO, S. A. </t>
         </is>
       </c>
       <c r="C33" s="31" t="inlineStr">
         <is>
-          <t>SERVSEGURO</t>
+          <t>A-500001</t>
         </is>
       </c>
       <c r="D33" s="30" t="inlineStr">
         <is>
-          <t>INSURANCE</t>
+          <t>CODIORGAN-A50, 1 KG</t>
         </is>
       </c>
       <c r="E33" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F33" s="18" t="n">
-        <v>1</v>
+        <v>368</v>
       </c>
       <c r="G33" s="18" t="n">
         <v>0</v>
       </c>
       <c r="H33" s="18" t="n">
-        <v>1</v>
+        <v>368</v>
       </c>
       <c r="I33" s="18">
         <f>MAX(0, E33-F33)</f>
@@ -12013,30 +12565,30 @@
     <row r="34">
       <c r="B34" s="27" t="inlineStr">
         <is>
-          <t>TÉCNICAS AGRÍCOLAS, S.A.</t>
+          <t xml:space="preserve">SERVICIOS AGROPECUARIOS EL LLANO, S. A. </t>
         </is>
       </c>
       <c r="C34" s="28" t="inlineStr">
         <is>
-          <t>SPCE0001</t>
+          <t>AGXCR0001</t>
         </is>
       </c>
       <c r="D34" s="27" t="inlineStr">
         <is>
-          <t>SPRINTENE ABONO CE, 1 L</t>
+          <t>AGROXILATO-K, 1 L</t>
         </is>
       </c>
       <c r="E34" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F34" s="14" t="n">
-        <v>180</v>
+        <v>540</v>
       </c>
       <c r="G34" s="14" t="n">
         <v>0</v>
       </c>
       <c r="H34" s="14" t="n">
-        <v>180</v>
+        <v>540</v>
       </c>
       <c r="I34" s="14">
         <f>MAX(0, E34-F34)</f>
@@ -12059,30 +12611,30 @@
     <row r="35">
       <c r="B35" s="30" t="inlineStr">
         <is>
-          <t>TÉCNICAS AGRÍCOLAS, S.A.</t>
+          <t xml:space="preserve">SERVICIOS AGROPECUARIOS EL LLANO, S. A. </t>
         </is>
       </c>
       <c r="C35" s="31" t="inlineStr">
         <is>
-          <t>SS0001</t>
+          <t>AGXCR0005</t>
         </is>
       </c>
       <c r="D35" s="30" t="inlineStr">
         <is>
-          <t>SAL WAX MAX, 1 KG</t>
+          <t>AGROXILATO-K, 5 L</t>
         </is>
       </c>
       <c r="E35" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F35" s="18" t="n">
-        <v>1584</v>
+        <v>300</v>
       </c>
       <c r="G35" s="18" t="n">
         <v>0</v>
       </c>
       <c r="H35" s="18" t="n">
-        <v>1584</v>
+        <v>300</v>
       </c>
       <c r="I35" s="18">
         <f>MAX(0, E35-F35)</f>
@@ -12102,48 +12654,416 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="24" customHeight="1">
-      <c r="B36" s="20" t="inlineStr">
+    <row r="36">
+      <c r="B36" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SERVICIOS AGROPECUARIOS EL LLANO, S. A. </t>
+        </is>
+      </c>
+      <c r="C36" s="28" t="inlineStr">
+        <is>
+          <t>AN0005</t>
+        </is>
+      </c>
+      <c r="D36" s="27" t="inlineStr">
+        <is>
+          <t>ALCAPLANT, 5 KG</t>
+        </is>
+      </c>
+      <c r="E36" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F36" s="14" t="n">
+        <v>7920</v>
+      </c>
+      <c r="G36" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H36" s="14" t="n">
+        <v>7920</v>
+      </c>
+      <c r="I36" s="14">
+        <f>MAX(0, E36-F36)</f>
+        <v/>
+      </c>
+      <c r="J36" s="14">
+        <f>F36-E36</f>
+        <v/>
+      </c>
+      <c r="K36" s="15">
+        <f>IF(E36&gt;0, F36/E36, IF(F36&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L36" s="29" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SERVICIOS AGROPECUARIOS EL LLANO, S. A. </t>
+        </is>
+      </c>
+      <c r="C37" s="31" t="inlineStr">
+        <is>
+          <t>B0001</t>
+        </is>
+      </c>
+      <c r="D37" s="30" t="inlineStr">
+        <is>
+          <t>FORTALEZA,1 L</t>
+        </is>
+      </c>
+      <c r="E37" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F37" s="18" t="n">
+        <v>540</v>
+      </c>
+      <c r="G37" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H37" s="18" t="n">
+        <v>540</v>
+      </c>
+      <c r="I37" s="18">
+        <f>MAX(0, E37-F37)</f>
+        <v/>
+      </c>
+      <c r="J37" s="18">
+        <f>F37-E37</f>
+        <v/>
+      </c>
+      <c r="K37" s="19">
+        <f>IF(E37&gt;0, F37/E37, IF(F37&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L37" s="29" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SERVICIOS AGROPECUARIOS EL LLANO, S. A. </t>
+        </is>
+      </c>
+      <c r="C38" s="28" t="inlineStr">
+        <is>
+          <t>C-CU0001</t>
+        </is>
+      </c>
+      <c r="D38" s="27" t="inlineStr">
+        <is>
+          <t>CODICOBRE, 1 L</t>
+        </is>
+      </c>
+      <c r="E38" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F38" s="14" t="n">
+        <v>840</v>
+      </c>
+      <c r="G38" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H38" s="14" t="n">
+        <v>840</v>
+      </c>
+      <c r="I38" s="14">
+        <f>MAX(0, E38-F38)</f>
+        <v/>
+      </c>
+      <c r="J38" s="14">
+        <f>F38-E38</f>
+        <v/>
+      </c>
+      <c r="K38" s="15">
+        <f>IF(E38&gt;0, F38/E38, IF(F38&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L38" s="29" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SERVICIOS AGROPECUARIOS EL LLANO, S. A. </t>
+        </is>
+      </c>
+      <c r="C39" s="31" t="inlineStr">
+        <is>
+          <t>C-CU0005</t>
+        </is>
+      </c>
+      <c r="D39" s="30" t="inlineStr">
+        <is>
+          <t>CODICOBRE, 5 L</t>
+        </is>
+      </c>
+      <c r="E39" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F39" s="18" t="n">
+        <v>600</v>
+      </c>
+      <c r="G39" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H39" s="18" t="n">
+        <v>600</v>
+      </c>
+      <c r="I39" s="18">
+        <f>MAX(0, E39-F39)</f>
+        <v/>
+      </c>
+      <c r="J39" s="18">
+        <f>F39-E39</f>
+        <v/>
+      </c>
+      <c r="K39" s="19">
+        <f>IF(E39&gt;0, F39/E39, IF(F39&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L39" s="29" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SERVICIOS AGROPECUARIOS EL LLANO, S. A. </t>
+        </is>
+      </c>
+      <c r="C40" s="28" t="inlineStr">
+        <is>
+          <t>SERVFLETE</t>
+        </is>
+      </c>
+      <c r="D40" s="27" t="inlineStr">
+        <is>
+          <t>FREIGHT</t>
+        </is>
+      </c>
+      <c r="E40" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F40" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="G40" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H40" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="I40" s="14">
+        <f>MAX(0, E40-F40)</f>
+        <v/>
+      </c>
+      <c r="J40" s="14">
+        <f>F40-E40</f>
+        <v/>
+      </c>
+      <c r="K40" s="15">
+        <f>IF(E40&gt;0, F40/E40, IF(F40&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L40" s="29" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SERVICIOS AGROPECUARIOS EL LLANO, S. A. </t>
+        </is>
+      </c>
+      <c r="C41" s="31" t="inlineStr">
+        <is>
+          <t>SERVSEGURO</t>
+        </is>
+      </c>
+      <c r="D41" s="30" t="inlineStr">
+        <is>
+          <t>INSURANCE</t>
+        </is>
+      </c>
+      <c r="E41" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F41" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="G41" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H41" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="I41" s="18">
+        <f>MAX(0, E41-F41)</f>
+        <v/>
+      </c>
+      <c r="J41" s="18">
+        <f>F41-E41</f>
+        <v/>
+      </c>
+      <c r="K41" s="19">
+        <f>IF(E41&gt;0, F41/E41, IF(F41&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L41" s="29" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SERVICIOS AGROPECUARIOS EL LLANO, S. A. </t>
+        </is>
+      </c>
+      <c r="C42" s="28" t="inlineStr">
+        <is>
+          <t>SPCE0001</t>
+        </is>
+      </c>
+      <c r="D42" s="27" t="inlineStr">
+        <is>
+          <t>SPRINTENE ABONO CE, 1 L</t>
+        </is>
+      </c>
+      <c r="E42" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F42" s="14" t="n">
+        <v>180</v>
+      </c>
+      <c r="G42" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H42" s="14" t="n">
+        <v>180</v>
+      </c>
+      <c r="I42" s="14">
+        <f>MAX(0, E42-F42)</f>
+        <v/>
+      </c>
+      <c r="J42" s="14">
+        <f>F42-E42</f>
+        <v/>
+      </c>
+      <c r="K42" s="15">
+        <f>IF(E42&gt;0, F42/E42, IF(F42&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L42" s="29" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SERVICIOS AGROPECUARIOS EL LLANO, S. A. </t>
+        </is>
+      </c>
+      <c r="C43" s="31" t="inlineStr">
+        <is>
+          <t>SS0001</t>
+        </is>
+      </c>
+      <c r="D43" s="30" t="inlineStr">
+        <is>
+          <t>SAL WAX MAX, 1 KG</t>
+        </is>
+      </c>
+      <c r="E43" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F43" s="18" t="n">
+        <v>1584</v>
+      </c>
+      <c r="G43" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H43" s="18" t="n">
+        <v>1584</v>
+      </c>
+      <c r="I43" s="18">
+        <f>MAX(0, E43-F43)</f>
+        <v/>
+      </c>
+      <c r="J43" s="18">
+        <f>F43-E43</f>
+        <v/>
+      </c>
+      <c r="K43" s="19">
+        <f>IF(E43&gt;0, F43/E43, IF(F43&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L43" s="29" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="24" customHeight="1">
+      <c r="B44" s="20" t="inlineStr">
         <is>
           <t>TOTAL RICARDO</t>
         </is>
       </c>
-      <c r="C36" s="33" t="inlineStr">
-        <is>
-          <t>136 líneas</t>
-        </is>
-      </c>
-      <c r="D36" s="34" t="inlineStr"/>
-      <c r="E36" s="22">
-        <f>SUM(E10:E35)</f>
-        <v/>
-      </c>
-      <c r="F36" s="22">
-        <f>SUM(F10:F35)</f>
-        <v/>
-      </c>
-      <c r="G36" s="22">
-        <f>SUM(G10:G35)</f>
-        <v/>
-      </c>
-      <c r="H36" s="22">
-        <f>SUM(H10:H35)</f>
-        <v/>
-      </c>
-      <c r="I36" s="22">
-        <f>SUM(I10:I35)</f>
-        <v/>
-      </c>
-      <c r="J36" s="22">
-        <f>SUM(J10:J35)</f>
-        <v/>
-      </c>
-      <c r="K36" s="23">
-        <f>IF(E36&gt;0, F36/E36, 0)</f>
-        <v/>
-      </c>
-      <c r="L36" s="21">
-        <f>IF(K36&gt;=1, "SUPERADO", "EN CURSO")</f>
+      <c r="C44" s="33" t="inlineStr">
+        <is>
+          <t>137 líneas</t>
+        </is>
+      </c>
+      <c r="D44" s="34" t="inlineStr"/>
+      <c r="E44" s="22">
+        <f>SUM(E10:E43)</f>
+        <v/>
+      </c>
+      <c r="F44" s="22">
+        <f>SUM(F10:F43)</f>
+        <v/>
+      </c>
+      <c r="G44" s="22">
+        <f>SUM(G10:G43)</f>
+        <v/>
+      </c>
+      <c r="H44" s="22">
+        <f>SUM(H10:H43)</f>
+        <v/>
+      </c>
+      <c r="I44" s="22">
+        <f>SUM(I10:I43)</f>
+        <v/>
+      </c>
+      <c r="J44" s="22">
+        <f>SUM(J10:J43)</f>
+        <v/>
+      </c>
+      <c r="K44" s="23">
+        <f>IF(E44&gt;0, F44/E44, 0)</f>
+        <v/>
+      </c>
+      <c r="L44" s="21">
+        <f>IF(K44&gt;=1, "SUPERADO", "EN CURSO")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizar pedidos a 01/10/2026 y sincronizar dashboard web y Excel
</commit_message>
<xml_diff>
--- a/Seguimiento_Presupuesto_Sep_2026.xlsx
+++ b/Seguimiento_Presupuesto_Sep_2026.xlsx
@@ -902,7 +902,7 @@
     <row r="3" ht="20" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Comparativa Estimación Septiembre (Unidades) vs Pedidos Reales a Fecha 30/09/2026 | Generado: 30/09/2026 07:33</t>
+          <t>Comparativa Estimación Septiembre (Unidades) vs Pedidos Reales a Fecha 01/10/2026 | Generado: 01/10/2026 07:26</t>
         </is>
       </c>
     </row>
@@ -946,13 +946,13 @@
       <c r="C6" s="4" t="n"/>
       <c r="D6" s="8" t="inlineStr">
         <is>
-          <t>233,625 u</t>
+          <t>236,105 u</t>
         </is>
       </c>
       <c r="E6" s="4" t="n"/>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>128.4%</t>
+          <t>129.8%</t>
         </is>
       </c>
       <c r="G6" s="4" t="n"/>
@@ -964,7 +964,7 @@
       <c r="I6" s="4" t="n"/>
       <c r="J6" s="7" t="inlineStr">
         <is>
-          <t>130,660 u</t>
+          <t>35,774 u</t>
         </is>
       </c>
     </row>
@@ -1063,19 +1063,19 @@
         </is>
       </c>
       <c r="C11" s="17" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D11" s="18" t="n">
         <v>37832</v>
       </c>
       <c r="E11" s="18" t="n">
-        <v>56212</v>
+        <v>57312</v>
       </c>
       <c r="F11" s="18" t="n">
-        <v>6996</v>
+        <v>57312</v>
       </c>
       <c r="G11" s="18" t="n">
-        <v>49216</v>
+        <v>0</v>
       </c>
       <c r="H11" s="18">
         <f>MAX(0, D11-E11)</f>
@@ -1106,10 +1106,10 @@
         <v>23674</v>
       </c>
       <c r="F12" s="14" t="n">
-        <v>14826</v>
+        <v>23674</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>8848</v>
+        <v>0</v>
       </c>
       <c r="H12" s="14">
         <f>MAX(0, D12-E12)</f>
@@ -1137,13 +1137,13 @@
         <v>17100</v>
       </c>
       <c r="E13" s="18" t="n">
-        <v>45669</v>
+        <v>47049</v>
       </c>
       <c r="F13" s="18" t="n">
-        <v>38359</v>
+        <v>42519</v>
       </c>
       <c r="G13" s="18" t="n">
-        <v>7310</v>
+        <v>4530</v>
       </c>
       <c r="H13" s="18">
         <f>MAX(0, D13-E13)</f>
@@ -1174,10 +1174,10 @@
         <v>32728</v>
       </c>
       <c r="F14" s="14" t="n">
-        <v>0</v>
+        <v>11668</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>32728</v>
+        <v>21060</v>
       </c>
       <c r="H14" s="14">
         <f>MAX(0, D14-E14)</f>
@@ -1208,10 +1208,10 @@
         <v>8560</v>
       </c>
       <c r="F15" s="18" t="n">
-        <v>7860</v>
+        <v>8560</v>
       </c>
       <c r="G15" s="18" t="n">
-        <v>700</v>
+        <v>0</v>
       </c>
       <c r="H15" s="18">
         <f>MAX(0, D15-E15)</f>
@@ -1242,10 +1242,10 @@
         <v>54908</v>
       </c>
       <c r="F16" s="14" t="n">
-        <v>23050</v>
+        <v>44724</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>31858</v>
+        <v>10184</v>
       </c>
       <c r="H16" s="14">
         <f>MAX(0, D16-E16)</f>
@@ -1350,7 +1350,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 30/09/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 01/10/2026</t>
         </is>
       </c>
     </row>
@@ -3005,7 +3005,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 30/09/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 01/10/2026</t>
         </is>
       </c>
     </row>
@@ -3050,13 +3050,13 @@
       <c r="C6" s="4" t="n"/>
       <c r="D6" s="25" t="inlineStr">
         <is>
-          <t>56,212 u</t>
+          <t>57,312 u</t>
         </is>
       </c>
       <c r="E6" s="4" t="n"/>
       <c r="F6" s="25" t="inlineStr">
         <is>
-          <t>148.6%</t>
+          <t>151.5%</t>
         </is>
       </c>
       <c r="G6" s="4" t="n"/>
@@ -3068,7 +3068,7 @@
       <c r="I6" s="4" t="n"/>
       <c r="J6" s="24" t="inlineStr">
         <is>
-          <t>49,216 u</t>
+          <t>0 u</t>
         </is>
       </c>
       <c r="K6" s="4" t="n"/>
@@ -3525,10 +3525,10 @@
         <v>1100</v>
       </c>
       <c r="F18" s="14" t="n">
-        <v>0</v>
+        <v>1100</v>
       </c>
       <c r="G18" s="14" t="n">
-        <v>0</v>
+        <v>1100</v>
       </c>
       <c r="H18" s="14" t="n">
         <v>0</v>
@@ -3545,9 +3545,9 @@
         <f>IF(E18&gt;0, F18/E18, IF(F18&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L18" s="35" t="inlineStr">
-        <is>
-          <t>Sin Pedido</t>
+      <c r="L18" s="29" t="inlineStr">
+        <is>
+          <t>Superado</t>
         </is>
       </c>
     </row>
@@ -3850,10 +3850,10 @@
         <v>21000</v>
       </c>
       <c r="G25" s="18" t="n">
-        <v>0</v>
+        <v>21000</v>
       </c>
       <c r="H25" s="18" t="n">
-        <v>21000</v>
+        <v>0</v>
       </c>
       <c r="I25" s="18">
         <f>MAX(0, E25-F25)</f>
@@ -3896,10 +3896,10 @@
         <v>400</v>
       </c>
       <c r="G26" s="14" t="n">
-        <v>0</v>
+        <v>400</v>
       </c>
       <c r="H26" s="14" t="n">
-        <v>400</v>
+        <v>0</v>
       </c>
       <c r="I26" s="14">
         <f>MAX(0, E26-F26)</f>
@@ -3942,10 +3942,10 @@
         <v>504</v>
       </c>
       <c r="G27" s="18" t="n">
-        <v>0</v>
+        <v>504</v>
       </c>
       <c r="H27" s="18" t="n">
-        <v>504</v>
+        <v>0</v>
       </c>
       <c r="I27" s="18">
         <f>MAX(0, E27-F27)</f>
@@ -3988,10 +3988,10 @@
         <v>800</v>
       </c>
       <c r="G28" s="14" t="n">
-        <v>0</v>
+        <v>800</v>
       </c>
       <c r="H28" s="14" t="n">
-        <v>800</v>
+        <v>0</v>
       </c>
       <c r="I28" s="14">
         <f>MAX(0, E28-F28)</f>
@@ -4034,10 +4034,10 @@
         <v>1080</v>
       </c>
       <c r="G29" s="18" t="n">
-        <v>0</v>
+        <v>1080</v>
       </c>
       <c r="H29" s="18" t="n">
-        <v>1080</v>
+        <v>0</v>
       </c>
       <c r="I29" s="18">
         <f>MAX(0, E29-F29)</f>
@@ -4080,10 +4080,10 @@
         <v>17500</v>
       </c>
       <c r="G30" s="14" t="n">
-        <v>0</v>
+        <v>17500</v>
       </c>
       <c r="H30" s="14" t="n">
-        <v>17500</v>
+        <v>0</v>
       </c>
       <c r="I30" s="14">
         <f>MAX(0, E30-F30)</f>
@@ -4264,10 +4264,10 @@
         <v>1056</v>
       </c>
       <c r="G34" s="14" t="n">
-        <v>0</v>
+        <v>1056</v>
       </c>
       <c r="H34" s="14" t="n">
-        <v>1056</v>
+        <v>0</v>
       </c>
       <c r="I34" s="14">
         <f>MAX(0, E34-F34)</f>
@@ -4310,10 +4310,10 @@
         <v>528</v>
       </c>
       <c r="G35" s="18" t="n">
-        <v>0</v>
+        <v>528</v>
       </c>
       <c r="H35" s="18" t="n">
-        <v>528</v>
+        <v>0</v>
       </c>
       <c r="I35" s="18">
         <f>MAX(0, E35-F35)</f>
@@ -4356,10 +4356,10 @@
         <v>396</v>
       </c>
       <c r="G36" s="14" t="n">
-        <v>0</v>
+        <v>396</v>
       </c>
       <c r="H36" s="14" t="n">
-        <v>396</v>
+        <v>0</v>
       </c>
       <c r="I36" s="14">
         <f>MAX(0, E36-F36)</f>
@@ -4402,10 +4402,10 @@
         <v>792</v>
       </c>
       <c r="G37" s="18" t="n">
-        <v>0</v>
+        <v>792</v>
       </c>
       <c r="H37" s="18" t="n">
-        <v>792</v>
+        <v>0</v>
       </c>
       <c r="I37" s="18">
         <f>MAX(0, E37-F37)</f>
@@ -4448,10 +4448,10 @@
         <v>600</v>
       </c>
       <c r="G38" s="14" t="n">
-        <v>0</v>
+        <v>600</v>
       </c>
       <c r="H38" s="14" t="n">
-        <v>600</v>
+        <v>0</v>
       </c>
       <c r="I38" s="14">
         <f>MAX(0, E38-F38)</f>
@@ -4494,10 +4494,10 @@
         <v>640</v>
       </c>
       <c r="G39" s="18" t="n">
-        <v>0</v>
+        <v>640</v>
       </c>
       <c r="H39" s="18" t="n">
-        <v>640</v>
+        <v>0</v>
       </c>
       <c r="I39" s="18">
         <f>MAX(0, E39-F39)</f>
@@ -4540,10 +4540,10 @@
         <v>792</v>
       </c>
       <c r="G40" s="14" t="n">
-        <v>0</v>
+        <v>792</v>
       </c>
       <c r="H40" s="14" t="n">
-        <v>792</v>
+        <v>0</v>
       </c>
       <c r="I40" s="14">
         <f>MAX(0, E40-F40)</f>
@@ -4586,10 +4586,10 @@
         <v>640</v>
       </c>
       <c r="G41" s="18" t="n">
-        <v>0</v>
+        <v>640</v>
       </c>
       <c r="H41" s="18" t="n">
-        <v>640</v>
+        <v>0</v>
       </c>
       <c r="I41" s="18">
         <f>MAX(0, E41-F41)</f>
@@ -4632,10 +4632,10 @@
         <v>792</v>
       </c>
       <c r="G42" s="14" t="n">
-        <v>0</v>
+        <v>792</v>
       </c>
       <c r="H42" s="14" t="n">
-        <v>792</v>
+        <v>0</v>
       </c>
       <c r="I42" s="14">
         <f>MAX(0, E42-F42)</f>
@@ -4678,10 +4678,10 @@
         <v>640</v>
       </c>
       <c r="G43" s="18" t="n">
-        <v>0</v>
+        <v>640</v>
       </c>
       <c r="H43" s="18" t="n">
-        <v>640</v>
+        <v>0</v>
       </c>
       <c r="I43" s="18">
         <f>MAX(0, E43-F43)</f>
@@ -4724,10 +4724,10 @@
         <v>1056</v>
       </c>
       <c r="G44" s="14" t="n">
-        <v>0</v>
+        <v>1056</v>
       </c>
       <c r="H44" s="14" t="n">
-        <v>1056</v>
+        <v>0</v>
       </c>
       <c r="I44" s="14">
         <f>MAX(0, E44-F44)</f>
@@ -5350,7 +5350,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 30/09/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 01/10/2026</t>
         </is>
       </c>
     </row>
@@ -5413,7 +5413,7 @@
       <c r="I6" s="4" t="n"/>
       <c r="J6" s="24" t="inlineStr">
         <is>
-          <t>8,848 u</t>
+          <t>0 u</t>
         </is>
       </c>
       <c r="K6" s="4" t="n"/>
@@ -5689,10 +5689,10 @@
         <v>2560</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>640</v>
+        <v>2560</v>
       </c>
       <c r="H14" s="14" t="n">
-        <v>1920</v>
+        <v>0</v>
       </c>
       <c r="I14" s="14">
         <f>MAX(0, E14-F14)</f>
@@ -5735,10 +5735,10 @@
         <v>640</v>
       </c>
       <c r="G15" s="18" t="n">
-        <v>0</v>
+        <v>640</v>
       </c>
       <c r="H15" s="18" t="n">
-        <v>640</v>
+        <v>0</v>
       </c>
       <c r="I15" s="18">
         <f>MAX(0, E15-F15)</f>
@@ -5919,10 +5919,10 @@
         <v>1300</v>
       </c>
       <c r="G19" s="18" t="n">
-        <v>700</v>
+        <v>1300</v>
       </c>
       <c r="H19" s="18" t="n">
-        <v>600</v>
+        <v>0</v>
       </c>
       <c r="I19" s="18">
         <f>MAX(0, E19-F19)</f>
@@ -5965,10 +5965,10 @@
         <v>1600</v>
       </c>
       <c r="G20" s="14" t="n">
-        <v>100</v>
+        <v>1600</v>
       </c>
       <c r="H20" s="14" t="n">
-        <v>1500</v>
+        <v>0</v>
       </c>
       <c r="I20" s="14">
         <f>MAX(0, E20-F20)</f>
@@ -6011,10 +6011,10 @@
         <v>4480</v>
       </c>
       <c r="G21" s="18" t="n">
-        <v>640</v>
+        <v>4480</v>
       </c>
       <c r="H21" s="18" t="n">
-        <v>3840</v>
+        <v>0</v>
       </c>
       <c r="I21" s="18">
         <f>MAX(0, E21-F21)</f>
@@ -6057,10 +6057,10 @@
         <v>48</v>
       </c>
       <c r="G22" s="14" t="n">
-        <v>0</v>
+        <v>48</v>
       </c>
       <c r="H22" s="14" t="n">
-        <v>48</v>
+        <v>0</v>
       </c>
       <c r="I22" s="14">
         <f>MAX(0, E22-F22)</f>
@@ -6103,10 +6103,10 @@
         <v>300</v>
       </c>
       <c r="G23" s="18" t="n">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="H23" s="18" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="I23" s="18">
         <f>MAX(0, E23-F23)</f>
@@ -7208,7 +7208,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:L54"/>
+  <dimension ref="B2:L56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -7235,7 +7235,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 30/09/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 01/10/2026</t>
         </is>
       </c>
     </row>
@@ -7280,13 +7280,13 @@
       <c r="C6" s="4" t="n"/>
       <c r="D6" s="25" t="inlineStr">
         <is>
-          <t>45,669 u</t>
+          <t>47,049 u</t>
         </is>
       </c>
       <c r="E6" s="4" t="n"/>
       <c r="F6" s="25" t="inlineStr">
         <is>
-          <t>267.1%</t>
+          <t>275.1%</t>
         </is>
       </c>
       <c r="G6" s="4" t="n"/>
@@ -7298,7 +7298,7 @@
       <c r="I6" s="4" t="n"/>
       <c r="J6" s="24" t="inlineStr">
         <is>
-          <t>7,310 u</t>
+          <t>4,530 u</t>
         </is>
       </c>
       <c r="K6" s="4" t="n"/>
@@ -7390,10 +7390,10 @@
         <v>3200</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>1600</v>
+        <v>3200</v>
       </c>
       <c r="H10" s="14" t="n">
-        <v>1600</v>
+        <v>0</v>
       </c>
       <c r="I10" s="14">
         <f>MAX(0, E10-F10)</f>
@@ -7804,10 +7804,10 @@
         <v>1280</v>
       </c>
       <c r="G19" s="18" t="n">
-        <v>0</v>
+        <v>1280</v>
       </c>
       <c r="H19" s="18" t="n">
-        <v>1280</v>
+        <v>0</v>
       </c>
       <c r="I19" s="18">
         <f>MAX(0, E19-F19)</f>
@@ -7896,10 +7896,10 @@
         <v>1280</v>
       </c>
       <c r="G21" s="18" t="n">
-        <v>0</v>
+        <v>1280</v>
       </c>
       <c r="H21" s="18" t="n">
-        <v>1280</v>
+        <v>0</v>
       </c>
       <c r="I21" s="18">
         <f>MAX(0, E21-F21)</f>
@@ -8341,25 +8341,25 @@
       </c>
       <c r="C31" s="31" t="inlineStr">
         <is>
-          <t>C-L0005</t>
+          <t>BIO0020</t>
         </is>
       </c>
       <c r="D31" s="30" t="inlineStr">
         <is>
-          <t>CODIBOR-L, 5 L</t>
+          <t>BIORAD-20, 20 L</t>
         </is>
       </c>
       <c r="E31" s="18" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="F31" s="18" t="n">
-        <v>200</v>
+        <v>640</v>
       </c>
       <c r="G31" s="18" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="H31" s="18" t="n">
-        <v>0</v>
+        <v>640</v>
       </c>
       <c r="I31" s="18">
         <f>MAX(0, E31-F31)</f>
@@ -8375,7 +8375,7 @@
       </c>
       <c r="L31" s="29" t="inlineStr">
         <is>
-          <t>Superado</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -8387,25 +8387,25 @@
       </c>
       <c r="C32" s="28" t="inlineStr">
         <is>
-          <t>C-L0020</t>
+          <t>C-CU0020</t>
         </is>
       </c>
       <c r="D32" s="27" t="inlineStr">
         <is>
-          <t>CODIBOR-L, 20 L</t>
+          <t>CODICOBRE, 20 L</t>
         </is>
       </c>
       <c r="E32" s="14" t="n">
-        <v>640</v>
+        <v>0</v>
       </c>
       <c r="F32" s="14" t="n">
-        <v>640</v>
+        <v>320</v>
       </c>
       <c r="G32" s="14" t="n">
-        <v>640</v>
+        <v>0</v>
       </c>
       <c r="H32" s="14" t="n">
-        <v>0</v>
+        <v>320</v>
       </c>
       <c r="I32" s="14">
         <f>MAX(0, E32-F32)</f>
@@ -8421,7 +8421,7 @@
       </c>
       <c r="L32" s="29" t="inlineStr">
         <is>
-          <t>Superado</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -8433,25 +8433,25 @@
       </c>
       <c r="C33" s="31" t="inlineStr">
         <is>
-          <t>PT0005</t>
+          <t>C-L0005</t>
         </is>
       </c>
       <c r="D33" s="30" t="inlineStr">
         <is>
-          <t>AGROPOTASION, 5 L</t>
+          <t>CODIBOR-L, 5 L</t>
         </is>
       </c>
       <c r="E33" s="18" t="n">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="F33" s="18" t="n">
+        <v>300</v>
+      </c>
+      <c r="G33" s="18" t="n">
+        <v>200</v>
+      </c>
+      <c r="H33" s="18" t="n">
         <v>100</v>
-      </c>
-      <c r="G33" s="18" t="n">
-        <v>100</v>
-      </c>
-      <c r="H33" s="18" t="n">
-        <v>0</v>
       </c>
       <c r="I33" s="18">
         <f>MAX(0, E33-F33)</f>
@@ -8467,7 +8467,7 @@
       </c>
       <c r="L33" s="29" t="inlineStr">
         <is>
-          <t>Extra Estimación</t>
+          <t>Superado</t>
         </is>
       </c>
     </row>
@@ -8479,25 +8479,25 @@
       </c>
       <c r="C34" s="28" t="inlineStr">
         <is>
-          <t>PT0020</t>
+          <t>C-L0020</t>
         </is>
       </c>
       <c r="D34" s="27" t="inlineStr">
         <is>
-          <t>AGROPOTASION, 20 L</t>
+          <t>CODIBOR-L, 20 L</t>
         </is>
       </c>
       <c r="E34" s="14" t="n">
-        <v>0</v>
+        <v>640</v>
       </c>
       <c r="F34" s="14" t="n">
-        <v>200</v>
+        <v>960</v>
       </c>
       <c r="G34" s="14" t="n">
-        <v>200</v>
+        <v>640</v>
       </c>
       <c r="H34" s="14" t="n">
-        <v>0</v>
+        <v>320</v>
       </c>
       <c r="I34" s="14">
         <f>MAX(0, E34-F34)</f>
@@ -8513,7 +8513,7 @@
       </c>
       <c r="L34" s="29" t="inlineStr">
         <is>
-          <t>Extra Estimación</t>
+          <t>Superado</t>
         </is>
       </c>
     </row>
@@ -8525,22 +8525,22 @@
       </c>
       <c r="C35" s="31" t="inlineStr">
         <is>
-          <t>SPCE2B0020</t>
+          <t>PT0005</t>
         </is>
       </c>
       <c r="D35" s="30" t="inlineStr">
         <is>
-          <t>SPRINTENE CON BORO, 20 L</t>
+          <t>AGROPOTASION, 5 L</t>
         </is>
       </c>
       <c r="E35" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F35" s="18" t="n">
-        <v>320</v>
+        <v>100</v>
       </c>
       <c r="G35" s="18" t="n">
-        <v>320</v>
+        <v>100</v>
       </c>
       <c r="H35" s="18" t="n">
         <v>0</v>
@@ -8566,27 +8566,27 @@
     <row r="36">
       <c r="B36" s="27" t="inlineStr">
         <is>
-          <t>FINCA DOÑA ANA C.B.</t>
+          <t>CODIMED EXPORT, S.L.</t>
         </is>
       </c>
       <c r="C36" s="28" t="inlineStr">
         <is>
-          <t>A-50(2)0020</t>
+          <t>PT0020</t>
         </is>
       </c>
       <c r="D36" s="27" t="inlineStr">
         <is>
-          <t>CODIORGAN-A50, 20 KG</t>
+          <t>AGROPOTASION, 20 L</t>
         </is>
       </c>
       <c r="E36" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F36" s="14" t="n">
-        <v>120</v>
+        <v>200</v>
       </c>
       <c r="G36" s="14" t="n">
-        <v>120</v>
+        <v>200</v>
       </c>
       <c r="H36" s="14" t="n">
         <v>0</v>
@@ -8612,27 +8612,27 @@
     <row r="37">
       <c r="B37" s="30" t="inlineStr">
         <is>
-          <t>FINCA DOÑA ANA C.B.</t>
+          <t>CODIMED EXPORT, S.L.</t>
         </is>
       </c>
       <c r="C37" s="31" t="inlineStr">
         <is>
-          <t>C-CU1000</t>
+          <t>SPCE2B0020</t>
         </is>
       </c>
       <c r="D37" s="30" t="inlineStr">
         <is>
-          <t>CODICOBRE, 1000 L</t>
+          <t>SPRINTENE CON BORO, 20 L</t>
         </is>
       </c>
       <c r="E37" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F37" s="18" t="n">
-        <v>1000</v>
+        <v>320</v>
       </c>
       <c r="G37" s="18" t="n">
-        <v>1000</v>
+        <v>320</v>
       </c>
       <c r="H37" s="18" t="n">
         <v>0</v>
@@ -8658,27 +8658,27 @@
     <row r="38">
       <c r="B38" s="27" t="inlineStr">
         <is>
-          <t>FITOSANITARIOS CARCAIXENT, S.L.</t>
+          <t>FINCA DOÑA ANA C.B.</t>
         </is>
       </c>
       <c r="C38" s="28" t="inlineStr">
         <is>
-          <t>C-CU0005</t>
+          <t>A-50(2)0020</t>
         </is>
       </c>
       <c r="D38" s="27" t="inlineStr">
         <is>
-          <t>CODICOBRE, 5 L</t>
+          <t>CODIORGAN-A50, 20 KG</t>
         </is>
       </c>
       <c r="E38" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F38" s="14" t="n">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="G38" s="14" t="n">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="H38" s="14" t="n">
         <v>0</v>
@@ -8704,27 +8704,27 @@
     <row r="39">
       <c r="B39" s="30" t="inlineStr">
         <is>
-          <t>FITOSANITARIOS CARCAIXENT, S.L.</t>
+          <t>FINCA DOÑA ANA C.B.</t>
         </is>
       </c>
       <c r="C39" s="31" t="inlineStr">
         <is>
-          <t>G30020</t>
+          <t>C-CU1000</t>
         </is>
       </c>
       <c r="D39" s="30" t="inlineStr">
         <is>
-          <t>GREEN-UP, 20 L</t>
+          <t>CODICOBRE, 1000 L</t>
         </is>
       </c>
       <c r="E39" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F39" s="18" t="n">
-        <v>200</v>
+        <v>1000</v>
       </c>
       <c r="G39" s="18" t="n">
-        <v>200</v>
+        <v>1000</v>
       </c>
       <c r="H39" s="18" t="n">
         <v>0</v>
@@ -8755,12 +8755,12 @@
       </c>
       <c r="C40" s="28" t="inlineStr">
         <is>
-          <t>HST0020</t>
+          <t>C-CU0005</t>
         </is>
       </c>
       <c r="D40" s="27" t="inlineStr">
         <is>
-          <t>HIDROSTRESS-40, 20 L</t>
+          <t>CODICOBRE, 5 L</t>
         </is>
       </c>
       <c r="E40" s="14" t="n">
@@ -8801,22 +8801,22 @@
       </c>
       <c r="C41" s="31" t="inlineStr">
         <is>
-          <t>PT0005</t>
+          <t>G30020</t>
         </is>
       </c>
       <c r="D41" s="30" t="inlineStr">
         <is>
-          <t>AGROPOTASION, 5 L</t>
+          <t>GREEN-UP, 20 L</t>
         </is>
       </c>
       <c r="E41" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F41" s="18" t="n">
-        <v>600</v>
+        <v>200</v>
       </c>
       <c r="G41" s="18" t="n">
-        <v>600</v>
+        <v>200</v>
       </c>
       <c r="H41" s="18" t="n">
         <v>0</v>
@@ -8847,22 +8847,22 @@
       </c>
       <c r="C42" s="28" t="inlineStr">
         <is>
-          <t>PT0020</t>
+          <t>HST0020</t>
         </is>
       </c>
       <c r="D42" s="27" t="inlineStr">
         <is>
-          <t>AGROPOTASION, 20 L</t>
+          <t>HIDROSTRESS-40, 20 L</t>
         </is>
       </c>
       <c r="E42" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F42" s="14" t="n">
-        <v>1920</v>
+        <v>100</v>
       </c>
       <c r="G42" s="14" t="n">
-        <v>1920</v>
+        <v>100</v>
       </c>
       <c r="H42" s="14" t="n">
         <v>0</v>
@@ -8888,27 +8888,27 @@
     <row r="43">
       <c r="B43" s="30" t="inlineStr">
         <is>
-          <t>FITOSANITARIOS DRAGO S.L.U</t>
+          <t>FITOSANITARIOS CARCAIXENT, S.L.</t>
         </is>
       </c>
       <c r="C43" s="31" t="inlineStr">
         <is>
-          <t>AGXK0200</t>
+          <t>PT0005</t>
         </is>
       </c>
       <c r="D43" s="30" t="inlineStr">
         <is>
-          <t>AGROXILATO-K, 200 L</t>
+          <t>AGROPOTASION, 5 L</t>
         </is>
       </c>
       <c r="E43" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F43" s="18" t="n">
-        <v>1600</v>
+        <v>600</v>
       </c>
       <c r="G43" s="18" t="n">
-        <v>1600</v>
+        <v>600</v>
       </c>
       <c r="H43" s="18" t="n">
         <v>0</v>
@@ -8934,27 +8934,27 @@
     <row r="44">
       <c r="B44" s="27" t="inlineStr">
         <is>
-          <t>FITOSANITARIOS DRAGO S.L.U</t>
+          <t>FITOSANITARIOS CARCAIXENT, S.L.</t>
         </is>
       </c>
       <c r="C44" s="28" t="inlineStr">
         <is>
-          <t>AGXK1000</t>
+          <t>PT0020</t>
         </is>
       </c>
       <c r="D44" s="27" t="inlineStr">
         <is>
-          <t>AGROXILATO-K, 1000 L</t>
+          <t>AGROPOTASION, 20 L</t>
         </is>
       </c>
       <c r="E44" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F44" s="14" t="n">
-        <v>10000</v>
+        <v>1920</v>
       </c>
       <c r="G44" s="14" t="n">
-        <v>10000</v>
+        <v>1920</v>
       </c>
       <c r="H44" s="14" t="n">
         <v>0</v>
@@ -8985,22 +8985,22 @@
       </c>
       <c r="C45" s="31" t="inlineStr">
         <is>
-          <t>C-CU0001</t>
+          <t>AGXK0200</t>
         </is>
       </c>
       <c r="D45" s="30" t="inlineStr">
         <is>
-          <t>CODICOBRE, 1 L</t>
+          <t>AGROXILATO-K, 200 L</t>
         </is>
       </c>
       <c r="E45" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F45" s="18" t="n">
-        <v>24</v>
+        <v>1600</v>
       </c>
       <c r="G45" s="18" t="n">
-        <v>24</v>
+        <v>1600</v>
       </c>
       <c r="H45" s="18" t="n">
         <v>0</v>
@@ -9031,22 +9031,22 @@
       </c>
       <c r="C46" s="28" t="inlineStr">
         <is>
-          <t>JF0020</t>
+          <t>AGXK1000</t>
         </is>
       </c>
       <c r="D46" s="27" t="inlineStr">
         <is>
-          <t>DRAGO-FOS, 20 L</t>
+          <t>AGROXILATO-K, 1000 L</t>
         </is>
       </c>
       <c r="E46" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F46" s="14" t="n">
-        <v>1280</v>
+        <v>10000</v>
       </c>
       <c r="G46" s="14" t="n">
-        <v>1280</v>
+        <v>10000</v>
       </c>
       <c r="H46" s="14" t="n">
         <v>0</v>
@@ -9077,22 +9077,22 @@
       </c>
       <c r="C47" s="31" t="inlineStr">
         <is>
-          <t>PHD0005</t>
+          <t>C-CU0001</t>
         </is>
       </c>
       <c r="D47" s="30" t="inlineStr">
         <is>
-          <t xml:space="preserve">PH-DOWNER, 5 L   </t>
+          <t>CODICOBRE, 1 L</t>
         </is>
       </c>
       <c r="E47" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F47" s="18" t="n">
-        <v>400</v>
+        <v>24</v>
       </c>
       <c r="G47" s="18" t="n">
-        <v>400</v>
+        <v>24</v>
       </c>
       <c r="H47" s="18" t="n">
         <v>0</v>
@@ -9123,22 +9123,22 @@
       </c>
       <c r="C48" s="28" t="inlineStr">
         <is>
-          <t>PHD0020</t>
+          <t>JF0020</t>
         </is>
       </c>
       <c r="D48" s="27" t="inlineStr">
         <is>
-          <t>PH-DOWNER, 20 L</t>
+          <t>DRAGO-FOS, 20 L</t>
         </is>
       </c>
       <c r="E48" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F48" s="14" t="n">
-        <v>640</v>
+        <v>1280</v>
       </c>
       <c r="G48" s="14" t="n">
-        <v>640</v>
+        <v>1280</v>
       </c>
       <c r="H48" s="14" t="n">
         <v>0</v>
@@ -9169,22 +9169,22 @@
       </c>
       <c r="C49" s="31" t="inlineStr">
         <is>
-          <t>S0200</t>
+          <t>PHD0005</t>
         </is>
       </c>
       <c r="D49" s="30" t="inlineStr">
         <is>
-          <t>SAL-WAX STAR, 200 L</t>
+          <t xml:space="preserve">PH-DOWNER, 5 L   </t>
         </is>
       </c>
       <c r="E49" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F49" s="18" t="n">
-        <v>800</v>
+        <v>400</v>
       </c>
       <c r="G49" s="18" t="n">
-        <v>800</v>
+        <v>400</v>
       </c>
       <c r="H49" s="18" t="n">
         <v>0</v>
@@ -9215,22 +9215,22 @@
       </c>
       <c r="C50" s="28" t="inlineStr">
         <is>
-          <t>SS0020</t>
+          <t>PHD0020</t>
         </is>
       </c>
       <c r="D50" s="27" t="inlineStr">
         <is>
-          <t>SALWAX-CA, 20 KG</t>
+          <t>PH-DOWNER, 20 L</t>
         </is>
       </c>
       <c r="E50" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F50" s="14" t="n">
-        <v>40</v>
+        <v>640</v>
       </c>
       <c r="G50" s="14" t="n">
-        <v>40</v>
+        <v>640</v>
       </c>
       <c r="H50" s="14" t="n">
         <v>0</v>
@@ -9256,27 +9256,27 @@
     <row r="51">
       <c r="B51" s="30" t="inlineStr">
         <is>
-          <t>FITOXENT S.C.L.V.</t>
+          <t>FITOSANITARIOS DRAGO S.L.U</t>
         </is>
       </c>
       <c r="C51" s="31" t="inlineStr">
         <is>
-          <t>FTK0005</t>
+          <t>S0200</t>
         </is>
       </c>
       <c r="D51" s="30" t="inlineStr">
         <is>
-          <t>FITOKONTROL CA FLOW, 5 KG</t>
+          <t>SAL-WAX STAR, 200 L</t>
         </is>
       </c>
       <c r="E51" s="18" t="n">
-        <v>4400</v>
+        <v>0</v>
       </c>
       <c r="F51" s="18" t="n">
-        <v>4400</v>
+        <v>800</v>
       </c>
       <c r="G51" s="18" t="n">
-        <v>4400</v>
+        <v>800</v>
       </c>
       <c r="H51" s="18" t="n">
         <v>0</v>
@@ -9295,34 +9295,34 @@
       </c>
       <c r="L51" s="29" t="inlineStr">
         <is>
-          <t>Superado</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="B52" s="27" t="inlineStr">
         <is>
-          <t>FITOXENT S.C.L.V.</t>
+          <t>FITOSANITARIOS DRAGO S.L.U</t>
         </is>
       </c>
       <c r="C52" s="28" t="inlineStr">
         <is>
-          <t>PT0020</t>
+          <t>SS0020</t>
         </is>
       </c>
       <c r="D52" s="27" t="inlineStr">
         <is>
-          <t>AGROPOTASION, 20 L</t>
+          <t>SALWAX-CA, 20 KG</t>
         </is>
       </c>
       <c r="E52" s="14" t="n">
-        <v>2560</v>
+        <v>0</v>
       </c>
       <c r="F52" s="14" t="n">
-        <v>1280</v>
+        <v>40</v>
       </c>
       <c r="G52" s="14" t="n">
-        <v>1280</v>
+        <v>40</v>
       </c>
       <c r="H52" s="14" t="n">
         <v>0</v>
@@ -9339,9 +9339,9 @@
         <f>IF(E52&gt;0, F52/E52, IF(F52&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L52" s="32" t="inlineStr">
-        <is>
-          <t>En Curso</t>
+      <c r="L52" s="29" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -9353,22 +9353,22 @@
       </c>
       <c r="C53" s="31" t="inlineStr">
         <is>
-          <t>S0020</t>
+          <t>FTK0005</t>
         </is>
       </c>
       <c r="D53" s="30" t="inlineStr">
         <is>
-          <t>SALWAX STAR, 20 L</t>
+          <t>FITOKONTROL CA FLOW, 5 KG</t>
         </is>
       </c>
       <c r="E53" s="18" t="n">
-        <v>0</v>
+        <v>4400</v>
       </c>
       <c r="F53" s="18" t="n">
-        <v>200</v>
+        <v>4400</v>
       </c>
       <c r="G53" s="18" t="n">
-        <v>200</v>
+        <v>4400</v>
       </c>
       <c r="H53" s="18" t="n">
         <v>0</v>
@@ -9387,52 +9387,144 @@
       </c>
       <c r="L53" s="29" t="inlineStr">
         <is>
-          <t>Extra Estimación</t>
-        </is>
-      </c>
-    </row>
-    <row r="54" ht="24" customHeight="1">
-      <c r="B54" s="20" t="inlineStr">
+          <t>Superado</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="B54" s="27" t="inlineStr">
+        <is>
+          <t>FITOXENT S.C.L.V.</t>
+        </is>
+      </c>
+      <c r="C54" s="28" t="inlineStr">
+        <is>
+          <t>PT0020</t>
+        </is>
+      </c>
+      <c r="D54" s="27" t="inlineStr">
+        <is>
+          <t>AGROPOTASION, 20 L</t>
+        </is>
+      </c>
+      <c r="E54" s="14" t="n">
+        <v>2560</v>
+      </c>
+      <c r="F54" s="14" t="n">
+        <v>1280</v>
+      </c>
+      <c r="G54" s="14" t="n">
+        <v>1280</v>
+      </c>
+      <c r="H54" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I54" s="14">
+        <f>MAX(0, E54-F54)</f>
+        <v/>
+      </c>
+      <c r="J54" s="14">
+        <f>F54-E54</f>
+        <v/>
+      </c>
+      <c r="K54" s="15">
+        <f>IF(E54&gt;0, F54/E54, IF(F54&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L54" s="32" t="inlineStr">
+        <is>
+          <t>En Curso</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="B55" s="30" t="inlineStr">
+        <is>
+          <t>FITOXENT S.C.L.V.</t>
+        </is>
+      </c>
+      <c r="C55" s="31" t="inlineStr">
+        <is>
+          <t>S0020</t>
+        </is>
+      </c>
+      <c r="D55" s="30" t="inlineStr">
+        <is>
+          <t>SALWAX STAR, 20 L</t>
+        </is>
+      </c>
+      <c r="E55" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F55" s="18" t="n">
+        <v>200</v>
+      </c>
+      <c r="G55" s="18" t="n">
+        <v>200</v>
+      </c>
+      <c r="H55" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="I55" s="18">
+        <f>MAX(0, E55-F55)</f>
+        <v/>
+      </c>
+      <c r="J55" s="18">
+        <f>F55-E55</f>
+        <v/>
+      </c>
+      <c r="K55" s="19">
+        <f>IF(E55&gt;0, F55/E55, IF(F55&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L55" s="29" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="24" customHeight="1">
+      <c r="B56" s="20" t="inlineStr">
         <is>
           <t>TOTAL JAVIER</t>
         </is>
       </c>
-      <c r="C54" s="33" t="inlineStr">
+      <c r="C56" s="33" t="inlineStr">
         <is>
           <t>186 líneas</t>
         </is>
       </c>
-      <c r="D54" s="34" t="inlineStr"/>
-      <c r="E54" s="22">
-        <f>SUM(E10:E53)</f>
-        <v/>
-      </c>
-      <c r="F54" s="22">
-        <f>SUM(F10:F53)</f>
-        <v/>
-      </c>
-      <c r="G54" s="22">
-        <f>SUM(G10:G53)</f>
-        <v/>
-      </c>
-      <c r="H54" s="22">
-        <f>SUM(H10:H53)</f>
-        <v/>
-      </c>
-      <c r="I54" s="22">
-        <f>SUM(I10:I53)</f>
-        <v/>
-      </c>
-      <c r="J54" s="22">
-        <f>SUM(J10:J53)</f>
-        <v/>
-      </c>
-      <c r="K54" s="23">
-        <f>IF(E54&gt;0, F54/E54, 0)</f>
-        <v/>
-      </c>
-      <c r="L54" s="21">
-        <f>IF(K54&gt;=1, "SUPERADO", "EN CURSO")</f>
+      <c r="D56" s="34" t="inlineStr"/>
+      <c r="E56" s="22">
+        <f>SUM(E10:E55)</f>
+        <v/>
+      </c>
+      <c r="F56" s="22">
+        <f>SUM(F10:F55)</f>
+        <v/>
+      </c>
+      <c r="G56" s="22">
+        <f>SUM(G10:G55)</f>
+        <v/>
+      </c>
+      <c r="H56" s="22">
+        <f>SUM(H10:H55)</f>
+        <v/>
+      </c>
+      <c r="I56" s="22">
+        <f>SUM(I10:I55)</f>
+        <v/>
+      </c>
+      <c r="J56" s="22">
+        <f>SUM(J10:J55)</f>
+        <v/>
+      </c>
+      <c r="K56" s="23">
+        <f>IF(E56&gt;0, F56/E56, 0)</f>
+        <v/>
+      </c>
+      <c r="L56" s="21">
+        <f>IF(K56&gt;=1, "SUPERADO", "EN CURSO")</f>
         <v/>
       </c>
     </row>
@@ -9488,7 +9580,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 30/09/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 01/10/2026</t>
         </is>
       </c>
     </row>
@@ -9551,7 +9643,7 @@
       <c r="I6" s="4" t="n"/>
       <c r="J6" s="24" t="inlineStr">
         <is>
-          <t>32,728 u</t>
+          <t>21,060 u</t>
         </is>
       </c>
       <c r="K6" s="4" t="n"/>
@@ -9643,10 +9735,10 @@
         <v>2200</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>0</v>
+        <v>2200</v>
       </c>
       <c r="H10" s="14" t="n">
-        <v>2200</v>
+        <v>0</v>
       </c>
       <c r="I10" s="14">
         <f>MAX(0, E10-F10)</f>
@@ -9781,10 +9873,10 @@
         <v>1000</v>
       </c>
       <c r="G13" s="18" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="H13" s="18" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="I13" s="18">
         <f>MAX(0, E13-F13)</f>
@@ -9827,10 +9919,10 @@
         <v>5500</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>0</v>
+        <v>5500</v>
       </c>
       <c r="H14" s="14" t="n">
-        <v>5500</v>
+        <v>0</v>
       </c>
       <c r="I14" s="14">
         <f>MAX(0, E14-F14)</f>
@@ -9873,10 +9965,10 @@
         <v>1000</v>
       </c>
       <c r="G15" s="18" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="H15" s="18" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="I15" s="18">
         <f>MAX(0, E15-F15)</f>
@@ -9919,10 +10011,10 @@
         <v>1968</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>0</v>
+        <v>1968</v>
       </c>
       <c r="H16" s="14" t="n">
-        <v>1968</v>
+        <v>0</v>
       </c>
       <c r="I16" s="14">
         <f>MAX(0, E16-F16)</f>
@@ -10039,7 +10131,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 30/09/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 01/10/2026</t>
         </is>
       </c>
     </row>
@@ -10102,7 +10194,7 @@
       <c r="I6" s="4" t="n"/>
       <c r="J6" s="24" t="inlineStr">
         <is>
-          <t>700 u</t>
+          <t>0 u</t>
         </is>
       </c>
       <c r="K6" s="4" t="n"/>
@@ -11022,10 +11114,10 @@
         <v>320</v>
       </c>
       <c r="G28" s="14" t="n">
-        <v>0</v>
+        <v>320</v>
       </c>
       <c r="H28" s="14" t="n">
-        <v>320</v>
+        <v>0</v>
       </c>
       <c r="I28" s="14">
         <f>MAX(0, E28-F28)</f>
@@ -11068,10 +11160,10 @@
         <v>60</v>
       </c>
       <c r="G29" s="18" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="H29" s="18" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="I29" s="18">
         <f>MAX(0, E29-F29)</f>
@@ -11114,10 +11206,10 @@
         <v>320</v>
       </c>
       <c r="G30" s="14" t="n">
-        <v>0</v>
+        <v>320</v>
       </c>
       <c r="H30" s="14" t="n">
-        <v>320</v>
+        <v>0</v>
       </c>
       <c r="I30" s="14">
         <f>MAX(0, E30-F30)</f>
@@ -11326,7 +11418,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 30/09/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 01/10/2026</t>
         </is>
       </c>
     </row>
@@ -11389,7 +11481,7 @@
       <c r="I6" s="4" t="n"/>
       <c r="J6" s="24" t="inlineStr">
         <is>
-          <t>31,858 u</t>
+          <t>10,184 u</t>
         </is>
       </c>
       <c r="K6" s="4" t="n"/>
@@ -11849,10 +11941,10 @@
         <v>2200</v>
       </c>
       <c r="G18" s="14" t="n">
-        <v>0</v>
+        <v>2200</v>
       </c>
       <c r="H18" s="14" t="n">
-        <v>2200</v>
+        <v>0</v>
       </c>
       <c r="I18" s="14">
         <f>MAX(0, E18-F18)</f>
@@ -11895,10 +11987,10 @@
         <v>6600</v>
       </c>
       <c r="G19" s="18" t="n">
-        <v>0</v>
+        <v>6600</v>
       </c>
       <c r="H19" s="18" t="n">
-        <v>6600</v>
+        <v>0</v>
       </c>
       <c r="I19" s="18">
         <f>MAX(0, E19-F19)</f>
@@ -12539,10 +12631,10 @@
         <v>368</v>
       </c>
       <c r="G33" s="18" t="n">
-        <v>0</v>
+        <v>368</v>
       </c>
       <c r="H33" s="18" t="n">
-        <v>368</v>
+        <v>0</v>
       </c>
       <c r="I33" s="18">
         <f>MAX(0, E33-F33)</f>
@@ -12585,10 +12677,10 @@
         <v>540</v>
       </c>
       <c r="G34" s="14" t="n">
-        <v>0</v>
+        <v>540</v>
       </c>
       <c r="H34" s="14" t="n">
-        <v>540</v>
+        <v>0</v>
       </c>
       <c r="I34" s="14">
         <f>MAX(0, E34-F34)</f>
@@ -12631,10 +12723,10 @@
         <v>300</v>
       </c>
       <c r="G35" s="18" t="n">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="H35" s="18" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="I35" s="18">
         <f>MAX(0, E35-F35)</f>
@@ -12677,10 +12769,10 @@
         <v>7920</v>
       </c>
       <c r="G36" s="14" t="n">
-        <v>0</v>
+        <v>7920</v>
       </c>
       <c r="H36" s="14" t="n">
-        <v>7920</v>
+        <v>0</v>
       </c>
       <c r="I36" s="14">
         <f>MAX(0, E36-F36)</f>
@@ -12723,10 +12815,10 @@
         <v>540</v>
       </c>
       <c r="G37" s="18" t="n">
-        <v>0</v>
+        <v>540</v>
       </c>
       <c r="H37" s="18" t="n">
-        <v>540</v>
+        <v>0</v>
       </c>
       <c r="I37" s="18">
         <f>MAX(0, E37-F37)</f>
@@ -12769,10 +12861,10 @@
         <v>840</v>
       </c>
       <c r="G38" s="14" t="n">
-        <v>0</v>
+        <v>840</v>
       </c>
       <c r="H38" s="14" t="n">
-        <v>840</v>
+        <v>0</v>
       </c>
       <c r="I38" s="14">
         <f>MAX(0, E38-F38)</f>
@@ -12815,10 +12907,10 @@
         <v>600</v>
       </c>
       <c r="G39" s="18" t="n">
-        <v>0</v>
+        <v>600</v>
       </c>
       <c r="H39" s="18" t="n">
-        <v>600</v>
+        <v>0</v>
       </c>
       <c r="I39" s="18">
         <f>MAX(0, E39-F39)</f>
@@ -12861,10 +12953,10 @@
         <v>1</v>
       </c>
       <c r="G40" s="14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H40" s="14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I40" s="14">
         <f>MAX(0, E40-F40)</f>
@@ -12907,10 +12999,10 @@
         <v>1</v>
       </c>
       <c r="G41" s="18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H41" s="18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I41" s="18">
         <f>MAX(0, E41-F41)</f>
@@ -12953,10 +13045,10 @@
         <v>180</v>
       </c>
       <c r="G42" s="14" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
       <c r="H42" s="14" t="n">
-        <v>180</v>
+        <v>0</v>
       </c>
       <c r="I42" s="14">
         <f>MAX(0, E42-F42)</f>
@@ -12999,10 +13091,10 @@
         <v>1584</v>
       </c>
       <c r="G43" s="18" t="n">
-        <v>0</v>
+        <v>1584</v>
       </c>
       <c r="H43" s="18" t="n">
-        <v>1584</v>
+        <v>0</v>
       </c>
       <c r="I43" s="18">
         <f>MAX(0, E43-F43)</f>

</xml_diff>

<commit_message>
Actualizacion pedidos y planificacion: 06/10/2026
</commit_message>
<xml_diff>
--- a/Seguimiento_Presupuesto_Sep_2026.xlsx
+++ b/Seguimiento_Presupuesto_Sep_2026.xlsx
@@ -906,7 +906,7 @@
     <row r="3" ht="20" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Comparativa Estimación Septiembre (Unidades) vs Pedidos Reales a Fecha 05/10/2026 | Generado: 05/10/2026 08:42</t>
+          <t>Comparativa Estimación Septiembre (Unidades) vs Pedidos Reales a Fecha 06/10/2026 | Generado: 06/10/2026 08:13</t>
         </is>
       </c>
     </row>
@@ -950,25 +950,25 @@
       <c r="C6" s="4" t="n"/>
       <c r="D6" s="8" t="inlineStr">
         <is>
-          <t>10,341 u</t>
+          <t>10,741 u</t>
         </is>
       </c>
       <c r="E6" s="4" t="n"/>
       <c r="F6" s="9" t="inlineStr">
         <is>
-          <t>5.7%</t>
+          <t>5.9%</t>
         </is>
       </c>
       <c r="G6" s="4" t="n"/>
       <c r="H6" s="10" t="inlineStr">
         <is>
-          <t>171,625 u</t>
+          <t>171,225 u</t>
         </is>
       </c>
       <c r="I6" s="4" t="n"/>
       <c r="J6" s="7" t="inlineStr">
         <is>
-          <t>2,000 u</t>
+          <t>0 u</t>
         </is>
       </c>
     </row>
@@ -1039,10 +1039,10 @@
         <v>2320</v>
       </c>
       <c r="E10" s="15" t="n">
-        <v>200</v>
+        <v>400</v>
       </c>
       <c r="F10" s="15" t="n">
-        <v>200</v>
+        <v>400</v>
       </c>
       <c r="G10" s="15" t="n">
         <v>0</v>
@@ -1110,10 +1110,10 @@
         <v>4841</v>
       </c>
       <c r="F12" s="15" t="n">
-        <v>4201</v>
+        <v>4841</v>
       </c>
       <c r="G12" s="15" t="n">
-        <v>640</v>
+        <v>0</v>
       </c>
       <c r="H12" s="15">
         <f>MAX(0, D12-E12)</f>
@@ -1141,13 +1141,13 @@
         <v>17100</v>
       </c>
       <c r="E13" s="19" t="n">
-        <v>620</v>
+        <v>820</v>
       </c>
       <c r="F13" s="19" t="n">
-        <v>0</v>
+        <v>820</v>
       </c>
       <c r="G13" s="19" t="n">
-        <v>620</v>
+        <v>0</v>
       </c>
       <c r="H13" s="19">
         <f>MAX(0, D13-E13)</f>
@@ -1212,10 +1212,10 @@
         <v>4680</v>
       </c>
       <c r="F15" s="19" t="n">
-        <v>3940</v>
+        <v>4680</v>
       </c>
       <c r="G15" s="19" t="n">
-        <v>740</v>
+        <v>0</v>
       </c>
       <c r="H15" s="19">
         <f>MAX(0, D15-E15)</f>
@@ -1354,7 +1354,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 05/10/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 06/10/2026</t>
         </is>
       </c>
     </row>
@@ -1399,19 +1399,19 @@
       <c r="C6" s="4" t="n"/>
       <c r="D6" s="25" t="inlineStr">
         <is>
-          <t>200 u</t>
+          <t>400 u</t>
         </is>
       </c>
       <c r="E6" s="4" t="n"/>
       <c r="F6" s="26" t="inlineStr">
         <is>
-          <t>8.6%</t>
+          <t>17.2%</t>
         </is>
       </c>
       <c r="G6" s="4" t="n"/>
       <c r="H6" s="26" t="inlineStr">
         <is>
-          <t>2,120 u</t>
+          <t>1,920 u</t>
         </is>
       </c>
       <c r="I6" s="4" t="n"/>
@@ -1598,10 +1598,10 @@
         <v>0</v>
       </c>
       <c r="F12" s="15" t="n">
-        <v>200</v>
+        <v>400</v>
       </c>
       <c r="G12" s="15" t="n">
-        <v>200</v>
+        <v>400</v>
       </c>
       <c r="H12" s="15" t="n">
         <v>0</v>
@@ -1767,7 +1767,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 05/10/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 06/10/2026</t>
         </is>
       </c>
     </row>
@@ -3100,7 +3100,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 05/10/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 06/10/2026</t>
         </is>
       </c>
     </row>
@@ -3163,7 +3163,7 @@
       <c r="I6" s="4" t="n"/>
       <c r="J6" s="25" t="inlineStr">
         <is>
-          <t>640 u</t>
+          <t>0 u</t>
         </is>
       </c>
       <c r="K6" s="4" t="n"/>
@@ -3715,10 +3715,10 @@
         <v>640</v>
       </c>
       <c r="G20" s="15" t="n">
-        <v>0</v>
+        <v>640</v>
       </c>
       <c r="H20" s="15" t="n">
-        <v>640</v>
+        <v>0</v>
       </c>
       <c r="I20" s="15">
         <f>MAX(0, E20-F20)</f>
@@ -4801,7 +4801,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 05/10/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 06/10/2026</t>
         </is>
       </c>
     </row>
@@ -4846,25 +4846,25 @@
       <c r="C6" s="4" t="n"/>
       <c r="D6" s="25" t="inlineStr">
         <is>
-          <t>620 u</t>
+          <t>820 u</t>
         </is>
       </c>
       <c r="E6" s="4" t="n"/>
       <c r="F6" s="26" t="inlineStr">
         <is>
-          <t>3.6%</t>
+          <t>4.8%</t>
         </is>
       </c>
       <c r="G6" s="4" t="n"/>
       <c r="H6" s="26" t="inlineStr">
         <is>
-          <t>16,480 u</t>
+          <t>16,280 u</t>
         </is>
       </c>
       <c r="I6" s="4" t="n"/>
       <c r="J6" s="25" t="inlineStr">
         <is>
-          <t>620 u</t>
+          <t>0 u</t>
         </is>
       </c>
       <c r="K6" s="4" t="n"/>
@@ -5091,13 +5091,13 @@
         <v>0</v>
       </c>
       <c r="F13" s="19" t="n">
-        <v>100</v>
+        <v>300</v>
       </c>
       <c r="G13" s="19" t="n">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="H13" s="19" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="I13" s="19">
         <f>MAX(0, E13-F13)</f>
@@ -5232,10 +5232,10 @@
         <v>200</v>
       </c>
       <c r="G16" s="15" t="n">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="H16" s="15" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="I16" s="15">
         <f>MAX(0, E16-F16)</f>
@@ -5278,10 +5278,10 @@
         <v>320</v>
       </c>
       <c r="G17" s="19" t="n">
-        <v>0</v>
+        <v>320</v>
       </c>
       <c r="H17" s="19" t="n">
-        <v>320</v>
+        <v>0</v>
       </c>
       <c r="I17" s="19">
         <f>MAX(0, E17-F17)</f>
@@ -5490,7 +5490,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 05/10/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 06/10/2026</t>
         </is>
       </c>
     </row>
@@ -5995,7 +5995,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 05/10/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 06/10/2026</t>
         </is>
       </c>
     </row>
@@ -6058,7 +6058,7 @@
       <c r="I6" s="4" t="n"/>
       <c r="J6" s="25" t="inlineStr">
         <is>
-          <t>740 u</t>
+          <t>0 u</t>
         </is>
       </c>
       <c r="K6" s="4" t="n"/>
@@ -6150,10 +6150,10 @@
         <v>640</v>
       </c>
       <c r="G10" s="15" t="n">
-        <v>0</v>
+        <v>640</v>
       </c>
       <c r="H10" s="15" t="n">
-        <v>640</v>
+        <v>0</v>
       </c>
       <c r="I10" s="15">
         <f>MAX(0, E10-F10)</f>
@@ -6334,10 +6334,10 @@
         <v>100</v>
       </c>
       <c r="G14" s="15" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="H14" s="15" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="I14" s="15">
         <f>MAX(0, E14-F14)</f>
@@ -6914,7 +6914,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 05/10/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 06/10/2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizacion dashboard, pedidos 07.10, modulo tesoreria cash flow y mejoras MRP
</commit_message>
<xml_diff>
--- a/Seguimiento_Presupuesto_Sep_2026.xlsx
+++ b/Seguimiento_Presupuesto_Sep_2026.xlsx
@@ -339,13 +339,13 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="8" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="16" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -906,7 +906,7 @@
     <row r="3" ht="20" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Comparativa Estimación Septiembre (Unidades) vs Pedidos Reales a Fecha 06/10/2026 | Generado: 06/10/2026 08:13</t>
+          <t>Comparativa Estimación Septiembre (Unidades) vs Pedidos Reales a Fecha 07/10/2026 | Generado: 07/10/2026 07:17</t>
         </is>
       </c>
     </row>
@@ -950,25 +950,25 @@
       <c r="C6" s="4" t="n"/>
       <c r="D6" s="8" t="inlineStr">
         <is>
-          <t>10,741 u</t>
+          <t>48,541 u</t>
         </is>
       </c>
       <c r="E6" s="4" t="n"/>
       <c r="F6" s="9" t="inlineStr">
         <is>
-          <t>5.9%</t>
+          <t>26.7%</t>
         </is>
       </c>
       <c r="G6" s="4" t="n"/>
       <c r="H6" s="10" t="inlineStr">
         <is>
-          <t>171,225 u</t>
+          <t>133,425 u</t>
         </is>
       </c>
       <c r="I6" s="4" t="n"/>
       <c r="J6" s="7" t="inlineStr">
         <is>
-          <t>0 u</t>
+          <t>37,801 u</t>
         </is>
       </c>
     </row>
@@ -1067,26 +1067,26 @@
         </is>
       </c>
       <c r="C11" s="18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D11" s="19" t="n">
         <v>37832</v>
       </c>
       <c r="E11" s="19" t="n">
-        <v>0</v>
+        <v>37800</v>
       </c>
       <c r="F11" s="19" t="n">
         <v>0</v>
       </c>
       <c r="G11" s="19" t="n">
-        <v>0</v>
+        <v>37800</v>
       </c>
       <c r="H11" s="19">
         <f>MAX(0, D11-E11)</f>
         <v/>
       </c>
       <c r="I11" s="19">
-        <f>'García'!J34</f>
+        <f>'García'!J35</f>
         <v/>
       </c>
       <c r="J11" s="20">
@@ -1110,10 +1110,10 @@
         <v>4841</v>
       </c>
       <c r="F12" s="15" t="n">
-        <v>4841</v>
+        <v>4840</v>
       </c>
       <c r="G12" s="15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H12" s="15">
         <f>MAX(0, D12-E12)</f>
@@ -1354,7 +1354,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 06/10/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 07/10/2026</t>
         </is>
       </c>
     </row>
@@ -1740,7 +1740,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:L34"/>
+  <dimension ref="B2:L35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1767,7 +1767,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 06/10/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 07/10/2026</t>
         </is>
       </c>
     </row>
@@ -1812,25 +1812,25 @@
       <c r="C6" s="4" t="n"/>
       <c r="D6" s="25" t="inlineStr">
         <is>
-          <t>0 u</t>
+          <t>37,800 u</t>
         </is>
       </c>
       <c r="E6" s="4" t="n"/>
       <c r="F6" s="26" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>99.9%</t>
         </is>
       </c>
       <c r="G6" s="4" t="n"/>
       <c r="H6" s="26" t="inlineStr">
         <is>
-          <t>37,832 u</t>
+          <t>32 u</t>
         </is>
       </c>
       <c r="I6" s="4" t="n"/>
       <c r="J6" s="25" t="inlineStr">
         <is>
-          <t>0 u</t>
+          <t>37,800 u</t>
         </is>
       </c>
       <c r="K6" s="4" t="n"/>
@@ -2551,25 +2551,25 @@
       </c>
       <c r="C24" s="29" t="inlineStr">
         <is>
-          <t>SSEG0005</t>
+          <t>AGXK0005</t>
         </is>
       </c>
       <c r="D24" s="28" t="inlineStr">
         <is>
-          <t>SAL-WAX Ca</t>
+          <t>AGROXILATO+K</t>
         </is>
       </c>
       <c r="E24" s="15" t="n">
-        <v>20000</v>
+        <v>0</v>
       </c>
       <c r="F24" s="15" t="n">
-        <v>0</v>
+        <v>16800</v>
       </c>
       <c r="G24" s="15" t="n">
         <v>0</v>
       </c>
       <c r="H24" s="15" t="n">
-        <v>0</v>
+        <v>16800</v>
       </c>
       <c r="I24" s="15">
         <f>MAX(0, E24-F24)</f>
@@ -2583,39 +2583,39 @@
         <f>IF(E24&gt;0, F24/E24, IF(F24&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L24" s="30" t="inlineStr">
-        <is>
-          <t>Sin Pedido</t>
+      <c r="L24" s="34" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="B25" s="31" t="inlineStr">
         <is>
-          <t>INIESTA DEL PINO DISTRIBUCIONES S.L.U</t>
+          <t>DOTRA CHEMICALS</t>
         </is>
       </c>
       <c r="C25" s="32" t="inlineStr">
         <is>
-          <t>AGXK0020</t>
+          <t>SSEG0005</t>
         </is>
       </c>
       <c r="D25" s="31" t="inlineStr">
         <is>
-          <t>AGROXILATO-K, 20 L</t>
+          <t>SAL-WAX Ca</t>
         </is>
       </c>
       <c r="E25" s="19" t="n">
-        <v>640</v>
+        <v>20000</v>
       </c>
       <c r="F25" s="19" t="n">
-        <v>0</v>
+        <v>21000</v>
       </c>
       <c r="G25" s="19" t="n">
         <v>0</v>
       </c>
       <c r="H25" s="19" t="n">
-        <v>0</v>
+        <v>21000</v>
       </c>
       <c r="I25" s="19">
         <f>MAX(0, E25-F25)</f>
@@ -2629,9 +2629,9 @@
         <f>IF(E25&gt;0, F25/E25, IF(F25&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L25" s="33" t="inlineStr">
-        <is>
-          <t>Sin Pedido</t>
+      <c r="L25" s="37" t="inlineStr">
+        <is>
+          <t>Superado</t>
         </is>
       </c>
     </row>
@@ -2643,16 +2643,16 @@
       </c>
       <c r="C26" s="29" t="inlineStr">
         <is>
-          <t>TRI0005</t>
+          <t>AGXK0020</t>
         </is>
       </c>
       <c r="D26" s="28" t="inlineStr">
         <is>
-          <t>TRIFENO-94, 5L</t>
+          <t>AGROXILATO-K, 20 L</t>
         </is>
       </c>
       <c r="E26" s="15" t="n">
-        <v>60</v>
+        <v>640</v>
       </c>
       <c r="F26" s="15" t="n">
         <v>0</v>
@@ -2684,21 +2684,21 @@
     <row r="27">
       <c r="B27" s="31" t="inlineStr">
         <is>
-          <t>SERVIAGRI´ 97, S.L.</t>
+          <t>INIESTA DEL PINO DISTRIBUCIONES S.L.U</t>
         </is>
       </c>
       <c r="C27" s="32" t="inlineStr">
         <is>
-          <t>AGXK0005</t>
+          <t>TRI0005</t>
         </is>
       </c>
       <c r="D27" s="31" t="inlineStr">
         <is>
-          <t>AGROXILATO-K, 5 L</t>
+          <t>TRIFENO-94, 5L</t>
         </is>
       </c>
       <c r="E27" s="19" t="n">
-        <v>200</v>
+        <v>60</v>
       </c>
       <c r="F27" s="19" t="n">
         <v>0</v>
@@ -2735,16 +2735,16 @@
       </c>
       <c r="C28" s="29" t="inlineStr">
         <is>
-          <t>AVAN0005</t>
+          <t>AGXK0005</t>
         </is>
       </c>
       <c r="D28" s="28" t="inlineStr">
         <is>
-          <t>FLORAMEC AVANCE, 5 L</t>
+          <t>AGROXILATO-K, 5 L</t>
         </is>
       </c>
       <c r="E28" s="15" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="F28" s="15" t="n">
         <v>0</v>
@@ -2781,16 +2781,16 @@
       </c>
       <c r="C29" s="32" t="inlineStr">
         <is>
-          <t>B0001</t>
+          <t>AVAN0005</t>
         </is>
       </c>
       <c r="D29" s="31" t="inlineStr">
         <is>
-          <t>BOROCAL,1 L</t>
+          <t>FLORAMEC AVANCE, 5 L</t>
         </is>
       </c>
       <c r="E29" s="19" t="n">
-        <v>12</v>
+        <v>100</v>
       </c>
       <c r="F29" s="19" t="n">
         <v>0</v>
@@ -2827,16 +2827,16 @@
       </c>
       <c r="C30" s="29" t="inlineStr">
         <is>
-          <t>BIO0005</t>
+          <t>B0001</t>
         </is>
       </c>
       <c r="D30" s="28" t="inlineStr">
         <is>
-          <t>BIORAD-20, 5L</t>
+          <t>BOROCAL,1 L</t>
         </is>
       </c>
       <c r="E30" s="15" t="n">
-        <v>300</v>
+        <v>12</v>
       </c>
       <c r="F30" s="15" t="n">
         <v>0</v>
@@ -2873,12 +2873,12 @@
       </c>
       <c r="C31" s="32" t="inlineStr">
         <is>
-          <t>FTK0005</t>
+          <t>BIO0005</t>
         </is>
       </c>
       <c r="D31" s="31" t="inlineStr">
         <is>
-          <t>FITOKONTROL CA FLOW, 5 KG</t>
+          <t>BIORAD-20, 5L</t>
         </is>
       </c>
       <c r="E31" s="19" t="n">
@@ -2919,16 +2919,16 @@
       </c>
       <c r="C32" s="29" t="inlineStr">
         <is>
-          <t>JF0005</t>
+          <t>FTK0005</t>
         </is>
       </c>
       <c r="D32" s="28" t="inlineStr">
         <is>
-          <t>CODIGIN-FOS, 5 L</t>
+          <t>FITOKONTROL CA FLOW, 5 KG</t>
         </is>
       </c>
       <c r="E32" s="15" t="n">
-        <v>100</v>
+        <v>300</v>
       </c>
       <c r="F32" s="15" t="n">
         <v>0</v>
@@ -2960,21 +2960,21 @@
     <row r="33">
       <c r="B33" s="31" t="inlineStr">
         <is>
-          <t>TRATAMIENTOS AGRICOLAS BRENES, S.L.</t>
+          <t>SERVIAGRI´ 97, S.L.</t>
         </is>
       </c>
       <c r="C33" s="32" t="inlineStr">
         <is>
-          <t>WHITE0020</t>
+          <t>JF0005</t>
         </is>
       </c>
       <c r="D33" s="31" t="inlineStr">
         <is>
-          <t>AGROWHITE, 20 KG</t>
+          <t>CODIGIN-FOS, 5 L</t>
         </is>
       </c>
       <c r="E33" s="19" t="n">
-        <v>1100</v>
+        <v>100</v>
       </c>
       <c r="F33" s="19" t="n">
         <v>0</v>
@@ -3003,48 +3003,94 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="24" customHeight="1">
-      <c r="B34" s="21" t="inlineStr">
+    <row r="34">
+      <c r="B34" s="28" t="inlineStr">
+        <is>
+          <t>TRATAMIENTOS AGRICOLAS BRENES, S.L.</t>
+        </is>
+      </c>
+      <c r="C34" s="29" t="inlineStr">
+        <is>
+          <t>WHITE0020</t>
+        </is>
+      </c>
+      <c r="D34" s="28" t="inlineStr">
+        <is>
+          <t>AGROWHITE, 20 KG</t>
+        </is>
+      </c>
+      <c r="E34" s="15" t="n">
+        <v>1100</v>
+      </c>
+      <c r="F34" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G34" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H34" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I34" s="15">
+        <f>MAX(0, E34-F34)</f>
+        <v/>
+      </c>
+      <c r="J34" s="15">
+        <f>ABS(F34-E34)</f>
+        <v/>
+      </c>
+      <c r="K34" s="16">
+        <f>IF(E34&gt;0, F34/E34, IF(F34&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L34" s="30" t="inlineStr">
+        <is>
+          <t>Sin Pedido</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="24" customHeight="1">
+      <c r="B35" s="21" t="inlineStr">
         <is>
           <t>TOTAL GARCÍA</t>
         </is>
       </c>
-      <c r="C34" s="35" t="inlineStr">
+      <c r="C35" s="35" t="inlineStr">
         <is>
           <t>230 líneas</t>
         </is>
       </c>
-      <c r="D34" s="36" t="inlineStr"/>
-      <c r="E34" s="23">
-        <f>SUM(E10:E33)</f>
-        <v/>
-      </c>
-      <c r="F34" s="23">
-        <f>SUM(F10:F33)</f>
-        <v/>
-      </c>
-      <c r="G34" s="23">
-        <f>SUM(G10:G33)</f>
-        <v/>
-      </c>
-      <c r="H34" s="23">
-        <f>SUM(H10:H33)</f>
-        <v/>
-      </c>
-      <c r="I34" s="23">
-        <f>SUM(I10:I33)</f>
-        <v/>
-      </c>
-      <c r="J34" s="23">
-        <f>SUM(J10:J33)</f>
-        <v/>
-      </c>
-      <c r="K34" s="24">
-        <f>IF(E34&gt;0, F34/E34, 0)</f>
-        <v/>
-      </c>
-      <c r="L34" s="22">
-        <f>IF(K34&gt;=1, "SUPERADO", "EN CURSO")</f>
+      <c r="D35" s="36" t="inlineStr"/>
+      <c r="E35" s="23">
+        <f>SUM(E10:E34)</f>
+        <v/>
+      </c>
+      <c r="F35" s="23">
+        <f>SUM(F10:F34)</f>
+        <v/>
+      </c>
+      <c r="G35" s="23">
+        <f>SUM(G10:G34)</f>
+        <v/>
+      </c>
+      <c r="H35" s="23">
+        <f>SUM(H10:H34)</f>
+        <v/>
+      </c>
+      <c r="I35" s="23">
+        <f>SUM(I10:I34)</f>
+        <v/>
+      </c>
+      <c r="J35" s="23">
+        <f>SUM(J10:J34)</f>
+        <v/>
+      </c>
+      <c r="K35" s="24">
+        <f>IF(E35&gt;0, F35/E35, 0)</f>
+        <v/>
+      </c>
+      <c r="L35" s="22">
+        <f>IF(K35&gt;=1, "SUPERADO", "EN CURSO")</f>
         <v/>
       </c>
     </row>
@@ -3100,7 +3146,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 06/10/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 07/10/2026</t>
         </is>
       </c>
     </row>
@@ -3163,7 +3209,7 @@
       <c r="I6" s="4" t="n"/>
       <c r="J6" s="25" t="inlineStr">
         <is>
-          <t>0 u</t>
+          <t>1 u</t>
         </is>
       </c>
       <c r="K6" s="4" t="n"/>
@@ -3732,7 +3778,7 @@
         <f>IF(E20&gt;0, F20/E20, IF(F20&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L20" s="37" t="inlineStr">
+      <c r="L20" s="38" t="inlineStr">
         <is>
           <t>En Curso</t>
         </is>
@@ -3824,7 +3870,7 @@
         <f>IF(E22&gt;0, F22/E22, IF(F22&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L22" s="38" t="inlineStr">
+      <c r="L22" s="39" t="inlineStr">
         <is>
           <t>Rezagado</t>
         </is>
@@ -3945,10 +3991,10 @@
         <v>1</v>
       </c>
       <c r="G25" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" s="19" t="n">
         <v>1</v>
-      </c>
-      <c r="H25" s="19" t="n">
-        <v>0</v>
       </c>
       <c r="I25" s="19">
         <f>MAX(0, E25-F25)</f>
@@ -3962,7 +4008,7 @@
         <f>IF(E25&gt;0, F25/E25, IF(F25&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L25" s="39" t="inlineStr">
+      <c r="L25" s="37" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -4100,7 +4146,7 @@
         <f>IF(E28&gt;0, F28/E28, IF(F28&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L28" s="37" t="inlineStr">
+      <c r="L28" s="38" t="inlineStr">
         <is>
           <t>En Curso</t>
         </is>
@@ -4146,7 +4192,7 @@
         <f>IF(E29&gt;0, F29/E29, IF(F29&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L29" s="39" t="inlineStr">
+      <c r="L29" s="37" t="inlineStr">
         <is>
           <t>Superado</t>
         </is>
@@ -4192,7 +4238,7 @@
         <f>IF(E30&gt;0, F30/E30, IF(F30&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L30" s="37" t="inlineStr">
+      <c r="L30" s="38" t="inlineStr">
         <is>
           <t>En Curso</t>
         </is>
@@ -4801,7 +4847,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 06/10/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 07/10/2026</t>
         </is>
       </c>
     </row>
@@ -5111,7 +5157,7 @@
         <f>IF(E13&gt;0, F13/E13, IF(F13&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L13" s="39" t="inlineStr">
+      <c r="L13" s="37" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -5295,7 +5341,7 @@
         <f>IF(E17&gt;0, F17/E17, IF(F17&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L17" s="39" t="inlineStr">
+      <c r="L17" s="37" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -5490,7 +5536,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 06/10/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 07/10/2026</t>
         </is>
       </c>
     </row>
@@ -5995,7 +6041,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 06/10/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 07/10/2026</t>
         </is>
       </c>
     </row>
@@ -6581,7 +6627,7 @@
         <f>IF(E19&gt;0, F19/E19, IF(F19&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L19" s="39" t="inlineStr">
+      <c r="L19" s="37" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -6673,7 +6719,7 @@
         <f>IF(E21&gt;0, F21/E21, IF(F21&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L21" s="39" t="inlineStr">
+      <c r="L21" s="37" t="inlineStr">
         <is>
           <t>Superado</t>
         </is>
@@ -6914,7 +6960,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 06/10/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 07/10/2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizacion diaria de pedidos y stock al 08.10.2026: 53.240 u pedidos en Octubre y 75.569 u pendientes en MRP
</commit_message>
<xml_diff>
--- a/Seguimiento_Presupuesto_Sep_2026.xlsx
+++ b/Seguimiento_Presupuesto_Sep_2026.xlsx
@@ -113,7 +113,8 @@
     </font>
     <font>
       <name val="Segoe UI"/>
-      <color rgb="0064748B"/>
+      <b val="1"/>
+      <color rgb="0092400E"/>
       <sz val="9"/>
     </font>
     <font>
@@ -124,8 +125,7 @@
     </font>
     <font>
       <name val="Segoe UI"/>
-      <b val="1"/>
-      <color rgb="0092400E"/>
+      <color rgb="0064748B"/>
       <sz val="9"/>
     </font>
     <font>
@@ -237,7 +237,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -320,7 +320,7 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -335,20 +335,23 @@
     <xf numFmtId="0" fontId="15" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="8" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -906,7 +909,7 @@
     <row r="3" ht="20" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Comparativa Estimación Septiembre (Unidades) vs Pedidos Reales a Fecha 07/10/2026 | Generado: 07/10/2026 07:17</t>
+          <t>Comparativa Estimación Septiembre (Unidades) vs Pedidos Reales a Fecha 08/10/2026 | Generado: 08/10/2026 07:30</t>
         </is>
       </c>
     </row>
@@ -950,25 +953,25 @@
       <c r="C6" s="4" t="n"/>
       <c r="D6" s="8" t="inlineStr">
         <is>
-          <t>48,541 u</t>
+          <t>53,240 u</t>
         </is>
       </c>
       <c r="E6" s="4" t="n"/>
       <c r="F6" s="9" t="inlineStr">
         <is>
-          <t>26.7%</t>
+          <t>29.3%</t>
         </is>
       </c>
       <c r="G6" s="4" t="n"/>
       <c r="H6" s="10" t="inlineStr">
         <is>
-          <t>133,425 u</t>
+          <t>128,726 u</t>
         </is>
       </c>
       <c r="I6" s="4" t="n"/>
       <c r="J6" s="7" t="inlineStr">
         <is>
-          <t>37,801 u</t>
+          <t>38,800 u</t>
         </is>
       </c>
     </row>
@@ -1033,16 +1036,16 @@
         </is>
       </c>
       <c r="C10" s="14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D10" s="15" t="n">
         <v>2320</v>
       </c>
       <c r="E10" s="15" t="n">
-        <v>400</v>
+        <v>1680</v>
       </c>
       <c r="F10" s="15" t="n">
-        <v>400</v>
+        <v>1680</v>
       </c>
       <c r="G10" s="15" t="n">
         <v>0</v>
@@ -1107,20 +1110,20 @@
         <v>21914</v>
       </c>
       <c r="E12" s="15" t="n">
-        <v>4841</v>
+        <v>6620</v>
       </c>
       <c r="F12" s="15" t="n">
-        <v>4840</v>
+        <v>6620</v>
       </c>
       <c r="G12" s="15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H12" s="15">
         <f>MAX(0, D12-E12)</f>
         <v/>
       </c>
       <c r="I12" s="15">
-        <f>'Irene'!J42</f>
+        <f>'Irene'!J45</f>
         <v/>
       </c>
       <c r="J12" s="16">
@@ -1135,26 +1138,26 @@
         </is>
       </c>
       <c r="C13" s="18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D13" s="19" t="n">
         <v>17100</v>
       </c>
       <c r="E13" s="19" t="n">
-        <v>820</v>
+        <v>2460</v>
       </c>
       <c r="F13" s="19" t="n">
-        <v>820</v>
+        <v>1460</v>
       </c>
       <c r="G13" s="19" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="H13" s="19">
         <f>MAX(0, D13-E13)</f>
         <v/>
       </c>
       <c r="I13" s="19">
-        <f>'Javier'!J20</f>
+        <f>'Javier'!J22</f>
         <v/>
       </c>
       <c r="J13" s="20">
@@ -1354,7 +1357,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 07/10/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 08/10/2026</t>
         </is>
       </c>
     </row>
@@ -1399,19 +1402,19 @@
       <c r="C6" s="4" t="n"/>
       <c r="D6" s="25" t="inlineStr">
         <is>
-          <t>400 u</t>
+          <t>1,680 u</t>
         </is>
       </c>
       <c r="E6" s="4" t="n"/>
       <c r="F6" s="26" t="inlineStr">
         <is>
-          <t>17.2%</t>
+          <t>72.4%</t>
         </is>
       </c>
       <c r="G6" s="4" t="n"/>
       <c r="H6" s="26" t="inlineStr">
         <is>
-          <t>1,920 u</t>
+          <t>640 u</t>
         </is>
       </c>
       <c r="I6" s="4" t="n"/>
@@ -1506,10 +1509,10 @@
         <v>960</v>
       </c>
       <c r="F10" s="15" t="n">
-        <v>0</v>
+        <v>640</v>
       </c>
       <c r="G10" s="15" t="n">
-        <v>0</v>
+        <v>640</v>
       </c>
       <c r="H10" s="15" t="n">
         <v>0</v>
@@ -1528,7 +1531,7 @@
       </c>
       <c r="L10" s="30" t="inlineStr">
         <is>
-          <t>Sin Pedido</t>
+          <t>En Curso</t>
         </is>
       </c>
     </row>
@@ -1552,10 +1555,10 @@
         <v>960</v>
       </c>
       <c r="F11" s="19" t="n">
-        <v>0</v>
+        <v>640</v>
       </c>
       <c r="G11" s="19" t="n">
-        <v>0</v>
+        <v>640</v>
       </c>
       <c r="H11" s="19" t="n">
         <v>0</v>
@@ -1574,7 +1577,7 @@
       </c>
       <c r="L11" s="33" t="inlineStr">
         <is>
-          <t>Sin Pedido</t>
+          <t>En Curso</t>
         </is>
       </c>
     </row>
@@ -1664,7 +1667,7 @@
         <f>IF(E13&gt;0, F13/E13, IF(F13&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L13" s="33" t="inlineStr">
+      <c r="L13" s="35" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -1676,12 +1679,12 @@
           <t>TOTAL ALFONSO</t>
         </is>
       </c>
-      <c r="C14" s="35" t="inlineStr">
+      <c r="C14" s="36" t="inlineStr">
         <is>
           <t>276 líneas</t>
         </is>
       </c>
-      <c r="D14" s="36" t="inlineStr"/>
+      <c r="D14" s="37" t="inlineStr"/>
       <c r="E14" s="23">
         <f>SUM(E10:E13)</f>
         <v/>
@@ -1767,7 +1770,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 07/10/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 08/10/2026</t>
         </is>
       </c>
     </row>
@@ -1939,7 +1942,7 @@
         <f>IF(E10&gt;0, F10/E10, IF(F10&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L10" s="30" t="inlineStr">
+      <c r="L10" s="38" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -1985,7 +1988,7 @@
         <f>IF(E11&gt;0, F11/E11, IF(F11&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L11" s="33" t="inlineStr">
+      <c r="L11" s="35" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -2031,7 +2034,7 @@
         <f>IF(E12&gt;0, F12/E12, IF(F12&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L12" s="30" t="inlineStr">
+      <c r="L12" s="38" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -2077,7 +2080,7 @@
         <f>IF(E13&gt;0, F13/E13, IF(F13&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L13" s="33" t="inlineStr">
+      <c r="L13" s="35" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -2123,7 +2126,7 @@
         <f>IF(E14&gt;0, F14/E14, IF(F14&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L14" s="30" t="inlineStr">
+      <c r="L14" s="38" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -2169,7 +2172,7 @@
         <f>IF(E15&gt;0, F15/E15, IF(F15&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L15" s="33" t="inlineStr">
+      <c r="L15" s="35" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -2215,7 +2218,7 @@
         <f>IF(E16&gt;0, F16/E16, IF(F16&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L16" s="30" t="inlineStr">
+      <c r="L16" s="38" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -2261,7 +2264,7 @@
         <f>IF(E17&gt;0, F17/E17, IF(F17&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L17" s="33" t="inlineStr">
+      <c r="L17" s="35" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -2307,7 +2310,7 @@
         <f>IF(E18&gt;0, F18/E18, IF(F18&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L18" s="30" t="inlineStr">
+      <c r="L18" s="38" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -2353,7 +2356,7 @@
         <f>IF(E19&gt;0, F19/E19, IF(F19&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L19" s="33" t="inlineStr">
+      <c r="L19" s="35" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -2399,7 +2402,7 @@
         <f>IF(E20&gt;0, F20/E20, IF(F20&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L20" s="30" t="inlineStr">
+      <c r="L20" s="38" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -2445,7 +2448,7 @@
         <f>IF(E21&gt;0, F21/E21, IF(F21&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L21" s="33" t="inlineStr">
+      <c r="L21" s="35" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -2491,7 +2494,7 @@
         <f>IF(E22&gt;0, F22/E22, IF(F22&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L22" s="30" t="inlineStr">
+      <c r="L22" s="38" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -2537,7 +2540,7 @@
         <f>IF(E23&gt;0, F23/E23, IF(F23&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L23" s="33" t="inlineStr">
+      <c r="L23" s="35" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -2629,7 +2632,7 @@
         <f>IF(E25&gt;0, F25/E25, IF(F25&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L25" s="37" t="inlineStr">
+      <c r="L25" s="39" t="inlineStr">
         <is>
           <t>Superado</t>
         </is>
@@ -2675,7 +2678,7 @@
         <f>IF(E26&gt;0, F26/E26, IF(F26&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L26" s="30" t="inlineStr">
+      <c r="L26" s="38" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -2721,7 +2724,7 @@
         <f>IF(E27&gt;0, F27/E27, IF(F27&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L27" s="33" t="inlineStr">
+      <c r="L27" s="35" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -2767,7 +2770,7 @@
         <f>IF(E28&gt;0, F28/E28, IF(F28&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L28" s="30" t="inlineStr">
+      <c r="L28" s="38" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -2813,7 +2816,7 @@
         <f>IF(E29&gt;0, F29/E29, IF(F29&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L29" s="33" t="inlineStr">
+      <c r="L29" s="35" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -2859,7 +2862,7 @@
         <f>IF(E30&gt;0, F30/E30, IF(F30&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L30" s="30" t="inlineStr">
+      <c r="L30" s="38" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -2905,7 +2908,7 @@
         <f>IF(E31&gt;0, F31/E31, IF(F31&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L31" s="33" t="inlineStr">
+      <c r="L31" s="35" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -2951,7 +2954,7 @@
         <f>IF(E32&gt;0, F32/E32, IF(F32&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L32" s="30" t="inlineStr">
+      <c r="L32" s="38" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -2997,7 +3000,7 @@
         <f>IF(E33&gt;0, F33/E33, IF(F33&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L33" s="33" t="inlineStr">
+      <c r="L33" s="35" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -3043,7 +3046,7 @@
         <f>IF(E34&gt;0, F34/E34, IF(F34&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L34" s="30" t="inlineStr">
+      <c r="L34" s="38" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -3055,12 +3058,12 @@
           <t>TOTAL GARCÍA</t>
         </is>
       </c>
-      <c r="C35" s="35" t="inlineStr">
+      <c r="C35" s="36" t="inlineStr">
         <is>
           <t>230 líneas</t>
         </is>
       </c>
-      <c r="D35" s="36" t="inlineStr"/>
+      <c r="D35" s="37" t="inlineStr"/>
       <c r="E35" s="23">
         <f>SUM(E10:E34)</f>
         <v/>
@@ -3119,7 +3122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:L42"/>
+  <dimension ref="B2:L45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -3146,7 +3149,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 07/10/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 08/10/2026</t>
         </is>
       </c>
     </row>
@@ -3191,25 +3194,25 @@
       <c r="C6" s="4" t="n"/>
       <c r="D6" s="25" t="inlineStr">
         <is>
-          <t>4,841 u</t>
+          <t>6,620 u</t>
         </is>
       </c>
       <c r="E6" s="4" t="n"/>
       <c r="F6" s="26" t="inlineStr">
         <is>
-          <t>22.1%</t>
+          <t>30.2%</t>
         </is>
       </c>
       <c r="G6" s="4" t="n"/>
       <c r="H6" s="26" t="inlineStr">
         <is>
-          <t>17,073 u</t>
+          <t>15,294 u</t>
         </is>
       </c>
       <c r="I6" s="4" t="n"/>
       <c r="J6" s="25" t="inlineStr">
         <is>
-          <t>1 u</t>
+          <t>0 u</t>
         </is>
       </c>
       <c r="K6" s="4" t="n"/>
@@ -3318,7 +3321,7 @@
         <f>IF(E10&gt;0, F10/E10, IF(F10&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L10" s="30" t="inlineStr">
+      <c r="L10" s="38" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -3364,7 +3367,7 @@
         <f>IF(E11&gt;0, F11/E11, IF(F11&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L11" s="33" t="inlineStr">
+      <c r="L11" s="35" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -3410,7 +3413,7 @@
         <f>IF(E12&gt;0, F12/E12, IF(F12&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L12" s="30" t="inlineStr">
+      <c r="L12" s="38" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -3456,7 +3459,7 @@
         <f>IF(E13&gt;0, F13/E13, IF(F13&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L13" s="33" t="inlineStr">
+      <c r="L13" s="35" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -3502,7 +3505,7 @@
         <f>IF(E14&gt;0, F14/E14, IF(F14&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L14" s="30" t="inlineStr">
+      <c r="L14" s="38" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -3548,7 +3551,7 @@
         <f>IF(E15&gt;0, F15/E15, IF(F15&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L15" s="33" t="inlineStr">
+      <c r="L15" s="35" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -3594,7 +3597,7 @@
         <f>IF(E16&gt;0, F16/E16, IF(F16&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L16" s="30" t="inlineStr">
+      <c r="L16" s="38" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -3640,7 +3643,7 @@
         <f>IF(E17&gt;0, F17/E17, IF(F17&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L17" s="33" t="inlineStr">
+      <c r="L17" s="35" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -3686,7 +3689,7 @@
         <f>IF(E18&gt;0, F18/E18, IF(F18&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L18" s="30" t="inlineStr">
+      <c r="L18" s="38" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -3732,7 +3735,7 @@
         <f>IF(E19&gt;0, F19/E19, IF(F19&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L19" s="33" t="inlineStr">
+      <c r="L19" s="35" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -3778,7 +3781,7 @@
         <f>IF(E20&gt;0, F20/E20, IF(F20&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L20" s="38" t="inlineStr">
+      <c r="L20" s="30" t="inlineStr">
         <is>
           <t>En Curso</t>
         </is>
@@ -3824,7 +3827,7 @@
         <f>IF(E21&gt;0, F21/E21, IF(F21&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L21" s="33" t="inlineStr">
+      <c r="L21" s="35" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -3870,7 +3873,7 @@
         <f>IF(E22&gt;0, F22/E22, IF(F22&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L22" s="39" t="inlineStr">
+      <c r="L22" s="40" t="inlineStr">
         <is>
           <t>Rezagado</t>
         </is>
@@ -3916,7 +3919,7 @@
         <f>IF(E23&gt;0, F23/E23, IF(F23&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L23" s="33" t="inlineStr">
+      <c r="L23" s="35" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -3962,7 +3965,7 @@
         <f>IF(E24&gt;0, F24/E24, IF(F24&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L24" s="30" t="inlineStr">
+      <c r="L24" s="38" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -3976,25 +3979,25 @@
       </c>
       <c r="C25" s="32" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>AGXK0020</t>
         </is>
       </c>
       <c r="D25" s="31" t="inlineStr">
         <is>
-          <t>descuento marketing</t>
+          <t>AGROXILATO-K, 20 L</t>
         </is>
       </c>
       <c r="E25" s="19" t="n">
-        <v>0</v>
+        <v>3200</v>
       </c>
       <c r="F25" s="19" t="n">
-        <v>1</v>
+        <v>640</v>
       </c>
       <c r="G25" s="19" t="n">
-        <v>0</v>
+        <v>640</v>
       </c>
       <c r="H25" s="19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I25" s="19">
         <f>MAX(0, E25-F25)</f>
@@ -4008,9 +4011,9 @@
         <f>IF(E25&gt;0, F25/E25, IF(F25&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L25" s="37" t="inlineStr">
-        <is>
-          <t>Extra Estimación</t>
+      <c r="L25" s="41" t="inlineStr">
+        <is>
+          <t>Rezagado</t>
         </is>
       </c>
     </row>
@@ -4022,16 +4025,16 @@
       </c>
       <c r="C26" s="29" t="inlineStr">
         <is>
-          <t>AGXK0020</t>
+          <t>AGXK0200</t>
         </is>
       </c>
       <c r="D26" s="28" t="inlineStr">
         <is>
-          <t>AGROXILATO-K, 20 L</t>
+          <t>AGROXILATO-K, 200 L</t>
         </is>
       </c>
       <c r="E26" s="15" t="n">
-        <v>3200</v>
+        <v>400</v>
       </c>
       <c r="F26" s="15" t="n">
         <v>0</v>
@@ -4054,7 +4057,7 @@
         <f>IF(E26&gt;0, F26/E26, IF(F26&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L26" s="30" t="inlineStr">
+      <c r="L26" s="38" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -4068,22 +4071,22 @@
       </c>
       <c r="C27" s="32" t="inlineStr">
         <is>
-          <t>AGXK0200</t>
+          <t>AGZ-M0001</t>
         </is>
       </c>
       <c r="D27" s="31" t="inlineStr">
         <is>
-          <t>AGROXILATO-K, 200 L</t>
+          <t>AGROXILATO-ZN-MN, 1 KG</t>
         </is>
       </c>
       <c r="E27" s="19" t="n">
-        <v>400</v>
+        <v>0</v>
       </c>
       <c r="F27" s="19" t="n">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="G27" s="19" t="n">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="H27" s="19" t="n">
         <v>0</v>
@@ -4100,9 +4103,9 @@
         <f>IF(E27&gt;0, F27/E27, IF(F27&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L27" s="33" t="inlineStr">
-        <is>
-          <t>Sin Pedido</t>
+      <c r="L27" s="39" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -4114,22 +4117,22 @@
       </c>
       <c r="C28" s="29" t="inlineStr">
         <is>
-          <t>AVAN0005</t>
+          <t>AGZ-M0005</t>
         </is>
       </c>
       <c r="D28" s="28" t="inlineStr">
         <is>
-          <t>FLORAMEC AVANCE, 5 L</t>
+          <t>AGROXILATO-ZN-MN, 5 KG</t>
         </is>
       </c>
       <c r="E28" s="15" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="F28" s="15" t="n">
-        <v>600</v>
+        <v>100</v>
       </c>
       <c r="G28" s="15" t="n">
-        <v>600</v>
+        <v>100</v>
       </c>
       <c r="H28" s="15" t="n">
         <v>0</v>
@@ -4146,9 +4149,9 @@
         <f>IF(E28&gt;0, F28/E28, IF(F28&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L28" s="38" t="inlineStr">
-        <is>
-          <t>En Curso</t>
+      <c r="L28" s="34" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -4160,22 +4163,22 @@
       </c>
       <c r="C29" s="32" t="inlineStr">
         <is>
-          <t>C-L0005</t>
+          <t>AVAN0005</t>
         </is>
       </c>
       <c r="D29" s="31" t="inlineStr">
         <is>
-          <t>CODIBOR-L, 5 L</t>
+          <t>FLORAMEC AVANCE, 5 L</t>
         </is>
       </c>
       <c r="E29" s="19" t="n">
-        <v>200</v>
+        <v>1200</v>
       </c>
       <c r="F29" s="19" t="n">
-        <v>200</v>
+        <v>600</v>
       </c>
       <c r="G29" s="19" t="n">
-        <v>200</v>
+        <v>600</v>
       </c>
       <c r="H29" s="19" t="n">
         <v>0</v>
@@ -4192,9 +4195,9 @@
         <f>IF(E29&gt;0, F29/E29, IF(F29&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L29" s="37" t="inlineStr">
-        <is>
-          <t>Superado</t>
+      <c r="L29" s="33" t="inlineStr">
+        <is>
+          <t>En Curso</t>
         </is>
       </c>
     </row>
@@ -4206,16 +4209,16 @@
       </c>
       <c r="C30" s="29" t="inlineStr">
         <is>
-          <t>C-MB0005</t>
+          <t>C-L0005</t>
         </is>
       </c>
       <c r="D30" s="28" t="inlineStr">
         <is>
-          <t>CODIFOL-MB, 5 L</t>
+          <t>CODIBOR-L, 5 L</t>
         </is>
       </c>
       <c r="E30" s="15" t="n">
-        <v>300</v>
+        <v>200</v>
       </c>
       <c r="F30" s="15" t="n">
         <v>200</v>
@@ -4238,9 +4241,9 @@
         <f>IF(E30&gt;0, F30/E30, IF(F30&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L30" s="38" t="inlineStr">
-        <is>
-          <t>En Curso</t>
+      <c r="L30" s="34" t="inlineStr">
+        <is>
+          <t>Superado</t>
         </is>
       </c>
     </row>
@@ -4252,22 +4255,22 @@
       </c>
       <c r="C31" s="32" t="inlineStr">
         <is>
-          <t>CPLUS0020</t>
+          <t>C-MB0005</t>
         </is>
       </c>
       <c r="D31" s="31" t="inlineStr">
         <is>
-          <t>CALCIPLUS, 20 L</t>
+          <t>CODIFOL-MB, 5 L</t>
         </is>
       </c>
       <c r="E31" s="19" t="n">
-        <v>640</v>
+        <v>300</v>
       </c>
       <c r="F31" s="19" t="n">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="G31" s="19" t="n">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="H31" s="19" t="n">
         <v>0</v>
@@ -4286,7 +4289,7 @@
       </c>
       <c r="L31" s="33" t="inlineStr">
         <is>
-          <t>Sin Pedido</t>
+          <t>En Curso</t>
         </is>
       </c>
     </row>
@@ -4298,22 +4301,22 @@
       </c>
       <c r="C32" s="29" t="inlineStr">
         <is>
-          <t>PIV0020</t>
+          <t>CPLUS0020</t>
         </is>
       </c>
       <c r="D32" s="28" t="inlineStr">
         <is>
-          <t>PGR IV, 20 L</t>
+          <t>CALCIPLUS, 20 L</t>
         </is>
       </c>
       <c r="E32" s="15" t="n">
-        <v>1280</v>
+        <v>640</v>
       </c>
       <c r="F32" s="15" t="n">
-        <v>2560</v>
+        <v>0</v>
       </c>
       <c r="G32" s="15" t="n">
-        <v>2560</v>
+        <v>0</v>
       </c>
       <c r="H32" s="15" t="n">
         <v>0</v>
@@ -4330,36 +4333,36 @@
         <f>IF(E32&gt;0, F32/E32, IF(F32&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L32" s="34" t="inlineStr">
-        <is>
-          <t>Superado</t>
+      <c r="L32" s="38" t="inlineStr">
+        <is>
+          <t>Sin Pedido</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="B33" s="31" t="inlineStr">
         <is>
-          <t>GUIVARTO AGRICOLA, S.L.</t>
+          <t>COOP.AGRIC. SAN ISIDRO S.C.A.</t>
         </is>
       </c>
       <c r="C33" s="32" t="inlineStr">
         <is>
-          <t>A-50(2)0005</t>
+          <t>PIV0020</t>
         </is>
       </c>
       <c r="D33" s="31" t="inlineStr">
         <is>
-          <t>CODIORGAN A-50, 5 KG</t>
+          <t>PGR IV, 20 L</t>
         </is>
       </c>
       <c r="E33" s="19" t="n">
-        <v>100</v>
+        <v>1280</v>
       </c>
       <c r="F33" s="19" t="n">
-        <v>0</v>
+        <v>2560</v>
       </c>
       <c r="G33" s="19" t="n">
-        <v>0</v>
+        <v>2560</v>
       </c>
       <c r="H33" s="19" t="n">
         <v>0</v>
@@ -4376,36 +4379,36 @@
         <f>IF(E33&gt;0, F33/E33, IF(F33&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L33" s="33" t="inlineStr">
-        <is>
-          <t>Sin Pedido</t>
+      <c r="L33" s="39" t="inlineStr">
+        <is>
+          <t>Superado</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="B34" s="28" t="inlineStr">
         <is>
-          <t>GUIVARTO AGRICOLA, S.L.</t>
+          <t>COOP.AGRIC. SAN ISIDRO S.C.A.</t>
         </is>
       </c>
       <c r="C34" s="29" t="inlineStr">
         <is>
-          <t>AGXK0020</t>
+          <t>PT0020</t>
         </is>
       </c>
       <c r="D34" s="28" t="inlineStr">
         <is>
-          <t>AGROXILATO-K, 20 L</t>
+          <t>AGROPOTASION, 20 L</t>
         </is>
       </c>
       <c r="E34" s="15" t="n">
-        <v>1240</v>
+        <v>0</v>
       </c>
       <c r="F34" s="15" t="n">
-        <v>0</v>
+        <v>320</v>
       </c>
       <c r="G34" s="15" t="n">
-        <v>0</v>
+        <v>320</v>
       </c>
       <c r="H34" s="15" t="n">
         <v>0</v>
@@ -4422,36 +4425,36 @@
         <f>IF(E34&gt;0, F34/E34, IF(F34&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L34" s="30" t="inlineStr">
-        <is>
-          <t>Sin Pedido</t>
+      <c r="L34" s="34" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="B35" s="31" t="inlineStr">
         <is>
-          <t>GUIVARTO AGRICOLA, S.L.</t>
+          <t>COOP.AGRIC. SAN ISIDRO S.C.A.</t>
         </is>
       </c>
       <c r="C35" s="32" t="inlineStr">
         <is>
-          <t>AGZNP0005</t>
+          <t>S0020</t>
         </is>
       </c>
       <c r="D35" s="31" t="inlineStr">
         <is>
-          <t>AGROXILATO-ZN PLUS, 5 KG</t>
+          <t>SAL-WAX STAR, 20 L</t>
         </is>
       </c>
       <c r="E35" s="19" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="F35" s="19" t="n">
-        <v>0</v>
+        <v>640</v>
       </c>
       <c r="G35" s="19" t="n">
-        <v>0</v>
+        <v>640</v>
       </c>
       <c r="H35" s="19" t="n">
         <v>0</v>
@@ -4468,9 +4471,9 @@
         <f>IF(E35&gt;0, F35/E35, IF(F35&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L35" s="33" t="inlineStr">
-        <is>
-          <t>Sin Pedido</t>
+      <c r="L35" s="39" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -4482,16 +4485,16 @@
       </c>
       <c r="C36" s="29" t="inlineStr">
         <is>
-          <t>AQUOM0005</t>
+          <t>A-50(2)0005</t>
         </is>
       </c>
       <c r="D36" s="28" t="inlineStr">
         <is>
-          <t>AQUOM, 5 L</t>
+          <t>CODIORGAN A-50, 5 KG</t>
         </is>
       </c>
       <c r="E36" s="15" t="n">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="F36" s="15" t="n">
         <v>0</v>
@@ -4514,7 +4517,7 @@
         <f>IF(E36&gt;0, F36/E36, IF(F36&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L36" s="30" t="inlineStr">
+      <c r="L36" s="38" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -4528,16 +4531,16 @@
       </c>
       <c r="C37" s="32" t="inlineStr">
         <is>
-          <t>AVAN0020</t>
+          <t>AGXK0020</t>
         </is>
       </c>
       <c r="D37" s="31" t="inlineStr">
         <is>
-          <t>FLORAMEC AVANCE, 20 L</t>
+          <t>AGROXILATO-K, 20 L</t>
         </is>
       </c>
       <c r="E37" s="19" t="n">
-        <v>640</v>
+        <v>1240</v>
       </c>
       <c r="F37" s="19" t="n">
         <v>0</v>
@@ -4560,7 +4563,7 @@
         <f>IF(E37&gt;0, F37/E37, IF(F37&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L37" s="33" t="inlineStr">
+      <c r="L37" s="35" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -4574,16 +4577,16 @@
       </c>
       <c r="C38" s="29" t="inlineStr">
         <is>
-          <t>BEY0020</t>
+          <t>AGZNP0005</t>
         </is>
       </c>
       <c r="D38" s="28" t="inlineStr">
         <is>
-          <t>FLORAMEC PLUS 20 L</t>
+          <t>AGROXILATO-ZN PLUS, 5 KG</t>
         </is>
       </c>
       <c r="E38" s="15" t="n">
-        <v>80</v>
+        <v>50</v>
       </c>
       <c r="F38" s="15" t="n">
         <v>0</v>
@@ -4606,7 +4609,7 @@
         <f>IF(E38&gt;0, F38/E38, IF(F38&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L38" s="30" t="inlineStr">
+      <c r="L38" s="38" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -4620,16 +4623,16 @@
       </c>
       <c r="C39" s="32" t="inlineStr">
         <is>
-          <t>BROTA0005</t>
+          <t>AQUOM0005</t>
         </is>
       </c>
       <c r="D39" s="31" t="inlineStr">
         <is>
-          <t>BROTAMEC, 5 L</t>
+          <t>AQUOM, 5 L</t>
         </is>
       </c>
       <c r="E39" s="19" t="n">
-        <v>600</v>
+        <v>200</v>
       </c>
       <c r="F39" s="19" t="n">
         <v>0</v>
@@ -4652,7 +4655,7 @@
         <f>IF(E39&gt;0, F39/E39, IF(F39&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L39" s="33" t="inlineStr">
+      <c r="L39" s="35" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -4666,16 +4669,16 @@
       </c>
       <c r="C40" s="29" t="inlineStr">
         <is>
-          <t>C-M-P0001</t>
+          <t>AVAN0020</t>
         </is>
       </c>
       <c r="D40" s="28" t="inlineStr">
         <is>
-          <t>CODIFOL Mo-PLUS, 1 L</t>
+          <t>FLORAMEC AVANCE, 20 L</t>
         </is>
       </c>
       <c r="E40" s="15" t="n">
-        <v>36</v>
+        <v>640</v>
       </c>
       <c r="F40" s="15" t="n">
         <v>0</v>
@@ -4698,7 +4701,7 @@
         <f>IF(E40&gt;0, F40/E40, IF(F40&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L40" s="30" t="inlineStr">
+      <c r="L40" s="38" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -4712,16 +4715,16 @@
       </c>
       <c r="C41" s="32" t="inlineStr">
         <is>
-          <t>FTK0005</t>
+          <t>BEY0020</t>
         </is>
       </c>
       <c r="D41" s="31" t="inlineStr">
         <is>
-          <t>FITOKONTROL CA FLOW, 5 KG</t>
+          <t>FLORAMEC PLUS 20 L</t>
         </is>
       </c>
       <c r="E41" s="19" t="n">
-        <v>800</v>
+        <v>80</v>
       </c>
       <c r="F41" s="19" t="n">
         <v>0</v>
@@ -4744,54 +4747,192 @@
         <f>IF(E41&gt;0, F41/E41, IF(F41&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L41" s="33" t="inlineStr">
+      <c r="L41" s="35" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
       </c>
     </row>
-    <row r="42" ht="24" customHeight="1">
-      <c r="B42" s="21" t="inlineStr">
+    <row r="42">
+      <c r="B42" s="28" t="inlineStr">
+        <is>
+          <t>GUIVARTO AGRICOLA, S.L.</t>
+        </is>
+      </c>
+      <c r="C42" s="29" t="inlineStr">
+        <is>
+          <t>BROTA0005</t>
+        </is>
+      </c>
+      <c r="D42" s="28" t="inlineStr">
+        <is>
+          <t>BROTAMEC, 5 L</t>
+        </is>
+      </c>
+      <c r="E42" s="15" t="n">
+        <v>600</v>
+      </c>
+      <c r="F42" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G42" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H42" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I42" s="15">
+        <f>MAX(0, E42-F42)</f>
+        <v/>
+      </c>
+      <c r="J42" s="15">
+        <f>ABS(F42-E42)</f>
+        <v/>
+      </c>
+      <c r="K42" s="16">
+        <f>IF(E42&gt;0, F42/E42, IF(F42&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L42" s="38" t="inlineStr">
+        <is>
+          <t>Sin Pedido</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" s="31" t="inlineStr">
+        <is>
+          <t>GUIVARTO AGRICOLA, S.L.</t>
+        </is>
+      </c>
+      <c r="C43" s="32" t="inlineStr">
+        <is>
+          <t>C-M-P0001</t>
+        </is>
+      </c>
+      <c r="D43" s="31" t="inlineStr">
+        <is>
+          <t>CODIFOL Mo-PLUS, 1 L</t>
+        </is>
+      </c>
+      <c r="E43" s="19" t="n">
+        <v>36</v>
+      </c>
+      <c r="F43" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G43" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H43" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I43" s="19">
+        <f>MAX(0, E43-F43)</f>
+        <v/>
+      </c>
+      <c r="J43" s="19">
+        <f>ABS(F43-E43)</f>
+        <v/>
+      </c>
+      <c r="K43" s="20">
+        <f>IF(E43&gt;0, F43/E43, IF(F43&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L43" s="35" t="inlineStr">
+        <is>
+          <t>Sin Pedido</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" s="28" t="inlineStr">
+        <is>
+          <t>GUIVARTO AGRICOLA, S.L.</t>
+        </is>
+      </c>
+      <c r="C44" s="29" t="inlineStr">
+        <is>
+          <t>FTK0005</t>
+        </is>
+      </c>
+      <c r="D44" s="28" t="inlineStr">
+        <is>
+          <t>FITOKONTROL CA FLOW, 5 KG</t>
+        </is>
+      </c>
+      <c r="E44" s="15" t="n">
+        <v>800</v>
+      </c>
+      <c r="F44" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G44" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H44" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I44" s="15">
+        <f>MAX(0, E44-F44)</f>
+        <v/>
+      </c>
+      <c r="J44" s="15">
+        <f>ABS(F44-E44)</f>
+        <v/>
+      </c>
+      <c r="K44" s="16">
+        <f>IF(E44&gt;0, F44/E44, IF(F44&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L44" s="38" t="inlineStr">
+        <is>
+          <t>Sin Pedido</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="24" customHeight="1">
+      <c r="B45" s="21" t="inlineStr">
         <is>
           <t>TOTAL IRENE</t>
         </is>
       </c>
-      <c r="C42" s="35" t="inlineStr">
-        <is>
-          <t>90 líneas</t>
-        </is>
-      </c>
-      <c r="D42" s="36" t="inlineStr"/>
-      <c r="E42" s="23">
-        <f>SUM(E10:E41)</f>
-        <v/>
-      </c>
-      <c r="F42" s="23">
-        <f>SUM(F10:F41)</f>
-        <v/>
-      </c>
-      <c r="G42" s="23">
-        <f>SUM(G10:G41)</f>
-        <v/>
-      </c>
-      <c r="H42" s="23">
-        <f>SUM(H10:H41)</f>
-        <v/>
-      </c>
-      <c r="I42" s="23">
-        <f>SUM(I10:I41)</f>
-        <v/>
-      </c>
-      <c r="J42" s="23">
-        <f>SUM(J10:J41)</f>
-        <v/>
-      </c>
-      <c r="K42" s="24">
-        <f>IF(E42&gt;0, F42/E42, 0)</f>
-        <v/>
-      </c>
-      <c r="L42" s="22">
-        <f>IF(K42&gt;=1, "SUPERADO", "EN CURSO")</f>
+      <c r="C45" s="36" t="inlineStr">
+        <is>
+          <t>89 líneas</t>
+        </is>
+      </c>
+      <c r="D45" s="37" t="inlineStr"/>
+      <c r="E45" s="23">
+        <f>SUM(E10:E44)</f>
+        <v/>
+      </c>
+      <c r="F45" s="23">
+        <f>SUM(F10:F44)</f>
+        <v/>
+      </c>
+      <c r="G45" s="23">
+        <f>SUM(G10:G44)</f>
+        <v/>
+      </c>
+      <c r="H45" s="23">
+        <f>SUM(H10:H44)</f>
+        <v/>
+      </c>
+      <c r="I45" s="23">
+        <f>SUM(I10:I44)</f>
+        <v/>
+      </c>
+      <c r="J45" s="23">
+        <f>SUM(J10:J44)</f>
+        <v/>
+      </c>
+      <c r="K45" s="24">
+        <f>IF(E45&gt;0, F45/E45, 0)</f>
+        <v/>
+      </c>
+      <c r="L45" s="22">
+        <f>IF(K45&gt;=1, "SUPERADO", "EN CURSO")</f>
         <v/>
       </c>
     </row>
@@ -4820,7 +4961,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:L20"/>
+  <dimension ref="B2:L22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -4847,7 +4988,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 07/10/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 08/10/2026</t>
         </is>
       </c>
     </row>
@@ -4892,25 +5033,25 @@
       <c r="C6" s="4" t="n"/>
       <c r="D6" s="25" t="inlineStr">
         <is>
-          <t>820 u</t>
+          <t>2,460 u</t>
         </is>
       </c>
       <c r="E6" s="4" t="n"/>
       <c r="F6" s="26" t="inlineStr">
         <is>
-          <t>4.8%</t>
+          <t>14.4%</t>
         </is>
       </c>
       <c r="G6" s="4" t="n"/>
       <c r="H6" s="26" t="inlineStr">
         <is>
-          <t>16,280 u</t>
+          <t>14,640 u</t>
         </is>
       </c>
       <c r="I6" s="4" t="n"/>
       <c r="J6" s="25" t="inlineStr">
         <is>
-          <t>0 u</t>
+          <t>1,000 u</t>
         </is>
       </c>
       <c r="K6" s="4" t="n"/>
@@ -5019,7 +5160,7 @@
         <f>IF(E10&gt;0, F10/E10, IF(F10&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L10" s="30" t="inlineStr">
+      <c r="L10" s="38" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -5065,7 +5206,7 @@
         <f>IF(E11&gt;0, F11/E11, IF(F11&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L11" s="33" t="inlineStr">
+      <c r="L11" s="35" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -5111,7 +5252,7 @@
         <f>IF(E12&gt;0, F12/E12, IF(F12&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L12" s="30" t="inlineStr">
+      <c r="L12" s="38" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -5157,7 +5298,7 @@
         <f>IF(E13&gt;0, F13/E13, IF(F13&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L13" s="37" t="inlineStr">
+      <c r="L13" s="39" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -5203,7 +5344,7 @@
         <f>IF(E14&gt;0, F14/E14, IF(F14&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L14" s="30" t="inlineStr">
+      <c r="L14" s="38" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -5249,7 +5390,7 @@
         <f>IF(E15&gt;0, F15/E15, IF(F15&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L15" s="33" t="inlineStr">
+      <c r="L15" s="35" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -5263,25 +5404,25 @@
       </c>
       <c r="C16" s="29" t="inlineStr">
         <is>
-          <t>PT0005</t>
+          <t>JF1000</t>
         </is>
       </c>
       <c r="D16" s="28" t="inlineStr">
         <is>
-          <t>AGROPOTASION, 5 L</t>
+          <t>CODIGIN-FOS, 1000 L</t>
         </is>
       </c>
       <c r="E16" s="15" t="n">
         <v>0</v>
       </c>
       <c r="F16" s="15" t="n">
-        <v>200</v>
+        <v>1000</v>
       </c>
       <c r="G16" s="15" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="H16" s="15" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="I16" s="15">
         <f>MAX(0, E16-F16)</f>
@@ -5309,22 +5450,22 @@
       </c>
       <c r="C17" s="32" t="inlineStr">
         <is>
-          <t>PT0020</t>
+          <t>PT0005</t>
         </is>
       </c>
       <c r="D17" s="31" t="inlineStr">
         <is>
-          <t>AGROPOTASION, 20 L</t>
+          <t>AGROPOTASION, 5 L</t>
         </is>
       </c>
       <c r="E17" s="19" t="n">
         <v>0</v>
       </c>
       <c r="F17" s="19" t="n">
-        <v>320</v>
+        <v>200</v>
       </c>
       <c r="G17" s="19" t="n">
-        <v>320</v>
+        <v>200</v>
       </c>
       <c r="H17" s="19" t="n">
         <v>0</v>
@@ -5341,7 +5482,7 @@
         <f>IF(E17&gt;0, F17/E17, IF(F17&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L17" s="37" t="inlineStr">
+      <c r="L17" s="39" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -5350,27 +5491,27 @@
     <row r="18">
       <c r="B18" s="28" t="inlineStr">
         <is>
-          <t>FITOXENT S.C.L.V.</t>
+          <t>CODIMED EXPORT, S.L.</t>
         </is>
       </c>
       <c r="C18" s="29" t="inlineStr">
         <is>
-          <t>FTK0005</t>
+          <t>PT0020</t>
         </is>
       </c>
       <c r="D18" s="28" t="inlineStr">
         <is>
-          <t>FITOKONTROL CA FLOW, 5 KG</t>
+          <t>AGROPOTASION, 20 L</t>
         </is>
       </c>
       <c r="E18" s="15" t="n">
-        <v>4400</v>
+        <v>0</v>
       </c>
       <c r="F18" s="15" t="n">
-        <v>0</v>
+        <v>320</v>
       </c>
       <c r="G18" s="15" t="n">
-        <v>0</v>
+        <v>320</v>
       </c>
       <c r="H18" s="15" t="n">
         <v>0</v>
@@ -5387,16 +5528,16 @@
         <f>IF(E18&gt;0, F18/E18, IF(F18&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L18" s="30" t="inlineStr">
-        <is>
-          <t>Sin Pedido</t>
+      <c r="L18" s="34" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="31" t="inlineStr">
         <is>
-          <t>FITOXENT S.C.L.V.</t>
+          <t>FITOSANITARIOS CARCAIXENT, S.L.</t>
         </is>
       </c>
       <c r="C19" s="32" t="inlineStr">
@@ -5410,13 +5551,13 @@
         </is>
       </c>
       <c r="E19" s="19" t="n">
-        <v>2560</v>
+        <v>0</v>
       </c>
       <c r="F19" s="19" t="n">
-        <v>0</v>
+        <v>640</v>
       </c>
       <c r="G19" s="19" t="n">
-        <v>0</v>
+        <v>640</v>
       </c>
       <c r="H19" s="19" t="n">
         <v>0</v>
@@ -5433,54 +5574,146 @@
         <f>IF(E19&gt;0, F19/E19, IF(F19&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L19" s="33" t="inlineStr">
+      <c r="L19" s="39" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="28" t="inlineStr">
+        <is>
+          <t>FITOXENT S.C.L.V.</t>
+        </is>
+      </c>
+      <c r="C20" s="29" t="inlineStr">
+        <is>
+          <t>FTK0005</t>
+        </is>
+      </c>
+      <c r="D20" s="28" t="inlineStr">
+        <is>
+          <t>FITOKONTROL CA FLOW, 5 KG</t>
+        </is>
+      </c>
+      <c r="E20" s="15" t="n">
+        <v>4400</v>
+      </c>
+      <c r="F20" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I20" s="15">
+        <f>MAX(0, E20-F20)</f>
+        <v/>
+      </c>
+      <c r="J20" s="15">
+        <f>ABS(F20-E20)</f>
+        <v/>
+      </c>
+      <c r="K20" s="16">
+        <f>IF(E20&gt;0, F20/E20, IF(F20&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L20" s="38" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="24" customHeight="1">
-      <c r="B20" s="21" t="inlineStr">
+    <row r="21">
+      <c r="B21" s="31" t="inlineStr">
+        <is>
+          <t>FITOXENT S.C.L.V.</t>
+        </is>
+      </c>
+      <c r="C21" s="32" t="inlineStr">
+        <is>
+          <t>PT0020</t>
+        </is>
+      </c>
+      <c r="D21" s="31" t="inlineStr">
+        <is>
+          <t>AGROPOTASION, 20 L</t>
+        </is>
+      </c>
+      <c r="E21" s="19" t="n">
+        <v>2560</v>
+      </c>
+      <c r="F21" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I21" s="19">
+        <f>MAX(0, E21-F21)</f>
+        <v/>
+      </c>
+      <c r="J21" s="19">
+        <f>ABS(F21-E21)</f>
+        <v/>
+      </c>
+      <c r="K21" s="20">
+        <f>IF(E21&gt;0, F21/E21, IF(F21&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L21" s="35" t="inlineStr">
+        <is>
+          <t>Sin Pedido</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="24" customHeight="1">
+      <c r="B22" s="21" t="inlineStr">
         <is>
           <t>TOTAL JAVIER</t>
         </is>
       </c>
-      <c r="C20" s="35" t="inlineStr">
-        <is>
-          <t>174 líneas</t>
-        </is>
-      </c>
-      <c r="D20" s="36" t="inlineStr"/>
-      <c r="E20" s="23">
-        <f>SUM(E10:E19)</f>
-        <v/>
-      </c>
-      <c r="F20" s="23">
-        <f>SUM(F10:F19)</f>
-        <v/>
-      </c>
-      <c r="G20" s="23">
-        <f>SUM(G10:G19)</f>
-        <v/>
-      </c>
-      <c r="H20" s="23">
-        <f>SUM(H10:H19)</f>
-        <v/>
-      </c>
-      <c r="I20" s="23">
-        <f>SUM(I10:I19)</f>
-        <v/>
-      </c>
-      <c r="J20" s="23">
-        <f>SUM(J10:J19)</f>
-        <v/>
-      </c>
-      <c r="K20" s="24">
-        <f>IF(E20&gt;0, F20/E20, 0)</f>
-        <v/>
-      </c>
-      <c r="L20" s="22">
-        <f>IF(K20&gt;=1, "SUPERADO", "EN CURSO")</f>
+      <c r="C22" s="36" t="inlineStr">
+        <is>
+          <t>175 líneas</t>
+        </is>
+      </c>
+      <c r="D22" s="37" t="inlineStr"/>
+      <c r="E22" s="23">
+        <f>SUM(E10:E21)</f>
+        <v/>
+      </c>
+      <c r="F22" s="23">
+        <f>SUM(F10:F21)</f>
+        <v/>
+      </c>
+      <c r="G22" s="23">
+        <f>SUM(G10:G21)</f>
+        <v/>
+      </c>
+      <c r="H22" s="23">
+        <f>SUM(H10:H21)</f>
+        <v/>
+      </c>
+      <c r="I22" s="23">
+        <f>SUM(I10:I21)</f>
+        <v/>
+      </c>
+      <c r="J22" s="23">
+        <f>SUM(J10:J21)</f>
+        <v/>
+      </c>
+      <c r="K22" s="24">
+        <f>IF(E22&gt;0, F22/E22, 0)</f>
+        <v/>
+      </c>
+      <c r="L22" s="22">
+        <f>IF(K22&gt;=1, "SUPERADO", "EN CURSO")</f>
         <v/>
       </c>
     </row>
@@ -5536,7 +5769,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 07/10/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 08/10/2026</t>
         </is>
       </c>
     </row>
@@ -5708,7 +5941,7 @@
         <f>IF(E10&gt;0, F10/E10, IF(F10&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L10" s="30" t="inlineStr">
+      <c r="L10" s="38" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -5754,7 +5987,7 @@
         <f>IF(E11&gt;0, F11/E11, IF(F11&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L11" s="33" t="inlineStr">
+      <c r="L11" s="35" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -5800,7 +6033,7 @@
         <f>IF(E12&gt;0, F12/E12, IF(F12&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L12" s="30" t="inlineStr">
+      <c r="L12" s="38" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -5846,7 +6079,7 @@
         <f>IF(E13&gt;0, F13/E13, IF(F13&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L13" s="33" t="inlineStr">
+      <c r="L13" s="35" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -5892,7 +6125,7 @@
         <f>IF(E14&gt;0, F14/E14, IF(F14&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L14" s="30" t="inlineStr">
+      <c r="L14" s="38" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -5938,7 +6171,7 @@
         <f>IF(E15&gt;0, F15/E15, IF(F15&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L15" s="33" t="inlineStr">
+      <c r="L15" s="35" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -5950,12 +6183,12 @@
           <t>TOTAL MEHMET</t>
         </is>
       </c>
-      <c r="C16" s="35" t="inlineStr">
+      <c r="C16" s="36" t="inlineStr">
         <is>
           <t>61 líneas</t>
         </is>
       </c>
-      <c r="D16" s="36" t="inlineStr"/>
+      <c r="D16" s="37" t="inlineStr"/>
       <c r="E16" s="23">
         <f>SUM(E10:E15)</f>
         <v/>
@@ -6041,7 +6274,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 07/10/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 08/10/2026</t>
         </is>
       </c>
     </row>
@@ -6259,7 +6492,7 @@
         <f>IF(E11&gt;0, F11/E11, IF(F11&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L11" s="33" t="inlineStr">
+      <c r="L11" s="35" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -6305,7 +6538,7 @@
         <f>IF(E12&gt;0, F12/E12, IF(F12&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L12" s="30" t="inlineStr">
+      <c r="L12" s="38" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -6351,7 +6584,7 @@
         <f>IF(E13&gt;0, F13/E13, IF(F13&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L13" s="33" t="inlineStr">
+      <c r="L13" s="35" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -6443,7 +6676,7 @@
         <f>IF(E15&gt;0, F15/E15, IF(F15&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L15" s="33" t="inlineStr">
+      <c r="L15" s="35" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -6489,7 +6722,7 @@
         <f>IF(E16&gt;0, F16/E16, IF(F16&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L16" s="30" t="inlineStr">
+      <c r="L16" s="38" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -6535,7 +6768,7 @@
         <f>IF(E17&gt;0, F17/E17, IF(F17&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L17" s="33" t="inlineStr">
+      <c r="L17" s="35" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -6581,7 +6814,7 @@
         <f>IF(E18&gt;0, F18/E18, IF(F18&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L18" s="30" t="inlineStr">
+      <c r="L18" s="38" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -6627,7 +6860,7 @@
         <f>IF(E19&gt;0, F19/E19, IF(F19&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L19" s="37" t="inlineStr">
+      <c r="L19" s="39" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -6719,7 +6952,7 @@
         <f>IF(E21&gt;0, F21/E21, IF(F21&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L21" s="37" t="inlineStr">
+      <c r="L21" s="39" t="inlineStr">
         <is>
           <t>Superado</t>
         </is>
@@ -6765,7 +6998,7 @@
         <f>IF(E22&gt;0, F22/E22, IF(F22&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L22" s="30" t="inlineStr">
+      <c r="L22" s="38" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -6811,7 +7044,7 @@
         <f>IF(E23&gt;0, F23/E23, IF(F23&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L23" s="40" t="inlineStr">
+      <c r="L23" s="33" t="inlineStr">
         <is>
           <t>En Curso</t>
         </is>
@@ -6869,12 +7102,12 @@
           <t>TOTAL PEDRO</t>
         </is>
       </c>
-      <c r="C25" s="35" t="inlineStr">
+      <c r="C25" s="36" t="inlineStr">
         <is>
           <t>104 líneas</t>
         </is>
       </c>
-      <c r="D25" s="36" t="inlineStr"/>
+      <c r="D25" s="37" t="inlineStr"/>
       <c r="E25" s="23">
         <f>SUM(E10:E24)</f>
         <v/>
@@ -6960,7 +7193,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 07/10/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 08/10/2026</t>
         </is>
       </c>
     </row>
@@ -7132,7 +7365,7 @@
         <f>IF(E10&gt;0, F10/E10, IF(F10&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L10" s="30" t="inlineStr">
+      <c r="L10" s="38" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -7178,7 +7411,7 @@
         <f>IF(E11&gt;0, F11/E11, IF(F11&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L11" s="33" t="inlineStr">
+      <c r="L11" s="35" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -7190,12 +7423,12 @@
           <t>TOTAL RICARDO</t>
         </is>
       </c>
-      <c r="C12" s="35" t="inlineStr">
+      <c r="C12" s="36" t="inlineStr">
         <is>
           <t>115 líneas</t>
         </is>
       </c>
-      <c r="D12" s="36" t="inlineStr"/>
+      <c r="D12" s="37" t="inlineStr"/>
       <c r="E12" s="23">
         <f>SUM(E10:E11)</f>
         <v/>

</xml_diff>

<commit_message>
Actualizacion pedidos al 15/10/2026 y correccion sintaxis MRP
</commit_message>
<xml_diff>
--- a/Seguimiento_Presupuesto_Sep_2026.xlsx
+++ b/Seguimiento_Presupuesto_Sep_2026.xlsx
@@ -102,7 +102,7 @@
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="00B45309"/>
+      <color rgb="00047857"/>
       <sz val="13"/>
     </font>
     <font>
@@ -131,7 +131,7 @@
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="00047857"/>
+      <color rgb="00B45309"/>
       <sz val="13"/>
     </font>
     <font>
@@ -316,7 +316,7 @@
     <xf numFmtId="0" fontId="11" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -341,20 +341,20 @@
     <xf numFmtId="0" fontId="15" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="8" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -918,7 +918,7 @@
     <row r="3" ht="20" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Comparativa Estimación Septiembre (Unidades) vs Pedidos Reales a Fecha 14/10/2026 | Generado: 14/10/2026 07:07</t>
+          <t>Comparativa Estimación Septiembre (Unidades) vs Pedidos Reales a Fecha 15/10/2026 | Generado: 15/10/2026 07:28</t>
         </is>
       </c>
     </row>
@@ -962,25 +962,25 @@
       <c r="C6" s="4" t="n"/>
       <c r="D6" s="8" t="inlineStr">
         <is>
-          <t>68,740 u</t>
+          <t>110,460 u</t>
         </is>
       </c>
       <c r="E6" s="4" t="n"/>
       <c r="F6" s="9" t="inlineStr">
         <is>
-          <t>37.8%</t>
+          <t>60.7%</t>
         </is>
       </c>
       <c r="G6" s="4" t="n"/>
       <c r="H6" s="10" t="inlineStr">
         <is>
-          <t>119,234 u</t>
+          <t>114,354 u</t>
         </is>
       </c>
       <c r="I6" s="4" t="n"/>
       <c r="J6" s="7" t="inlineStr">
         <is>
-          <t>46,100 u</t>
+          <t>81,300 u</t>
         </is>
       </c>
     </row>
@@ -1045,16 +1045,16 @@
         </is>
       </c>
       <c r="C10" s="14" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D10" s="15" t="n">
         <v>2320</v>
       </c>
       <c r="E10" s="15" t="n">
-        <v>1680</v>
+        <v>2320</v>
       </c>
       <c r="F10" s="15" t="n">
-        <v>1680</v>
+        <v>2320</v>
       </c>
       <c r="G10" s="15" t="n">
         <v>0</v>
@@ -1064,7 +1064,7 @@
         <v/>
       </c>
       <c r="I10" s="15">
-        <f>'Alfonso'!J14</f>
+        <f>'Alfonso'!J15</f>
         <v/>
       </c>
       <c r="J10" s="16">
@@ -1079,26 +1079,26 @@
         </is>
       </c>
       <c r="C11" s="18" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D11" s="19" t="n">
         <v>37832</v>
       </c>
       <c r="E11" s="19" t="n">
-        <v>43840</v>
+        <v>80676</v>
       </c>
       <c r="F11" s="19" t="n">
-        <v>3040</v>
+        <v>6680</v>
       </c>
       <c r="G11" s="19" t="n">
-        <v>40800</v>
+        <v>73996</v>
       </c>
       <c r="H11" s="19">
         <f>MAX(0, D11-E11)</f>
         <v/>
       </c>
       <c r="I11" s="19">
-        <f>'García'!J37</f>
+        <f>'García'!J48</f>
         <v/>
       </c>
       <c r="J11" s="20">
@@ -1113,16 +1113,16 @@
         </is>
       </c>
       <c r="C12" s="14" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D12" s="15" t="n">
         <v>21914</v>
       </c>
       <c r="E12" s="15" t="n">
-        <v>9580</v>
+        <v>11820</v>
       </c>
       <c r="F12" s="15" t="n">
-        <v>9580</v>
+        <v>11820</v>
       </c>
       <c r="G12" s="15" t="n">
         <v>0</v>
@@ -1132,7 +1132,7 @@
         <v/>
       </c>
       <c r="I12" s="15">
-        <f>'Irene'!J46</f>
+        <f>'Irene'!J48</f>
         <v/>
       </c>
       <c r="J12" s="16">
@@ -1147,26 +1147,26 @@
         </is>
       </c>
       <c r="C13" s="18" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D13" s="19" t="n">
         <v>17100</v>
       </c>
       <c r="E13" s="19" t="n">
-        <v>6760</v>
+        <v>7760</v>
       </c>
       <c r="F13" s="19" t="n">
         <v>1460</v>
       </c>
       <c r="G13" s="19" t="n">
-        <v>5300</v>
+        <v>6300</v>
       </c>
       <c r="H13" s="19">
         <f>MAX(0, D13-E13)</f>
         <v/>
       </c>
       <c r="I13" s="19">
-        <f>'Javier'!J26</f>
+        <f>'Javier'!J27</f>
         <v/>
       </c>
       <c r="J13" s="20">
@@ -1215,26 +1215,26 @@
         </is>
       </c>
       <c r="C15" s="18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D15" s="19" t="n">
         <v>17340</v>
       </c>
       <c r="E15" s="19" t="n">
-        <v>6880</v>
+        <v>7880</v>
       </c>
       <c r="F15" s="19" t="n">
         <v>6880</v>
       </c>
       <c r="G15" s="19" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="H15" s="19">
         <f>MAX(0, D15-E15)</f>
         <v/>
       </c>
       <c r="I15" s="19">
-        <f>'Pedro'!J25</f>
+        <f>'Pedro'!J26</f>
         <v/>
       </c>
       <c r="J15" s="20">
@@ -1339,7 +1339,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:L14"/>
+  <dimension ref="B2:L15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1366,7 +1366,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 14/10/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 15/10/2026</t>
         </is>
       </c>
     </row>
@@ -1377,19 +1377,19 @@
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D5" s="5" t="inlineStr">
         <is>
           <t>PEDIDOS REALES (U)</t>
         </is>
       </c>
       <c r="E5" s="4" t="n"/>
-      <c r="F5" s="6" t="inlineStr">
+      <c r="F5" s="5" t="inlineStr">
         <is>
           <t>% CONSECUCIÓN</t>
         </is>
       </c>
       <c r="G5" s="4" t="n"/>
-      <c r="H5" s="6" t="inlineStr">
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>FALTA CONSEGUIR (GAP)</t>
         </is>
@@ -1409,21 +1409,21 @@
         </is>
       </c>
       <c r="C6" s="4" t="n"/>
-      <c r="D6" s="25" t="inlineStr">
-        <is>
-          <t>1,680 u</t>
+      <c r="D6" s="26" t="inlineStr">
+        <is>
+          <t>2,320 u</t>
         </is>
       </c>
       <c r="E6" s="4" t="n"/>
       <c r="F6" s="26" t="inlineStr">
         <is>
-          <t>72.4%</t>
+          <t>100.0%</t>
         </is>
       </c>
       <c r="G6" s="4" t="n"/>
       <c r="H6" s="26" t="inlineStr">
         <is>
-          <t>640 u</t>
+          <t>0 u</t>
         </is>
       </c>
       <c r="I6" s="4" t="n"/>
@@ -1593,27 +1593,27 @@
     <row r="12">
       <c r="B12" s="28" t="inlineStr">
         <is>
-          <t>AGROTÉCNICA DEL NORTE, S.L</t>
+          <t>AGROCAMP CANET S.L.</t>
         </is>
       </c>
       <c r="C12" s="29" t="inlineStr">
         <is>
-          <t>PT0005</t>
+          <t>AGXK0020</t>
         </is>
       </c>
       <c r="D12" s="28" t="inlineStr">
         <is>
-          <t>AGROPOTASION, 5 L</t>
+          <t>AGROXILATO-K, 20 L</t>
         </is>
       </c>
       <c r="E12" s="15" t="n">
         <v>0</v>
       </c>
       <c r="F12" s="15" t="n">
-        <v>400</v>
+        <v>640</v>
       </c>
       <c r="G12" s="15" t="n">
-        <v>400</v>
+        <v>640</v>
       </c>
       <c r="H12" s="15" t="n">
         <v>0</v>
@@ -1639,27 +1639,27 @@
     <row r="13">
       <c r="B13" s="31" t="inlineStr">
         <is>
-          <t>AGROVEYCA,S.L</t>
+          <t>AGROTÉCNICA DEL NORTE, S.L</t>
         </is>
       </c>
       <c r="C13" s="32" t="inlineStr">
         <is>
-          <t>BIO0020</t>
+          <t>PT0005</t>
         </is>
       </c>
       <c r="D13" s="31" t="inlineStr">
         <is>
-          <t>BIORAD-20, 20 L</t>
+          <t>AGROPOTASION, 5 L</t>
         </is>
       </c>
       <c r="E13" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="19" t="n">
         <v>400</v>
       </c>
-      <c r="F13" s="19" t="n">
-        <v>0</v>
-      </c>
       <c r="G13" s="19" t="n">
-        <v>0</v>
+        <v>400</v>
       </c>
       <c r="H13" s="19" t="n">
         <v>0</v>
@@ -1678,52 +1678,98 @@
       </c>
       <c r="L13" s="35" t="inlineStr">
         <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="28" t="inlineStr">
+        <is>
+          <t>AGROVEYCA,S.L</t>
+        </is>
+      </c>
+      <c r="C14" s="29" t="inlineStr">
+        <is>
+          <t>BIO0020</t>
+        </is>
+      </c>
+      <c r="D14" s="28" t="inlineStr">
+        <is>
+          <t>BIORAD-20, 20 L</t>
+        </is>
+      </c>
+      <c r="E14" s="15" t="n">
+        <v>400</v>
+      </c>
+      <c r="F14" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" s="15">
+        <f>MAX(0, E14-F14)</f>
+        <v/>
+      </c>
+      <c r="J14" s="15">
+        <f>ABS(F14-E14)</f>
+        <v/>
+      </c>
+      <c r="K14" s="16">
+        <f>IF(E14&gt;0, F14/E14, IF(F14&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L14" s="36" t="inlineStr">
+        <is>
           <t>Sin Pedido</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="24" customHeight="1">
-      <c r="B14" s="21" t="inlineStr">
+    <row r="15" ht="24" customHeight="1">
+      <c r="B15" s="21" t="inlineStr">
         <is>
           <t>TOTAL ALFONSO</t>
         </is>
       </c>
-      <c r="C14" s="36" t="inlineStr">
+      <c r="C15" s="37" t="inlineStr">
         <is>
           <t>276 líneas</t>
         </is>
       </c>
-      <c r="D14" s="37" t="inlineStr"/>
-      <c r="E14" s="23">
-        <f>SUM(E10:E13)</f>
-        <v/>
-      </c>
-      <c r="F14" s="23">
-        <f>SUM(F10:F13)</f>
-        <v/>
-      </c>
-      <c r="G14" s="23">
-        <f>SUM(G10:G13)</f>
-        <v/>
-      </c>
-      <c r="H14" s="23">
-        <f>SUM(H10:H13)</f>
-        <v/>
-      </c>
-      <c r="I14" s="23">
-        <f>SUM(I10:I13)</f>
-        <v/>
-      </c>
-      <c r="J14" s="23">
-        <f>SUM(J10:J13)</f>
-        <v/>
-      </c>
-      <c r="K14" s="24">
-        <f>IF(E14&gt;0, F14/E14, 0)</f>
-        <v/>
-      </c>
-      <c r="L14" s="22">
-        <f>IF(K14&gt;=1, "SUPERADO", "EN CURSO")</f>
+      <c r="D15" s="38" t="inlineStr"/>
+      <c r="E15" s="23">
+        <f>SUM(E10:E14)</f>
+        <v/>
+      </c>
+      <c r="F15" s="23">
+        <f>SUM(F10:F14)</f>
+        <v/>
+      </c>
+      <c r="G15" s="23">
+        <f>SUM(G10:G14)</f>
+        <v/>
+      </c>
+      <c r="H15" s="23">
+        <f>SUM(H10:H14)</f>
+        <v/>
+      </c>
+      <c r="I15" s="23">
+        <f>SUM(I10:I14)</f>
+        <v/>
+      </c>
+      <c r="J15" s="23">
+        <f>SUM(J10:J14)</f>
+        <v/>
+      </c>
+      <c r="K15" s="24">
+        <f>IF(E15&gt;0, F15/E15, 0)</f>
+        <v/>
+      </c>
+      <c r="L15" s="22">
+        <f>IF(K15&gt;=1, "SUPERADO", "EN CURSO")</f>
         <v/>
       </c>
     </row>
@@ -1752,7 +1798,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:L37"/>
+  <dimension ref="B2:L48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1779,7 +1825,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 14/10/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 15/10/2026</t>
         </is>
       </c>
     </row>
@@ -1822,19 +1868,19 @@
         </is>
       </c>
       <c r="C6" s="4" t="n"/>
-      <c r="D6" s="38" t="inlineStr">
-        <is>
-          <t>43,840 u</t>
+      <c r="D6" s="26" t="inlineStr">
+        <is>
+          <t>80,676 u</t>
         </is>
       </c>
       <c r="E6" s="4" t="n"/>
-      <c r="F6" s="38" t="inlineStr">
-        <is>
-          <t>115.9%</t>
+      <c r="F6" s="26" t="inlineStr">
+        <is>
+          <t>213.2%</t>
         </is>
       </c>
       <c r="G6" s="4" t="n"/>
-      <c r="H6" s="38" t="inlineStr">
+      <c r="H6" s="26" t="inlineStr">
         <is>
           <t>0 u</t>
         </is>
@@ -1842,7 +1888,7 @@
       <c r="I6" s="4" t="n"/>
       <c r="J6" s="25" t="inlineStr">
         <is>
-          <t>40,800 u</t>
+          <t>73,996 u</t>
         </is>
       </c>
       <c r="K6" s="4" t="n"/>
@@ -1951,7 +1997,7 @@
         <f>IF(E10&gt;0, F10/E10, IF(F10&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L10" s="39" t="inlineStr">
+      <c r="L10" s="36" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -1997,7 +2043,7 @@
         <f>IF(E11&gt;0, F11/E11, IF(F11&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L11" s="35" t="inlineStr">
+      <c r="L11" s="39" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -2043,7 +2089,7 @@
         <f>IF(E12&gt;0, F12/E12, IF(F12&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L12" s="39" t="inlineStr">
+      <c r="L12" s="36" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -2135,7 +2181,7 @@
         <f>IF(E14&gt;0, F14/E14, IF(F14&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L14" s="39" t="inlineStr">
+      <c r="L14" s="36" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -2181,7 +2227,7 @@
         <f>IF(E15&gt;0, F15/E15, IF(F15&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L15" s="35" t="inlineStr">
+      <c r="L15" s="39" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -2227,7 +2273,7 @@
         <f>IF(E16&gt;0, F16/E16, IF(F16&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L16" s="39" t="inlineStr">
+      <c r="L16" s="36" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -2273,7 +2319,7 @@
         <f>IF(E17&gt;0, F17/E17, IF(F17&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L17" s="35" t="inlineStr">
+      <c r="L17" s="39" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -2319,7 +2365,7 @@
         <f>IF(E18&gt;0, F18/E18, IF(F18&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L18" s="39" t="inlineStr">
+      <c r="L18" s="36" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -2365,7 +2411,7 @@
         <f>IF(E19&gt;0, F19/E19, IF(F19&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L19" s="35" t="inlineStr">
+      <c r="L19" s="39" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -2411,7 +2457,7 @@
         <f>IF(E20&gt;0, F20/E20, IF(F20&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L20" s="39" t="inlineStr">
+      <c r="L20" s="36" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -2457,7 +2503,7 @@
         <f>IF(E21&gt;0, F21/E21, IF(F21&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L21" s="35" t="inlineStr">
+      <c r="L21" s="39" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -2503,7 +2549,7 @@
         <f>IF(E22&gt;0, F22/E22, IF(F22&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L22" s="39" t="inlineStr">
+      <c r="L22" s="36" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -2549,7 +2595,7 @@
         <f>IF(E23&gt;0, F23/E23, IF(F23&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L23" s="35" t="inlineStr">
+      <c r="L23" s="39" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -2609,25 +2655,25 @@
       </c>
       <c r="C25" s="32" t="inlineStr">
         <is>
-          <t>SSEG0005</t>
+          <t>SPAR0001</t>
         </is>
       </c>
       <c r="D25" s="31" t="inlineStr">
         <is>
-          <t>SAL-WAX Ca</t>
+          <t>SPRINTENE ARABIA, 1 L</t>
         </is>
       </c>
       <c r="E25" s="19" t="n">
-        <v>20000</v>
+        <v>0</v>
       </c>
       <c r="F25" s="19" t="n">
-        <v>21000</v>
+        <v>10296</v>
       </c>
       <c r="G25" s="19" t="n">
         <v>0</v>
       </c>
       <c r="H25" s="19" t="n">
-        <v>21000</v>
+        <v>10296</v>
       </c>
       <c r="I25" s="19">
         <f>MAX(0, E25-F25)</f>
@@ -2641,39 +2687,39 @@
         <f>IF(E25&gt;0, F25/E25, IF(F25&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L25" s="40" t="inlineStr">
-        <is>
-          <t>Superado</t>
+      <c r="L25" s="35" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="B26" s="28" t="inlineStr">
         <is>
-          <t>INIESTA DEL PINO DISTRIBUCIONES S.L.U</t>
+          <t>DOTRA CHEMICALS</t>
         </is>
       </c>
       <c r="C26" s="29" t="inlineStr">
         <is>
-          <t>AGXK0020</t>
+          <t>SSEG0005</t>
         </is>
       </c>
       <c r="D26" s="28" t="inlineStr">
         <is>
-          <t>AGROXILATO-K, 20 L</t>
+          <t>SAL-WAX Ca</t>
         </is>
       </c>
       <c r="E26" s="15" t="n">
-        <v>640</v>
+        <v>20000</v>
       </c>
       <c r="F26" s="15" t="n">
-        <v>1920</v>
+        <v>21000</v>
       </c>
       <c r="G26" s="15" t="n">
-        <v>1920</v>
+        <v>0</v>
       </c>
       <c r="H26" s="15" t="n">
-        <v>0</v>
+        <v>21000</v>
       </c>
       <c r="I26" s="15">
         <f>MAX(0, E26-F26)</f>
@@ -2696,30 +2742,30 @@
     <row r="27">
       <c r="B27" s="31" t="inlineStr">
         <is>
-          <t>INIESTA DEL PINO DISTRIBUCIONES S.L.U</t>
+          <t>DOTRA CHEMICALS</t>
         </is>
       </c>
       <c r="C27" s="32" t="inlineStr">
         <is>
-          <t>CBROT0005</t>
+          <t>SSEG0005EG</t>
         </is>
       </c>
       <c r="D27" s="31" t="inlineStr">
         <is>
-          <t>CODIBROT, 5 L</t>
+          <t>SALWAX CALCIO EGIPTO, 5 KG</t>
         </is>
       </c>
       <c r="E27" s="19" t="n">
         <v>0</v>
       </c>
       <c r="F27" s="19" t="n">
-        <v>20</v>
+        <v>8000</v>
       </c>
       <c r="G27" s="19" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="H27" s="19" t="n">
-        <v>0</v>
+        <v>8000</v>
       </c>
       <c r="I27" s="19">
         <f>MAX(0, E27-F27)</f>
@@ -2733,7 +2779,7 @@
         <f>IF(E27&gt;0, F27/E27, IF(F27&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L27" s="40" t="inlineStr">
+      <c r="L27" s="35" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -2747,22 +2793,22 @@
       </c>
       <c r="C28" s="29" t="inlineStr">
         <is>
-          <t>TRI0005</t>
+          <t>AGXK0020</t>
         </is>
       </c>
       <c r="D28" s="28" t="inlineStr">
         <is>
-          <t>TRIFENO-94, 5L</t>
+          <t>AGROXILATO-K, 20 L</t>
         </is>
       </c>
       <c r="E28" s="15" t="n">
-        <v>60</v>
+        <v>640</v>
       </c>
       <c r="F28" s="15" t="n">
-        <v>0</v>
+        <v>1920</v>
       </c>
       <c r="G28" s="15" t="n">
-        <v>0</v>
+        <v>1920</v>
       </c>
       <c r="H28" s="15" t="n">
         <v>0</v>
@@ -2779,36 +2825,36 @@
         <f>IF(E28&gt;0, F28/E28, IF(F28&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L28" s="39" t="inlineStr">
-        <is>
-          <t>Sin Pedido</t>
+      <c r="L28" s="34" t="inlineStr">
+        <is>
+          <t>Superado</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="B29" s="31" t="inlineStr">
         <is>
-          <t>SERVIAGRI´ 97, S.L.</t>
+          <t>INIESTA DEL PINO DISTRIBUCIONES S.L.U</t>
         </is>
       </c>
       <c r="C29" s="32" t="inlineStr">
         <is>
-          <t>AGXK0005</t>
+          <t>CBROT0005</t>
         </is>
       </c>
       <c r="D29" s="31" t="inlineStr">
         <is>
-          <t>AGROXILATO-K, 5 L</t>
+          <t>CODIBROT, 5 L</t>
         </is>
       </c>
       <c r="E29" s="19" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="F29" s="19" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="G29" s="19" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="H29" s="19" t="n">
         <v>0</v>
@@ -2827,28 +2873,28 @@
       </c>
       <c r="L29" s="35" t="inlineStr">
         <is>
-          <t>Sin Pedido</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="B30" s="28" t="inlineStr">
         <is>
-          <t>SERVIAGRI´ 97, S.L.</t>
+          <t>INIESTA DEL PINO DISTRIBUCIONES S.L.U</t>
         </is>
       </c>
       <c r="C30" s="29" t="inlineStr">
         <is>
-          <t>AVAN0005</t>
+          <t>TRI0005</t>
         </is>
       </c>
       <c r="D30" s="28" t="inlineStr">
         <is>
-          <t>FLORAMEC AVANCE, 5 L</t>
+          <t>TRIFENO-94, 5L</t>
         </is>
       </c>
       <c r="E30" s="15" t="n">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="F30" s="15" t="n">
         <v>0</v>
@@ -2871,7 +2917,7 @@
         <f>IF(E30&gt;0, F30/E30, IF(F30&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L30" s="39" t="inlineStr">
+      <c r="L30" s="36" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -2885,16 +2931,16 @@
       </c>
       <c r="C31" s="32" t="inlineStr">
         <is>
-          <t>B0001</t>
+          <t>AGXK0005</t>
         </is>
       </c>
       <c r="D31" s="31" t="inlineStr">
         <is>
-          <t>BOROCAL,1 L</t>
+          <t>AGROXILATO-K, 5 L</t>
         </is>
       </c>
       <c r="E31" s="19" t="n">
-        <v>12</v>
+        <v>200</v>
       </c>
       <c r="F31" s="19" t="n">
         <v>0</v>
@@ -2917,7 +2963,7 @@
         <f>IF(E31&gt;0, F31/E31, IF(F31&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L31" s="35" t="inlineStr">
+      <c r="L31" s="39" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -2931,16 +2977,16 @@
       </c>
       <c r="C32" s="29" t="inlineStr">
         <is>
-          <t>BIO0005</t>
+          <t>AVAN0005</t>
         </is>
       </c>
       <c r="D32" s="28" t="inlineStr">
         <is>
-          <t>BIORAD-20, 5L</t>
+          <t>FLORAMEC AVANCE, 5 L</t>
         </is>
       </c>
       <c r="E32" s="15" t="n">
-        <v>300</v>
+        <v>100</v>
       </c>
       <c r="F32" s="15" t="n">
         <v>0</v>
@@ -2963,7 +3009,7 @@
         <f>IF(E32&gt;0, F32/E32, IF(F32&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L32" s="39" t="inlineStr">
+      <c r="L32" s="36" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -2977,25 +3023,25 @@
       </c>
       <c r="C33" s="32" t="inlineStr">
         <is>
-          <t>BIO1000</t>
+          <t>B0001</t>
         </is>
       </c>
       <c r="D33" s="31" t="inlineStr">
         <is>
-          <t>BIORAD-20, 1000 L</t>
+          <t>BOROCAL,1 L</t>
         </is>
       </c>
       <c r="E33" s="19" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="F33" s="19" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="G33" s="19" t="n">
         <v>0</v>
       </c>
       <c r="H33" s="19" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="I33" s="19">
         <f>MAX(0, E33-F33)</f>
@@ -3009,9 +3055,9 @@
         <f>IF(E33&gt;0, F33/E33, IF(F33&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L33" s="40" t="inlineStr">
-        <is>
-          <t>Extra Estimación</t>
+      <c r="L33" s="39" t="inlineStr">
+        <is>
+          <t>Sin Pedido</t>
         </is>
       </c>
     </row>
@@ -3023,12 +3069,12 @@
       </c>
       <c r="C34" s="29" t="inlineStr">
         <is>
-          <t>FTK0005</t>
+          <t>BIO0005</t>
         </is>
       </c>
       <c r="D34" s="28" t="inlineStr">
         <is>
-          <t>FITOKONTROL CA FLOW, 5 KG</t>
+          <t>BIORAD-20, 5L</t>
         </is>
       </c>
       <c r="E34" s="15" t="n">
@@ -3055,7 +3101,7 @@
         <f>IF(E34&gt;0, F34/E34, IF(F34&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L34" s="39" t="inlineStr">
+      <c r="L34" s="36" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -3069,22 +3115,22 @@
       </c>
       <c r="C35" s="32" t="inlineStr">
         <is>
-          <t>JF0005</t>
+          <t>BIO1000</t>
         </is>
       </c>
       <c r="D35" s="31" t="inlineStr">
         <is>
-          <t>CODIGIN-FOS, 5 L</t>
+          <t>BIORAD-20, 1000 L</t>
         </is>
       </c>
       <c r="E35" s="19" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="F35" s="19" t="n">
-        <v>0</v>
+        <v>3000</v>
       </c>
       <c r="G35" s="19" t="n">
-        <v>0</v>
+        <v>3000</v>
       </c>
       <c r="H35" s="19" t="n">
         <v>0</v>
@@ -3103,28 +3149,28 @@
       </c>
       <c r="L35" s="35" t="inlineStr">
         <is>
-          <t>Sin Pedido</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="B36" s="28" t="inlineStr">
         <is>
-          <t>TRATAMIENTOS AGRICOLAS BRENES, S.L.</t>
+          <t>SERVIAGRI´ 97, S.L.</t>
         </is>
       </c>
       <c r="C36" s="29" t="inlineStr">
         <is>
-          <t>WHITE0020</t>
+          <t>FTK0005</t>
         </is>
       </c>
       <c r="D36" s="28" t="inlineStr">
         <is>
-          <t>AGROWHITE, 20 KG</t>
+          <t>FITOKONTROL CA FLOW, 5 KG</t>
         </is>
       </c>
       <c r="E36" s="15" t="n">
-        <v>1100</v>
+        <v>300</v>
       </c>
       <c r="F36" s="15" t="n">
         <v>0</v>
@@ -3147,54 +3193,560 @@
         <f>IF(E36&gt;0, F36/E36, IF(F36&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L36" s="39" t="inlineStr">
+      <c r="L36" s="36" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="24" customHeight="1">
-      <c r="B37" s="21" t="inlineStr">
+    <row r="37">
+      <c r="B37" s="31" t="inlineStr">
+        <is>
+          <t>SERVIAGRI´ 97, S.L.</t>
+        </is>
+      </c>
+      <c r="C37" s="32" t="inlineStr">
+        <is>
+          <t>JF0005</t>
+        </is>
+      </c>
+      <c r="D37" s="31" t="inlineStr">
+        <is>
+          <t>CODIGIN-FOS, 5 L</t>
+        </is>
+      </c>
+      <c r="E37" s="19" t="n">
+        <v>100</v>
+      </c>
+      <c r="F37" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G37" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H37" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I37" s="19">
+        <f>MAX(0, E37-F37)</f>
+        <v/>
+      </c>
+      <c r="J37" s="19">
+        <f>ABS(F37-E37)</f>
+        <v/>
+      </c>
+      <c r="K37" s="20">
+        <f>IF(E37&gt;0, F37/E37, IF(F37&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L37" s="39" t="inlineStr">
+        <is>
+          <t>Sin Pedido</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" s="28" t="inlineStr">
+        <is>
+          <t>STE BBMAGRI, SARL</t>
+        </is>
+      </c>
+      <c r="C38" s="29" t="inlineStr">
+        <is>
+          <t>A-500020</t>
+        </is>
+      </c>
+      <c r="D38" s="28" t="inlineStr">
+        <is>
+          <t>CODIORGAN-A50, 20 KG</t>
+        </is>
+      </c>
+      <c r="E38" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F38" s="15" t="n">
+        <v>1500</v>
+      </c>
+      <c r="G38" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H38" s="15" t="n">
+        <v>1500</v>
+      </c>
+      <c r="I38" s="15">
+        <f>MAX(0, E38-F38)</f>
+        <v/>
+      </c>
+      <c r="J38" s="15">
+        <f>ABS(F38-E38)</f>
+        <v/>
+      </c>
+      <c r="K38" s="16">
+        <f>IF(E38&gt;0, F38/E38, IF(F38&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L38" s="34" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" s="31" t="inlineStr">
+        <is>
+          <t>STE BBMAGRI, SARL</t>
+        </is>
+      </c>
+      <c r="C39" s="32" t="inlineStr">
+        <is>
+          <t>AGXCR0020</t>
+        </is>
+      </c>
+      <c r="D39" s="31" t="inlineStr">
+        <is>
+          <t>GREEN MAX</t>
+        </is>
+      </c>
+      <c r="E39" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F39" s="19" t="n">
+        <v>7000</v>
+      </c>
+      <c r="G39" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H39" s="19" t="n">
+        <v>7000</v>
+      </c>
+      <c r="I39" s="19">
+        <f>MAX(0, E39-F39)</f>
+        <v/>
+      </c>
+      <c r="J39" s="19">
+        <f>ABS(F39-E39)</f>
+        <v/>
+      </c>
+      <c r="K39" s="20">
+        <f>IF(E39&gt;0, F39/E39, IF(F39&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L39" s="35" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" s="28" t="inlineStr">
+        <is>
+          <t>STE BBMAGRI, SARL</t>
+        </is>
+      </c>
+      <c r="C40" s="29" t="inlineStr">
+        <is>
+          <t>AVAN0020</t>
+        </is>
+      </c>
+      <c r="D40" s="28" t="inlineStr">
+        <is>
+          <t>FLORAMEC AVANCE</t>
+        </is>
+      </c>
+      <c r="E40" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F40" s="15" t="n">
+        <v>2000</v>
+      </c>
+      <c r="G40" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H40" s="15" t="n">
+        <v>2000</v>
+      </c>
+      <c r="I40" s="15">
+        <f>MAX(0, E40-F40)</f>
+        <v/>
+      </c>
+      <c r="J40" s="15">
+        <f>ABS(F40-E40)</f>
+        <v/>
+      </c>
+      <c r="K40" s="16">
+        <f>IF(E40&gt;0, F40/E40, IF(F40&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L40" s="34" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" s="31" t="inlineStr">
+        <is>
+          <t>STE BBMAGRI, SARL</t>
+        </is>
+      </c>
+      <c r="C41" s="32" t="inlineStr">
+        <is>
+          <t>BR-590005</t>
+        </is>
+      </c>
+      <c r="D41" s="31" t="inlineStr">
+        <is>
+          <t>BR-59</t>
+        </is>
+      </c>
+      <c r="E41" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F41" s="19" t="n">
+        <v>800</v>
+      </c>
+      <c r="G41" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H41" s="19" t="n">
+        <v>800</v>
+      </c>
+      <c r="I41" s="19">
+        <f>MAX(0, E41-F41)</f>
+        <v/>
+      </c>
+      <c r="J41" s="19">
+        <f>ABS(F41-E41)</f>
+        <v/>
+      </c>
+      <c r="K41" s="20">
+        <f>IF(E41&gt;0, F41/E41, IF(F41&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L41" s="35" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" s="28" t="inlineStr">
+        <is>
+          <t>STE BBMAGRI, SARL</t>
+        </is>
+      </c>
+      <c r="C42" s="29" t="inlineStr">
+        <is>
+          <t>C-CU20005</t>
+        </is>
+      </c>
+      <c r="D42" s="28" t="inlineStr">
+        <is>
+          <t>CODICOBRE (EGIPTO), 5 L</t>
+        </is>
+      </c>
+      <c r="E42" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F42" s="15" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G42" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H42" s="15" t="n">
+        <v>1000</v>
+      </c>
+      <c r="I42" s="15">
+        <f>MAX(0, E42-F42)</f>
+        <v/>
+      </c>
+      <c r="J42" s="15">
+        <f>ABS(F42-E42)</f>
+        <v/>
+      </c>
+      <c r="K42" s="16">
+        <f>IF(E42&gt;0, F42/E42, IF(F42&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L42" s="34" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" s="31" t="inlineStr">
+        <is>
+          <t>STE BBMAGRI, SARL</t>
+        </is>
+      </c>
+      <c r="C43" s="32" t="inlineStr">
+        <is>
+          <t>PHD0020</t>
+        </is>
+      </c>
+      <c r="D43" s="31" t="inlineStr">
+        <is>
+          <t>PH-DOWNER</t>
+        </is>
+      </c>
+      <c r="E43" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F43" s="19" t="n">
+        <v>600</v>
+      </c>
+      <c r="G43" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H43" s="19" t="n">
+        <v>600</v>
+      </c>
+      <c r="I43" s="19">
+        <f>MAX(0, E43-F43)</f>
+        <v/>
+      </c>
+      <c r="J43" s="19">
+        <f>ABS(F43-E43)</f>
+        <v/>
+      </c>
+      <c r="K43" s="20">
+        <f>IF(E43&gt;0, F43/E43, IF(F43&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L43" s="35" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" s="28" t="inlineStr">
+        <is>
+          <t>STE BBMAGRI, SARL</t>
+        </is>
+      </c>
+      <c r="C44" s="29" t="inlineStr">
+        <is>
+          <t>PT0020</t>
+        </is>
+      </c>
+      <c r="D44" s="28" t="inlineStr">
+        <is>
+          <t>AGROPOTASION</t>
+        </is>
+      </c>
+      <c r="E44" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F44" s="15" t="n">
+        <v>3000</v>
+      </c>
+      <c r="G44" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H44" s="15" t="n">
+        <v>3000</v>
+      </c>
+      <c r="I44" s="15">
+        <f>MAX(0, E44-F44)</f>
+        <v/>
+      </c>
+      <c r="J44" s="15">
+        <f>ABS(F44-E44)</f>
+        <v/>
+      </c>
+      <c r="K44" s="16">
+        <f>IF(E44&gt;0, F44/E44, IF(F44&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L44" s="34" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" s="31" t="inlineStr">
+        <is>
+          <t>STE BBMAGRI, SARL</t>
+        </is>
+      </c>
+      <c r="C45" s="32" t="inlineStr">
+        <is>
+          <t>SS0020</t>
+        </is>
+      </c>
+      <c r="D45" s="31" t="inlineStr">
+        <is>
+          <t>SAL-WAX-Ca</t>
+        </is>
+      </c>
+      <c r="E45" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F45" s="19" t="n">
+        <v>2000</v>
+      </c>
+      <c r="G45" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H45" s="19" t="n">
+        <v>2000</v>
+      </c>
+      <c r="I45" s="19">
+        <f>MAX(0, E45-F45)</f>
+        <v/>
+      </c>
+      <c r="J45" s="19">
+        <f>ABS(F45-E45)</f>
+        <v/>
+      </c>
+      <c r="K45" s="20">
+        <f>IF(E45&gt;0, F45/E45, IF(F45&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L45" s="35" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" s="28" t="inlineStr">
+        <is>
+          <t>TRATAMIENTOS AGRICOLAS BRENES, S.L.</t>
+        </is>
+      </c>
+      <c r="C46" s="29" t="inlineStr">
+        <is>
+          <t>PT0020</t>
+        </is>
+      </c>
+      <c r="D46" s="28" t="inlineStr">
+        <is>
+          <t>AGROPOTASION, 20 L</t>
+        </is>
+      </c>
+      <c r="E46" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F46" s="15" t="n">
+        <v>640</v>
+      </c>
+      <c r="G46" s="15" t="n">
+        <v>640</v>
+      </c>
+      <c r="H46" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I46" s="15">
+        <f>MAX(0, E46-F46)</f>
+        <v/>
+      </c>
+      <c r="J46" s="15">
+        <f>ABS(F46-E46)</f>
+        <v/>
+      </c>
+      <c r="K46" s="16">
+        <f>IF(E46&gt;0, F46/E46, IF(F46&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L46" s="34" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="B47" s="31" t="inlineStr">
+        <is>
+          <t>TRATAMIENTOS AGRICOLAS BRENES, S.L.</t>
+        </is>
+      </c>
+      <c r="C47" s="32" t="inlineStr">
+        <is>
+          <t>WHITE0020</t>
+        </is>
+      </c>
+      <c r="D47" s="31" t="inlineStr">
+        <is>
+          <t>AGROWHITE, 20 KG</t>
+        </is>
+      </c>
+      <c r="E47" s="19" t="n">
+        <v>1100</v>
+      </c>
+      <c r="F47" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G47" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H47" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I47" s="19">
+        <f>MAX(0, E47-F47)</f>
+        <v/>
+      </c>
+      <c r="J47" s="19">
+        <f>ABS(F47-E47)</f>
+        <v/>
+      </c>
+      <c r="K47" s="20">
+        <f>IF(E47&gt;0, F47/E47, IF(F47&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L47" s="39" t="inlineStr">
+        <is>
+          <t>Sin Pedido</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="24" customHeight="1">
+      <c r="B48" s="21" t="inlineStr">
         <is>
           <t>TOTAL GARCÍA</t>
         </is>
       </c>
-      <c r="C37" s="36" t="inlineStr">
-        <is>
-          <t>232 líneas</t>
-        </is>
-      </c>
-      <c r="D37" s="37" t="inlineStr"/>
-      <c r="E37" s="23">
-        <f>SUM(E10:E36)</f>
-        <v/>
-      </c>
-      <c r="F37" s="23">
-        <f>SUM(F10:F36)</f>
-        <v/>
-      </c>
-      <c r="G37" s="23">
-        <f>SUM(G10:G36)</f>
-        <v/>
-      </c>
-      <c r="H37" s="23">
-        <f>SUM(H10:H36)</f>
-        <v/>
-      </c>
-      <c r="I37" s="23">
-        <f>SUM(I10:I36)</f>
-        <v/>
-      </c>
-      <c r="J37" s="23">
-        <f>SUM(J10:J36)</f>
-        <v/>
-      </c>
-      <c r="K37" s="24">
-        <f>IF(E37&gt;0, F37/E37, 0)</f>
-        <v/>
-      </c>
-      <c r="L37" s="22">
-        <f>IF(K37&gt;=1, "SUPERADO", "EN CURSO")</f>
+      <c r="C48" s="37" t="inlineStr">
+        <is>
+          <t>236 líneas</t>
+        </is>
+      </c>
+      <c r="D48" s="38" t="inlineStr"/>
+      <c r="E48" s="23">
+        <f>SUM(E10:E47)</f>
+        <v/>
+      </c>
+      <c r="F48" s="23">
+        <f>SUM(F10:F47)</f>
+        <v/>
+      </c>
+      <c r="G48" s="23">
+        <f>SUM(G10:G47)</f>
+        <v/>
+      </c>
+      <c r="H48" s="23">
+        <f>SUM(H10:H47)</f>
+        <v/>
+      </c>
+      <c r="I48" s="23">
+        <f>SUM(I10:I47)</f>
+        <v/>
+      </c>
+      <c r="J48" s="23">
+        <f>SUM(J10:J47)</f>
+        <v/>
+      </c>
+      <c r="K48" s="24">
+        <f>IF(E48&gt;0, F48/E48, 0)</f>
+        <v/>
+      </c>
+      <c r="L48" s="22">
+        <f>IF(K48&gt;=1, "SUPERADO", "EN CURSO")</f>
         <v/>
       </c>
     </row>
@@ -3223,7 +3775,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:L46"/>
+  <dimension ref="B2:L48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -3250,7 +3802,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 14/10/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 15/10/2026</t>
         </is>
       </c>
     </row>
@@ -3295,19 +3847,19 @@
       <c r="C6" s="4" t="n"/>
       <c r="D6" s="25" t="inlineStr">
         <is>
-          <t>9,580 u</t>
+          <t>11,820 u</t>
         </is>
       </c>
       <c r="E6" s="4" t="n"/>
-      <c r="F6" s="26" t="inlineStr">
-        <is>
-          <t>43.7%</t>
+      <c r="F6" s="40" t="inlineStr">
+        <is>
+          <t>53.9%</t>
         </is>
       </c>
       <c r="G6" s="4" t="n"/>
-      <c r="H6" s="26" t="inlineStr">
-        <is>
-          <t>12,334 u</t>
+      <c r="H6" s="40" t="inlineStr">
+        <is>
+          <t>10,094 u</t>
         </is>
       </c>
       <c r="I6" s="4" t="n"/>
@@ -3422,7 +3974,7 @@
         <f>IF(E10&gt;0, F10/E10, IF(F10&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L10" s="39" t="inlineStr">
+      <c r="L10" s="36" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -3652,7 +4204,7 @@
         <f>IF(E15&gt;0, F15/E15, IF(F15&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L15" s="35" t="inlineStr">
+      <c r="L15" s="39" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -3698,7 +4250,7 @@
         <f>IF(E16&gt;0, F16/E16, IF(F16&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L16" s="39" t="inlineStr">
+      <c r="L16" s="36" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -3744,7 +4296,7 @@
         <f>IF(E17&gt;0, F17/E17, IF(F17&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L17" s="35" t="inlineStr">
+      <c r="L17" s="39" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -3790,7 +4342,7 @@
         <f>IF(E18&gt;0, F18/E18, IF(F18&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L18" s="39" t="inlineStr">
+      <c r="L18" s="36" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -3882,7 +4434,7 @@
         <f>IF(E20&gt;0, F20/E20, IF(F20&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L20" s="39" t="inlineStr">
+      <c r="L20" s="36" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -3928,7 +4480,7 @@
         <f>IF(E21&gt;0, F21/E21, IF(F21&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L21" s="40" t="inlineStr">
+      <c r="L21" s="35" t="inlineStr">
         <is>
           <t>Superado</t>
         </is>
@@ -3974,7 +4526,7 @@
         <f>IF(E22&gt;0, F22/E22, IF(F22&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L22" s="39" t="inlineStr">
+      <c r="L22" s="36" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -4066,7 +4618,7 @@
         <f>IF(E24&gt;0, F24/E24, IF(F24&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L24" s="39" t="inlineStr">
+      <c r="L24" s="36" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -4112,7 +4664,7 @@
         <f>IF(E25&gt;0, F25/E25, IF(F25&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L25" s="35" t="inlineStr">
+      <c r="L25" s="39" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -4204,7 +4756,7 @@
         <f>IF(E27&gt;0, F27/E27, IF(F27&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L27" s="35" t="inlineStr">
+      <c r="L27" s="39" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -4296,7 +4848,7 @@
         <f>IF(E29&gt;0, F29/E29, IF(F29&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L29" s="40" t="inlineStr">
+      <c r="L29" s="35" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -4388,7 +4940,7 @@
         <f>IF(E31&gt;0, F31/E31, IF(F31&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L31" s="40" t="inlineStr">
+      <c r="L31" s="35" t="inlineStr">
         <is>
           <t>Superado</t>
         </is>
@@ -4480,7 +5032,7 @@
         <f>IF(E33&gt;0, F33/E33, IF(F33&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L33" s="35" t="inlineStr">
+      <c r="L33" s="39" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -4572,7 +5124,7 @@
         <f>IF(E35&gt;0, F35/E35, IF(F35&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L35" s="40" t="inlineStr">
+      <c r="L35" s="35" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -4644,10 +5196,10 @@
         <v>100</v>
       </c>
       <c r="F37" s="19" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="G37" s="19" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="H37" s="19" t="n">
         <v>0</v>
@@ -4666,7 +5218,7 @@
       </c>
       <c r="L37" s="35" t="inlineStr">
         <is>
-          <t>Sin Pedido</t>
+          <t>Superado</t>
         </is>
       </c>
     </row>
@@ -4710,7 +5262,7 @@
         <f>IF(E38&gt;0, F38/E38, IF(F38&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L38" s="39" t="inlineStr">
+      <c r="L38" s="36" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -4756,7 +5308,7 @@
         <f>IF(E39&gt;0, F39/E39, IF(F39&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L39" s="35" t="inlineStr">
+      <c r="L39" s="39" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -4802,7 +5354,7 @@
         <f>IF(E40&gt;0, F40/E40, IF(F40&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L40" s="39" t="inlineStr">
+      <c r="L40" s="36" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -4816,22 +5368,22 @@
       </c>
       <c r="C41" s="32" t="inlineStr">
         <is>
-          <t>AVAN0020</t>
+          <t>AVAN0005</t>
         </is>
       </c>
       <c r="D41" s="31" t="inlineStr">
         <is>
-          <t>FLORAMEC AVANCE, 20 L</t>
+          <t>FLORAMEC AVANCE, 5 L</t>
         </is>
       </c>
       <c r="E41" s="19" t="n">
-        <v>640</v>
+        <v>0</v>
       </c>
       <c r="F41" s="19" t="n">
-        <v>0</v>
+        <v>600</v>
       </c>
       <c r="G41" s="19" t="n">
-        <v>0</v>
+        <v>600</v>
       </c>
       <c r="H41" s="19" t="n">
         <v>0</v>
@@ -4850,7 +5402,7 @@
       </c>
       <c r="L41" s="35" t="inlineStr">
         <is>
-          <t>Sin Pedido</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -4862,22 +5414,22 @@
       </c>
       <c r="C42" s="29" t="inlineStr">
         <is>
-          <t>BEY0020</t>
+          <t>AVAN0020</t>
         </is>
       </c>
       <c r="D42" s="28" t="inlineStr">
         <is>
-          <t>FLORAMEC PLUS 20 L</t>
+          <t>FLORAMEC AVANCE, 20 L</t>
         </is>
       </c>
       <c r="E42" s="15" t="n">
-        <v>80</v>
+        <v>640</v>
       </c>
       <c r="F42" s="15" t="n">
-        <v>0</v>
+        <v>640</v>
       </c>
       <c r="G42" s="15" t="n">
-        <v>0</v>
+        <v>640</v>
       </c>
       <c r="H42" s="15" t="n">
         <v>0</v>
@@ -4894,9 +5446,9 @@
         <f>IF(E42&gt;0, F42/E42, IF(F42&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L42" s="39" t="inlineStr">
-        <is>
-          <t>Sin Pedido</t>
+      <c r="L42" s="34" t="inlineStr">
+        <is>
+          <t>Superado</t>
         </is>
       </c>
     </row>
@@ -4908,16 +5460,16 @@
       </c>
       <c r="C43" s="32" t="inlineStr">
         <is>
-          <t>BROTA0005</t>
+          <t>BEY0020</t>
         </is>
       </c>
       <c r="D43" s="31" t="inlineStr">
         <is>
-          <t>BROTAMEC, 5 L</t>
+          <t>FLORAMEC PLUS 20 L</t>
         </is>
       </c>
       <c r="E43" s="19" t="n">
-        <v>600</v>
+        <v>80</v>
       </c>
       <c r="F43" s="19" t="n">
         <v>0</v>
@@ -4940,7 +5492,7 @@
         <f>IF(E43&gt;0, F43/E43, IF(F43&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L43" s="35" t="inlineStr">
+      <c r="L43" s="39" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -4954,22 +5506,22 @@
       </c>
       <c r="C44" s="29" t="inlineStr">
         <is>
-          <t>C-M-P0001</t>
+          <t>BROTA0005</t>
         </is>
       </c>
       <c r="D44" s="28" t="inlineStr">
         <is>
-          <t>CODIFOL Mo-PLUS, 1 L</t>
+          <t>BROTAMEC, 5 L</t>
         </is>
       </c>
       <c r="E44" s="15" t="n">
-        <v>36</v>
+        <v>600</v>
       </c>
       <c r="F44" s="15" t="n">
-        <v>0</v>
+        <v>600</v>
       </c>
       <c r="G44" s="15" t="n">
-        <v>0</v>
+        <v>600</v>
       </c>
       <c r="H44" s="15" t="n">
         <v>0</v>
@@ -4986,9 +5538,9 @@
         <f>IF(E44&gt;0, F44/E44, IF(F44&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L44" s="39" t="inlineStr">
-        <is>
-          <t>Sin Pedido</t>
+      <c r="L44" s="34" t="inlineStr">
+        <is>
+          <t>Superado</t>
         </is>
       </c>
     </row>
@@ -5000,16 +5552,16 @@
       </c>
       <c r="C45" s="32" t="inlineStr">
         <is>
-          <t>FTK0005</t>
+          <t>C-M-P0001</t>
         </is>
       </c>
       <c r="D45" s="31" t="inlineStr">
         <is>
-          <t>FITOKONTROL CA FLOW, 5 KG</t>
+          <t>CODIFOL Mo-PLUS, 1 L</t>
         </is>
       </c>
       <c r="E45" s="19" t="n">
-        <v>800</v>
+        <v>36</v>
       </c>
       <c r="F45" s="19" t="n">
         <v>0</v>
@@ -5032,54 +5584,146 @@
         <f>IF(E45&gt;0, F45/E45, IF(F45&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L45" s="35" t="inlineStr">
+      <c r="L45" s="39" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
       </c>
     </row>
-    <row r="46" ht="24" customHeight="1">
-      <c r="B46" s="21" t="inlineStr">
+    <row r="46">
+      <c r="B46" s="28" t="inlineStr">
+        <is>
+          <t>GUIVARTO AGRICOLA, S.L.</t>
+        </is>
+      </c>
+      <c r="C46" s="29" t="inlineStr">
+        <is>
+          <t>FTK0005</t>
+        </is>
+      </c>
+      <c r="D46" s="28" t="inlineStr">
+        <is>
+          <t>FITOKONTROL CA FLOW, 5 KG</t>
+        </is>
+      </c>
+      <c r="E46" s="15" t="n">
+        <v>800</v>
+      </c>
+      <c r="F46" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G46" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H46" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I46" s="15">
+        <f>MAX(0, E46-F46)</f>
+        <v/>
+      </c>
+      <c r="J46" s="15">
+        <f>ABS(F46-E46)</f>
+        <v/>
+      </c>
+      <c r="K46" s="16">
+        <f>IF(E46&gt;0, F46/E46, IF(F46&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L46" s="36" t="inlineStr">
+        <is>
+          <t>Sin Pedido</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="B47" s="31" t="inlineStr">
+        <is>
+          <t>GUIVARTO AGRICOLA, S.L.</t>
+        </is>
+      </c>
+      <c r="C47" s="32" t="inlineStr">
+        <is>
+          <t>TRI0005</t>
+        </is>
+      </c>
+      <c r="D47" s="31" t="inlineStr">
+        <is>
+          <t>TRIFENO-94, 5L</t>
+        </is>
+      </c>
+      <c r="E47" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F47" s="19" t="n">
+        <v>300</v>
+      </c>
+      <c r="G47" s="19" t="n">
+        <v>300</v>
+      </c>
+      <c r="H47" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I47" s="19">
+        <f>MAX(0, E47-F47)</f>
+        <v/>
+      </c>
+      <c r="J47" s="19">
+        <f>ABS(F47-E47)</f>
+        <v/>
+      </c>
+      <c r="K47" s="20">
+        <f>IF(E47&gt;0, F47/E47, IF(F47&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L47" s="35" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="24" customHeight="1">
+      <c r="B48" s="21" t="inlineStr">
         <is>
           <t>TOTAL IRENE</t>
         </is>
       </c>
-      <c r="C46" s="36" t="inlineStr">
+      <c r="C48" s="37" t="inlineStr">
         <is>
           <t>89 líneas</t>
         </is>
       </c>
-      <c r="D46" s="37" t="inlineStr"/>
-      <c r="E46" s="23">
-        <f>SUM(E10:E45)</f>
-        <v/>
-      </c>
-      <c r="F46" s="23">
-        <f>SUM(F10:F45)</f>
-        <v/>
-      </c>
-      <c r="G46" s="23">
-        <f>SUM(G10:G45)</f>
-        <v/>
-      </c>
-      <c r="H46" s="23">
-        <f>SUM(H10:H45)</f>
-        <v/>
-      </c>
-      <c r="I46" s="23">
-        <f>SUM(I10:I45)</f>
-        <v/>
-      </c>
-      <c r="J46" s="23">
-        <f>SUM(J10:J45)</f>
-        <v/>
-      </c>
-      <c r="K46" s="24">
-        <f>IF(E46&gt;0, F46/E46, 0)</f>
-        <v/>
-      </c>
-      <c r="L46" s="22">
-        <f>IF(K46&gt;=1, "SUPERADO", "EN CURSO")</f>
+      <c r="D48" s="38" t="inlineStr"/>
+      <c r="E48" s="23">
+        <f>SUM(E10:E47)</f>
+        <v/>
+      </c>
+      <c r="F48" s="23">
+        <f>SUM(F10:F47)</f>
+        <v/>
+      </c>
+      <c r="G48" s="23">
+        <f>SUM(G10:G47)</f>
+        <v/>
+      </c>
+      <c r="H48" s="23">
+        <f>SUM(H10:H47)</f>
+        <v/>
+      </c>
+      <c r="I48" s="23">
+        <f>SUM(I10:I47)</f>
+        <v/>
+      </c>
+      <c r="J48" s="23">
+        <f>SUM(J10:J47)</f>
+        <v/>
+      </c>
+      <c r="K48" s="24">
+        <f>IF(E48&gt;0, F48/E48, 0)</f>
+        <v/>
+      </c>
+      <c r="L48" s="22">
+        <f>IF(K48&gt;=1, "SUPERADO", "EN CURSO")</f>
         <v/>
       </c>
     </row>
@@ -5108,7 +5752,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:L26"/>
+  <dimension ref="B2:L27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -5135,7 +5779,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 14/10/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 15/10/2026</t>
         </is>
       </c>
     </row>
@@ -5180,25 +5824,25 @@
       <c r="C6" s="4" t="n"/>
       <c r="D6" s="25" t="inlineStr">
         <is>
-          <t>6,760 u</t>
+          <t>7,760 u</t>
         </is>
       </c>
       <c r="E6" s="4" t="n"/>
-      <c r="F6" s="26" t="inlineStr">
-        <is>
-          <t>39.5%</t>
+      <c r="F6" s="40" t="inlineStr">
+        <is>
+          <t>45.4%</t>
         </is>
       </c>
       <c r="G6" s="4" t="n"/>
-      <c r="H6" s="26" t="inlineStr">
-        <is>
-          <t>10,340 u</t>
+      <c r="H6" s="40" t="inlineStr">
+        <is>
+          <t>9,340 u</t>
         </is>
       </c>
       <c r="I6" s="4" t="n"/>
       <c r="J6" s="25" t="inlineStr">
         <is>
-          <t>5,300 u</t>
+          <t>6,300 u</t>
         </is>
       </c>
       <c r="K6" s="4" t="n"/>
@@ -5353,7 +5997,7 @@
         <f>IF(E11&gt;0, F11/E11, IF(F11&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L11" s="40" t="inlineStr">
+      <c r="L11" s="35" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -5445,7 +6089,7 @@
         <f>IF(E13&gt;0, F13/E13, IF(F13&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L13" s="40" t="inlineStr">
+      <c r="L13" s="35" t="inlineStr">
         <is>
           <t>Superado</t>
         </is>
@@ -5537,7 +6181,7 @@
         <f>IF(E15&gt;0, F15/E15, IF(F15&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L15" s="40" t="inlineStr">
+      <c r="L15" s="35" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -5583,7 +6227,7 @@
         <f>IF(E16&gt;0, F16/E16, IF(F16&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L16" s="39" t="inlineStr">
+      <c r="L16" s="36" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -5629,7 +6273,7 @@
         <f>IF(E17&gt;0, F17/E17, IF(F17&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L17" s="40" t="inlineStr">
+      <c r="L17" s="35" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -5675,7 +6319,7 @@
         <f>IF(E18&gt;0, F18/E18, IF(F18&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L18" s="39" t="inlineStr">
+      <c r="L18" s="36" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -5721,7 +6365,7 @@
         <f>IF(E19&gt;0, F19/E19, IF(F19&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L19" s="35" t="inlineStr">
+      <c r="L19" s="39" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -5813,7 +6457,7 @@
         <f>IF(E21&gt;0, F21/E21, IF(F21&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L21" s="40" t="inlineStr">
+      <c r="L21" s="35" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -5868,30 +6512,30 @@
     <row r="23">
       <c r="B23" s="31" t="inlineStr">
         <is>
-          <t>FITOSANITARIOS CARCAIXENT, S.L.</t>
+          <t>FINCA DOÑA ANA C.B.</t>
         </is>
       </c>
       <c r="C23" s="32" t="inlineStr">
         <is>
-          <t>PT0020</t>
+          <t>PT1000</t>
         </is>
       </c>
       <c r="D23" s="31" t="inlineStr">
         <is>
-          <t>AGROPOTASION, 20 L</t>
+          <t>AGROPOTASION, 1000 L</t>
         </is>
       </c>
       <c r="E23" s="19" t="n">
         <v>0</v>
       </c>
       <c r="F23" s="19" t="n">
-        <v>640</v>
+        <v>1000</v>
       </c>
       <c r="G23" s="19" t="n">
-        <v>640</v>
+        <v>0</v>
       </c>
       <c r="H23" s="19" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="I23" s="19">
         <f>MAX(0, E23-F23)</f>
@@ -5905,7 +6549,7 @@
         <f>IF(E23&gt;0, F23/E23, IF(F23&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L23" s="40" t="inlineStr">
+      <c r="L23" s="35" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -5914,27 +6558,27 @@
     <row r="24">
       <c r="B24" s="28" t="inlineStr">
         <is>
-          <t>FITOXENT S.C.L.V.</t>
+          <t>FITOSANITARIOS CARCAIXENT, S.L.</t>
         </is>
       </c>
       <c r="C24" s="29" t="inlineStr">
         <is>
-          <t>FTK0005</t>
+          <t>PT0020</t>
         </is>
       </c>
       <c r="D24" s="28" t="inlineStr">
         <is>
-          <t>FITOKONTROL CA FLOW, 5 KG</t>
+          <t>AGROPOTASION, 20 L</t>
         </is>
       </c>
       <c r="E24" s="15" t="n">
-        <v>4400</v>
+        <v>0</v>
       </c>
       <c r="F24" s="15" t="n">
-        <v>0</v>
+        <v>640</v>
       </c>
       <c r="G24" s="15" t="n">
-        <v>0</v>
+        <v>640</v>
       </c>
       <c r="H24" s="15" t="n">
         <v>0</v>
@@ -5951,9 +6595,9 @@
         <f>IF(E24&gt;0, F24/E24, IF(F24&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L24" s="39" t="inlineStr">
-        <is>
-          <t>Sin Pedido</t>
+      <c r="L24" s="34" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -5965,16 +6609,16 @@
       </c>
       <c r="C25" s="32" t="inlineStr">
         <is>
-          <t>PT0020</t>
+          <t>FTK0005</t>
         </is>
       </c>
       <c r="D25" s="31" t="inlineStr">
         <is>
-          <t>AGROPOTASION, 20 L</t>
+          <t>FITOKONTROL CA FLOW, 5 KG</t>
         </is>
       </c>
       <c r="E25" s="19" t="n">
-        <v>2560</v>
+        <v>4400</v>
       </c>
       <c r="F25" s="19" t="n">
         <v>0</v>
@@ -5997,54 +6641,100 @@
         <f>IF(E25&gt;0, F25/E25, IF(F25&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L25" s="35" t="inlineStr">
+      <c r="L25" s="39" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="24" customHeight="1">
-      <c r="B26" s="21" t="inlineStr">
+    <row r="26">
+      <c r="B26" s="28" t="inlineStr">
+        <is>
+          <t>FITOXENT S.C.L.V.</t>
+        </is>
+      </c>
+      <c r="C26" s="29" t="inlineStr">
+        <is>
+          <t>PT0020</t>
+        </is>
+      </c>
+      <c r="D26" s="28" t="inlineStr">
+        <is>
+          <t>AGROPOTASION, 20 L</t>
+        </is>
+      </c>
+      <c r="E26" s="15" t="n">
+        <v>2560</v>
+      </c>
+      <c r="F26" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G26" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I26" s="15">
+        <f>MAX(0, E26-F26)</f>
+        <v/>
+      </c>
+      <c r="J26" s="15">
+        <f>ABS(F26-E26)</f>
+        <v/>
+      </c>
+      <c r="K26" s="16">
+        <f>IF(E26&gt;0, F26/E26, IF(F26&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L26" s="36" t="inlineStr">
+        <is>
+          <t>Sin Pedido</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="24" customHeight="1">
+      <c r="B27" s="21" t="inlineStr">
         <is>
           <t>TOTAL JAVIER</t>
         </is>
       </c>
-      <c r="C26" s="36" t="inlineStr">
-        <is>
-          <t>175 líneas</t>
-        </is>
-      </c>
-      <c r="D26" s="37" t="inlineStr"/>
-      <c r="E26" s="23">
-        <f>SUM(E10:E25)</f>
-        <v/>
-      </c>
-      <c r="F26" s="23">
-        <f>SUM(F10:F25)</f>
-        <v/>
-      </c>
-      <c r="G26" s="23">
-        <f>SUM(G10:G25)</f>
-        <v/>
-      </c>
-      <c r="H26" s="23">
-        <f>SUM(H10:H25)</f>
-        <v/>
-      </c>
-      <c r="I26" s="23">
-        <f>SUM(I10:I25)</f>
-        <v/>
-      </c>
-      <c r="J26" s="23">
-        <f>SUM(J10:J25)</f>
-        <v/>
-      </c>
-      <c r="K26" s="24">
-        <f>IF(E26&gt;0, F26/E26, 0)</f>
-        <v/>
-      </c>
-      <c r="L26" s="22">
-        <f>IF(K26&gt;=1, "SUPERADO", "EN CURSO")</f>
+      <c r="C27" s="37" t="inlineStr">
+        <is>
+          <t>176 líneas</t>
+        </is>
+      </c>
+      <c r="D27" s="38" t="inlineStr"/>
+      <c r="E27" s="23">
+        <f>SUM(E10:E26)</f>
+        <v/>
+      </c>
+      <c r="F27" s="23">
+        <f>SUM(F10:F26)</f>
+        <v/>
+      </c>
+      <c r="G27" s="23">
+        <f>SUM(G10:G26)</f>
+        <v/>
+      </c>
+      <c r="H27" s="23">
+        <f>SUM(H10:H26)</f>
+        <v/>
+      </c>
+      <c r="I27" s="23">
+        <f>SUM(I10:I26)</f>
+        <v/>
+      </c>
+      <c r="J27" s="23">
+        <f>SUM(J10:J26)</f>
+        <v/>
+      </c>
+      <c r="K27" s="24">
+        <f>IF(E27&gt;0, F27/E27, 0)</f>
+        <v/>
+      </c>
+      <c r="L27" s="22">
+        <f>IF(K27&gt;=1, "SUPERADO", "EN CURSO")</f>
         <v/>
       </c>
     </row>
@@ -6100,7 +6790,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 14/10/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 15/10/2026</t>
         </is>
       </c>
     </row>
@@ -6149,13 +6839,13 @@
         </is>
       </c>
       <c r="E6" s="4" t="n"/>
-      <c r="F6" s="26" t="inlineStr">
+      <c r="F6" s="40" t="inlineStr">
         <is>
           <t>0.0%</t>
         </is>
       </c>
       <c r="G6" s="4" t="n"/>
-      <c r="H6" s="26" t="inlineStr">
+      <c r="H6" s="40" t="inlineStr">
         <is>
           <t>39,460 u</t>
         </is>
@@ -6272,7 +6962,7 @@
         <f>IF(E10&gt;0, F10/E10, IF(F10&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L10" s="39" t="inlineStr">
+      <c r="L10" s="36" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -6318,7 +7008,7 @@
         <f>IF(E11&gt;0, F11/E11, IF(F11&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L11" s="35" t="inlineStr">
+      <c r="L11" s="39" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -6364,7 +7054,7 @@
         <f>IF(E12&gt;0, F12/E12, IF(F12&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L12" s="39" t="inlineStr">
+      <c r="L12" s="36" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -6410,7 +7100,7 @@
         <f>IF(E13&gt;0, F13/E13, IF(F13&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L13" s="35" t="inlineStr">
+      <c r="L13" s="39" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -6456,7 +7146,7 @@
         <f>IF(E14&gt;0, F14/E14, IF(F14&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L14" s="39" t="inlineStr">
+      <c r="L14" s="36" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -6502,7 +7192,7 @@
         <f>IF(E15&gt;0, F15/E15, IF(F15&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L15" s="35" t="inlineStr">
+      <c r="L15" s="39" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -6514,12 +7204,12 @@
           <t>TOTAL MEHMET</t>
         </is>
       </c>
-      <c r="C16" s="36" t="inlineStr">
+      <c r="C16" s="37" t="inlineStr">
         <is>
           <t>61 líneas</t>
         </is>
       </c>
-      <c r="D16" s="37" t="inlineStr"/>
+      <c r="D16" s="38" t="inlineStr"/>
       <c r="E16" s="23">
         <f>SUM(E10:E15)</f>
         <v/>
@@ -6578,7 +7268,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:L25"/>
+  <dimension ref="B2:L26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -6605,7 +7295,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 14/10/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 15/10/2026</t>
         </is>
       </c>
     </row>
@@ -6650,25 +7340,25 @@
       <c r="C6" s="4" t="n"/>
       <c r="D6" s="25" t="inlineStr">
         <is>
-          <t>6,880 u</t>
+          <t>7,880 u</t>
         </is>
       </c>
       <c r="E6" s="4" t="n"/>
-      <c r="F6" s="26" t="inlineStr">
-        <is>
-          <t>39.7%</t>
+      <c r="F6" s="40" t="inlineStr">
+        <is>
+          <t>45.4%</t>
         </is>
       </c>
       <c r="G6" s="4" t="n"/>
-      <c r="H6" s="26" t="inlineStr">
-        <is>
-          <t>10,460 u</t>
+      <c r="H6" s="40" t="inlineStr">
+        <is>
+          <t>9,460 u</t>
         </is>
       </c>
       <c r="I6" s="4" t="n"/>
       <c r="J6" s="25" t="inlineStr">
         <is>
-          <t>0 u</t>
+          <t>1,000 u</t>
         </is>
       </c>
       <c r="K6" s="4" t="n"/>
@@ -6823,7 +7513,7 @@
         <f>IF(E11&gt;0, F11/E11, IF(F11&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L11" s="35" t="inlineStr">
+      <c r="L11" s="39" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -6869,7 +7559,7 @@
         <f>IF(E12&gt;0, F12/E12, IF(F12&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L12" s="39" t="inlineStr">
+      <c r="L12" s="36" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -6915,7 +7605,7 @@
         <f>IF(E13&gt;0, F13/E13, IF(F13&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L13" s="35" t="inlineStr">
+      <c r="L13" s="39" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -7007,7 +7697,7 @@
         <f>IF(E15&gt;0, F15/E15, IF(F15&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L15" s="35" t="inlineStr">
+      <c r="L15" s="39" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -7053,7 +7743,7 @@
         <f>IF(E16&gt;0, F16/E16, IF(F16&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L16" s="39" t="inlineStr">
+      <c r="L16" s="36" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -7099,7 +7789,7 @@
         <f>IF(E17&gt;0, F17/E17, IF(F17&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L17" s="35" t="inlineStr">
+      <c r="L17" s="39" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -7191,7 +7881,7 @@
         <f>IF(E19&gt;0, F19/E19, IF(F19&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L19" s="40" t="inlineStr">
+      <c r="L19" s="35" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -7283,7 +7973,7 @@
         <f>IF(E21&gt;0, F21/E21, IF(F21&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L21" s="40" t="inlineStr">
+      <c r="L21" s="35" t="inlineStr">
         <is>
           <t>Superado</t>
         </is>
@@ -7329,7 +8019,7 @@
         <f>IF(E22&gt;0, F22/E22, IF(F22&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L22" s="39" t="inlineStr">
+      <c r="L22" s="36" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -7427,48 +8117,94 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="24" customHeight="1">
-      <c r="B25" s="21" t="inlineStr">
+    <row r="25">
+      <c r="B25" s="31" t="inlineStr">
+        <is>
+          <t>FITOMURCIA S.L.</t>
+        </is>
+      </c>
+      <c r="C25" s="32" t="inlineStr">
+        <is>
+          <t>BIO1000</t>
+        </is>
+      </c>
+      <c r="D25" s="31" t="inlineStr">
+        <is>
+          <t>BIORAD-20, 1000 L</t>
+        </is>
+      </c>
+      <c r="E25" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" s="19" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G25" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" s="19" t="n">
+        <v>1000</v>
+      </c>
+      <c r="I25" s="19">
+        <f>MAX(0, E25-F25)</f>
+        <v/>
+      </c>
+      <c r="J25" s="19">
+        <f>ABS(F25-E25)</f>
+        <v/>
+      </c>
+      <c r="K25" s="20">
+        <f>IF(E25&gt;0, F25/E25, IF(F25&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L25" s="35" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="24" customHeight="1">
+      <c r="B26" s="21" t="inlineStr">
         <is>
           <t>TOTAL PEDRO</t>
         </is>
       </c>
-      <c r="C25" s="36" t="inlineStr">
+      <c r="C26" s="37" t="inlineStr">
         <is>
           <t>104 líneas</t>
         </is>
       </c>
-      <c r="D25" s="37" t="inlineStr"/>
-      <c r="E25" s="23">
-        <f>SUM(E10:E24)</f>
-        <v/>
-      </c>
-      <c r="F25" s="23">
-        <f>SUM(F10:F24)</f>
-        <v/>
-      </c>
-      <c r="G25" s="23">
-        <f>SUM(G10:G24)</f>
-        <v/>
-      </c>
-      <c r="H25" s="23">
-        <f>SUM(H10:H24)</f>
-        <v/>
-      </c>
-      <c r="I25" s="23">
-        <f>SUM(I10:I24)</f>
-        <v/>
-      </c>
-      <c r="J25" s="23">
-        <f>SUM(J10:J24)</f>
-        <v/>
-      </c>
-      <c r="K25" s="24">
-        <f>IF(E25&gt;0, F25/E25, 0)</f>
-        <v/>
-      </c>
-      <c r="L25" s="22">
-        <f>IF(K25&gt;=1, "SUPERADO", "EN CURSO")</f>
+      <c r="D26" s="38" t="inlineStr"/>
+      <c r="E26" s="23">
+        <f>SUM(E10:E25)</f>
+        <v/>
+      </c>
+      <c r="F26" s="23">
+        <f>SUM(F10:F25)</f>
+        <v/>
+      </c>
+      <c r="G26" s="23">
+        <f>SUM(G10:G25)</f>
+        <v/>
+      </c>
+      <c r="H26" s="23">
+        <f>SUM(H10:H25)</f>
+        <v/>
+      </c>
+      <c r="I26" s="23">
+        <f>SUM(I10:I25)</f>
+        <v/>
+      </c>
+      <c r="J26" s="23">
+        <f>SUM(J10:J25)</f>
+        <v/>
+      </c>
+      <c r="K26" s="24">
+        <f>IF(E26&gt;0, F26/E26, 0)</f>
+        <v/>
+      </c>
+      <c r="L26" s="22">
+        <f>IF(K26&gt;=1, "SUPERADO", "EN CURSO")</f>
         <v/>
       </c>
     </row>
@@ -7524,7 +8260,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 14/10/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 15/10/2026</t>
         </is>
       </c>
     </row>
@@ -7573,13 +8309,13 @@
         </is>
       </c>
       <c r="E6" s="4" t="n"/>
-      <c r="F6" s="26" t="inlineStr">
+      <c r="F6" s="40" t="inlineStr">
         <is>
           <t>0.0%</t>
         </is>
       </c>
       <c r="G6" s="4" t="n"/>
-      <c r="H6" s="26" t="inlineStr">
+      <c r="H6" s="40" t="inlineStr">
         <is>
           <t>46,000 u</t>
         </is>
@@ -7696,7 +8432,7 @@
         <f>IF(E10&gt;0, F10/E10, IF(F10&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L10" s="39" t="inlineStr">
+      <c r="L10" s="36" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -7742,7 +8478,7 @@
         <f>IF(E11&gt;0, F11/E11, IF(F11&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L11" s="35" t="inlineStr">
+      <c r="L11" s="39" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -7754,12 +8490,12 @@
           <t>TOTAL RICARDO</t>
         </is>
       </c>
-      <c r="C12" s="36" t="inlineStr">
+      <c r="C12" s="37" t="inlineStr">
         <is>
           <t>115 líneas</t>
         </is>
       </c>
-      <c r="D12" s="37" t="inlineStr"/>
+      <c r="D12" s="38" t="inlineStr"/>
       <c r="E12" s="23">
         <f>SUM(E10:E11)</f>
         <v/>

</xml_diff>

<commit_message>
Actualizacion pedidos al 16/10/2026
</commit_message>
<xml_diff>
--- a/Seguimiento_Presupuesto_Sep_2026.xlsx
+++ b/Seguimiento_Presupuesto_Sep_2026.xlsx
@@ -918,7 +918,7 @@
     <row r="3" ht="20" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Comparativa Estimación Septiembre (Unidades) vs Pedidos Reales a Fecha 15/10/2026 | Generado: 15/10/2026 07:28</t>
+          <t>Comparativa Estimación Septiembre (Unidades) vs Pedidos Reales a Fecha 16/10/2026 | Generado: 16/10/2026 07:16</t>
         </is>
       </c>
     </row>
@@ -962,25 +962,25 @@
       <c r="C6" s="4" t="n"/>
       <c r="D6" s="8" t="inlineStr">
         <is>
-          <t>110,460 u</t>
+          <t>135,360 u</t>
         </is>
       </c>
       <c r="E6" s="4" t="n"/>
       <c r="F6" s="9" t="inlineStr">
         <is>
-          <t>60.7%</t>
+          <t>74.4%</t>
         </is>
       </c>
       <c r="G6" s="4" t="n"/>
       <c r="H6" s="10" t="inlineStr">
         <is>
-          <t>114,354 u</t>
+          <t>90,054 u</t>
         </is>
       </c>
       <c r="I6" s="4" t="n"/>
       <c r="J6" s="7" t="inlineStr">
         <is>
-          <t>81,300 u</t>
+          <t>97,816 u</t>
         </is>
       </c>
     </row>
@@ -1045,16 +1045,16 @@
         </is>
       </c>
       <c r="C10" s="14" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D10" s="15" t="n">
         <v>2320</v>
       </c>
       <c r="E10" s="15" t="n">
-        <v>2320</v>
+        <v>2924</v>
       </c>
       <c r="F10" s="15" t="n">
-        <v>2320</v>
+        <v>2924</v>
       </c>
       <c r="G10" s="15" t="n">
         <v>0</v>
@@ -1064,7 +1064,7 @@
         <v/>
       </c>
       <c r="I10" s="15">
-        <f>'Alfonso'!J15</f>
+        <f>'Alfonso'!J21</f>
         <v/>
       </c>
       <c r="J10" s="16">
@@ -1113,16 +1113,16 @@
         </is>
       </c>
       <c r="C12" s="14" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D12" s="15" t="n">
         <v>21914</v>
       </c>
       <c r="E12" s="15" t="n">
-        <v>11820</v>
+        <v>13320</v>
       </c>
       <c r="F12" s="15" t="n">
-        <v>11820</v>
+        <v>13320</v>
       </c>
       <c r="G12" s="15" t="n">
         <v>0</v>
@@ -1132,7 +1132,7 @@
         <v/>
       </c>
       <c r="I12" s="15">
-        <f>'Irene'!J48</f>
+        <f>'Irene'!J50</f>
         <v/>
       </c>
       <c r="J12" s="16">
@@ -1156,10 +1156,10 @@
         <v>7760</v>
       </c>
       <c r="F13" s="19" t="n">
-        <v>1460</v>
+        <v>6740</v>
       </c>
       <c r="G13" s="19" t="n">
-        <v>6300</v>
+        <v>1020</v>
       </c>
       <c r="H13" s="19">
         <f>MAX(0, D13-E13)</f>
@@ -1224,10 +1224,10 @@
         <v>7880</v>
       </c>
       <c r="F15" s="19" t="n">
-        <v>6880</v>
+        <v>7880</v>
       </c>
       <c r="G15" s="19" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="H15" s="19">
         <f>MAX(0, D15-E15)</f>
@@ -1249,26 +1249,26 @@
         </is>
       </c>
       <c r="C16" s="14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D16" s="15" t="n">
         <v>46000</v>
       </c>
       <c r="E16" s="15" t="n">
-        <v>0</v>
+        <v>22800</v>
       </c>
       <c r="F16" s="15" t="n">
         <v>0</v>
       </c>
       <c r="G16" s="15" t="n">
-        <v>0</v>
+        <v>22800</v>
       </c>
       <c r="H16" s="15">
         <f>MAX(0, D16-E16)</f>
         <v/>
       </c>
       <c r="I16" s="15">
-        <f>'Ricardo'!J12</f>
+        <f>'Ricardo'!J13</f>
         <v/>
       </c>
       <c r="J16" s="16">
@@ -1339,7 +1339,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:L15"/>
+  <dimension ref="B2:L21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1366,7 +1366,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 15/10/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 16/10/2026</t>
         </is>
       </c>
     </row>
@@ -1411,13 +1411,13 @@
       <c r="C6" s="4" t="n"/>
       <c r="D6" s="26" t="inlineStr">
         <is>
-          <t>2,320 u</t>
+          <t>2,924 u</t>
         </is>
       </c>
       <c r="E6" s="4" t="n"/>
       <c r="F6" s="26" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>126.0%</t>
         </is>
       </c>
       <c r="G6" s="4" t="n"/>
@@ -1728,48 +1728,324 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="24" customHeight="1">
-      <c r="B15" s="21" t="inlineStr">
+    <row r="15">
+      <c r="B15" s="31" t="inlineStr">
+        <is>
+          <t>VILLALTA SATIVUM, S.L.</t>
+        </is>
+      </c>
+      <c r="C15" s="32" t="inlineStr">
+        <is>
+          <t>AGXKAEP0020</t>
+        </is>
+      </c>
+      <c r="D15" s="31" t="inlineStr">
+        <is>
+          <t>BIOCULTURE POTASIO PLUS, 20 L</t>
+        </is>
+      </c>
+      <c r="E15" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="19" t="n">
+        <v>140</v>
+      </c>
+      <c r="G15" s="19" t="n">
+        <v>140</v>
+      </c>
+      <c r="H15" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" s="19">
+        <f>MAX(0, E15-F15)</f>
+        <v/>
+      </c>
+      <c r="J15" s="19">
+        <f>ABS(F15-E15)</f>
+        <v/>
+      </c>
+      <c r="K15" s="20">
+        <f>IF(E15&gt;0, F15/E15, IF(F15&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L15" s="35" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="28" t="inlineStr">
+        <is>
+          <t>VILLALTA SATIVUM, S.L.</t>
+        </is>
+      </c>
+      <c r="C16" s="29" t="inlineStr">
+        <is>
+          <t>AQUOM0020</t>
+        </is>
+      </c>
+      <c r="D16" s="28" t="inlineStr">
+        <is>
+          <t>AQUOM, 20 L</t>
+        </is>
+      </c>
+      <c r="E16" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="15" t="n">
+        <v>40</v>
+      </c>
+      <c r="G16" s="15" t="n">
+        <v>40</v>
+      </c>
+      <c r="H16" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" s="15">
+        <f>MAX(0, E16-F16)</f>
+        <v/>
+      </c>
+      <c r="J16" s="15">
+        <f>ABS(F16-E16)</f>
+        <v/>
+      </c>
+      <c r="K16" s="16">
+        <f>IF(E16&gt;0, F16/E16, IF(F16&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L16" s="34" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="31" t="inlineStr">
+        <is>
+          <t>VILLALTA SATIVUM, S.L.</t>
+        </is>
+      </c>
+      <c r="C17" s="32" t="inlineStr">
+        <is>
+          <t>C-CUAE0020</t>
+        </is>
+      </c>
+      <c r="D17" s="31" t="inlineStr">
+        <is>
+          <t>CUPRAMEC, 20 L</t>
+        </is>
+      </c>
+      <c r="E17" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="19" t="n">
+        <v>200</v>
+      </c>
+      <c r="G17" s="19" t="n">
+        <v>200</v>
+      </c>
+      <c r="H17" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" s="19">
+        <f>MAX(0, E17-F17)</f>
+        <v/>
+      </c>
+      <c r="J17" s="19">
+        <f>ABS(F17-E17)</f>
+        <v/>
+      </c>
+      <c r="K17" s="20">
+        <f>IF(E17&gt;0, F17/E17, IF(F17&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L17" s="35" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="28" t="inlineStr">
+        <is>
+          <t>VILLALTA SATIVUM, S.L.</t>
+        </is>
+      </c>
+      <c r="C18" s="29" t="inlineStr">
+        <is>
+          <t>PT0001</t>
+        </is>
+      </c>
+      <c r="D18" s="28" t="inlineStr">
+        <is>
+          <t>AGROPOTASION, 1 L</t>
+        </is>
+      </c>
+      <c r="E18" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" s="15" t="n">
+        <v>24</v>
+      </c>
+      <c r="G18" s="15" t="n">
+        <v>24</v>
+      </c>
+      <c r="H18" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" s="15">
+        <f>MAX(0, E18-F18)</f>
+        <v/>
+      </c>
+      <c r="J18" s="15">
+        <f>ABS(F18-E18)</f>
+        <v/>
+      </c>
+      <c r="K18" s="16">
+        <f>IF(E18&gt;0, F18/E18, IF(F18&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L18" s="34" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="31" t="inlineStr">
+        <is>
+          <t>VILLALTA SATIVUM, S.L.</t>
+        </is>
+      </c>
+      <c r="C19" s="32" t="inlineStr">
+        <is>
+          <t>PT0005</t>
+        </is>
+      </c>
+      <c r="D19" s="31" t="inlineStr">
+        <is>
+          <t>AGROPOTASION, 5 L</t>
+        </is>
+      </c>
+      <c r="E19" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" s="19" t="n">
+        <v>100</v>
+      </c>
+      <c r="G19" s="19" t="n">
+        <v>100</v>
+      </c>
+      <c r="H19" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I19" s="19">
+        <f>MAX(0, E19-F19)</f>
+        <v/>
+      </c>
+      <c r="J19" s="19">
+        <f>ABS(F19-E19)</f>
+        <v/>
+      </c>
+      <c r="K19" s="20">
+        <f>IF(E19&gt;0, F19/E19, IF(F19&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L19" s="35" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="28" t="inlineStr">
+        <is>
+          <t>VILLALTA SATIVUM, S.L.</t>
+        </is>
+      </c>
+      <c r="C20" s="29" t="inlineStr">
+        <is>
+          <t>PT0020</t>
+        </is>
+      </c>
+      <c r="D20" s="28" t="inlineStr">
+        <is>
+          <t>AGROPOTASION, 20 L</t>
+        </is>
+      </c>
+      <c r="E20" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" s="15" t="n">
+        <v>100</v>
+      </c>
+      <c r="G20" s="15" t="n">
+        <v>100</v>
+      </c>
+      <c r="H20" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I20" s="15">
+        <f>MAX(0, E20-F20)</f>
+        <v/>
+      </c>
+      <c r="J20" s="15">
+        <f>ABS(F20-E20)</f>
+        <v/>
+      </c>
+      <c r="K20" s="16">
+        <f>IF(E20&gt;0, F20/E20, IF(F20&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L20" s="34" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="24" customHeight="1">
+      <c r="B21" s="21" t="inlineStr">
         <is>
           <t>TOTAL ALFONSO</t>
         </is>
       </c>
-      <c r="C15" s="37" t="inlineStr">
-        <is>
-          <t>276 líneas</t>
-        </is>
-      </c>
-      <c r="D15" s="38" t="inlineStr"/>
-      <c r="E15" s="23">
-        <f>SUM(E10:E14)</f>
-        <v/>
-      </c>
-      <c r="F15" s="23">
-        <f>SUM(F10:F14)</f>
-        <v/>
-      </c>
-      <c r="G15" s="23">
-        <f>SUM(G10:G14)</f>
-        <v/>
-      </c>
-      <c r="H15" s="23">
-        <f>SUM(H10:H14)</f>
-        <v/>
-      </c>
-      <c r="I15" s="23">
-        <f>SUM(I10:I14)</f>
-        <v/>
-      </c>
-      <c r="J15" s="23">
-        <f>SUM(J10:J14)</f>
-        <v/>
-      </c>
-      <c r="K15" s="24">
-        <f>IF(E15&gt;0, F15/E15, 0)</f>
-        <v/>
-      </c>
-      <c r="L15" s="22">
-        <f>IF(K15&gt;=1, "SUPERADO", "EN CURSO")</f>
+      <c r="C21" s="37" t="inlineStr">
+        <is>
+          <t>279 líneas</t>
+        </is>
+      </c>
+      <c r="D21" s="38" t="inlineStr"/>
+      <c r="E21" s="23">
+        <f>SUM(E10:E20)</f>
+        <v/>
+      </c>
+      <c r="F21" s="23">
+        <f>SUM(F10:F20)</f>
+        <v/>
+      </c>
+      <c r="G21" s="23">
+        <f>SUM(G10:G20)</f>
+        <v/>
+      </c>
+      <c r="H21" s="23">
+        <f>SUM(H10:H20)</f>
+        <v/>
+      </c>
+      <c r="I21" s="23">
+        <f>SUM(I10:I20)</f>
+        <v/>
+      </c>
+      <c r="J21" s="23">
+        <f>SUM(J10:J20)</f>
+        <v/>
+      </c>
+      <c r="K21" s="24">
+        <f>IF(E21&gt;0, F21/E21, 0)</f>
+        <v/>
+      </c>
+      <c r="L21" s="22">
+        <f>IF(K21&gt;=1, "SUPERADO", "EN CURSO")</f>
         <v/>
       </c>
     </row>
@@ -1825,7 +2101,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 15/10/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 16/10/2026</t>
         </is>
       </c>
     </row>
@@ -2655,12 +2931,12 @@
       </c>
       <c r="C25" s="32" t="inlineStr">
         <is>
-          <t>SPAR0001</t>
+          <t>SPCE2B0001</t>
         </is>
       </c>
       <c r="D25" s="31" t="inlineStr">
         <is>
-          <t>SPRINTENE ARABIA, 1 L</t>
+          <t>NEW SPRINTENE</t>
         </is>
       </c>
       <c r="E25" s="19" t="n">
@@ -3299,12 +3575,12 @@
       </c>
       <c r="C39" s="32" t="inlineStr">
         <is>
-          <t>AGXCR0020</t>
+          <t>AGXK0020</t>
         </is>
       </c>
       <c r="D39" s="31" t="inlineStr">
         <is>
-          <t>GREEN MAX</t>
+          <t>AGROXILATO-K</t>
         </is>
       </c>
       <c r="E39" s="19" t="n">
@@ -3437,12 +3713,12 @@
       </c>
       <c r="C42" s="29" t="inlineStr">
         <is>
-          <t>C-CU20005</t>
+          <t>C-CU0005</t>
         </is>
       </c>
       <c r="D42" s="28" t="inlineStr">
         <is>
-          <t>CODICOBRE (EGIPTO), 5 L</t>
+          <t>CODICOBRE</t>
         </is>
       </c>
       <c r="E42" s="15" t="n">
@@ -3713,7 +3989,7 @@
       </c>
       <c r="C48" s="37" t="inlineStr">
         <is>
-          <t>236 líneas</t>
+          <t>234 líneas</t>
         </is>
       </c>
       <c r="D48" s="38" t="inlineStr"/>
@@ -3775,7 +4051,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:L48"/>
+  <dimension ref="B2:L50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -3802,7 +4078,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 15/10/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 16/10/2026</t>
         </is>
       </c>
     </row>
@@ -3847,19 +4123,19 @@
       <c r="C6" s="4" t="n"/>
       <c r="D6" s="25" t="inlineStr">
         <is>
-          <t>11,820 u</t>
+          <t>13,320 u</t>
         </is>
       </c>
       <c r="E6" s="4" t="n"/>
       <c r="F6" s="40" t="inlineStr">
         <is>
-          <t>53.9%</t>
+          <t>60.8%</t>
         </is>
       </c>
       <c r="G6" s="4" t="n"/>
       <c r="H6" s="40" t="inlineStr">
         <is>
-          <t>10,094 u</t>
+          <t>8,594 u</t>
         </is>
       </c>
       <c r="I6" s="4" t="n"/>
@@ -5242,10 +5518,10 @@
         <v>1240</v>
       </c>
       <c r="F38" s="15" t="n">
-        <v>0</v>
+        <v>640</v>
       </c>
       <c r="G38" s="15" t="n">
-        <v>0</v>
+        <v>640</v>
       </c>
       <c r="H38" s="15" t="n">
         <v>0</v>
@@ -5262,9 +5538,9 @@
         <f>IF(E38&gt;0, F38/E38, IF(F38&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L38" s="36" t="inlineStr">
-        <is>
-          <t>Sin Pedido</t>
+      <c r="L38" s="30" t="inlineStr">
+        <is>
+          <t>En Curso</t>
         </is>
       </c>
     </row>
@@ -5460,22 +5736,22 @@
       </c>
       <c r="C43" s="32" t="inlineStr">
         <is>
-          <t>BEY0020</t>
+          <t>BEY0005</t>
         </is>
       </c>
       <c r="D43" s="31" t="inlineStr">
         <is>
-          <t>FLORAMEC PLUS 20 L</t>
+          <t>FLORAMEC PLUS, 5 L</t>
         </is>
       </c>
       <c r="E43" s="19" t="n">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="F43" s="19" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="G43" s="19" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="H43" s="19" t="n">
         <v>0</v>
@@ -5492,9 +5768,9 @@
         <f>IF(E43&gt;0, F43/E43, IF(F43&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L43" s="39" t="inlineStr">
-        <is>
-          <t>Sin Pedido</t>
+      <c r="L43" s="35" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -5506,22 +5782,22 @@
       </c>
       <c r="C44" s="29" t="inlineStr">
         <is>
-          <t>BROTA0005</t>
+          <t>BEY0020</t>
         </is>
       </c>
       <c r="D44" s="28" t="inlineStr">
         <is>
-          <t>BROTAMEC, 5 L</t>
+          <t>FLORAMEC PLUS 20 L</t>
         </is>
       </c>
       <c r="E44" s="15" t="n">
-        <v>600</v>
+        <v>80</v>
       </c>
       <c r="F44" s="15" t="n">
-        <v>600</v>
+        <v>120</v>
       </c>
       <c r="G44" s="15" t="n">
-        <v>600</v>
+        <v>120</v>
       </c>
       <c r="H44" s="15" t="n">
         <v>0</v>
@@ -5552,22 +5828,22 @@
       </c>
       <c r="C45" s="32" t="inlineStr">
         <is>
-          <t>C-M-P0001</t>
+          <t>BROTA0005</t>
         </is>
       </c>
       <c r="D45" s="31" t="inlineStr">
         <is>
-          <t>CODIFOL Mo-PLUS, 1 L</t>
+          <t>BROTAMEC, 5 L</t>
         </is>
       </c>
       <c r="E45" s="19" t="n">
-        <v>36</v>
+        <v>600</v>
       </c>
       <c r="F45" s="19" t="n">
-        <v>0</v>
+        <v>600</v>
       </c>
       <c r="G45" s="19" t="n">
-        <v>0</v>
+        <v>600</v>
       </c>
       <c r="H45" s="19" t="n">
         <v>0</v>
@@ -5584,9 +5860,9 @@
         <f>IF(E45&gt;0, F45/E45, IF(F45&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L45" s="39" t="inlineStr">
-        <is>
-          <t>Sin Pedido</t>
+      <c r="L45" s="35" t="inlineStr">
+        <is>
+          <t>Superado</t>
         </is>
       </c>
     </row>
@@ -5598,16 +5874,16 @@
       </c>
       <c r="C46" s="29" t="inlineStr">
         <is>
-          <t>FTK0005</t>
+          <t>C-M-P0001</t>
         </is>
       </c>
       <c r="D46" s="28" t="inlineStr">
         <is>
-          <t>FITOKONTROL CA FLOW, 5 KG</t>
+          <t>CODIFOL Mo-PLUS, 1 L</t>
         </is>
       </c>
       <c r="E46" s="15" t="n">
-        <v>800</v>
+        <v>36</v>
       </c>
       <c r="F46" s="15" t="n">
         <v>0</v>
@@ -5644,22 +5920,22 @@
       </c>
       <c r="C47" s="32" t="inlineStr">
         <is>
-          <t>TRI0005</t>
+          <t>FTK0005</t>
         </is>
       </c>
       <c r="D47" s="31" t="inlineStr">
         <is>
-          <t>TRIFENO-94, 5L</t>
+          <t>FITOKONTROL CA FLOW, 5 KG</t>
         </is>
       </c>
       <c r="E47" s="19" t="n">
-        <v>0</v>
+        <v>800</v>
       </c>
       <c r="F47" s="19" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="G47" s="19" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="H47" s="19" t="n">
         <v>0</v>
@@ -5676,54 +5952,146 @@
         <f>IF(E47&gt;0, F47/E47, IF(F47&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L47" s="35" t="inlineStr">
+      <c r="L47" s="39" t="inlineStr">
+        <is>
+          <t>Sin Pedido</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="B48" s="28" t="inlineStr">
+        <is>
+          <t>GUIVARTO AGRICOLA, S.L.</t>
+        </is>
+      </c>
+      <c r="C48" s="29" t="inlineStr">
+        <is>
+          <t>TRI0005</t>
+        </is>
+      </c>
+      <c r="D48" s="28" t="inlineStr">
+        <is>
+          <t>TRIFENO-94, 5L</t>
+        </is>
+      </c>
+      <c r="E48" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F48" s="15" t="n">
+        <v>300</v>
+      </c>
+      <c r="G48" s="15" t="n">
+        <v>300</v>
+      </c>
+      <c r="H48" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I48" s="15">
+        <f>MAX(0, E48-F48)</f>
+        <v/>
+      </c>
+      <c r="J48" s="15">
+        <f>ABS(F48-E48)</f>
+        <v/>
+      </c>
+      <c r="K48" s="16">
+        <f>IF(E48&gt;0, F48/E48, IF(F48&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L48" s="34" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
       </c>
     </row>
-    <row r="48" ht="24" customHeight="1">
-      <c r="B48" s="21" t="inlineStr">
+    <row r="49">
+      <c r="B49" s="31" t="inlineStr">
+        <is>
+          <t>SUCA, S.C.A.</t>
+        </is>
+      </c>
+      <c r="C49" s="32" t="inlineStr">
+        <is>
+          <t>AGXK0020</t>
+        </is>
+      </c>
+      <c r="D49" s="31" t="inlineStr">
+        <is>
+          <t>AGROXILATO-K, 20 L</t>
+        </is>
+      </c>
+      <c r="E49" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F49" s="19" t="n">
+        <v>640</v>
+      </c>
+      <c r="G49" s="19" t="n">
+        <v>640</v>
+      </c>
+      <c r="H49" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I49" s="19">
+        <f>MAX(0, E49-F49)</f>
+        <v/>
+      </c>
+      <c r="J49" s="19">
+        <f>ABS(F49-E49)</f>
+        <v/>
+      </c>
+      <c r="K49" s="20">
+        <f>IF(E49&gt;0, F49/E49, IF(F49&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L49" s="35" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="24" customHeight="1">
+      <c r="B50" s="21" t="inlineStr">
         <is>
           <t>TOTAL IRENE</t>
         </is>
       </c>
-      <c r="C48" s="37" t="inlineStr">
+      <c r="C50" s="37" t="inlineStr">
         <is>
           <t>89 líneas</t>
         </is>
       </c>
-      <c r="D48" s="38" t="inlineStr"/>
-      <c r="E48" s="23">
-        <f>SUM(E10:E47)</f>
-        <v/>
-      </c>
-      <c r="F48" s="23">
-        <f>SUM(F10:F47)</f>
-        <v/>
-      </c>
-      <c r="G48" s="23">
-        <f>SUM(G10:G47)</f>
-        <v/>
-      </c>
-      <c r="H48" s="23">
-        <f>SUM(H10:H47)</f>
-        <v/>
-      </c>
-      <c r="I48" s="23">
-        <f>SUM(I10:I47)</f>
-        <v/>
-      </c>
-      <c r="J48" s="23">
-        <f>SUM(J10:J47)</f>
-        <v/>
-      </c>
-      <c r="K48" s="24">
-        <f>IF(E48&gt;0, F48/E48, 0)</f>
-        <v/>
-      </c>
-      <c r="L48" s="22">
-        <f>IF(K48&gt;=1, "SUPERADO", "EN CURSO")</f>
+      <c r="D50" s="38" t="inlineStr"/>
+      <c r="E50" s="23">
+        <f>SUM(E10:E49)</f>
+        <v/>
+      </c>
+      <c r="F50" s="23">
+        <f>SUM(F10:F49)</f>
+        <v/>
+      </c>
+      <c r="G50" s="23">
+        <f>SUM(G10:G49)</f>
+        <v/>
+      </c>
+      <c r="H50" s="23">
+        <f>SUM(H10:H49)</f>
+        <v/>
+      </c>
+      <c r="I50" s="23">
+        <f>SUM(I10:I49)</f>
+        <v/>
+      </c>
+      <c r="J50" s="23">
+        <f>SUM(J10:J49)</f>
+        <v/>
+      </c>
+      <c r="K50" s="24">
+        <f>IF(E50&gt;0, F50/E50, 0)</f>
+        <v/>
+      </c>
+      <c r="L50" s="22">
+        <f>IF(K50&gt;=1, "SUPERADO", "EN CURSO")</f>
         <v/>
       </c>
     </row>
@@ -5779,7 +6147,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 15/10/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 16/10/2026</t>
         </is>
       </c>
     </row>
@@ -5842,7 +6210,7 @@
       <c r="I6" s="4" t="n"/>
       <c r="J6" s="25" t="inlineStr">
         <is>
-          <t>6,300 u</t>
+          <t>1,020 u</t>
         </is>
       </c>
       <c r="K6" s="4" t="n"/>
@@ -5934,10 +6302,10 @@
         <v>20</v>
       </c>
       <c r="G10" s="15" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="H10" s="15" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="I10" s="15">
         <f>MAX(0, E10-F10)</f>
@@ -5980,10 +6348,10 @@
         <v>640</v>
       </c>
       <c r="G11" s="19" t="n">
-        <v>0</v>
+        <v>640</v>
       </c>
       <c r="H11" s="19" t="n">
-        <v>640</v>
+        <v>0</v>
       </c>
       <c r="I11" s="19">
         <f>MAX(0, E11-F11)</f>
@@ -6026,10 +6394,10 @@
         <v>2400</v>
       </c>
       <c r="G12" s="15" t="n">
-        <v>0</v>
+        <v>2400</v>
       </c>
       <c r="H12" s="15" t="n">
-        <v>2400</v>
+        <v>0</v>
       </c>
       <c r="I12" s="15">
         <f>MAX(0, E12-F12)</f>
@@ -6072,10 +6440,10 @@
         <v>1100</v>
       </c>
       <c r="G13" s="19" t="n">
-        <v>0</v>
+        <v>1100</v>
       </c>
       <c r="H13" s="19" t="n">
-        <v>1100</v>
+        <v>0</v>
       </c>
       <c r="I13" s="19">
         <f>MAX(0, E13-F13)</f>
@@ -6118,10 +6486,10 @@
         <v>100</v>
       </c>
       <c r="G14" s="15" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="H14" s="15" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="I14" s="15">
         <f>MAX(0, E14-F14)</f>
@@ -6164,10 +6532,10 @@
         <v>40</v>
       </c>
       <c r="G15" s="19" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="H15" s="19" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="I15" s="19">
         <f>MAX(0, E15-F15)</f>
@@ -6532,10 +6900,10 @@
         <v>1000</v>
       </c>
       <c r="G23" s="19" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="H23" s="19" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="I23" s="19">
         <f>MAX(0, E23-F23)</f>
@@ -6790,7 +7158,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 15/10/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 16/10/2026</t>
         </is>
       </c>
     </row>
@@ -7295,7 +7663,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 15/10/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 16/10/2026</t>
         </is>
       </c>
     </row>
@@ -7358,7 +7726,7 @@
       <c r="I6" s="4" t="n"/>
       <c r="J6" s="25" t="inlineStr">
         <is>
-          <t>1,000 u</t>
+          <t>0 u</t>
         </is>
       </c>
       <c r="K6" s="4" t="n"/>
@@ -8140,10 +8508,10 @@
         <v>1000</v>
       </c>
       <c r="G25" s="19" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="H25" s="19" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="I25" s="19">
         <f>MAX(0, E25-F25)</f>
@@ -8233,7 +8601,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:L12"/>
+  <dimension ref="B2:L13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -8260,7 +8628,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 15/10/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 16/10/2026</t>
         </is>
       </c>
     </row>
@@ -8305,25 +8673,25 @@
       <c r="C6" s="4" t="n"/>
       <c r="D6" s="25" t="inlineStr">
         <is>
-          <t>0 u</t>
+          <t>22,800 u</t>
         </is>
       </c>
       <c r="E6" s="4" t="n"/>
       <c r="F6" s="40" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>49.6%</t>
         </is>
       </c>
       <c r="G6" s="4" t="n"/>
       <c r="H6" s="40" t="inlineStr">
         <is>
-          <t>46,000 u</t>
+          <t>23,200 u</t>
         </is>
       </c>
       <c r="I6" s="4" t="n"/>
       <c r="J6" s="25" t="inlineStr">
         <is>
-          <t>0 u</t>
+          <t>22,800 u</t>
         </is>
       </c>
       <c r="K6" s="4" t="n"/>
@@ -8458,13 +8826,13 @@
         <v>44000</v>
       </c>
       <c r="F11" s="19" t="n">
-        <v>0</v>
+        <v>19800</v>
       </c>
       <c r="G11" s="19" t="n">
         <v>0</v>
       </c>
       <c r="H11" s="19" t="n">
-        <v>0</v>
+        <v>19800</v>
       </c>
       <c r="I11" s="19">
         <f>MAX(0, E11-F11)</f>
@@ -8478,54 +8846,100 @@
         <f>IF(E11&gt;0, F11/E11, IF(F11&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L11" s="39" t="inlineStr">
-        <is>
-          <t>Sin Pedido</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="24" customHeight="1">
-      <c r="B12" s="21" t="inlineStr">
+      <c r="L11" s="41" t="inlineStr">
+        <is>
+          <t>Rezagado</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="28" t="inlineStr">
+        <is>
+          <t>LEKKERBIO B.V.</t>
+        </is>
+      </c>
+      <c r="C12" s="29" t="inlineStr">
+        <is>
+          <t>DECA0020</t>
+        </is>
+      </c>
+      <c r="D12" s="28" t="inlineStr">
+        <is>
+          <t>DEFENS-CA-AE, 20 KG</t>
+        </is>
+      </c>
+      <c r="E12" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="15" t="n">
+        <v>3000</v>
+      </c>
+      <c r="G12" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="15" t="n">
+        <v>3000</v>
+      </c>
+      <c r="I12" s="15">
+        <f>MAX(0, E12-F12)</f>
+        <v/>
+      </c>
+      <c r="J12" s="15">
+        <f>ABS(F12-E12)</f>
+        <v/>
+      </c>
+      <c r="K12" s="16">
+        <f>IF(E12&gt;0, F12/E12, IF(F12&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L12" s="34" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="24" customHeight="1">
+      <c r="B13" s="21" t="inlineStr">
         <is>
           <t>TOTAL RICARDO</t>
         </is>
       </c>
-      <c r="C12" s="37" t="inlineStr">
-        <is>
-          <t>115 líneas</t>
-        </is>
-      </c>
-      <c r="D12" s="38" t="inlineStr"/>
-      <c r="E12" s="23">
-        <f>SUM(E10:E11)</f>
-        <v/>
-      </c>
-      <c r="F12" s="23">
-        <f>SUM(F10:F11)</f>
-        <v/>
-      </c>
-      <c r="G12" s="23">
-        <f>SUM(G10:G11)</f>
-        <v/>
-      </c>
-      <c r="H12" s="23">
-        <f>SUM(H10:H11)</f>
-        <v/>
-      </c>
-      <c r="I12" s="23">
-        <f>SUM(I10:I11)</f>
-        <v/>
-      </c>
-      <c r="J12" s="23">
-        <f>SUM(J10:J11)</f>
-        <v/>
-      </c>
-      <c r="K12" s="24">
-        <f>IF(E12&gt;0, F12/E12, 0)</f>
-        <v/>
-      </c>
-      <c r="L12" s="22">
-        <f>IF(K12&gt;=1, "SUPERADO", "EN CURSO")</f>
+      <c r="C13" s="37" t="inlineStr">
+        <is>
+          <t>116 líneas</t>
+        </is>
+      </c>
+      <c r="D13" s="38" t="inlineStr"/>
+      <c r="E13" s="23">
+        <f>SUM(E10:E12)</f>
+        <v/>
+      </c>
+      <c r="F13" s="23">
+        <f>SUM(F10:F12)</f>
+        <v/>
+      </c>
+      <c r="G13" s="23">
+        <f>SUM(G10:G12)</f>
+        <v/>
+      </c>
+      <c r="H13" s="23">
+        <f>SUM(H10:H12)</f>
+        <v/>
+      </c>
+      <c r="I13" s="23">
+        <f>SUM(I10:I12)</f>
+        <v/>
+      </c>
+      <c r="J13" s="23">
+        <f>SUM(J10:J12)</f>
+        <v/>
+      </c>
+      <c r="K13" s="24">
+        <f>IF(E13&gt;0, F13/E13, 0)</f>
+        <v/>
+      </c>
+      <c r="L13" s="22">
+        <f>IF(K13&gt;=1, "SUPERADO", "EN CURSO")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizacion pedidos al 21.10.2026 y sincronizacion de dashboards
</commit_message>
<xml_diff>
--- a/Seguimiento_Presupuesto_Sep_2026.xlsx
+++ b/Seguimiento_Presupuesto_Sep_2026.xlsx
@@ -918,7 +918,7 @@
     <row r="3" ht="20" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Comparativa Estimación Septiembre (Unidades) vs Pedidos Reales a Fecha 20/10/2026 | Generado: 20/10/2026 08:14</t>
+          <t>Comparativa Estimación Septiembre (Unidades) vs Pedidos Reales a Fecha 21/10/2026 | Generado: 21/10/2026 08:20</t>
         </is>
       </c>
     </row>
@@ -962,19 +962,19 @@
       <c r="C6" s="4" t="n"/>
       <c r="D6" s="8" t="inlineStr">
         <is>
-          <t>144,765 u</t>
+          <t>152,805 u</t>
         </is>
       </c>
       <c r="E6" s="4" t="n"/>
       <c r="F6" s="9" t="inlineStr">
         <is>
-          <t>79.6%</t>
+          <t>84.0%</t>
         </is>
       </c>
       <c r="G6" s="4" t="n"/>
       <c r="H6" s="10" t="inlineStr">
         <is>
-          <t>80,649 u</t>
+          <t>72,669 u</t>
         </is>
       </c>
       <c r="I6" s="4" t="n"/>
@@ -1153,10 +1153,10 @@
         <v>17100</v>
       </c>
       <c r="E13" s="19" t="n">
-        <v>12960</v>
+        <v>13560</v>
       </c>
       <c r="F13" s="19" t="n">
-        <v>11940</v>
+        <v>12540</v>
       </c>
       <c r="G13" s="19" t="n">
         <v>1020</v>
@@ -1166,7 +1166,7 @@
         <v/>
       </c>
       <c r="I13" s="19">
-        <f>'Javier'!J30</f>
+        <f>'Javier'!J33</f>
         <v/>
       </c>
       <c r="J13" s="20">
@@ -1221,10 +1221,10 @@
         <v>17340</v>
       </c>
       <c r="E15" s="19" t="n">
-        <v>9960</v>
+        <v>17400</v>
       </c>
       <c r="F15" s="19" t="n">
-        <v>9960</v>
+        <v>17400</v>
       </c>
       <c r="G15" s="19" t="n">
         <v>0</v>
@@ -1234,7 +1234,7 @@
         <v/>
       </c>
       <c r="I15" s="19">
-        <f>'Pedro'!J26</f>
+        <f>'Pedro'!J27</f>
         <v/>
       </c>
       <c r="J15" s="20">
@@ -1366,7 +1366,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 20/10/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 21/10/2026</t>
         </is>
       </c>
     </row>
@@ -2101,7 +2101,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 20/10/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 21/10/2026</t>
         </is>
       </c>
     </row>
@@ -4078,7 +4078,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 20/10/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 21/10/2026</t>
         </is>
       </c>
     </row>
@@ -6120,7 +6120,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:L30"/>
+  <dimension ref="B2:L33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -6147,7 +6147,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 20/10/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 21/10/2026</t>
         </is>
       </c>
     </row>
@@ -6192,19 +6192,19 @@
       <c r="C6" s="4" t="n"/>
       <c r="D6" s="25" t="inlineStr">
         <is>
-          <t>12,960 u</t>
+          <t>13,560 u</t>
         </is>
       </c>
       <c r="E6" s="4" t="n"/>
       <c r="F6" s="40" t="inlineStr">
         <is>
-          <t>75.8%</t>
+          <t>79.3%</t>
         </is>
       </c>
       <c r="G6" s="4" t="n"/>
       <c r="H6" s="40" t="inlineStr">
         <is>
-          <t>4,140 u</t>
+          <t>3,540 u</t>
         </is>
       </c>
       <c r="I6" s="4" t="n"/>
@@ -7069,22 +7069,22 @@
       </c>
       <c r="C27" s="32" t="inlineStr">
         <is>
-          <t>PT0020</t>
+          <t>BIO0020</t>
         </is>
       </c>
       <c r="D27" s="31" t="inlineStr">
         <is>
-          <t>AGROPOTASION, 20 L</t>
+          <t>BIORAD-20, 20 L</t>
         </is>
       </c>
       <c r="E27" s="19" t="n">
         <v>0</v>
       </c>
       <c r="F27" s="19" t="n">
-        <v>640</v>
+        <v>200</v>
       </c>
       <c r="G27" s="19" t="n">
-        <v>640</v>
+        <v>200</v>
       </c>
       <c r="H27" s="19" t="n">
         <v>0</v>
@@ -7110,27 +7110,27 @@
     <row r="28">
       <c r="B28" s="28" t="inlineStr">
         <is>
-          <t>FITOXENT S.C.L.V.</t>
+          <t>FITOSANITARIOS CARCAIXENT, S.L.</t>
         </is>
       </c>
       <c r="C28" s="29" t="inlineStr">
         <is>
-          <t>FTK0005</t>
+          <t>BR-590005</t>
         </is>
       </c>
       <c r="D28" s="28" t="inlineStr">
         <is>
-          <t>FITOKONTROL CA FLOW, 5 KG</t>
+          <t>BR-59, 5 KG</t>
         </is>
       </c>
       <c r="E28" s="15" t="n">
-        <v>4400</v>
+        <v>0</v>
       </c>
       <c r="F28" s="15" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="G28" s="15" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="H28" s="15" t="n">
         <v>0</v>
@@ -7147,36 +7147,36 @@
         <f>IF(E28&gt;0, F28/E28, IF(F28&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L28" s="36" t="inlineStr">
-        <is>
-          <t>Sin Pedido</t>
+      <c r="L28" s="34" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="B29" s="31" t="inlineStr">
         <is>
-          <t>FITOXENT S.C.L.V.</t>
+          <t>FITOSANITARIOS CARCAIXENT, S.L.</t>
         </is>
       </c>
       <c r="C29" s="32" t="inlineStr">
         <is>
-          <t>PT0020</t>
+          <t>FTK0005</t>
         </is>
       </c>
       <c r="D29" s="31" t="inlineStr">
         <is>
-          <t>AGROPOTASION, 20 L</t>
+          <t>FITOKONTROL CA FLOW, 5 KG</t>
         </is>
       </c>
       <c r="E29" s="19" t="n">
-        <v>2560</v>
+        <v>0</v>
       </c>
       <c r="F29" s="19" t="n">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="G29" s="19" t="n">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="H29" s="19" t="n">
         <v>0</v>
@@ -7193,54 +7193,192 @@
         <f>IF(E29&gt;0, F29/E29, IF(F29&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L29" s="39" t="inlineStr">
+      <c r="L29" s="35" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="28" t="inlineStr">
+        <is>
+          <t>FITOSANITARIOS CARCAIXENT, S.L.</t>
+        </is>
+      </c>
+      <c r="C30" s="29" t="inlineStr">
+        <is>
+          <t>PT0020</t>
+        </is>
+      </c>
+      <c r="D30" s="28" t="inlineStr">
+        <is>
+          <t>AGROPOTASION, 20 L</t>
+        </is>
+      </c>
+      <c r="E30" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" s="15" t="n">
+        <v>740</v>
+      </c>
+      <c r="G30" s="15" t="n">
+        <v>740</v>
+      </c>
+      <c r="H30" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I30" s="15">
+        <f>MAX(0, E30-F30)</f>
+        <v/>
+      </c>
+      <c r="J30" s="15">
+        <f>ABS(F30-E30)</f>
+        <v/>
+      </c>
+      <c r="K30" s="16">
+        <f>IF(E30&gt;0, F30/E30, IF(F30&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L30" s="34" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="31" t="inlineStr">
+        <is>
+          <t>FITOXENT S.C.L.V.</t>
+        </is>
+      </c>
+      <c r="C31" s="32" t="inlineStr">
+        <is>
+          <t>FTK0005</t>
+        </is>
+      </c>
+      <c r="D31" s="31" t="inlineStr">
+        <is>
+          <t>FITOKONTROL CA FLOW, 5 KG</t>
+        </is>
+      </c>
+      <c r="E31" s="19" t="n">
+        <v>4400</v>
+      </c>
+      <c r="F31" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H31" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I31" s="19">
+        <f>MAX(0, E31-F31)</f>
+        <v/>
+      </c>
+      <c r="J31" s="19">
+        <f>ABS(F31-E31)</f>
+        <v/>
+      </c>
+      <c r="K31" s="20">
+        <f>IF(E31&gt;0, F31/E31, IF(F31&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L31" s="39" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="24" customHeight="1">
-      <c r="B30" s="21" t="inlineStr">
+    <row r="32">
+      <c r="B32" s="28" t="inlineStr">
+        <is>
+          <t>FITOXENT S.C.L.V.</t>
+        </is>
+      </c>
+      <c r="C32" s="29" t="inlineStr">
+        <is>
+          <t>PT0020</t>
+        </is>
+      </c>
+      <c r="D32" s="28" t="inlineStr">
+        <is>
+          <t>AGROPOTASION, 20 L</t>
+        </is>
+      </c>
+      <c r="E32" s="15" t="n">
+        <v>2560</v>
+      </c>
+      <c r="F32" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G32" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H32" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I32" s="15">
+        <f>MAX(0, E32-F32)</f>
+        <v/>
+      </c>
+      <c r="J32" s="15">
+        <f>ABS(F32-E32)</f>
+        <v/>
+      </c>
+      <c r="K32" s="16">
+        <f>IF(E32&gt;0, F32/E32, IF(F32&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L32" s="36" t="inlineStr">
+        <is>
+          <t>Sin Pedido</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="24" customHeight="1">
+      <c r="B33" s="21" t="inlineStr">
         <is>
           <t>TOTAL JAVIER</t>
         </is>
       </c>
-      <c r="C30" s="37" t="inlineStr">
-        <is>
-          <t>176 líneas</t>
-        </is>
-      </c>
-      <c r="D30" s="38" t="inlineStr"/>
-      <c r="E30" s="23">
-        <f>SUM(E10:E29)</f>
-        <v/>
-      </c>
-      <c r="F30" s="23">
-        <f>SUM(F10:F29)</f>
-        <v/>
-      </c>
-      <c r="G30" s="23">
-        <f>SUM(G10:G29)</f>
-        <v/>
-      </c>
-      <c r="H30" s="23">
-        <f>SUM(H10:H29)</f>
-        <v/>
-      </c>
-      <c r="I30" s="23">
-        <f>SUM(I10:I29)</f>
-        <v/>
-      </c>
-      <c r="J30" s="23">
-        <f>SUM(J10:J29)</f>
-        <v/>
-      </c>
-      <c r="K30" s="24">
-        <f>IF(E30&gt;0, F30/E30, 0)</f>
-        <v/>
-      </c>
-      <c r="L30" s="22">
-        <f>IF(K30&gt;=1, "SUPERADO", "EN CURSO")</f>
+      <c r="C33" s="37" t="inlineStr">
+        <is>
+          <t>179 líneas</t>
+        </is>
+      </c>
+      <c r="D33" s="38" t="inlineStr"/>
+      <c r="E33" s="23">
+        <f>SUM(E10:E32)</f>
+        <v/>
+      </c>
+      <c r="F33" s="23">
+        <f>SUM(F10:F32)</f>
+        <v/>
+      </c>
+      <c r="G33" s="23">
+        <f>SUM(G10:G32)</f>
+        <v/>
+      </c>
+      <c r="H33" s="23">
+        <f>SUM(H10:H32)</f>
+        <v/>
+      </c>
+      <c r="I33" s="23">
+        <f>SUM(I10:I32)</f>
+        <v/>
+      </c>
+      <c r="J33" s="23">
+        <f>SUM(J10:J32)</f>
+        <v/>
+      </c>
+      <c r="K33" s="24">
+        <f>IF(E33&gt;0, F33/E33, 0)</f>
+        <v/>
+      </c>
+      <c r="L33" s="22">
+        <f>IF(K33&gt;=1, "SUPERADO", "EN CURSO")</f>
         <v/>
       </c>
     </row>
@@ -7296,7 +7434,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 20/10/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 21/10/2026</t>
         </is>
       </c>
     </row>
@@ -7774,7 +7912,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:L26"/>
+  <dimension ref="B2:L27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -7801,7 +7939,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 20/10/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 21/10/2026</t>
         </is>
       </c>
     </row>
@@ -7812,19 +7950,19 @@
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D5" s="5" t="inlineStr">
         <is>
           <t>PEDIDOS REALES (U)</t>
         </is>
       </c>
       <c r="E5" s="4" t="n"/>
-      <c r="F5" s="6" t="inlineStr">
+      <c r="F5" s="5" t="inlineStr">
         <is>
           <t>% CONSECUCIÓN</t>
         </is>
       </c>
       <c r="G5" s="4" t="n"/>
-      <c r="H5" s="6" t="inlineStr">
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>FALTA CONSEGUIR (GAP)</t>
         </is>
@@ -7844,21 +7982,21 @@
         </is>
       </c>
       <c r="C6" s="4" t="n"/>
-      <c r="D6" s="25" t="inlineStr">
-        <is>
-          <t>9,960 u</t>
+      <c r="D6" s="26" t="inlineStr">
+        <is>
+          <t>17,400 u</t>
         </is>
       </c>
       <c r="E6" s="4" t="n"/>
-      <c r="F6" s="40" t="inlineStr">
-        <is>
-          <t>57.4%</t>
+      <c r="F6" s="26" t="inlineStr">
+        <is>
+          <t>100.3%</t>
         </is>
       </c>
       <c r="G6" s="4" t="n"/>
-      <c r="H6" s="40" t="inlineStr">
-        <is>
-          <t>7,380 u</t>
+      <c r="H6" s="26" t="inlineStr">
+        <is>
+          <t>0 u</t>
         </is>
       </c>
       <c r="I6" s="4" t="n"/>
@@ -8321,10 +8459,10 @@
         <v>2200</v>
       </c>
       <c r="F18" s="15" t="n">
-        <v>2200</v>
+        <v>5500</v>
       </c>
       <c r="G18" s="15" t="n">
-        <v>2200</v>
+        <v>5500</v>
       </c>
       <c r="H18" s="15" t="n">
         <v>0</v>
@@ -8355,22 +8493,22 @@
       </c>
       <c r="C19" s="32" t="inlineStr">
         <is>
-          <t>AQUOM0005</t>
+          <t>ANAE0020</t>
         </is>
       </c>
       <c r="D19" s="31" t="inlineStr">
         <is>
-          <t>AQUOM, 5 L</t>
+          <t>ALCAPLANT NEW AE, 20 KG</t>
         </is>
       </c>
       <c r="E19" s="19" t="n">
         <v>0</v>
       </c>
       <c r="F19" s="19" t="n">
-        <v>100</v>
+        <v>1100</v>
       </c>
       <c r="G19" s="19" t="n">
-        <v>100</v>
+        <v>1100</v>
       </c>
       <c r="H19" s="19" t="n">
         <v>0</v>
@@ -8401,22 +8539,22 @@
       </c>
       <c r="C20" s="29" t="inlineStr">
         <is>
-          <t>S0020</t>
+          <t>AQUOM0005</t>
         </is>
       </c>
       <c r="D20" s="28" t="inlineStr">
         <is>
-          <t>SAL-WAX STAR, 20 L</t>
+          <t>AQUOM, 5 L</t>
         </is>
       </c>
       <c r="E20" s="15" t="n">
-        <v>640</v>
+        <v>0</v>
       </c>
       <c r="F20" s="15" t="n">
-        <v>1920</v>
+        <v>100</v>
       </c>
       <c r="G20" s="15" t="n">
-        <v>1920</v>
+        <v>100</v>
       </c>
       <c r="H20" s="15" t="n">
         <v>0</v>
@@ -8435,7 +8573,7 @@
       </c>
       <c r="L20" s="34" t="inlineStr">
         <is>
-          <t>Superado</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -8447,22 +8585,22 @@
       </c>
       <c r="C21" s="32" t="inlineStr">
         <is>
-          <t>S0200</t>
+          <t>S0020</t>
         </is>
       </c>
       <c r="D21" s="31" t="inlineStr">
         <is>
-          <t>SAL-WAX STAR, 200 L</t>
+          <t>SAL-WAX STAR, 20 L</t>
         </is>
       </c>
       <c r="E21" s="19" t="n">
-        <v>400</v>
+        <v>640</v>
       </c>
       <c r="F21" s="19" t="n">
-        <v>800</v>
+        <v>2560</v>
       </c>
       <c r="G21" s="19" t="n">
-        <v>800</v>
+        <v>2560</v>
       </c>
       <c r="H21" s="19" t="n">
         <v>0</v>
@@ -8493,22 +8631,22 @@
       </c>
       <c r="C22" s="29" t="inlineStr">
         <is>
-          <t>S1000</t>
+          <t>S0200</t>
         </is>
       </c>
       <c r="D22" s="28" t="inlineStr">
         <is>
-          <t>SAL-WAX STAR, 1000 L</t>
+          <t>SAL-WAX STAR, 200 L</t>
         </is>
       </c>
       <c r="E22" s="15" t="n">
-        <v>5000</v>
+        <v>400</v>
       </c>
       <c r="F22" s="15" t="n">
-        <v>0</v>
+        <v>3200</v>
       </c>
       <c r="G22" s="15" t="n">
-        <v>0</v>
+        <v>3200</v>
       </c>
       <c r="H22" s="15" t="n">
         <v>0</v>
@@ -8525,9 +8663,9 @@
         <f>IF(E22&gt;0, F22/E22, IF(F22&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L22" s="36" t="inlineStr">
-        <is>
-          <t>Sin Pedido</t>
+      <c r="L22" s="34" t="inlineStr">
+        <is>
+          <t>Superado</t>
         </is>
       </c>
     </row>
@@ -8539,22 +8677,22 @@
       </c>
       <c r="C23" s="32" t="inlineStr">
         <is>
-          <t>SPCE2B0020</t>
+          <t>S1000</t>
         </is>
       </c>
       <c r="D23" s="31" t="inlineStr">
         <is>
-          <t>SPRINTENE CON BORO, 20 L</t>
+          <t>SAL-WAX STAR, 1000 L</t>
         </is>
       </c>
       <c r="E23" s="19" t="n">
-        <v>640</v>
+        <v>5000</v>
       </c>
       <c r="F23" s="19" t="n">
-        <v>320</v>
+        <v>0</v>
       </c>
       <c r="G23" s="19" t="n">
-        <v>320</v>
+        <v>0</v>
       </c>
       <c r="H23" s="19" t="n">
         <v>0</v>
@@ -8571,9 +8709,9 @@
         <f>IF(E23&gt;0, F23/E23, IF(F23&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L23" s="33" t="inlineStr">
-        <is>
-          <t>En Curso</t>
+      <c r="L23" s="39" t="inlineStr">
+        <is>
+          <t>Sin Pedido</t>
         </is>
       </c>
     </row>
@@ -8585,22 +8723,22 @@
       </c>
       <c r="C24" s="29" t="inlineStr">
         <is>
-          <t>SS0020</t>
+          <t>SPCE2B0020</t>
         </is>
       </c>
       <c r="D24" s="28" t="inlineStr">
         <is>
-          <t>SAL-WAX-Ca sólido, 20 KG</t>
+          <t>SPRINTENE CON BORO, 20 L</t>
         </is>
       </c>
       <c r="E24" s="15" t="n">
-        <v>0</v>
+        <v>640</v>
       </c>
       <c r="F24" s="15" t="n">
-        <v>1600</v>
+        <v>320</v>
       </c>
       <c r="G24" s="15" t="n">
-        <v>1600</v>
+        <v>320</v>
       </c>
       <c r="H24" s="15" t="n">
         <v>0</v>
@@ -8617,36 +8755,36 @@
         <f>IF(E24&gt;0, F24/E24, IF(F24&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L24" s="34" t="inlineStr">
-        <is>
-          <t>Extra Estimación</t>
+      <c r="L24" s="30" t="inlineStr">
+        <is>
+          <t>En Curso</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="B25" s="31" t="inlineStr">
         <is>
-          <t>FITOMURCIA S.L.</t>
+          <t>COMERCIAL TÉCNICA FITOCARTHAGO, S.L.</t>
         </is>
       </c>
       <c r="C25" s="32" t="inlineStr">
         <is>
-          <t>BIO1000</t>
+          <t>SS0020</t>
         </is>
       </c>
       <c r="D25" s="31" t="inlineStr">
         <is>
-          <t>BIORAD-20, 1000 L</t>
+          <t>SAL-WAX-Ca sólido, 20 KG</t>
         </is>
       </c>
       <c r="E25" s="19" t="n">
         <v>0</v>
       </c>
       <c r="F25" s="19" t="n">
-        <v>1000</v>
+        <v>1600</v>
       </c>
       <c r="G25" s="19" t="n">
-        <v>1000</v>
+        <v>1600</v>
       </c>
       <c r="H25" s="19" t="n">
         <v>0</v>
@@ -8669,48 +8807,94 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="24" customHeight="1">
-      <c r="B26" s="21" t="inlineStr">
+    <row r="26">
+      <c r="B26" s="28" t="inlineStr">
+        <is>
+          <t>FITOMURCIA S.L.</t>
+        </is>
+      </c>
+      <c r="C26" s="29" t="inlineStr">
+        <is>
+          <t>BIO1000</t>
+        </is>
+      </c>
+      <c r="D26" s="28" t="inlineStr">
+        <is>
+          <t>BIORAD-20, 1000 L</t>
+        </is>
+      </c>
+      <c r="E26" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" s="15" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G26" s="15" t="n">
+        <v>1000</v>
+      </c>
+      <c r="H26" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I26" s="15">
+        <f>MAX(0, E26-F26)</f>
+        <v/>
+      </c>
+      <c r="J26" s="15">
+        <f>ABS(F26-E26)</f>
+        <v/>
+      </c>
+      <c r="K26" s="16">
+        <f>IF(E26&gt;0, F26/E26, IF(F26&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L26" s="34" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="24" customHeight="1">
+      <c r="B27" s="21" t="inlineStr">
         <is>
           <t>TOTAL PEDRO</t>
         </is>
       </c>
-      <c r="C26" s="37" t="inlineStr">
+      <c r="C27" s="37" t="inlineStr">
         <is>
           <t>104 líneas</t>
         </is>
       </c>
-      <c r="D26" s="38" t="inlineStr"/>
-      <c r="E26" s="23">
-        <f>SUM(E10:E25)</f>
-        <v/>
-      </c>
-      <c r="F26" s="23">
-        <f>SUM(F10:F25)</f>
-        <v/>
-      </c>
-      <c r="G26" s="23">
-        <f>SUM(G10:G25)</f>
-        <v/>
-      </c>
-      <c r="H26" s="23">
-        <f>SUM(H10:H25)</f>
-        <v/>
-      </c>
-      <c r="I26" s="23">
-        <f>SUM(I10:I25)</f>
-        <v/>
-      </c>
-      <c r="J26" s="23">
-        <f>SUM(J10:J25)</f>
-        <v/>
-      </c>
-      <c r="K26" s="24">
-        <f>IF(E26&gt;0, F26/E26, 0)</f>
-        <v/>
-      </c>
-      <c r="L26" s="22">
-        <f>IF(K26&gt;=1, "SUPERADO", "EN CURSO")</f>
+      <c r="D27" s="38" t="inlineStr"/>
+      <c r="E27" s="23">
+        <f>SUM(E10:E26)</f>
+        <v/>
+      </c>
+      <c r="F27" s="23">
+        <f>SUM(F10:F26)</f>
+        <v/>
+      </c>
+      <c r="G27" s="23">
+        <f>SUM(G10:G26)</f>
+        <v/>
+      </c>
+      <c r="H27" s="23">
+        <f>SUM(H10:H26)</f>
+        <v/>
+      </c>
+      <c r="I27" s="23">
+        <f>SUM(I10:I26)</f>
+        <v/>
+      </c>
+      <c r="J27" s="23">
+        <f>SUM(J10:J26)</f>
+        <v/>
+      </c>
+      <c r="K27" s="24">
+        <f>IF(E27&gt;0, F27/E27, 0)</f>
+        <v/>
+      </c>
+      <c r="L27" s="22">
+        <f>IF(K27&gt;=1, "SUPERADO", "EN CURSO")</f>
         <v/>
       </c>
     </row>
@@ -8766,7 +8950,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 20/10/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 21/10/2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizacion pedidos 26.10: comercial, MRP y seguimiento
</commit_message>
<xml_diff>
--- a/Seguimiento_Presupuesto_Sep_2026.xlsx
+++ b/Seguimiento_Presupuesto_Sep_2026.xlsx
@@ -114,18 +114,18 @@
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="0092400E"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <b val="1"/>
       <color rgb="00166534"/>
       <sz val="9"/>
     </font>
     <font>
       <name val="Segoe UI"/>
       <color rgb="0064748B"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="0092400E"/>
       <sz val="9"/>
     </font>
     <font>
@@ -323,7 +323,7 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -335,23 +335,23 @@
     <xf numFmtId="0" fontId="14" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="8" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="16" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -915,7 +915,7 @@
     <row r="3" ht="20" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Comparativa Estimación Septiembre (Unidades) vs Pedidos Reales a Fecha 23/10/2026 | Generado: 23/10/2026 08:56</t>
+          <t>Comparativa Estimación Septiembre (Unidades) vs Pedidos Reales a Fecha 26/10/2026 | Generado: 26/10/2026 08:04</t>
         </is>
       </c>
     </row>
@@ -959,25 +959,25 @@
       <c r="C6" s="4" t="n"/>
       <c r="D6" s="8" t="inlineStr">
         <is>
-          <t>233,677 u</t>
+          <t>247,817 u</t>
         </is>
       </c>
       <c r="E6" s="4" t="n"/>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>128.4%</t>
+          <t>136.2%</t>
         </is>
       </c>
       <c r="G6" s="4" t="n"/>
       <c r="H6" s="9" t="inlineStr">
         <is>
-          <t>48,869 u</t>
+          <t>44,669 u</t>
         </is>
       </c>
       <c r="I6" s="4" t="n"/>
       <c r="J6" s="7" t="inlineStr">
         <is>
-          <t>180,008 u</t>
+          <t>190,808 u</t>
         </is>
       </c>
     </row>
@@ -1042,16 +1042,16 @@
         </is>
       </c>
       <c r="C10" s="13" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D10" s="14" t="n">
         <v>2320</v>
       </c>
       <c r="E10" s="14" t="n">
-        <v>3524</v>
+        <v>6864</v>
       </c>
       <c r="F10" s="14" t="n">
-        <v>3524</v>
+        <v>6864</v>
       </c>
       <c r="G10" s="14" t="n">
         <v>0</v>
@@ -1061,7 +1061,7 @@
         <v/>
       </c>
       <c r="I10" s="14">
-        <f>'Alfonso'!J23</f>
+        <f>'Alfonso'!J26</f>
         <v/>
       </c>
       <c r="J10" s="15">
@@ -1116,20 +1116,20 @@
         <v>21914</v>
       </c>
       <c r="E12" s="14" t="n">
-        <v>16045</v>
+        <v>20245</v>
       </c>
       <c r="F12" s="14" t="n">
         <v>13525</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>2520</v>
+        <v>6720</v>
       </c>
       <c r="H12" s="14">
         <f>MAX(0, D12-E12)</f>
         <v/>
       </c>
       <c r="I12" s="14">
-        <f>'Irene'!J51</f>
+        <f>'Irene'!J52</f>
         <v/>
       </c>
       <c r="J12" s="15">
@@ -1246,26 +1246,26 @@
         </is>
       </c>
       <c r="C16" s="13" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D16" s="14" t="n">
         <v>46000</v>
       </c>
       <c r="E16" s="14" t="n">
-        <v>102472</v>
+        <v>109072</v>
       </c>
       <c r="F16" s="14" t="n">
         <v>0</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>102472</v>
+        <v>109072</v>
       </c>
       <c r="H16" s="14">
         <f>MAX(0, D16-E16)</f>
         <v/>
       </c>
       <c r="I16" s="14">
-        <f>'Ricardo'!J45</f>
+        <f>'Ricardo'!J47</f>
         <v/>
       </c>
       <c r="J16" s="15">
@@ -1336,7 +1336,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:L23"/>
+  <dimension ref="B2:L26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1363,7 +1363,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 23/10/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 26/10/2026</t>
         </is>
       </c>
     </row>
@@ -1408,13 +1408,13 @@
       <c r="C6" s="4" t="n"/>
       <c r="D6" s="25" t="inlineStr">
         <is>
-          <t>3,524 u</t>
+          <t>6,864 u</t>
         </is>
       </c>
       <c r="E6" s="4" t="n"/>
       <c r="F6" s="25" t="inlineStr">
         <is>
-          <t>151.9%</t>
+          <t>295.9%</t>
         </is>
       </c>
       <c r="G6" s="4" t="n"/>
@@ -1515,10 +1515,10 @@
         <v>960</v>
       </c>
       <c r="F10" s="14" t="n">
-        <v>640</v>
+        <v>1280</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>640</v>
+        <v>1280</v>
       </c>
       <c r="H10" s="14" t="n">
         <v>0</v>
@@ -1537,7 +1537,7 @@
       </c>
       <c r="L10" s="29" t="inlineStr">
         <is>
-          <t>En Curso</t>
+          <t>Superado</t>
         </is>
       </c>
     </row>
@@ -1561,10 +1561,10 @@
         <v>960</v>
       </c>
       <c r="F11" s="18" t="n">
-        <v>640</v>
+        <v>1280</v>
       </c>
       <c r="G11" s="18" t="n">
-        <v>640</v>
+        <v>1280</v>
       </c>
       <c r="H11" s="18" t="n">
         <v>0</v>
@@ -1583,7 +1583,7 @@
       </c>
       <c r="L11" s="32" t="inlineStr">
         <is>
-          <t>En Curso</t>
+          <t>Superado</t>
         </is>
       </c>
     </row>
@@ -1627,7 +1627,7 @@
         <f>IF(E12&gt;0, F12/E12, IF(F12&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L12" s="33" t="inlineStr">
+      <c r="L12" s="29" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -1673,7 +1673,7 @@
         <f>IF(E13&gt;0, F13/E13, IF(F13&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L13" s="34" t="inlineStr">
+      <c r="L13" s="32" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -1719,7 +1719,7 @@
         <f>IF(E14&gt;0, F14/E14, IF(F14&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L14" s="33" t="inlineStr">
+      <c r="L14" s="29" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -1765,7 +1765,7 @@
         <f>IF(E15&gt;0, F15/E15, IF(F15&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L15" s="34" t="inlineStr">
+      <c r="L15" s="32" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -1779,22 +1779,22 @@
       </c>
       <c r="C16" s="28" t="inlineStr">
         <is>
-          <t>BIO0020</t>
+          <t>AN0020</t>
         </is>
       </c>
       <c r="D16" s="27" t="inlineStr">
         <is>
-          <t>BIORAD-20, 20 L</t>
+          <t>ALCAPLANT NEW, 20 KG</t>
         </is>
       </c>
       <c r="E16" s="14" t="n">
-        <v>400</v>
+        <v>0</v>
       </c>
       <c r="F16" s="14" t="n">
-        <v>0</v>
+        <v>1100</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>0</v>
+        <v>1100</v>
       </c>
       <c r="H16" s="14" t="n">
         <v>0</v>
@@ -1811,36 +1811,36 @@
         <f>IF(E16&gt;0, F16/E16, IF(F16&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L16" s="35" t="inlineStr">
-        <is>
-          <t>Sin Pedido</t>
+      <c r="L16" s="29" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="30" t="inlineStr">
         <is>
-          <t>VILLALTA SATIVUM, S.L.</t>
+          <t>AGROVEYCA,S.L</t>
         </is>
       </c>
       <c r="C17" s="31" t="inlineStr">
         <is>
-          <t>AGXKAEP0020</t>
+          <t>AQUOM0020</t>
         </is>
       </c>
       <c r="D17" s="30" t="inlineStr">
         <is>
-          <t>BIOCULTURE POTASIO PLUS, 20 L</t>
+          <t>AQUOM, 20 L</t>
         </is>
       </c>
       <c r="E17" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F17" s="18" t="n">
-        <v>140</v>
+        <v>320</v>
       </c>
       <c r="G17" s="18" t="n">
-        <v>140</v>
+        <v>320</v>
       </c>
       <c r="H17" s="18" t="n">
         <v>0</v>
@@ -1857,7 +1857,7 @@
         <f>IF(E17&gt;0, F17/E17, IF(F17&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L17" s="34" t="inlineStr">
+      <c r="L17" s="32" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -1866,27 +1866,27 @@
     <row r="18">
       <c r="B18" s="27" t="inlineStr">
         <is>
-          <t>VILLALTA SATIVUM, S.L.</t>
+          <t>AGROVEYCA,S.L</t>
         </is>
       </c>
       <c r="C18" s="28" t="inlineStr">
         <is>
-          <t>AQUOM0020</t>
+          <t>BIO0020</t>
         </is>
       </c>
       <c r="D18" s="27" t="inlineStr">
         <is>
-          <t>AQUOM, 20 L</t>
+          <t>BIORAD-20, 20 L</t>
         </is>
       </c>
       <c r="E18" s="14" t="n">
-        <v>0</v>
+        <v>400</v>
       </c>
       <c r="F18" s="14" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="G18" s="14" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="H18" s="14" t="n">
         <v>0</v>
@@ -1905,34 +1905,34 @@
       </c>
       <c r="L18" s="33" t="inlineStr">
         <is>
-          <t>Extra Estimación</t>
+          <t>Sin Pedido</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="30" t="inlineStr">
         <is>
-          <t>VILLALTA SATIVUM, S.L.</t>
+          <t>AGROVEYCA,S.L</t>
         </is>
       </c>
       <c r="C19" s="31" t="inlineStr">
         <is>
-          <t>C-CUAE0020</t>
+          <t>S0020</t>
         </is>
       </c>
       <c r="D19" s="30" t="inlineStr">
         <is>
-          <t>CUPRAMEC, 20 L</t>
+          <t>SAL-WAX STAR, 20 L</t>
         </is>
       </c>
       <c r="E19" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F19" s="18" t="n">
-        <v>200</v>
+        <v>640</v>
       </c>
       <c r="G19" s="18" t="n">
-        <v>200</v>
+        <v>640</v>
       </c>
       <c r="H19" s="18" t="n">
         <v>0</v>
@@ -1949,7 +1949,7 @@
         <f>IF(E19&gt;0, F19/E19, IF(F19&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L19" s="34" t="inlineStr">
+      <c r="L19" s="32" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -1963,22 +1963,22 @@
       </c>
       <c r="C20" s="28" t="inlineStr">
         <is>
-          <t>PT0001</t>
+          <t>AGXKAEP0020</t>
         </is>
       </c>
       <c r="D20" s="27" t="inlineStr">
         <is>
-          <t>AGROPOTASION, 1 L</t>
+          <t>BIOCULTURE POTASIO PLUS, 20 L</t>
         </is>
       </c>
       <c r="E20" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F20" s="14" t="n">
-        <v>24</v>
+        <v>140</v>
       </c>
       <c r="G20" s="14" t="n">
-        <v>24</v>
+        <v>140</v>
       </c>
       <c r="H20" s="14" t="n">
         <v>0</v>
@@ -1995,7 +1995,7 @@
         <f>IF(E20&gt;0, F20/E20, IF(F20&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L20" s="33" t="inlineStr">
+      <c r="L20" s="29" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -2009,22 +2009,22 @@
       </c>
       <c r="C21" s="31" t="inlineStr">
         <is>
-          <t>PT0005</t>
+          <t>AQUOM0020</t>
         </is>
       </c>
       <c r="D21" s="30" t="inlineStr">
         <is>
-          <t>AGROPOTASION, 5 L</t>
+          <t>AQUOM, 20 L</t>
         </is>
       </c>
       <c r="E21" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F21" s="18" t="n">
-        <v>100</v>
+        <v>40</v>
       </c>
       <c r="G21" s="18" t="n">
-        <v>100</v>
+        <v>40</v>
       </c>
       <c r="H21" s="18" t="n">
         <v>0</v>
@@ -2041,7 +2041,7 @@
         <f>IF(E21&gt;0, F21/E21, IF(F21&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L21" s="34" t="inlineStr">
+      <c r="L21" s="32" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -2055,22 +2055,22 @@
       </c>
       <c r="C22" s="28" t="inlineStr">
         <is>
-          <t>PT0020</t>
+          <t>C-CUAE0020</t>
         </is>
       </c>
       <c r="D22" s="27" t="inlineStr">
         <is>
-          <t>AGROPOTASION, 20 L</t>
+          <t>CUPRAMEC, 20 L</t>
         </is>
       </c>
       <c r="E22" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F22" s="14" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="G22" s="14" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="H22" s="14" t="n">
         <v>0</v>
@@ -2087,54 +2087,192 @@
         <f>IF(E22&gt;0, F22/E22, IF(F22&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L22" s="33" t="inlineStr">
+      <c r="L22" s="29" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="24" customHeight="1">
-      <c r="B23" s="20" t="inlineStr">
+    <row r="23">
+      <c r="B23" s="30" t="inlineStr">
+        <is>
+          <t>VILLALTA SATIVUM, S.L.</t>
+        </is>
+      </c>
+      <c r="C23" s="31" t="inlineStr">
+        <is>
+          <t>PT0001</t>
+        </is>
+      </c>
+      <c r="D23" s="30" t="inlineStr">
+        <is>
+          <t>AGROPOTASION, 1 L</t>
+        </is>
+      </c>
+      <c r="E23" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" s="18" t="n">
+        <v>24</v>
+      </c>
+      <c r="G23" s="18" t="n">
+        <v>24</v>
+      </c>
+      <c r="H23" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="I23" s="18">
+        <f>MAX(0, E23-F23)</f>
+        <v/>
+      </c>
+      <c r="J23" s="18">
+        <f>ABS(F23-E23)</f>
+        <v/>
+      </c>
+      <c r="K23" s="19">
+        <f>IF(E23&gt;0, F23/E23, IF(F23&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L23" s="32" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="27" t="inlineStr">
+        <is>
+          <t>VILLALTA SATIVUM, S.L.</t>
+        </is>
+      </c>
+      <c r="C24" s="28" t="inlineStr">
+        <is>
+          <t>PT0005</t>
+        </is>
+      </c>
+      <c r="D24" s="27" t="inlineStr">
+        <is>
+          <t>AGROPOTASION, 5 L</t>
+        </is>
+      </c>
+      <c r="E24" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" s="14" t="n">
+        <v>100</v>
+      </c>
+      <c r="G24" s="14" t="n">
+        <v>100</v>
+      </c>
+      <c r="H24" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I24" s="14">
+        <f>MAX(0, E24-F24)</f>
+        <v/>
+      </c>
+      <c r="J24" s="14">
+        <f>ABS(F24-E24)</f>
+        <v/>
+      </c>
+      <c r="K24" s="15">
+        <f>IF(E24&gt;0, F24/E24, IF(F24&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L24" s="29" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="30" t="inlineStr">
+        <is>
+          <t>VILLALTA SATIVUM, S.L.</t>
+        </is>
+      </c>
+      <c r="C25" s="31" t="inlineStr">
+        <is>
+          <t>PT0020</t>
+        </is>
+      </c>
+      <c r="D25" s="30" t="inlineStr">
+        <is>
+          <t>AGROPOTASION, 20 L</t>
+        </is>
+      </c>
+      <c r="E25" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" s="18" t="n">
+        <v>100</v>
+      </c>
+      <c r="G25" s="18" t="n">
+        <v>100</v>
+      </c>
+      <c r="H25" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="I25" s="18">
+        <f>MAX(0, E25-F25)</f>
+        <v/>
+      </c>
+      <c r="J25" s="18">
+        <f>ABS(F25-E25)</f>
+        <v/>
+      </c>
+      <c r="K25" s="19">
+        <f>IF(E25&gt;0, F25/E25, IF(F25&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L25" s="32" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="24" customHeight="1">
+      <c r="B26" s="20" t="inlineStr">
         <is>
           <t>TOTAL ALFONSO</t>
         </is>
       </c>
-      <c r="C23" s="36" t="inlineStr">
+      <c r="C26" s="34" t="inlineStr">
         <is>
           <t>279 líneas</t>
         </is>
       </c>
-      <c r="D23" s="37" t="inlineStr"/>
-      <c r="E23" s="22">
-        <f>SUM(E10:E22)</f>
-        <v/>
-      </c>
-      <c r="F23" s="22">
-        <f>SUM(F10:F22)</f>
-        <v/>
-      </c>
-      <c r="G23" s="22">
-        <f>SUM(G10:G22)</f>
-        <v/>
-      </c>
-      <c r="H23" s="22">
-        <f>SUM(H10:H22)</f>
-        <v/>
-      </c>
-      <c r="I23" s="22">
-        <f>SUM(I10:I22)</f>
-        <v/>
-      </c>
-      <c r="J23" s="22">
-        <f>SUM(J10:J22)</f>
-        <v/>
-      </c>
-      <c r="K23" s="23">
-        <f>IF(E23&gt;0, F23/E23, 0)</f>
-        <v/>
-      </c>
-      <c r="L23" s="21">
-        <f>IF(K23&gt;=1, "SUPERADO", "EN CURSO")</f>
+      <c r="D26" s="35" t="inlineStr"/>
+      <c r="E26" s="22">
+        <f>SUM(E10:E25)</f>
+        <v/>
+      </c>
+      <c r="F26" s="22">
+        <f>SUM(F10:F25)</f>
+        <v/>
+      </c>
+      <c r="G26" s="22">
+        <f>SUM(G10:G25)</f>
+        <v/>
+      </c>
+      <c r="H26" s="22">
+        <f>SUM(H10:H25)</f>
+        <v/>
+      </c>
+      <c r="I26" s="22">
+        <f>SUM(I10:I25)</f>
+        <v/>
+      </c>
+      <c r="J26" s="22">
+        <f>SUM(J10:J25)</f>
+        <v/>
+      </c>
+      <c r="K26" s="23">
+        <f>IF(E26&gt;0, F26/E26, 0)</f>
+        <v/>
+      </c>
+      <c r="L26" s="21">
+        <f>IF(K26&gt;=1, "SUPERADO", "EN CURSO")</f>
         <v/>
       </c>
     </row>
@@ -2190,7 +2328,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 23/10/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 26/10/2026</t>
         </is>
       </c>
     </row>
@@ -2362,7 +2500,7 @@
         <f>IF(E10&gt;0, F10/E10, IF(F10&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L10" s="35" t="inlineStr">
+      <c r="L10" s="33" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -2408,7 +2546,7 @@
         <f>IF(E11&gt;0, F11/E11, IF(F11&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L11" s="38" t="inlineStr">
+      <c r="L11" s="36" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -2454,7 +2592,7 @@
         <f>IF(E12&gt;0, F12/E12, IF(F12&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L12" s="35" t="inlineStr">
+      <c r="L12" s="33" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -2500,7 +2638,7 @@
         <f>IF(E13&gt;0, F13/E13, IF(F13&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L13" s="32" t="inlineStr">
+      <c r="L13" s="37" t="inlineStr">
         <is>
           <t>En Curso</t>
         </is>
@@ -2546,7 +2684,7 @@
         <f>IF(E14&gt;0, F14/E14, IF(F14&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L14" s="35" t="inlineStr">
+      <c r="L14" s="33" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -2592,7 +2730,7 @@
         <f>IF(E15&gt;0, F15/E15, IF(F15&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L15" s="38" t="inlineStr">
+      <c r="L15" s="36" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -2638,7 +2776,7 @@
         <f>IF(E16&gt;0, F16/E16, IF(F16&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L16" s="35" t="inlineStr">
+      <c r="L16" s="33" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -2684,7 +2822,7 @@
         <f>IF(E17&gt;0, F17/E17, IF(F17&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L17" s="38" t="inlineStr">
+      <c r="L17" s="36" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -2730,7 +2868,7 @@
         <f>IF(E18&gt;0, F18/E18, IF(F18&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L18" s="35" t="inlineStr">
+      <c r="L18" s="33" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -2776,7 +2914,7 @@
         <f>IF(E19&gt;0, F19/E19, IF(F19&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L19" s="38" t="inlineStr">
+      <c r="L19" s="36" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -2822,7 +2960,7 @@
         <f>IF(E20&gt;0, F20/E20, IF(F20&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L20" s="35" t="inlineStr">
+      <c r="L20" s="33" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -2868,7 +3006,7 @@
         <f>IF(E21&gt;0, F21/E21, IF(F21&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L21" s="38" t="inlineStr">
+      <c r="L21" s="36" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -2914,7 +3052,7 @@
         <f>IF(E22&gt;0, F22/E22, IF(F22&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L22" s="35" t="inlineStr">
+      <c r="L22" s="33" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -2960,7 +3098,7 @@
         <f>IF(E23&gt;0, F23/E23, IF(F23&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L23" s="38" t="inlineStr">
+      <c r="L23" s="36" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -3006,7 +3144,7 @@
         <f>IF(E24&gt;0, F24/E24, IF(F24&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L24" s="33" t="inlineStr">
+      <c r="L24" s="29" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -3052,7 +3190,7 @@
         <f>IF(E25&gt;0, F25/E25, IF(F25&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L25" s="34" t="inlineStr">
+      <c r="L25" s="32" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -3098,7 +3236,7 @@
         <f>IF(E26&gt;0, F26/E26, IF(F26&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L26" s="33" t="inlineStr">
+      <c r="L26" s="29" t="inlineStr">
         <is>
           <t>Superado</t>
         </is>
@@ -3144,7 +3282,7 @@
         <f>IF(E27&gt;0, F27/E27, IF(F27&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L27" s="34" t="inlineStr">
+      <c r="L27" s="32" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -3190,7 +3328,7 @@
         <f>IF(E28&gt;0, F28/E28, IF(F28&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L28" s="33" t="inlineStr">
+      <c r="L28" s="29" t="inlineStr">
         <is>
           <t>Superado</t>
         </is>
@@ -3236,7 +3374,7 @@
         <f>IF(E29&gt;0, F29/E29, IF(F29&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L29" s="34" t="inlineStr">
+      <c r="L29" s="32" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -3282,7 +3420,7 @@
         <f>IF(E30&gt;0, F30/E30, IF(F30&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L30" s="35" t="inlineStr">
+      <c r="L30" s="33" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -3328,7 +3466,7 @@
         <f>IF(E31&gt;0, F31/E31, IF(F31&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L31" s="38" t="inlineStr">
+      <c r="L31" s="36" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -3374,7 +3512,7 @@
         <f>IF(E32&gt;0, F32/E32, IF(F32&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L32" s="35" t="inlineStr">
+      <c r="L32" s="33" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -3420,7 +3558,7 @@
         <f>IF(E33&gt;0, F33/E33, IF(F33&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L33" s="38" t="inlineStr">
+      <c r="L33" s="36" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -3466,7 +3604,7 @@
         <f>IF(E34&gt;0, F34/E34, IF(F34&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L34" s="35" t="inlineStr">
+      <c r="L34" s="33" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -3512,7 +3650,7 @@
         <f>IF(E35&gt;0, F35/E35, IF(F35&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L35" s="34" t="inlineStr">
+      <c r="L35" s="32" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -3558,7 +3696,7 @@
         <f>IF(E36&gt;0, F36/E36, IF(F36&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L36" s="35" t="inlineStr">
+      <c r="L36" s="33" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -3604,7 +3742,7 @@
         <f>IF(E37&gt;0, F37/E37, IF(F37&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L37" s="38" t="inlineStr">
+      <c r="L37" s="36" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -3650,7 +3788,7 @@
         <f>IF(E38&gt;0, F38/E38, IF(F38&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L38" s="33" t="inlineStr">
+      <c r="L38" s="29" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -3696,7 +3834,7 @@
         <f>IF(E39&gt;0, F39/E39, IF(F39&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L39" s="34" t="inlineStr">
+      <c r="L39" s="32" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -3742,7 +3880,7 @@
         <f>IF(E40&gt;0, F40/E40, IF(F40&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L40" s="33" t="inlineStr">
+      <c r="L40" s="29" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -3788,7 +3926,7 @@
         <f>IF(E41&gt;0, F41/E41, IF(F41&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L41" s="34" t="inlineStr">
+      <c r="L41" s="32" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -3834,7 +3972,7 @@
         <f>IF(E42&gt;0, F42/E42, IF(F42&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L42" s="33" t="inlineStr">
+      <c r="L42" s="29" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -3880,7 +4018,7 @@
         <f>IF(E43&gt;0, F43/E43, IF(F43&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L43" s="34" t="inlineStr">
+      <c r="L43" s="32" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -3926,7 +4064,7 @@
         <f>IF(E44&gt;0, F44/E44, IF(F44&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L44" s="33" t="inlineStr">
+      <c r="L44" s="29" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -3972,7 +4110,7 @@
         <f>IF(E45&gt;0, F45/E45, IF(F45&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L45" s="34" t="inlineStr">
+      <c r="L45" s="32" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -4018,7 +4156,7 @@
         <f>IF(E46&gt;0, F46/E46, IF(F46&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L46" s="33" t="inlineStr">
+      <c r="L46" s="29" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -4064,7 +4202,7 @@
         <f>IF(E47&gt;0, F47/E47, IF(F47&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L47" s="38" t="inlineStr">
+      <c r="L47" s="36" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -4076,12 +4214,12 @@
           <t>TOTAL GARCÍA</t>
         </is>
       </c>
-      <c r="C48" s="36" t="inlineStr">
+      <c r="C48" s="34" t="inlineStr">
         <is>
           <t>234 líneas</t>
         </is>
       </c>
-      <c r="D48" s="37" t="inlineStr"/>
+      <c r="D48" s="35" t="inlineStr"/>
       <c r="E48" s="22">
         <f>SUM(E10:E47)</f>
         <v/>
@@ -4140,7 +4278,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:L51"/>
+  <dimension ref="B2:L52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -4167,7 +4305,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 23/10/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 26/10/2026</t>
         </is>
       </c>
     </row>
@@ -4212,25 +4350,25 @@
       <c r="C6" s="4" t="n"/>
       <c r="D6" s="24" t="inlineStr">
         <is>
-          <t>16,045 u</t>
+          <t>20,245 u</t>
         </is>
       </c>
       <c r="E6" s="4" t="n"/>
-      <c r="F6" s="39" t="inlineStr">
-        <is>
-          <t>73.2%</t>
+      <c r="F6" s="38" t="inlineStr">
+        <is>
+          <t>92.4%</t>
         </is>
       </c>
       <c r="G6" s="4" t="n"/>
-      <c r="H6" s="39" t="inlineStr">
-        <is>
-          <t>5,869 u</t>
+      <c r="H6" s="38" t="inlineStr">
+        <is>
+          <t>1,669 u</t>
         </is>
       </c>
       <c r="I6" s="4" t="n"/>
       <c r="J6" s="24" t="inlineStr">
         <is>
-          <t>2,520 u</t>
+          <t>6,720 u</t>
         </is>
       </c>
       <c r="K6" s="4" t="n"/>
@@ -4339,7 +4477,7 @@
         <f>IF(E10&gt;0, F10/E10, IF(F10&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L10" s="35" t="inlineStr">
+      <c r="L10" s="33" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -4365,13 +4503,13 @@
         <v>1920</v>
       </c>
       <c r="F11" s="18" t="n">
-        <v>1280</v>
+        <v>3200</v>
       </c>
       <c r="G11" s="18" t="n">
         <v>1280</v>
       </c>
       <c r="H11" s="18" t="n">
-        <v>0</v>
+        <v>1920</v>
       </c>
       <c r="I11" s="18">
         <f>MAX(0, E11-F11)</f>
@@ -4387,7 +4525,7 @@
       </c>
       <c r="L11" s="32" t="inlineStr">
         <is>
-          <t>En Curso</t>
+          <t>Superado</t>
         </is>
       </c>
     </row>
@@ -4431,7 +4569,7 @@
         <f>IF(E12&gt;0, F12/E12, IF(F12&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L12" s="29" t="inlineStr">
+      <c r="L12" s="39" t="inlineStr">
         <is>
           <t>En Curso</t>
         </is>
@@ -4477,7 +4615,7 @@
         <f>IF(E13&gt;0, F13/E13, IF(F13&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L13" s="34" t="inlineStr">
+      <c r="L13" s="32" t="inlineStr">
         <is>
           <t>Superado</t>
         </is>
@@ -4523,7 +4661,7 @@
         <f>IF(E14&gt;0, F14/E14, IF(F14&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L14" s="33" t="inlineStr">
+      <c r="L14" s="29" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -4569,7 +4707,7 @@
         <f>IF(E15&gt;0, F15/E15, IF(F15&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L15" s="38" t="inlineStr">
+      <c r="L15" s="36" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -4615,7 +4753,7 @@
         <f>IF(E16&gt;0, F16/E16, IF(F16&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L16" s="35" t="inlineStr">
+      <c r="L16" s="33" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -4661,7 +4799,7 @@
         <f>IF(E17&gt;0, F17/E17, IF(F17&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L17" s="38" t="inlineStr">
+      <c r="L17" s="36" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -4707,7 +4845,7 @@
         <f>IF(E18&gt;0, F18/E18, IF(F18&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L18" s="35" t="inlineStr">
+      <c r="L18" s="33" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -4799,7 +4937,7 @@
         <f>IF(E20&gt;0, F20/E20, IF(F20&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L20" s="35" t="inlineStr">
+      <c r="L20" s="33" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -4845,7 +4983,7 @@
         <f>IF(E21&gt;0, F21/E21, IF(F21&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L21" s="34" t="inlineStr">
+      <c r="L21" s="32" t="inlineStr">
         <is>
           <t>Superado</t>
         </is>
@@ -4891,7 +5029,7 @@
         <f>IF(E22&gt;0, F22/E22, IF(F22&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L22" s="33" t="inlineStr">
+      <c r="L22" s="29" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -4937,7 +5075,7 @@
         <f>IF(E23&gt;0, F23/E23, IF(F23&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L23" s="38" t="inlineStr">
+      <c r="L23" s="36" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -5029,7 +5167,7 @@
         <f>IF(E25&gt;0, F25/E25, IF(F25&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L25" s="38" t="inlineStr">
+      <c r="L25" s="36" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -5075,7 +5213,7 @@
         <f>IF(E26&gt;0, F26/E26, IF(F26&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L26" s="33" t="inlineStr">
+      <c r="L26" s="29" t="inlineStr">
         <is>
           <t>Superado</t>
         </is>
@@ -5121,7 +5259,7 @@
         <f>IF(E27&gt;0, F27/E27, IF(F27&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L27" s="32" t="inlineStr">
+      <c r="L27" s="37" t="inlineStr">
         <is>
           <t>En Curso</t>
         </is>
@@ -5167,7 +5305,7 @@
         <f>IF(E28&gt;0, F28/E28, IF(F28&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L28" s="35" t="inlineStr">
+      <c r="L28" s="33" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -5213,7 +5351,7 @@
         <f>IF(E29&gt;0, F29/E29, IF(F29&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L29" s="34" t="inlineStr">
+      <c r="L29" s="32" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -5259,7 +5397,7 @@
         <f>IF(E30&gt;0, F30/E30, IF(F30&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L30" s="33" t="inlineStr">
+      <c r="L30" s="29" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -5305,7 +5443,7 @@
         <f>IF(E31&gt;0, F31/E31, IF(F31&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L31" s="32" t="inlineStr">
+      <c r="L31" s="37" t="inlineStr">
         <is>
           <t>En Curso</t>
         </is>
@@ -5351,7 +5489,7 @@
         <f>IF(E32&gt;0, F32/E32, IF(F32&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L32" s="33" t="inlineStr">
+      <c r="L32" s="29" t="inlineStr">
         <is>
           <t>Superado</t>
         </is>
@@ -5397,7 +5535,7 @@
         <f>IF(E33&gt;0, F33/E33, IF(F33&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L33" s="32" t="inlineStr">
+      <c r="L33" s="37" t="inlineStr">
         <is>
           <t>En Curso</t>
         </is>
@@ -5443,7 +5581,7 @@
         <f>IF(E34&gt;0, F34/E34, IF(F34&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L34" s="35" t="inlineStr">
+      <c r="L34" s="33" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -5489,7 +5627,7 @@
         <f>IF(E35&gt;0, F35/E35, IF(F35&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L35" s="34" t="inlineStr">
+      <c r="L35" s="32" t="inlineStr">
         <is>
           <t>Superado</t>
         </is>
@@ -5535,7 +5673,7 @@
         <f>IF(E36&gt;0, F36/E36, IF(F36&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L36" s="33" t="inlineStr">
+      <c r="L36" s="29" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -5581,7 +5719,7 @@
         <f>IF(E37&gt;0, F37/E37, IF(F37&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L37" s="34" t="inlineStr">
+      <c r="L37" s="32" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -5627,7 +5765,7 @@
         <f>IF(E38&gt;0, F38/E38, IF(F38&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L38" s="33" t="inlineStr">
+      <c r="L38" s="29" t="inlineStr">
         <is>
           <t>Superado</t>
         </is>
@@ -5653,13 +5791,13 @@
         <v>1240</v>
       </c>
       <c r="F39" s="18" t="n">
-        <v>640</v>
+        <v>2560</v>
       </c>
       <c r="G39" s="18" t="n">
         <v>640</v>
       </c>
       <c r="H39" s="18" t="n">
-        <v>0</v>
+        <v>1920</v>
       </c>
       <c r="I39" s="18">
         <f>MAX(0, E39-F39)</f>
@@ -5675,7 +5813,7 @@
       </c>
       <c r="L39" s="32" t="inlineStr">
         <is>
-          <t>En Curso</t>
+          <t>Superado</t>
         </is>
       </c>
     </row>
@@ -5719,7 +5857,7 @@
         <f>IF(E40&gt;0, F40/E40, IF(F40&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L40" s="35" t="inlineStr">
+      <c r="L40" s="33" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -5765,7 +5903,7 @@
         <f>IF(E41&gt;0, F41/E41, IF(F41&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L41" s="38" t="inlineStr">
+      <c r="L41" s="36" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -5811,7 +5949,7 @@
         <f>IF(E42&gt;0, F42/E42, IF(F42&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L42" s="33" t="inlineStr">
+      <c r="L42" s="29" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -5857,7 +5995,7 @@
         <f>IF(E43&gt;0, F43/E43, IF(F43&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L43" s="34" t="inlineStr">
+      <c r="L43" s="32" t="inlineStr">
         <is>
           <t>Superado</t>
         </is>
@@ -5903,7 +6041,7 @@
         <f>IF(E44&gt;0, F44/E44, IF(F44&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L44" s="33" t="inlineStr">
+      <c r="L44" s="29" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -5949,7 +6087,7 @@
         <f>IF(E45&gt;0, F45/E45, IF(F45&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L45" s="34" t="inlineStr">
+      <c r="L45" s="32" t="inlineStr">
         <is>
           <t>Superado</t>
         </is>
@@ -5995,7 +6133,7 @@
         <f>IF(E46&gt;0, F46/E46, IF(F46&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L46" s="33" t="inlineStr">
+      <c r="L46" s="29" t="inlineStr">
         <is>
           <t>Superado</t>
         </is>
@@ -6041,7 +6179,7 @@
         <f>IF(E47&gt;0, F47/E47, IF(F47&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L47" s="38" t="inlineStr">
+      <c r="L47" s="36" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -6087,7 +6225,7 @@
         <f>IF(E48&gt;0, F48/E48, IF(F48&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L48" s="35" t="inlineStr">
+      <c r="L48" s="33" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -6101,25 +6239,25 @@
       </c>
       <c r="C49" s="31" t="inlineStr">
         <is>
-          <t>TRI0005</t>
+          <t>TRI0001</t>
         </is>
       </c>
       <c r="D49" s="30" t="inlineStr">
         <is>
-          <t>TRIFENO-94, 5L</t>
+          <t>TRIFENO-94, 1 L</t>
         </is>
       </c>
       <c r="E49" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F49" s="18" t="n">
-        <v>300</v>
+        <v>60</v>
       </c>
       <c r="G49" s="18" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="H49" s="18" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="I49" s="18">
         <f>MAX(0, E49-F49)</f>
@@ -6133,7 +6271,7 @@
         <f>IF(E49&gt;0, F49/E49, IF(F49&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L49" s="34" t="inlineStr">
+      <c r="L49" s="32" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -6142,30 +6280,30 @@
     <row r="50">
       <c r="B50" s="27" t="inlineStr">
         <is>
-          <t>SUCA, S.C.A.</t>
+          <t>GUIVARTO AGRICOLA, S.L.</t>
         </is>
       </c>
       <c r="C50" s="28" t="inlineStr">
         <is>
-          <t>AGXK0020</t>
+          <t>TRI0005</t>
         </is>
       </c>
       <c r="D50" s="27" t="inlineStr">
         <is>
-          <t>AGROXILATO-K, 20 L</t>
+          <t>TRIFENO-94, 5L</t>
         </is>
       </c>
       <c r="E50" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F50" s="14" t="n">
-        <v>640</v>
+        <v>600</v>
       </c>
       <c r="G50" s="14" t="n">
-        <v>640</v>
+        <v>300</v>
       </c>
       <c r="H50" s="14" t="n">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="I50" s="14">
         <f>MAX(0, E50-F50)</f>
@@ -6179,54 +6317,100 @@
         <f>IF(E50&gt;0, F50/E50, IF(F50&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L50" s="33" t="inlineStr">
+      <c r="L50" s="29" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
       </c>
     </row>
-    <row r="51" ht="24" customHeight="1">
-      <c r="B51" s="20" t="inlineStr">
+    <row r="51">
+      <c r="B51" s="30" t="inlineStr">
+        <is>
+          <t>SUCA, S.C.A.</t>
+        </is>
+      </c>
+      <c r="C51" s="31" t="inlineStr">
+        <is>
+          <t>AGXK0020</t>
+        </is>
+      </c>
+      <c r="D51" s="30" t="inlineStr">
+        <is>
+          <t>AGROXILATO-K, 20 L</t>
+        </is>
+      </c>
+      <c r="E51" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F51" s="18" t="n">
+        <v>640</v>
+      </c>
+      <c r="G51" s="18" t="n">
+        <v>640</v>
+      </c>
+      <c r="H51" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="I51" s="18">
+        <f>MAX(0, E51-F51)</f>
+        <v/>
+      </c>
+      <c r="J51" s="18">
+        <f>ABS(F51-E51)</f>
+        <v/>
+      </c>
+      <c r="K51" s="19">
+        <f>IF(E51&gt;0, F51/E51, IF(F51&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L51" s="32" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="24" customHeight="1">
+      <c r="B52" s="20" t="inlineStr">
         <is>
           <t>TOTAL IRENE</t>
         </is>
       </c>
-      <c r="C51" s="36" t="inlineStr">
+      <c r="C52" s="34" t="inlineStr">
         <is>
           <t>89 líneas</t>
         </is>
       </c>
-      <c r="D51" s="37" t="inlineStr"/>
-      <c r="E51" s="22">
-        <f>SUM(E10:E50)</f>
-        <v/>
-      </c>
-      <c r="F51" s="22">
-        <f>SUM(F10:F50)</f>
-        <v/>
-      </c>
-      <c r="G51" s="22">
-        <f>SUM(G10:G50)</f>
-        <v/>
-      </c>
-      <c r="H51" s="22">
-        <f>SUM(H10:H50)</f>
-        <v/>
-      </c>
-      <c r="I51" s="22">
-        <f>SUM(I10:I50)</f>
-        <v/>
-      </c>
-      <c r="J51" s="22">
-        <f>SUM(J10:J50)</f>
-        <v/>
-      </c>
-      <c r="K51" s="23">
-        <f>IF(E51&gt;0, F51/E51, 0)</f>
-        <v/>
-      </c>
-      <c r="L51" s="21">
-        <f>IF(K51&gt;=1, "SUPERADO", "EN CURSO")</f>
+      <c r="D52" s="35" t="inlineStr"/>
+      <c r="E52" s="22">
+        <f>SUM(E10:E51)</f>
+        <v/>
+      </c>
+      <c r="F52" s="22">
+        <f>SUM(F10:F51)</f>
+        <v/>
+      </c>
+      <c r="G52" s="22">
+        <f>SUM(G10:G51)</f>
+        <v/>
+      </c>
+      <c r="H52" s="22">
+        <f>SUM(H10:H51)</f>
+        <v/>
+      </c>
+      <c r="I52" s="22">
+        <f>SUM(I10:I51)</f>
+        <v/>
+      </c>
+      <c r="J52" s="22">
+        <f>SUM(J10:J51)</f>
+        <v/>
+      </c>
+      <c r="K52" s="23">
+        <f>IF(E52&gt;0, F52/E52, 0)</f>
+        <v/>
+      </c>
+      <c r="L52" s="21">
+        <f>IF(K52&gt;=1, "SUPERADO", "EN CURSO")</f>
         <v/>
       </c>
     </row>
@@ -6282,7 +6466,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 23/10/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 26/10/2026</t>
         </is>
       </c>
     </row>
@@ -6331,13 +6515,13 @@
         </is>
       </c>
       <c r="E6" s="4" t="n"/>
-      <c r="F6" s="39" t="inlineStr">
+      <c r="F6" s="38" t="inlineStr">
         <is>
           <t>79.3%</t>
         </is>
       </c>
       <c r="G6" s="4" t="n"/>
-      <c r="H6" s="39" t="inlineStr">
+      <c r="H6" s="38" t="inlineStr">
         <is>
           <t>3,540 u</t>
         </is>
@@ -6454,7 +6638,7 @@
         <f>IF(E10&gt;0, F10/E10, IF(F10&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L10" s="33" t="inlineStr">
+      <c r="L10" s="29" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -6500,7 +6684,7 @@
         <f>IF(E11&gt;0, F11/E11, IF(F11&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L11" s="34" t="inlineStr">
+      <c r="L11" s="32" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -6546,7 +6730,7 @@
         <f>IF(E12&gt;0, F12/E12, IF(F12&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L12" s="33" t="inlineStr">
+      <c r="L12" s="29" t="inlineStr">
         <is>
           <t>Superado</t>
         </is>
@@ -6592,7 +6776,7 @@
         <f>IF(E13&gt;0, F13/E13, IF(F13&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L13" s="34" t="inlineStr">
+      <c r="L13" s="32" t="inlineStr">
         <is>
           <t>Superado</t>
         </is>
@@ -6638,7 +6822,7 @@
         <f>IF(E14&gt;0, F14/E14, IF(F14&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L14" s="33" t="inlineStr">
+      <c r="L14" s="29" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -6684,7 +6868,7 @@
         <f>IF(E15&gt;0, F15/E15, IF(F15&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L15" s="34" t="inlineStr">
+      <c r="L15" s="32" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -6776,7 +6960,7 @@
         <f>IF(E17&gt;0, F17/E17, IF(F17&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L17" s="34" t="inlineStr">
+      <c r="L17" s="32" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -6822,7 +7006,7 @@
         <f>IF(E18&gt;0, F18/E18, IF(F18&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L18" s="33" t="inlineStr">
+      <c r="L18" s="29" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -6868,7 +7052,7 @@
         <f>IF(E19&gt;0, F19/E19, IF(F19&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L19" s="34" t="inlineStr">
+      <c r="L19" s="32" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -6914,7 +7098,7 @@
         <f>IF(E20&gt;0, F20/E20, IF(F20&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L20" s="33" t="inlineStr">
+      <c r="L20" s="29" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -6960,7 +7144,7 @@
         <f>IF(E21&gt;0, F21/E21, IF(F21&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L21" s="38" t="inlineStr">
+      <c r="L21" s="36" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -7006,7 +7190,7 @@
         <f>IF(E22&gt;0, F22/E22, IF(F22&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L22" s="35" t="inlineStr">
+      <c r="L22" s="33" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -7052,7 +7236,7 @@
         <f>IF(E23&gt;0, F23/E23, IF(F23&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L23" s="34" t="inlineStr">
+      <c r="L23" s="32" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -7098,7 +7282,7 @@
         <f>IF(E24&gt;0, F24/E24, IF(F24&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L24" s="33" t="inlineStr">
+      <c r="L24" s="29" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -7144,7 +7328,7 @@
         <f>IF(E25&gt;0, F25/E25, IF(F25&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L25" s="34" t="inlineStr">
+      <c r="L25" s="32" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -7190,7 +7374,7 @@
         <f>IF(E26&gt;0, F26/E26, IF(F26&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L26" s="33" t="inlineStr">
+      <c r="L26" s="29" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -7236,7 +7420,7 @@
         <f>IF(E27&gt;0, F27/E27, IF(F27&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L27" s="34" t="inlineStr">
+      <c r="L27" s="32" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -7282,7 +7466,7 @@
         <f>IF(E28&gt;0, F28/E28, IF(F28&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L28" s="33" t="inlineStr">
+      <c r="L28" s="29" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -7328,7 +7512,7 @@
         <f>IF(E29&gt;0, F29/E29, IF(F29&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L29" s="34" t="inlineStr">
+      <c r="L29" s="32" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -7374,7 +7558,7 @@
         <f>IF(E30&gt;0, F30/E30, IF(F30&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L30" s="33" t="inlineStr">
+      <c r="L30" s="29" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -7420,7 +7604,7 @@
         <f>IF(E31&gt;0, F31/E31, IF(F31&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L31" s="38" t="inlineStr">
+      <c r="L31" s="36" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -7466,7 +7650,7 @@
         <f>IF(E32&gt;0, F32/E32, IF(F32&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L32" s="35" t="inlineStr">
+      <c r="L32" s="33" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -7478,12 +7662,12 @@
           <t>TOTAL JAVIER</t>
         </is>
       </c>
-      <c r="C33" s="36" t="inlineStr">
+      <c r="C33" s="34" t="inlineStr">
         <is>
           <t>179 líneas</t>
         </is>
       </c>
-      <c r="D33" s="37" t="inlineStr"/>
+      <c r="D33" s="35" t="inlineStr"/>
       <c r="E33" s="22">
         <f>SUM(E10:E32)</f>
         <v/>
@@ -7569,7 +7753,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 23/10/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 26/10/2026</t>
         </is>
       </c>
     </row>
@@ -7618,13 +7802,13 @@
         </is>
       </c>
       <c r="E6" s="4" t="n"/>
-      <c r="F6" s="39" t="inlineStr">
+      <c r="F6" s="38" t="inlineStr">
         <is>
           <t>0.0%</t>
         </is>
       </c>
       <c r="G6" s="4" t="n"/>
-      <c r="H6" s="39" t="inlineStr">
+      <c r="H6" s="38" t="inlineStr">
         <is>
           <t>39,460 u</t>
         </is>
@@ -7741,7 +7925,7 @@
         <f>IF(E10&gt;0, F10/E10, IF(F10&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L10" s="35" t="inlineStr">
+      <c r="L10" s="33" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -7787,7 +7971,7 @@
         <f>IF(E11&gt;0, F11/E11, IF(F11&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L11" s="38" t="inlineStr">
+      <c r="L11" s="36" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -7833,7 +8017,7 @@
         <f>IF(E12&gt;0, F12/E12, IF(F12&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L12" s="35" t="inlineStr">
+      <c r="L12" s="33" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -7879,7 +8063,7 @@
         <f>IF(E13&gt;0, F13/E13, IF(F13&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L13" s="38" t="inlineStr">
+      <c r="L13" s="36" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -7925,7 +8109,7 @@
         <f>IF(E14&gt;0, F14/E14, IF(F14&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L14" s="35" t="inlineStr">
+      <c r="L14" s="33" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -7971,7 +8155,7 @@
         <f>IF(E15&gt;0, F15/E15, IF(F15&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L15" s="38" t="inlineStr">
+      <c r="L15" s="36" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -7983,12 +8167,12 @@
           <t>TOTAL MEHMET</t>
         </is>
       </c>
-      <c r="C16" s="36" t="inlineStr">
+      <c r="C16" s="34" t="inlineStr">
         <is>
           <t>61 líneas</t>
         </is>
       </c>
-      <c r="D16" s="37" t="inlineStr"/>
+      <c r="D16" s="35" t="inlineStr"/>
       <c r="E16" s="22">
         <f>SUM(E10:E15)</f>
         <v/>
@@ -8074,7 +8258,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 23/10/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 26/10/2026</t>
         </is>
       </c>
     </row>
@@ -8246,7 +8430,7 @@
         <f>IF(E10&gt;0, F10/E10, IF(F10&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L10" s="33" t="inlineStr">
+      <c r="L10" s="29" t="inlineStr">
         <is>
           <t>Superado</t>
         </is>
@@ -8292,7 +8476,7 @@
         <f>IF(E11&gt;0, F11/E11, IF(F11&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L11" s="38" t="inlineStr">
+      <c r="L11" s="36" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -8338,7 +8522,7 @@
         <f>IF(E12&gt;0, F12/E12, IF(F12&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L12" s="35" t="inlineStr">
+      <c r="L12" s="33" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -8384,7 +8568,7 @@
         <f>IF(E13&gt;0, F13/E13, IF(F13&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L13" s="32" t="inlineStr">
+      <c r="L13" s="37" t="inlineStr">
         <is>
           <t>En Curso</t>
         </is>
@@ -8430,7 +8614,7 @@
         <f>IF(E14&gt;0, F14/E14, IF(F14&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L14" s="33" t="inlineStr">
+      <c r="L14" s="29" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -8522,7 +8706,7 @@
         <f>IF(E16&gt;0, F16/E16, IF(F16&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L16" s="35" t="inlineStr">
+      <c r="L16" s="33" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -8568,7 +8752,7 @@
         <f>IF(E17&gt;0, F17/E17, IF(F17&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L17" s="38" t="inlineStr">
+      <c r="L17" s="36" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -8614,7 +8798,7 @@
         <f>IF(E18&gt;0, F18/E18, IF(F18&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L18" s="33" t="inlineStr">
+      <c r="L18" s="29" t="inlineStr">
         <is>
           <t>Superado</t>
         </is>
@@ -8660,7 +8844,7 @@
         <f>IF(E19&gt;0, F19/E19, IF(F19&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L19" s="34" t="inlineStr">
+      <c r="L19" s="32" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -8706,7 +8890,7 @@
         <f>IF(E20&gt;0, F20/E20, IF(F20&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L20" s="33" t="inlineStr">
+      <c r="L20" s="29" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -8752,7 +8936,7 @@
         <f>IF(E21&gt;0, F21/E21, IF(F21&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L21" s="34" t="inlineStr">
+      <c r="L21" s="32" t="inlineStr">
         <is>
           <t>Superado</t>
         </is>
@@ -8798,7 +8982,7 @@
         <f>IF(E22&gt;0, F22/E22, IF(F22&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L22" s="33" t="inlineStr">
+      <c r="L22" s="29" t="inlineStr">
         <is>
           <t>Superado</t>
         </is>
@@ -8844,7 +9028,7 @@
         <f>IF(E23&gt;0, F23/E23, IF(F23&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L23" s="38" t="inlineStr">
+      <c r="L23" s="36" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -8890,7 +9074,7 @@
         <f>IF(E24&gt;0, F24/E24, IF(F24&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L24" s="29" t="inlineStr">
+      <c r="L24" s="39" t="inlineStr">
         <is>
           <t>En Curso</t>
         </is>
@@ -8936,7 +9120,7 @@
         <f>IF(E25&gt;0, F25/E25, IF(F25&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L25" s="34" t="inlineStr">
+      <c r="L25" s="32" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -8982,7 +9166,7 @@
         <f>IF(E26&gt;0, F26/E26, IF(F26&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L26" s="33" t="inlineStr">
+      <c r="L26" s="29" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -8994,12 +9178,12 @@
           <t>TOTAL PEDRO</t>
         </is>
       </c>
-      <c r="C27" s="36" t="inlineStr">
+      <c r="C27" s="34" t="inlineStr">
         <is>
           <t>104 líneas</t>
         </is>
       </c>
-      <c r="D27" s="37" t="inlineStr"/>
+      <c r="D27" s="35" t="inlineStr"/>
       <c r="E27" s="22">
         <f>SUM(E10:E26)</f>
         <v/>
@@ -9058,7 +9242,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:L45"/>
+  <dimension ref="B2:L47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -9085,7 +9269,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 23/10/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 26/10/2026</t>
         </is>
       </c>
     </row>
@@ -9130,13 +9314,13 @@
       <c r="C6" s="4" t="n"/>
       <c r="D6" s="25" t="inlineStr">
         <is>
-          <t>102,472 u</t>
+          <t>109,072 u</t>
         </is>
       </c>
       <c r="E6" s="4" t="n"/>
       <c r="F6" s="25" t="inlineStr">
         <is>
-          <t>222.8%</t>
+          <t>237.1%</t>
         </is>
       </c>
       <c r="G6" s="4" t="n"/>
@@ -9148,7 +9332,7 @@
       <c r="I6" s="4" t="n"/>
       <c r="J6" s="24" t="inlineStr">
         <is>
-          <t>102,472 u</t>
+          <t>109,072 u</t>
         </is>
       </c>
       <c r="K6" s="4" t="n"/>
@@ -9220,30 +9404,30 @@
     <row r="10">
       <c r="B10" s="27" t="inlineStr">
         <is>
-          <t>EUROFERTIL, S.A.</t>
+          <t>ECUAQUIMICA</t>
         </is>
       </c>
       <c r="C10" s="28" t="inlineStr">
         <is>
-          <t>F-A1000</t>
+          <t>AN0005</t>
         </is>
       </c>
       <c r="D10" s="27" t="inlineStr">
         <is>
-          <t>FITOLIN AGRO</t>
+          <t>ALCAPLANT NEW</t>
         </is>
       </c>
       <c r="E10" s="14" t="n">
-        <v>2000</v>
+        <v>0</v>
       </c>
       <c r="F10" s="14" t="n">
-        <v>0</v>
+        <v>2200</v>
       </c>
       <c r="G10" s="14" t="n">
         <v>0</v>
       </c>
       <c r="H10" s="14" t="n">
-        <v>0</v>
+        <v>2200</v>
       </c>
       <c r="I10" s="14">
         <f>MAX(0, E10-F10)</f>
@@ -9257,39 +9441,39 @@
         <f>IF(E10&gt;0, F10/E10, IF(F10&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L10" s="35" t="inlineStr">
-        <is>
-          <t>Sin Pedido</t>
+      <c r="L10" s="29" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="B11" s="30" t="inlineStr">
         <is>
-          <t xml:space="preserve">EUROFERTIL, S.A.    </t>
+          <t>ECUAQUIMICA</t>
         </is>
       </c>
       <c r="C11" s="31" t="inlineStr">
         <is>
-          <t>AGXCR1000</t>
+          <t>AN0020</t>
         </is>
       </c>
       <c r="D11" s="30" t="inlineStr">
         <is>
-          <t>AGROXILATO-K, 1000 L</t>
+          <t>ALCAPLANT NEW</t>
         </is>
       </c>
       <c r="E11" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F11" s="18" t="n">
-        <v>4000</v>
+        <v>4400</v>
       </c>
       <c r="G11" s="18" t="n">
         <v>0</v>
       </c>
       <c r="H11" s="18" t="n">
-        <v>4000</v>
+        <v>4400</v>
       </c>
       <c r="I11" s="18">
         <f>MAX(0, E11-F11)</f>
@@ -9303,7 +9487,7 @@
         <f>IF(E11&gt;0, F11/E11, IF(F11&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L11" s="34" t="inlineStr">
+      <c r="L11" s="32" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -9312,30 +9496,30 @@
     <row r="12">
       <c r="B12" s="27" t="inlineStr">
         <is>
-          <t xml:space="preserve">EUROFERTIL, S.A.    </t>
+          <t>EUROFERTIL, S.A.</t>
         </is>
       </c>
       <c r="C12" s="28" t="inlineStr">
         <is>
-          <t>AN0020</t>
+          <t>F-A1000</t>
         </is>
       </c>
       <c r="D12" s="27" t="inlineStr">
         <is>
-          <t>ALCAPLANT, 20 KG</t>
+          <t>FITOLIN AGRO</t>
         </is>
       </c>
       <c r="E12" s="14" t="n">
-        <v>0</v>
+        <v>2000</v>
       </c>
       <c r="F12" s="14" t="n">
-        <v>22000</v>
+        <v>0</v>
       </c>
       <c r="G12" s="14" t="n">
         <v>0</v>
       </c>
       <c r="H12" s="14" t="n">
-        <v>22000</v>
+        <v>0</v>
       </c>
       <c r="I12" s="14">
         <f>MAX(0, E12-F12)</f>
@@ -9351,7 +9535,7 @@
       </c>
       <c r="L12" s="33" t="inlineStr">
         <is>
-          <t>Extra Estimación</t>
+          <t>Sin Pedido</t>
         </is>
       </c>
     </row>
@@ -9363,25 +9547,25 @@
       </c>
       <c r="C13" s="31" t="inlineStr">
         <is>
-          <t>B1000</t>
+          <t>AGXCR1000</t>
         </is>
       </c>
       <c r="D13" s="30" t="inlineStr">
         <is>
-          <t>FORTALEZA, 1000 L</t>
+          <t>AGROXILATO-K, 1000 L</t>
         </is>
       </c>
       <c r="E13" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F13" s="18" t="n">
-        <v>2000</v>
+        <v>4000</v>
       </c>
       <c r="G13" s="18" t="n">
         <v>0</v>
       </c>
       <c r="H13" s="18" t="n">
-        <v>2000</v>
+        <v>4000</v>
       </c>
       <c r="I13" s="18">
         <f>MAX(0, E13-F13)</f>
@@ -9395,7 +9579,7 @@
         <f>IF(E13&gt;0, F13/E13, IF(F13&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L13" s="34" t="inlineStr">
+      <c r="L13" s="32" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -9409,25 +9593,25 @@
       </c>
       <c r="C14" s="28" t="inlineStr">
         <is>
-          <t>C-CU1000</t>
+          <t>AN0020</t>
         </is>
       </c>
       <c r="D14" s="27" t="inlineStr">
         <is>
-          <t>CODICOBRE, 1000 L</t>
+          <t>ALCAPLANT, 20 KG</t>
         </is>
       </c>
       <c r="E14" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F14" s="14" t="n">
-        <v>1000</v>
+        <v>22000</v>
       </c>
       <c r="G14" s="14" t="n">
         <v>0</v>
       </c>
       <c r="H14" s="14" t="n">
-        <v>1000</v>
+        <v>22000</v>
       </c>
       <c r="I14" s="14">
         <f>MAX(0, E14-F14)</f>
@@ -9441,7 +9625,7 @@
         <f>IF(E14&gt;0, F14/E14, IF(F14&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L14" s="33" t="inlineStr">
+      <c r="L14" s="29" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -9455,25 +9639,25 @@
       </c>
       <c r="C15" s="31" t="inlineStr">
         <is>
-          <t>CODIR1000</t>
+          <t>B1000</t>
         </is>
       </c>
       <c r="D15" s="30" t="inlineStr">
         <is>
-          <t>CODIRESIST, 1000 L</t>
+          <t>FORTALEZA, 1000 L</t>
         </is>
       </c>
       <c r="E15" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F15" s="18" t="n">
-        <v>1000</v>
+        <v>2000</v>
       </c>
       <c r="G15" s="18" t="n">
         <v>0</v>
       </c>
       <c r="H15" s="18" t="n">
-        <v>1000</v>
+        <v>2000</v>
       </c>
       <c r="I15" s="18">
         <f>MAX(0, E15-F15)</f>
@@ -9487,7 +9671,7 @@
         <f>IF(E15&gt;0, F15/E15, IF(F15&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L15" s="34" t="inlineStr">
+      <c r="L15" s="32" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -9501,25 +9685,25 @@
       </c>
       <c r="C16" s="28" t="inlineStr">
         <is>
-          <t>DECA0005</t>
+          <t>C-CU1000</t>
         </is>
       </c>
       <c r="D16" s="27" t="inlineStr">
         <is>
-          <t>DEFENS-CA-AE, 5 KG</t>
+          <t>CODICOBRE, 1000 L</t>
         </is>
       </c>
       <c r="E16" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F16" s="14" t="n">
-        <v>2200</v>
+        <v>1000</v>
       </c>
       <c r="G16" s="14" t="n">
         <v>0</v>
       </c>
       <c r="H16" s="14" t="n">
-        <v>2200</v>
+        <v>1000</v>
       </c>
       <c r="I16" s="14">
         <f>MAX(0, E16-F16)</f>
@@ -9533,7 +9717,7 @@
         <f>IF(E16&gt;0, F16/E16, IF(F16&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L16" s="33" t="inlineStr">
+      <c r="L16" s="29" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -9547,25 +9731,25 @@
       </c>
       <c r="C17" s="31" t="inlineStr">
         <is>
-          <t>FLORCR1000</t>
+          <t>CODIR1000</t>
         </is>
       </c>
       <c r="D17" s="30" t="inlineStr">
         <is>
-          <t>FLORAMEC, 1000 L</t>
+          <t>CODIRESIST, 1000 L</t>
         </is>
       </c>
       <c r="E17" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F17" s="18" t="n">
-        <v>2000</v>
+        <v>1000</v>
       </c>
       <c r="G17" s="18" t="n">
         <v>0</v>
       </c>
       <c r="H17" s="18" t="n">
-        <v>2000</v>
+        <v>1000</v>
       </c>
       <c r="I17" s="18">
         <f>MAX(0, E17-F17)</f>
@@ -9579,7 +9763,7 @@
         <f>IF(E17&gt;0, F17/E17, IF(F17&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L17" s="34" t="inlineStr">
+      <c r="L17" s="32" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -9593,25 +9777,25 @@
       </c>
       <c r="C18" s="28" t="inlineStr">
         <is>
-          <t>G1000</t>
+          <t>DECA0005</t>
         </is>
       </c>
       <c r="D18" s="27" t="inlineStr">
         <is>
-          <t>TRANSLOCADOR, 1000 L</t>
+          <t>DEFENS-CA-AE, 5 KG</t>
         </is>
       </c>
       <c r="E18" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F18" s="14" t="n">
-        <v>1000</v>
+        <v>2200</v>
       </c>
       <c r="G18" s="14" t="n">
         <v>0</v>
       </c>
       <c r="H18" s="14" t="n">
-        <v>1000</v>
+        <v>2200</v>
       </c>
       <c r="I18" s="14">
         <f>MAX(0, E18-F18)</f>
@@ -9625,7 +9809,7 @@
         <f>IF(E18&gt;0, F18/E18, IF(F18&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L18" s="33" t="inlineStr">
+      <c r="L18" s="29" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -9639,12 +9823,12 @@
       </c>
       <c r="C19" s="31" t="inlineStr">
         <is>
-          <t>NB1000</t>
+          <t>FLORCR1000</t>
         </is>
       </c>
       <c r="D19" s="30" t="inlineStr">
         <is>
-          <t>NITROBALANCE, 1000 L</t>
+          <t>FLORAMEC, 1000 L</t>
         </is>
       </c>
       <c r="E19" s="18" t="n">
@@ -9671,7 +9855,7 @@
         <f>IF(E19&gt;0, F19/E19, IF(F19&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L19" s="34" t="inlineStr">
+      <c r="L19" s="32" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -9685,25 +9869,25 @@
       </c>
       <c r="C20" s="28" t="inlineStr">
         <is>
-          <t>PT1000</t>
+          <t>G1000</t>
         </is>
       </c>
       <c r="D20" s="27" t="inlineStr">
         <is>
-          <t>POTASION PLUS, 1000 L</t>
+          <t>TRANSLOCADOR, 1000 L</t>
         </is>
       </c>
       <c r="E20" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F20" s="14" t="n">
-        <v>4000</v>
+        <v>1000</v>
       </c>
       <c r="G20" s="14" t="n">
         <v>0</v>
       </c>
       <c r="H20" s="14" t="n">
-        <v>4000</v>
+        <v>1000</v>
       </c>
       <c r="I20" s="14">
         <f>MAX(0, E20-F20)</f>
@@ -9717,7 +9901,7 @@
         <f>IF(E20&gt;0, F20/E20, IF(F20&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L20" s="33" t="inlineStr">
+      <c r="L20" s="29" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -9731,25 +9915,25 @@
       </c>
       <c r="C21" s="31" t="inlineStr">
         <is>
-          <t>SS0020</t>
+          <t>NB1000</t>
         </is>
       </c>
       <c r="D21" s="30" t="inlineStr">
         <is>
-          <t>SAL WAX MAX, 20 KG</t>
+          <t>NITROBALANCE, 1000 L</t>
         </is>
       </c>
       <c r="E21" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F21" s="18" t="n">
-        <v>640</v>
+        <v>2000</v>
       </c>
       <c r="G21" s="18" t="n">
         <v>0</v>
       </c>
       <c r="H21" s="18" t="n">
-        <v>640</v>
+        <v>2000</v>
       </c>
       <c r="I21" s="18">
         <f>MAX(0, E21-F21)</f>
@@ -9763,7 +9947,7 @@
         <f>IF(E21&gt;0, F21/E21, IF(F21&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L21" s="34" t="inlineStr">
+      <c r="L21" s="32" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -9772,30 +9956,30 @@
     <row r="22">
       <c r="B22" s="27" t="inlineStr">
         <is>
-          <t>JUAN JIMENEZ, SRL</t>
+          <t xml:space="preserve">EUROFERTIL, S.A.    </t>
         </is>
       </c>
       <c r="C22" s="28" t="inlineStr">
         <is>
-          <t>A-50(2)0001</t>
+          <t>PT1000</t>
         </is>
       </c>
       <c r="D22" s="27" t="inlineStr">
         <is>
-          <t>CODIORGAN A-50</t>
+          <t>POTASION PLUS, 1000 L</t>
         </is>
       </c>
       <c r="E22" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F22" s="14" t="n">
-        <v>2448</v>
+        <v>4000</v>
       </c>
       <c r="G22" s="14" t="n">
         <v>0</v>
       </c>
       <c r="H22" s="14" t="n">
-        <v>2448</v>
+        <v>4000</v>
       </c>
       <c r="I22" s="14">
         <f>MAX(0, E22-F22)</f>
@@ -9809,7 +9993,7 @@
         <f>IF(E22&gt;0, F22/E22, IF(F22&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L22" s="33" t="inlineStr">
+      <c r="L22" s="29" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -9818,30 +10002,30 @@
     <row r="23">
       <c r="B23" s="30" t="inlineStr">
         <is>
-          <t>JUAN JIMENEZ, SRL</t>
+          <t xml:space="preserve">EUROFERTIL, S.A.    </t>
         </is>
       </c>
       <c r="C23" s="31" t="inlineStr">
         <is>
-          <t>AGXK0001</t>
+          <t>SS0020</t>
         </is>
       </c>
       <c r="D23" s="30" t="inlineStr">
         <is>
-          <t>AGROXILATO-K</t>
+          <t>SAL WAX MAX, 20 KG</t>
         </is>
       </c>
       <c r="E23" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F23" s="18" t="n">
-        <v>1788</v>
+        <v>640</v>
       </c>
       <c r="G23" s="18" t="n">
         <v>0</v>
       </c>
       <c r="H23" s="18" t="n">
-        <v>1788</v>
+        <v>640</v>
       </c>
       <c r="I23" s="18">
         <f>MAX(0, E23-F23)</f>
@@ -9855,7 +10039,7 @@
         <f>IF(E23&gt;0, F23/E23, IF(F23&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L23" s="34" t="inlineStr">
+      <c r="L23" s="32" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -9869,25 +10053,25 @@
       </c>
       <c r="C24" s="28" t="inlineStr">
         <is>
-          <t>AN0005</t>
+          <t>A-50(2)0001</t>
         </is>
       </c>
       <c r="D24" s="27" t="inlineStr">
         <is>
-          <t>ALCAPLANT NEW</t>
+          <t>CODIORGAN A-50</t>
         </is>
       </c>
       <c r="E24" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F24" s="14" t="n">
-        <v>1800</v>
+        <v>2448</v>
       </c>
       <c r="G24" s="14" t="n">
         <v>0</v>
       </c>
       <c r="H24" s="14" t="n">
-        <v>1800</v>
+        <v>2448</v>
       </c>
       <c r="I24" s="14">
         <f>MAX(0, E24-F24)</f>
@@ -9901,7 +10085,7 @@
         <f>IF(E24&gt;0, F24/E24, IF(F24&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L24" s="33" t="inlineStr">
+      <c r="L24" s="29" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -9915,25 +10099,25 @@
       </c>
       <c r="C25" s="31" t="inlineStr">
         <is>
-          <t>B0001</t>
+          <t>AGXK0001</t>
         </is>
       </c>
       <c r="D25" s="30" t="inlineStr">
         <is>
-          <t>BOROCAL</t>
+          <t>AGROXILATO-K</t>
         </is>
       </c>
       <c r="E25" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F25" s="18" t="n">
-        <v>2808</v>
+        <v>1788</v>
       </c>
       <c r="G25" s="18" t="n">
         <v>0</v>
       </c>
       <c r="H25" s="18" t="n">
-        <v>2808</v>
+        <v>1788</v>
       </c>
       <c r="I25" s="18">
         <f>MAX(0, E25-F25)</f>
@@ -9947,7 +10131,7 @@
         <f>IF(E25&gt;0, F25/E25, IF(F25&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L25" s="34" t="inlineStr">
+      <c r="L25" s="32" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -9961,25 +10145,25 @@
       </c>
       <c r="C26" s="28" t="inlineStr">
         <is>
-          <t>BEY0001</t>
+          <t>AN0005</t>
         </is>
       </c>
       <c r="D26" s="27" t="inlineStr">
         <is>
-          <t>BERRY-FLOR, 1 L</t>
+          <t>ALCAPLANT NEW</t>
         </is>
       </c>
       <c r="E26" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F26" s="14" t="n">
-        <v>36</v>
+        <v>1800</v>
       </c>
       <c r="G26" s="14" t="n">
         <v>0</v>
       </c>
       <c r="H26" s="14" t="n">
-        <v>36</v>
+        <v>1800</v>
       </c>
       <c r="I26" s="14">
         <f>MAX(0, E26-F26)</f>
@@ -9993,7 +10177,7 @@
         <f>IF(E26&gt;0, F26/E26, IF(F26&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L26" s="33" t="inlineStr">
+      <c r="L26" s="29" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -10007,25 +10191,25 @@
       </c>
       <c r="C27" s="31" t="inlineStr">
         <is>
-          <t>BIO0001</t>
+          <t>B0001</t>
         </is>
       </c>
       <c r="D27" s="30" t="inlineStr">
         <is>
-          <t>BIORAD-20</t>
+          <t>BOROCAL</t>
         </is>
       </c>
       <c r="E27" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F27" s="18" t="n">
-        <v>2892</v>
+        <v>2808</v>
       </c>
       <c r="G27" s="18" t="n">
         <v>0</v>
       </c>
       <c r="H27" s="18" t="n">
-        <v>2892</v>
+        <v>2808</v>
       </c>
       <c r="I27" s="18">
         <f>MAX(0, E27-F27)</f>
@@ -10039,7 +10223,7 @@
         <f>IF(E27&gt;0, F27/E27, IF(F27&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L27" s="34" t="inlineStr">
+      <c r="L27" s="32" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -10053,25 +10237,25 @@
       </c>
       <c r="C28" s="28" t="inlineStr">
         <is>
-          <t>BIO0005</t>
+          <t>BEY0001</t>
         </is>
       </c>
       <c r="D28" s="27" t="inlineStr">
         <is>
-          <t>BIORAD-20</t>
+          <t>BERRY-FLOR, 1 L</t>
         </is>
       </c>
       <c r="E28" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F28" s="14" t="n">
-        <v>3900</v>
+        <v>36</v>
       </c>
       <c r="G28" s="14" t="n">
         <v>0</v>
       </c>
       <c r="H28" s="14" t="n">
-        <v>3900</v>
+        <v>36</v>
       </c>
       <c r="I28" s="14">
         <f>MAX(0, E28-F28)</f>
@@ -10085,7 +10269,7 @@
         <f>IF(E28&gt;0, F28/E28, IF(F28&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L28" s="33" t="inlineStr">
+      <c r="L28" s="29" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -10099,7 +10283,7 @@
       </c>
       <c r="C29" s="31" t="inlineStr">
         <is>
-          <t>BIO0020</t>
+          <t>BIO0001</t>
         </is>
       </c>
       <c r="D29" s="30" t="inlineStr">
@@ -10111,13 +10295,13 @@
         <v>0</v>
       </c>
       <c r="F29" s="18" t="n">
-        <v>6400</v>
+        <v>2892</v>
       </c>
       <c r="G29" s="18" t="n">
         <v>0</v>
       </c>
       <c r="H29" s="18" t="n">
-        <v>6400</v>
+        <v>2892</v>
       </c>
       <c r="I29" s="18">
         <f>MAX(0, E29-F29)</f>
@@ -10131,7 +10315,7 @@
         <f>IF(E29&gt;0, F29/E29, IF(F29&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L29" s="34" t="inlineStr">
+      <c r="L29" s="32" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -10145,25 +10329,25 @@
       </c>
       <c r="C30" s="28" t="inlineStr">
         <is>
-          <t>BR-590005</t>
+          <t>BIO0005</t>
         </is>
       </c>
       <c r="D30" s="27" t="inlineStr">
         <is>
-          <t>BR-59, 5 KG</t>
+          <t>BIORAD-20</t>
         </is>
       </c>
       <c r="E30" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F30" s="14" t="n">
-        <v>480</v>
+        <v>3900</v>
       </c>
       <c r="G30" s="14" t="n">
         <v>0</v>
       </c>
       <c r="H30" s="14" t="n">
-        <v>480</v>
+        <v>3900</v>
       </c>
       <c r="I30" s="14">
         <f>MAX(0, E30-F30)</f>
@@ -10177,7 +10361,7 @@
         <f>IF(E30&gt;0, F30/E30, IF(F30&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L30" s="33" t="inlineStr">
+      <c r="L30" s="29" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -10191,25 +10375,25 @@
       </c>
       <c r="C31" s="31" t="inlineStr">
         <is>
-          <t>C-CU0001</t>
+          <t>BIO0020</t>
         </is>
       </c>
       <c r="D31" s="30" t="inlineStr">
         <is>
-          <t>CODICOBRE</t>
+          <t>BIORAD-20</t>
         </is>
       </c>
       <c r="E31" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F31" s="18" t="n">
-        <v>1200</v>
+        <v>6400</v>
       </c>
       <c r="G31" s="18" t="n">
         <v>0</v>
       </c>
       <c r="H31" s="18" t="n">
-        <v>1200</v>
+        <v>6400</v>
       </c>
       <c r="I31" s="18">
         <f>MAX(0, E31-F31)</f>
@@ -10223,7 +10407,7 @@
         <f>IF(E31&gt;0, F31/E31, IF(F31&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L31" s="34" t="inlineStr">
+      <c r="L31" s="32" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -10237,25 +10421,25 @@
       </c>
       <c r="C32" s="28" t="inlineStr">
         <is>
-          <t>C-L0001</t>
+          <t>BR-590005</t>
         </is>
       </c>
       <c r="D32" s="27" t="inlineStr">
         <is>
-          <t>CODIBOR-L, 1 L</t>
+          <t>BR-59, 5 KG</t>
         </is>
       </c>
       <c r="E32" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F32" s="14" t="n">
-        <v>84</v>
+        <v>480</v>
       </c>
       <c r="G32" s="14" t="n">
         <v>0</v>
       </c>
       <c r="H32" s="14" t="n">
-        <v>84</v>
+        <v>480</v>
       </c>
       <c r="I32" s="14">
         <f>MAX(0, E32-F32)</f>
@@ -10269,7 +10453,7 @@
         <f>IF(E32&gt;0, F32/E32, IF(F32&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L32" s="33" t="inlineStr">
+      <c r="L32" s="29" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -10283,25 +10467,25 @@
       </c>
       <c r="C33" s="31" t="inlineStr">
         <is>
-          <t>F-A0001</t>
+          <t>C-CU0001</t>
         </is>
       </c>
       <c r="D33" s="30" t="inlineStr">
         <is>
-          <t>FITOLIN-AGRO</t>
+          <t>CODICOBRE</t>
         </is>
       </c>
       <c r="E33" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F33" s="18" t="n">
-        <v>984</v>
+        <v>1200</v>
       </c>
       <c r="G33" s="18" t="n">
         <v>0</v>
       </c>
       <c r="H33" s="18" t="n">
-        <v>984</v>
+        <v>1200</v>
       </c>
       <c r="I33" s="18">
         <f>MAX(0, E33-F33)</f>
@@ -10315,7 +10499,7 @@
         <f>IF(E33&gt;0, F33/E33, IF(F33&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L33" s="34" t="inlineStr">
+      <c r="L33" s="32" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -10329,25 +10513,25 @@
       </c>
       <c r="C34" s="28" t="inlineStr">
         <is>
-          <t>F-A0005</t>
+          <t>C-L0001</t>
         </is>
       </c>
       <c r="D34" s="27" t="inlineStr">
         <is>
-          <t>FITOLIN-AGRO</t>
+          <t>CODIBOR-L, 1 L</t>
         </is>
       </c>
       <c r="E34" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F34" s="14" t="n">
-        <v>2040</v>
+        <v>84</v>
       </c>
       <c r="G34" s="14" t="n">
         <v>0</v>
       </c>
       <c r="H34" s="14" t="n">
-        <v>2040</v>
+        <v>84</v>
       </c>
       <c r="I34" s="14">
         <f>MAX(0, E34-F34)</f>
@@ -10361,7 +10545,7 @@
         <f>IF(E34&gt;0, F34/E34, IF(F34&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L34" s="33" t="inlineStr">
+      <c r="L34" s="29" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -10375,25 +10559,25 @@
       </c>
       <c r="C35" s="31" t="inlineStr">
         <is>
-          <t>FLOR0001</t>
+          <t>F-A0001</t>
         </is>
       </c>
       <c r="D35" s="30" t="inlineStr">
         <is>
-          <t>FLORAMEC</t>
+          <t>FITOLIN-AGRO</t>
         </is>
       </c>
       <c r="E35" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F35" s="18" t="n">
-        <v>648</v>
+        <v>984</v>
       </c>
       <c r="G35" s="18" t="n">
         <v>0</v>
       </c>
       <c r="H35" s="18" t="n">
-        <v>648</v>
+        <v>984</v>
       </c>
       <c r="I35" s="18">
         <f>MAX(0, E35-F35)</f>
@@ -10407,7 +10591,7 @@
         <f>IF(E35&gt;0, F35/E35, IF(F35&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L35" s="34" t="inlineStr">
+      <c r="L35" s="32" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -10421,25 +10605,25 @@
       </c>
       <c r="C36" s="28" t="inlineStr">
         <is>
-          <t>LP0001</t>
+          <t>F-A0005</t>
         </is>
       </c>
       <c r="D36" s="27" t="inlineStr">
         <is>
-          <t>LAVAPLANT GRANEL</t>
+          <t>FITOLIN-AGRO</t>
         </is>
       </c>
       <c r="E36" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F36" s="14" t="n">
-        <v>1092</v>
+        <v>2040</v>
       </c>
       <c r="G36" s="14" t="n">
         <v>0</v>
       </c>
       <c r="H36" s="14" t="n">
-        <v>1092</v>
+        <v>2040</v>
       </c>
       <c r="I36" s="14">
         <f>MAX(0, E36-F36)</f>
@@ -10453,7 +10637,7 @@
         <f>IF(E36&gt;0, F36/E36, IF(F36&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L36" s="33" t="inlineStr">
+      <c r="L36" s="29" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -10467,25 +10651,25 @@
       </c>
       <c r="C37" s="31" t="inlineStr">
         <is>
-          <t>LP0005</t>
+          <t>FLOR0001</t>
         </is>
       </c>
       <c r="D37" s="30" t="inlineStr">
         <is>
-          <t>LAVAPLANT, 5 L</t>
+          <t>FLORAMEC</t>
         </is>
       </c>
       <c r="E37" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F37" s="18" t="n">
-        <v>1160</v>
+        <v>648</v>
       </c>
       <c r="G37" s="18" t="n">
         <v>0</v>
       </c>
       <c r="H37" s="18" t="n">
-        <v>1160</v>
+        <v>648</v>
       </c>
       <c r="I37" s="18">
         <f>MAX(0, E37-F37)</f>
@@ -10499,7 +10683,7 @@
         <f>IF(E37&gt;0, F37/E37, IF(F37&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L37" s="34" t="inlineStr">
+      <c r="L37" s="32" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -10513,25 +10697,25 @@
       </c>
       <c r="C38" s="28" t="inlineStr">
         <is>
-          <t>PT0001</t>
+          <t>LP0001</t>
         </is>
       </c>
       <c r="D38" s="27" t="inlineStr">
         <is>
-          <t>AGROPOTASION</t>
+          <t>LAVAPLANT GRANEL</t>
         </is>
       </c>
       <c r="E38" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F38" s="14" t="n">
-        <v>2520</v>
+        <v>1092</v>
       </c>
       <c r="G38" s="14" t="n">
         <v>0</v>
       </c>
       <c r="H38" s="14" t="n">
-        <v>2520</v>
+        <v>1092</v>
       </c>
       <c r="I38" s="14">
         <f>MAX(0, E38-F38)</f>
@@ -10545,7 +10729,7 @@
         <f>IF(E38&gt;0, F38/E38, IF(F38&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L38" s="33" t="inlineStr">
+      <c r="L38" s="29" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -10559,25 +10743,25 @@
       </c>
       <c r="C39" s="31" t="inlineStr">
         <is>
-          <t>PT0005</t>
+          <t>LP0005</t>
         </is>
       </c>
       <c r="D39" s="30" t="inlineStr">
         <is>
-          <t>AGROPOTASION, 5 L</t>
+          <t>LAVAPLANT, 5 L</t>
         </is>
       </c>
       <c r="E39" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F39" s="18" t="n">
-        <v>1260</v>
+        <v>1160</v>
       </c>
       <c r="G39" s="18" t="n">
         <v>0</v>
       </c>
       <c r="H39" s="18" t="n">
-        <v>1260</v>
+        <v>1160</v>
       </c>
       <c r="I39" s="18">
         <f>MAX(0, E39-F39)</f>
@@ -10591,7 +10775,7 @@
         <f>IF(E39&gt;0, F39/E39, IF(F39&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L39" s="34" t="inlineStr">
+      <c r="L39" s="32" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -10605,25 +10789,25 @@
       </c>
       <c r="C40" s="28" t="inlineStr">
         <is>
-          <t>SPCE2B0001</t>
+          <t>PT0001</t>
         </is>
       </c>
       <c r="D40" s="27" t="inlineStr">
         <is>
-          <t>SPRINTENE</t>
+          <t>AGROPOTASION</t>
         </is>
       </c>
       <c r="E40" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F40" s="14" t="n">
-        <v>300</v>
+        <v>2520</v>
       </c>
       <c r="G40" s="14" t="n">
         <v>0</v>
       </c>
       <c r="H40" s="14" t="n">
-        <v>300</v>
+        <v>2520</v>
       </c>
       <c r="I40" s="14">
         <f>MAX(0, E40-F40)</f>
@@ -10637,7 +10821,7 @@
         <f>IF(E40&gt;0, F40/E40, IF(F40&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L40" s="33" t="inlineStr">
+      <c r="L40" s="29" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -10651,25 +10835,25 @@
       </c>
       <c r="C41" s="31" t="inlineStr">
         <is>
-          <t>SS0001</t>
+          <t>PT0005</t>
         </is>
       </c>
       <c r="D41" s="30" t="inlineStr">
         <is>
-          <t>SAL-WAX</t>
+          <t>AGROPOTASION, 5 L</t>
         </is>
       </c>
       <c r="E41" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F41" s="18" t="n">
-        <v>1088</v>
+        <v>1260</v>
       </c>
       <c r="G41" s="18" t="n">
         <v>0</v>
       </c>
       <c r="H41" s="18" t="n">
-        <v>1088</v>
+        <v>1260</v>
       </c>
       <c r="I41" s="18">
         <f>MAX(0, E41-F41)</f>
@@ -10683,7 +10867,7 @@
         <f>IF(E41&gt;0, F41/E41, IF(F41&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L41" s="34" t="inlineStr">
+      <c r="L41" s="32" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -10697,25 +10881,25 @@
       </c>
       <c r="C42" s="28" t="inlineStr">
         <is>
-          <t>START20001</t>
+          <t>SPCE2B0001</t>
         </is>
       </c>
       <c r="D42" s="27" t="inlineStr">
         <is>
-          <t>RADISOL</t>
+          <t>SPRINTENE</t>
         </is>
       </c>
       <c r="E42" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F42" s="14" t="n">
-        <v>2904</v>
+        <v>300</v>
       </c>
       <c r="G42" s="14" t="n">
         <v>0</v>
       </c>
       <c r="H42" s="14" t="n">
-        <v>2904</v>
+        <v>300</v>
       </c>
       <c r="I42" s="14">
         <f>MAX(0, E42-F42)</f>
@@ -10729,7 +10913,7 @@
         <f>IF(E42&gt;0, F42/E42, IF(F42&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L42" s="33" t="inlineStr">
+      <c r="L42" s="29" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
@@ -10738,30 +10922,30 @@
     <row r="43">
       <c r="B43" s="30" t="inlineStr">
         <is>
-          <t>LEKKERBIO B.V.</t>
+          <t>JUAN JIMENEZ, SRL</t>
         </is>
       </c>
       <c r="C43" s="31" t="inlineStr">
         <is>
-          <t>AO0020</t>
+          <t>SS0001</t>
         </is>
       </c>
       <c r="D43" s="30" t="inlineStr">
         <is>
-          <t>ALCAPLANT NEW</t>
+          <t>SAL-WAX</t>
         </is>
       </c>
       <c r="E43" s="18" t="n">
-        <v>44000</v>
+        <v>0</v>
       </c>
       <c r="F43" s="18" t="n">
-        <v>19800</v>
+        <v>1088</v>
       </c>
       <c r="G43" s="18" t="n">
         <v>0</v>
       </c>
       <c r="H43" s="18" t="n">
-        <v>19800</v>
+        <v>1088</v>
       </c>
       <c r="I43" s="18">
         <f>MAX(0, E43-F43)</f>
@@ -10775,39 +10959,39 @@
         <f>IF(E43&gt;0, F43/E43, IF(F43&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L43" s="40" t="inlineStr">
-        <is>
-          <t>Rezagado</t>
+      <c r="L43" s="32" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="B44" s="27" t="inlineStr">
         <is>
-          <t>LEKKERBIO B.V.</t>
+          <t>JUAN JIMENEZ, SRL</t>
         </is>
       </c>
       <c r="C44" s="28" t="inlineStr">
         <is>
-          <t>DECA0020</t>
+          <t>START20001</t>
         </is>
       </c>
       <c r="D44" s="27" t="inlineStr">
         <is>
-          <t>DEFENS-CA-AE, 20 KG</t>
+          <t>RADISOL</t>
         </is>
       </c>
       <c r="E44" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F44" s="14" t="n">
-        <v>3000</v>
+        <v>2904</v>
       </c>
       <c r="G44" s="14" t="n">
         <v>0</v>
       </c>
       <c r="H44" s="14" t="n">
-        <v>3000</v>
+        <v>2904</v>
       </c>
       <c r="I44" s="14">
         <f>MAX(0, E44-F44)</f>
@@ -10821,54 +11005,146 @@
         <f>IF(E44&gt;0, F44/E44, IF(F44&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L44" s="33" t="inlineStr">
+      <c r="L44" s="29" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
       </c>
     </row>
-    <row r="45" ht="24" customHeight="1">
-      <c r="B45" s="20" t="inlineStr">
+    <row r="45">
+      <c r="B45" s="30" t="inlineStr">
+        <is>
+          <t>LEKKERBIO B.V.</t>
+        </is>
+      </c>
+      <c r="C45" s="31" t="inlineStr">
+        <is>
+          <t>AO0020</t>
+        </is>
+      </c>
+      <c r="D45" s="30" t="inlineStr">
+        <is>
+          <t>ALCAPLANT NEW</t>
+        </is>
+      </c>
+      <c r="E45" s="18" t="n">
+        <v>44000</v>
+      </c>
+      <c r="F45" s="18" t="n">
+        <v>19800</v>
+      </c>
+      <c r="G45" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H45" s="18" t="n">
+        <v>19800</v>
+      </c>
+      <c r="I45" s="18">
+        <f>MAX(0, E45-F45)</f>
+        <v/>
+      </c>
+      <c r="J45" s="18">
+        <f>ABS(F45-E45)</f>
+        <v/>
+      </c>
+      <c r="K45" s="19">
+        <f>IF(E45&gt;0, F45/E45, IF(F45&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L45" s="40" t="inlineStr">
+        <is>
+          <t>Rezagado</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" s="27" t="inlineStr">
+        <is>
+          <t>LEKKERBIO B.V.</t>
+        </is>
+      </c>
+      <c r="C46" s="28" t="inlineStr">
+        <is>
+          <t>DECA0020</t>
+        </is>
+      </c>
+      <c r="D46" s="27" t="inlineStr">
+        <is>
+          <t>DEFENS-CA-AE, 20 KG</t>
+        </is>
+      </c>
+      <c r="E46" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F46" s="14" t="n">
+        <v>3000</v>
+      </c>
+      <c r="G46" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H46" s="14" t="n">
+        <v>3000</v>
+      </c>
+      <c r="I46" s="14">
+        <f>MAX(0, E46-F46)</f>
+        <v/>
+      </c>
+      <c r="J46" s="14">
+        <f>ABS(F46-E46)</f>
+        <v/>
+      </c>
+      <c r="K46" s="15">
+        <f>IF(E46&gt;0, F46/E46, IF(F46&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L46" s="29" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="24" customHeight="1">
+      <c r="B47" s="20" t="inlineStr">
         <is>
           <t>TOTAL RICARDO</t>
         </is>
       </c>
-      <c r="C45" s="36" t="inlineStr">
+      <c r="C47" s="34" t="inlineStr">
         <is>
           <t>128 líneas</t>
         </is>
       </c>
-      <c r="D45" s="37" t="inlineStr"/>
-      <c r="E45" s="22">
-        <f>SUM(E10:E44)</f>
-        <v/>
-      </c>
-      <c r="F45" s="22">
-        <f>SUM(F10:F44)</f>
-        <v/>
-      </c>
-      <c r="G45" s="22">
-        <f>SUM(G10:G44)</f>
-        <v/>
-      </c>
-      <c r="H45" s="22">
-        <f>SUM(H10:H44)</f>
-        <v/>
-      </c>
-      <c r="I45" s="22">
-        <f>SUM(I10:I44)</f>
-        <v/>
-      </c>
-      <c r="J45" s="22">
-        <f>SUM(J10:J44)</f>
-        <v/>
-      </c>
-      <c r="K45" s="23">
-        <f>IF(E45&gt;0, F45/E45, 0)</f>
-        <v/>
-      </c>
-      <c r="L45" s="21">
-        <f>IF(K45&gt;=1, "SUPERADO", "EN CURSO")</f>
+      <c r="D47" s="35" t="inlineStr"/>
+      <c r="E47" s="22">
+        <f>SUM(E10:E46)</f>
+        <v/>
+      </c>
+      <c r="F47" s="22">
+        <f>SUM(F10:F46)</f>
+        <v/>
+      </c>
+      <c r="G47" s="22">
+        <f>SUM(G10:G46)</f>
+        <v/>
+      </c>
+      <c r="H47" s="22">
+        <f>SUM(H10:H46)</f>
+        <v/>
+      </c>
+      <c r="I47" s="22">
+        <f>SUM(I10:I46)</f>
+        <v/>
+      </c>
+      <c r="J47" s="22">
+        <f>SUM(J10:J46)</f>
+        <v/>
+      </c>
+      <c r="K47" s="23">
+        <f>IF(E47&gt;0, F47/E47, 0)</f>
+        <v/>
+      </c>
+      <c r="L47" s="21">
+        <f>IF(K47&gt;=1, "SUPERADO", "EN CURSO")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Reorganizacion estructural: scripts, informes, antiguos, BI intelligence y pedidos 27.10
</commit_message>
<xml_diff>
--- a/Seguimiento_Presupuesto_Sep_2026.xlsx
+++ b/Seguimiento_Presupuesto_Sep_2026.xlsx
@@ -131,14 +131,14 @@
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="00B45309"/>
-      <sz val="13"/>
+      <color rgb="00991B1B"/>
+      <sz val="9"/>
     </font>
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="00991B1B"/>
-      <sz val="9"/>
+      <color rgb="00B45309"/>
+      <sz val="13"/>
     </font>
   </fonts>
   <fills count="11">
@@ -348,16 +348,16 @@
     <xf numFmtId="0" fontId="16" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="16" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -915,7 +915,7 @@
     <row r="3" ht="20" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Comparativa Estimación Septiembre (Unidades) vs Pedidos Reales a Fecha 26/10/2026 | Generado: 26/10/2026 08:04</t>
+          <t>Comparativa Estimación Septiembre (Unidades) vs Pedidos Reales a Fecha 27/10/2026 | Generado: 27/10/2026 07:39</t>
         </is>
       </c>
     </row>
@@ -959,25 +959,25 @@
       <c r="C6" s="4" t="n"/>
       <c r="D6" s="8" t="inlineStr">
         <is>
-          <t>247,817 u</t>
+          <t>254,091 u</t>
         </is>
       </c>
       <c r="E6" s="4" t="n"/>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>136.2%</t>
+          <t>139.6%</t>
         </is>
       </c>
       <c r="G6" s="4" t="n"/>
       <c r="H6" s="9" t="inlineStr">
         <is>
-          <t>44,669 u</t>
+          <t>41,738 u</t>
         </is>
       </c>
       <c r="I6" s="4" t="n"/>
       <c r="J6" s="7" t="inlineStr">
         <is>
-          <t>190,808 u</t>
+          <t>187,680 u</t>
         </is>
       </c>
     </row>
@@ -1042,16 +1042,16 @@
         </is>
       </c>
       <c r="C10" s="13" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D10" s="14" t="n">
         <v>2320</v>
       </c>
       <c r="E10" s="14" t="n">
-        <v>6864</v>
+        <v>7164</v>
       </c>
       <c r="F10" s="14" t="n">
-        <v>6864</v>
+        <v>7164</v>
       </c>
       <c r="G10" s="14" t="n">
         <v>0</v>
@@ -1061,7 +1061,7 @@
         <v/>
       </c>
       <c r="I10" s="14">
-        <f>'Alfonso'!J26</f>
+        <f>'Alfonso'!J28</f>
         <v/>
       </c>
       <c r="J10" s="15">
@@ -1082,20 +1082,20 @@
         <v>37832</v>
       </c>
       <c r="E11" s="18" t="n">
-        <v>80676</v>
+        <v>81476</v>
       </c>
       <c r="F11" s="18" t="n">
         <v>6680</v>
       </c>
       <c r="G11" s="18" t="n">
-        <v>73996</v>
+        <v>74796</v>
       </c>
       <c r="H11" s="18">
         <f>MAX(0, D11-E11)</f>
         <v/>
       </c>
       <c r="I11" s="18">
-        <f>'García'!J48</f>
+        <f>'García'!J50</f>
         <v/>
       </c>
       <c r="J11" s="19">
@@ -1116,20 +1116,20 @@
         <v>21914</v>
       </c>
       <c r="E12" s="14" t="n">
+        <v>23753</v>
+      </c>
+      <c r="F12" s="14" t="n">
         <v>20245</v>
       </c>
-      <c r="F12" s="14" t="n">
-        <v>13525</v>
-      </c>
       <c r="G12" s="14" t="n">
-        <v>6720</v>
+        <v>3508</v>
       </c>
       <c r="H12" s="14">
         <f>MAX(0, D12-E12)</f>
         <v/>
       </c>
       <c r="I12" s="14">
-        <f>'Irene'!J52</f>
+        <f>'Irene'!J55</f>
         <v/>
       </c>
       <c r="J12" s="15">
@@ -1144,26 +1144,26 @@
         </is>
       </c>
       <c r="C13" s="17" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D13" s="18" t="n">
         <v>17100</v>
       </c>
       <c r="E13" s="18" t="n">
-        <v>13560</v>
+        <v>14822</v>
       </c>
       <c r="F13" s="18" t="n">
-        <v>12540</v>
+        <v>14822</v>
       </c>
       <c r="G13" s="18" t="n">
-        <v>1020</v>
+        <v>0</v>
       </c>
       <c r="H13" s="18">
         <f>MAX(0, D13-E13)</f>
         <v/>
       </c>
       <c r="I13" s="18">
-        <f>'Javier'!J33</f>
+        <f>'Javier'!J37</f>
         <v/>
       </c>
       <c r="J13" s="19">
@@ -1218,10 +1218,10 @@
         <v>17340</v>
       </c>
       <c r="E15" s="18" t="n">
-        <v>17400</v>
+        <v>17500</v>
       </c>
       <c r="F15" s="18" t="n">
-        <v>17400</v>
+        <v>17500</v>
       </c>
       <c r="G15" s="18" t="n">
         <v>0</v>
@@ -1231,7 +1231,7 @@
         <v/>
       </c>
       <c r="I15" s="18">
-        <f>'Pedro'!J27</f>
+        <f>'Pedro'!J28</f>
         <v/>
       </c>
       <c r="J15" s="19">
@@ -1252,20 +1252,20 @@
         <v>46000</v>
       </c>
       <c r="E16" s="14" t="n">
-        <v>109072</v>
+        <v>109376</v>
       </c>
       <c r="F16" s="14" t="n">
         <v>0</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>109072</v>
+        <v>109376</v>
       </c>
       <c r="H16" s="14">
         <f>MAX(0, D16-E16)</f>
         <v/>
       </c>
       <c r="I16" s="14">
-        <f>'Ricardo'!J47</f>
+        <f>'Ricardo'!J50</f>
         <v/>
       </c>
       <c r="J16" s="15">
@@ -1336,7 +1336,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:L26"/>
+  <dimension ref="B2:L28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1363,7 +1363,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 26/10/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 27/10/2026</t>
         </is>
       </c>
     </row>
@@ -1408,13 +1408,13 @@
       <c r="C6" s="4" t="n"/>
       <c r="D6" s="25" t="inlineStr">
         <is>
-          <t>6,864 u</t>
+          <t>7,164 u</t>
         </is>
       </c>
       <c r="E6" s="4" t="n"/>
       <c r="F6" s="25" t="inlineStr">
         <is>
-          <t>295.9%</t>
+          <t>308.8%</t>
         </is>
       </c>
       <c r="G6" s="4" t="n"/>
@@ -1958,27 +1958,27 @@
     <row r="20">
       <c r="B20" s="27" t="inlineStr">
         <is>
-          <t>VILLALTA SATIVUM, S.L.</t>
+          <t>PLANTALDIA SLU</t>
         </is>
       </c>
       <c r="C20" s="28" t="inlineStr">
         <is>
-          <t>AGXKAEP0020</t>
+          <t>A-50(2)0005</t>
         </is>
       </c>
       <c r="D20" s="27" t="inlineStr">
         <is>
-          <t>BIOCULTURE POTASIO PLUS, 20 L</t>
+          <t>CODIORGAN A-50, 5 KG</t>
         </is>
       </c>
       <c r="E20" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F20" s="14" t="n">
-        <v>140</v>
+        <v>100</v>
       </c>
       <c r="G20" s="14" t="n">
-        <v>140</v>
+        <v>100</v>
       </c>
       <c r="H20" s="14" t="n">
         <v>0</v>
@@ -2004,27 +2004,27 @@
     <row r="21">
       <c r="B21" s="30" t="inlineStr">
         <is>
-          <t>VILLALTA SATIVUM, S.L.</t>
+          <t>PLANTALDIA SLU</t>
         </is>
       </c>
       <c r="C21" s="31" t="inlineStr">
         <is>
-          <t>AQUOM0020</t>
+          <t>C-L0005</t>
         </is>
       </c>
       <c r="D21" s="30" t="inlineStr">
         <is>
-          <t>AQUOM, 20 L</t>
+          <t>CODIBOR-L, 5 L</t>
         </is>
       </c>
       <c r="E21" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F21" s="18" t="n">
-        <v>40</v>
+        <v>200</v>
       </c>
       <c r="G21" s="18" t="n">
-        <v>40</v>
+        <v>200</v>
       </c>
       <c r="H21" s="18" t="n">
         <v>0</v>
@@ -2055,22 +2055,22 @@
       </c>
       <c r="C22" s="28" t="inlineStr">
         <is>
-          <t>C-CUAE0020</t>
+          <t>AGXKAEP0020</t>
         </is>
       </c>
       <c r="D22" s="27" t="inlineStr">
         <is>
-          <t>CUPRAMEC, 20 L</t>
+          <t>BIOCULTURE POTASIO PLUS, 20 L</t>
         </is>
       </c>
       <c r="E22" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F22" s="14" t="n">
-        <v>200</v>
+        <v>140</v>
       </c>
       <c r="G22" s="14" t="n">
-        <v>200</v>
+        <v>140</v>
       </c>
       <c r="H22" s="14" t="n">
         <v>0</v>
@@ -2101,22 +2101,22 @@
       </c>
       <c r="C23" s="31" t="inlineStr">
         <is>
-          <t>PT0001</t>
+          <t>AQUOM0020</t>
         </is>
       </c>
       <c r="D23" s="30" t="inlineStr">
         <is>
-          <t>AGROPOTASION, 1 L</t>
+          <t>AQUOM, 20 L</t>
         </is>
       </c>
       <c r="E23" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F23" s="18" t="n">
-        <v>24</v>
+        <v>40</v>
       </c>
       <c r="G23" s="18" t="n">
-        <v>24</v>
+        <v>40</v>
       </c>
       <c r="H23" s="18" t="n">
         <v>0</v>
@@ -2147,22 +2147,22 @@
       </c>
       <c r="C24" s="28" t="inlineStr">
         <is>
-          <t>PT0005</t>
+          <t>C-CUAE0020</t>
         </is>
       </c>
       <c r="D24" s="27" t="inlineStr">
         <is>
-          <t>AGROPOTASION, 5 L</t>
+          <t>CUPRAMEC, 20 L</t>
         </is>
       </c>
       <c r="E24" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F24" s="14" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="G24" s="14" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="H24" s="14" t="n">
         <v>0</v>
@@ -2193,22 +2193,22 @@
       </c>
       <c r="C25" s="31" t="inlineStr">
         <is>
-          <t>PT0020</t>
+          <t>PT0001</t>
         </is>
       </c>
       <c r="D25" s="30" t="inlineStr">
         <is>
-          <t>AGROPOTASION, 20 L</t>
+          <t>AGROPOTASION, 1 L</t>
         </is>
       </c>
       <c r="E25" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F25" s="18" t="n">
-        <v>100</v>
+        <v>24</v>
       </c>
       <c r="G25" s="18" t="n">
-        <v>100</v>
+        <v>24</v>
       </c>
       <c r="H25" s="18" t="n">
         <v>0</v>
@@ -2231,48 +2231,140 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="24" customHeight="1">
-      <c r="B26" s="20" t="inlineStr">
+    <row r="26">
+      <c r="B26" s="27" t="inlineStr">
+        <is>
+          <t>VILLALTA SATIVUM, S.L.</t>
+        </is>
+      </c>
+      <c r="C26" s="28" t="inlineStr">
+        <is>
+          <t>PT0005</t>
+        </is>
+      </c>
+      <c r="D26" s="27" t="inlineStr">
+        <is>
+          <t>AGROPOTASION, 5 L</t>
+        </is>
+      </c>
+      <c r="E26" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" s="14" t="n">
+        <v>100</v>
+      </c>
+      <c r="G26" s="14" t="n">
+        <v>100</v>
+      </c>
+      <c r="H26" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I26" s="14">
+        <f>MAX(0, E26-F26)</f>
+        <v/>
+      </c>
+      <c r="J26" s="14">
+        <f>ABS(F26-E26)</f>
+        <v/>
+      </c>
+      <c r="K26" s="15">
+        <f>IF(E26&gt;0, F26/E26, IF(F26&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L26" s="29" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="30" t="inlineStr">
+        <is>
+          <t>VILLALTA SATIVUM, S.L.</t>
+        </is>
+      </c>
+      <c r="C27" s="31" t="inlineStr">
+        <is>
+          <t>PT0020</t>
+        </is>
+      </c>
+      <c r="D27" s="30" t="inlineStr">
+        <is>
+          <t>AGROPOTASION, 20 L</t>
+        </is>
+      </c>
+      <c r="E27" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" s="18" t="n">
+        <v>100</v>
+      </c>
+      <c r="G27" s="18" t="n">
+        <v>100</v>
+      </c>
+      <c r="H27" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="I27" s="18">
+        <f>MAX(0, E27-F27)</f>
+        <v/>
+      </c>
+      <c r="J27" s="18">
+        <f>ABS(F27-E27)</f>
+        <v/>
+      </c>
+      <c r="K27" s="19">
+        <f>IF(E27&gt;0, F27/E27, IF(F27&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L27" s="32" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="24" customHeight="1">
+      <c r="B28" s="20" t="inlineStr">
         <is>
           <t>TOTAL ALFONSO</t>
         </is>
       </c>
-      <c r="C26" s="34" t="inlineStr">
+      <c r="C28" s="34" t="inlineStr">
         <is>
           <t>279 líneas</t>
         </is>
       </c>
-      <c r="D26" s="35" t="inlineStr"/>
-      <c r="E26" s="22">
-        <f>SUM(E10:E25)</f>
-        <v/>
-      </c>
-      <c r="F26" s="22">
-        <f>SUM(F10:F25)</f>
-        <v/>
-      </c>
-      <c r="G26" s="22">
-        <f>SUM(G10:G25)</f>
-        <v/>
-      </c>
-      <c r="H26" s="22">
-        <f>SUM(H10:H25)</f>
-        <v/>
-      </c>
-      <c r="I26" s="22">
-        <f>SUM(I10:I25)</f>
-        <v/>
-      </c>
-      <c r="J26" s="22">
-        <f>SUM(J10:J25)</f>
-        <v/>
-      </c>
-      <c r="K26" s="23">
-        <f>IF(E26&gt;0, F26/E26, 0)</f>
-        <v/>
-      </c>
-      <c r="L26" s="21">
-        <f>IF(K26&gt;=1, "SUPERADO", "EN CURSO")</f>
+      <c r="D28" s="35" t="inlineStr"/>
+      <c r="E28" s="22">
+        <f>SUM(E10:E27)</f>
+        <v/>
+      </c>
+      <c r="F28" s="22">
+        <f>SUM(F10:F27)</f>
+        <v/>
+      </c>
+      <c r="G28" s="22">
+        <f>SUM(G10:G27)</f>
+        <v/>
+      </c>
+      <c r="H28" s="22">
+        <f>SUM(H10:H27)</f>
+        <v/>
+      </c>
+      <c r="I28" s="22">
+        <f>SUM(I10:I27)</f>
+        <v/>
+      </c>
+      <c r="J28" s="22">
+        <f>SUM(J10:J27)</f>
+        <v/>
+      </c>
+      <c r="K28" s="23">
+        <f>IF(E28&gt;0, F28/E28, 0)</f>
+        <v/>
+      </c>
+      <c r="L28" s="21">
+        <f>IF(K28&gt;=1, "SUPERADO", "EN CURSO")</f>
         <v/>
       </c>
     </row>
@@ -2301,7 +2393,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:L48"/>
+  <dimension ref="B2:L50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -2328,7 +2420,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 26/10/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 27/10/2026</t>
         </is>
       </c>
     </row>
@@ -2373,13 +2465,13 @@
       <c r="C6" s="4" t="n"/>
       <c r="D6" s="25" t="inlineStr">
         <is>
-          <t>80,676 u</t>
+          <t>81,476 u</t>
         </is>
       </c>
       <c r="E6" s="4" t="n"/>
       <c r="F6" s="25" t="inlineStr">
         <is>
-          <t>213.2%</t>
+          <t>215.4%</t>
         </is>
       </c>
       <c r="G6" s="4" t="n"/>
@@ -2391,7 +2483,7 @@
       <c r="I6" s="4" t="n"/>
       <c r="J6" s="24" t="inlineStr">
         <is>
-          <t>73,996 u</t>
+          <t>74,796 u</t>
         </is>
       </c>
       <c r="K6" s="4" t="n"/>
@@ -3112,12 +3204,12 @@
       </c>
       <c r="C24" s="28" t="inlineStr">
         <is>
-          <t>AGXK0005</t>
+          <t>AGXK0005EG</t>
         </is>
       </c>
       <c r="D24" s="27" t="inlineStr">
         <is>
-          <t>AGROXILATO+K</t>
+          <t>AGROXILATO-K, 5 L</t>
         </is>
       </c>
       <c r="E24" s="14" t="n">
@@ -3158,12 +3250,12 @@
       </c>
       <c r="C25" s="31" t="inlineStr">
         <is>
-          <t>SPCE2B0001</t>
+          <t>SPCE2B0001EG</t>
         </is>
       </c>
       <c r="D25" s="30" t="inlineStr">
         <is>
-          <t>NEW SPRINTENE</t>
+          <t>SPRINTENE CON BORO, 1 L</t>
         </is>
       </c>
       <c r="E25" s="18" t="n">
@@ -3756,7 +3848,7 @@
       </c>
       <c r="C38" s="28" t="inlineStr">
         <is>
-          <t>A-500020</t>
+          <t>A-500020MA</t>
         </is>
       </c>
       <c r="D38" s="27" t="inlineStr">
@@ -3802,12 +3894,12 @@
       </c>
       <c r="C39" s="31" t="inlineStr">
         <is>
-          <t>AGXK0020</t>
+          <t>AGXK0020MA</t>
         </is>
       </c>
       <c r="D39" s="30" t="inlineStr">
         <is>
-          <t>AGROXILATO-K</t>
+          <t>AGROXILATO-K, 20 L</t>
         </is>
       </c>
       <c r="E39" s="18" t="n">
@@ -3848,12 +3940,12 @@
       </c>
       <c r="C40" s="28" t="inlineStr">
         <is>
-          <t>AVAN0020</t>
+          <t>AVAN0020MA</t>
         </is>
       </c>
       <c r="D40" s="27" t="inlineStr">
         <is>
-          <t>FLORAMEC AVANCE</t>
+          <t>FLORAMEC AVANCE, 20 L</t>
         </is>
       </c>
       <c r="E40" s="14" t="n">
@@ -3894,12 +3986,12 @@
       </c>
       <c r="C41" s="31" t="inlineStr">
         <is>
-          <t>BR-590005</t>
+          <t>BR-590005MA</t>
         </is>
       </c>
       <c r="D41" s="30" t="inlineStr">
         <is>
-          <t>BR-59</t>
+          <t>BR-59, 5 KG</t>
         </is>
       </c>
       <c r="E41" s="18" t="n">
@@ -3940,25 +4032,25 @@
       </c>
       <c r="C42" s="28" t="inlineStr">
         <is>
-          <t>C-CU0005</t>
+          <t>BROTA0005</t>
         </is>
       </c>
       <c r="D42" s="27" t="inlineStr">
         <is>
-          <t>CODICOBRE</t>
+          <t>BROTAMEC, 5 L</t>
         </is>
       </c>
       <c r="E42" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F42" s="14" t="n">
-        <v>1000</v>
+        <v>200</v>
       </c>
       <c r="G42" s="14" t="n">
         <v>0</v>
       </c>
       <c r="H42" s="14" t="n">
-        <v>1000</v>
+        <v>200</v>
       </c>
       <c r="I42" s="14">
         <f>MAX(0, E42-F42)</f>
@@ -3986,25 +4078,25 @@
       </c>
       <c r="C43" s="31" t="inlineStr">
         <is>
-          <t>PHD0020</t>
+          <t>C-CU0005MA</t>
         </is>
       </c>
       <c r="D43" s="30" t="inlineStr">
         <is>
-          <t>PH-DOWNER</t>
+          <t>CODICOBRE, 5 L</t>
         </is>
       </c>
       <c r="E43" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F43" s="18" t="n">
-        <v>600</v>
+        <v>1000</v>
       </c>
       <c r="G43" s="18" t="n">
         <v>0</v>
       </c>
       <c r="H43" s="18" t="n">
-        <v>600</v>
+        <v>1000</v>
       </c>
       <c r="I43" s="18">
         <f>MAX(0, E43-F43)</f>
@@ -4032,25 +4124,25 @@
       </c>
       <c r="C44" s="28" t="inlineStr">
         <is>
-          <t>PT0020</t>
+          <t>PHD0005</t>
         </is>
       </c>
       <c r="D44" s="27" t="inlineStr">
         <is>
-          <t>AGROPOTASION</t>
+          <t>PH-DOWNER, 5 L</t>
         </is>
       </c>
       <c r="E44" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F44" s="14" t="n">
-        <v>3000</v>
+        <v>600</v>
       </c>
       <c r="G44" s="14" t="n">
         <v>0</v>
       </c>
       <c r="H44" s="14" t="n">
-        <v>3000</v>
+        <v>600</v>
       </c>
       <c r="I44" s="14">
         <f>MAX(0, E44-F44)</f>
@@ -4078,25 +4170,25 @@
       </c>
       <c r="C45" s="31" t="inlineStr">
         <is>
-          <t>SS0020</t>
+          <t>PHD0020MA</t>
         </is>
       </c>
       <c r="D45" s="30" t="inlineStr">
         <is>
-          <t>SAL-WAX-Ca</t>
+          <t xml:space="preserve">PH-DOWNER, 20 L   </t>
         </is>
       </c>
       <c r="E45" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F45" s="18" t="n">
-        <v>2000</v>
+        <v>600</v>
       </c>
       <c r="G45" s="18" t="n">
         <v>0</v>
       </c>
       <c r="H45" s="18" t="n">
-        <v>2000</v>
+        <v>600</v>
       </c>
       <c r="I45" s="18">
         <f>MAX(0, E45-F45)</f>
@@ -4119,12 +4211,12 @@
     <row r="46">
       <c r="B46" s="27" t="inlineStr">
         <is>
-          <t>TRATAMIENTOS AGRICOLAS BRENES, S.L.</t>
+          <t>STE BBMAGRI, SARL</t>
         </is>
       </c>
       <c r="C46" s="28" t="inlineStr">
         <is>
-          <t>PT0020</t>
+          <t>PT0020MA</t>
         </is>
       </c>
       <c r="D46" s="27" t="inlineStr">
@@ -4136,13 +4228,13 @@
         <v>0</v>
       </c>
       <c r="F46" s="14" t="n">
-        <v>640</v>
+        <v>3000</v>
       </c>
       <c r="G46" s="14" t="n">
-        <v>640</v>
+        <v>0</v>
       </c>
       <c r="H46" s="14" t="n">
-        <v>0</v>
+        <v>3000</v>
       </c>
       <c r="I46" s="14">
         <f>MAX(0, E46-F46)</f>
@@ -4165,30 +4257,30 @@
     <row r="47">
       <c r="B47" s="30" t="inlineStr">
         <is>
-          <t>TRATAMIENTOS AGRICOLAS BRENES, S.L.</t>
+          <t>STE BBMAGRI, SARL</t>
         </is>
       </c>
       <c r="C47" s="31" t="inlineStr">
         <is>
-          <t>WHITE0020</t>
+          <t>SS0020MA</t>
         </is>
       </c>
       <c r="D47" s="30" t="inlineStr">
         <is>
-          <t>AGROWHITE, 20 KG</t>
+          <t>SALWAX-CA, 20 KG</t>
         </is>
       </c>
       <c r="E47" s="18" t="n">
-        <v>1100</v>
+        <v>0</v>
       </c>
       <c r="F47" s="18" t="n">
-        <v>0</v>
+        <v>2000</v>
       </c>
       <c r="G47" s="18" t="n">
         <v>0</v>
       </c>
       <c r="H47" s="18" t="n">
-        <v>0</v>
+        <v>2000</v>
       </c>
       <c r="I47" s="18">
         <f>MAX(0, E47-F47)</f>
@@ -4202,54 +4294,146 @@
         <f>IF(E47&gt;0, F47/E47, IF(F47&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L47" s="36" t="inlineStr">
+      <c r="L47" s="32" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="B48" s="27" t="inlineStr">
+        <is>
+          <t>TRATAMIENTOS AGRICOLAS BRENES, S.L.</t>
+        </is>
+      </c>
+      <c r="C48" s="28" t="inlineStr">
+        <is>
+          <t>PT0020</t>
+        </is>
+      </c>
+      <c r="D48" s="27" t="inlineStr">
+        <is>
+          <t>AGROPOTASION, 20 L</t>
+        </is>
+      </c>
+      <c r="E48" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F48" s="14" t="n">
+        <v>640</v>
+      </c>
+      <c r="G48" s="14" t="n">
+        <v>640</v>
+      </c>
+      <c r="H48" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I48" s="14">
+        <f>MAX(0, E48-F48)</f>
+        <v/>
+      </c>
+      <c r="J48" s="14">
+        <f>ABS(F48-E48)</f>
+        <v/>
+      </c>
+      <c r="K48" s="15">
+        <f>IF(E48&gt;0, F48/E48, IF(F48&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L48" s="29" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="B49" s="30" t="inlineStr">
+        <is>
+          <t>TRATAMIENTOS AGRICOLAS BRENES, S.L.</t>
+        </is>
+      </c>
+      <c r="C49" s="31" t="inlineStr">
+        <is>
+          <t>WHITE0020</t>
+        </is>
+      </c>
+      <c r="D49" s="30" t="inlineStr">
+        <is>
+          <t>AGROWHITE, 20 KG</t>
+        </is>
+      </c>
+      <c r="E49" s="18" t="n">
+        <v>1100</v>
+      </c>
+      <c r="F49" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G49" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H49" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="I49" s="18">
+        <f>MAX(0, E49-F49)</f>
+        <v/>
+      </c>
+      <c r="J49" s="18">
+        <f>ABS(F49-E49)</f>
+        <v/>
+      </c>
+      <c r="K49" s="19">
+        <f>IF(E49&gt;0, F49/E49, IF(F49&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L49" s="36" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
       </c>
     </row>
-    <row r="48" ht="24" customHeight="1">
-      <c r="B48" s="20" t="inlineStr">
+    <row r="50" ht="24" customHeight="1">
+      <c r="B50" s="20" t="inlineStr">
         <is>
           <t>TOTAL GARCÍA</t>
         </is>
       </c>
-      <c r="C48" s="34" t="inlineStr">
-        <is>
-          <t>234 líneas</t>
-        </is>
-      </c>
-      <c r="D48" s="35" t="inlineStr"/>
-      <c r="E48" s="22">
-        <f>SUM(E10:E47)</f>
-        <v/>
-      </c>
-      <c r="F48" s="22">
-        <f>SUM(F10:F47)</f>
-        <v/>
-      </c>
-      <c r="G48" s="22">
-        <f>SUM(G10:G47)</f>
-        <v/>
-      </c>
-      <c r="H48" s="22">
-        <f>SUM(H10:H47)</f>
-        <v/>
-      </c>
-      <c r="I48" s="22">
-        <f>SUM(I10:I47)</f>
-        <v/>
-      </c>
-      <c r="J48" s="22">
-        <f>SUM(J10:J47)</f>
-        <v/>
-      </c>
-      <c r="K48" s="23">
-        <f>IF(E48&gt;0, F48/E48, 0)</f>
-        <v/>
-      </c>
-      <c r="L48" s="21">
-        <f>IF(K48&gt;=1, "SUPERADO", "EN CURSO")</f>
+      <c r="C50" s="34" t="inlineStr">
+        <is>
+          <t>244 líneas</t>
+        </is>
+      </c>
+      <c r="D50" s="35" t="inlineStr"/>
+      <c r="E50" s="22">
+        <f>SUM(E10:E49)</f>
+        <v/>
+      </c>
+      <c r="F50" s="22">
+        <f>SUM(F10:F49)</f>
+        <v/>
+      </c>
+      <c r="G50" s="22">
+        <f>SUM(G10:G49)</f>
+        <v/>
+      </c>
+      <c r="H50" s="22">
+        <f>SUM(H10:H49)</f>
+        <v/>
+      </c>
+      <c r="I50" s="22">
+        <f>SUM(I10:I49)</f>
+        <v/>
+      </c>
+      <c r="J50" s="22">
+        <f>SUM(J10:J49)</f>
+        <v/>
+      </c>
+      <c r="K50" s="23">
+        <f>IF(E50&gt;0, F50/E50, 0)</f>
+        <v/>
+      </c>
+      <c r="L50" s="21">
+        <f>IF(K50&gt;=1, "SUPERADO", "EN CURSO")</f>
         <v/>
       </c>
     </row>
@@ -4278,7 +4462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:L52"/>
+  <dimension ref="B2:L55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -4305,7 +4489,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 26/10/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 27/10/2026</t>
         </is>
       </c>
     </row>
@@ -4316,19 +4500,19 @@
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D5" s="5" t="inlineStr">
         <is>
           <t>PEDIDOS REALES (U)</t>
         </is>
       </c>
       <c r="E5" s="4" t="n"/>
-      <c r="F5" s="6" t="inlineStr">
+      <c r="F5" s="5" t="inlineStr">
         <is>
           <t>% CONSECUCIÓN</t>
         </is>
       </c>
       <c r="G5" s="4" t="n"/>
-      <c r="H5" s="6" t="inlineStr">
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>FALTA CONSEGUIR (GAP)</t>
         </is>
@@ -4348,27 +4532,27 @@
         </is>
       </c>
       <c r="C6" s="4" t="n"/>
-      <c r="D6" s="24" t="inlineStr">
-        <is>
-          <t>20,245 u</t>
+      <c r="D6" s="25" t="inlineStr">
+        <is>
+          <t>23,753 u</t>
         </is>
       </c>
       <c r="E6" s="4" t="n"/>
-      <c r="F6" s="38" t="inlineStr">
-        <is>
-          <t>92.4%</t>
+      <c r="F6" s="25" t="inlineStr">
+        <is>
+          <t>108.4%</t>
         </is>
       </c>
       <c r="G6" s="4" t="n"/>
-      <c r="H6" s="38" t="inlineStr">
-        <is>
-          <t>1,669 u</t>
+      <c r="H6" s="25" t="inlineStr">
+        <is>
+          <t>0 u</t>
         </is>
       </c>
       <c r="I6" s="4" t="n"/>
       <c r="J6" s="24" t="inlineStr">
         <is>
-          <t>6,720 u</t>
+          <t>3,508 u</t>
         </is>
       </c>
       <c r="K6" s="4" t="n"/>
@@ -4506,10 +4690,10 @@
         <v>3200</v>
       </c>
       <c r="G11" s="18" t="n">
-        <v>1280</v>
+        <v>3200</v>
       </c>
       <c r="H11" s="18" t="n">
-        <v>1920</v>
+        <v>0</v>
       </c>
       <c r="I11" s="18">
         <f>MAX(0, E11-F11)</f>
@@ -4569,7 +4753,7 @@
         <f>IF(E12&gt;0, F12/E12, IF(F12&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L12" s="39" t="inlineStr">
+      <c r="L12" s="38" t="inlineStr">
         <is>
           <t>En Curso</t>
         </is>
@@ -4598,10 +4782,10 @@
         <v>1280</v>
       </c>
       <c r="G13" s="18" t="n">
-        <v>640</v>
+        <v>1280</v>
       </c>
       <c r="H13" s="18" t="n">
-        <v>640</v>
+        <v>0</v>
       </c>
       <c r="I13" s="18">
         <f>MAX(0, E13-F13)</f>
@@ -4891,7 +5075,7 @@
         <f>IF(E19&gt;0, F19/E19, IF(F19&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L19" s="40" t="inlineStr">
+      <c r="L19" s="39" t="inlineStr">
         <is>
           <t>Rezagado</t>
         </is>
@@ -5012,10 +5196,10 @@
         <v>600</v>
       </c>
       <c r="G22" s="14" t="n">
-        <v>0</v>
+        <v>600</v>
       </c>
       <c r="H22" s="14" t="n">
-        <v>600</v>
+        <v>0</v>
       </c>
       <c r="I22" s="14">
         <f>MAX(0, E22-F22)</f>
@@ -5121,7 +5305,7 @@
         <f>IF(E24&gt;0, F24/E24, IF(F24&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L24" s="41" t="inlineStr">
+      <c r="L24" s="40" t="inlineStr">
         <is>
           <t>Rezagado</t>
         </is>
@@ -5239,13 +5423,13 @@
         <v>3200</v>
       </c>
       <c r="F27" s="18" t="n">
+        <v>4480</v>
+      </c>
+      <c r="G27" s="18" t="n">
         <v>1920</v>
       </c>
-      <c r="G27" s="18" t="n">
-        <v>640</v>
-      </c>
       <c r="H27" s="18" t="n">
-        <v>1280</v>
+        <v>2560</v>
       </c>
       <c r="I27" s="18">
         <f>MAX(0, E27-F27)</f>
@@ -5259,9 +5443,9 @@
         <f>IF(E27&gt;0, F27/E27, IF(F27&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L27" s="37" t="inlineStr">
-        <is>
-          <t>En Curso</t>
+      <c r="L27" s="32" t="inlineStr">
+        <is>
+          <t>Superado</t>
         </is>
       </c>
     </row>
@@ -5411,25 +5595,25 @@
       </c>
       <c r="C31" s="31" t="inlineStr">
         <is>
-          <t>AVAN0005</t>
+          <t>AMIMG0020</t>
         </is>
       </c>
       <c r="D31" s="30" t="inlineStr">
         <is>
-          <t>FLORAMEC AVANCE, 5 L</t>
+          <t>AMINOSOIL MG, 20 L</t>
         </is>
       </c>
       <c r="E31" s="18" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="F31" s="18" t="n">
-        <v>600</v>
+        <v>640</v>
       </c>
       <c r="G31" s="18" t="n">
-        <v>600</v>
+        <v>0</v>
       </c>
       <c r="H31" s="18" t="n">
-        <v>0</v>
+        <v>640</v>
       </c>
       <c r="I31" s="18">
         <f>MAX(0, E31-F31)</f>
@@ -5443,9 +5627,9 @@
         <f>IF(E31&gt;0, F31/E31, IF(F31&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L31" s="37" t="inlineStr">
-        <is>
-          <t>En Curso</t>
+      <c r="L31" s="32" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -5457,22 +5641,22 @@
       </c>
       <c r="C32" s="28" t="inlineStr">
         <is>
-          <t>C-L0005</t>
+          <t>AVAN0005</t>
         </is>
       </c>
       <c r="D32" s="27" t="inlineStr">
         <is>
-          <t>CODIBOR-L, 5 L</t>
+          <t>FLORAMEC AVANCE, 5 L</t>
         </is>
       </c>
       <c r="E32" s="14" t="n">
-        <v>200</v>
+        <v>1200</v>
       </c>
       <c r="F32" s="14" t="n">
-        <v>200</v>
+        <v>600</v>
       </c>
       <c r="G32" s="14" t="n">
-        <v>200</v>
+        <v>600</v>
       </c>
       <c r="H32" s="14" t="n">
         <v>0</v>
@@ -5489,9 +5673,9 @@
         <f>IF(E32&gt;0, F32/E32, IF(F32&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L32" s="29" t="inlineStr">
-        <is>
-          <t>Superado</t>
+      <c r="L32" s="38" t="inlineStr">
+        <is>
+          <t>En Curso</t>
         </is>
       </c>
     </row>
@@ -5503,16 +5687,16 @@
       </c>
       <c r="C33" s="31" t="inlineStr">
         <is>
-          <t>C-MB0005</t>
+          <t>C-L0005</t>
         </is>
       </c>
       <c r="D33" s="30" t="inlineStr">
         <is>
-          <t>CODIFOL-MB, 5 L</t>
+          <t>CODIBOR-L, 5 L</t>
         </is>
       </c>
       <c r="E33" s="18" t="n">
-        <v>300</v>
+        <v>200</v>
       </c>
       <c r="F33" s="18" t="n">
         <v>200</v>
@@ -5535,9 +5719,9 @@
         <f>IF(E33&gt;0, F33/E33, IF(F33&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L33" s="37" t="inlineStr">
-        <is>
-          <t>En Curso</t>
+      <c r="L33" s="32" t="inlineStr">
+        <is>
+          <t>Superado</t>
         </is>
       </c>
     </row>
@@ -5549,22 +5733,22 @@
       </c>
       <c r="C34" s="28" t="inlineStr">
         <is>
-          <t>CPLUS0020</t>
+          <t>C-MB0005</t>
         </is>
       </c>
       <c r="D34" s="27" t="inlineStr">
         <is>
-          <t>CALCIPLUS, 20 L</t>
+          <t>CODIFOL-MB, 5 L</t>
         </is>
       </c>
       <c r="E34" s="14" t="n">
-        <v>640</v>
+        <v>300</v>
       </c>
       <c r="F34" s="14" t="n">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="G34" s="14" t="n">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="H34" s="14" t="n">
         <v>0</v>
@@ -5581,9 +5765,9 @@
         <f>IF(E34&gt;0, F34/E34, IF(F34&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L34" s="33" t="inlineStr">
-        <is>
-          <t>Sin Pedido</t>
+      <c r="L34" s="38" t="inlineStr">
+        <is>
+          <t>En Curso</t>
         </is>
       </c>
     </row>
@@ -5595,22 +5779,22 @@
       </c>
       <c r="C35" s="31" t="inlineStr">
         <is>
-          <t>PIV0020</t>
+          <t>CPLUS0020</t>
         </is>
       </c>
       <c r="D35" s="30" t="inlineStr">
         <is>
-          <t>PGR IV, 20 L</t>
+          <t>CALCIPLUS, 20 L</t>
         </is>
       </c>
       <c r="E35" s="18" t="n">
-        <v>1280</v>
+        <v>640</v>
       </c>
       <c r="F35" s="18" t="n">
-        <v>2560</v>
+        <v>0</v>
       </c>
       <c r="G35" s="18" t="n">
-        <v>2560</v>
+        <v>0</v>
       </c>
       <c r="H35" s="18" t="n">
         <v>0</v>
@@ -5627,9 +5811,9 @@
         <f>IF(E35&gt;0, F35/E35, IF(F35&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L35" s="32" t="inlineStr">
-        <is>
-          <t>Superado</t>
+      <c r="L35" s="36" t="inlineStr">
+        <is>
+          <t>Sin Pedido</t>
         </is>
       </c>
     </row>
@@ -5641,22 +5825,22 @@
       </c>
       <c r="C36" s="28" t="inlineStr">
         <is>
-          <t>PT0020</t>
+          <t>PIV0020</t>
         </is>
       </c>
       <c r="D36" s="27" t="inlineStr">
         <is>
-          <t>AGROPOTASION, 20 L</t>
+          <t>PGR IV, 20 L</t>
         </is>
       </c>
       <c r="E36" s="14" t="n">
-        <v>0</v>
+        <v>1280</v>
       </c>
       <c r="F36" s="14" t="n">
-        <v>320</v>
+        <v>2560</v>
       </c>
       <c r="G36" s="14" t="n">
-        <v>320</v>
+        <v>2560</v>
       </c>
       <c r="H36" s="14" t="n">
         <v>0</v>
@@ -5675,7 +5859,7 @@
       </c>
       <c r="L36" s="29" t="inlineStr">
         <is>
-          <t>Extra Estimación</t>
+          <t>Superado</t>
         </is>
       </c>
     </row>
@@ -5687,25 +5871,25 @@
       </c>
       <c r="C37" s="31" t="inlineStr">
         <is>
-          <t>S0020</t>
+          <t>PT0005</t>
         </is>
       </c>
       <c r="D37" s="30" t="inlineStr">
         <is>
-          <t>SAL-WAX STAR, 20 L</t>
+          <t>AGROPOTASION, 5 L</t>
         </is>
       </c>
       <c r="E37" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F37" s="18" t="n">
-        <v>640</v>
+        <v>200</v>
       </c>
       <c r="G37" s="18" t="n">
-        <v>640</v>
+        <v>0</v>
       </c>
       <c r="H37" s="18" t="n">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="I37" s="18">
         <f>MAX(0, E37-F37)</f>
@@ -5728,27 +5912,27 @@
     <row r="38">
       <c r="B38" s="27" t="inlineStr">
         <is>
-          <t>GUIVARTO AGRICOLA, S.L.</t>
+          <t>COOP.AGRIC. SAN ISIDRO S.C.A.</t>
         </is>
       </c>
       <c r="C38" s="28" t="inlineStr">
         <is>
-          <t>A-50(2)0005</t>
+          <t>PT0020</t>
         </is>
       </c>
       <c r="D38" s="27" t="inlineStr">
         <is>
-          <t>CODIORGAN A-50, 5 KG</t>
+          <t>AGROPOTASION, 20 L</t>
         </is>
       </c>
       <c r="E38" s="14" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="F38" s="14" t="n">
-        <v>100</v>
+        <v>320</v>
       </c>
       <c r="G38" s="14" t="n">
-        <v>100</v>
+        <v>320</v>
       </c>
       <c r="H38" s="14" t="n">
         <v>0</v>
@@ -5767,37 +5951,37 @@
       </c>
       <c r="L38" s="29" t="inlineStr">
         <is>
-          <t>Superado</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="B39" s="30" t="inlineStr">
         <is>
-          <t>GUIVARTO AGRICOLA, S.L.</t>
+          <t>COOP.AGRIC. SAN ISIDRO S.C.A.</t>
         </is>
       </c>
       <c r="C39" s="31" t="inlineStr">
         <is>
-          <t>AGXK0020</t>
+          <t>S0020</t>
         </is>
       </c>
       <c r="D39" s="30" t="inlineStr">
         <is>
-          <t>AGROXILATO-K, 20 L</t>
+          <t>SAL-WAX STAR, 20 L</t>
         </is>
       </c>
       <c r="E39" s="18" t="n">
-        <v>1240</v>
+        <v>0</v>
       </c>
       <c r="F39" s="18" t="n">
-        <v>2560</v>
+        <v>640</v>
       </c>
       <c r="G39" s="18" t="n">
         <v>640</v>
       </c>
       <c r="H39" s="18" t="n">
-        <v>1920</v>
+        <v>0</v>
       </c>
       <c r="I39" s="18">
         <f>MAX(0, E39-F39)</f>
@@ -5813,37 +5997,37 @@
       </c>
       <c r="L39" s="32" t="inlineStr">
         <is>
-          <t>Superado</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="B40" s="27" t="inlineStr">
         <is>
-          <t>GUIVARTO AGRICOLA, S.L.</t>
+          <t>COOP.AGRIC. SAN ISIDRO S.C.A.</t>
         </is>
       </c>
       <c r="C40" s="28" t="inlineStr">
         <is>
-          <t>AGZNP0005</t>
+          <t>TRI0001</t>
         </is>
       </c>
       <c r="D40" s="27" t="inlineStr">
         <is>
-          <t>AGROXILATO-ZN PLUS, 5 KG</t>
+          <t>TRIFENO-94, 1 L</t>
         </is>
       </c>
       <c r="E40" s="14" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="F40" s="14" t="n">
-        <v>0</v>
+        <v>108</v>
       </c>
       <c r="G40" s="14" t="n">
         <v>0</v>
       </c>
       <c r="H40" s="14" t="n">
-        <v>0</v>
+        <v>108</v>
       </c>
       <c r="I40" s="14">
         <f>MAX(0, E40-F40)</f>
@@ -5857,9 +6041,9 @@
         <f>IF(E40&gt;0, F40/E40, IF(F40&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L40" s="33" t="inlineStr">
-        <is>
-          <t>Sin Pedido</t>
+      <c r="L40" s="29" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -5871,22 +6055,22 @@
       </c>
       <c r="C41" s="31" t="inlineStr">
         <is>
-          <t>AQUOM0005</t>
+          <t>A-50(2)0005</t>
         </is>
       </c>
       <c r="D41" s="30" t="inlineStr">
         <is>
-          <t>AQUOM, 5 L</t>
+          <t>CODIORGAN A-50, 5 KG</t>
         </is>
       </c>
       <c r="E41" s="18" t="n">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="F41" s="18" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="G41" s="18" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="H41" s="18" t="n">
         <v>0</v>
@@ -5903,9 +6087,9 @@
         <f>IF(E41&gt;0, F41/E41, IF(F41&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L41" s="36" t="inlineStr">
-        <is>
-          <t>Sin Pedido</t>
+      <c r="L41" s="32" t="inlineStr">
+        <is>
+          <t>Superado</t>
         </is>
       </c>
     </row>
@@ -5917,22 +6101,22 @@
       </c>
       <c r="C42" s="28" t="inlineStr">
         <is>
-          <t>AVAN0005</t>
+          <t>AGXK0020</t>
         </is>
       </c>
       <c r="D42" s="27" t="inlineStr">
         <is>
-          <t>FLORAMEC AVANCE, 5 L</t>
+          <t>AGROXILATO-K, 20 L</t>
         </is>
       </c>
       <c r="E42" s="14" t="n">
-        <v>0</v>
+        <v>1240</v>
       </c>
       <c r="F42" s="14" t="n">
-        <v>600</v>
+        <v>2560</v>
       </c>
       <c r="G42" s="14" t="n">
-        <v>600</v>
+        <v>2560</v>
       </c>
       <c r="H42" s="14" t="n">
         <v>0</v>
@@ -5951,7 +6135,7 @@
       </c>
       <c r="L42" s="29" t="inlineStr">
         <is>
-          <t>Extra Estimación</t>
+          <t>Superado</t>
         </is>
       </c>
     </row>
@@ -5963,22 +6147,22 @@
       </c>
       <c r="C43" s="31" t="inlineStr">
         <is>
-          <t>AVAN0020</t>
+          <t>AGZNP0005</t>
         </is>
       </c>
       <c r="D43" s="30" t="inlineStr">
         <is>
-          <t>FLORAMEC AVANCE, 20 L</t>
+          <t>AGROXILATO-ZN PLUS, 5 KG</t>
         </is>
       </c>
       <c r="E43" s="18" t="n">
-        <v>640</v>
+        <v>50</v>
       </c>
       <c r="F43" s="18" t="n">
-        <v>640</v>
+        <v>0</v>
       </c>
       <c r="G43" s="18" t="n">
-        <v>640</v>
+        <v>0</v>
       </c>
       <c r="H43" s="18" t="n">
         <v>0</v>
@@ -5995,9 +6179,9 @@
         <f>IF(E43&gt;0, F43/E43, IF(F43&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L43" s="32" t="inlineStr">
-        <is>
-          <t>Superado</t>
+      <c r="L43" s="36" t="inlineStr">
+        <is>
+          <t>Sin Pedido</t>
         </is>
       </c>
     </row>
@@ -6009,22 +6193,22 @@
       </c>
       <c r="C44" s="28" t="inlineStr">
         <is>
-          <t>BEY0005</t>
+          <t>AQUOM0005</t>
         </is>
       </c>
       <c r="D44" s="27" t="inlineStr">
         <is>
-          <t>FLORAMEC PLUS, 5 L</t>
+          <t>AQUOM, 5 L</t>
         </is>
       </c>
       <c r="E44" s="14" t="n">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="F44" s="14" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G44" s="14" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="H44" s="14" t="n">
         <v>0</v>
@@ -6041,9 +6225,9 @@
         <f>IF(E44&gt;0, F44/E44, IF(F44&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L44" s="29" t="inlineStr">
-        <is>
-          <t>Extra Estimación</t>
+      <c r="L44" s="33" t="inlineStr">
+        <is>
+          <t>Sin Pedido</t>
         </is>
       </c>
     </row>
@@ -6055,22 +6239,22 @@
       </c>
       <c r="C45" s="31" t="inlineStr">
         <is>
-          <t>BEY0020</t>
+          <t>AVAN0005</t>
         </is>
       </c>
       <c r="D45" s="30" t="inlineStr">
         <is>
-          <t>FLORAMEC PLUS 20 L</t>
+          <t>FLORAMEC AVANCE, 5 L</t>
         </is>
       </c>
       <c r="E45" s="18" t="n">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="F45" s="18" t="n">
-        <v>120</v>
+        <v>600</v>
       </c>
       <c r="G45" s="18" t="n">
-        <v>120</v>
+        <v>600</v>
       </c>
       <c r="H45" s="18" t="n">
         <v>0</v>
@@ -6089,7 +6273,7 @@
       </c>
       <c r="L45" s="32" t="inlineStr">
         <is>
-          <t>Superado</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -6101,22 +6285,22 @@
       </c>
       <c r="C46" s="28" t="inlineStr">
         <is>
-          <t>BROTA0005</t>
+          <t>AVAN0020</t>
         </is>
       </c>
       <c r="D46" s="27" t="inlineStr">
         <is>
-          <t>BROTAMEC, 5 L</t>
+          <t>FLORAMEC AVANCE, 20 L</t>
         </is>
       </c>
       <c r="E46" s="14" t="n">
-        <v>600</v>
+        <v>640</v>
       </c>
       <c r="F46" s="14" t="n">
-        <v>600</v>
+        <v>640</v>
       </c>
       <c r="G46" s="14" t="n">
-        <v>600</v>
+        <v>640</v>
       </c>
       <c r="H46" s="14" t="n">
         <v>0</v>
@@ -6147,22 +6331,22 @@
       </c>
       <c r="C47" s="31" t="inlineStr">
         <is>
-          <t>C-M-P0001</t>
+          <t>BEY0005</t>
         </is>
       </c>
       <c r="D47" s="30" t="inlineStr">
         <is>
-          <t>CODIFOL Mo-PLUS, 1 L</t>
+          <t>FLORAMEC PLUS, 5 L</t>
         </is>
       </c>
       <c r="E47" s="18" t="n">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="F47" s="18" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="G47" s="18" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="H47" s="18" t="n">
         <v>0</v>
@@ -6179,9 +6363,9 @@
         <f>IF(E47&gt;0, F47/E47, IF(F47&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L47" s="36" t="inlineStr">
-        <is>
-          <t>Sin Pedido</t>
+      <c r="L47" s="32" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -6193,22 +6377,22 @@
       </c>
       <c r="C48" s="28" t="inlineStr">
         <is>
-          <t>FTK0005</t>
+          <t>BEY0020</t>
         </is>
       </c>
       <c r="D48" s="27" t="inlineStr">
         <is>
-          <t>FITOKONTROL CA FLOW, 5 KG</t>
+          <t>FLORAMEC PLUS 20 L</t>
         </is>
       </c>
       <c r="E48" s="14" t="n">
-        <v>800</v>
+        <v>80</v>
       </c>
       <c r="F48" s="14" t="n">
-        <v>0</v>
+        <v>120</v>
       </c>
       <c r="G48" s="14" t="n">
-        <v>0</v>
+        <v>120</v>
       </c>
       <c r="H48" s="14" t="n">
         <v>0</v>
@@ -6225,9 +6409,9 @@
         <f>IF(E48&gt;0, F48/E48, IF(F48&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L48" s="33" t="inlineStr">
-        <is>
-          <t>Sin Pedido</t>
+      <c r="L48" s="29" t="inlineStr">
+        <is>
+          <t>Superado</t>
         </is>
       </c>
     </row>
@@ -6239,25 +6423,25 @@
       </c>
       <c r="C49" s="31" t="inlineStr">
         <is>
-          <t>TRI0001</t>
+          <t>BROTA0005</t>
         </is>
       </c>
       <c r="D49" s="30" t="inlineStr">
         <is>
-          <t>TRIFENO-94, 1 L</t>
+          <t>BROTAMEC, 5 L</t>
         </is>
       </c>
       <c r="E49" s="18" t="n">
-        <v>0</v>
+        <v>600</v>
       </c>
       <c r="F49" s="18" t="n">
-        <v>60</v>
+        <v>600</v>
       </c>
       <c r="G49" s="18" t="n">
-        <v>0</v>
+        <v>600</v>
       </c>
       <c r="H49" s="18" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="I49" s="18">
         <f>MAX(0, E49-F49)</f>
@@ -6273,7 +6457,7 @@
       </c>
       <c r="L49" s="32" t="inlineStr">
         <is>
-          <t>Extra Estimación</t>
+          <t>Superado</t>
         </is>
       </c>
     </row>
@@ -6285,25 +6469,25 @@
       </c>
       <c r="C50" s="28" t="inlineStr">
         <is>
-          <t>TRI0005</t>
+          <t>C-M-P0001</t>
         </is>
       </c>
       <c r="D50" s="27" t="inlineStr">
         <is>
-          <t>TRIFENO-94, 5L</t>
+          <t>CODIFOL Mo-PLUS, 1 L</t>
         </is>
       </c>
       <c r="E50" s="14" t="n">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="F50" s="14" t="n">
-        <v>600</v>
+        <v>0</v>
       </c>
       <c r="G50" s="14" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="H50" s="14" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="I50" s="14">
         <f>MAX(0, E50-F50)</f>
@@ -6317,36 +6501,36 @@
         <f>IF(E50&gt;0, F50/E50, IF(F50&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L50" s="29" t="inlineStr">
-        <is>
-          <t>Extra Estimación</t>
+      <c r="L50" s="33" t="inlineStr">
+        <is>
+          <t>Sin Pedido</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="B51" s="30" t="inlineStr">
         <is>
-          <t>SUCA, S.C.A.</t>
+          <t>GUIVARTO AGRICOLA, S.L.</t>
         </is>
       </c>
       <c r="C51" s="31" t="inlineStr">
         <is>
-          <t>AGXK0020</t>
+          <t>FTK0005</t>
         </is>
       </c>
       <c r="D51" s="30" t="inlineStr">
         <is>
-          <t>AGROXILATO-K, 20 L</t>
+          <t>FITOKONTROL CA FLOW, 5 KG</t>
         </is>
       </c>
       <c r="E51" s="18" t="n">
-        <v>0</v>
+        <v>800</v>
       </c>
       <c r="F51" s="18" t="n">
-        <v>640</v>
+        <v>0</v>
       </c>
       <c r="G51" s="18" t="n">
-        <v>640</v>
+        <v>0</v>
       </c>
       <c r="H51" s="18" t="n">
         <v>0</v>
@@ -6363,54 +6547,192 @@
         <f>IF(E51&gt;0, F51/E51, IF(F51&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L51" s="32" t="inlineStr">
+      <c r="L51" s="36" t="inlineStr">
+        <is>
+          <t>Sin Pedido</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="B52" s="27" t="inlineStr">
+        <is>
+          <t>GUIVARTO AGRICOLA, S.L.</t>
+        </is>
+      </c>
+      <c r="C52" s="28" t="inlineStr">
+        <is>
+          <t>TRI0001</t>
+        </is>
+      </c>
+      <c r="D52" s="27" t="inlineStr">
+        <is>
+          <t>TRIFENO-94, 1 L</t>
+        </is>
+      </c>
+      <c r="E52" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F52" s="14" t="n">
+        <v>60</v>
+      </c>
+      <c r="G52" s="14" t="n">
+        <v>60</v>
+      </c>
+      <c r="H52" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I52" s="14">
+        <f>MAX(0, E52-F52)</f>
+        <v/>
+      </c>
+      <c r="J52" s="14">
+        <f>ABS(F52-E52)</f>
+        <v/>
+      </c>
+      <c r="K52" s="15">
+        <f>IF(E52&gt;0, F52/E52, IF(F52&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L52" s="29" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
       </c>
     </row>
-    <row r="52" ht="24" customHeight="1">
-      <c r="B52" s="20" t="inlineStr">
+    <row r="53">
+      <c r="B53" s="30" t="inlineStr">
+        <is>
+          <t>GUIVARTO AGRICOLA, S.L.</t>
+        </is>
+      </c>
+      <c r="C53" s="31" t="inlineStr">
+        <is>
+          <t>TRI0005</t>
+        </is>
+      </c>
+      <c r="D53" s="30" t="inlineStr">
+        <is>
+          <t>TRIFENO-94, 5L</t>
+        </is>
+      </c>
+      <c r="E53" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F53" s="18" t="n">
+        <v>600</v>
+      </c>
+      <c r="G53" s="18" t="n">
+        <v>600</v>
+      </c>
+      <c r="H53" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="I53" s="18">
+        <f>MAX(0, E53-F53)</f>
+        <v/>
+      </c>
+      <c r="J53" s="18">
+        <f>ABS(F53-E53)</f>
+        <v/>
+      </c>
+      <c r="K53" s="19">
+        <f>IF(E53&gt;0, F53/E53, IF(F53&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L53" s="32" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="B54" s="27" t="inlineStr">
+        <is>
+          <t>SUCA, S.C.A.</t>
+        </is>
+      </c>
+      <c r="C54" s="28" t="inlineStr">
+        <is>
+          <t>AGXK0020</t>
+        </is>
+      </c>
+      <c r="D54" s="27" t="inlineStr">
+        <is>
+          <t>AGROXILATO-K, 20 L</t>
+        </is>
+      </c>
+      <c r="E54" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F54" s="14" t="n">
+        <v>640</v>
+      </c>
+      <c r="G54" s="14" t="n">
+        <v>640</v>
+      </c>
+      <c r="H54" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I54" s="14">
+        <f>MAX(0, E54-F54)</f>
+        <v/>
+      </c>
+      <c r="J54" s="14">
+        <f>ABS(F54-E54)</f>
+        <v/>
+      </c>
+      <c r="K54" s="15">
+        <f>IF(E54&gt;0, F54/E54, IF(F54&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L54" s="29" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="24" customHeight="1">
+      <c r="B55" s="20" t="inlineStr">
         <is>
           <t>TOTAL IRENE</t>
         </is>
       </c>
-      <c r="C52" s="34" t="inlineStr">
+      <c r="C55" s="34" t="inlineStr">
         <is>
           <t>89 líneas</t>
         </is>
       </c>
-      <c r="D52" s="35" t="inlineStr"/>
-      <c r="E52" s="22">
-        <f>SUM(E10:E51)</f>
-        <v/>
-      </c>
-      <c r="F52" s="22">
-        <f>SUM(F10:F51)</f>
-        <v/>
-      </c>
-      <c r="G52" s="22">
-        <f>SUM(G10:G51)</f>
-        <v/>
-      </c>
-      <c r="H52" s="22">
-        <f>SUM(H10:H51)</f>
-        <v/>
-      </c>
-      <c r="I52" s="22">
-        <f>SUM(I10:I51)</f>
-        <v/>
-      </c>
-      <c r="J52" s="22">
-        <f>SUM(J10:J51)</f>
-        <v/>
-      </c>
-      <c r="K52" s="23">
-        <f>IF(E52&gt;0, F52/E52, 0)</f>
-        <v/>
-      </c>
-      <c r="L52" s="21">
-        <f>IF(K52&gt;=1, "SUPERADO", "EN CURSO")</f>
+      <c r="D55" s="35" t="inlineStr"/>
+      <c r="E55" s="22">
+        <f>SUM(E10:E54)</f>
+        <v/>
+      </c>
+      <c r="F55" s="22">
+        <f>SUM(F10:F54)</f>
+        <v/>
+      </c>
+      <c r="G55" s="22">
+        <f>SUM(G10:G54)</f>
+        <v/>
+      </c>
+      <c r="H55" s="22">
+        <f>SUM(H10:H54)</f>
+        <v/>
+      </c>
+      <c r="I55" s="22">
+        <f>SUM(I10:I54)</f>
+        <v/>
+      </c>
+      <c r="J55" s="22">
+        <f>SUM(J10:J54)</f>
+        <v/>
+      </c>
+      <c r="K55" s="23">
+        <f>IF(E55&gt;0, F55/E55, 0)</f>
+        <v/>
+      </c>
+      <c r="L55" s="21">
+        <f>IF(K55&gt;=1, "SUPERADO", "EN CURSO")</f>
         <v/>
       </c>
     </row>
@@ -6439,7 +6761,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:L33"/>
+  <dimension ref="B2:L37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -6466,7 +6788,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 26/10/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 27/10/2026</t>
         </is>
       </c>
     </row>
@@ -6511,25 +6833,25 @@
       <c r="C6" s="4" t="n"/>
       <c r="D6" s="24" t="inlineStr">
         <is>
-          <t>13,560 u</t>
+          <t>14,822 u</t>
         </is>
       </c>
       <c r="E6" s="4" t="n"/>
-      <c r="F6" s="38" t="inlineStr">
-        <is>
-          <t>79.3%</t>
+      <c r="F6" s="41" t="inlineStr">
+        <is>
+          <t>86.7%</t>
         </is>
       </c>
       <c r="G6" s="4" t="n"/>
-      <c r="H6" s="38" t="inlineStr">
-        <is>
-          <t>3,540 u</t>
+      <c r="H6" s="41" t="inlineStr">
+        <is>
+          <t>2,278 u</t>
         </is>
       </c>
       <c r="I6" s="4" t="n"/>
       <c r="J6" s="24" t="inlineStr">
         <is>
-          <t>1,020 u</t>
+          <t>0 u</t>
         </is>
       </c>
       <c r="K6" s="4" t="n"/>
@@ -6851,10 +7173,10 @@
         <v>40</v>
       </c>
       <c r="G15" s="18" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="H15" s="18" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="I15" s="18">
         <f>MAX(0, E15-F15)</f>
@@ -6914,7 +7236,7 @@
         <f>IF(E16&gt;0, F16/E16, IF(F16&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L16" s="41" t="inlineStr">
+      <c r="L16" s="40" t="inlineStr">
         <is>
           <t>Rezagado</t>
         </is>
@@ -7219,10 +7541,10 @@
         <v>1000</v>
       </c>
       <c r="G23" s="18" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="H23" s="18" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="I23" s="18">
         <f>MAX(0, E23-F23)</f>
@@ -7567,27 +7889,27 @@
     <row r="31">
       <c r="B31" s="30" t="inlineStr">
         <is>
-          <t>FITOXENT S.C.L.V.</t>
+          <t>FITOSANITARIOS DRAGO S.L.U</t>
         </is>
       </c>
       <c r="C31" s="31" t="inlineStr">
         <is>
-          <t>FTK0005</t>
+          <t>AGZNP0005</t>
         </is>
       </c>
       <c r="D31" s="30" t="inlineStr">
         <is>
-          <t>FITOKONTROL CA FLOW, 5 KG</t>
+          <t>AGROXILATO ZN PLUS, 5 KG</t>
         </is>
       </c>
       <c r="E31" s="18" t="n">
-        <v>4400</v>
+        <v>0</v>
       </c>
       <c r="F31" s="18" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="G31" s="18" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="H31" s="18" t="n">
         <v>0</v>
@@ -7604,36 +7926,36 @@
         <f>IF(E31&gt;0, F31/E31, IF(F31&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L31" s="36" t="inlineStr">
-        <is>
-          <t>Sin Pedido</t>
+      <c r="L31" s="32" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="B32" s="27" t="inlineStr">
         <is>
-          <t>FITOXENT S.C.L.V.</t>
+          <t>FITOSANITARIOS DRAGO S.L.U</t>
         </is>
       </c>
       <c r="C32" s="28" t="inlineStr">
         <is>
-          <t>PT0020</t>
+          <t>B0001</t>
         </is>
       </c>
       <c r="D32" s="27" t="inlineStr">
         <is>
-          <t>AGROPOTASION, 20 L</t>
+          <t>BOROCAL,1 L</t>
         </is>
       </c>
       <c r="E32" s="14" t="n">
-        <v>2560</v>
+        <v>0</v>
       </c>
       <c r="F32" s="14" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="G32" s="14" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="H32" s="14" t="n">
         <v>0</v>
@@ -7650,54 +7972,238 @@
         <f>IF(E32&gt;0, F32/E32, IF(F32&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L32" s="33" t="inlineStr">
+      <c r="L32" s="29" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="30" t="inlineStr">
+        <is>
+          <t>FITOSANITARIOS DRAGO S.L.U</t>
+        </is>
+      </c>
+      <c r="C33" s="31" t="inlineStr">
+        <is>
+          <t>C-CU0005</t>
+        </is>
+      </c>
+      <c r="D33" s="30" t="inlineStr">
+        <is>
+          <t>CODICOBRE, 5 L</t>
+        </is>
+      </c>
+      <c r="E33" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F33" s="18" t="n">
+        <v>200</v>
+      </c>
+      <c r="G33" s="18" t="n">
+        <v>200</v>
+      </c>
+      <c r="H33" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="I33" s="18">
+        <f>MAX(0, E33-F33)</f>
+        <v/>
+      </c>
+      <c r="J33" s="18">
+        <f>ABS(F33-E33)</f>
+        <v/>
+      </c>
+      <c r="K33" s="19">
+        <f>IF(E33&gt;0, F33/E33, IF(F33&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L33" s="32" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="27" t="inlineStr">
+        <is>
+          <t>FITOSANITARIOS DRAGO S.L.U</t>
+        </is>
+      </c>
+      <c r="C34" s="28" t="inlineStr">
+        <is>
+          <t>S1000</t>
+        </is>
+      </c>
+      <c r="D34" s="27" t="inlineStr">
+        <is>
+          <t>SAL-WAX STAR, 1000 L</t>
+        </is>
+      </c>
+      <c r="E34" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" s="14" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G34" s="14" t="n">
+        <v>1000</v>
+      </c>
+      <c r="H34" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I34" s="14">
+        <f>MAX(0, E34-F34)</f>
+        <v/>
+      </c>
+      <c r="J34" s="14">
+        <f>ABS(F34-E34)</f>
+        <v/>
+      </c>
+      <c r="K34" s="15">
+        <f>IF(E34&gt;0, F34/E34, IF(F34&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L34" s="29" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="30" t="inlineStr">
+        <is>
+          <t>FITOXENT S.C.L.V.</t>
+        </is>
+      </c>
+      <c r="C35" s="31" t="inlineStr">
+        <is>
+          <t>FTK0005</t>
+        </is>
+      </c>
+      <c r="D35" s="30" t="inlineStr">
+        <is>
+          <t>FITOKONTROL CA FLOW, 5 KG</t>
+        </is>
+      </c>
+      <c r="E35" s="18" t="n">
+        <v>4400</v>
+      </c>
+      <c r="F35" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G35" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H35" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="I35" s="18">
+        <f>MAX(0, E35-F35)</f>
+        <v/>
+      </c>
+      <c r="J35" s="18">
+        <f>ABS(F35-E35)</f>
+        <v/>
+      </c>
+      <c r="K35" s="19">
+        <f>IF(E35&gt;0, F35/E35, IF(F35&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L35" s="36" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="24" customHeight="1">
-      <c r="B33" s="20" t="inlineStr">
+    <row r="36">
+      <c r="B36" s="27" t="inlineStr">
+        <is>
+          <t>FITOXENT S.C.L.V.</t>
+        </is>
+      </c>
+      <c r="C36" s="28" t="inlineStr">
+        <is>
+          <t>PT0020</t>
+        </is>
+      </c>
+      <c r="D36" s="27" t="inlineStr">
+        <is>
+          <t>AGROPOTASION, 20 L</t>
+        </is>
+      </c>
+      <c r="E36" s="14" t="n">
+        <v>2560</v>
+      </c>
+      <c r="F36" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G36" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H36" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I36" s="14">
+        <f>MAX(0, E36-F36)</f>
+        <v/>
+      </c>
+      <c r="J36" s="14">
+        <f>ABS(F36-E36)</f>
+        <v/>
+      </c>
+      <c r="K36" s="15">
+        <f>IF(E36&gt;0, F36/E36, IF(F36&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L36" s="33" t="inlineStr">
+        <is>
+          <t>Sin Pedido</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="24" customHeight="1">
+      <c r="B37" s="20" t="inlineStr">
         <is>
           <t>TOTAL JAVIER</t>
         </is>
       </c>
-      <c r="C33" s="34" t="inlineStr">
-        <is>
-          <t>179 líneas</t>
-        </is>
-      </c>
-      <c r="D33" s="35" t="inlineStr"/>
-      <c r="E33" s="22">
-        <f>SUM(E10:E32)</f>
-        <v/>
-      </c>
-      <c r="F33" s="22">
-        <f>SUM(F10:F32)</f>
-        <v/>
-      </c>
-      <c r="G33" s="22">
-        <f>SUM(G10:G32)</f>
-        <v/>
-      </c>
-      <c r="H33" s="22">
-        <f>SUM(H10:H32)</f>
-        <v/>
-      </c>
-      <c r="I33" s="22">
-        <f>SUM(I10:I32)</f>
-        <v/>
-      </c>
-      <c r="J33" s="22">
-        <f>SUM(J10:J32)</f>
-        <v/>
-      </c>
-      <c r="K33" s="23">
-        <f>IF(E33&gt;0, F33/E33, 0)</f>
-        <v/>
-      </c>
-      <c r="L33" s="21">
-        <f>IF(K33&gt;=1, "SUPERADO", "EN CURSO")</f>
+      <c r="C37" s="34" t="inlineStr">
+        <is>
+          <t>180 líneas</t>
+        </is>
+      </c>
+      <c r="D37" s="35" t="inlineStr"/>
+      <c r="E37" s="22">
+        <f>SUM(E10:E36)</f>
+        <v/>
+      </c>
+      <c r="F37" s="22">
+        <f>SUM(F10:F36)</f>
+        <v/>
+      </c>
+      <c r="G37" s="22">
+        <f>SUM(G10:G36)</f>
+        <v/>
+      </c>
+      <c r="H37" s="22">
+        <f>SUM(H10:H36)</f>
+        <v/>
+      </c>
+      <c r="I37" s="22">
+        <f>SUM(I10:I36)</f>
+        <v/>
+      </c>
+      <c r="J37" s="22">
+        <f>SUM(J10:J36)</f>
+        <v/>
+      </c>
+      <c r="K37" s="23">
+        <f>IF(E37&gt;0, F37/E37, 0)</f>
+        <v/>
+      </c>
+      <c r="L37" s="21">
+        <f>IF(K37&gt;=1, "SUPERADO", "EN CURSO")</f>
         <v/>
       </c>
     </row>
@@ -7753,7 +8259,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 26/10/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 27/10/2026</t>
         </is>
       </c>
     </row>
@@ -7802,13 +8308,13 @@
         </is>
       </c>
       <c r="E6" s="4" t="n"/>
-      <c r="F6" s="38" t="inlineStr">
+      <c r="F6" s="41" t="inlineStr">
         <is>
           <t>0.0%</t>
         </is>
       </c>
       <c r="G6" s="4" t="n"/>
-      <c r="H6" s="38" t="inlineStr">
+      <c r="H6" s="41" t="inlineStr">
         <is>
           <t>39,460 u</t>
         </is>
@@ -8231,7 +8737,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:L27"/>
+  <dimension ref="B2:L28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -8258,7 +8764,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 26/10/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 27/10/2026</t>
         </is>
       </c>
     </row>
@@ -8303,13 +8809,13 @@
       <c r="C6" s="4" t="n"/>
       <c r="D6" s="25" t="inlineStr">
         <is>
-          <t>17,400 u</t>
+          <t>17,500 u</t>
         </is>
       </c>
       <c r="E6" s="4" t="n"/>
       <c r="F6" s="25" t="inlineStr">
         <is>
-          <t>100.3%</t>
+          <t>100.9%</t>
         </is>
       </c>
       <c r="G6" s="4" t="n"/>
@@ -8660,7 +9166,7 @@
         <f>IF(E15&gt;0, F15/E15, IF(F15&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L15" s="40" t="inlineStr">
+      <c r="L15" s="39" t="inlineStr">
         <is>
           <t>Rezagado</t>
         </is>
@@ -9074,7 +9580,7 @@
         <f>IF(E24&gt;0, F24/E24, IF(F24&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L24" s="39" t="inlineStr">
+      <c r="L24" s="38" t="inlineStr">
         <is>
           <t>En Curso</t>
         </is>
@@ -9172,48 +9678,94 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="24" customHeight="1">
-      <c r="B27" s="20" t="inlineStr">
+    <row r="27">
+      <c r="B27" s="30" t="inlineStr">
+        <is>
+          <t>FITOMURCIA S.L.</t>
+        </is>
+      </c>
+      <c r="C27" s="31" t="inlineStr">
+        <is>
+          <t>C-M-P0005</t>
+        </is>
+      </c>
+      <c r="D27" s="30" t="inlineStr">
+        <is>
+          <t>CODIFOL MO-PLUS, 5 L</t>
+        </is>
+      </c>
+      <c r="E27" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" s="18" t="n">
+        <v>100</v>
+      </c>
+      <c r="G27" s="18" t="n">
+        <v>100</v>
+      </c>
+      <c r="H27" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="I27" s="18">
+        <f>MAX(0, E27-F27)</f>
+        <v/>
+      </c>
+      <c r="J27" s="18">
+        <f>ABS(F27-E27)</f>
+        <v/>
+      </c>
+      <c r="K27" s="19">
+        <f>IF(E27&gt;0, F27/E27, IF(F27&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L27" s="32" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="24" customHeight="1">
+      <c r="B28" s="20" t="inlineStr">
         <is>
           <t>TOTAL PEDRO</t>
         </is>
       </c>
-      <c r="C27" s="34" t="inlineStr">
+      <c r="C28" s="34" t="inlineStr">
         <is>
           <t>104 líneas</t>
         </is>
       </c>
-      <c r="D27" s="35" t="inlineStr"/>
-      <c r="E27" s="22">
-        <f>SUM(E10:E26)</f>
-        <v/>
-      </c>
-      <c r="F27" s="22">
-        <f>SUM(F10:F26)</f>
-        <v/>
-      </c>
-      <c r="G27" s="22">
-        <f>SUM(G10:G26)</f>
-        <v/>
-      </c>
-      <c r="H27" s="22">
-        <f>SUM(H10:H26)</f>
-        <v/>
-      </c>
-      <c r="I27" s="22">
-        <f>SUM(I10:I26)</f>
-        <v/>
-      </c>
-      <c r="J27" s="22">
-        <f>SUM(J10:J26)</f>
-        <v/>
-      </c>
-      <c r="K27" s="23">
-        <f>IF(E27&gt;0, F27/E27, 0)</f>
-        <v/>
-      </c>
-      <c r="L27" s="21">
-        <f>IF(K27&gt;=1, "SUPERADO", "EN CURSO")</f>
+      <c r="D28" s="35" t="inlineStr"/>
+      <c r="E28" s="22">
+        <f>SUM(E10:E27)</f>
+        <v/>
+      </c>
+      <c r="F28" s="22">
+        <f>SUM(F10:F27)</f>
+        <v/>
+      </c>
+      <c r="G28" s="22">
+        <f>SUM(G10:G27)</f>
+        <v/>
+      </c>
+      <c r="H28" s="22">
+        <f>SUM(H10:H27)</f>
+        <v/>
+      </c>
+      <c r="I28" s="22">
+        <f>SUM(I10:I27)</f>
+        <v/>
+      </c>
+      <c r="J28" s="22">
+        <f>SUM(J10:J27)</f>
+        <v/>
+      </c>
+      <c r="K28" s="23">
+        <f>IF(E28&gt;0, F28/E28, 0)</f>
+        <v/>
+      </c>
+      <c r="L28" s="21">
+        <f>IF(K28&gt;=1, "SUPERADO", "EN CURSO")</f>
         <v/>
       </c>
     </row>
@@ -9242,7 +9794,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:L47"/>
+  <dimension ref="B2:L50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -9269,7 +9821,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 26/10/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 27/10/2026</t>
         </is>
       </c>
     </row>
@@ -9314,13 +9866,13 @@
       <c r="C6" s="4" t="n"/>
       <c r="D6" s="25" t="inlineStr">
         <is>
-          <t>109,072 u</t>
+          <t>109,376 u</t>
         </is>
       </c>
       <c r="E6" s="4" t="n"/>
       <c r="F6" s="25" t="inlineStr">
         <is>
-          <t>237.1%</t>
+          <t>237.8%</t>
         </is>
       </c>
       <c r="G6" s="4" t="n"/>
@@ -9332,7 +9884,7 @@
       <c r="I6" s="4" t="n"/>
       <c r="J6" s="24" t="inlineStr">
         <is>
-          <t>109,072 u</t>
+          <t>109,376 u</t>
         </is>
       </c>
       <c r="K6" s="4" t="n"/>
@@ -10881,25 +11433,25 @@
       </c>
       <c r="C42" s="28" t="inlineStr">
         <is>
-          <t>SPCE2B0001</t>
+          <t>RUN0001</t>
         </is>
       </c>
       <c r="D42" s="27" t="inlineStr">
         <is>
-          <t>SPRINTENE</t>
+          <t>RUN STRESS</t>
         </is>
       </c>
       <c r="E42" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F42" s="14" t="n">
-        <v>300</v>
+        <v>204</v>
       </c>
       <c r="G42" s="14" t="n">
         <v>0</v>
       </c>
       <c r="H42" s="14" t="n">
-        <v>300</v>
+        <v>204</v>
       </c>
       <c r="I42" s="14">
         <f>MAX(0, E42-F42)</f>
@@ -10927,25 +11479,25 @@
       </c>
       <c r="C43" s="31" t="inlineStr">
         <is>
-          <t>SS0001</t>
+          <t>SPCE2B0001</t>
         </is>
       </c>
       <c r="D43" s="30" t="inlineStr">
         <is>
-          <t>SAL-WAX</t>
+          <t>SPRINTENE</t>
         </is>
       </c>
       <c r="E43" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F43" s="18" t="n">
-        <v>1088</v>
+        <v>300</v>
       </c>
       <c r="G43" s="18" t="n">
         <v>0</v>
       </c>
       <c r="H43" s="18" t="n">
-        <v>1088</v>
+        <v>300</v>
       </c>
       <c r="I43" s="18">
         <f>MAX(0, E43-F43)</f>
@@ -10973,25 +11525,25 @@
       </c>
       <c r="C44" s="28" t="inlineStr">
         <is>
-          <t>START20001</t>
+          <t>SS0001</t>
         </is>
       </c>
       <c r="D44" s="27" t="inlineStr">
         <is>
-          <t>RADISOL</t>
+          <t>SAL-WAX</t>
         </is>
       </c>
       <c r="E44" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F44" s="14" t="n">
-        <v>2904</v>
+        <v>1088</v>
       </c>
       <c r="G44" s="14" t="n">
         <v>0</v>
       </c>
       <c r="H44" s="14" t="n">
-        <v>2904</v>
+        <v>1088</v>
       </c>
       <c r="I44" s="14">
         <f>MAX(0, E44-F44)</f>
@@ -11014,30 +11566,30 @@
     <row r="45">
       <c r="B45" s="30" t="inlineStr">
         <is>
-          <t>LEKKERBIO B.V.</t>
+          <t>JUAN JIMENEZ, SRL</t>
         </is>
       </c>
       <c r="C45" s="31" t="inlineStr">
         <is>
-          <t>AO0020</t>
+          <t>START20001</t>
         </is>
       </c>
       <c r="D45" s="30" t="inlineStr">
         <is>
-          <t>ALCAPLANT NEW</t>
+          <t>RADISOL</t>
         </is>
       </c>
       <c r="E45" s="18" t="n">
-        <v>44000</v>
+        <v>0</v>
       </c>
       <c r="F45" s="18" t="n">
-        <v>19800</v>
+        <v>2904</v>
       </c>
       <c r="G45" s="18" t="n">
         <v>0</v>
       </c>
       <c r="H45" s="18" t="n">
-        <v>19800</v>
+        <v>2904</v>
       </c>
       <c r="I45" s="18">
         <f>MAX(0, E45-F45)</f>
@@ -11051,9 +11603,9 @@
         <f>IF(E45&gt;0, F45/E45, IF(F45&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L45" s="40" t="inlineStr">
-        <is>
-          <t>Rezagado</t>
+      <c r="L45" s="32" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -11065,25 +11617,25 @@
       </c>
       <c r="C46" s="28" t="inlineStr">
         <is>
-          <t>DECA0020</t>
+          <t>AO0020</t>
         </is>
       </c>
       <c r="D46" s="27" t="inlineStr">
         <is>
-          <t>DEFENS-CA-AE, 20 KG</t>
+          <t>ALCAPLANT NEW</t>
         </is>
       </c>
       <c r="E46" s="14" t="n">
-        <v>0</v>
+        <v>44000</v>
       </c>
       <c r="F46" s="14" t="n">
-        <v>3000</v>
+        <v>19800</v>
       </c>
       <c r="G46" s="14" t="n">
         <v>0</v>
       </c>
       <c r="H46" s="14" t="n">
-        <v>3000</v>
+        <v>19800</v>
       </c>
       <c r="I46" s="14">
         <f>MAX(0, E46-F46)</f>
@@ -11097,54 +11649,192 @@
         <f>IF(E46&gt;0, F46/E46, IF(F46&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L46" s="29" t="inlineStr">
+      <c r="L46" s="40" t="inlineStr">
+        <is>
+          <t>Rezagado</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="B47" s="30" t="inlineStr">
+        <is>
+          <t>LEKKERBIO B.V.</t>
+        </is>
+      </c>
+      <c r="C47" s="31" t="inlineStr">
+        <is>
+          <t>CAG</t>
+        </is>
+      </c>
+      <c r="D47" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAJA "CODIAGRO NUEVA CALIDAD"  5L       </t>
+        </is>
+      </c>
+      <c r="E47" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F47" s="18" t="n">
+        <v>60</v>
+      </c>
+      <c r="G47" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H47" s="18" t="n">
+        <v>60</v>
+      </c>
+      <c r="I47" s="18">
+        <f>MAX(0, E47-F47)</f>
+        <v/>
+      </c>
+      <c r="J47" s="18">
+        <f>ABS(F47-E47)</f>
+        <v/>
+      </c>
+      <c r="K47" s="19">
+        <f>IF(E47&gt;0, F47/E47, IF(F47&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L47" s="32" t="inlineStr">
         <is>
           <t>Extra Estimación</t>
         </is>
       </c>
     </row>
-    <row r="47" ht="24" customHeight="1">
-      <c r="B47" s="20" t="inlineStr">
+    <row r="48">
+      <c r="B48" s="27" t="inlineStr">
+        <is>
+          <t>LEKKERBIO B.V.</t>
+        </is>
+      </c>
+      <c r="C48" s="28" t="inlineStr">
+        <is>
+          <t>CWH</t>
+        </is>
+      </c>
+      <c r="D48" s="27" t="inlineStr">
+        <is>
+          <t>CAJA AGROWHITE</t>
+        </is>
+      </c>
+      <c r="E48" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F48" s="14" t="n">
+        <v>40</v>
+      </c>
+      <c r="G48" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H48" s="14" t="n">
+        <v>40</v>
+      </c>
+      <c r="I48" s="14">
+        <f>MAX(0, E48-F48)</f>
+        <v/>
+      </c>
+      <c r="J48" s="14">
+        <f>ABS(F48-E48)</f>
+        <v/>
+      </c>
+      <c r="K48" s="15">
+        <f>IF(E48&gt;0, F48/E48, IF(F48&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L48" s="29" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="B49" s="30" t="inlineStr">
+        <is>
+          <t>LEKKERBIO B.V.</t>
+        </is>
+      </c>
+      <c r="C49" s="31" t="inlineStr">
+        <is>
+          <t>DECA0020</t>
+        </is>
+      </c>
+      <c r="D49" s="30" t="inlineStr">
+        <is>
+          <t>DEFENS-CA-AE, 20 KG</t>
+        </is>
+      </c>
+      <c r="E49" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F49" s="18" t="n">
+        <v>3000</v>
+      </c>
+      <c r="G49" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H49" s="18" t="n">
+        <v>3000</v>
+      </c>
+      <c r="I49" s="18">
+        <f>MAX(0, E49-F49)</f>
+        <v/>
+      </c>
+      <c r="J49" s="18">
+        <f>ABS(F49-E49)</f>
+        <v/>
+      </c>
+      <c r="K49" s="19">
+        <f>IF(E49&gt;0, F49/E49, IF(F49&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L49" s="32" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="24" customHeight="1">
+      <c r="B50" s="20" t="inlineStr">
         <is>
           <t>TOTAL RICARDO</t>
         </is>
       </c>
-      <c r="C47" s="34" t="inlineStr">
-        <is>
-          <t>128 líneas</t>
-        </is>
-      </c>
-      <c r="D47" s="35" t="inlineStr"/>
-      <c r="E47" s="22">
-        <f>SUM(E10:E46)</f>
-        <v/>
-      </c>
-      <c r="F47" s="22">
-        <f>SUM(F10:F46)</f>
-        <v/>
-      </c>
-      <c r="G47" s="22">
-        <f>SUM(G10:G46)</f>
-        <v/>
-      </c>
-      <c r="H47" s="22">
-        <f>SUM(H10:H46)</f>
-        <v/>
-      </c>
-      <c r="I47" s="22">
-        <f>SUM(I10:I46)</f>
-        <v/>
-      </c>
-      <c r="J47" s="22">
-        <f>SUM(J10:J46)</f>
-        <v/>
-      </c>
-      <c r="K47" s="23">
-        <f>IF(E47&gt;0, F47/E47, 0)</f>
-        <v/>
-      </c>
-      <c r="L47" s="21">
-        <f>IF(K47&gt;=1, "SUPERADO", "EN CURSO")</f>
+      <c r="C50" s="34" t="inlineStr">
+        <is>
+          <t>130 líneas</t>
+        </is>
+      </c>
+      <c r="D50" s="35" t="inlineStr"/>
+      <c r="E50" s="22">
+        <f>SUM(E10:E49)</f>
+        <v/>
+      </c>
+      <c r="F50" s="22">
+        <f>SUM(F10:F49)</f>
+        <v/>
+      </c>
+      <c r="G50" s="22">
+        <f>SUM(G10:G49)</f>
+        <v/>
+      </c>
+      <c r="H50" s="22">
+        <f>SUM(H10:H49)</f>
+        <v/>
+      </c>
+      <c r="I50" s="22">
+        <f>SUM(I10:I49)</f>
+        <v/>
+      </c>
+      <c r="J50" s="22">
+        <f>SUM(J10:J49)</f>
+        <v/>
+      </c>
+      <c r="K50" s="23">
+        <f>IF(E50&gt;0, F50/E50, 0)</f>
+        <v/>
+      </c>
+      <c r="L50" s="21">
+        <f>IF(K50&gt;=1, "SUPERADO", "EN CURSO")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizacion pedidos 28.10: comercial, MRP, tesoreria y seguimiento
</commit_message>
<xml_diff>
--- a/Seguimiento_Presupuesto_Sep_2026.xlsx
+++ b/Seguimiento_Presupuesto_Sep_2026.xlsx
@@ -335,14 +335,14 @@
     <xf numFmtId="0" fontId="14" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="8" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -915,7 +915,7 @@
     <row r="3" ht="20" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Comparativa Estimación Septiembre (Unidades) vs Pedidos Reales a Fecha 27/10/2026 | Generado: 27/10/2026 07:39</t>
+          <t>Comparativa Estimación Septiembre (Unidades) vs Pedidos Reales a Fecha 28/10/2026 | Generado: 28/10/2026 09:31</t>
         </is>
       </c>
     </row>
@@ -959,25 +959,25 @@
       <c r="C6" s="4" t="n"/>
       <c r="D6" s="8" t="inlineStr">
         <is>
-          <t>254,091 u</t>
+          <t>264,355 u</t>
         </is>
       </c>
       <c r="E6" s="4" t="n"/>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>139.6%</t>
+          <t>145.3%</t>
         </is>
       </c>
       <c r="G6" s="4" t="n"/>
       <c r="H6" s="9" t="inlineStr">
         <is>
-          <t>41,738 u</t>
+          <t>34,106 u</t>
         </is>
       </c>
       <c r="I6" s="4" t="n"/>
       <c r="J6" s="7" t="inlineStr">
         <is>
-          <t>187,680 u</t>
+          <t>194,436 u</t>
         </is>
       </c>
     </row>
@@ -1048,20 +1048,20 @@
         <v>2320</v>
       </c>
       <c r="E10" s="14" t="n">
-        <v>7164</v>
+        <v>7804</v>
       </c>
       <c r="F10" s="14" t="n">
         <v>7164</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>0</v>
+        <v>640</v>
       </c>
       <c r="H10" s="14">
         <f>MAX(0, D10-E10)</f>
         <v/>
       </c>
       <c r="I10" s="14">
-        <f>'Alfonso'!J28</f>
+        <f>'Alfonso'!J29</f>
         <v/>
       </c>
       <c r="J10" s="15">
@@ -1110,26 +1110,26 @@
         </is>
       </c>
       <c r="C12" s="13" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D12" s="14" t="n">
         <v>21914</v>
       </c>
       <c r="E12" s="14" t="n">
+        <v>25745</v>
+      </c>
+      <c r="F12" s="14" t="n">
         <v>23753</v>
       </c>
-      <c r="F12" s="14" t="n">
-        <v>20245</v>
-      </c>
       <c r="G12" s="14" t="n">
-        <v>3508</v>
+        <v>1992</v>
       </c>
       <c r="H12" s="14">
         <f>MAX(0, D12-E12)</f>
         <v/>
       </c>
       <c r="I12" s="14">
-        <f>'Irene'!J55</f>
+        <f>'Irene'!J57</f>
         <v/>
       </c>
       <c r="J12" s="15">
@@ -1178,26 +1178,26 @@
         </is>
       </c>
       <c r="C14" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D14" s="14" t="n">
         <v>39460</v>
       </c>
       <c r="E14" s="14" t="n">
-        <v>0</v>
+        <v>7632</v>
       </c>
       <c r="F14" s="14" t="n">
         <v>0</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>0</v>
+        <v>7632</v>
       </c>
       <c r="H14" s="14">
         <f>MAX(0, D14-E14)</f>
         <v/>
       </c>
       <c r="I14" s="14">
-        <f>'Mehmet'!J16</f>
+        <f>'Mehmet'!J23</f>
         <v/>
       </c>
       <c r="J14" s="15">
@@ -1336,7 +1336,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:L28"/>
+  <dimension ref="B2:L29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1363,7 +1363,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 27/10/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 28/10/2026</t>
         </is>
       </c>
     </row>
@@ -1408,13 +1408,13 @@
       <c r="C6" s="4" t="n"/>
       <c r="D6" s="25" t="inlineStr">
         <is>
-          <t>7,164 u</t>
+          <t>7,804 u</t>
         </is>
       </c>
       <c r="E6" s="4" t="n"/>
       <c r="F6" s="25" t="inlineStr">
         <is>
-          <t>308.8%</t>
+          <t>336.4%</t>
         </is>
       </c>
       <c r="G6" s="4" t="n"/>
@@ -1426,7 +1426,7 @@
       <c r="I6" s="4" t="n"/>
       <c r="J6" s="24" t="inlineStr">
         <is>
-          <t>0 u</t>
+          <t>640 u</t>
         </is>
       </c>
       <c r="K6" s="4" t="n"/>
@@ -1590,17 +1590,17 @@
     <row r="12">
       <c r="B12" s="27" t="inlineStr">
         <is>
-          <t>AGROCAMP CANET S.L.</t>
+          <t>ACTIV. PRODUC. Y COMERC. LA VEGUILLA, SL</t>
         </is>
       </c>
       <c r="C12" s="28" t="inlineStr">
         <is>
-          <t>AGXK0020</t>
+          <t>C-CU0020</t>
         </is>
       </c>
       <c r="D12" s="27" t="inlineStr">
         <is>
-          <t>AGROXILATO-K, 20 L</t>
+          <t>CODICOBRE, 20 L</t>
         </is>
       </c>
       <c r="E12" s="14" t="n">
@@ -1610,10 +1610,10 @@
         <v>640</v>
       </c>
       <c r="G12" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="14" t="n">
         <v>640</v>
-      </c>
-      <c r="H12" s="14" t="n">
-        <v>0</v>
       </c>
       <c r="I12" s="14">
         <f>MAX(0, E12-F12)</f>
@@ -1636,27 +1636,27 @@
     <row r="13">
       <c r="B13" s="30" t="inlineStr">
         <is>
-          <t>AGROTÉCNICA DEL NORTE, S.L</t>
+          <t>AGROCAMP CANET S.L.</t>
         </is>
       </c>
       <c r="C13" s="31" t="inlineStr">
         <is>
-          <t>A-50(2)0005</t>
+          <t>AGXK0020</t>
         </is>
       </c>
       <c r="D13" s="30" t="inlineStr">
         <is>
-          <t>CODIORGAN-A50, 5 KG</t>
+          <t>AGROXILATO-K, 20 L</t>
         </is>
       </c>
       <c r="E13" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F13" s="18" t="n">
-        <v>300</v>
+        <v>640</v>
       </c>
       <c r="G13" s="18" t="n">
-        <v>300</v>
+        <v>640</v>
       </c>
       <c r="H13" s="18" t="n">
         <v>0</v>
@@ -1687,12 +1687,12 @@
       </c>
       <c r="C14" s="28" t="inlineStr">
         <is>
-          <t>BR-590005</t>
+          <t>A-50(2)0005</t>
         </is>
       </c>
       <c r="D14" s="27" t="inlineStr">
         <is>
-          <t>BR-59, 5 KG</t>
+          <t>CODIORGAN-A50, 5 KG</t>
         </is>
       </c>
       <c r="E14" s="14" t="n">
@@ -1733,22 +1733,22 @@
       </c>
       <c r="C15" s="31" t="inlineStr">
         <is>
-          <t>PT0005</t>
+          <t>BR-590005</t>
         </is>
       </c>
       <c r="D15" s="30" t="inlineStr">
         <is>
-          <t>AGROPOTASION, 5 L</t>
+          <t>BR-59, 5 KG</t>
         </is>
       </c>
       <c r="E15" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F15" s="18" t="n">
-        <v>400</v>
+        <v>300</v>
       </c>
       <c r="G15" s="18" t="n">
-        <v>400</v>
+        <v>300</v>
       </c>
       <c r="H15" s="18" t="n">
         <v>0</v>
@@ -1774,27 +1774,27 @@
     <row r="16">
       <c r="B16" s="27" t="inlineStr">
         <is>
-          <t>AGROVEYCA,S.L</t>
+          <t>AGROTÉCNICA DEL NORTE, S.L</t>
         </is>
       </c>
       <c r="C16" s="28" t="inlineStr">
         <is>
-          <t>AN0020</t>
+          <t>PT0005</t>
         </is>
       </c>
       <c r="D16" s="27" t="inlineStr">
         <is>
-          <t>ALCAPLANT NEW, 20 KG</t>
+          <t>AGROPOTASION, 5 L</t>
         </is>
       </c>
       <c r="E16" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F16" s="14" t="n">
-        <v>1100</v>
+        <v>400</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>1100</v>
+        <v>400</v>
       </c>
       <c r="H16" s="14" t="n">
         <v>0</v>
@@ -1825,22 +1825,22 @@
       </c>
       <c r="C17" s="31" t="inlineStr">
         <is>
-          <t>AQUOM0020</t>
+          <t>AN0020</t>
         </is>
       </c>
       <c r="D17" s="30" t="inlineStr">
         <is>
-          <t>AQUOM, 20 L</t>
+          <t>ALCAPLANT NEW, 20 KG</t>
         </is>
       </c>
       <c r="E17" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F17" s="18" t="n">
-        <v>320</v>
+        <v>1100</v>
       </c>
       <c r="G17" s="18" t="n">
-        <v>320</v>
+        <v>1100</v>
       </c>
       <c r="H17" s="18" t="n">
         <v>0</v>
@@ -1871,22 +1871,22 @@
       </c>
       <c r="C18" s="28" t="inlineStr">
         <is>
-          <t>BIO0020</t>
+          <t>AQUOM0020</t>
         </is>
       </c>
       <c r="D18" s="27" t="inlineStr">
         <is>
-          <t>BIORAD-20, 20 L</t>
+          <t>AQUOM, 20 L</t>
         </is>
       </c>
       <c r="E18" s="14" t="n">
-        <v>400</v>
+        <v>0</v>
       </c>
       <c r="F18" s="14" t="n">
-        <v>0</v>
+        <v>320</v>
       </c>
       <c r="G18" s="14" t="n">
-        <v>0</v>
+        <v>320</v>
       </c>
       <c r="H18" s="14" t="n">
         <v>0</v>
@@ -1903,9 +1903,9 @@
         <f>IF(E18&gt;0, F18/E18, IF(F18&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L18" s="33" t="inlineStr">
-        <is>
-          <t>Sin Pedido</t>
+      <c r="L18" s="29" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -1917,22 +1917,22 @@
       </c>
       <c r="C19" s="31" t="inlineStr">
         <is>
-          <t>S0020</t>
+          <t>BIO0020</t>
         </is>
       </c>
       <c r="D19" s="30" t="inlineStr">
         <is>
-          <t>SAL-WAX STAR, 20 L</t>
+          <t>BIORAD-20, 20 L</t>
         </is>
       </c>
       <c r="E19" s="18" t="n">
-        <v>0</v>
+        <v>400</v>
       </c>
       <c r="F19" s="18" t="n">
-        <v>640</v>
+        <v>0</v>
       </c>
       <c r="G19" s="18" t="n">
-        <v>640</v>
+        <v>0</v>
       </c>
       <c r="H19" s="18" t="n">
         <v>0</v>
@@ -1949,36 +1949,36 @@
         <f>IF(E19&gt;0, F19/E19, IF(F19&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L19" s="32" t="inlineStr">
-        <is>
-          <t>Extra Estimación</t>
+      <c r="L19" s="33" t="inlineStr">
+        <is>
+          <t>Sin Pedido</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="B20" s="27" t="inlineStr">
         <is>
-          <t>PLANTALDIA SLU</t>
+          <t>AGROVEYCA,S.L</t>
         </is>
       </c>
       <c r="C20" s="28" t="inlineStr">
         <is>
-          <t>A-50(2)0005</t>
+          <t>S0020</t>
         </is>
       </c>
       <c r="D20" s="27" t="inlineStr">
         <is>
-          <t>CODIORGAN A-50, 5 KG</t>
+          <t>SAL-WAX STAR, 20 L</t>
         </is>
       </c>
       <c r="E20" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F20" s="14" t="n">
-        <v>100</v>
+        <v>640</v>
       </c>
       <c r="G20" s="14" t="n">
-        <v>100</v>
+        <v>640</v>
       </c>
       <c r="H20" s="14" t="n">
         <v>0</v>
@@ -2009,22 +2009,22 @@
       </c>
       <c r="C21" s="31" t="inlineStr">
         <is>
-          <t>C-L0005</t>
+          <t>A-50(2)0005</t>
         </is>
       </c>
       <c r="D21" s="30" t="inlineStr">
         <is>
-          <t>CODIBOR-L, 5 L</t>
+          <t>CODIORGAN A-50, 5 KG</t>
         </is>
       </c>
       <c r="E21" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F21" s="18" t="n">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="G21" s="18" t="n">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="H21" s="18" t="n">
         <v>0</v>
@@ -2050,27 +2050,27 @@
     <row r="22">
       <c r="B22" s="27" t="inlineStr">
         <is>
-          <t>VILLALTA SATIVUM, S.L.</t>
+          <t>PLANTALDIA SLU</t>
         </is>
       </c>
       <c r="C22" s="28" t="inlineStr">
         <is>
-          <t>AGXKAEP0020</t>
+          <t>C-L0005</t>
         </is>
       </c>
       <c r="D22" s="27" t="inlineStr">
         <is>
-          <t>BIOCULTURE POTASIO PLUS, 20 L</t>
+          <t>CODIBOR-L, 5 L</t>
         </is>
       </c>
       <c r="E22" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F22" s="14" t="n">
-        <v>140</v>
+        <v>200</v>
       </c>
       <c r="G22" s="14" t="n">
-        <v>140</v>
+        <v>200</v>
       </c>
       <c r="H22" s="14" t="n">
         <v>0</v>
@@ -2101,22 +2101,22 @@
       </c>
       <c r="C23" s="31" t="inlineStr">
         <is>
-          <t>AQUOM0020</t>
+          <t>AGXKAEP0020</t>
         </is>
       </c>
       <c r="D23" s="30" t="inlineStr">
         <is>
-          <t>AQUOM, 20 L</t>
+          <t>BIOCULTURE POTASIO PLUS, 20 L</t>
         </is>
       </c>
       <c r="E23" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F23" s="18" t="n">
-        <v>40</v>
+        <v>140</v>
       </c>
       <c r="G23" s="18" t="n">
-        <v>40</v>
+        <v>140</v>
       </c>
       <c r="H23" s="18" t="n">
         <v>0</v>
@@ -2147,22 +2147,22 @@
       </c>
       <c r="C24" s="28" t="inlineStr">
         <is>
-          <t>C-CUAE0020</t>
+          <t>AQUOM0020</t>
         </is>
       </c>
       <c r="D24" s="27" t="inlineStr">
         <is>
-          <t>CUPRAMEC, 20 L</t>
+          <t>AQUOM, 20 L</t>
         </is>
       </c>
       <c r="E24" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F24" s="14" t="n">
-        <v>200</v>
+        <v>40</v>
       </c>
       <c r="G24" s="14" t="n">
-        <v>200</v>
+        <v>40</v>
       </c>
       <c r="H24" s="14" t="n">
         <v>0</v>
@@ -2193,22 +2193,22 @@
       </c>
       <c r="C25" s="31" t="inlineStr">
         <is>
-          <t>PT0001</t>
+          <t>C-CUAE0020</t>
         </is>
       </c>
       <c r="D25" s="30" t="inlineStr">
         <is>
-          <t>AGROPOTASION, 1 L</t>
+          <t>CUPRAMEC, 20 L</t>
         </is>
       </c>
       <c r="E25" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F25" s="18" t="n">
-        <v>24</v>
+        <v>200</v>
       </c>
       <c r="G25" s="18" t="n">
-        <v>24</v>
+        <v>200</v>
       </c>
       <c r="H25" s="18" t="n">
         <v>0</v>
@@ -2239,22 +2239,22 @@
       </c>
       <c r="C26" s="28" t="inlineStr">
         <is>
-          <t>PT0005</t>
+          <t>PT0001</t>
         </is>
       </c>
       <c r="D26" s="27" t="inlineStr">
         <is>
-          <t>AGROPOTASION, 5 L</t>
+          <t>AGROPOTASION, 1 L</t>
         </is>
       </c>
       <c r="E26" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F26" s="14" t="n">
-        <v>100</v>
+        <v>24</v>
       </c>
       <c r="G26" s="14" t="n">
-        <v>100</v>
+        <v>24</v>
       </c>
       <c r="H26" s="14" t="n">
         <v>0</v>
@@ -2285,12 +2285,12 @@
       </c>
       <c r="C27" s="31" t="inlineStr">
         <is>
-          <t>PT0020</t>
+          <t>PT0005</t>
         </is>
       </c>
       <c r="D27" s="30" t="inlineStr">
         <is>
-          <t>AGROPOTASION, 20 L</t>
+          <t>AGROPOTASION, 5 L</t>
         </is>
       </c>
       <c r="E27" s="18" t="n">
@@ -2323,48 +2323,94 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="24" customHeight="1">
-      <c r="B28" s="20" t="inlineStr">
+    <row r="28">
+      <c r="B28" s="27" t="inlineStr">
+        <is>
+          <t>VILLALTA SATIVUM, S.L.</t>
+        </is>
+      </c>
+      <c r="C28" s="28" t="inlineStr">
+        <is>
+          <t>PT0020</t>
+        </is>
+      </c>
+      <c r="D28" s="27" t="inlineStr">
+        <is>
+          <t>AGROPOTASION, 20 L</t>
+        </is>
+      </c>
+      <c r="E28" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" s="14" t="n">
+        <v>100</v>
+      </c>
+      <c r="G28" s="14" t="n">
+        <v>100</v>
+      </c>
+      <c r="H28" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I28" s="14">
+        <f>MAX(0, E28-F28)</f>
+        <v/>
+      </c>
+      <c r="J28" s="14">
+        <f>ABS(F28-E28)</f>
+        <v/>
+      </c>
+      <c r="K28" s="15">
+        <f>IF(E28&gt;0, F28/E28, IF(F28&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L28" s="29" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="24" customHeight="1">
+      <c r="B29" s="20" t="inlineStr">
         <is>
           <t>TOTAL ALFONSO</t>
         </is>
       </c>
-      <c r="C28" s="34" t="inlineStr">
-        <is>
-          <t>279 líneas</t>
-        </is>
-      </c>
-      <c r="D28" s="35" t="inlineStr"/>
-      <c r="E28" s="22">
-        <f>SUM(E10:E27)</f>
-        <v/>
-      </c>
-      <c r="F28" s="22">
-        <f>SUM(F10:F27)</f>
-        <v/>
-      </c>
-      <c r="G28" s="22">
-        <f>SUM(G10:G27)</f>
-        <v/>
-      </c>
-      <c r="H28" s="22">
-        <f>SUM(H10:H27)</f>
-        <v/>
-      </c>
-      <c r="I28" s="22">
-        <f>SUM(I10:I27)</f>
-        <v/>
-      </c>
-      <c r="J28" s="22">
-        <f>SUM(J10:J27)</f>
-        <v/>
-      </c>
-      <c r="K28" s="23">
-        <f>IF(E28&gt;0, F28/E28, 0)</f>
-        <v/>
-      </c>
-      <c r="L28" s="21">
-        <f>IF(K28&gt;=1, "SUPERADO", "EN CURSO")</f>
+      <c r="C29" s="34" t="inlineStr">
+        <is>
+          <t>280 líneas</t>
+        </is>
+      </c>
+      <c r="D29" s="35" t="inlineStr"/>
+      <c r="E29" s="22">
+        <f>SUM(E10:E28)</f>
+        <v/>
+      </c>
+      <c r="F29" s="22">
+        <f>SUM(F10:F28)</f>
+        <v/>
+      </c>
+      <c r="G29" s="22">
+        <f>SUM(G10:G28)</f>
+        <v/>
+      </c>
+      <c r="H29" s="22">
+        <f>SUM(H10:H28)</f>
+        <v/>
+      </c>
+      <c r="I29" s="22">
+        <f>SUM(I10:I28)</f>
+        <v/>
+      </c>
+      <c r="J29" s="22">
+        <f>SUM(J10:J28)</f>
+        <v/>
+      </c>
+      <c r="K29" s="23">
+        <f>IF(E29&gt;0, F29/E29, 0)</f>
+        <v/>
+      </c>
+      <c r="L29" s="21">
+        <f>IF(K29&gt;=1, "SUPERADO", "EN CURSO")</f>
         <v/>
       </c>
     </row>
@@ -2420,7 +2466,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 27/10/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 28/10/2026</t>
         </is>
       </c>
     </row>
@@ -2592,7 +2638,7 @@
         <f>IF(E10&gt;0, F10/E10, IF(F10&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L10" s="33" t="inlineStr">
+      <c r="L10" s="36" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -2638,7 +2684,7 @@
         <f>IF(E11&gt;0, F11/E11, IF(F11&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L11" s="36" t="inlineStr">
+      <c r="L11" s="33" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -2684,7 +2730,7 @@
         <f>IF(E12&gt;0, F12/E12, IF(F12&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L12" s="33" t="inlineStr">
+      <c r="L12" s="36" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -2776,7 +2822,7 @@
         <f>IF(E14&gt;0, F14/E14, IF(F14&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L14" s="33" t="inlineStr">
+      <c r="L14" s="36" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -2822,7 +2868,7 @@
         <f>IF(E15&gt;0, F15/E15, IF(F15&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L15" s="36" t="inlineStr">
+      <c r="L15" s="33" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -2868,7 +2914,7 @@
         <f>IF(E16&gt;0, F16/E16, IF(F16&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L16" s="33" t="inlineStr">
+      <c r="L16" s="36" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -2914,7 +2960,7 @@
         <f>IF(E17&gt;0, F17/E17, IF(F17&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L17" s="36" t="inlineStr">
+      <c r="L17" s="33" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -2960,7 +3006,7 @@
         <f>IF(E18&gt;0, F18/E18, IF(F18&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L18" s="33" t="inlineStr">
+      <c r="L18" s="36" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -3006,7 +3052,7 @@
         <f>IF(E19&gt;0, F19/E19, IF(F19&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L19" s="36" t="inlineStr">
+      <c r="L19" s="33" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -3052,7 +3098,7 @@
         <f>IF(E20&gt;0, F20/E20, IF(F20&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L20" s="33" t="inlineStr">
+      <c r="L20" s="36" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -3098,7 +3144,7 @@
         <f>IF(E21&gt;0, F21/E21, IF(F21&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L21" s="36" t="inlineStr">
+      <c r="L21" s="33" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -3144,7 +3190,7 @@
         <f>IF(E22&gt;0, F22/E22, IF(F22&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L22" s="33" t="inlineStr">
+      <c r="L22" s="36" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -3190,7 +3236,7 @@
         <f>IF(E23&gt;0, F23/E23, IF(F23&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L23" s="36" t="inlineStr">
+      <c r="L23" s="33" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -3512,7 +3558,7 @@
         <f>IF(E30&gt;0, F30/E30, IF(F30&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L30" s="33" t="inlineStr">
+      <c r="L30" s="36" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -3558,7 +3604,7 @@
         <f>IF(E31&gt;0, F31/E31, IF(F31&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L31" s="36" t="inlineStr">
+      <c r="L31" s="33" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -3604,7 +3650,7 @@
         <f>IF(E32&gt;0, F32/E32, IF(F32&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L32" s="33" t="inlineStr">
+      <c r="L32" s="36" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -3650,7 +3696,7 @@
         <f>IF(E33&gt;0, F33/E33, IF(F33&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L33" s="36" t="inlineStr">
+      <c r="L33" s="33" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -3696,7 +3742,7 @@
         <f>IF(E34&gt;0, F34/E34, IF(F34&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L34" s="33" t="inlineStr">
+      <c r="L34" s="36" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -3788,7 +3834,7 @@
         <f>IF(E36&gt;0, F36/E36, IF(F36&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L36" s="33" t="inlineStr">
+      <c r="L36" s="36" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -3834,7 +3880,7 @@
         <f>IF(E37&gt;0, F37/E37, IF(F37&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L37" s="36" t="inlineStr">
+      <c r="L37" s="33" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -4386,7 +4432,7 @@
         <f>IF(E49&gt;0, F49/E49, IF(F49&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L49" s="36" t="inlineStr">
+      <c r="L49" s="33" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -4462,7 +4508,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:L55"/>
+  <dimension ref="B2:L57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -4489,7 +4535,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 27/10/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 28/10/2026</t>
         </is>
       </c>
     </row>
@@ -4534,13 +4580,13 @@
       <c r="C6" s="4" t="n"/>
       <c r="D6" s="25" t="inlineStr">
         <is>
-          <t>23,753 u</t>
+          <t>25,745 u</t>
         </is>
       </c>
       <c r="E6" s="4" t="n"/>
       <c r="F6" s="25" t="inlineStr">
         <is>
-          <t>108.4%</t>
+          <t>117.5%</t>
         </is>
       </c>
       <c r="G6" s="4" t="n"/>
@@ -4552,7 +4598,7 @@
       <c r="I6" s="4" t="n"/>
       <c r="J6" s="24" t="inlineStr">
         <is>
-          <t>3,508 u</t>
+          <t>1,992 u</t>
         </is>
       </c>
       <c r="K6" s="4" t="n"/>
@@ -4661,7 +4707,7 @@
         <f>IF(E10&gt;0, F10/E10, IF(F10&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L10" s="33" t="inlineStr">
+      <c r="L10" s="36" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -4687,13 +4733,13 @@
         <v>1920</v>
       </c>
       <c r="F11" s="18" t="n">
-        <v>3200</v>
+        <v>3840</v>
       </c>
       <c r="G11" s="18" t="n">
         <v>3200</v>
       </c>
       <c r="H11" s="18" t="n">
-        <v>0</v>
+        <v>640</v>
       </c>
       <c r="I11" s="18">
         <f>MAX(0, E11-F11)</f>
@@ -4891,7 +4937,7 @@
         <f>IF(E15&gt;0, F15/E15, IF(F15&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L15" s="36" t="inlineStr">
+      <c r="L15" s="33" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -4937,7 +4983,7 @@
         <f>IF(E16&gt;0, F16/E16, IF(F16&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L16" s="33" t="inlineStr">
+      <c r="L16" s="36" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -4963,13 +5009,13 @@
         <v>300</v>
       </c>
       <c r="F17" s="18" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="G17" s="18" t="n">
         <v>0</v>
       </c>
       <c r="H17" s="18" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="I17" s="18">
         <f>MAX(0, E17-F17)</f>
@@ -4983,9 +5029,9 @@
         <f>IF(E17&gt;0, F17/E17, IF(F17&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L17" s="36" t="inlineStr">
-        <is>
-          <t>Sin Pedido</t>
+      <c r="L17" s="39" t="inlineStr">
+        <is>
+          <t>Rezagado</t>
         </is>
       </c>
     </row>
@@ -4997,25 +5043,25 @@
       </c>
       <c r="C18" s="28" t="inlineStr">
         <is>
-          <t>C-MB0001</t>
+          <t>C-M-P0001</t>
         </is>
       </c>
       <c r="D18" s="27" t="inlineStr">
         <is>
-          <t>CODIFOL-MB, 1 L</t>
+          <t>CODIFOL Mo-PLUS, 1 L</t>
         </is>
       </c>
       <c r="E18" s="14" t="n">
-        <v>48</v>
+        <v>0</v>
       </c>
       <c r="F18" s="14" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="G18" s="14" t="n">
         <v>0</v>
       </c>
       <c r="H18" s="14" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="I18" s="14">
         <f>MAX(0, E18-F18)</f>
@@ -5029,9 +5075,9 @@
         <f>IF(E18&gt;0, F18/E18, IF(F18&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L18" s="33" t="inlineStr">
-        <is>
-          <t>Sin Pedido</t>
+      <c r="L18" s="29" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -5043,22 +5089,22 @@
       </c>
       <c r="C19" s="31" t="inlineStr">
         <is>
-          <t>C-MB0005</t>
+          <t>C-MB0001</t>
         </is>
       </c>
       <c r="D19" s="30" t="inlineStr">
         <is>
-          <t>CODIFOL-MB, 5 L</t>
+          <t>CODIFOL-MB, 1 L</t>
         </is>
       </c>
       <c r="E19" s="18" t="n">
-        <v>400</v>
+        <v>48</v>
       </c>
       <c r="F19" s="18" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G19" s="18" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="H19" s="18" t="n">
         <v>0</v>
@@ -5075,9 +5121,9 @@
         <f>IF(E19&gt;0, F19/E19, IF(F19&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L19" s="39" t="inlineStr">
-        <is>
-          <t>Rezagado</t>
+      <c r="L19" s="33" t="inlineStr">
+        <is>
+          <t>Sin Pedido</t>
         </is>
       </c>
     </row>
@@ -5089,22 +5135,22 @@
       </c>
       <c r="C20" s="28" t="inlineStr">
         <is>
-          <t>CALCIO0005</t>
+          <t>C-MB0005</t>
         </is>
       </c>
       <c r="D20" s="27" t="inlineStr">
         <is>
-          <t>CALCIAMEC, 5 KG</t>
+          <t>CODIFOL-MB, 5 L</t>
         </is>
       </c>
       <c r="E20" s="14" t="n">
-        <v>800</v>
+        <v>400</v>
       </c>
       <c r="F20" s="14" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="G20" s="14" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="H20" s="14" t="n">
         <v>0</v>
@@ -5121,9 +5167,9 @@
         <f>IF(E20&gt;0, F20/E20, IF(F20&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L20" s="33" t="inlineStr">
-        <is>
-          <t>Sin Pedido</t>
+      <c r="L20" s="40" t="inlineStr">
+        <is>
+          <t>Rezagado</t>
         </is>
       </c>
     </row>
@@ -5135,22 +5181,22 @@
       </c>
       <c r="C21" s="31" t="inlineStr">
         <is>
-          <t>CPLUS0020</t>
+          <t>CALCIO0005</t>
         </is>
       </c>
       <c r="D21" s="30" t="inlineStr">
         <is>
-          <t>CALCIPLUS, 20 L</t>
+          <t>CALCIAMEC, 5 KG</t>
         </is>
       </c>
       <c r="E21" s="18" t="n">
-        <v>1280</v>
+        <v>800</v>
       </c>
       <c r="F21" s="18" t="n">
-        <v>1280</v>
+        <v>0</v>
       </c>
       <c r="G21" s="18" t="n">
-        <v>1280</v>
+        <v>0</v>
       </c>
       <c r="H21" s="18" t="n">
         <v>0</v>
@@ -5167,9 +5213,9 @@
         <f>IF(E21&gt;0, F21/E21, IF(F21&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L21" s="32" t="inlineStr">
-        <is>
-          <t>Superado</t>
+      <c r="L21" s="33" t="inlineStr">
+        <is>
+          <t>Sin Pedido</t>
         </is>
       </c>
     </row>
@@ -5181,22 +5227,22 @@
       </c>
       <c r="C22" s="28" t="inlineStr">
         <is>
-          <t>JF0005</t>
+          <t>CPLUS0020</t>
         </is>
       </c>
       <c r="D22" s="27" t="inlineStr">
         <is>
-          <t>CODIGIN-FOS, 5 L</t>
+          <t>CALCIPLUS, 20 L</t>
         </is>
       </c>
       <c r="E22" s="14" t="n">
-        <v>0</v>
+        <v>1280</v>
       </c>
       <c r="F22" s="14" t="n">
-        <v>600</v>
+        <v>1280</v>
       </c>
       <c r="G22" s="14" t="n">
-        <v>600</v>
+        <v>1280</v>
       </c>
       <c r="H22" s="14" t="n">
         <v>0</v>
@@ -5215,7 +5261,7 @@
       </c>
       <c r="L22" s="29" t="inlineStr">
         <is>
-          <t>Extra Estimación</t>
+          <t>Superado</t>
         </is>
       </c>
     </row>
@@ -5227,22 +5273,22 @@
       </c>
       <c r="C23" s="31" t="inlineStr">
         <is>
-          <t>PHD0005</t>
+          <t>JF0005</t>
         </is>
       </c>
       <c r="D23" s="30" t="inlineStr">
         <is>
-          <t>PH-DOWNER, 5 L</t>
+          <t>CODIGIN-FOS, 5 L</t>
         </is>
       </c>
       <c r="E23" s="18" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="F23" s="18" t="n">
-        <v>0</v>
+        <v>600</v>
       </c>
       <c r="G23" s="18" t="n">
-        <v>0</v>
+        <v>600</v>
       </c>
       <c r="H23" s="18" t="n">
         <v>0</v>
@@ -5259,9 +5305,9 @@
         <f>IF(E23&gt;0, F23/E23, IF(F23&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L23" s="36" t="inlineStr">
-        <is>
-          <t>Sin Pedido</t>
+      <c r="L23" s="32" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -5273,22 +5319,22 @@
       </c>
       <c r="C24" s="28" t="inlineStr">
         <is>
-          <t>PIV0020</t>
+          <t>PHD0005</t>
         </is>
       </c>
       <c r="D24" s="27" t="inlineStr">
         <is>
-          <t>PGR IV, 20 L</t>
+          <t>PH-DOWNER, 5 L</t>
         </is>
       </c>
       <c r="E24" s="14" t="n">
-        <v>3200</v>
+        <v>100</v>
       </c>
       <c r="F24" s="14" t="n">
-        <v>640</v>
+        <v>0</v>
       </c>
       <c r="G24" s="14" t="n">
-        <v>640</v>
+        <v>0</v>
       </c>
       <c r="H24" s="14" t="n">
         <v>0</v>
@@ -5305,9 +5351,9 @@
         <f>IF(E24&gt;0, F24/E24, IF(F24&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L24" s="40" t="inlineStr">
-        <is>
-          <t>Rezagado</t>
+      <c r="L24" s="36" t="inlineStr">
+        <is>
+          <t>Sin Pedido</t>
         </is>
       </c>
     </row>
@@ -5319,25 +5365,25 @@
       </c>
       <c r="C25" s="31" t="inlineStr">
         <is>
-          <t>S0020</t>
+          <t>PIV0020</t>
         </is>
       </c>
       <c r="D25" s="30" t="inlineStr">
         <is>
-          <t>SAL-WAX STAR, 20 L</t>
+          <t>PGR IV, 20 L</t>
         </is>
       </c>
       <c r="E25" s="18" t="n">
+        <v>3200</v>
+      </c>
+      <c r="F25" s="18" t="n">
+        <v>1280</v>
+      </c>
+      <c r="G25" s="18" t="n">
         <v>640</v>
       </c>
-      <c r="F25" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G25" s="18" t="n">
-        <v>0</v>
-      </c>
       <c r="H25" s="18" t="n">
-        <v>0</v>
+        <v>640</v>
       </c>
       <c r="I25" s="18">
         <f>MAX(0, E25-F25)</f>
@@ -5351,9 +5397,9 @@
         <f>IF(E25&gt;0, F25/E25, IF(F25&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L25" s="36" t="inlineStr">
-        <is>
-          <t>Sin Pedido</t>
+      <c r="L25" s="39" t="inlineStr">
+        <is>
+          <t>Rezagado</t>
         </is>
       </c>
     </row>
@@ -5365,22 +5411,22 @@
       </c>
       <c r="C26" s="28" t="inlineStr">
         <is>
-          <t>TRI0005</t>
+          <t>S0020</t>
         </is>
       </c>
       <c r="D26" s="27" t="inlineStr">
         <is>
-          <t>TRIFENO-94, 5L</t>
+          <t>SAL-WAX STAR, 20 L</t>
         </is>
       </c>
       <c r="E26" s="14" t="n">
-        <v>100</v>
+        <v>640</v>
       </c>
       <c r="F26" s="14" t="n">
-        <v>205</v>
+        <v>0</v>
       </c>
       <c r="G26" s="14" t="n">
-        <v>205</v>
+        <v>0</v>
       </c>
       <c r="H26" s="14" t="n">
         <v>0</v>
@@ -5397,39 +5443,39 @@
         <f>IF(E26&gt;0, F26/E26, IF(F26&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L26" s="29" t="inlineStr">
-        <is>
-          <t>Superado</t>
+      <c r="L26" s="36" t="inlineStr">
+        <is>
+          <t>Sin Pedido</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="B27" s="30" t="inlineStr">
         <is>
-          <t>COOP.AGRIC. SAN ISIDRO S.C.A.</t>
+          <t>CAMPOEJIDO S.C.A.</t>
         </is>
       </c>
       <c r="C27" s="31" t="inlineStr">
         <is>
-          <t>AGXK0020</t>
+          <t>TRI0005</t>
         </is>
       </c>
       <c r="D27" s="30" t="inlineStr">
         <is>
-          <t>AGROXILATO-K, 20 L</t>
+          <t>TRIFENO-94, 5L</t>
         </is>
       </c>
       <c r="E27" s="18" t="n">
-        <v>3200</v>
+        <v>100</v>
       </c>
       <c r="F27" s="18" t="n">
-        <v>4480</v>
+        <v>205</v>
       </c>
       <c r="G27" s="18" t="n">
-        <v>1920</v>
+        <v>205</v>
       </c>
       <c r="H27" s="18" t="n">
-        <v>2560</v>
+        <v>0</v>
       </c>
       <c r="I27" s="18">
         <f>MAX(0, E27-F27)</f>
@@ -5457,22 +5503,22 @@
       </c>
       <c r="C28" s="28" t="inlineStr">
         <is>
-          <t>AGXK0200</t>
+          <t>AGXK0020</t>
         </is>
       </c>
       <c r="D28" s="27" t="inlineStr">
         <is>
-          <t>AGROXILATO-K, 200 L</t>
+          <t>AGROXILATO-K, 20 L</t>
         </is>
       </c>
       <c r="E28" s="14" t="n">
-        <v>400</v>
+        <v>3200</v>
       </c>
       <c r="F28" s="14" t="n">
-        <v>0</v>
+        <v>4480</v>
       </c>
       <c r="G28" s="14" t="n">
-        <v>0</v>
+        <v>4480</v>
       </c>
       <c r="H28" s="14" t="n">
         <v>0</v>
@@ -5489,9 +5535,9 @@
         <f>IF(E28&gt;0, F28/E28, IF(F28&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L28" s="33" t="inlineStr">
-        <is>
-          <t>Sin Pedido</t>
+      <c r="L28" s="29" t="inlineStr">
+        <is>
+          <t>Superado</t>
         </is>
       </c>
     </row>
@@ -5503,22 +5549,22 @@
       </c>
       <c r="C29" s="31" t="inlineStr">
         <is>
-          <t>AGZ-M0001</t>
+          <t>AGXK0200</t>
         </is>
       </c>
       <c r="D29" s="30" t="inlineStr">
         <is>
-          <t>AGROXILATO-ZN-MN, 1 KG</t>
+          <t>AGROXILATO-K, 200 L</t>
         </is>
       </c>
       <c r="E29" s="18" t="n">
-        <v>0</v>
+        <v>400</v>
       </c>
       <c r="F29" s="18" t="n">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="G29" s="18" t="n">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="H29" s="18" t="n">
         <v>0</v>
@@ -5535,9 +5581,9 @@
         <f>IF(E29&gt;0, F29/E29, IF(F29&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L29" s="32" t="inlineStr">
-        <is>
-          <t>Extra Estimación</t>
+      <c r="L29" s="33" t="inlineStr">
+        <is>
+          <t>Sin Pedido</t>
         </is>
       </c>
     </row>
@@ -5549,22 +5595,22 @@
       </c>
       <c r="C30" s="28" t="inlineStr">
         <is>
-          <t>AGZ-M0005</t>
+          <t>AGZ-M0001</t>
         </is>
       </c>
       <c r="D30" s="27" t="inlineStr">
         <is>
-          <t>AGROXILATO-ZN-MN, 5 KG</t>
+          <t>AGROXILATO-ZN-MN, 1 KG</t>
         </is>
       </c>
       <c r="E30" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F30" s="14" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="G30" s="14" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="H30" s="14" t="n">
         <v>0</v>
@@ -5595,25 +5641,25 @@
       </c>
       <c r="C31" s="31" t="inlineStr">
         <is>
-          <t>AMIMG0020</t>
+          <t>AGZ-M0005</t>
         </is>
       </c>
       <c r="D31" s="30" t="inlineStr">
         <is>
-          <t>AMINOSOIL MG, 20 L</t>
+          <t>AGROXILATO-ZN-MN, 5 KG</t>
         </is>
       </c>
       <c r="E31" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F31" s="18" t="n">
-        <v>640</v>
+        <v>100</v>
       </c>
       <c r="G31" s="18" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="H31" s="18" t="n">
-        <v>640</v>
+        <v>0</v>
       </c>
       <c r="I31" s="18">
         <f>MAX(0, E31-F31)</f>
@@ -5641,22 +5687,22 @@
       </c>
       <c r="C32" s="28" t="inlineStr">
         <is>
-          <t>AVAN0005</t>
+          <t>AMIMG0020</t>
         </is>
       </c>
       <c r="D32" s="27" t="inlineStr">
         <is>
-          <t>FLORAMEC AVANCE, 5 L</t>
+          <t>AMINOSOIL MG, 20 L</t>
         </is>
       </c>
       <c r="E32" s="14" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="F32" s="14" t="n">
-        <v>600</v>
+        <v>640</v>
       </c>
       <c r="G32" s="14" t="n">
-        <v>600</v>
+        <v>640</v>
       </c>
       <c r="H32" s="14" t="n">
         <v>0</v>
@@ -5673,9 +5719,9 @@
         <f>IF(E32&gt;0, F32/E32, IF(F32&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L32" s="38" t="inlineStr">
-        <is>
-          <t>En Curso</t>
+      <c r="L32" s="29" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -5687,22 +5733,22 @@
       </c>
       <c r="C33" s="31" t="inlineStr">
         <is>
-          <t>C-L0005</t>
+          <t>AVAN0005</t>
         </is>
       </c>
       <c r="D33" s="30" t="inlineStr">
         <is>
-          <t>CODIBOR-L, 5 L</t>
+          <t>FLORAMEC AVANCE, 5 L</t>
         </is>
       </c>
       <c r="E33" s="18" t="n">
-        <v>200</v>
+        <v>1200</v>
       </c>
       <c r="F33" s="18" t="n">
-        <v>200</v>
+        <v>600</v>
       </c>
       <c r="G33" s="18" t="n">
-        <v>200</v>
+        <v>600</v>
       </c>
       <c r="H33" s="18" t="n">
         <v>0</v>
@@ -5719,9 +5765,9 @@
         <f>IF(E33&gt;0, F33/E33, IF(F33&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L33" s="32" t="inlineStr">
-        <is>
-          <t>Superado</t>
+      <c r="L33" s="37" t="inlineStr">
+        <is>
+          <t>En Curso</t>
         </is>
       </c>
     </row>
@@ -5733,16 +5779,16 @@
       </c>
       <c r="C34" s="28" t="inlineStr">
         <is>
-          <t>C-MB0005</t>
+          <t>C-L0005</t>
         </is>
       </c>
       <c r="D34" s="27" t="inlineStr">
         <is>
-          <t>CODIFOL-MB, 5 L</t>
+          <t>CODIBOR-L, 5 L</t>
         </is>
       </c>
       <c r="E34" s="14" t="n">
-        <v>300</v>
+        <v>200</v>
       </c>
       <c r="F34" s="14" t="n">
         <v>200</v>
@@ -5765,9 +5811,9 @@
         <f>IF(E34&gt;0, F34/E34, IF(F34&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L34" s="38" t="inlineStr">
-        <is>
-          <t>En Curso</t>
+      <c r="L34" s="29" t="inlineStr">
+        <is>
+          <t>Superado</t>
         </is>
       </c>
     </row>
@@ -5779,22 +5825,22 @@
       </c>
       <c r="C35" s="31" t="inlineStr">
         <is>
-          <t>CPLUS0020</t>
+          <t>C-MB0005</t>
         </is>
       </c>
       <c r="D35" s="30" t="inlineStr">
         <is>
-          <t>CALCIPLUS, 20 L</t>
+          <t>CODIFOL-MB, 5 L</t>
         </is>
       </c>
       <c r="E35" s="18" t="n">
-        <v>640</v>
+        <v>300</v>
       </c>
       <c r="F35" s="18" t="n">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="G35" s="18" t="n">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="H35" s="18" t="n">
         <v>0</v>
@@ -5811,9 +5857,9 @@
         <f>IF(E35&gt;0, F35/E35, IF(F35&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L35" s="36" t="inlineStr">
-        <is>
-          <t>Sin Pedido</t>
+      <c r="L35" s="37" t="inlineStr">
+        <is>
+          <t>En Curso</t>
         </is>
       </c>
     </row>
@@ -5825,22 +5871,22 @@
       </c>
       <c r="C36" s="28" t="inlineStr">
         <is>
-          <t>PIV0020</t>
+          <t>CPLUS0020</t>
         </is>
       </c>
       <c r="D36" s="27" t="inlineStr">
         <is>
-          <t>PGR IV, 20 L</t>
+          <t>CALCIPLUS, 20 L</t>
         </is>
       </c>
       <c r="E36" s="14" t="n">
-        <v>1280</v>
+        <v>640</v>
       </c>
       <c r="F36" s="14" t="n">
-        <v>2560</v>
+        <v>0</v>
       </c>
       <c r="G36" s="14" t="n">
-        <v>2560</v>
+        <v>0</v>
       </c>
       <c r="H36" s="14" t="n">
         <v>0</v>
@@ -5857,9 +5903,9 @@
         <f>IF(E36&gt;0, F36/E36, IF(F36&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L36" s="29" t="inlineStr">
-        <is>
-          <t>Superado</t>
+      <c r="L36" s="36" t="inlineStr">
+        <is>
+          <t>Sin Pedido</t>
         </is>
       </c>
     </row>
@@ -5871,25 +5917,25 @@
       </c>
       <c r="C37" s="31" t="inlineStr">
         <is>
-          <t>PT0005</t>
+          <t>PIV0020</t>
         </is>
       </c>
       <c r="D37" s="30" t="inlineStr">
         <is>
-          <t>AGROPOTASION, 5 L</t>
+          <t>PGR IV, 20 L</t>
         </is>
       </c>
       <c r="E37" s="18" t="n">
-        <v>0</v>
+        <v>1280</v>
       </c>
       <c r="F37" s="18" t="n">
-        <v>200</v>
+        <v>2560</v>
       </c>
       <c r="G37" s="18" t="n">
-        <v>0</v>
+        <v>2560</v>
       </c>
       <c r="H37" s="18" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="I37" s="18">
         <f>MAX(0, E37-F37)</f>
@@ -5905,7 +5951,7 @@
       </c>
       <c r="L37" s="32" t="inlineStr">
         <is>
-          <t>Extra Estimación</t>
+          <t>Superado</t>
         </is>
       </c>
     </row>
@@ -5917,22 +5963,22 @@
       </c>
       <c r="C38" s="28" t="inlineStr">
         <is>
-          <t>PT0020</t>
+          <t>PT0005</t>
         </is>
       </c>
       <c r="D38" s="27" t="inlineStr">
         <is>
-          <t>AGROPOTASION, 20 L</t>
+          <t>AGROPOTASION, 5 L</t>
         </is>
       </c>
       <c r="E38" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F38" s="14" t="n">
-        <v>320</v>
+        <v>200</v>
       </c>
       <c r="G38" s="14" t="n">
-        <v>320</v>
+        <v>200</v>
       </c>
       <c r="H38" s="14" t="n">
         <v>0</v>
@@ -5963,22 +6009,22 @@
       </c>
       <c r="C39" s="31" t="inlineStr">
         <is>
-          <t>S0020</t>
+          <t>PT0020</t>
         </is>
       </c>
       <c r="D39" s="30" t="inlineStr">
         <is>
-          <t>SAL-WAX STAR, 20 L</t>
+          <t>AGROPOTASION, 20 L</t>
         </is>
       </c>
       <c r="E39" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F39" s="18" t="n">
-        <v>640</v>
+        <v>320</v>
       </c>
       <c r="G39" s="18" t="n">
-        <v>640</v>
+        <v>320</v>
       </c>
       <c r="H39" s="18" t="n">
         <v>0</v>
@@ -6009,25 +6055,25 @@
       </c>
       <c r="C40" s="28" t="inlineStr">
         <is>
-          <t>TRI0001</t>
+          <t>S0020</t>
         </is>
       </c>
       <c r="D40" s="27" t="inlineStr">
         <is>
-          <t>TRIFENO-94, 1 L</t>
+          <t>SAL-WAX STAR, 20 L</t>
         </is>
       </c>
       <c r="E40" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F40" s="14" t="n">
-        <v>108</v>
+        <v>640</v>
       </c>
       <c r="G40" s="14" t="n">
-        <v>0</v>
+        <v>640</v>
       </c>
       <c r="H40" s="14" t="n">
-        <v>108</v>
+        <v>0</v>
       </c>
       <c r="I40" s="14">
         <f>MAX(0, E40-F40)</f>
@@ -6050,27 +6096,27 @@
     <row r="41">
       <c r="B41" s="30" t="inlineStr">
         <is>
-          <t>GUIVARTO AGRICOLA, S.L.</t>
+          <t>COOP.AGRIC. SAN ISIDRO S.C.A.</t>
         </is>
       </c>
       <c r="C41" s="31" t="inlineStr">
         <is>
-          <t>A-50(2)0005</t>
+          <t>TRI0001</t>
         </is>
       </c>
       <c r="D41" s="30" t="inlineStr">
         <is>
-          <t>CODIORGAN A-50, 5 KG</t>
+          <t>TRIFENO-94, 1 L</t>
         </is>
       </c>
       <c r="E41" s="18" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="F41" s="18" t="n">
-        <v>100</v>
+        <v>108</v>
       </c>
       <c r="G41" s="18" t="n">
-        <v>100</v>
+        <v>108</v>
       </c>
       <c r="H41" s="18" t="n">
         <v>0</v>
@@ -6089,7 +6135,7 @@
       </c>
       <c r="L41" s="32" t="inlineStr">
         <is>
-          <t>Superado</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -6101,22 +6147,22 @@
       </c>
       <c r="C42" s="28" t="inlineStr">
         <is>
-          <t>AGXK0020</t>
+          <t>A-50(2)0005</t>
         </is>
       </c>
       <c r="D42" s="27" t="inlineStr">
         <is>
-          <t>AGROXILATO-K, 20 L</t>
+          <t>CODIORGAN A-50, 5 KG</t>
         </is>
       </c>
       <c r="E42" s="14" t="n">
-        <v>1240</v>
+        <v>100</v>
       </c>
       <c r="F42" s="14" t="n">
-        <v>2560</v>
+        <v>100</v>
       </c>
       <c r="G42" s="14" t="n">
-        <v>2560</v>
+        <v>100</v>
       </c>
       <c r="H42" s="14" t="n">
         <v>0</v>
@@ -6147,22 +6193,22 @@
       </c>
       <c r="C43" s="31" t="inlineStr">
         <is>
-          <t>AGZNP0005</t>
+          <t>AGXK0020</t>
         </is>
       </c>
       <c r="D43" s="30" t="inlineStr">
         <is>
-          <t>AGROXILATO-ZN PLUS, 5 KG</t>
+          <t>AGROXILATO-K, 20 L</t>
         </is>
       </c>
       <c r="E43" s="18" t="n">
-        <v>50</v>
+        <v>1240</v>
       </c>
       <c r="F43" s="18" t="n">
-        <v>0</v>
+        <v>2560</v>
       </c>
       <c r="G43" s="18" t="n">
-        <v>0</v>
+        <v>2560</v>
       </c>
       <c r="H43" s="18" t="n">
         <v>0</v>
@@ -6179,9 +6225,9 @@
         <f>IF(E43&gt;0, F43/E43, IF(F43&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L43" s="36" t="inlineStr">
-        <is>
-          <t>Sin Pedido</t>
+      <c r="L43" s="32" t="inlineStr">
+        <is>
+          <t>Superado</t>
         </is>
       </c>
     </row>
@@ -6193,16 +6239,16 @@
       </c>
       <c r="C44" s="28" t="inlineStr">
         <is>
-          <t>AQUOM0005</t>
+          <t>AGZNP0005</t>
         </is>
       </c>
       <c r="D44" s="27" t="inlineStr">
         <is>
-          <t>AQUOM, 5 L</t>
+          <t>AGROXILATO-ZN PLUS, 5 KG</t>
         </is>
       </c>
       <c r="E44" s="14" t="n">
-        <v>200</v>
+        <v>50</v>
       </c>
       <c r="F44" s="14" t="n">
         <v>0</v>
@@ -6225,7 +6271,7 @@
         <f>IF(E44&gt;0, F44/E44, IF(F44&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L44" s="33" t="inlineStr">
+      <c r="L44" s="36" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -6239,22 +6285,22 @@
       </c>
       <c r="C45" s="31" t="inlineStr">
         <is>
-          <t>AVAN0005</t>
+          <t>AQUOM0005</t>
         </is>
       </c>
       <c r="D45" s="30" t="inlineStr">
         <is>
-          <t>FLORAMEC AVANCE, 5 L</t>
+          <t>AQUOM, 5 L</t>
         </is>
       </c>
       <c r="E45" s="18" t="n">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="F45" s="18" t="n">
-        <v>600</v>
+        <v>0</v>
       </c>
       <c r="G45" s="18" t="n">
-        <v>600</v>
+        <v>0</v>
       </c>
       <c r="H45" s="18" t="n">
         <v>0</v>
@@ -6271,9 +6317,9 @@
         <f>IF(E45&gt;0, F45/E45, IF(F45&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L45" s="32" t="inlineStr">
-        <is>
-          <t>Extra Estimación</t>
+      <c r="L45" s="33" t="inlineStr">
+        <is>
+          <t>Sin Pedido</t>
         </is>
       </c>
     </row>
@@ -6285,22 +6331,22 @@
       </c>
       <c r="C46" s="28" t="inlineStr">
         <is>
-          <t>AVAN0020</t>
+          <t>AVAN0005</t>
         </is>
       </c>
       <c r="D46" s="27" t="inlineStr">
         <is>
-          <t>FLORAMEC AVANCE, 20 L</t>
+          <t>FLORAMEC AVANCE, 5 L</t>
         </is>
       </c>
       <c r="E46" s="14" t="n">
-        <v>640</v>
+        <v>0</v>
       </c>
       <c r="F46" s="14" t="n">
-        <v>640</v>
+        <v>600</v>
       </c>
       <c r="G46" s="14" t="n">
-        <v>640</v>
+        <v>600</v>
       </c>
       <c r="H46" s="14" t="n">
         <v>0</v>
@@ -6319,7 +6365,7 @@
       </c>
       <c r="L46" s="29" t="inlineStr">
         <is>
-          <t>Superado</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -6331,22 +6377,22 @@
       </c>
       <c r="C47" s="31" t="inlineStr">
         <is>
-          <t>BEY0005</t>
+          <t>AVAN0020</t>
         </is>
       </c>
       <c r="D47" s="30" t="inlineStr">
         <is>
-          <t>FLORAMEC PLUS, 5 L</t>
+          <t>FLORAMEC AVANCE, 20 L</t>
         </is>
       </c>
       <c r="E47" s="18" t="n">
-        <v>0</v>
+        <v>640</v>
       </c>
       <c r="F47" s="18" t="n">
-        <v>100</v>
+        <v>640</v>
       </c>
       <c r="G47" s="18" t="n">
-        <v>100</v>
+        <v>640</v>
       </c>
       <c r="H47" s="18" t="n">
         <v>0</v>
@@ -6365,7 +6411,7 @@
       </c>
       <c r="L47" s="32" t="inlineStr">
         <is>
-          <t>Extra Estimación</t>
+          <t>Superado</t>
         </is>
       </c>
     </row>
@@ -6377,22 +6423,22 @@
       </c>
       <c r="C48" s="28" t="inlineStr">
         <is>
-          <t>BEY0020</t>
+          <t>BEY0005</t>
         </is>
       </c>
       <c r="D48" s="27" t="inlineStr">
         <is>
-          <t>FLORAMEC PLUS 20 L</t>
+          <t>FLORAMEC PLUS, 5 L</t>
         </is>
       </c>
       <c r="E48" s="14" t="n">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="F48" s="14" t="n">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="G48" s="14" t="n">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="H48" s="14" t="n">
         <v>0</v>
@@ -6411,7 +6457,7 @@
       </c>
       <c r="L48" s="29" t="inlineStr">
         <is>
-          <t>Superado</t>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
@@ -6423,22 +6469,22 @@
       </c>
       <c r="C49" s="31" t="inlineStr">
         <is>
-          <t>BROTA0005</t>
+          <t>BEY0020</t>
         </is>
       </c>
       <c r="D49" s="30" t="inlineStr">
         <is>
-          <t>BROTAMEC, 5 L</t>
+          <t>FLORAMEC PLUS 20 L</t>
         </is>
       </c>
       <c r="E49" s="18" t="n">
-        <v>600</v>
+        <v>80</v>
       </c>
       <c r="F49" s="18" t="n">
-        <v>600</v>
+        <v>120</v>
       </c>
       <c r="G49" s="18" t="n">
-        <v>600</v>
+        <v>120</v>
       </c>
       <c r="H49" s="18" t="n">
         <v>0</v>
@@ -6469,22 +6515,22 @@
       </c>
       <c r="C50" s="28" t="inlineStr">
         <is>
-          <t>C-M-P0001</t>
+          <t>BROTA0005</t>
         </is>
       </c>
       <c r="D50" s="27" t="inlineStr">
         <is>
-          <t>CODIFOL Mo-PLUS, 1 L</t>
+          <t>BROTAMEC, 5 L</t>
         </is>
       </c>
       <c r="E50" s="14" t="n">
-        <v>36</v>
+        <v>600</v>
       </c>
       <c r="F50" s="14" t="n">
-        <v>0</v>
+        <v>600</v>
       </c>
       <c r="G50" s="14" t="n">
-        <v>0</v>
+        <v>600</v>
       </c>
       <c r="H50" s="14" t="n">
         <v>0</v>
@@ -6501,9 +6547,9 @@
         <f>IF(E50&gt;0, F50/E50, IF(F50&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L50" s="33" t="inlineStr">
-        <is>
-          <t>Sin Pedido</t>
+      <c r="L50" s="29" t="inlineStr">
+        <is>
+          <t>Superado</t>
         </is>
       </c>
     </row>
@@ -6515,16 +6561,16 @@
       </c>
       <c r="C51" s="31" t="inlineStr">
         <is>
-          <t>FTK0005</t>
+          <t>C-M-P0001</t>
         </is>
       </c>
       <c r="D51" s="30" t="inlineStr">
         <is>
-          <t>FITOKONTROL CA FLOW, 5 KG</t>
+          <t>CODIFOL Mo-PLUS, 1 L</t>
         </is>
       </c>
       <c r="E51" s="18" t="n">
-        <v>800</v>
+        <v>36</v>
       </c>
       <c r="F51" s="18" t="n">
         <v>0</v>
@@ -6547,7 +6593,7 @@
         <f>IF(E51&gt;0, F51/E51, IF(F51&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L51" s="36" t="inlineStr">
+      <c r="L51" s="33" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -6561,22 +6607,22 @@
       </c>
       <c r="C52" s="28" t="inlineStr">
         <is>
-          <t>TRI0001</t>
+          <t>FTK0005</t>
         </is>
       </c>
       <c r="D52" s="27" t="inlineStr">
         <is>
-          <t>TRIFENO-94, 1 L</t>
+          <t>FITOKONTROL CA FLOW, 5 KG</t>
         </is>
       </c>
       <c r="E52" s="14" t="n">
-        <v>0</v>
+        <v>800</v>
       </c>
       <c r="F52" s="14" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="G52" s="14" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="H52" s="14" t="n">
         <v>0</v>
@@ -6593,9 +6639,9 @@
         <f>IF(E52&gt;0, F52/E52, IF(F52&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L52" s="29" t="inlineStr">
-        <is>
-          <t>Extra Estimación</t>
+      <c r="L52" s="36" t="inlineStr">
+        <is>
+          <t>Sin Pedido</t>
         </is>
       </c>
     </row>
@@ -6607,22 +6653,22 @@
       </c>
       <c r="C53" s="31" t="inlineStr">
         <is>
-          <t>TRI0005</t>
+          <t>TRI0001</t>
         </is>
       </c>
       <c r="D53" s="30" t="inlineStr">
         <is>
-          <t>TRIFENO-94, 5L</t>
+          <t>TRIFENO-94, 1 L</t>
         </is>
       </c>
       <c r="E53" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F53" s="18" t="n">
-        <v>600</v>
+        <v>60</v>
       </c>
       <c r="G53" s="18" t="n">
-        <v>600</v>
+        <v>60</v>
       </c>
       <c r="H53" s="18" t="n">
         <v>0</v>
@@ -6648,27 +6694,27 @@
     <row r="54">
       <c r="B54" s="27" t="inlineStr">
         <is>
-          <t>SUCA, S.C.A.</t>
+          <t>GUIVARTO AGRICOLA, S.L.</t>
         </is>
       </c>
       <c r="C54" s="28" t="inlineStr">
         <is>
-          <t>AGXK0020</t>
+          <t>TRI0005</t>
         </is>
       </c>
       <c r="D54" s="27" t="inlineStr">
         <is>
-          <t>AGROXILATO-K, 20 L</t>
+          <t>TRIFENO-94, 5L</t>
         </is>
       </c>
       <c r="E54" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F54" s="14" t="n">
-        <v>640</v>
+        <v>600</v>
       </c>
       <c r="G54" s="14" t="n">
-        <v>640</v>
+        <v>600</v>
       </c>
       <c r="H54" s="14" t="n">
         <v>0</v>
@@ -6691,48 +6737,140 @@
         </is>
       </c>
     </row>
-    <row r="55" ht="24" customHeight="1">
-      <c r="B55" s="20" t="inlineStr">
+    <row r="55">
+      <c r="B55" s="30" t="inlineStr">
+        <is>
+          <t>HORTOCAMPO, S.A.</t>
+        </is>
+      </c>
+      <c r="C55" s="31" t="inlineStr">
+        <is>
+          <t>BROTA0005</t>
+        </is>
+      </c>
+      <c r="D55" s="30" t="inlineStr">
+        <is>
+          <t>CODECROP BROTIUM, 5 L</t>
+        </is>
+      </c>
+      <c r="E55" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F55" s="18" t="n">
+        <v>600</v>
+      </c>
+      <c r="G55" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H55" s="18" t="n">
+        <v>600</v>
+      </c>
+      <c r="I55" s="18">
+        <f>MAX(0, E55-F55)</f>
+        <v/>
+      </c>
+      <c r="J55" s="18">
+        <f>ABS(F55-E55)</f>
+        <v/>
+      </c>
+      <c r="K55" s="19">
+        <f>IF(E55&gt;0, F55/E55, IF(F55&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L55" s="32" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="B56" s="27" t="inlineStr">
+        <is>
+          <t>SUCA, S.C.A.</t>
+        </is>
+      </c>
+      <c r="C56" s="28" t="inlineStr">
+        <is>
+          <t>AGXK0020</t>
+        </is>
+      </c>
+      <c r="D56" s="27" t="inlineStr">
+        <is>
+          <t>AGROXILATO-K, 20 L</t>
+        </is>
+      </c>
+      <c r="E56" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F56" s="14" t="n">
+        <v>640</v>
+      </c>
+      <c r="G56" s="14" t="n">
+        <v>640</v>
+      </c>
+      <c r="H56" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I56" s="14">
+        <f>MAX(0, E56-F56)</f>
+        <v/>
+      </c>
+      <c r="J56" s="14">
+        <f>ABS(F56-E56)</f>
+        <v/>
+      </c>
+      <c r="K56" s="15">
+        <f>IF(E56&gt;0, F56/E56, IF(F56&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L56" s="29" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="24" customHeight="1">
+      <c r="B57" s="20" t="inlineStr">
         <is>
           <t>TOTAL IRENE</t>
         </is>
       </c>
-      <c r="C55" s="34" t="inlineStr">
+      <c r="C57" s="34" t="inlineStr">
         <is>
           <t>89 líneas</t>
         </is>
       </c>
-      <c r="D55" s="35" t="inlineStr"/>
-      <c r="E55" s="22">
-        <f>SUM(E10:E54)</f>
-        <v/>
-      </c>
-      <c r="F55" s="22">
-        <f>SUM(F10:F54)</f>
-        <v/>
-      </c>
-      <c r="G55" s="22">
-        <f>SUM(G10:G54)</f>
-        <v/>
-      </c>
-      <c r="H55" s="22">
-        <f>SUM(H10:H54)</f>
-        <v/>
-      </c>
-      <c r="I55" s="22">
-        <f>SUM(I10:I54)</f>
-        <v/>
-      </c>
-      <c r="J55" s="22">
-        <f>SUM(J10:J54)</f>
-        <v/>
-      </c>
-      <c r="K55" s="23">
-        <f>IF(E55&gt;0, F55/E55, 0)</f>
-        <v/>
-      </c>
-      <c r="L55" s="21">
-        <f>IF(K55&gt;=1, "SUPERADO", "EN CURSO")</f>
+      <c r="D57" s="35" t="inlineStr"/>
+      <c r="E57" s="22">
+        <f>SUM(E10:E56)</f>
+        <v/>
+      </c>
+      <c r="F57" s="22">
+        <f>SUM(F10:F56)</f>
+        <v/>
+      </c>
+      <c r="G57" s="22">
+        <f>SUM(G10:G56)</f>
+        <v/>
+      </c>
+      <c r="H57" s="22">
+        <f>SUM(H10:H56)</f>
+        <v/>
+      </c>
+      <c r="I57" s="22">
+        <f>SUM(I10:I56)</f>
+        <v/>
+      </c>
+      <c r="J57" s="22">
+        <f>SUM(J10:J56)</f>
+        <v/>
+      </c>
+      <c r="K57" s="23">
+        <f>IF(E57&gt;0, F57/E57, 0)</f>
+        <v/>
+      </c>
+      <c r="L57" s="21">
+        <f>IF(K57&gt;=1, "SUPERADO", "EN CURSO")</f>
         <v/>
       </c>
     </row>
@@ -6788,7 +6926,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 27/10/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 28/10/2026</t>
         </is>
       </c>
     </row>
@@ -7466,7 +7604,7 @@
         <f>IF(E21&gt;0, F21/E21, IF(F21&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L21" s="36" t="inlineStr">
+      <c r="L21" s="33" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -7512,7 +7650,7 @@
         <f>IF(E22&gt;0, F22/E22, IF(F22&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L22" s="33" t="inlineStr">
+      <c r="L22" s="36" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -8110,7 +8248,7 @@
         <f>IF(E35&gt;0, F35/E35, IF(F35&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L35" s="36" t="inlineStr">
+      <c r="L35" s="33" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -8156,7 +8294,7 @@
         <f>IF(E36&gt;0, F36/E36, IF(F36&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L36" s="33" t="inlineStr">
+      <c r="L36" s="36" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -8232,7 +8370,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:L16"/>
+  <dimension ref="B2:L23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -8259,7 +8397,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 27/10/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 28/10/2026</t>
         </is>
       </c>
     </row>
@@ -8304,25 +8442,25 @@
       <c r="C6" s="4" t="n"/>
       <c r="D6" s="24" t="inlineStr">
         <is>
-          <t>0 u</t>
+          <t>7,632 u</t>
         </is>
       </c>
       <c r="E6" s="4" t="n"/>
       <c r="F6" s="41" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>19.3%</t>
         </is>
       </c>
       <c r="G6" s="4" t="n"/>
       <c r="H6" s="41" t="inlineStr">
         <is>
-          <t>39,460 u</t>
+          <t>31,828 u</t>
         </is>
       </c>
       <c r="I6" s="4" t="n"/>
       <c r="J6" s="24" t="inlineStr">
         <is>
-          <t>0 u</t>
+          <t>7,632 u</t>
         </is>
       </c>
       <c r="K6" s="4" t="n"/>
@@ -8394,30 +8532,30 @@
     <row r="10">
       <c r="B10" s="27" t="inlineStr">
         <is>
-          <t>ÇITAR ÇIÇEK TARIM TIC. LTD. STI</t>
+          <t>PLANTA SANA, D.O.O.</t>
         </is>
       </c>
       <c r="C10" s="28" t="inlineStr">
         <is>
-          <t>AN0005</t>
+          <t>A-50(2)0001</t>
         </is>
       </c>
       <c r="D10" s="27" t="inlineStr">
         <is>
-          <t>ALCAPLANT NEW, 5 KG</t>
+          <t>CODIORGAN-A50</t>
         </is>
       </c>
       <c r="E10" s="14" t="n">
-        <v>5500</v>
+        <v>0</v>
       </c>
       <c r="F10" s="14" t="n">
-        <v>0</v>
+        <v>2112</v>
       </c>
       <c r="G10" s="14" t="n">
         <v>0</v>
       </c>
       <c r="H10" s="14" t="n">
-        <v>0</v>
+        <v>2112</v>
       </c>
       <c r="I10" s="14">
         <f>MAX(0, E10-F10)</f>
@@ -8431,39 +8569,39 @@
         <f>IF(E10&gt;0, F10/E10, IF(F10&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L10" s="33" t="inlineStr">
-        <is>
-          <t>Sin Pedido</t>
+      <c r="L10" s="29" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="B11" s="30" t="inlineStr">
         <is>
-          <t>ÇITAR ÇIÇEK TARIM TIC. LTD. STI</t>
+          <t>PLANTA SANA, D.O.O.</t>
         </is>
       </c>
       <c r="C11" s="31" t="inlineStr">
         <is>
-          <t>BIO0020</t>
+          <t>A-50(2)0020</t>
         </is>
       </c>
       <c r="D11" s="30" t="inlineStr">
         <is>
-          <t>BIORAD-20, 20 L</t>
+          <t>CODIORGAN-A50, 20 KG</t>
         </is>
       </c>
       <c r="E11" s="18" t="n">
-        <v>10000</v>
+        <v>0</v>
       </c>
       <c r="F11" s="18" t="n">
-        <v>0</v>
+        <v>500</v>
       </c>
       <c r="G11" s="18" t="n">
         <v>0</v>
       </c>
       <c r="H11" s="18" t="n">
-        <v>0</v>
+        <v>500</v>
       </c>
       <c r="I11" s="18">
         <f>MAX(0, E11-F11)</f>
@@ -8477,39 +8615,39 @@
         <f>IF(E11&gt;0, F11/E11, IF(F11&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L11" s="36" t="inlineStr">
-        <is>
-          <t>Sin Pedido</t>
+      <c r="L11" s="32" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="B12" s="27" t="inlineStr">
         <is>
-          <t>ÇITAR ÇIÇEK TARIM TIC. LTD. STI</t>
+          <t>PLANTA SANA, D.O.O.</t>
         </is>
       </c>
       <c r="C12" s="28" t="inlineStr">
         <is>
-          <t>BIO1000</t>
+          <t>AVAN0001</t>
         </is>
       </c>
       <c r="D12" s="27" t="inlineStr">
         <is>
-          <t>BIORAD-20, 1000 L</t>
+          <t>FLORAMEC AVANCE</t>
         </is>
       </c>
       <c r="E12" s="14" t="n">
-        <v>10000</v>
+        <v>0</v>
       </c>
       <c r="F12" s="14" t="n">
-        <v>0</v>
+        <v>600</v>
       </c>
       <c r="G12" s="14" t="n">
         <v>0</v>
       </c>
       <c r="H12" s="14" t="n">
-        <v>0</v>
+        <v>600</v>
       </c>
       <c r="I12" s="14">
         <f>MAX(0, E12-F12)</f>
@@ -8523,39 +8661,39 @@
         <f>IF(E12&gt;0, F12/E12, IF(F12&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L12" s="33" t="inlineStr">
-        <is>
-          <t>Sin Pedido</t>
+      <c r="L12" s="29" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="B13" s="30" t="inlineStr">
         <is>
-          <t>ÇITAR ÇIÇEK TARIM TIC. LTD. STI</t>
+          <t>PLANTA SANA, D.O.O.</t>
         </is>
       </c>
       <c r="C13" s="31" t="inlineStr">
         <is>
-          <t>C-CU1000</t>
+          <t>C-CU0001</t>
         </is>
       </c>
       <c r="D13" s="30" t="inlineStr">
         <is>
-          <t>CODICOBRE, 1000 L</t>
+          <t>CODICOBRE</t>
         </is>
       </c>
       <c r="E13" s="18" t="n">
-        <v>2000</v>
+        <v>0</v>
       </c>
       <c r="F13" s="18" t="n">
-        <v>0</v>
+        <v>1008</v>
       </c>
       <c r="G13" s="18" t="n">
         <v>0</v>
       </c>
       <c r="H13" s="18" t="n">
-        <v>0</v>
+        <v>1008</v>
       </c>
       <c r="I13" s="18">
         <f>MAX(0, E13-F13)</f>
@@ -8569,16 +8707,16 @@
         <f>IF(E13&gt;0, F13/E13, IF(F13&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L13" s="36" t="inlineStr">
-        <is>
-          <t>Sin Pedido</t>
+      <c r="L13" s="32" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="B14" s="27" t="inlineStr">
         <is>
-          <t>ÇITAR ÇIÇEK TARIM TIC. LTD. STI</t>
+          <t>PLANTA SANA, D.O.O.</t>
         </is>
       </c>
       <c r="C14" s="28" t="inlineStr">
@@ -8588,20 +8726,20 @@
       </c>
       <c r="D14" s="27" t="inlineStr">
         <is>
-          <t>FITOKONTROL CA FLOW, 5 KG</t>
+          <t>FITOKONTROL CA FLOW</t>
         </is>
       </c>
       <c r="E14" s="14" t="n">
-        <v>10000</v>
+        <v>0</v>
       </c>
       <c r="F14" s="14" t="n">
-        <v>0</v>
+        <v>2200</v>
       </c>
       <c r="G14" s="14" t="n">
         <v>0</v>
       </c>
       <c r="H14" s="14" t="n">
-        <v>0</v>
+        <v>2200</v>
       </c>
       <c r="I14" s="14">
         <f>MAX(0, E14-F14)</f>
@@ -8615,39 +8753,39 @@
         <f>IF(E14&gt;0, F14/E14, IF(F14&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L14" s="33" t="inlineStr">
-        <is>
-          <t>Sin Pedido</t>
+      <c r="L14" s="29" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="30" t="inlineStr">
         <is>
-          <t>ÇITAR ÇIÇEK TARIM TIC. LTD. STI</t>
+          <t>PLANTA SANA, D.O.O.</t>
         </is>
       </c>
       <c r="C15" s="31" t="inlineStr">
         <is>
-          <t>RUN0001</t>
+          <t>FU0001</t>
         </is>
       </c>
       <c r="D15" s="30" t="inlineStr">
         <is>
-          <t>RUN STRESS, 1 L</t>
+          <t>FULVIGIN</t>
         </is>
       </c>
       <c r="E15" s="18" t="n">
-        <v>1960</v>
+        <v>0</v>
       </c>
       <c r="F15" s="18" t="n">
-        <v>0</v>
+        <v>204</v>
       </c>
       <c r="G15" s="18" t="n">
         <v>0</v>
       </c>
       <c r="H15" s="18" t="n">
-        <v>0</v>
+        <v>204</v>
       </c>
       <c r="I15" s="18">
         <f>MAX(0, E15-F15)</f>
@@ -8661,54 +8799,376 @@
         <f>IF(E15&gt;0, F15/E15, IF(F15&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L15" s="36" t="inlineStr">
+      <c r="L15" s="32" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="27" t="inlineStr">
+        <is>
+          <t>PLANTA SANA, D.O.O.</t>
+        </is>
+      </c>
+      <c r="C16" s="28" t="inlineStr">
+        <is>
+          <t>RUN0001</t>
+        </is>
+      </c>
+      <c r="D16" s="27" t="inlineStr">
+        <is>
+          <t>RUN STRESS, 1 L</t>
+        </is>
+      </c>
+      <c r="E16" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="14" t="n">
+        <v>1008</v>
+      </c>
+      <c r="G16" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="14" t="n">
+        <v>1008</v>
+      </c>
+      <c r="I16" s="14">
+        <f>MAX(0, E16-F16)</f>
+        <v/>
+      </c>
+      <c r="J16" s="14">
+        <f>ABS(F16-E16)</f>
+        <v/>
+      </c>
+      <c r="K16" s="15">
+        <f>IF(E16&gt;0, F16/E16, IF(F16&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L16" s="29" t="inlineStr">
+        <is>
+          <t>Extra Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="30" t="inlineStr">
+        <is>
+          <t>ÇITAR ÇIÇEK TARIM TIC. LTD. STI</t>
+        </is>
+      </c>
+      <c r="C17" s="31" t="inlineStr">
+        <is>
+          <t>AN0005</t>
+        </is>
+      </c>
+      <c r="D17" s="30" t="inlineStr">
+        <is>
+          <t>ALCAPLANT NEW, 5 KG</t>
+        </is>
+      </c>
+      <c r="E17" s="18" t="n">
+        <v>5500</v>
+      </c>
+      <c r="F17" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" s="18">
+        <f>MAX(0, E17-F17)</f>
+        <v/>
+      </c>
+      <c r="J17" s="18">
+        <f>ABS(F17-E17)</f>
+        <v/>
+      </c>
+      <c r="K17" s="19">
+        <f>IF(E17&gt;0, F17/E17, IF(F17&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L17" s="33" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="24" customHeight="1">
-      <c r="B16" s="20" t="inlineStr">
+    <row r="18">
+      <c r="B18" s="27" t="inlineStr">
+        <is>
+          <t>ÇITAR ÇIÇEK TARIM TIC. LTD. STI</t>
+        </is>
+      </c>
+      <c r="C18" s="28" t="inlineStr">
+        <is>
+          <t>BIO0020</t>
+        </is>
+      </c>
+      <c r="D18" s="27" t="inlineStr">
+        <is>
+          <t>BIORAD-20, 20 L</t>
+        </is>
+      </c>
+      <c r="E18" s="14" t="n">
+        <v>10000</v>
+      </c>
+      <c r="F18" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" s="14">
+        <f>MAX(0, E18-F18)</f>
+        <v/>
+      </c>
+      <c r="J18" s="14">
+        <f>ABS(F18-E18)</f>
+        <v/>
+      </c>
+      <c r="K18" s="15">
+        <f>IF(E18&gt;0, F18/E18, IF(F18&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L18" s="36" t="inlineStr">
+        <is>
+          <t>Sin Pedido</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="30" t="inlineStr">
+        <is>
+          <t>ÇITAR ÇIÇEK TARIM TIC. LTD. STI</t>
+        </is>
+      </c>
+      <c r="C19" s="31" t="inlineStr">
+        <is>
+          <t>BIO1000</t>
+        </is>
+      </c>
+      <c r="D19" s="30" t="inlineStr">
+        <is>
+          <t>BIORAD-20, 1000 L</t>
+        </is>
+      </c>
+      <c r="E19" s="18" t="n">
+        <v>10000</v>
+      </c>
+      <c r="F19" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="I19" s="18">
+        <f>MAX(0, E19-F19)</f>
+        <v/>
+      </c>
+      <c r="J19" s="18">
+        <f>ABS(F19-E19)</f>
+        <v/>
+      </c>
+      <c r="K19" s="19">
+        <f>IF(E19&gt;0, F19/E19, IF(F19&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L19" s="33" t="inlineStr">
+        <is>
+          <t>Sin Pedido</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="27" t="inlineStr">
+        <is>
+          <t>ÇITAR ÇIÇEK TARIM TIC. LTD. STI</t>
+        </is>
+      </c>
+      <c r="C20" s="28" t="inlineStr">
+        <is>
+          <t>C-CU1000</t>
+        </is>
+      </c>
+      <c r="D20" s="27" t="inlineStr">
+        <is>
+          <t>CODICOBRE, 1000 L</t>
+        </is>
+      </c>
+      <c r="E20" s="14" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F20" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I20" s="14">
+        <f>MAX(0, E20-F20)</f>
+        <v/>
+      </c>
+      <c r="J20" s="14">
+        <f>ABS(F20-E20)</f>
+        <v/>
+      </c>
+      <c r="K20" s="15">
+        <f>IF(E20&gt;0, F20/E20, IF(F20&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L20" s="36" t="inlineStr">
+        <is>
+          <t>Sin Pedido</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="30" t="inlineStr">
+        <is>
+          <t>ÇITAR ÇIÇEK TARIM TIC. LTD. STI</t>
+        </is>
+      </c>
+      <c r="C21" s="31" t="inlineStr">
+        <is>
+          <t>FTK0005</t>
+        </is>
+      </c>
+      <c r="D21" s="30" t="inlineStr">
+        <is>
+          <t>FITOKONTROL CA FLOW, 5 KG</t>
+        </is>
+      </c>
+      <c r="E21" s="18" t="n">
+        <v>10000</v>
+      </c>
+      <c r="F21" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="I21" s="18">
+        <f>MAX(0, E21-F21)</f>
+        <v/>
+      </c>
+      <c r="J21" s="18">
+        <f>ABS(F21-E21)</f>
+        <v/>
+      </c>
+      <c r="K21" s="19">
+        <f>IF(E21&gt;0, F21/E21, IF(F21&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L21" s="33" t="inlineStr">
+        <is>
+          <t>Sin Pedido</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="27" t="inlineStr">
+        <is>
+          <t>ÇITAR ÇIÇEK TARIM TIC. LTD. STI</t>
+        </is>
+      </c>
+      <c r="C22" s="28" t="inlineStr">
+        <is>
+          <t>RUN0001</t>
+        </is>
+      </c>
+      <c r="D22" s="27" t="inlineStr">
+        <is>
+          <t>RUN STRESS, 1 L</t>
+        </is>
+      </c>
+      <c r="E22" s="14" t="n">
+        <v>1960</v>
+      </c>
+      <c r="F22" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I22" s="14">
+        <f>MAX(0, E22-F22)</f>
+        <v/>
+      </c>
+      <c r="J22" s="14">
+        <f>ABS(F22-E22)</f>
+        <v/>
+      </c>
+      <c r="K22" s="15">
+        <f>IF(E22&gt;0, F22/E22, IF(F22&gt;0, 1, 0))</f>
+        <v/>
+      </c>
+      <c r="L22" s="36" t="inlineStr">
+        <is>
+          <t>Sin Pedido</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="24" customHeight="1">
+      <c r="B23" s="20" t="inlineStr">
         <is>
           <t>TOTAL MEHMET</t>
         </is>
       </c>
-      <c r="C16" s="34" t="inlineStr">
-        <is>
-          <t>61 líneas</t>
-        </is>
-      </c>
-      <c r="D16" s="35" t="inlineStr"/>
-      <c r="E16" s="22">
-        <f>SUM(E10:E15)</f>
-        <v/>
-      </c>
-      <c r="F16" s="22">
-        <f>SUM(F10:F15)</f>
-        <v/>
-      </c>
-      <c r="G16" s="22">
-        <f>SUM(G10:G15)</f>
-        <v/>
-      </c>
-      <c r="H16" s="22">
-        <f>SUM(H10:H15)</f>
-        <v/>
-      </c>
-      <c r="I16" s="22">
-        <f>SUM(I10:I15)</f>
-        <v/>
-      </c>
-      <c r="J16" s="22">
-        <f>SUM(J10:J15)</f>
-        <v/>
-      </c>
-      <c r="K16" s="23">
-        <f>IF(E16&gt;0, F16/E16, 0)</f>
-        <v/>
-      </c>
-      <c r="L16" s="21">
-        <f>IF(K16&gt;=1, "SUPERADO", "EN CURSO")</f>
+      <c r="C23" s="34" t="inlineStr">
+        <is>
+          <t>62 líneas</t>
+        </is>
+      </c>
+      <c r="D23" s="35" t="inlineStr"/>
+      <c r="E23" s="22">
+        <f>SUM(E10:E22)</f>
+        <v/>
+      </c>
+      <c r="F23" s="22">
+        <f>SUM(F10:F22)</f>
+        <v/>
+      </c>
+      <c r="G23" s="22">
+        <f>SUM(G10:G22)</f>
+        <v/>
+      </c>
+      <c r="H23" s="22">
+        <f>SUM(H10:H22)</f>
+        <v/>
+      </c>
+      <c r="I23" s="22">
+        <f>SUM(I10:I22)</f>
+        <v/>
+      </c>
+      <c r="J23" s="22">
+        <f>SUM(J10:J22)</f>
+        <v/>
+      </c>
+      <c r="K23" s="23">
+        <f>IF(E23&gt;0, F23/E23, 0)</f>
+        <v/>
+      </c>
+      <c r="L23" s="21">
+        <f>IF(K23&gt;=1, "SUPERADO", "EN CURSO")</f>
         <v/>
       </c>
     </row>
@@ -8764,7 +9224,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 27/10/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 28/10/2026</t>
         </is>
       </c>
     </row>
@@ -8982,7 +9442,7 @@
         <f>IF(E11&gt;0, F11/E11, IF(F11&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L11" s="36" t="inlineStr">
+      <c r="L11" s="33" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -9028,7 +9488,7 @@
         <f>IF(E12&gt;0, F12/E12, IF(F12&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L12" s="33" t="inlineStr">
+      <c r="L12" s="36" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -9212,7 +9672,7 @@
         <f>IF(E16&gt;0, F16/E16, IF(F16&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L16" s="33" t="inlineStr">
+      <c r="L16" s="36" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -9258,7 +9718,7 @@
         <f>IF(E17&gt;0, F17/E17, IF(F17&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L17" s="36" t="inlineStr">
+      <c r="L17" s="33" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -9534,7 +9994,7 @@
         <f>IF(E23&gt;0, F23/E23, IF(F23&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L23" s="36" t="inlineStr">
+      <c r="L23" s="33" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>
@@ -9821,7 +10281,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 27/10/2026</t>
+          <t>Seguimiento diario de Previsión Septiembre 2026 vs Pedidos a Fecha 28/10/2026</t>
         </is>
       </c>
     </row>
@@ -10085,7 +10545,7 @@
         <f>IF(E12&gt;0, F12/E12, IF(F12&gt;0, 1, 0))</f>
         <v/>
       </c>
-      <c r="L12" s="33" t="inlineStr">
+      <c r="L12" s="36" t="inlineStr">
         <is>
           <t>Sin Pedido</t>
         </is>

</xml_diff>